<commit_message>
Add BUAD-281 course calendar parser and workbook sheet
Extend auto_dissect.py with a Course Calendar fallback for point-based
schedules (exams, certifications, homework). Process BUAD-281 Managerial
Accounting calendar into syllabi.xlsx with PDF detail documents.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-281" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -46,7 +47,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +67,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCEFEF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF7F0E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEBDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF6EE"/>
       </patternFill>
     </fill>
   </fills>
@@ -95,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -205,6 +221,30 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -903,4 +943,288 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FF7F0E"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>BUAD-281 — Managerial Accounting</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Instructor</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Braunegg</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fall 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Required for an A</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Grading scale</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Total graded points in calendar: 1055 (letter scale not in document)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="40" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="C7" s="40" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="D7" s="40" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="E7" s="40" t="inlineStr">
+        <is>
+          <t>Group Project</t>
+        </is>
+      </c>
+      <c r="F7" s="40" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="41" t="inlineStr">
+        <is>
+          <t>Midterm 1</t>
+        </is>
+      </c>
+      <c r="B8" s="42" t="inlineStr">
+        <is>
+          <t>250 pts</t>
+        </is>
+      </c>
+      <c r="C8" s="42" t="inlineStr"/>
+      <c r="D8" s="42" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E8" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F8" s="43">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-midterm-1.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="44" t="inlineStr">
+        <is>
+          <t>Midterm 2</t>
+        </is>
+      </c>
+      <c r="B9" s="45" t="inlineStr">
+        <is>
+          <t>250 pts</t>
+        </is>
+      </c>
+      <c r="C9" s="45" t="inlineStr"/>
+      <c r="D9" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="E9" s="45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" s="46">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-midterm-2.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="41" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+      <c r="B10" s="42" t="inlineStr">
+        <is>
+          <t>250 pts</t>
+        </is>
+      </c>
+      <c r="C10" s="42" t="inlineStr"/>
+      <c r="D10" s="42" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="E10" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" s="43">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-final-exam.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="44" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B11" s="45" t="inlineStr">
+        <is>
+          <t>155 pts</t>
+        </is>
+      </c>
+      <c r="C11" s="45" t="inlineStr"/>
+      <c r="D11" s="45" t="inlineStr"/>
+      <c r="E11" s="45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" s="46">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-homework.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="41" t="inlineStr">
+        <is>
+          <t>LinkedIn Learning Excel Certification</t>
+        </is>
+      </c>
+      <c r="B12" s="42" t="inlineStr">
+        <is>
+          <t>75 pts</t>
+        </is>
+      </c>
+      <c r="C12" s="42" t="inlineStr"/>
+      <c r="D12" s="42" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E12" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F12" s="43">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-linkedin-learning-excel-certification.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="44" t="inlineStr">
+        <is>
+          <t>Stukent Simternship</t>
+        </is>
+      </c>
+      <c r="B13" s="45" t="inlineStr">
+        <is>
+          <t>75 pts</t>
+        </is>
+      </c>
+      <c r="C13" s="45" t="inlineStr"/>
+      <c r="D13" s="45" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E13" s="45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" s="46">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-stukent-simternship.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>1055 pts</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B5:F5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Retrain calendar extraction: PDF tables for clean verbatim
Past errors on BUAD-281 (~4/10): grep-only on table PDFs produced garbled
200-char fragments with cross-category noise. Fix:

- extract_text.py: embed pdfplumber table rows as CALENDAR_TABLE_JSON
- auto_dissect.py: structured row-per-line verbatim for calendar categories
- SKILL.md + reference.md: document two document types, past errors, quality rubric

Regenerate BUAD-281 PDFs with clean homework rows and scoped exam/review content.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -111,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -240,6 +240,30 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1014,7 +1038,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Total graded points in calendar: 1055 (letter scale not in document)</t>
+          <t>Total graded points in calendar: 1070 (letter scale not in document)</t>
         </is>
       </c>
     </row>
@@ -1056,23 +1080,23 @@
           <t>Midterm 1</t>
         </is>
       </c>
-      <c r="B8" s="42" t="inlineStr">
+      <c r="B8" s="51" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C8" s="42" t="inlineStr"/>
-      <c r="D8" s="42" t="inlineStr">
+      <c r="C8" s="51" t="inlineStr"/>
+      <c r="D8" s="51" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="E8" s="42" t="inlineStr">
+      <c r="E8" s="51" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F8" s="43">
+      <c r="F8" s="52">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-midterm-1.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1083,23 +1107,23 @@
           <t>Midterm 2</t>
         </is>
       </c>
-      <c r="B9" s="45" t="inlineStr">
+      <c r="B9" s="53" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C9" s="45" t="inlineStr"/>
-      <c r="D9" s="45" t="inlineStr">
+      <c r="C9" s="53" t="inlineStr"/>
+      <c r="D9" s="53" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E9" s="45" t="inlineStr">
+      <c r="E9" s="53" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F9" s="46">
+      <c r="F9" s="54">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-midterm-2.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1110,23 +1134,23 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B10" s="42" t="inlineStr">
+      <c r="B10" s="51" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C10" s="42" t="inlineStr"/>
-      <c r="D10" s="42" t="inlineStr">
+      <c r="C10" s="51" t="inlineStr"/>
+      <c r="D10" s="51" t="inlineStr">
         <is>
           <t>2026-12-16</t>
         </is>
       </c>
-      <c r="E10" s="42" t="inlineStr">
+      <c r="E10" s="51" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F10" s="43">
+      <c r="F10" s="52">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-final-exam.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1137,19 +1161,19 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B11" s="45" t="inlineStr">
-        <is>
-          <t>155 pts</t>
-        </is>
-      </c>
-      <c r="C11" s="45" t="inlineStr"/>
-      <c r="D11" s="45" t="inlineStr"/>
-      <c r="E11" s="45" t="inlineStr">
+      <c r="B11" s="53" t="inlineStr">
+        <is>
+          <t>170 pts</t>
+        </is>
+      </c>
+      <c r="C11" s="53" t="inlineStr"/>
+      <c r="D11" s="53" t="inlineStr"/>
+      <c r="E11" s="53" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F11" s="46">
+      <c r="F11" s="54">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-homework.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1160,23 +1184,23 @@
           <t>LinkedIn Learning Excel Certification</t>
         </is>
       </c>
-      <c r="B12" s="42" t="inlineStr">
+      <c r="B12" s="51" t="inlineStr">
         <is>
           <t>75 pts</t>
         </is>
       </c>
-      <c r="C12" s="42" t="inlineStr"/>
-      <c r="D12" s="42" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E12" s="42" t="inlineStr">
+      <c r="C12" s="51" t="inlineStr"/>
+      <c r="D12" s="51" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="E12" s="51" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F12" s="43">
+      <c r="F12" s="52">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-linkedin-learning-excel-certification.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1187,23 +1211,23 @@
           <t>Stukent Simternship</t>
         </is>
       </c>
-      <c r="B13" s="45" t="inlineStr">
+      <c r="B13" s="53" t="inlineStr">
         <is>
           <t>75 pts</t>
         </is>
       </c>
-      <c r="C13" s="45" t="inlineStr"/>
-      <c r="D13" s="45" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E13" s="45" t="inlineStr">
+      <c r="C13" s="53" t="inlineStr"/>
+      <c r="D13" s="53" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="E13" s="53" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F13" s="46">
+      <c r="F13" s="54">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-stukent-simternship.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1216,7 +1240,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>1055 pts</t>
+          <t>1070 pts</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Calendar v3: ISO homework dates, split certs, merged final, supplement merge
- Per-homework ISO due dates from calendar date column; Excel shows Sep 9 - Nov 16 range
- Split LinkedIn/Stukent into separate announcement vs submission lines per cert
- Merge final exam points, schedule, chapters, prerequisites into one Exam block
- Add --supplement flag to merge full syllabus for cert rubrics/instructions
- Strip cert noise from midterm review rows; fix cert start/due date inference

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -111,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -240,6 +240,30 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1080,23 +1104,23 @@
           <t>Midterm 1</t>
         </is>
       </c>
-      <c r="B8" s="51" t="inlineStr">
+      <c r="B8" s="59" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C8" s="51" t="inlineStr"/>
-      <c r="D8" s="51" t="inlineStr">
+      <c r="C8" s="59" t="inlineStr"/>
+      <c r="D8" s="59" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="E8" s="51" t="inlineStr">
+      <c r="E8" s="59" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F8" s="52">
+      <c r="F8" s="60">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-midterm-1.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1107,23 +1131,23 @@
           <t>Midterm 2</t>
         </is>
       </c>
-      <c r="B9" s="53" t="inlineStr">
+      <c r="B9" s="61" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C9" s="53" t="inlineStr"/>
-      <c r="D9" s="53" t="inlineStr">
+      <c r="C9" s="61" t="inlineStr"/>
+      <c r="D9" s="61" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E9" s="53" t="inlineStr">
+      <c r="E9" s="61" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F9" s="54">
+      <c r="F9" s="62">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-midterm-2.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1134,23 +1158,23 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B10" s="51" t="inlineStr">
+      <c r="B10" s="59" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C10" s="51" t="inlineStr"/>
-      <c r="D10" s="51" t="inlineStr">
+      <c r="C10" s="59" t="inlineStr"/>
+      <c r="D10" s="59" t="inlineStr">
         <is>
           <t>2026-12-16</t>
         </is>
       </c>
-      <c r="E10" s="51" t="inlineStr">
+      <c r="E10" s="59" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F10" s="52">
+      <c r="F10" s="60">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-final-exam.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1161,19 +1185,27 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B11" s="53" t="inlineStr">
+      <c r="B11" s="61" t="inlineStr">
         <is>
           <t>170 pts</t>
         </is>
       </c>
-      <c r="C11" s="53" t="inlineStr"/>
-      <c r="D11" s="53" t="inlineStr"/>
-      <c r="E11" s="53" t="inlineStr">
+      <c r="C11" s="61" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="D11" s="61" t="inlineStr">
+        <is>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="E11" s="61" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F11" s="54">
+      <c r="F11" s="62">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-homework.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1184,23 +1216,27 @@
           <t>LinkedIn Learning Excel Certification</t>
         </is>
       </c>
-      <c r="B12" s="51" t="inlineStr">
+      <c r="B12" s="59" t="inlineStr">
         <is>
           <t>75 pts</t>
         </is>
       </c>
-      <c r="C12" s="51" t="inlineStr"/>
-      <c r="D12" s="51" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="E12" s="51" t="inlineStr">
+      <c r="C12" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D12" s="59" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E12" s="59" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F12" s="52">
+      <c r="F12" s="60">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-linkedin-learning-excel-certification.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1211,23 +1247,27 @@
           <t>Stukent Simternship</t>
         </is>
       </c>
-      <c r="B13" s="53" t="inlineStr">
+      <c r="B13" s="61" t="inlineStr">
         <is>
           <t>75 pts</t>
         </is>
       </c>
-      <c r="C13" s="53" t="inlineStr"/>
-      <c r="D13" s="53" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="E13" s="53" t="inlineStr">
+      <c r="C13" s="61" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D13" s="61" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E13" s="61" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F13" s="54">
+      <c r="F13" s="62">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-stukent-simternship.pdf","Open PDF")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Integrate BUAD-304 research guide and Marshall schedule dates
Add Marshall syllabus mode for Course Evaluation + Course Schedule syllabi:
- Parse deliverable due dates from schedule prose (split-line and OCR fixes)
- Merge research participation guide into Participation category via --research-guide
- Fix is_group_project false positive for Participation
- Host research guide PDF in output/sources with research_guide_url in JSON
- Document BUAD-304 patterns in SKILL.md and reference.md

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -138,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -210,6 +210,30 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1346,23 +1370,23 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B9" s="32" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="C9" s="23" t="inlineStr"/>
-      <c r="D9" s="23" t="inlineStr">
+      <c r="C9" s="32" t="inlineStr"/>
+      <c r="D9" s="32" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E9" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F9" s="24">
+      <c r="E9" s="32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" s="33">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-final-exam.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1373,19 +1397,27 @@
           <t>Participation</t>
         </is>
       </c>
-      <c r="B10" s="26" t="inlineStr">
+      <c r="B10" s="34" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C10" s="26" t="inlineStr"/>
-      <c r="D10" s="26" t="inlineStr"/>
-      <c r="E10" s="26" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F10" s="27">
+      <c r="C10" s="34" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D10" s="34" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E10" s="34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" s="35">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-participation.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1396,19 +1428,23 @@
           <t>Midterm Exam</t>
         </is>
       </c>
-      <c r="B11" s="23" t="inlineStr">
+      <c r="B11" s="32" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C11" s="23" t="inlineStr"/>
-      <c r="D11" s="23" t="inlineStr"/>
-      <c r="E11" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F11" s="24">
+      <c r="C11" s="32" t="inlineStr"/>
+      <c r="D11" s="32" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E11" s="32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" s="33">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-midterm-exam.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1419,23 +1455,23 @@
           <t>Team Project Paper</t>
         </is>
       </c>
-      <c r="B12" s="26" t="inlineStr">
+      <c r="B12" s="34" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C12" s="26" t="inlineStr"/>
-      <c r="D12" s="26" t="inlineStr">
-        <is>
-          <t>2026-12-09</t>
-        </is>
-      </c>
-      <c r="E12" s="26" t="inlineStr">
+      <c r="C12" s="34" t="inlineStr"/>
+      <c r="D12" s="34" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E12" s="34" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F12" s="27">
+      <c r="F12" s="35">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-team-project-paper.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1446,23 +1482,23 @@
           <t>Final Reflection Paper</t>
         </is>
       </c>
-      <c r="B13" s="23" t="inlineStr">
+      <c r="B13" s="32" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C13" s="23" t="inlineStr"/>
-      <c r="D13" s="23" t="inlineStr">
-        <is>
-          <t>2026-12-09</t>
-        </is>
-      </c>
-      <c r="E13" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F13" s="24">
+      <c r="C13" s="32" t="inlineStr"/>
+      <c r="D13" s="32" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E13" s="32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" s="33">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-final-reflection-paper.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1473,23 +1509,23 @@
           <t>Presentation</t>
         </is>
       </c>
-      <c r="B14" s="26" t="inlineStr">
+      <c r="B14" s="34" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C14" s="26" t="inlineStr"/>
-      <c r="D14" s="26" t="inlineStr">
-        <is>
-          <t>2026-12-09</t>
-        </is>
-      </c>
-      <c r="E14" s="26" t="inlineStr">
+      <c r="C14" s="34" t="inlineStr"/>
+      <c r="D14" s="34" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E14" s="34" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F14" s="27">
+      <c r="F14" s="35">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-presentation.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1500,19 +1536,27 @@
           <t>Case Analysis Assignments</t>
         </is>
       </c>
-      <c r="B15" s="23" t="inlineStr">
+      <c r="B15" s="32" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C15" s="23" t="inlineStr"/>
-      <c r="D15" s="23" t="inlineStr"/>
-      <c r="E15" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F15" s="24">
+      <c r="C15" s="32" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="D15" s="32" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E15" s="32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F15" s="33">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-case-analysis-assignments.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1523,19 +1567,23 @@
           <t>Proposal &amp; Team Contract</t>
         </is>
       </c>
-      <c r="B16" s="26" t="inlineStr">
+      <c r="B16" s="34" t="inlineStr">
         <is>
           <t>3%</t>
         </is>
       </c>
-      <c r="C16" s="26" t="inlineStr"/>
-      <c r="D16" s="26" t="inlineStr"/>
-      <c r="E16" s="26" t="inlineStr">
+      <c r="C16" s="34" t="inlineStr"/>
+      <c r="D16" s="34" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E16" s="34" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F16" s="27">
+      <c r="F16" s="35">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-proposal-team-contract.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1546,23 +1594,23 @@
           <t>Self &amp; Peer Evaluation</t>
         </is>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B17" s="32" t="inlineStr">
         <is>
           <t>2%</t>
         </is>
       </c>
-      <c r="C17" s="23" t="inlineStr"/>
-      <c r="D17" s="23" t="inlineStr">
-        <is>
-          <t>2026-12-09</t>
-        </is>
-      </c>
-      <c r="E17" s="23" t="inlineStr">
+      <c r="C17" s="32" t="inlineStr"/>
+      <c r="D17" s="32" t="inlineStr">
+        <is>
+          <t>2026-11-18</t>
+        </is>
+      </c>
+      <c r="E17" s="32" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F17" s="24">
+      <c r="F17" s="33">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-self-peer-evaluation.pdf","Open PDF")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Populate BUAD-304 start dates from full Course Schedule
Infer start dates from schedule prose (team project explained 8/31,
USC-CT videos 8/26, first class 8/24). Add dated session rows per
category, team project outline due 10/19, and refresh source PDF.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -138,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -210,6 +210,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1370,23 +1382,27 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B9" s="32" t="inlineStr">
+      <c r="B9" s="36" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="C9" s="32" t="inlineStr"/>
-      <c r="D9" s="32" t="inlineStr">
+      <c r="C9" s="36" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D9" s="36" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E9" s="32" t="inlineStr">
+      <c r="E9" s="36" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F9" s="33">
+      <c r="F9" s="37">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-final-exam.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1397,27 +1413,27 @@
           <t>Participation</t>
         </is>
       </c>
-      <c r="B10" s="34" t="inlineStr">
+      <c r="B10" s="38" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C10" s="34" t="inlineStr">
+      <c r="C10" s="38" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D10" s="34" t="inlineStr">
+      <c r="D10" s="38" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E10" s="34" t="inlineStr">
+      <c r="E10" s="38" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F10" s="35">
+      <c r="F10" s="39">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-participation.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1428,23 +1444,27 @@
           <t>Midterm Exam</t>
         </is>
       </c>
-      <c r="B11" s="32" t="inlineStr">
+      <c r="B11" s="36" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C11" s="32" t="inlineStr"/>
-      <c r="D11" s="32" t="inlineStr">
+      <c r="C11" s="36" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D11" s="36" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E11" s="32" t="inlineStr">
+      <c r="E11" s="36" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F11" s="33">
+      <c r="F11" s="37">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-midterm-exam.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1455,23 +1475,27 @@
           <t>Team Project Paper</t>
         </is>
       </c>
-      <c r="B12" s="34" t="inlineStr">
+      <c r="B12" s="38" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C12" s="34" t="inlineStr"/>
-      <c r="D12" s="34" t="inlineStr">
+      <c r="C12" s="38" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D12" s="38" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E12" s="34" t="inlineStr">
+      <c r="E12" s="38" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F12" s="35">
+      <c r="F12" s="39">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-team-project-paper.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1482,23 +1506,27 @@
           <t>Final Reflection Paper</t>
         </is>
       </c>
-      <c r="B13" s="32" t="inlineStr">
+      <c r="B13" s="36" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C13" s="32" t="inlineStr"/>
-      <c r="D13" s="32" t="inlineStr">
+      <c r="C13" s="36" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D13" s="36" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E13" s="32" t="inlineStr">
+      <c r="E13" s="36" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F13" s="33">
+      <c r="F13" s="37">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-final-reflection-paper.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1509,23 +1537,27 @@
           <t>Presentation</t>
         </is>
       </c>
-      <c r="B14" s="34" t="inlineStr">
+      <c r="B14" s="38" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C14" s="34" t="inlineStr"/>
-      <c r="D14" s="34" t="inlineStr">
+      <c r="C14" s="38" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D14" s="38" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E14" s="34" t="inlineStr">
+      <c r="E14" s="38" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F14" s="35">
+      <c r="F14" s="39">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-presentation.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1536,27 +1568,27 @@
           <t>Case Analysis Assignments</t>
         </is>
       </c>
-      <c r="B15" s="32" t="inlineStr">
+      <c r="B15" s="36" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C15" s="32" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="D15" s="32" t="inlineStr">
+      <c r="C15" s="36" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D15" s="36" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E15" s="32" t="inlineStr">
+      <c r="E15" s="36" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F15" s="33">
+      <c r="F15" s="37">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-case-analysis-assignments.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1567,23 +1599,27 @@
           <t>Proposal &amp; Team Contract</t>
         </is>
       </c>
-      <c r="B16" s="34" t="inlineStr">
+      <c r="B16" s="38" t="inlineStr">
         <is>
           <t>3%</t>
         </is>
       </c>
-      <c r="C16" s="34" t="inlineStr"/>
-      <c r="D16" s="34" t="inlineStr">
+      <c r="C16" s="38" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D16" s="38" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E16" s="34" t="inlineStr">
+      <c r="E16" s="38" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F16" s="35">
+      <c r="F16" s="39">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-proposal-team-contract.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1594,23 +1630,27 @@
           <t>Self &amp; Peer Evaluation</t>
         </is>
       </c>
-      <c r="B17" s="32" t="inlineStr">
+      <c r="B17" s="36" t="inlineStr">
         <is>
           <t>2%</t>
         </is>
       </c>
-      <c r="C17" s="32" t="inlineStr"/>
-      <c r="D17" s="32" t="inlineStr">
+      <c r="C17" s="36" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D17" s="36" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E17" s="32" t="inlineStr">
+      <c r="E17" s="36" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F17" s="33">
+      <c r="F17" s="37">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-self-peer-evaluation.pdf","Open PDF")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add per-assignment start/due sub-rows on each Excel category
Expand BUAD-304 tabs with indented homework rows: Connect self-assessments
(Aug 24 - Dec 20), Sharpen Companion, research milestones, and each graded
deliverable from the Course Schedule. Calendar courses get one row per
homework problem set under the Homework category.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,8 +53,12 @@
       <color rgb="000563C1"/>
       <u val="single"/>
     </font>
+    <font>
+      <color rgb="00404040"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -111,6 +115,11 @@
         <fgColor rgb="00EFF5F9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F6F9FC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -138,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -245,6 +254,39 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1272,7 +1314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1382,286 +1424,982 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B9" s="36" t="inlineStr">
+      <c r="B9" s="46" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="C9" s="36" t="inlineStr">
+      <c r="C9" s="46" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D9" s="36" t="inlineStr">
+      <c r="D9" s="46" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E9" s="36" t="inlineStr">
+      <c r="E9" s="46" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F9" s="37">
+      <c r="F9" s="47">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-final-exam.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Final Exam</t>
+        </is>
+      </c>
+      <c r="B10" s="48" t="inlineStr"/>
+      <c r="C10" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D10" s="48" t="inlineStr">
+        <is>
+          <t>2026-12-09</t>
+        </is>
+      </c>
+      <c r="E10" s="48" t="inlineStr"/>
+      <c r="F10" s="48" t="inlineStr">
+        <is>
+          <t>Course Schedule due date</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="25" t="inlineStr">
         <is>
           <t>Participation</t>
         </is>
       </c>
-      <c r="B10" s="38" t="inlineStr">
+      <c r="B11" s="49" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C10" s="38" t="inlineStr">
+      <c r="C11" s="49" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D10" s="38" t="inlineStr">
+      <c r="D11" s="49" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E10" s="38" t="inlineStr">
+      <c r="E11" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F10" s="39">
+      <c r="F11" s="50">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-participation.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="22" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Research: Setup deadline (registration, prescreening, contacts)</t>
+        </is>
+      </c>
+      <c r="B12" s="48" t="inlineStr"/>
+      <c r="C12" s="48" t="inlineStr"/>
+      <c r="D12" s="48" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E12" s="48" t="inlineStr"/>
+      <c r="F12" s="48" t="inlineStr">
+        <is>
+          <t>Research Participation Guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Research: Employee contact surveys sent</t>
+        </is>
+      </c>
+      <c r="B13" s="48" t="inlineStr"/>
+      <c r="C13" s="48" t="inlineStr"/>
+      <c r="D13" s="48" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="E13" s="48" t="inlineStr"/>
+      <c r="F13" s="48" t="inlineStr">
+        <is>
+          <t>Research Participation Guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Research: Complete 2.0 research credits</t>
+        </is>
+      </c>
+      <c r="B14" s="48" t="inlineStr"/>
+      <c r="C14" s="48" t="inlineStr"/>
+      <c r="D14" s="48" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E14" s="48" t="inlineStr"/>
+      <c r="F14" s="48" t="inlineStr">
+        <is>
+          <t>Research Participation Guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Connect: Sharpen Companion</t>
+        </is>
+      </c>
+      <c r="B15" s="48" t="inlineStr"/>
+      <c r="C15" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="D15" s="48" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="E15" s="48" t="inlineStr"/>
+      <c r="F15" s="48" t="inlineStr">
+        <is>
+          <t>Brightspace Connect module</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Research: SONA registration opens</t>
+        </is>
+      </c>
+      <c r="B16" s="48" t="inlineStr"/>
+      <c r="C16" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D16" s="48" t="inlineStr"/>
+      <c r="E16" s="48" t="inlineStr"/>
+      <c r="F16" s="48" t="inlineStr">
+        <is>
+          <t>Research Participation Guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Connect: Self-Assessment 11.01 - What is my</t>
+        </is>
+      </c>
+      <c r="B17" s="48" t="inlineStr"/>
+      <c r="C17" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D17" s="48" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E17" s="48" t="inlineStr"/>
+      <c r="F17" s="48" t="inlineStr">
+        <is>
+          <t>Assigned in class week of 2026-09-09; Connect window</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Connect: Self-Assessment 11.02 - What is my</t>
+        </is>
+      </c>
+      <c r="B18" s="48" t="inlineStr"/>
+      <c r="C18" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D18" s="48" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E18" s="48" t="inlineStr"/>
+      <c r="F18" s="48" t="inlineStr">
+        <is>
+          <t>Assigned in class week of 2026-09-09; Connect window</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Connect: Self-Assessment 12.02 - Which influence</t>
+        </is>
+      </c>
+      <c r="B19" s="48" t="inlineStr"/>
+      <c r="C19" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D19" s="48" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E19" s="48" t="inlineStr"/>
+      <c r="F19" s="48" t="inlineStr">
+        <is>
+          <t>Assigned in class week of 2026-08-24; Connect window</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
+        </is>
+      </c>
+      <c r="B20" s="48" t="inlineStr"/>
+      <c r="C20" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D20" s="48" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E20" s="48" t="inlineStr"/>
+      <c r="F20" s="48" t="inlineStr">
+        <is>
+          <t>Assigned in class week of 2026-08-31; Connect window</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Connect: Self-Assessment 3.04 - What Is Your Level</t>
+        </is>
+      </c>
+      <c r="B21" s="48" t="inlineStr"/>
+      <c r="C21" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D21" s="48" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E21" s="48" t="inlineStr"/>
+      <c r="F21" s="48" t="inlineStr">
+        <is>
+          <t>Assigned in class week of 2026-08-31; Connect window</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Connect: Self-Assessment 5.01 - Assessing Your</t>
+        </is>
+      </c>
+      <c r="B22" s="48" t="inlineStr"/>
+      <c r="C22" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D22" s="48" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E22" s="48" t="inlineStr"/>
+      <c r="F22" s="48" t="inlineStr">
+        <is>
+          <t>Assigned in class week of 2026-09-02; Connect window</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Research: Prescreening questionnaire opens</t>
+        </is>
+      </c>
+      <c r="B23" s="48" t="inlineStr"/>
+      <c r="C23" s="48" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="D23" s="48" t="inlineStr"/>
+      <c r="E23" s="48" t="inlineStr"/>
+      <c r="F23" s="48" t="inlineStr">
+        <is>
+          <t>Research Participation Guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Research: Study invitations begin (after setup)</t>
+        </is>
+      </c>
+      <c r="B24" s="48" t="inlineStr"/>
+      <c r="C24" s="48" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="D24" s="48" t="inlineStr"/>
+      <c r="E24" s="48" t="inlineStr"/>
+      <c r="F24" s="48" t="inlineStr">
+        <is>
+          <t>Research Participation Guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="22" t="inlineStr">
         <is>
           <t>Midterm Exam</t>
         </is>
       </c>
-      <c r="B11" s="36" t="inlineStr">
+      <c r="B25" s="46" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C11" s="36" t="inlineStr">
+      <c r="C25" s="46" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D11" s="36" t="inlineStr">
+      <c r="D25" s="46" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E11" s="36" t="inlineStr">
+      <c r="E25" s="46" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F11" s="37">
+      <c r="F25" s="47">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-midterm-exam.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="25" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Midterm Exam</t>
+        </is>
+      </c>
+      <c r="B26" s="48" t="inlineStr"/>
+      <c r="C26" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D26" s="48" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E26" s="48" t="inlineStr"/>
+      <c r="F26" s="48" t="inlineStr">
+        <is>
+          <t>Course Schedule due date</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="25" t="inlineStr">
         <is>
           <t>Team Project Paper</t>
         </is>
       </c>
-      <c r="B12" s="38" t="inlineStr">
+      <c r="B27" s="49" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C12" s="38" t="inlineStr">
+      <c r="C27" s="49" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D12" s="38" t="inlineStr">
+      <c r="D27" s="49" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E12" s="38" t="inlineStr">
+      <c r="E27" s="49" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F12" s="39">
+      <c r="F27" s="50">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-team-project-paper.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="22" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Connect: Self-Assessment 14.02 - What Type of Organizational Culture Do I</t>
+        </is>
+      </c>
+      <c r="B28" s="48" t="inlineStr"/>
+      <c r="C28" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D28" s="48" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E28" s="48" t="inlineStr"/>
+      <c r="F28" s="48" t="inlineStr">
+        <is>
+          <t>Assigned in class week of 2026-11-04; Connect window</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Connect: Self-Assessment 8.01 - Group</t>
+        </is>
+      </c>
+      <c r="B29" s="48" t="inlineStr"/>
+      <c r="C29" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D29" s="48" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E29" s="48" t="inlineStr"/>
+      <c r="F29" s="48" t="inlineStr">
+        <is>
+          <t>Assigned in class week of 2026-10-19; Connect window</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Team project outline</t>
+        </is>
+      </c>
+      <c r="B30" s="48" t="inlineStr"/>
+      <c r="C30" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D30" s="48" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E30" s="48" t="inlineStr"/>
+      <c r="F30" s="48" t="inlineStr">
+        <is>
+          <t>Course Schedule due date</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Team project paper</t>
+        </is>
+      </c>
+      <c r="B31" s="48" t="inlineStr"/>
+      <c r="C31" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D31" s="48" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E31" s="48" t="inlineStr"/>
+      <c r="F31" s="48" t="inlineStr">
+        <is>
+          <t>Course Schedule due date</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="22" t="inlineStr">
         <is>
           <t>Final Reflection Paper</t>
         </is>
       </c>
-      <c r="B13" s="36" t="inlineStr">
+      <c r="B32" s="46" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C13" s="36" t="inlineStr">
+      <c r="C32" s="46" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D13" s="36" t="inlineStr">
+      <c r="D32" s="46" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E13" s="36" t="inlineStr">
+      <c r="E32" s="46" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F13" s="37">
+      <c r="F32" s="47">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-final-reflection-paper.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="25" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Connect: Self-Assessment 16.02 - What Is Your</t>
+        </is>
+      </c>
+      <c r="B33" s="48" t="inlineStr"/>
+      <c r="C33" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D33" s="48" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E33" s="48" t="inlineStr"/>
+      <c r="F33" s="48" t="inlineStr">
+        <is>
+          <t>Assigned in class week of 2026-11-30; Connect window</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Connect: Self-Assessment 16.03 - Assessing Your</t>
+        </is>
+      </c>
+      <c r="B34" s="48" t="inlineStr"/>
+      <c r="C34" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D34" s="48" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E34" s="48" t="inlineStr"/>
+      <c r="F34" s="48" t="inlineStr">
+        <is>
+          <t>Assigned in class week of 2026-11-30; Connect window</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Final Exam</t>
+        </is>
+      </c>
+      <c r="B35" s="48" t="inlineStr"/>
+      <c r="C35" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D35" s="48" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E35" s="48" t="inlineStr"/>
+      <c r="F35" s="48" t="inlineStr">
+        <is>
+          <t>Course Schedule due date</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="25" t="inlineStr">
         <is>
           <t>Presentation</t>
         </is>
       </c>
-      <c r="B14" s="38" t="inlineStr">
+      <c r="B36" s="49" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C14" s="38" t="inlineStr">
+      <c r="C36" s="49" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D14" s="38" t="inlineStr">
+      <c r="D36" s="49" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E14" s="38" t="inlineStr">
+      <c r="E36" s="49" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F14" s="39">
+      <c r="F36" s="50">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-presentation.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="22" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Presentation slides</t>
+        </is>
+      </c>
+      <c r="B37" s="48" t="inlineStr"/>
+      <c r="C37" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D37" s="48" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E37" s="48" t="inlineStr"/>
+      <c r="F37" s="48" t="inlineStr">
+        <is>
+          <t>Course Schedule due date</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="22" t="inlineStr">
         <is>
           <t>Case Analysis Assignments</t>
         </is>
       </c>
-      <c r="B15" s="36" t="inlineStr">
+      <c r="B38" s="46" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C15" s="36" t="inlineStr">
+      <c r="C38" s="46" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D15" s="36" t="inlineStr">
+      <c r="D38" s="46" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E15" s="36" t="inlineStr">
+      <c r="E38" s="46" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F15" s="37">
+      <c r="F38" s="47">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-case-analysis-assignments.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="25" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Connect: Self-Assessment 12.01 - What kind of</t>
+        </is>
+      </c>
+      <c r="B39" s="48" t="inlineStr"/>
+      <c r="C39" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D39" s="48" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E39" s="48" t="inlineStr"/>
+      <c r="F39" s="48" t="inlineStr">
+        <is>
+          <t>Assigned in class week of 2026-09-16; Connect window</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Thomas Green Case Analysis Memo</t>
+        </is>
+      </c>
+      <c r="B40" s="48" t="inlineStr"/>
+      <c r="C40" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D40" s="48" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E40" s="48" t="inlineStr"/>
+      <c r="F40" s="48" t="inlineStr">
+        <is>
+          <t>Course Schedule due date</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ SkillsForTomorrow Analysis Memo</t>
+        </is>
+      </c>
+      <c r="B41" s="48" t="inlineStr"/>
+      <c r="C41" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D41" s="48" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E41" s="48" t="inlineStr"/>
+      <c r="F41" s="48" t="inlineStr">
+        <is>
+          <t>Course Schedule due date</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="25" t="inlineStr">
         <is>
           <t>Proposal &amp; Team Contract</t>
         </is>
       </c>
-      <c r="B16" s="38" t="inlineStr">
+      <c r="B42" s="49" t="inlineStr">
         <is>
           <t>3%</t>
         </is>
       </c>
-      <c r="C16" s="38" t="inlineStr">
+      <c r="C42" s="49" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D16" s="38" t="inlineStr">
+      <c r="D42" s="49" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E16" s="38" t="inlineStr">
+      <c r="E42" s="49" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F16" s="39">
+      <c r="F42" s="50">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-proposal-team-contract.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="22" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Connect: Self-Assessment 10.5 - Preferred Conflict</t>
+        </is>
+      </c>
+      <c r="B43" s="48" t="inlineStr"/>
+      <c r="C43" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D43" s="48" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E43" s="48" t="inlineStr"/>
+      <c r="F43" s="48" t="inlineStr">
+        <is>
+          <t>Assigned in class week of 2026-09-28; Connect window</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Connect: Self-Assessment 9.01 - Assessing My</t>
+        </is>
+      </c>
+      <c r="B44" s="48" t="inlineStr"/>
+      <c r="C44" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D44" s="48" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E44" s="48" t="inlineStr"/>
+      <c r="F44" s="48" t="inlineStr">
+        <is>
+          <t>Assigned in class week of 2026-09-28; Connect window</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Team project proposal &amp; team contract</t>
+        </is>
+      </c>
+      <c r="B45" s="48" t="inlineStr"/>
+      <c r="C45" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D45" s="48" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E45" s="48" t="inlineStr"/>
+      <c r="F45" s="48" t="inlineStr">
+        <is>
+          <t>Course Schedule due date</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="22" t="inlineStr">
         <is>
           <t>Self &amp; Peer Evaluation</t>
         </is>
       </c>
-      <c r="B17" s="36" t="inlineStr">
+      <c r="B46" s="46" t="inlineStr">
         <is>
           <t>2%</t>
         </is>
       </c>
-      <c r="C17" s="36" t="inlineStr">
+      <c r="C46" s="46" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D17" s="36" t="inlineStr">
+      <c r="D46" s="46" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E17" s="36" t="inlineStr">
+      <c r="E46" s="46" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F17" s="37">
+      <c r="F46" s="47">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-self-peer-evaluation.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Self &amp; peer evaluation</t>
+        </is>
+      </c>
+      <c r="B47" s="48" t="inlineStr"/>
+      <c r="C47" s="48" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D47" s="48" t="inlineStr">
+        <is>
+          <t>2026-11-18</t>
+        </is>
+      </c>
+      <c r="E47" s="48" t="inlineStr"/>
+      <c r="F47" s="48" t="inlineStr">
+        <is>
+          <t>Course Schedule due date</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>100%</t>
         </is>

</xml_diff>

<commit_message>
Show N/A for start dates before August 1 of the term year
Applies to category rows and sub-assignments (e.g. Sharpen Companion
Jul 6 start becomes N/A for Fall 2026).

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -147,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -270,6 +270,21 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1424,27 +1439,27 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B9" s="46" t="inlineStr">
+      <c r="B9" s="51" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="C9" s="46" t="inlineStr">
+      <c r="C9" s="51" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D9" s="46" t="inlineStr">
+      <c r="D9" s="51" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E9" s="46" t="inlineStr">
+      <c r="E9" s="51" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F9" s="47">
+      <c r="F9" s="52">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-final-exam.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1455,19 +1470,19 @@
           <t xml:space="preserve">  ↳ Final Exam</t>
         </is>
       </c>
-      <c r="B10" s="48" t="inlineStr"/>
-      <c r="C10" s="48" t="inlineStr">
+      <c r="B10" s="53" t="inlineStr"/>
+      <c r="C10" s="53" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D10" s="48" t="inlineStr">
+      <c r="D10" s="53" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E10" s="48" t="inlineStr"/>
-      <c r="F10" s="48" t="inlineStr">
+      <c r="E10" s="53" t="inlineStr"/>
+      <c r="F10" s="53" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>
@@ -1479,27 +1494,27 @@
           <t>Participation</t>
         </is>
       </c>
-      <c r="B11" s="49" t="inlineStr">
+      <c r="B11" s="54" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C11" s="49" t="inlineStr">
+      <c r="C11" s="54" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D11" s="49" t="inlineStr">
+      <c r="D11" s="54" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E11" s="49" t="inlineStr">
+      <c r="E11" s="54" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F11" s="50">
+      <c r="F11" s="55">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-participation.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1510,15 +1525,15 @@
           <t xml:space="preserve">  ↳ Research: Setup deadline (registration, prescreening, contacts)</t>
         </is>
       </c>
-      <c r="B12" s="48" t="inlineStr"/>
-      <c r="C12" s="48" t="inlineStr"/>
-      <c r="D12" s="48" t="inlineStr">
+      <c r="B12" s="53" t="inlineStr"/>
+      <c r="C12" s="53" t="inlineStr"/>
+      <c r="D12" s="53" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="E12" s="48" t="inlineStr"/>
-      <c r="F12" s="48" t="inlineStr">
+      <c r="E12" s="53" t="inlineStr"/>
+      <c r="F12" s="53" t="inlineStr">
         <is>
           <t>Research Participation Guide</t>
         </is>
@@ -1530,15 +1545,15 @@
           <t xml:space="preserve">  ↳ Research: Employee contact surveys sent</t>
         </is>
       </c>
-      <c r="B13" s="48" t="inlineStr"/>
-      <c r="C13" s="48" t="inlineStr"/>
-      <c r="D13" s="48" t="inlineStr">
+      <c r="B13" s="53" t="inlineStr"/>
+      <c r="C13" s="53" t="inlineStr"/>
+      <c r="D13" s="53" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E13" s="48" t="inlineStr"/>
-      <c r="F13" s="48" t="inlineStr">
+      <c r="E13" s="53" t="inlineStr"/>
+      <c r="F13" s="53" t="inlineStr">
         <is>
           <t>Research Participation Guide</t>
         </is>
@@ -1550,15 +1565,15 @@
           <t xml:space="preserve">  ↳ Research: Complete 2.0 research credits</t>
         </is>
       </c>
-      <c r="B14" s="48" t="inlineStr"/>
-      <c r="C14" s="48" t="inlineStr"/>
-      <c r="D14" s="48" t="inlineStr">
+      <c r="B14" s="53" t="inlineStr"/>
+      <c r="C14" s="53" t="inlineStr"/>
+      <c r="D14" s="53" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E14" s="48" t="inlineStr"/>
-      <c r="F14" s="48" t="inlineStr">
+      <c r="E14" s="53" t="inlineStr"/>
+      <c r="F14" s="53" t="inlineStr">
         <is>
           <t>Research Participation Guide</t>
         </is>
@@ -1570,19 +1585,19 @@
           <t xml:space="preserve">  ↳ Connect: Sharpen Companion</t>
         </is>
       </c>
-      <c r="B15" s="48" t="inlineStr"/>
-      <c r="C15" s="48" t="inlineStr">
-        <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="D15" s="48" t="inlineStr">
+      <c r="B15" s="53" t="inlineStr"/>
+      <c r="C15" s="53" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D15" s="53" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E15" s="48" t="inlineStr"/>
-      <c r="F15" s="48" t="inlineStr">
+      <c r="E15" s="53" t="inlineStr"/>
+      <c r="F15" s="53" t="inlineStr">
         <is>
           <t>Brightspace Connect module</t>
         </is>
@@ -1594,15 +1609,15 @@
           <t xml:space="preserve">  ↳ Research: SONA registration opens</t>
         </is>
       </c>
-      <c r="B16" s="48" t="inlineStr"/>
-      <c r="C16" s="48" t="inlineStr">
+      <c r="B16" s="53" t="inlineStr"/>
+      <c r="C16" s="53" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D16" s="48" t="inlineStr"/>
-      <c r="E16" s="48" t="inlineStr"/>
-      <c r="F16" s="48" t="inlineStr">
+      <c r="D16" s="53" t="inlineStr"/>
+      <c r="E16" s="53" t="inlineStr"/>
+      <c r="F16" s="53" t="inlineStr">
         <is>
           <t>Research Participation Guide</t>
         </is>
@@ -1614,19 +1629,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 11.01 - What is my</t>
         </is>
       </c>
-      <c r="B17" s="48" t="inlineStr"/>
-      <c r="C17" s="48" t="inlineStr">
+      <c r="B17" s="53" t="inlineStr"/>
+      <c r="C17" s="53" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D17" s="48" t="inlineStr">
+      <c r="D17" s="53" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E17" s="48" t="inlineStr"/>
-      <c r="F17" s="48" t="inlineStr">
+      <c r="E17" s="53" t="inlineStr"/>
+      <c r="F17" s="53" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-09-09; Connect window</t>
         </is>
@@ -1638,19 +1653,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 11.02 - What is my</t>
         </is>
       </c>
-      <c r="B18" s="48" t="inlineStr"/>
-      <c r="C18" s="48" t="inlineStr">
+      <c r="B18" s="53" t="inlineStr"/>
+      <c r="C18" s="53" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D18" s="48" t="inlineStr">
+      <c r="D18" s="53" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E18" s="48" t="inlineStr"/>
-      <c r="F18" s="48" t="inlineStr">
+      <c r="E18" s="53" t="inlineStr"/>
+      <c r="F18" s="53" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-09-09; Connect window</t>
         </is>
@@ -1662,19 +1677,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 12.02 - Which influence</t>
         </is>
       </c>
-      <c r="B19" s="48" t="inlineStr"/>
-      <c r="C19" s="48" t="inlineStr">
+      <c r="B19" s="53" t="inlineStr"/>
+      <c r="C19" s="53" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D19" s="48" t="inlineStr">
+      <c r="D19" s="53" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E19" s="48" t="inlineStr"/>
-      <c r="F19" s="48" t="inlineStr">
+      <c r="E19" s="53" t="inlineStr"/>
+      <c r="F19" s="53" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-08-24; Connect window</t>
         </is>
@@ -1686,19 +1701,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
         </is>
       </c>
-      <c r="B20" s="48" t="inlineStr"/>
-      <c r="C20" s="48" t="inlineStr">
+      <c r="B20" s="53" t="inlineStr"/>
+      <c r="C20" s="53" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D20" s="48" t="inlineStr">
+      <c r="D20" s="53" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E20" s="48" t="inlineStr"/>
-      <c r="F20" s="48" t="inlineStr">
+      <c r="E20" s="53" t="inlineStr"/>
+      <c r="F20" s="53" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-08-31; Connect window</t>
         </is>
@@ -1710,19 +1725,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 3.04 - What Is Your Level</t>
         </is>
       </c>
-      <c r="B21" s="48" t="inlineStr"/>
-      <c r="C21" s="48" t="inlineStr">
+      <c r="B21" s="53" t="inlineStr"/>
+      <c r="C21" s="53" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D21" s="48" t="inlineStr">
+      <c r="D21" s="53" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E21" s="48" t="inlineStr"/>
-      <c r="F21" s="48" t="inlineStr">
+      <c r="E21" s="53" t="inlineStr"/>
+      <c r="F21" s="53" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-08-31; Connect window</t>
         </is>
@@ -1734,19 +1749,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 5.01 - Assessing Your</t>
         </is>
       </c>
-      <c r="B22" s="48" t="inlineStr"/>
-      <c r="C22" s="48" t="inlineStr">
+      <c r="B22" s="53" t="inlineStr"/>
+      <c r="C22" s="53" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D22" s="48" t="inlineStr">
+      <c r="D22" s="53" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E22" s="48" t="inlineStr"/>
-      <c r="F22" s="48" t="inlineStr">
+      <c r="E22" s="53" t="inlineStr"/>
+      <c r="F22" s="53" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-09-02; Connect window</t>
         </is>
@@ -1758,15 +1773,15 @@
           <t xml:space="preserve">  ↳ Research: Prescreening questionnaire opens</t>
         </is>
       </c>
-      <c r="B23" s="48" t="inlineStr"/>
-      <c r="C23" s="48" t="inlineStr">
+      <c r="B23" s="53" t="inlineStr"/>
+      <c r="C23" s="53" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="D23" s="48" t="inlineStr"/>
-      <c r="E23" s="48" t="inlineStr"/>
-      <c r="F23" s="48" t="inlineStr">
+      <c r="D23" s="53" t="inlineStr"/>
+      <c r="E23" s="53" t="inlineStr"/>
+      <c r="F23" s="53" t="inlineStr">
         <is>
           <t>Research Participation Guide</t>
         </is>
@@ -1778,15 +1793,15 @@
           <t xml:space="preserve">  ↳ Research: Study invitations begin (after setup)</t>
         </is>
       </c>
-      <c r="B24" s="48" t="inlineStr"/>
-      <c r="C24" s="48" t="inlineStr">
+      <c r="B24" s="53" t="inlineStr"/>
+      <c r="C24" s="53" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="D24" s="48" t="inlineStr"/>
-      <c r="E24" s="48" t="inlineStr"/>
-      <c r="F24" s="48" t="inlineStr">
+      <c r="D24" s="53" t="inlineStr"/>
+      <c r="E24" s="53" t="inlineStr"/>
+      <c r="F24" s="53" t="inlineStr">
         <is>
           <t>Research Participation Guide</t>
         </is>
@@ -1798,27 +1813,27 @@
           <t>Midterm Exam</t>
         </is>
       </c>
-      <c r="B25" s="46" t="inlineStr">
+      <c r="B25" s="51" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C25" s="46" t="inlineStr">
+      <c r="C25" s="51" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D25" s="46" t="inlineStr">
+      <c r="D25" s="51" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E25" s="46" t="inlineStr">
+      <c r="E25" s="51" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F25" s="47">
+      <c r="F25" s="52">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-midterm-exam.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1829,19 +1844,19 @@
           <t xml:space="preserve">  ↳ Midterm Exam</t>
         </is>
       </c>
-      <c r="B26" s="48" t="inlineStr"/>
-      <c r="C26" s="48" t="inlineStr">
+      <c r="B26" s="53" t="inlineStr"/>
+      <c r="C26" s="53" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D26" s="48" t="inlineStr">
+      <c r="D26" s="53" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E26" s="48" t="inlineStr"/>
-      <c r="F26" s="48" t="inlineStr">
+      <c r="E26" s="53" t="inlineStr"/>
+      <c r="F26" s="53" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>
@@ -1853,27 +1868,27 @@
           <t>Team Project Paper</t>
         </is>
       </c>
-      <c r="B27" s="49" t="inlineStr">
+      <c r="B27" s="54" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C27" s="49" t="inlineStr">
+      <c r="C27" s="54" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D27" s="49" t="inlineStr">
+      <c r="D27" s="54" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E27" s="49" t="inlineStr">
+      <c r="E27" s="54" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F27" s="50">
+      <c r="F27" s="55">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-team-project-paper.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1884,19 +1899,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 14.02 - What Type of Organizational Culture Do I</t>
         </is>
       </c>
-      <c r="B28" s="48" t="inlineStr"/>
-      <c r="C28" s="48" t="inlineStr">
+      <c r="B28" s="53" t="inlineStr"/>
+      <c r="C28" s="53" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D28" s="48" t="inlineStr">
+      <c r="D28" s="53" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E28" s="48" t="inlineStr"/>
-      <c r="F28" s="48" t="inlineStr">
+      <c r="E28" s="53" t="inlineStr"/>
+      <c r="F28" s="53" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-11-04; Connect window</t>
         </is>
@@ -1908,19 +1923,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 8.01 - Group</t>
         </is>
       </c>
-      <c r="B29" s="48" t="inlineStr"/>
-      <c r="C29" s="48" t="inlineStr">
+      <c r="B29" s="53" t="inlineStr"/>
+      <c r="C29" s="53" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D29" s="48" t="inlineStr">
+      <c r="D29" s="53" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E29" s="48" t="inlineStr"/>
-      <c r="F29" s="48" t="inlineStr">
+      <c r="E29" s="53" t="inlineStr"/>
+      <c r="F29" s="53" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-10-19; Connect window</t>
         </is>
@@ -1932,19 +1947,19 @@
           <t xml:space="preserve">  ↳ Team project outline</t>
         </is>
       </c>
-      <c r="B30" s="48" t="inlineStr"/>
-      <c r="C30" s="48" t="inlineStr">
+      <c r="B30" s="53" t="inlineStr"/>
+      <c r="C30" s="53" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D30" s="48" t="inlineStr">
+      <c r="D30" s="53" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E30" s="48" t="inlineStr"/>
-      <c r="F30" s="48" t="inlineStr">
+      <c r="E30" s="53" t="inlineStr"/>
+      <c r="F30" s="53" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>
@@ -1956,19 +1971,19 @@
           <t xml:space="preserve">  ↳ Team project paper</t>
         </is>
       </c>
-      <c r="B31" s="48" t="inlineStr"/>
-      <c r="C31" s="48" t="inlineStr">
+      <c r="B31" s="53" t="inlineStr"/>
+      <c r="C31" s="53" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D31" s="48" t="inlineStr">
+      <c r="D31" s="53" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E31" s="48" t="inlineStr"/>
-      <c r="F31" s="48" t="inlineStr">
+      <c r="E31" s="53" t="inlineStr"/>
+      <c r="F31" s="53" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>
@@ -1980,27 +1995,27 @@
           <t>Final Reflection Paper</t>
         </is>
       </c>
-      <c r="B32" s="46" t="inlineStr">
+      <c r="B32" s="51" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C32" s="46" t="inlineStr">
+      <c r="C32" s="51" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D32" s="46" t="inlineStr">
+      <c r="D32" s="51" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E32" s="46" t="inlineStr">
+      <c r="E32" s="51" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F32" s="47">
+      <c r="F32" s="52">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-final-reflection-paper.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -2011,19 +2026,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 16.02 - What Is Your</t>
         </is>
       </c>
-      <c r="B33" s="48" t="inlineStr"/>
-      <c r="C33" s="48" t="inlineStr">
+      <c r="B33" s="53" t="inlineStr"/>
+      <c r="C33" s="53" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D33" s="48" t="inlineStr">
+      <c r="D33" s="53" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E33" s="48" t="inlineStr"/>
-      <c r="F33" s="48" t="inlineStr">
+      <c r="E33" s="53" t="inlineStr"/>
+      <c r="F33" s="53" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-11-30; Connect window</t>
         </is>
@@ -2035,19 +2050,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 16.03 - Assessing Your</t>
         </is>
       </c>
-      <c r="B34" s="48" t="inlineStr"/>
-      <c r="C34" s="48" t="inlineStr">
+      <c r="B34" s="53" t="inlineStr"/>
+      <c r="C34" s="53" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D34" s="48" t="inlineStr">
+      <c r="D34" s="53" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E34" s="48" t="inlineStr"/>
-      <c r="F34" s="48" t="inlineStr">
+      <c r="E34" s="53" t="inlineStr"/>
+      <c r="F34" s="53" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-11-30; Connect window</t>
         </is>
@@ -2056,22 +2071,22 @@
     <row r="35">
       <c r="A35" s="42" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ Final Exam</t>
-        </is>
-      </c>
-      <c r="B35" s="48" t="inlineStr"/>
-      <c r="C35" s="48" t="inlineStr">
+          <t xml:space="preserve">  ↳ Personal Reflection Paper</t>
+        </is>
+      </c>
+      <c r="B35" s="53" t="inlineStr"/>
+      <c r="C35" s="53" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D35" s="48" t="inlineStr">
+      <c r="D35" s="53" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E35" s="48" t="inlineStr"/>
-      <c r="F35" s="48" t="inlineStr">
+      <c r="E35" s="53" t="inlineStr"/>
+      <c r="F35" s="53" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>
@@ -2083,27 +2098,27 @@
           <t>Presentation</t>
         </is>
       </c>
-      <c r="B36" s="49" t="inlineStr">
+      <c r="B36" s="54" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C36" s="49" t="inlineStr">
+      <c r="C36" s="54" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D36" s="49" t="inlineStr">
+      <c r="D36" s="54" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E36" s="49" t="inlineStr">
+      <c r="E36" s="54" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F36" s="50">
+      <c r="F36" s="55">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-presentation.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -2114,19 +2129,19 @@
           <t xml:space="preserve">  ↳ Presentation slides</t>
         </is>
       </c>
-      <c r="B37" s="48" t="inlineStr"/>
-      <c r="C37" s="48" t="inlineStr">
+      <c r="B37" s="53" t="inlineStr"/>
+      <c r="C37" s="53" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D37" s="48" t="inlineStr">
+      <c r="D37" s="53" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E37" s="48" t="inlineStr"/>
-      <c r="F37" s="48" t="inlineStr">
+      <c r="E37" s="53" t="inlineStr"/>
+      <c r="F37" s="53" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>
@@ -2138,27 +2153,27 @@
           <t>Case Analysis Assignments</t>
         </is>
       </c>
-      <c r="B38" s="46" t="inlineStr">
+      <c r="B38" s="51" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C38" s="46" t="inlineStr">
+      <c r="C38" s="51" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D38" s="46" t="inlineStr">
+      <c r="D38" s="51" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E38" s="46" t="inlineStr">
+      <c r="E38" s="51" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F38" s="47">
+      <c r="F38" s="52">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-case-analysis-assignments.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -2169,19 +2184,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 12.01 - What kind of</t>
         </is>
       </c>
-      <c r="B39" s="48" t="inlineStr"/>
-      <c r="C39" s="48" t="inlineStr">
+      <c r="B39" s="53" t="inlineStr"/>
+      <c r="C39" s="53" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D39" s="48" t="inlineStr">
+      <c r="D39" s="53" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E39" s="48" t="inlineStr"/>
-      <c r="F39" s="48" t="inlineStr">
+      <c r="E39" s="53" t="inlineStr"/>
+      <c r="F39" s="53" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-09-16; Connect window</t>
         </is>
@@ -2193,19 +2208,19 @@
           <t xml:space="preserve">  ↳ Thomas Green Case Analysis Memo</t>
         </is>
       </c>
-      <c r="B40" s="48" t="inlineStr"/>
-      <c r="C40" s="48" t="inlineStr">
+      <c r="B40" s="53" t="inlineStr"/>
+      <c r="C40" s="53" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D40" s="48" t="inlineStr">
+      <c r="D40" s="53" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E40" s="48" t="inlineStr"/>
-      <c r="F40" s="48" t="inlineStr">
+      <c r="E40" s="53" t="inlineStr"/>
+      <c r="F40" s="53" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>
@@ -2217,19 +2232,19 @@
           <t xml:space="preserve">  ↳ SkillsForTomorrow Analysis Memo</t>
         </is>
       </c>
-      <c r="B41" s="48" t="inlineStr"/>
-      <c r="C41" s="48" t="inlineStr">
+      <c r="B41" s="53" t="inlineStr"/>
+      <c r="C41" s="53" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D41" s="48" t="inlineStr">
+      <c r="D41" s="53" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E41" s="48" t="inlineStr"/>
-      <c r="F41" s="48" t="inlineStr">
+      <c r="E41" s="53" t="inlineStr"/>
+      <c r="F41" s="53" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>
@@ -2241,27 +2256,27 @@
           <t>Proposal &amp; Team Contract</t>
         </is>
       </c>
-      <c r="B42" s="49" t="inlineStr">
+      <c r="B42" s="54" t="inlineStr">
         <is>
           <t>3%</t>
         </is>
       </c>
-      <c r="C42" s="49" t="inlineStr">
+      <c r="C42" s="54" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D42" s="49" t="inlineStr">
+      <c r="D42" s="54" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E42" s="49" t="inlineStr">
+      <c r="E42" s="54" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F42" s="50">
+      <c r="F42" s="55">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-proposal-team-contract.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -2272,19 +2287,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 10.5 - Preferred Conflict</t>
         </is>
       </c>
-      <c r="B43" s="48" t="inlineStr"/>
-      <c r="C43" s="48" t="inlineStr">
+      <c r="B43" s="53" t="inlineStr"/>
+      <c r="C43" s="53" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D43" s="48" t="inlineStr">
+      <c r="D43" s="53" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E43" s="48" t="inlineStr"/>
-      <c r="F43" s="48" t="inlineStr">
+      <c r="E43" s="53" t="inlineStr"/>
+      <c r="F43" s="53" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-09-28; Connect window</t>
         </is>
@@ -2296,19 +2311,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 9.01 - Assessing My</t>
         </is>
       </c>
-      <c r="B44" s="48" t="inlineStr"/>
-      <c r="C44" s="48" t="inlineStr">
+      <c r="B44" s="53" t="inlineStr"/>
+      <c r="C44" s="53" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D44" s="48" t="inlineStr">
+      <c r="D44" s="53" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E44" s="48" t="inlineStr"/>
-      <c r="F44" s="48" t="inlineStr">
+      <c r="E44" s="53" t="inlineStr"/>
+      <c r="F44" s="53" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-09-28; Connect window</t>
         </is>
@@ -2320,19 +2335,19 @@
           <t xml:space="preserve">  ↳ Team project proposal &amp; team contract</t>
         </is>
       </c>
-      <c r="B45" s="48" t="inlineStr"/>
-      <c r="C45" s="48" t="inlineStr">
+      <c r="B45" s="53" t="inlineStr"/>
+      <c r="C45" s="53" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D45" s="48" t="inlineStr">
+      <c r="D45" s="53" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E45" s="48" t="inlineStr"/>
-      <c r="F45" s="48" t="inlineStr">
+      <c r="E45" s="53" t="inlineStr"/>
+      <c r="F45" s="53" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>
@@ -2344,27 +2359,27 @@
           <t>Self &amp; Peer Evaluation</t>
         </is>
       </c>
-      <c r="B46" s="46" t="inlineStr">
+      <c r="B46" s="51" t="inlineStr">
         <is>
           <t>2%</t>
         </is>
       </c>
-      <c r="C46" s="46" t="inlineStr">
+      <c r="C46" s="51" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D46" s="46" t="inlineStr">
+      <c r="D46" s="51" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E46" s="46" t="inlineStr">
+      <c r="E46" s="51" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F46" s="47">
+      <c r="F46" s="52">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-self-peer-evaluation.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -2375,19 +2390,19 @@
           <t xml:space="preserve">  ↳ Self &amp; peer evaluation</t>
         </is>
       </c>
-      <c r="B47" s="48" t="inlineStr"/>
-      <c r="C47" s="48" t="inlineStr">
+      <c r="B47" s="53" t="inlineStr"/>
+      <c r="C47" s="53" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D47" s="48" t="inlineStr">
+      <c r="D47" s="53" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E47" s="48" t="inlineStr"/>
-      <c r="F47" s="48" t="inlineStr">
+      <c r="E47" s="53" t="inlineStr"/>
+      <c r="F47" s="53" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>

</xml_diff>

<commit_message>
Add weekly homework/readings sub-rows for all classes in workbook
- HIST-103: parse full week-by-week schedule (readings, section prep, dues)
- BUAD-281: calendar rows include required reading and homework per class
- BUAD-304: unchanged Marshall Connect/deliverable sub-rows
- Regenerate all three sheets; start dates before Aug 1 show N/A

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -58,7 +58,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -120,6 +120,16 @@
         <fgColor rgb="00F6F9FC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDF6F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9F5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -147,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -293,6 +303,57 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -676,7 +737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -786,220 +847,1180 @@
           <t>Sleep Paper</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="56" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>2026-03-20</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="C9" s="56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D9" s="56" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="56" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="57">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-sleep-paper.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Sleep Paper Due</t>
+        </is>
+      </c>
+      <c r="B10" s="59" t="inlineStr"/>
+      <c r="C10" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D10" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="E10" s="59" t="inlineStr"/>
+      <c r="F10" s="59" t="inlineStr">
+        <is>
+          <t>Due date (course schedule)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 15-18: Renaissance</t>
+        </is>
+      </c>
+      <c r="B11" s="59" t="inlineStr"/>
+      <c r="C11" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D11" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="E11" s="59" t="inlineStr"/>
+      <c r="F11" s="59" t="inlineStr">
+        <is>
+          <t>Weekly schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Witchcraft Paper</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B12" s="60" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C12" s="60" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="D12" s="60" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E12" s="60" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F10" s="11">
+      <c r="F12" s="61">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-witchcraft-paper.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Witchcraft Paper Due</t>
+        </is>
+      </c>
+      <c r="B13" s="59" t="inlineStr"/>
+      <c r="C13" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="D13" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="E13" s="59" t="inlineStr"/>
+      <c r="F13" s="59" t="inlineStr">
+        <is>
+          <t>Due date (course schedule)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Nov 10-13: Enlightenment</t>
+        </is>
+      </c>
+      <c r="B14" s="59" t="inlineStr"/>
+      <c r="C14" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="D14" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-13</t>
+        </is>
+      </c>
+      <c r="E14" s="59" t="inlineStr"/>
+      <c r="F14" s="59" t="inlineStr">
+        <is>
+          <t>Weekly schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Mid-term</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B15" s="56" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C15" s="56" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D15" s="56" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E15" s="56" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F11" s="8">
+      <c r="F15" s="57">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-mid-term.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Midterm Exam</t>
+        </is>
+      </c>
+      <c r="B16" s="59" t="inlineStr"/>
+      <c r="C16" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="D16" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="E16" s="59" t="inlineStr"/>
+      <c r="F16" s="59" t="inlineStr">
+        <is>
+          <t>Oct 6: Midterm</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Oct 6-9: Midterm &amp; Break</t>
+        </is>
+      </c>
+      <c r="B17" s="59" t="inlineStr"/>
+      <c r="C17" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="D17" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E17" s="59" t="inlineStr"/>
+      <c r="F17" s="59" t="inlineStr">
+        <is>
+          <t>Weekly schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Dec 1-4: Modern Europe?</t>
+        </is>
+      </c>
+      <c r="B18" s="59" t="inlineStr"/>
+      <c r="C18" s="59" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="D18" s="59" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E18" s="59" t="inlineStr"/>
+      <c r="F18" s="59" t="inlineStr">
+        <is>
+          <t>Weekly schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B19" s="60" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>2026-12-10</t>
-        </is>
-      </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="C19" s="60" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D19" s="60" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E19" s="60" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F12" s="11">
+      <c r="F19" s="61">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-final-exam.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Final Exam</t>
+        </is>
+      </c>
+      <c r="B20" s="59" t="inlineStr"/>
+      <c r="C20" s="59" t="inlineStr">
+        <is>
+          <t>2026-12-10</t>
+        </is>
+      </c>
+      <c r="D20" s="59" t="inlineStr">
+        <is>
+          <t>2026-12-10</t>
+        </is>
+      </c>
+      <c r="E20" s="59" t="inlineStr"/>
+      <c r="F20" s="59" t="inlineStr">
+        <is>
+          <t>Dec 10: Final Exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Discussion Section</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B21" s="56" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C21" s="56" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D21" s="56" t="inlineStr">
         <is>
           <t>2026-11-12</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E21" s="56" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F13" s="8">
+      <c r="F21" s="57">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-discussion-section.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Aug 25-29: Intro &amp; Black Death</t>
+        </is>
+      </c>
+      <c r="B22" s="59" t="inlineStr"/>
+      <c r="C22" s="59" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D22" s="59" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="E22" s="59" t="inlineStr"/>
+      <c r="F22" s="59" t="inlineStr">
+        <is>
+          <t>Weekly schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Aug 25-29: Intro &amp; Black Death  -  Section readings 1</t>
+        </is>
+      </c>
+      <c r="B23" s="59" t="inlineStr"/>
+      <c r="C23" s="59" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D23" s="59" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="E23" s="59" t="inlineStr"/>
+      <c r="F23" s="59" t="inlineStr">
+        <is>
+          <t>-- 13 of 33 -- Lizzie Wade, “From Black Death to fatal flu, past pandemics show why people on the margins suffer most,” Science, May 14, 2020 Alex Brown and Grace Owen, “What a list of Black Death Sur</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 1-4: Everyday Life</t>
+        </is>
+      </c>
+      <c r="B24" s="59" t="inlineStr"/>
+      <c r="C24" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D24" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="E24" s="59" t="inlineStr"/>
+      <c r="F24" s="59" t="inlineStr">
+        <is>
+          <t>Weekly schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 1-4: Everyday Life  -  Section readings 1</t>
+        </is>
+      </c>
+      <c r="B25" s="59" t="inlineStr"/>
+      <c r="C25" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D25" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="E25" s="59" t="inlineStr"/>
+      <c r="F25" s="59" t="inlineStr">
+        <is>
+          <t>A Roger Ekirch, “Sleep we have lost: Pre-Industrial Slumber in the British Isles, The American Historical Review, April 2001, pg. 343-365 Sasha Handley, Sleep in Early Modern England, Introduction &amp; C</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 8-11: Renaissance</t>
+        </is>
+      </c>
+      <c r="B26" s="59" t="inlineStr"/>
+      <c r="C26" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="D26" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E26" s="59" t="inlineStr"/>
+      <c r="F26" s="59" t="inlineStr">
+        <is>
+          <t>Weekly schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 8-11: Renaissance  -  Section readings 1</t>
+        </is>
+      </c>
+      <c r="B27" s="59" t="inlineStr"/>
+      <c r="C27" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="D27" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E27" s="59" t="inlineStr"/>
+      <c r="F27" s="59" t="inlineStr">
+        <is>
+          <t>-- 14 of 33 -- Kay Daly, “Diverting the Flood of History: Ada Palmer’s Inventing the Renaissance,” Chicago Review of Books, 25 March 2025 Ada Palmer, “Black Death, COVID, and Why We Keep Telling the M</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 15-18: Renaissance  -  Section readings 1</t>
+        </is>
+      </c>
+      <c r="B28" s="59" t="inlineStr"/>
+      <c r="C28" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D28" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="E28" s="59" t="inlineStr"/>
+      <c r="F28" s="59" t="inlineStr">
+        <is>
+          <t>Vasari, Lives of the Artists: Leonardo da Vinci &amp; Properzia de’ Rossi Video: The Story of Women and Art, Part 1(1hr) Vasari on da Vinci PDF document Vasari on d'Rossi PDF document</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 20-24: European Expansion</t>
+        </is>
+      </c>
+      <c r="B29" s="59" t="inlineStr"/>
+      <c r="C29" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D29" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E29" s="59" t="inlineStr"/>
+      <c r="F29" s="59" t="inlineStr">
+        <is>
+          <t>Weekly schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 20-24: European Expansion  -  Section readings 1</t>
+        </is>
+      </c>
+      <c r="B30" s="59" t="inlineStr"/>
+      <c r="C30" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D30" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E30" s="59" t="inlineStr"/>
+      <c r="F30" s="59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jerry Brotton, The Renaissance Bazaar, Chap 1 (15 pgs) Read Columbus’ Letter on his Return: MacGregor, The History of the World in 100 Objects Read or listen to the stories behind these objects: Part </t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 20-24: European Expansion  -  Section readings 2</t>
+        </is>
+      </c>
+      <c r="B31" s="59" t="inlineStr"/>
+      <c r="C31" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D31" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E31" s="59" t="inlineStr"/>
+      <c r="F31" s="59" t="inlineStr">
+        <is>
+          <t>Bernal Diaz del Castillo, The True History of the Conquest of New Spain, pg 121-171 Miguel León Portilla, Broken Spears: The Aztec Account of the Conquest of Mexico, Appendix, Chap 8-10 (37 pgs) Broke</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Oct 13-16: The Reformation</t>
+        </is>
+      </c>
+      <c r="B32" s="59" t="inlineStr"/>
+      <c r="C32" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="D32" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="E32" s="59" t="inlineStr"/>
+      <c r="F32" s="59" t="inlineStr">
+        <is>
+          <t>Weekly schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Oct 20-23: The Reformation</t>
+        </is>
+      </c>
+      <c r="B33" s="59" t="inlineStr"/>
+      <c r="C33" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="D33" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="E33" s="59" t="inlineStr"/>
+      <c r="F33" s="59" t="inlineStr">
+        <is>
+          <t>Weekly schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Oct 27-30: Reformation</t>
+        </is>
+      </c>
+      <c r="B34" s="59" t="inlineStr"/>
+      <c r="C34" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="D34" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="E34" s="59" t="inlineStr"/>
+      <c r="F34" s="59" t="inlineStr">
+        <is>
+          <t>Weekly schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Oct 27-30: Reformation  -  Section readings 1</t>
+        </is>
+      </c>
+      <c r="B35" s="59" t="inlineStr"/>
+      <c r="C35" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="D35" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="E35" s="59" t="inlineStr"/>
+      <c r="F35" s="59" t="inlineStr">
+        <is>
+          <t>Barbara Diefendorf, ed., The Saint Bartholomew’s Day Massacre: A Brief History with Documents, Introduction, Documents 2-6, 9-11, 16-21, 31, 33</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Nov 3-6: Witches &amp; Science</t>
+        </is>
+      </c>
+      <c r="B36" s="59" t="inlineStr"/>
+      <c r="C36" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="D36" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="E36" s="59" t="inlineStr"/>
+      <c r="F36" s="59" t="inlineStr">
+        <is>
+          <t>Weekly schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Nov 3-6: Witches &amp; Science  -  Section readings 1</t>
+        </is>
+      </c>
+      <c r="B37" s="59" t="inlineStr"/>
+      <c r="C37" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="D37" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="E37" s="59" t="inlineStr"/>
+      <c r="F37" s="59" t="inlineStr">
+        <is>
+          <t>Brian Levack, The Witchcraft Sourcebook, Chaps 36-44, 46-47 103.Levack.36 PDF document 103.Levack.37 PDF document 103.Levack.38 PDF document 103.Levack.39 PDF document 103.Levack.40 PDF document 103.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Nov 10-13: Enlightenment  -  Section readings 1</t>
+        </is>
+      </c>
+      <c r="B38" s="59" t="inlineStr"/>
+      <c r="C38" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="D38" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-13</t>
+        </is>
+      </c>
+      <c r="E38" s="59" t="inlineStr"/>
+      <c r="F38" s="59" t="inlineStr">
+        <is>
+          <t>Excerpt: John Locke, Two Treatises of Government (1689) Excerpt: Rousseau, The Social Contract (1762) Enlightenment Primary Source Activity [Ungraded, but counts towards participation. Due in section]</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Nov 17-20: Enlightenment</t>
+        </is>
+      </c>
+      <c r="B39" s="59" t="inlineStr"/>
+      <c r="C39" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-17</t>
+        </is>
+      </c>
+      <c r="D39" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="E39" s="59" t="inlineStr"/>
+      <c r="F39" s="59" t="inlineStr">
+        <is>
+          <t>Weekly schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Nov 17-20: Enlightenment  -  Section readings 1</t>
+        </is>
+      </c>
+      <c r="B40" s="59" t="inlineStr"/>
+      <c r="C40" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-17</t>
+        </is>
+      </c>
+      <c r="D40" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="E40" s="59" t="inlineStr"/>
+      <c r="F40" s="59" t="inlineStr">
+        <is>
+          <t>Video: Africa &amp; Britain, A Forgotten History, Episode 2: Freedom (50 min) Slavery and the African Presence in London Activity [Ungraded but counts towards participation. Due in section] 103.Act.Enslav</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
         <is>
           <t>Identification Quizzes</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B41" s="60" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C41" s="60" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D41" s="60" t="inlineStr">
         <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="E41" s="60" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F14" s="11">
+      <c r="F41" s="61">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-identification-quizzes.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Aug 25-29: Intro &amp; Black Death (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B42" s="59" t="inlineStr"/>
+      <c r="C42" s="59" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D42" s="59" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="E42" s="59" t="inlineStr"/>
+      <c r="F42" s="59" t="inlineStr">
+        <is>
+          <t>Weekly lecture - quiz prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 1-4: Everyday Life (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B43" s="59" t="inlineStr"/>
+      <c r="C43" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D43" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="E43" s="59" t="inlineStr"/>
+      <c r="F43" s="59" t="inlineStr">
+        <is>
+          <t>Weekly lecture - quiz prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 8-11: Renaissance (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B44" s="59" t="inlineStr"/>
+      <c r="C44" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="D44" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E44" s="59" t="inlineStr"/>
+      <c r="F44" s="59" t="inlineStr">
+        <is>
+          <t>Weekly lecture - quiz prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 15-18: Renaissance (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B45" s="59" t="inlineStr"/>
+      <c r="C45" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D45" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="E45" s="59" t="inlineStr"/>
+      <c r="F45" s="59" t="inlineStr">
+        <is>
+          <t>Weekly lecture - quiz prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 20-24: European Expansion (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B46" s="59" t="inlineStr"/>
+      <c r="C46" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D46" s="59" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E46" s="59" t="inlineStr"/>
+      <c r="F46" s="59" t="inlineStr">
+        <is>
+          <t>Weekly lecture - quiz prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Oct 6-9: Midterm &amp; Break (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B47" s="59" t="inlineStr"/>
+      <c r="C47" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="D47" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E47" s="59" t="inlineStr"/>
+      <c r="F47" s="59" t="inlineStr">
+        <is>
+          <t>Weekly lecture - quiz prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Oct 13-16: The Reformation (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B48" s="59" t="inlineStr"/>
+      <c r="C48" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="D48" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="E48" s="59" t="inlineStr"/>
+      <c r="F48" s="59" t="inlineStr">
+        <is>
+          <t>Weekly lecture - quiz prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Oct 20-23: The Reformation (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B49" s="59" t="inlineStr"/>
+      <c r="C49" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="D49" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="E49" s="59" t="inlineStr"/>
+      <c r="F49" s="59" t="inlineStr">
+        <is>
+          <t>Weekly lecture - quiz prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Oct 27-30: Reformation (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B50" s="59" t="inlineStr"/>
+      <c r="C50" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="D50" s="59" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="E50" s="59" t="inlineStr"/>
+      <c r="F50" s="59" t="inlineStr">
+        <is>
+          <t>Weekly lecture - quiz prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Nov 3-6: Witches &amp; Science (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B51" s="59" t="inlineStr"/>
+      <c r="C51" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="D51" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="E51" s="59" t="inlineStr"/>
+      <c r="F51" s="59" t="inlineStr">
+        <is>
+          <t>Weekly lecture - quiz prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Nov 10-13: Enlightenment (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B52" s="59" t="inlineStr"/>
+      <c r="C52" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="D52" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-13</t>
+        </is>
+      </c>
+      <c r="E52" s="59" t="inlineStr"/>
+      <c r="F52" s="59" t="inlineStr">
+        <is>
+          <t>Weekly lecture - quiz prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Nov 17-20: Enlightenment (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B53" s="59" t="inlineStr"/>
+      <c r="C53" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-17</t>
+        </is>
+      </c>
+      <c r="D53" s="59" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="E53" s="59" t="inlineStr"/>
+      <c r="F53" s="59" t="inlineStr">
+        <is>
+          <t>Weekly lecture - quiz prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Dec 1-4: Modern Europe? (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B54" s="59" t="inlineStr"/>
+      <c r="C54" s="59" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="D54" s="59" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E54" s="59" t="inlineStr"/>
+      <c r="F54" s="59" t="inlineStr">
+        <is>
+          <t>Weekly lecture - quiz prep</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t>Extra Credit</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B55" s="56" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr"/>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="C55" s="56" t="inlineStr"/>
+      <c r="D55" s="56" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E55" s="56" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F15" s="8">
+      <c r="F55" s="57">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-extra-credit.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
@@ -1022,7 +2043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1132,181 +2153,973 @@
           <t>Midterm 1</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="62" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr"/>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="C9" s="62" t="inlineStr"/>
+      <c r="D9" s="62" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="62" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F9" s="16">
+      <c r="F9" s="63">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-midterm-1.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ 9/30 Midterm 1: 250 Points Chapters 1, 2, 3, 4, 5, 8</t>
+        </is>
+      </c>
+      <c r="B10" s="65" t="inlineStr"/>
+      <c r="C10" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="D10" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E10" s="65" t="inlineStr"/>
+      <c r="F10" s="65" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Midterm 2</t>
         </is>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B11" s="66" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C10" s="18" t="inlineStr"/>
-      <c r="D10" s="18" t="inlineStr">
+      <c r="C11" s="66" t="inlineStr"/>
+      <c r="D11" s="66" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E10" s="18" t="inlineStr">
+      <c r="E11" s="66" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F10" s="19">
+      <c r="F11" s="67">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-midterm-2.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ 10/26 Midterm 2: 250 Points Chapters 6, 7, 9, &amp; 16</t>
+        </is>
+      </c>
+      <c r="B12" s="65" t="inlineStr"/>
+      <c r="C12" s="65" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="D12" s="65" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="E12" s="65" t="inlineStr"/>
+      <c r="F12" s="65" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B11" s="15" t="inlineStr">
+      <c r="B13" s="62" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr"/>
-      <c r="D11" s="15" t="inlineStr">
+      <c r="C13" s="62" t="inlineStr"/>
+      <c r="D13" s="62" t="inlineStr">
         <is>
           <t>2026-12-16</t>
         </is>
       </c>
-      <c r="E11" s="15" t="inlineStr">
+      <c r="E13" s="62" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F11" s="16">
+      <c r="F13" s="63">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-final-exam.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Final Exam</t>
+        </is>
+      </c>
+      <c r="B14" s="65" t="inlineStr"/>
+      <c r="C14" s="65" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="D14" s="65" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="E14" s="65" t="inlineStr"/>
+      <c r="F14" s="65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Final Exam: 250 Points | Final Exam; Wednesday,; December 16th; 8:00 AM -10:00 AM PST | ISO date: 2026-12-16 | Chapters </t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="B12" s="18" t="inlineStr">
+      <c r="B15" s="66" t="inlineStr">
         <is>
           <t>170 pts</t>
         </is>
       </c>
-      <c r="C12" s="18" t="inlineStr">
+      <c r="C15" s="66" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="D12" s="18" t="inlineStr">
+      <c r="D15" s="66" t="inlineStr">
         <is>
           <t>2026-11-16</t>
         </is>
       </c>
-      <c r="E12" s="18" t="inlineStr">
+      <c r="E15" s="66" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F12" s="19">
+      <c r="F15" s="67">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-homework.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 1 (8/24)  -  Course Overview &amp; Introductions</t>
+        </is>
+      </c>
+      <c r="B16" s="65" t="inlineStr"/>
+      <c r="C16" s="65" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D16" s="65" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="E16" s="65" t="inlineStr"/>
+      <c r="F16" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Course Overview &amp; Introductions</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 2 (8/26)  -  Role of Managerial accounting</t>
+        </is>
+      </c>
+      <c r="B17" s="65" t="inlineStr"/>
+      <c r="C17" s="65" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D17" s="65" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="E17" s="65" t="inlineStr"/>
+      <c r="F17" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Role of Managerial accounting | Required Reading: Chapter 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 3 (8/31)  -  Basic Cost Mgt Concepts</t>
+        </is>
+      </c>
+      <c r="B18" s="65" t="inlineStr"/>
+      <c r="C18" s="65" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D18" s="65" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E18" s="65" t="inlineStr"/>
+      <c r="F18" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Basic Cost Mgt Concepts | Required Reading: Chapter 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 4 (9/2)  -  Basic Cost Mgt Concepts</t>
+        </is>
+      </c>
+      <c r="B19" s="65" t="inlineStr"/>
+      <c r="C19" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="D19" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E19" s="65" t="inlineStr"/>
+      <c r="F19" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Basic Cost Mgt Concepts | Required Reading: Chapter 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ 9/7  -  No Class Labor Day Holiday</t>
+        </is>
+      </c>
+      <c r="B20" s="65" t="inlineStr"/>
+      <c r="C20" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="D20" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="E20" s="65" t="inlineStr"/>
+      <c r="F20" s="65" t="inlineStr">
+        <is>
+          <t>Topic: No Class Labor Day Holiday</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 5 (9/9)  -  Product Cost Accumulation: Job; Order Costing</t>
+        </is>
+      </c>
+      <c r="B21" s="65" t="inlineStr"/>
+      <c r="C21" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="D21" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="E21" s="65" t="inlineStr"/>
+      <c r="F21" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Product Cost Accumulation: Job; Order Costing | Required Reading: Chapter 3 | Homework: 2-29, 2-30, 2-40; 15 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 6 (9/14)  -  Manufacturing Overhead Normal; Costing</t>
+        </is>
+      </c>
+      <c r="B22" s="65" t="inlineStr"/>
+      <c r="C22" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D22" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="E22" s="65" t="inlineStr"/>
+      <c r="F22" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Manufacturing Overhead Normal; Costing | Required Reading: Chapter 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 7 (9/16)  -  Activity Based Costing</t>
+        </is>
+      </c>
+      <c r="B23" s="65" t="inlineStr"/>
+      <c r="C23" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="D23" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E23" s="65" t="inlineStr"/>
+      <c r="F23" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Activity Based Costing | Required Reading: Chapter 5- ONLY; LO 5.1, 2, 4 &amp; 5 | Homework: 3-24, 3-28, 3-32; 15 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 8 (9/21)  -  Product Cost Accumulation: Pro-; cess Costing</t>
+        </is>
+      </c>
+      <c r="B24" s="65" t="inlineStr"/>
+      <c r="C24" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="D24" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E24" s="65" t="inlineStr"/>
+      <c r="F24" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Product Cost Accumulation: Pro-; cess Costing | Required Reading: Chapter 4- ONLY; LO 4.1, 3, 4, &amp; 5 | Homework: 5-27 5-46; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 9 (9/23)  -  Cost of Quality &amp; ESG &amp;; Overview of; • Linked In Learning Excel - 75 </t>
+        </is>
+      </c>
+      <c r="B25" s="65" t="inlineStr"/>
+      <c r="C25" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D25" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E25" s="65" t="inlineStr"/>
+      <c r="F25" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Cost of Quality &amp; ESG &amp;; Overview of; • Linked In Learning Excel - 75 Points; • Stukent Simternship  | Required Reading: Chapter 8 - ONLY; LO 8.7, 8, 9 | Homework: 4-21, 4-22; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 10 (9/28)  -  Catchup &amp; Midterm Review</t>
+        </is>
+      </c>
+      <c r="B26" s="65" t="inlineStr"/>
+      <c r="C26" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="D26" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E26" s="65" t="inlineStr"/>
+      <c r="F26" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Catchup &amp; Midterm Review | Homework: 8-28, 8-29; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 11 (10/5)  -  Cost Estimation</t>
+        </is>
+      </c>
+      <c r="B27" s="65" t="inlineStr"/>
+      <c r="C27" s="65" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="D27" s="65" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="E27" s="65" t="inlineStr"/>
+      <c r="F27" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Cost Estimation | Required Reading: Chapter 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 12 (10/7)  -  Cost volume profit analysis</t>
+        </is>
+      </c>
+      <c r="B28" s="65" t="inlineStr"/>
+      <c r="C28" s="65" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D28" s="65" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E28" s="65" t="inlineStr"/>
+      <c r="F28" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Cost volume profit analysis | Required Reading: Chapter 7 | Homework: 6-24, 6-25, 6-34; 15 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 13 (10/12)  -  Cost volume profit analysis &amp;</t>
+        </is>
+      </c>
+      <c r="B29" s="65" t="inlineStr"/>
+      <c r="C29" s="65" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="D29" s="65" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E29" s="65" t="inlineStr"/>
+      <c r="F29" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Cost volume profit analysis &amp; | Required Reading: Chapter 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 14 (10/14)  -  Financial planning and analysis:; Static Master Budget;</t>
+        </is>
+      </c>
+      <c r="B30" s="65" t="inlineStr"/>
+      <c r="C30" s="65" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="D30" s="65" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E30" s="65" t="inlineStr"/>
+      <c r="F30" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Financial planning and analysis:; Static Master Budget; | Required Reading: Chapter 9 | Homework: 7-29, 7-33, 7-40; 15 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 15 (10/19)  -  Capital Budgeting; Practice Midterm Questions Posted to Brightspace by</t>
+        </is>
+      </c>
+      <c r="B31" s="65" t="inlineStr"/>
+      <c r="C31" s="65" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="D31" s="65" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E31" s="65" t="inlineStr"/>
+      <c r="F31" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Capital Budgeting; Practice Midterm Questions Posted to Brightspace by; 5:00 PM | Required Reading: Chapter 16- ONLY; LO 16.1, 2, 3 | Homework: 9-25, 9-28, 9-37; 15 - Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 16 (10/21)  -  Catchup &amp; Midterm Review</t>
+        </is>
+      </c>
+      <c r="B32" s="65" t="inlineStr"/>
+      <c r="C32" s="65" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="D32" s="65" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E32" s="65" t="inlineStr"/>
+      <c r="F32" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Catchup &amp; Midterm Review | Homework: 16-28, 16-40; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 17 (10/28)  -  Guest Speaker</t>
+        </is>
+      </c>
+      <c r="B33" s="65" t="inlineStr"/>
+      <c r="C33" s="65" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="D33" s="65" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="E33" s="65" t="inlineStr"/>
+      <c r="F33" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Guest Speaker</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 19 (11/2)  -  Standard Costing &amp; Direct Cost; Variance Analysis</t>
+        </is>
+      </c>
+      <c r="B34" s="65" t="inlineStr"/>
+      <c r="C34" s="65" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="D34" s="65" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="E34" s="65" t="inlineStr"/>
+      <c r="F34" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Standard Costing &amp; Direct Cost; Variance Analysis | Required Reading: Chapter 10 – ONLY; LO 10.1 thru 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 19 (11/4)  -  Sales Variance Analysis; Flexible Budgeting</t>
+        </is>
+      </c>
+      <c r="B35" s="65" t="inlineStr"/>
+      <c r="C35" s="65" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="D35" s="65" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="E35" s="65" t="inlineStr"/>
+      <c r="F35" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Sales Variance Analysis; Flexible Budgeting | Required Reading: Chapter 11 - ONLY; LO 11.1, 11.2 &amp;; Appendix B | Homework: 10-26, 10-30; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 20 (11/9)  -  Investment Centers</t>
+        </is>
+      </c>
+      <c r="B36" s="65" t="inlineStr"/>
+      <c r="C36" s="65" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="D36" s="65" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E36" s="65" t="inlineStr"/>
+      <c r="F36" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Investment Centers | Required Reading: Chapter 13- ONLY; LO 13-1, 2, 3, 4 | Homework: 11-31, 11-52; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ 11/11  -  No Class Veterans Day</t>
+        </is>
+      </c>
+      <c r="B37" s="65" t="inlineStr"/>
+      <c r="C37" s="65" t="inlineStr">
+        <is>
+          <t>2026-11-11</t>
+        </is>
+      </c>
+      <c r="D37" s="65" t="inlineStr">
+        <is>
+          <t>2026-11-11</t>
+        </is>
+      </c>
+      <c r="E37" s="65" t="inlineStr"/>
+      <c r="F37" s="65" t="inlineStr">
+        <is>
+          <t>Topic: No Class Veterans Day</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 21 (11/16)  -  AI &amp; FP&amp;A</t>
+        </is>
+      </c>
+      <c r="B38" s="65" t="inlineStr"/>
+      <c r="C38" s="65" t="inlineStr">
+        <is>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="D38" s="65" t="inlineStr">
+        <is>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="E38" s="65" t="inlineStr"/>
+      <c r="F38" s="65" t="inlineStr">
+        <is>
+          <t>Topic: AI &amp; FP&amp;A | Homework: 13-29, 13-33; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 22 (11/18)  -  Decision-making: relevant costs; and benefits</t>
+        </is>
+      </c>
+      <c r="B39" s="65" t="inlineStr"/>
+      <c r="C39" s="65" t="inlineStr">
+        <is>
+          <t>2026-11-18</t>
+        </is>
+      </c>
+      <c r="D39" s="65" t="inlineStr">
+        <is>
+          <t>2026-11-18</t>
+        </is>
+      </c>
+      <c r="E39" s="65" t="inlineStr"/>
+      <c r="F39" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Decision-making: relevant costs; and benefits | Required Reading: Chapter 14; (Part 1 of 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 23 (11/23)  -  Decision-making: relevant costs; and benefits</t>
+        </is>
+      </c>
+      <c r="B40" s="65" t="inlineStr"/>
+      <c r="C40" s="65" t="inlineStr">
+        <is>
+          <t>2026-11-23</t>
+        </is>
+      </c>
+      <c r="D40" s="65" t="inlineStr">
+        <is>
+          <t>2026-11-23</t>
+        </is>
+      </c>
+      <c r="E40" s="65" t="inlineStr"/>
+      <c r="F40" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Decision-making: relevant costs; and benefits | Required Reading: Chapter 14; (Part 2 of 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ 11/25  -  No Class Thanksgiving Holiday</t>
+        </is>
+      </c>
+      <c r="B41" s="65" t="inlineStr"/>
+      <c r="C41" s="65" t="inlineStr">
+        <is>
+          <t>2026-11-25</t>
+        </is>
+      </c>
+      <c r="D41" s="65" t="inlineStr">
+        <is>
+          <t>2026-11-25</t>
+        </is>
+      </c>
+      <c r="E41" s="65" t="inlineStr"/>
+      <c r="F41" s="65" t="inlineStr">
+        <is>
+          <t>Topic: No Class Thanksgiving Holiday</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 24 (11/30)  -  Decision-making: relevant costs; and benefits</t>
+        </is>
+      </c>
+      <c r="B42" s="65" t="inlineStr"/>
+      <c r="C42" s="65" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="D42" s="65" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="E42" s="65" t="inlineStr"/>
+      <c r="F42" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Decision-making: relevant costs; and benefits | Required Reading: Chapter 14; (Part 3 of 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Class 2 (12/2)  -  Catchup &amp; Final Review; Practice Final Questions Posted to Brightspace</t>
+        </is>
+      </c>
+      <c r="B43" s="65" t="inlineStr"/>
+      <c r="C43" s="65" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="D43" s="65" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E43" s="65" t="inlineStr"/>
+      <c r="F43" s="65" t="inlineStr">
+        <is>
+          <t>Topic: Catchup &amp; Final Review; Practice Final Questions Posted to Brightspace at; 5:00 PM | Homework: 14-35, 14-41; 10 Points; Assignments listed Be-; low Due by11:59 PM; Linked In Learning; Excel Certi</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
         <is>
           <t>LinkedIn Learning Excel Certification</t>
         </is>
       </c>
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B44" s="62" t="inlineStr">
         <is>
           <t>75 pts</t>
         </is>
       </c>
-      <c r="C13" s="15" t="inlineStr">
+      <c r="C44" s="62" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D13" s="15" t="inlineStr">
+      <c r="D44" s="62" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E13" s="15" t="inlineStr">
+      <c r="E44" s="62" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F13" s="16">
+      <c r="F44" s="63">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-linkedin-learning-excel-certification.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ LinkedIn Learning Excel Certification</t>
+        </is>
+      </c>
+      <c r="B45" s="65" t="inlineStr"/>
+      <c r="C45" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D45" s="65" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E45" s="65" t="inlineStr"/>
+      <c r="F45" s="65" t="inlineStr">
+        <is>
+          <t>Certification (Course Calendar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="17" t="inlineStr">
         <is>
           <t>Stukent Simternship</t>
         </is>
       </c>
-      <c r="B14" s="18" t="inlineStr">
+      <c r="B46" s="66" t="inlineStr">
         <is>
           <t>75 pts</t>
         </is>
       </c>
-      <c r="C14" s="18" t="inlineStr">
+      <c r="C46" s="66" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D14" s="18" t="inlineStr">
+      <c r="D46" s="66" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E14" s="18" t="inlineStr">
+      <c r="E46" s="66" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F14" s="19">
+      <c r="F46" s="67">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-stukent-simternship.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Stukent Simternship</t>
+        </is>
+      </c>
+      <c r="B47" s="65" t="inlineStr"/>
+      <c r="C47" s="65" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D47" s="65" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E47" s="65" t="inlineStr"/>
+      <c r="F47" s="65" t="inlineStr">
+        <is>
+          <t>Certification (Course Calendar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>1070 pts</t>
         </is>
@@ -1439,27 +3252,27 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B9" s="51" t="inlineStr">
+      <c r="B9" s="68" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="C9" s="51" t="inlineStr">
+      <c r="C9" s="68" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D9" s="51" t="inlineStr">
+      <c r="D9" s="68" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E9" s="51" t="inlineStr">
+      <c r="E9" s="68" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F9" s="52">
+      <c r="F9" s="69">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-final-exam.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1470,19 +3283,19 @@
           <t xml:space="preserve">  ↳ Final Exam</t>
         </is>
       </c>
-      <c r="B10" s="53" t="inlineStr"/>
-      <c r="C10" s="53" t="inlineStr">
+      <c r="B10" s="70" t="inlineStr"/>
+      <c r="C10" s="70" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D10" s="53" t="inlineStr">
+      <c r="D10" s="70" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E10" s="53" t="inlineStr"/>
-      <c r="F10" s="53" t="inlineStr">
+      <c r="E10" s="70" t="inlineStr"/>
+      <c r="F10" s="70" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>
@@ -1494,27 +3307,27 @@
           <t>Participation</t>
         </is>
       </c>
-      <c r="B11" s="54" t="inlineStr">
+      <c r="B11" s="71" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C11" s="54" t="inlineStr">
+      <c r="C11" s="71" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D11" s="54" t="inlineStr">
+      <c r="D11" s="71" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E11" s="54" t="inlineStr">
+      <c r="E11" s="71" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F11" s="55">
+      <c r="F11" s="72">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-participation.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1525,15 +3338,15 @@
           <t xml:space="preserve">  ↳ Research: Setup deadline (registration, prescreening, contacts)</t>
         </is>
       </c>
-      <c r="B12" s="53" t="inlineStr"/>
-      <c r="C12" s="53" t="inlineStr"/>
-      <c r="D12" s="53" t="inlineStr">
+      <c r="B12" s="70" t="inlineStr"/>
+      <c r="C12" s="70" t="inlineStr"/>
+      <c r="D12" s="70" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="E12" s="53" t="inlineStr"/>
-      <c r="F12" s="53" t="inlineStr">
+      <c r="E12" s="70" t="inlineStr"/>
+      <c r="F12" s="70" t="inlineStr">
         <is>
           <t>Research Participation Guide</t>
         </is>
@@ -1545,15 +3358,15 @@
           <t xml:space="preserve">  ↳ Research: Employee contact surveys sent</t>
         </is>
       </c>
-      <c r="B13" s="53" t="inlineStr"/>
-      <c r="C13" s="53" t="inlineStr"/>
-      <c r="D13" s="53" t="inlineStr">
+      <c r="B13" s="70" t="inlineStr"/>
+      <c r="C13" s="70" t="inlineStr"/>
+      <c r="D13" s="70" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E13" s="53" t="inlineStr"/>
-      <c r="F13" s="53" t="inlineStr">
+      <c r="E13" s="70" t="inlineStr"/>
+      <c r="F13" s="70" t="inlineStr">
         <is>
           <t>Research Participation Guide</t>
         </is>
@@ -1565,15 +3378,15 @@
           <t xml:space="preserve">  ↳ Research: Complete 2.0 research credits</t>
         </is>
       </c>
-      <c r="B14" s="53" t="inlineStr"/>
-      <c r="C14" s="53" t="inlineStr"/>
-      <c r="D14" s="53" t="inlineStr">
+      <c r="B14" s="70" t="inlineStr"/>
+      <c r="C14" s="70" t="inlineStr"/>
+      <c r="D14" s="70" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E14" s="53" t="inlineStr"/>
-      <c r="F14" s="53" t="inlineStr">
+      <c r="E14" s="70" t="inlineStr"/>
+      <c r="F14" s="70" t="inlineStr">
         <is>
           <t>Research Participation Guide</t>
         </is>
@@ -1585,19 +3398,19 @@
           <t xml:space="preserve">  ↳ Connect: Sharpen Companion</t>
         </is>
       </c>
-      <c r="B15" s="53" t="inlineStr"/>
-      <c r="C15" s="53" t="inlineStr">
+      <c r="B15" s="70" t="inlineStr"/>
+      <c r="C15" s="70" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="D15" s="53" t="inlineStr">
+      <c r="D15" s="70" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E15" s="53" t="inlineStr"/>
-      <c r="F15" s="53" t="inlineStr">
+      <c r="E15" s="70" t="inlineStr"/>
+      <c r="F15" s="70" t="inlineStr">
         <is>
           <t>Brightspace Connect module</t>
         </is>
@@ -1609,15 +3422,15 @@
           <t xml:space="preserve">  ↳ Research: SONA registration opens</t>
         </is>
       </c>
-      <c r="B16" s="53" t="inlineStr"/>
-      <c r="C16" s="53" t="inlineStr">
+      <c r="B16" s="70" t="inlineStr"/>
+      <c r="C16" s="70" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D16" s="53" t="inlineStr"/>
-      <c r="E16" s="53" t="inlineStr"/>
-      <c r="F16" s="53" t="inlineStr">
+      <c r="D16" s="70" t="inlineStr"/>
+      <c r="E16" s="70" t="inlineStr"/>
+      <c r="F16" s="70" t="inlineStr">
         <is>
           <t>Research Participation Guide</t>
         </is>
@@ -1629,19 +3442,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 11.01 - What is my</t>
         </is>
       </c>
-      <c r="B17" s="53" t="inlineStr"/>
-      <c r="C17" s="53" t="inlineStr">
+      <c r="B17" s="70" t="inlineStr"/>
+      <c r="C17" s="70" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D17" s="53" t="inlineStr">
+      <c r="D17" s="70" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E17" s="53" t="inlineStr"/>
-      <c r="F17" s="53" t="inlineStr">
+      <c r="E17" s="70" t="inlineStr"/>
+      <c r="F17" s="70" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-09-09; Connect window</t>
         </is>
@@ -1653,19 +3466,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 11.02 - What is my</t>
         </is>
       </c>
-      <c r="B18" s="53" t="inlineStr"/>
-      <c r="C18" s="53" t="inlineStr">
+      <c r="B18" s="70" t="inlineStr"/>
+      <c r="C18" s="70" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D18" s="53" t="inlineStr">
+      <c r="D18" s="70" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E18" s="53" t="inlineStr"/>
-      <c r="F18" s="53" t="inlineStr">
+      <c r="E18" s="70" t="inlineStr"/>
+      <c r="F18" s="70" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-09-09; Connect window</t>
         </is>
@@ -1677,19 +3490,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 12.02 - Which influence</t>
         </is>
       </c>
-      <c r="B19" s="53" t="inlineStr"/>
-      <c r="C19" s="53" t="inlineStr">
+      <c r="B19" s="70" t="inlineStr"/>
+      <c r="C19" s="70" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D19" s="53" t="inlineStr">
+      <c r="D19" s="70" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E19" s="53" t="inlineStr"/>
-      <c r="F19" s="53" t="inlineStr">
+      <c r="E19" s="70" t="inlineStr"/>
+      <c r="F19" s="70" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-08-24; Connect window</t>
         </is>
@@ -1701,19 +3514,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
         </is>
       </c>
-      <c r="B20" s="53" t="inlineStr"/>
-      <c r="C20" s="53" t="inlineStr">
+      <c r="B20" s="70" t="inlineStr"/>
+      <c r="C20" s="70" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D20" s="53" t="inlineStr">
+      <c r="D20" s="70" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E20" s="53" t="inlineStr"/>
-      <c r="F20" s="53" t="inlineStr">
+      <c r="E20" s="70" t="inlineStr"/>
+      <c r="F20" s="70" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-08-31; Connect window</t>
         </is>
@@ -1725,19 +3538,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 3.04 - What Is Your Level</t>
         </is>
       </c>
-      <c r="B21" s="53" t="inlineStr"/>
-      <c r="C21" s="53" t="inlineStr">
+      <c r="B21" s="70" t="inlineStr"/>
+      <c r="C21" s="70" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D21" s="53" t="inlineStr">
+      <c r="D21" s="70" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E21" s="53" t="inlineStr"/>
-      <c r="F21" s="53" t="inlineStr">
+      <c r="E21" s="70" t="inlineStr"/>
+      <c r="F21" s="70" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-08-31; Connect window</t>
         </is>
@@ -1749,19 +3562,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 5.01 - Assessing Your</t>
         </is>
       </c>
-      <c r="B22" s="53" t="inlineStr"/>
-      <c r="C22" s="53" t="inlineStr">
+      <c r="B22" s="70" t="inlineStr"/>
+      <c r="C22" s="70" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D22" s="53" t="inlineStr">
+      <c r="D22" s="70" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E22" s="53" t="inlineStr"/>
-      <c r="F22" s="53" t="inlineStr">
+      <c r="E22" s="70" t="inlineStr"/>
+      <c r="F22" s="70" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-09-02; Connect window</t>
         </is>
@@ -1773,15 +3586,15 @@
           <t xml:space="preserve">  ↳ Research: Prescreening questionnaire opens</t>
         </is>
       </c>
-      <c r="B23" s="53" t="inlineStr"/>
-      <c r="C23" s="53" t="inlineStr">
+      <c r="B23" s="70" t="inlineStr"/>
+      <c r="C23" s="70" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="D23" s="53" t="inlineStr"/>
-      <c r="E23" s="53" t="inlineStr"/>
-      <c r="F23" s="53" t="inlineStr">
+      <c r="D23" s="70" t="inlineStr"/>
+      <c r="E23" s="70" t="inlineStr"/>
+      <c r="F23" s="70" t="inlineStr">
         <is>
           <t>Research Participation Guide</t>
         </is>
@@ -1793,15 +3606,15 @@
           <t xml:space="preserve">  ↳ Research: Study invitations begin (after setup)</t>
         </is>
       </c>
-      <c r="B24" s="53" t="inlineStr"/>
-      <c r="C24" s="53" t="inlineStr">
+      <c r="B24" s="70" t="inlineStr"/>
+      <c r="C24" s="70" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="D24" s="53" t="inlineStr"/>
-      <c r="E24" s="53" t="inlineStr"/>
-      <c r="F24" s="53" t="inlineStr">
+      <c r="D24" s="70" t="inlineStr"/>
+      <c r="E24" s="70" t="inlineStr"/>
+      <c r="F24" s="70" t="inlineStr">
         <is>
           <t>Research Participation Guide</t>
         </is>
@@ -1813,27 +3626,27 @@
           <t>Midterm Exam</t>
         </is>
       </c>
-      <c r="B25" s="51" t="inlineStr">
+      <c r="B25" s="68" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C25" s="51" t="inlineStr">
+      <c r="C25" s="68" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D25" s="51" t="inlineStr">
+      <c r="D25" s="68" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E25" s="51" t="inlineStr">
+      <c r="E25" s="68" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F25" s="52">
+      <c r="F25" s="69">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-midterm-exam.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1844,19 +3657,19 @@
           <t xml:space="preserve">  ↳ Midterm Exam</t>
         </is>
       </c>
-      <c r="B26" s="53" t="inlineStr"/>
-      <c r="C26" s="53" t="inlineStr">
+      <c r="B26" s="70" t="inlineStr"/>
+      <c r="C26" s="70" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D26" s="53" t="inlineStr">
+      <c r="D26" s="70" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E26" s="53" t="inlineStr"/>
-      <c r="F26" s="53" t="inlineStr">
+      <c r="E26" s="70" t="inlineStr"/>
+      <c r="F26" s="70" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>
@@ -1868,27 +3681,27 @@
           <t>Team Project Paper</t>
         </is>
       </c>
-      <c r="B27" s="54" t="inlineStr">
+      <c r="B27" s="71" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C27" s="54" t="inlineStr">
+      <c r="C27" s="71" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D27" s="54" t="inlineStr">
+      <c r="D27" s="71" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E27" s="54" t="inlineStr">
+      <c r="E27" s="71" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F27" s="55">
+      <c r="F27" s="72">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-team-project-paper.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -1899,19 +3712,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 14.02 - What Type of Organizational Culture Do I</t>
         </is>
       </c>
-      <c r="B28" s="53" t="inlineStr"/>
-      <c r="C28" s="53" t="inlineStr">
+      <c r="B28" s="70" t="inlineStr"/>
+      <c r="C28" s="70" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D28" s="53" t="inlineStr">
+      <c r="D28" s="70" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E28" s="53" t="inlineStr"/>
-      <c r="F28" s="53" t="inlineStr">
+      <c r="E28" s="70" t="inlineStr"/>
+      <c r="F28" s="70" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-11-04; Connect window</t>
         </is>
@@ -1923,19 +3736,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 8.01 - Group</t>
         </is>
       </c>
-      <c r="B29" s="53" t="inlineStr"/>
-      <c r="C29" s="53" t="inlineStr">
+      <c r="B29" s="70" t="inlineStr"/>
+      <c r="C29" s="70" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D29" s="53" t="inlineStr">
+      <c r="D29" s="70" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E29" s="53" t="inlineStr"/>
-      <c r="F29" s="53" t="inlineStr">
+      <c r="E29" s="70" t="inlineStr"/>
+      <c r="F29" s="70" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-10-19; Connect window</t>
         </is>
@@ -1947,19 +3760,19 @@
           <t xml:space="preserve">  ↳ Team project outline</t>
         </is>
       </c>
-      <c r="B30" s="53" t="inlineStr"/>
-      <c r="C30" s="53" t="inlineStr">
+      <c r="B30" s="70" t="inlineStr"/>
+      <c r="C30" s="70" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D30" s="53" t="inlineStr">
+      <c r="D30" s="70" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E30" s="53" t="inlineStr"/>
-      <c r="F30" s="53" t="inlineStr">
+      <c r="E30" s="70" t="inlineStr"/>
+      <c r="F30" s="70" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>
@@ -1971,19 +3784,19 @@
           <t xml:space="preserve">  ↳ Team project paper</t>
         </is>
       </c>
-      <c r="B31" s="53" t="inlineStr"/>
-      <c r="C31" s="53" t="inlineStr">
+      <c r="B31" s="70" t="inlineStr"/>
+      <c r="C31" s="70" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D31" s="53" t="inlineStr">
+      <c r="D31" s="70" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E31" s="53" t="inlineStr"/>
-      <c r="F31" s="53" t="inlineStr">
+      <c r="E31" s="70" t="inlineStr"/>
+      <c r="F31" s="70" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>
@@ -1995,27 +3808,27 @@
           <t>Final Reflection Paper</t>
         </is>
       </c>
-      <c r="B32" s="51" t="inlineStr">
+      <c r="B32" s="68" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C32" s="51" t="inlineStr">
+      <c r="C32" s="68" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D32" s="51" t="inlineStr">
+      <c r="D32" s="68" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E32" s="51" t="inlineStr">
+      <c r="E32" s="68" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F32" s="52">
+      <c r="F32" s="69">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-final-reflection-paper.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -2026,19 +3839,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 16.02 - What Is Your</t>
         </is>
       </c>
-      <c r="B33" s="53" t="inlineStr"/>
-      <c r="C33" s="53" t="inlineStr">
+      <c r="B33" s="70" t="inlineStr"/>
+      <c r="C33" s="70" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D33" s="53" t="inlineStr">
+      <c r="D33" s="70" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E33" s="53" t="inlineStr"/>
-      <c r="F33" s="53" t="inlineStr">
+      <c r="E33" s="70" t="inlineStr"/>
+      <c r="F33" s="70" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-11-30; Connect window</t>
         </is>
@@ -2050,19 +3863,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 16.03 - Assessing Your</t>
         </is>
       </c>
-      <c r="B34" s="53" t="inlineStr"/>
-      <c r="C34" s="53" t="inlineStr">
+      <c r="B34" s="70" t="inlineStr"/>
+      <c r="C34" s="70" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D34" s="53" t="inlineStr">
+      <c r="D34" s="70" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E34" s="53" t="inlineStr"/>
-      <c r="F34" s="53" t="inlineStr">
+      <c r="E34" s="70" t="inlineStr"/>
+      <c r="F34" s="70" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-11-30; Connect window</t>
         </is>
@@ -2074,19 +3887,19 @@
           <t xml:space="preserve">  ↳ Personal Reflection Paper</t>
         </is>
       </c>
-      <c r="B35" s="53" t="inlineStr"/>
-      <c r="C35" s="53" t="inlineStr">
+      <c r="B35" s="70" t="inlineStr"/>
+      <c r="C35" s="70" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D35" s="53" t="inlineStr">
+      <c r="D35" s="70" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E35" s="53" t="inlineStr"/>
-      <c r="F35" s="53" t="inlineStr">
+      <c r="E35" s="70" t="inlineStr"/>
+      <c r="F35" s="70" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>
@@ -2098,27 +3911,27 @@
           <t>Presentation</t>
         </is>
       </c>
-      <c r="B36" s="54" t="inlineStr">
+      <c r="B36" s="71" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C36" s="54" t="inlineStr">
+      <c r="C36" s="71" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D36" s="54" t="inlineStr">
+      <c r="D36" s="71" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E36" s="54" t="inlineStr">
+      <c r="E36" s="71" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F36" s="55">
+      <c r="F36" s="72">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-presentation.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -2129,19 +3942,19 @@
           <t xml:space="preserve">  ↳ Presentation slides</t>
         </is>
       </c>
-      <c r="B37" s="53" t="inlineStr"/>
-      <c r="C37" s="53" t="inlineStr">
+      <c r="B37" s="70" t="inlineStr"/>
+      <c r="C37" s="70" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D37" s="53" t="inlineStr">
+      <c r="D37" s="70" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E37" s="53" t="inlineStr"/>
-      <c r="F37" s="53" t="inlineStr">
+      <c r="E37" s="70" t="inlineStr"/>
+      <c r="F37" s="70" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>
@@ -2153,27 +3966,27 @@
           <t>Case Analysis Assignments</t>
         </is>
       </c>
-      <c r="B38" s="51" t="inlineStr">
+      <c r="B38" s="68" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C38" s="51" t="inlineStr">
+      <c r="C38" s="68" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D38" s="51" t="inlineStr">
+      <c r="D38" s="68" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E38" s="51" t="inlineStr">
+      <c r="E38" s="68" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F38" s="52">
+      <c r="F38" s="69">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-case-analysis-assignments.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -2184,19 +3997,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 12.01 - What kind of</t>
         </is>
       </c>
-      <c r="B39" s="53" t="inlineStr"/>
-      <c r="C39" s="53" t="inlineStr">
+      <c r="B39" s="70" t="inlineStr"/>
+      <c r="C39" s="70" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D39" s="53" t="inlineStr">
+      <c r="D39" s="70" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E39" s="53" t="inlineStr"/>
-      <c r="F39" s="53" t="inlineStr">
+      <c r="E39" s="70" t="inlineStr"/>
+      <c r="F39" s="70" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-09-16; Connect window</t>
         </is>
@@ -2208,19 +4021,19 @@
           <t xml:space="preserve">  ↳ Thomas Green Case Analysis Memo</t>
         </is>
       </c>
-      <c r="B40" s="53" t="inlineStr"/>
-      <c r="C40" s="53" t="inlineStr">
+      <c r="B40" s="70" t="inlineStr"/>
+      <c r="C40" s="70" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D40" s="53" t="inlineStr">
+      <c r="D40" s="70" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E40" s="53" t="inlineStr"/>
-      <c r="F40" s="53" t="inlineStr">
+      <c r="E40" s="70" t="inlineStr"/>
+      <c r="F40" s="70" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>
@@ -2232,19 +4045,19 @@
           <t xml:space="preserve">  ↳ SkillsForTomorrow Analysis Memo</t>
         </is>
       </c>
-      <c r="B41" s="53" t="inlineStr"/>
-      <c r="C41" s="53" t="inlineStr">
+      <c r="B41" s="70" t="inlineStr"/>
+      <c r="C41" s="70" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D41" s="53" t="inlineStr">
+      <c r="D41" s="70" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E41" s="53" t="inlineStr"/>
-      <c r="F41" s="53" t="inlineStr">
+      <c r="E41" s="70" t="inlineStr"/>
+      <c r="F41" s="70" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>
@@ -2256,27 +4069,27 @@
           <t>Proposal &amp; Team Contract</t>
         </is>
       </c>
-      <c r="B42" s="54" t="inlineStr">
+      <c r="B42" s="71" t="inlineStr">
         <is>
           <t>3%</t>
         </is>
       </c>
-      <c r="C42" s="54" t="inlineStr">
+      <c r="C42" s="71" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D42" s="54" t="inlineStr">
+      <c r="D42" s="71" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E42" s="54" t="inlineStr">
+      <c r="E42" s="71" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F42" s="55">
+      <c r="F42" s="72">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-proposal-team-contract.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -2287,19 +4100,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 10.5 - Preferred Conflict</t>
         </is>
       </c>
-      <c r="B43" s="53" t="inlineStr"/>
-      <c r="C43" s="53" t="inlineStr">
+      <c r="B43" s="70" t="inlineStr"/>
+      <c r="C43" s="70" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D43" s="53" t="inlineStr">
+      <c r="D43" s="70" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E43" s="53" t="inlineStr"/>
-      <c r="F43" s="53" t="inlineStr">
+      <c r="E43" s="70" t="inlineStr"/>
+      <c r="F43" s="70" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-09-28; Connect window</t>
         </is>
@@ -2311,19 +4124,19 @@
           <t xml:space="preserve">  ↳ Connect: Self-Assessment 9.01 - Assessing My</t>
         </is>
       </c>
-      <c r="B44" s="53" t="inlineStr"/>
-      <c r="C44" s="53" t="inlineStr">
+      <c r="B44" s="70" t="inlineStr"/>
+      <c r="C44" s="70" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D44" s="53" t="inlineStr">
+      <c r="D44" s="70" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E44" s="53" t="inlineStr"/>
-      <c r="F44" s="53" t="inlineStr">
+      <c r="E44" s="70" t="inlineStr"/>
+      <c r="F44" s="70" t="inlineStr">
         <is>
           <t>Assigned in class week of 2026-09-28; Connect window</t>
         </is>
@@ -2335,19 +4148,19 @@
           <t xml:space="preserve">  ↳ Team project proposal &amp; team contract</t>
         </is>
       </c>
-      <c r="B45" s="53" t="inlineStr"/>
-      <c r="C45" s="53" t="inlineStr">
+      <c r="B45" s="70" t="inlineStr"/>
+      <c r="C45" s="70" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D45" s="53" t="inlineStr">
+      <c r="D45" s="70" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E45" s="53" t="inlineStr"/>
-      <c r="F45" s="53" t="inlineStr">
+      <c r="E45" s="70" t="inlineStr"/>
+      <c r="F45" s="70" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>
@@ -2359,27 +4172,27 @@
           <t>Self &amp; Peer Evaluation</t>
         </is>
       </c>
-      <c r="B46" s="51" t="inlineStr">
+      <c r="B46" s="68" t="inlineStr">
         <is>
           <t>2%</t>
         </is>
       </c>
-      <c r="C46" s="51" t="inlineStr">
+      <c r="C46" s="68" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D46" s="51" t="inlineStr">
+      <c r="D46" s="68" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E46" s="51" t="inlineStr">
+      <c r="E46" s="68" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F46" s="52">
+      <c r="F46" s="69">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-self-peer-evaluation.pdf","Open PDF")</f>
         <v/>
       </c>
@@ -2390,19 +4203,19 @@
           <t xml:space="preserve">  ↳ Self &amp; peer evaluation</t>
         </is>
       </c>
-      <c r="B47" s="53" t="inlineStr"/>
-      <c r="C47" s="53" t="inlineStr">
+      <c r="B47" s="70" t="inlineStr"/>
+      <c r="C47" s="70" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D47" s="53" t="inlineStr">
+      <c r="D47" s="70" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E47" s="53" t="inlineStr"/>
-      <c r="F47" s="53" t="inlineStr">
+      <c r="E47" s="70" t="inlineStr"/>
+      <c r="F47" s="70" t="inlineStr">
         <is>
           <t>Course Schedule due date</t>
         </is>

</xml_diff>

<commit_message>
Label HIST-103 weekly readings as Homework in Excel Details column
Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -7,9 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-281" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-304" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-281" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-304" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -157,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -369,6 +369,21 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -733,1312 +748,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00D62728"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F56"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>HIST-103 — The Emergence of Modern Europe</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="2">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/sources/hist-103-source.pdf","SEE HERE")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Instructor</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Dr. Lindsay O'Neill</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Term</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Fall 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Required for an A</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>93% (100-93)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Grading scale</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>A: 100-93; A-: 92-90; B+: 89-87; B: 86-83; B-: 82-80; C+: 79-77; C: 76-73; C- 72-70 D+: 69-67; D: 66-63; D-: 62-60; F: 59-0</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Weight</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Due Date</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Group Project</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Sleep Paper</t>
-        </is>
-      </c>
-      <c r="B9" s="56" t="inlineStr">
-        <is>
-          <t>20%</t>
-        </is>
-      </c>
-      <c r="C9" s="56" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D9" s="56" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="E9" s="56" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F9" s="57">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-sleep-paper.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Sleep Paper Due</t>
-        </is>
-      </c>
-      <c r="B10" s="59" t="inlineStr"/>
-      <c r="C10" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="D10" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="E10" s="59" t="inlineStr"/>
-      <c r="F10" s="59" t="inlineStr">
-        <is>
-          <t>Due date (course schedule)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Sep 15-18: Renaissance</t>
-        </is>
-      </c>
-      <c r="B11" s="59" t="inlineStr"/>
-      <c r="C11" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="D11" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="E11" s="59" t="inlineStr"/>
-      <c r="F11" s="59" t="inlineStr">
-        <is>
-          <t>Weekly schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>Witchcraft Paper</t>
-        </is>
-      </c>
-      <c r="B12" s="60" t="inlineStr">
-        <is>
-          <t>20%</t>
-        </is>
-      </c>
-      <c r="C12" s="60" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="D12" s="60" t="inlineStr">
-        <is>
-          <t>2026-11-10</t>
-        </is>
-      </c>
-      <c r="E12" s="60" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F12" s="61">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-witchcraft-paper.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Witchcraft Paper Due</t>
-        </is>
-      </c>
-      <c r="B13" s="59" t="inlineStr"/>
-      <c r="C13" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-10</t>
-        </is>
-      </c>
-      <c r="D13" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-10</t>
-        </is>
-      </c>
-      <c r="E13" s="59" t="inlineStr"/>
-      <c r="F13" s="59" t="inlineStr">
-        <is>
-          <t>Due date (course schedule)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Nov 10-13: Enlightenment</t>
-        </is>
-      </c>
-      <c r="B14" s="59" t="inlineStr"/>
-      <c r="C14" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-10</t>
-        </is>
-      </c>
-      <c r="D14" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-13</t>
-        </is>
-      </c>
-      <c r="E14" s="59" t="inlineStr"/>
-      <c r="F14" s="59" t="inlineStr">
-        <is>
-          <t>Weekly schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Mid-term</t>
-        </is>
-      </c>
-      <c r="B15" s="56" t="inlineStr">
-        <is>
-          <t>20%</t>
-        </is>
-      </c>
-      <c r="C15" s="56" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="D15" s="56" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E15" s="56" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F15" s="57">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-mid-term.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Midterm Exam</t>
-        </is>
-      </c>
-      <c r="B16" s="59" t="inlineStr"/>
-      <c r="C16" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="D16" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="E16" s="59" t="inlineStr"/>
-      <c r="F16" s="59" t="inlineStr">
-        <is>
-          <t>Oct 6: Midterm</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Oct 6-9: Midterm &amp; Break</t>
-        </is>
-      </c>
-      <c r="B17" s="59" t="inlineStr"/>
-      <c r="C17" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="D17" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E17" s="59" t="inlineStr"/>
-      <c r="F17" s="59" t="inlineStr">
-        <is>
-          <t>Weekly schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Dec 1-4: Modern Europe?</t>
-        </is>
-      </c>
-      <c r="B18" s="59" t="inlineStr"/>
-      <c r="C18" s="59" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
-      <c r="D18" s="59" t="inlineStr">
-        <is>
-          <t>2026-12-04</t>
-        </is>
-      </c>
-      <c r="E18" s="59" t="inlineStr"/>
-      <c r="F18" s="59" t="inlineStr">
-        <is>
-          <t>Weekly schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>Final Exam</t>
-        </is>
-      </c>
-      <c r="B19" s="60" t="inlineStr">
-        <is>
-          <t>20%</t>
-        </is>
-      </c>
-      <c r="C19" s="60" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D19" s="60" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="E19" s="60" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F19" s="61">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-final-exam.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Final Exam</t>
-        </is>
-      </c>
-      <c r="B20" s="59" t="inlineStr"/>
-      <c r="C20" s="59" t="inlineStr">
-        <is>
-          <t>2026-12-10</t>
-        </is>
-      </c>
-      <c r="D20" s="59" t="inlineStr">
-        <is>
-          <t>2026-12-10</t>
-        </is>
-      </c>
-      <c r="E20" s="59" t="inlineStr"/>
-      <c r="F20" s="59" t="inlineStr">
-        <is>
-          <t>Dec 10: Final Exam</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Discussion Section</t>
-        </is>
-      </c>
-      <c r="B21" s="56" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="C21" s="56" t="inlineStr">
-        <is>
-          <t>2026-11-10</t>
-        </is>
-      </c>
-      <c r="D21" s="56" t="inlineStr">
-        <is>
-          <t>2026-11-12</t>
-        </is>
-      </c>
-      <c r="E21" s="56" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F21" s="57">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-discussion-section.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Aug 25-29: Intro &amp; Black Death</t>
-        </is>
-      </c>
-      <c r="B22" s="59" t="inlineStr"/>
-      <c r="C22" s="59" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="D22" s="59" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
-      </c>
-      <c r="E22" s="59" t="inlineStr"/>
-      <c r="F22" s="59" t="inlineStr">
-        <is>
-          <t>Weekly schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Aug 25-29: Intro &amp; Black Death  -  Section readings 1</t>
-        </is>
-      </c>
-      <c r="B23" s="59" t="inlineStr"/>
-      <c r="C23" s="59" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="D23" s="59" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
-      </c>
-      <c r="E23" s="59" t="inlineStr"/>
-      <c r="F23" s="59" t="inlineStr">
-        <is>
-          <t>-- 13 of 33 -- Lizzie Wade, “From Black Death to fatal flu, past pandemics show why people on the margins suffer most,” Science, May 14, 2020 Alex Brown and Grace Owen, “What a list of Black Death Sur</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Sep 1-4: Everyday Life</t>
-        </is>
-      </c>
-      <c r="B24" s="59" t="inlineStr"/>
-      <c r="C24" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="D24" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="E24" s="59" t="inlineStr"/>
-      <c r="F24" s="59" t="inlineStr">
-        <is>
-          <t>Weekly schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Sep 1-4: Everyday Life  -  Section readings 1</t>
-        </is>
-      </c>
-      <c r="B25" s="59" t="inlineStr"/>
-      <c r="C25" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="D25" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="E25" s="59" t="inlineStr"/>
-      <c r="F25" s="59" t="inlineStr">
-        <is>
-          <t>A Roger Ekirch, “Sleep we have lost: Pre-Industrial Slumber in the British Isles, The American Historical Review, April 2001, pg. 343-365 Sasha Handley, Sleep in Early Modern England, Introduction &amp; C</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Sep 8-11: Renaissance</t>
-        </is>
-      </c>
-      <c r="B26" s="59" t="inlineStr"/>
-      <c r="C26" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="D26" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="E26" s="59" t="inlineStr"/>
-      <c r="F26" s="59" t="inlineStr">
-        <is>
-          <t>Weekly schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Sep 8-11: Renaissance  -  Section readings 1</t>
-        </is>
-      </c>
-      <c r="B27" s="59" t="inlineStr"/>
-      <c r="C27" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="D27" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="E27" s="59" t="inlineStr"/>
-      <c r="F27" s="59" t="inlineStr">
-        <is>
-          <t>-- 14 of 33 -- Kay Daly, “Diverting the Flood of History: Ada Palmer’s Inventing the Renaissance,” Chicago Review of Books, 25 March 2025 Ada Palmer, “Black Death, COVID, and Why We Keep Telling the M</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Sep 15-18: Renaissance  -  Section readings 1</t>
-        </is>
-      </c>
-      <c r="B28" s="59" t="inlineStr"/>
-      <c r="C28" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="D28" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="E28" s="59" t="inlineStr"/>
-      <c r="F28" s="59" t="inlineStr">
-        <is>
-          <t>Vasari, Lives of the Artists: Leonardo da Vinci &amp; Properzia de’ Rossi Video: The Story of Women and Art, Part 1(1hr) Vasari on da Vinci PDF document Vasari on d'Rossi PDF document</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Sep 20-24: European Expansion</t>
-        </is>
-      </c>
-      <c r="B29" s="59" t="inlineStr"/>
-      <c r="C29" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="D29" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="E29" s="59" t="inlineStr"/>
-      <c r="F29" s="59" t="inlineStr">
-        <is>
-          <t>Weekly schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Sep 20-24: European Expansion  -  Section readings 1</t>
-        </is>
-      </c>
-      <c r="B30" s="59" t="inlineStr"/>
-      <c r="C30" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="D30" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="E30" s="59" t="inlineStr"/>
-      <c r="F30" s="59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jerry Brotton, The Renaissance Bazaar, Chap 1 (15 pgs) Read Columbus’ Letter on his Return: MacGregor, The History of the World in 100 Objects Read or listen to the stories behind these objects: Part </t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Sep 20-24: European Expansion  -  Section readings 2</t>
-        </is>
-      </c>
-      <c r="B31" s="59" t="inlineStr"/>
-      <c r="C31" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="D31" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="E31" s="59" t="inlineStr"/>
-      <c r="F31" s="59" t="inlineStr">
-        <is>
-          <t>Bernal Diaz del Castillo, The True History of the Conquest of New Spain, pg 121-171 Miguel León Portilla, Broken Spears: The Aztec Account of the Conquest of Mexico, Appendix, Chap 8-10 (37 pgs) Broke</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Oct 13-16: The Reformation</t>
-        </is>
-      </c>
-      <c r="B32" s="59" t="inlineStr"/>
-      <c r="C32" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="D32" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="E32" s="59" t="inlineStr"/>
-      <c r="F32" s="59" t="inlineStr">
-        <is>
-          <t>Weekly schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Oct 20-23: The Reformation</t>
-        </is>
-      </c>
-      <c r="B33" s="59" t="inlineStr"/>
-      <c r="C33" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="D33" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="E33" s="59" t="inlineStr"/>
-      <c r="F33" s="59" t="inlineStr">
-        <is>
-          <t>Weekly schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Oct 27-30: Reformation</t>
-        </is>
-      </c>
-      <c r="B34" s="59" t="inlineStr"/>
-      <c r="C34" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-27</t>
-        </is>
-      </c>
-      <c r="D34" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-30</t>
-        </is>
-      </c>
-      <c r="E34" s="59" t="inlineStr"/>
-      <c r="F34" s="59" t="inlineStr">
-        <is>
-          <t>Weekly schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Oct 27-30: Reformation  -  Section readings 1</t>
-        </is>
-      </c>
-      <c r="B35" s="59" t="inlineStr"/>
-      <c r="C35" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-27</t>
-        </is>
-      </c>
-      <c r="D35" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-30</t>
-        </is>
-      </c>
-      <c r="E35" s="59" t="inlineStr"/>
-      <c r="F35" s="59" t="inlineStr">
-        <is>
-          <t>Barbara Diefendorf, ed., The Saint Bartholomew’s Day Massacre: A Brief History with Documents, Introduction, Documents 2-6, 9-11, 16-21, 31, 33</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Nov 3-6: Witches &amp; Science</t>
-        </is>
-      </c>
-      <c r="B36" s="59" t="inlineStr"/>
-      <c r="C36" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-03</t>
-        </is>
-      </c>
-      <c r="D36" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-06</t>
-        </is>
-      </c>
-      <c r="E36" s="59" t="inlineStr"/>
-      <c r="F36" s="59" t="inlineStr">
-        <is>
-          <t>Weekly schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Nov 3-6: Witches &amp; Science  -  Section readings 1</t>
-        </is>
-      </c>
-      <c r="B37" s="59" t="inlineStr"/>
-      <c r="C37" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-03</t>
-        </is>
-      </c>
-      <c r="D37" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-06</t>
-        </is>
-      </c>
-      <c r="E37" s="59" t="inlineStr"/>
-      <c r="F37" s="59" t="inlineStr">
-        <is>
-          <t>Brian Levack, The Witchcraft Sourcebook, Chaps 36-44, 46-47 103.Levack.36 PDF document 103.Levack.37 PDF document 103.Levack.38 PDF document 103.Levack.39 PDF document 103.Levack.40 PDF document 103.L</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Nov 10-13: Enlightenment  -  Section readings 1</t>
-        </is>
-      </c>
-      <c r="B38" s="59" t="inlineStr"/>
-      <c r="C38" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-10</t>
-        </is>
-      </c>
-      <c r="D38" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-13</t>
-        </is>
-      </c>
-      <c r="E38" s="59" t="inlineStr"/>
-      <c r="F38" s="59" t="inlineStr">
-        <is>
-          <t>Excerpt: John Locke, Two Treatises of Government (1689) Excerpt: Rousseau, The Social Contract (1762) Enlightenment Primary Source Activity [Ungraded, but counts towards participation. Due in section]</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Nov 17-20: Enlightenment</t>
-        </is>
-      </c>
-      <c r="B39" s="59" t="inlineStr"/>
-      <c r="C39" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-17</t>
-        </is>
-      </c>
-      <c r="D39" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-20</t>
-        </is>
-      </c>
-      <c r="E39" s="59" t="inlineStr"/>
-      <c r="F39" s="59" t="inlineStr">
-        <is>
-          <t>Weekly schedule</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Nov 17-20: Enlightenment  -  Section readings 1</t>
-        </is>
-      </c>
-      <c r="B40" s="59" t="inlineStr"/>
-      <c r="C40" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-17</t>
-        </is>
-      </c>
-      <c r="D40" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-20</t>
-        </is>
-      </c>
-      <c r="E40" s="59" t="inlineStr"/>
-      <c r="F40" s="59" t="inlineStr">
-        <is>
-          <t>Video: Africa &amp; Britain, A Forgotten History, Episode 2: Freedom (50 min) Slavery and the African Presence in London Activity [Ungraded but counts towards participation. Due in section] 103.Act.Enslav</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="9" t="inlineStr">
-        <is>
-          <t>Identification Quizzes</t>
-        </is>
-      </c>
-      <c r="B41" s="60" t="inlineStr">
-        <is>
-          <t>5%</t>
-        </is>
-      </c>
-      <c r="C41" s="60" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="D41" s="60" t="inlineStr">
-        <is>
-          <t>2026-12-10</t>
-        </is>
-      </c>
-      <c r="E41" s="60" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F41" s="61">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-identification-quizzes.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Aug 25-29: Intro &amp; Black Death (lecture topics)</t>
-        </is>
-      </c>
-      <c r="B42" s="59" t="inlineStr"/>
-      <c r="C42" s="59" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="D42" s="59" t="inlineStr">
-        <is>
-          <t>2026-08-29</t>
-        </is>
-      </c>
-      <c r="E42" s="59" t="inlineStr"/>
-      <c r="F42" s="59" t="inlineStr">
-        <is>
-          <t>Weekly lecture - quiz prep</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Sep 1-4: Everyday Life (lecture topics)</t>
-        </is>
-      </c>
-      <c r="B43" s="59" t="inlineStr"/>
-      <c r="C43" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="D43" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="E43" s="59" t="inlineStr"/>
-      <c r="F43" s="59" t="inlineStr">
-        <is>
-          <t>Weekly lecture - quiz prep</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Sep 8-11: Renaissance (lecture topics)</t>
-        </is>
-      </c>
-      <c r="B44" s="59" t="inlineStr"/>
-      <c r="C44" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="D44" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="E44" s="59" t="inlineStr"/>
-      <c r="F44" s="59" t="inlineStr">
-        <is>
-          <t>Weekly lecture - quiz prep</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Sep 15-18: Renaissance (lecture topics)</t>
-        </is>
-      </c>
-      <c r="B45" s="59" t="inlineStr"/>
-      <c r="C45" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="D45" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="E45" s="59" t="inlineStr"/>
-      <c r="F45" s="59" t="inlineStr">
-        <is>
-          <t>Weekly lecture - quiz prep</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Sep 20-24: European Expansion (lecture topics)</t>
-        </is>
-      </c>
-      <c r="B46" s="59" t="inlineStr"/>
-      <c r="C46" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="D46" s="59" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="E46" s="59" t="inlineStr"/>
-      <c r="F46" s="59" t="inlineStr">
-        <is>
-          <t>Weekly lecture - quiz prep</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Oct 6-9: Midterm &amp; Break (lecture topics)</t>
-        </is>
-      </c>
-      <c r="B47" s="59" t="inlineStr"/>
-      <c r="C47" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="D47" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="E47" s="59" t="inlineStr"/>
-      <c r="F47" s="59" t="inlineStr">
-        <is>
-          <t>Weekly lecture - quiz prep</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Oct 13-16: The Reformation (lecture topics)</t>
-        </is>
-      </c>
-      <c r="B48" s="59" t="inlineStr"/>
-      <c r="C48" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="D48" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="E48" s="59" t="inlineStr"/>
-      <c r="F48" s="59" t="inlineStr">
-        <is>
-          <t>Weekly lecture - quiz prep</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Oct 20-23: The Reformation (lecture topics)</t>
-        </is>
-      </c>
-      <c r="B49" s="59" t="inlineStr"/>
-      <c r="C49" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="D49" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="E49" s="59" t="inlineStr"/>
-      <c r="F49" s="59" t="inlineStr">
-        <is>
-          <t>Weekly lecture - quiz prep</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Oct 27-30: Reformation (lecture topics)</t>
-        </is>
-      </c>
-      <c r="B50" s="59" t="inlineStr"/>
-      <c r="C50" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-27</t>
-        </is>
-      </c>
-      <c r="D50" s="59" t="inlineStr">
-        <is>
-          <t>2026-10-30</t>
-        </is>
-      </c>
-      <c r="E50" s="59" t="inlineStr"/>
-      <c r="F50" s="59" t="inlineStr">
-        <is>
-          <t>Weekly lecture - quiz prep</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Nov 3-6: Witches &amp; Science (lecture topics)</t>
-        </is>
-      </c>
-      <c r="B51" s="59" t="inlineStr"/>
-      <c r="C51" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-03</t>
-        </is>
-      </c>
-      <c r="D51" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-06</t>
-        </is>
-      </c>
-      <c r="E51" s="59" t="inlineStr"/>
-      <c r="F51" s="59" t="inlineStr">
-        <is>
-          <t>Weekly lecture - quiz prep</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Nov 10-13: Enlightenment (lecture topics)</t>
-        </is>
-      </c>
-      <c r="B52" s="59" t="inlineStr"/>
-      <c r="C52" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-10</t>
-        </is>
-      </c>
-      <c r="D52" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-13</t>
-        </is>
-      </c>
-      <c r="E52" s="59" t="inlineStr"/>
-      <c r="F52" s="59" t="inlineStr">
-        <is>
-          <t>Weekly lecture - quiz prep</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Nov 17-20: Enlightenment (lecture topics)</t>
-        </is>
-      </c>
-      <c r="B53" s="59" t="inlineStr"/>
-      <c r="C53" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-17</t>
-        </is>
-      </c>
-      <c r="D53" s="59" t="inlineStr">
-        <is>
-          <t>2026-11-20</t>
-        </is>
-      </c>
-      <c r="E53" s="59" t="inlineStr"/>
-      <c r="F53" s="59" t="inlineStr">
-        <is>
-          <t>Weekly lecture - quiz prep</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ↳ Week Dec 1-4: Modern Europe? (lecture topics)</t>
-        </is>
-      </c>
-      <c r="B54" s="59" t="inlineStr"/>
-      <c r="C54" s="59" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
-      <c r="D54" s="59" t="inlineStr">
-        <is>
-          <t>2026-12-04</t>
-        </is>
-      </c>
-      <c r="E54" s="59" t="inlineStr"/>
-      <c r="F54" s="59" t="inlineStr">
-        <is>
-          <t>Weekly lecture - quiz prep</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="6" t="inlineStr">
-        <is>
-          <t>Extra Credit</t>
-        </is>
-      </c>
-      <c r="B55" s="56" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C55" s="56" t="inlineStr"/>
-      <c r="D55" s="56" t="inlineStr">
-        <is>
-          <t>2026-12-04</t>
-        </is>
-      </c>
-      <c r="E55" s="56" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F55" s="57">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-extra-credit.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B6:F6"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
     <tabColor rgb="00FF7F0E"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -3135,7 +1844,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001F77B4"/>
@@ -4241,4 +2950,1310 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00D62728"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>HIST-103 — The Emergence of Modern Europe</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="2">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/sources/hist-103-source.pdf","SEE HERE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Instructor</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Dr. Lindsay O'Neill</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fall 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Required for an A</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>93% (100-93)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Grading scale</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>A: 100-93; A-: 92-90; B+: 89-87; B: 86-83; B-: 82-80; C+: 79-77; C: 76-73; C- 72-70 D+: 69-67; D: 66-63; D-: 62-60; F: 59-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Group Project</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Sleep Paper</t>
+        </is>
+      </c>
+      <c r="B9" s="73" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="C9" s="73" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D9" s="73" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="E9" s="73" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" s="74">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-sleep-paper.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Sleep Paper Due</t>
+        </is>
+      </c>
+      <c r="B10" s="75" t="inlineStr"/>
+      <c r="C10" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D10" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="E10" s="75" t="inlineStr"/>
+      <c r="F10" s="75" t="inlineStr">
+        <is>
+          <t>Due date (course schedule)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 15-18: Renaissance</t>
+        </is>
+      </c>
+      <c r="B11" s="75" t="inlineStr"/>
+      <c r="C11" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D11" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="E11" s="75" t="inlineStr"/>
+      <c r="F11" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Witchcraft Paper</t>
+        </is>
+      </c>
+      <c r="B12" s="76" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="C12" s="76" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D12" s="76" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="E12" s="76" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F12" s="77">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-witchcraft-paper.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Witchcraft Paper Due</t>
+        </is>
+      </c>
+      <c r="B13" s="75" t="inlineStr"/>
+      <c r="C13" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="D13" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="E13" s="75" t="inlineStr"/>
+      <c r="F13" s="75" t="inlineStr">
+        <is>
+          <t>Due date (course schedule)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Nov 10-13: Enlightenment</t>
+        </is>
+      </c>
+      <c r="B14" s="75" t="inlineStr"/>
+      <c r="C14" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="D14" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-13</t>
+        </is>
+      </c>
+      <c r="E14" s="75" t="inlineStr"/>
+      <c r="F14" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Mid-term</t>
+        </is>
+      </c>
+      <c r="B15" s="73" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="C15" s="73" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D15" s="73" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E15" s="73" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F15" s="74">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-mid-term.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Midterm Exam</t>
+        </is>
+      </c>
+      <c r="B16" s="75" t="inlineStr"/>
+      <c r="C16" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="D16" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="E16" s="75" t="inlineStr"/>
+      <c r="F16" s="75" t="inlineStr">
+        <is>
+          <t>Oct 6: Midterm</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Oct 6-9: Midterm &amp; Break</t>
+        </is>
+      </c>
+      <c r="B17" s="75" t="inlineStr"/>
+      <c r="C17" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="D17" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E17" s="75" t="inlineStr"/>
+      <c r="F17" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Dec 1-4: Modern Europe?</t>
+        </is>
+      </c>
+      <c r="B18" s="75" t="inlineStr"/>
+      <c r="C18" s="75" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="D18" s="75" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E18" s="75" t="inlineStr"/>
+      <c r="F18" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+      <c r="B19" s="76" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="C19" s="76" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D19" s="76" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E19" s="76" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F19" s="77">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-final-exam.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Final Exam</t>
+        </is>
+      </c>
+      <c r="B20" s="75" t="inlineStr"/>
+      <c r="C20" s="75" t="inlineStr">
+        <is>
+          <t>2026-12-10</t>
+        </is>
+      </c>
+      <c r="D20" s="75" t="inlineStr">
+        <is>
+          <t>2026-12-10</t>
+        </is>
+      </c>
+      <c r="E20" s="75" t="inlineStr"/>
+      <c r="F20" s="75" t="inlineStr">
+        <is>
+          <t>Dec 10: Final Exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Discussion Section</t>
+        </is>
+      </c>
+      <c r="B21" s="73" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="C21" s="73" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="D21" s="73" t="inlineStr">
+        <is>
+          <t>2026-11-12</t>
+        </is>
+      </c>
+      <c r="E21" s="73" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F21" s="74">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-discussion-section.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Aug 25-29: Intro &amp; Black Death</t>
+        </is>
+      </c>
+      <c r="B22" s="75" t="inlineStr"/>
+      <c r="C22" s="75" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D22" s="75" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="E22" s="75" t="inlineStr"/>
+      <c r="F22" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Aug 25-29: Intro &amp; Black Death  -  Section readings 1</t>
+        </is>
+      </c>
+      <c r="B23" s="75" t="inlineStr"/>
+      <c r="C23" s="75" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D23" s="75" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="E23" s="75" t="inlineStr"/>
+      <c r="F23" s="75" t="inlineStr">
+        <is>
+          <t>Homework - -- 13 of 33 -- Lizzie Wade, “From Black Death to fatal flu, past pandemics show why people on the margins suffer most,” Science, May 14, 2020 Alex Brown and Grace Owen, “What a list of Black Death Sur</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 1-4: Everyday Life</t>
+        </is>
+      </c>
+      <c r="B24" s="75" t="inlineStr"/>
+      <c r="C24" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D24" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="E24" s="75" t="inlineStr"/>
+      <c r="F24" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 1-4: Everyday Life  -  Section readings 1</t>
+        </is>
+      </c>
+      <c r="B25" s="75" t="inlineStr"/>
+      <c r="C25" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D25" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="E25" s="75" t="inlineStr"/>
+      <c r="F25" s="75" t="inlineStr">
+        <is>
+          <t>Homework - A Roger Ekirch, “Sleep we have lost: Pre-Industrial Slumber in the British Isles, The American Historical Review, April 2001, pg. 343-365 Sasha Handley, Sleep in Early Modern England, Introduction &amp; C</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 8-11: Renaissance</t>
+        </is>
+      </c>
+      <c r="B26" s="75" t="inlineStr"/>
+      <c r="C26" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="D26" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E26" s="75" t="inlineStr"/>
+      <c r="F26" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 8-11: Renaissance  -  Section readings 1</t>
+        </is>
+      </c>
+      <c r="B27" s="75" t="inlineStr"/>
+      <c r="C27" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="D27" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E27" s="75" t="inlineStr"/>
+      <c r="F27" s="75" t="inlineStr">
+        <is>
+          <t>Homework - -- 14 of 33 -- Kay Daly, “Diverting the Flood of History: Ada Palmer’s Inventing the Renaissance,” Chicago Review of Books, 25 March 2025 Ada Palmer, “Black Death, COVID, and Why We Keep Telling the M</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 15-18: Renaissance  -  Section readings 1</t>
+        </is>
+      </c>
+      <c r="B28" s="75" t="inlineStr"/>
+      <c r="C28" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D28" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="E28" s="75" t="inlineStr"/>
+      <c r="F28" s="75" t="inlineStr">
+        <is>
+          <t>Homework - Vasari, Lives of the Artists: Leonardo da Vinci &amp; Properzia de’ Rossi Video: The Story of Women and Art, Part 1(1hr) Vasari on da Vinci PDF document Vasari on d'Rossi PDF document</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 20-24: European Expansion</t>
+        </is>
+      </c>
+      <c r="B29" s="75" t="inlineStr"/>
+      <c r="C29" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D29" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E29" s="75" t="inlineStr"/>
+      <c r="F29" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 20-24: European Expansion  -  Section readings 1</t>
+        </is>
+      </c>
+      <c r="B30" s="75" t="inlineStr"/>
+      <c r="C30" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D30" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E30" s="75" t="inlineStr"/>
+      <c r="F30" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Homework - Jerry Brotton, The Renaissance Bazaar, Chap 1 (15 pgs) Read Columbus’ Letter on his Return: MacGregor, The History of the World in 100 Objects Read or listen to the stories behind these objects: Part </t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 20-24: European Expansion  -  Section readings 2</t>
+        </is>
+      </c>
+      <c r="B31" s="75" t="inlineStr"/>
+      <c r="C31" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D31" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E31" s="75" t="inlineStr"/>
+      <c r="F31" s="75" t="inlineStr">
+        <is>
+          <t>Homework - Bernal Diaz del Castillo, The True History of the Conquest of New Spain, pg 121-171 Miguel León Portilla, Broken Spears: The Aztec Account of the Conquest of Mexico, Appendix, Chap 8-10 (37 pgs) Broke</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Oct 13-16: The Reformation</t>
+        </is>
+      </c>
+      <c r="B32" s="75" t="inlineStr"/>
+      <c r="C32" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="D32" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="E32" s="75" t="inlineStr"/>
+      <c r="F32" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Oct 20-23: The Reformation</t>
+        </is>
+      </c>
+      <c r="B33" s="75" t="inlineStr"/>
+      <c r="C33" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="D33" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="E33" s="75" t="inlineStr"/>
+      <c r="F33" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Oct 27-30: Reformation</t>
+        </is>
+      </c>
+      <c r="B34" s="75" t="inlineStr"/>
+      <c r="C34" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="D34" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="E34" s="75" t="inlineStr"/>
+      <c r="F34" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Oct 27-30: Reformation  -  Section readings 1</t>
+        </is>
+      </c>
+      <c r="B35" s="75" t="inlineStr"/>
+      <c r="C35" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="D35" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="E35" s="75" t="inlineStr"/>
+      <c r="F35" s="75" t="inlineStr">
+        <is>
+          <t>Homework - Barbara Diefendorf, ed., The Saint Bartholomew’s Day Massacre: A Brief History with Documents, Introduction, Documents 2-6, 9-11, 16-21, 31, 33</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Nov 3-6: Witches &amp; Science</t>
+        </is>
+      </c>
+      <c r="B36" s="75" t="inlineStr"/>
+      <c r="C36" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="D36" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="E36" s="75" t="inlineStr"/>
+      <c r="F36" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Nov 3-6: Witches &amp; Science  -  Section readings 1</t>
+        </is>
+      </c>
+      <c r="B37" s="75" t="inlineStr"/>
+      <c r="C37" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="D37" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="E37" s="75" t="inlineStr"/>
+      <c r="F37" s="75" t="inlineStr">
+        <is>
+          <t>Homework - Brian Levack, The Witchcraft Sourcebook, Chaps 36-44, 46-47 103.Levack.36 PDF document 103.Levack.37 PDF document 103.Levack.38 PDF document 103.Levack.39 PDF document 103.Levack.40 PDF document 103.L</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Nov 10-13: Enlightenment  -  Section readings 1</t>
+        </is>
+      </c>
+      <c r="B38" s="75" t="inlineStr"/>
+      <c r="C38" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="D38" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-13</t>
+        </is>
+      </c>
+      <c r="E38" s="75" t="inlineStr"/>
+      <c r="F38" s="75" t="inlineStr">
+        <is>
+          <t>Homework - Excerpt: John Locke, Two Treatises of Government (1689) Excerpt: Rousseau, The Social Contract (1762) Enlightenment Primary Source Activity [Ungraded, but counts towards participation. Due in section]</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Nov 17-20: Enlightenment</t>
+        </is>
+      </c>
+      <c r="B39" s="75" t="inlineStr"/>
+      <c r="C39" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-17</t>
+        </is>
+      </c>
+      <c r="D39" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="E39" s="75" t="inlineStr"/>
+      <c r="F39" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Nov 17-20: Enlightenment  -  Section readings 1</t>
+        </is>
+      </c>
+      <c r="B40" s="75" t="inlineStr"/>
+      <c r="C40" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-17</t>
+        </is>
+      </c>
+      <c r="D40" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="E40" s="75" t="inlineStr"/>
+      <c r="F40" s="75" t="inlineStr">
+        <is>
+          <t>Homework - Video: Africa &amp; Britain, A Forgotten History, Episode 2: Freedom (50 min) Slavery and the African Presence in London Activity [Ungraded but counts towards participation. Due in section] 103.Act.Enslav</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>Identification Quizzes</t>
+        </is>
+      </c>
+      <c r="B41" s="76" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="C41" s="76" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D41" s="76" t="inlineStr">
+        <is>
+          <t>2026-12-10</t>
+        </is>
+      </c>
+      <c r="E41" s="76" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F41" s="77">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-identification-quizzes.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Aug 25-29: Intro &amp; Black Death (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B42" s="75" t="inlineStr"/>
+      <c r="C42" s="75" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="D42" s="75" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="E42" s="75" t="inlineStr"/>
+      <c r="F42" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 1-4: Everyday Life (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B43" s="75" t="inlineStr"/>
+      <c r="C43" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D43" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="E43" s="75" t="inlineStr"/>
+      <c r="F43" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 8-11: Renaissance (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B44" s="75" t="inlineStr"/>
+      <c r="C44" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="D44" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E44" s="75" t="inlineStr"/>
+      <c r="F44" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 15-18: Renaissance (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B45" s="75" t="inlineStr"/>
+      <c r="C45" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="D45" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="E45" s="75" t="inlineStr"/>
+      <c r="F45" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Sep 20-24: European Expansion (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B46" s="75" t="inlineStr"/>
+      <c r="C46" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D46" s="75" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E46" s="75" t="inlineStr"/>
+      <c r="F46" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Oct 6-9: Midterm &amp; Break (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B47" s="75" t="inlineStr"/>
+      <c r="C47" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="D47" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E47" s="75" t="inlineStr"/>
+      <c r="F47" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Oct 13-16: The Reformation (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B48" s="75" t="inlineStr"/>
+      <c r="C48" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="D48" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="E48" s="75" t="inlineStr"/>
+      <c r="F48" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Oct 20-23: The Reformation (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B49" s="75" t="inlineStr"/>
+      <c r="C49" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="D49" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="E49" s="75" t="inlineStr"/>
+      <c r="F49" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Oct 27-30: Reformation (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B50" s="75" t="inlineStr"/>
+      <c r="C50" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="D50" s="75" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="E50" s="75" t="inlineStr"/>
+      <c r="F50" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Nov 3-6: Witches &amp; Science (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B51" s="75" t="inlineStr"/>
+      <c r="C51" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="D51" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="E51" s="75" t="inlineStr"/>
+      <c r="F51" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Nov 10-13: Enlightenment (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B52" s="75" t="inlineStr"/>
+      <c r="C52" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="D52" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-13</t>
+        </is>
+      </c>
+      <c r="E52" s="75" t="inlineStr"/>
+      <c r="F52" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Nov 17-20: Enlightenment (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B53" s="75" t="inlineStr"/>
+      <c r="C53" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-17</t>
+        </is>
+      </c>
+      <c r="D53" s="75" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="E53" s="75" t="inlineStr"/>
+      <c r="F53" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ↳ Week Dec 1-4: Modern Europe? (lecture topics)</t>
+        </is>
+      </c>
+      <c r="B54" s="75" t="inlineStr"/>
+      <c r="C54" s="75" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="D54" s="75" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E54" s="75" t="inlineStr"/>
+      <c r="F54" s="75" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>Extra Credit</t>
+        </is>
+      </c>
+      <c r="B55" s="73" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C55" s="73" t="inlineStr"/>
+      <c r="D55" s="73" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E55" s="73" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F55" s="74">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/hist-103-extra-credit.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B6:F6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Only show verified start dates; blank when not in syllabus
- parse_dates_from_text and calendar date parsers: due only, no inferred start
- Marshall deliverables: start only from MARSHALL_INFERRED_STARTS prose matches
- HIST-103 due lines and major assignments: blank start, due only
- Pre-Aug 1 and N/A starts become empty cells in Excel
- Document verified-only start date policy in SKILL.md and reference.md
- Regenerated all three class sheets

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -221,7 +221,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="134">
+  <cellXfs count="146">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -612,6 +612,42 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1088,22 +1124,18 @@
           <t>Sleep Paper</t>
         </is>
       </c>
-      <c r="B9" s="94" t="inlineStr">
+      <c r="B9" s="134" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C9" s="95" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D9" s="95" t="inlineStr">
+      <c r="C9" s="135" t="inlineStr"/>
+      <c r="D9" s="135" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="E9" s="95" t="inlineStr">
+      <c r="E9" s="135" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1119,18 +1151,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B10" s="98" t="inlineStr"/>
-      <c r="C10" s="98" t="inlineStr">
+      <c r="B10" s="136" t="inlineStr"/>
+      <c r="C10" s="136" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D10" s="98" t="inlineStr">
+      <c r="D10" s="136" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E10" s="98" t="inlineStr"/>
+      <c r="E10" s="136" t="inlineStr"/>
       <c r="F10" s="99" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance</t>
@@ -1143,18 +1175,14 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B11" s="98" t="inlineStr"/>
-      <c r="C11" s="98" t="inlineStr">
+      <c r="B11" s="136" t="inlineStr"/>
+      <c r="C11" s="136" t="inlineStr"/>
+      <c r="D11" s="136" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D11" s="98" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="E11" s="98" t="inlineStr"/>
+      <c r="E11" s="136" t="inlineStr"/>
       <c r="F11" s="99" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
@@ -1167,22 +1195,18 @@
           <t>Witchcraft Paper</t>
         </is>
       </c>
-      <c r="B12" s="94" t="inlineStr">
+      <c r="B12" s="134" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C12" s="102" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="D12" s="102" t="inlineStr">
+      <c r="C12" s="137" t="inlineStr"/>
+      <c r="D12" s="137" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="E12" s="102" t="inlineStr">
+      <c r="E12" s="137" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1198,18 +1222,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B13" s="98" t="inlineStr"/>
-      <c r="C13" s="98" t="inlineStr">
+      <c r="B13" s="136" t="inlineStr"/>
+      <c r="C13" s="136" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D13" s="98" t="inlineStr">
+      <c r="D13" s="136" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E13" s="98" t="inlineStr"/>
+      <c r="E13" s="136" t="inlineStr"/>
       <c r="F13" s="99" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment</t>
@@ -1222,18 +1246,14 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B14" s="98" t="inlineStr"/>
-      <c r="C14" s="98" t="inlineStr">
+      <c r="B14" s="136" t="inlineStr"/>
+      <c r="C14" s="136" t="inlineStr"/>
+      <c r="D14" s="136" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D14" s="98" t="inlineStr">
-        <is>
-          <t>2026-11-10</t>
-        </is>
-      </c>
-      <c r="E14" s="98" t="inlineStr"/>
+      <c r="E14" s="136" t="inlineStr"/>
       <c r="F14" s="99" t="inlineStr">
         <is>
           <t>Witchcraft Paper Due</t>
@@ -1246,22 +1266,18 @@
           <t>Mid-term</t>
         </is>
       </c>
-      <c r="B15" s="94" t="inlineStr">
+      <c r="B15" s="134" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C15" s="95" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="D15" s="95" t="inlineStr">
+      <c r="C15" s="135" t="inlineStr"/>
+      <c r="D15" s="135" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E15" s="95" t="inlineStr">
+      <c r="E15" s="135" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1277,18 +1293,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B16" s="98" t="inlineStr"/>
-      <c r="C16" s="98" t="inlineStr">
+      <c r="B16" s="136" t="inlineStr"/>
+      <c r="C16" s="136" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="D16" s="98" t="inlineStr">
+      <c r="D16" s="136" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E16" s="98" t="inlineStr"/>
+      <c r="E16" s="136" t="inlineStr"/>
       <c r="F16" s="99" t="inlineStr">
         <is>
           <t>Week Oct 6-9: Midterm &amp; Break</t>
@@ -1301,18 +1317,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B17" s="98" t="inlineStr"/>
-      <c r="C17" s="98" t="inlineStr">
+      <c r="B17" s="136" t="inlineStr"/>
+      <c r="C17" s="136" t="inlineStr">
         <is>
           <t>2026-12-01</t>
         </is>
       </c>
-      <c r="D17" s="98" t="inlineStr">
+      <c r="D17" s="136" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E17" s="98" t="inlineStr"/>
+      <c r="E17" s="136" t="inlineStr"/>
       <c r="F17" s="99" t="inlineStr">
         <is>
           <t>Week Dec 1-4: Modern Europe?</t>
@@ -1325,18 +1341,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B18" s="98" t="inlineStr"/>
-      <c r="C18" s="98" t="inlineStr">
+      <c r="B18" s="136" t="inlineStr"/>
+      <c r="C18" s="136" t="inlineStr"/>
+      <c r="D18" s="136" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="D18" s="98" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="E18" s="98" t="inlineStr"/>
+      <c r="E18" s="136" t="inlineStr"/>
       <c r="F18" s="99" t="inlineStr">
         <is>
           <t>Midterm Exam</t>
@@ -1349,22 +1361,18 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B19" s="94" t="inlineStr">
+      <c r="B19" s="134" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C19" s="102" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D19" s="102" t="inlineStr">
+      <c r="C19" s="137" t="inlineStr"/>
+      <c r="D19" s="137" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="E19" s="102" t="inlineStr">
+      <c r="E19" s="137" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1380,18 +1388,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B20" s="98" t="inlineStr"/>
-      <c r="C20" s="98" t="inlineStr">
+      <c r="B20" s="136" t="inlineStr"/>
+      <c r="C20" s="136" t="inlineStr"/>
+      <c r="D20" s="136" t="inlineStr">
         <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="D20" s="98" t="inlineStr">
-        <is>
-          <t>2026-12-10</t>
-        </is>
-      </c>
-      <c r="E20" s="98" t="inlineStr"/>
+      <c r="E20" s="136" t="inlineStr"/>
       <c r="F20" s="99" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -1404,22 +1408,18 @@
           <t>Discussion Section</t>
         </is>
       </c>
-      <c r="B21" s="94" t="inlineStr">
+      <c r="B21" s="134" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C21" s="95" t="inlineStr">
-        <is>
-          <t>2026-11-10</t>
-        </is>
-      </c>
-      <c r="D21" s="95" t="inlineStr">
+      <c r="C21" s="135" t="inlineStr"/>
+      <c r="D21" s="135" t="inlineStr">
         <is>
           <t>2026-11-12</t>
         </is>
       </c>
-      <c r="E21" s="95" t="inlineStr">
+      <c r="E21" s="135" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1435,18 +1435,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B22" s="98" t="inlineStr"/>
-      <c r="C22" s="98" t="inlineStr">
+      <c r="B22" s="136" t="inlineStr"/>
+      <c r="C22" s="136" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D22" s="98" t="inlineStr">
+      <c r="D22" s="136" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E22" s="98" t="inlineStr"/>
+      <c r="E22" s="136" t="inlineStr"/>
       <c r="F22" s="99" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death</t>
@@ -1459,18 +1459,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B23" s="98" t="inlineStr"/>
-      <c r="C23" s="98" t="inlineStr">
+      <c r="B23" s="136" t="inlineStr"/>
+      <c r="C23" s="136" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D23" s="98" t="inlineStr">
+      <c r="D23" s="136" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E23" s="98" t="inlineStr"/>
+      <c r="E23" s="136" t="inlineStr"/>
       <c r="F23" s="99" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death - Section reading 1: -- 13 of 33 -- Lizzie Wade, “From Black Death to fatal flu, pas</t>
@@ -1483,18 +1483,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B24" s="98" t="inlineStr"/>
-      <c r="C24" s="98" t="inlineStr">
+      <c r="B24" s="136" t="inlineStr"/>
+      <c r="C24" s="136" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D24" s="98" t="inlineStr">
+      <c r="D24" s="136" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E24" s="98" t="inlineStr"/>
+      <c r="E24" s="136" t="inlineStr"/>
       <c r="F24" s="99" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life</t>
@@ -1507,18 +1507,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B25" s="98" t="inlineStr"/>
-      <c r="C25" s="98" t="inlineStr">
+      <c r="B25" s="136" t="inlineStr"/>
+      <c r="C25" s="136" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D25" s="98" t="inlineStr">
+      <c r="D25" s="136" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E25" s="98" t="inlineStr"/>
+      <c r="E25" s="136" t="inlineStr"/>
       <c r="F25" s="99" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life - Section reading 1: A Roger Ekirch, “Sleep we have lost: Pre-Industrial Slumber in the Brit</t>
@@ -1531,18 +1531,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B26" s="98" t="inlineStr"/>
-      <c r="C26" s="98" t="inlineStr">
+      <c r="B26" s="136" t="inlineStr"/>
+      <c r="C26" s="136" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D26" s="98" t="inlineStr">
+      <c r="D26" s="136" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E26" s="98" t="inlineStr"/>
+      <c r="E26" s="136" t="inlineStr"/>
       <c r="F26" s="99" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance</t>
@@ -1555,18 +1555,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B27" s="98" t="inlineStr"/>
-      <c r="C27" s="98" t="inlineStr">
+      <c r="B27" s="136" t="inlineStr"/>
+      <c r="C27" s="136" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D27" s="98" t="inlineStr">
+      <c r="D27" s="136" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E27" s="98" t="inlineStr"/>
+      <c r="E27" s="136" t="inlineStr"/>
       <c r="F27" s="99" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance - Section reading 1: -- 14 of 33 -- Kay Daly, “Diverting the Flood of History: Ada Palmer’s I</t>
@@ -1579,18 +1579,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B28" s="98" t="inlineStr"/>
-      <c r="C28" s="98" t="inlineStr">
+      <c r="B28" s="136" t="inlineStr"/>
+      <c r="C28" s="136" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D28" s="98" t="inlineStr">
+      <c r="D28" s="136" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E28" s="98" t="inlineStr"/>
+      <c r="E28" s="136" t="inlineStr"/>
       <c r="F28" s="99" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance - Section reading 1: Vasari, Lives of the Artists: Leonardo da Vinci &amp; Properzia de’ Rossi V</t>
@@ -1603,18 +1603,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B29" s="98" t="inlineStr"/>
-      <c r="C29" s="98" t="inlineStr">
+      <c r="B29" s="136" t="inlineStr"/>
+      <c r="C29" s="136" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D29" s="98" t="inlineStr">
+      <c r="D29" s="136" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E29" s="98" t="inlineStr"/>
+      <c r="E29" s="136" t="inlineStr"/>
       <c r="F29" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion</t>
@@ -1627,18 +1627,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B30" s="98" t="inlineStr"/>
-      <c r="C30" s="98" t="inlineStr">
+      <c r="B30" s="136" t="inlineStr"/>
+      <c r="C30" s="136" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D30" s="98" t="inlineStr">
+      <c r="D30" s="136" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E30" s="98" t="inlineStr"/>
+      <c r="E30" s="136" t="inlineStr"/>
       <c r="F30" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion - Section reading 1: Jerry Brotton, The Renaissance Bazaar, Chap 1 (15 pgs) Read Colu</t>
@@ -1651,18 +1651,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B31" s="98" t="inlineStr"/>
-      <c r="C31" s="98" t="inlineStr">
+      <c r="B31" s="136" t="inlineStr"/>
+      <c r="C31" s="136" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D31" s="98" t="inlineStr">
+      <c r="D31" s="136" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E31" s="98" t="inlineStr"/>
+      <c r="E31" s="136" t="inlineStr"/>
       <c r="F31" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion - Section reading 2: Bernal Diaz del Castillo, The True History of the Conquest of Ne</t>
@@ -1675,18 +1675,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B32" s="98" t="inlineStr"/>
-      <c r="C32" s="98" t="inlineStr">
+      <c r="B32" s="136" t="inlineStr"/>
+      <c r="C32" s="136" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="D32" s="98" t="inlineStr">
+      <c r="D32" s="136" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="E32" s="98" t="inlineStr"/>
+      <c r="E32" s="136" t="inlineStr"/>
       <c r="F32" s="99" t="inlineStr">
         <is>
           <t>Week Oct 13-16: The Reformation</t>
@@ -1699,18 +1699,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B33" s="98" t="inlineStr"/>
-      <c r="C33" s="98" t="inlineStr">
+      <c r="B33" s="136" t="inlineStr"/>
+      <c r="C33" s="136" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="D33" s="98" t="inlineStr">
+      <c r="D33" s="136" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="E33" s="98" t="inlineStr"/>
+      <c r="E33" s="136" t="inlineStr"/>
       <c r="F33" s="99" t="inlineStr">
         <is>
           <t>Week Oct 20-23: The Reformation</t>
@@ -1723,18 +1723,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B34" s="98" t="inlineStr"/>
-      <c r="C34" s="98" t="inlineStr">
+      <c r="B34" s="136" t="inlineStr"/>
+      <c r="C34" s="136" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D34" s="98" t="inlineStr">
+      <c r="D34" s="136" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E34" s="98" t="inlineStr"/>
+      <c r="E34" s="136" t="inlineStr"/>
       <c r="F34" s="99" t="inlineStr">
         <is>
           <t>Week Oct 27-30: Reformation</t>
@@ -1747,18 +1747,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B35" s="98" t="inlineStr"/>
-      <c r="C35" s="98" t="inlineStr">
+      <c r="B35" s="136" t="inlineStr"/>
+      <c r="C35" s="136" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D35" s="98" t="inlineStr">
+      <c r="D35" s="136" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E35" s="98" t="inlineStr"/>
+      <c r="E35" s="136" t="inlineStr"/>
       <c r="F35" s="99" t="inlineStr">
         <is>
           <t xml:space="preserve">Week Oct 27-30: Reformation - Section reading 1: Barbara Diefendorf, ed., The Saint Bartholomew’s Day Massacre: A Brief </t>
@@ -1771,18 +1771,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B36" s="98" t="inlineStr"/>
-      <c r="C36" s="98" t="inlineStr">
+      <c r="B36" s="136" t="inlineStr"/>
+      <c r="C36" s="136" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D36" s="98" t="inlineStr">
+      <c r="D36" s="136" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E36" s="98" t="inlineStr"/>
+      <c r="E36" s="136" t="inlineStr"/>
       <c r="F36" s="99" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science</t>
@@ -1795,18 +1795,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B37" s="98" t="inlineStr"/>
-      <c r="C37" s="98" t="inlineStr">
+      <c r="B37" s="136" t="inlineStr"/>
+      <c r="C37" s="136" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D37" s="98" t="inlineStr">
+      <c r="D37" s="136" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E37" s="98" t="inlineStr"/>
+      <c r="E37" s="136" t="inlineStr"/>
       <c r="F37" s="99" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science - Section reading 1: Brian Levack, The Witchcraft Sourcebook, Chaps 36-44, 46-47 103.Lev</t>
@@ -1819,18 +1819,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B38" s="98" t="inlineStr"/>
-      <c r="C38" s="98" t="inlineStr">
+      <c r="B38" s="136" t="inlineStr"/>
+      <c r="C38" s="136" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D38" s="98" t="inlineStr">
+      <c r="D38" s="136" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E38" s="98" t="inlineStr"/>
+      <c r="E38" s="136" t="inlineStr"/>
       <c r="F38" s="99" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment - Section reading 1: Excerpt: John Locke, Two Treatises of Government (1689) Excerpt: Rous</t>
@@ -1843,18 +1843,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B39" s="98" t="inlineStr"/>
-      <c r="C39" s="98" t="inlineStr">
+      <c r="B39" s="136" t="inlineStr"/>
+      <c r="C39" s="136" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D39" s="98" t="inlineStr">
+      <c r="D39" s="136" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E39" s="98" t="inlineStr"/>
+      <c r="E39" s="136" t="inlineStr"/>
       <c r="F39" s="99" t="inlineStr">
         <is>
           <t>Week Nov 17-20: Enlightenment</t>
@@ -1867,18 +1867,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B40" s="98" t="inlineStr"/>
-      <c r="C40" s="98" t="inlineStr">
+      <c r="B40" s="136" t="inlineStr"/>
+      <c r="C40" s="136" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D40" s="98" t="inlineStr">
+      <c r="D40" s="136" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E40" s="98" t="inlineStr"/>
+      <c r="E40" s="136" t="inlineStr"/>
       <c r="F40" s="99" t="inlineStr">
         <is>
           <t xml:space="preserve">Week Nov 17-20: Enlightenment - Section reading 1: Video: Africa &amp; Britain, A Forgotten History, Episode 2: Freedom (50 </t>
@@ -1891,22 +1891,18 @@
           <t>Identification Quizzes</t>
         </is>
       </c>
-      <c r="B41" s="94" t="inlineStr">
+      <c r="B41" s="134" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C41" s="102" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="D41" s="102" t="inlineStr">
+      <c r="C41" s="137" t="inlineStr"/>
+      <c r="D41" s="137" t="inlineStr">
         <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="E41" s="102" t="inlineStr">
+      <c r="E41" s="137" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1922,18 +1918,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B42" s="98" t="inlineStr"/>
-      <c r="C42" s="98" t="inlineStr">
+      <c r="B42" s="136" t="inlineStr"/>
+      <c r="C42" s="136" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D42" s="98" t="inlineStr">
+      <c r="D42" s="136" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E42" s="98" t="inlineStr"/>
+      <c r="E42" s="136" t="inlineStr"/>
       <c r="F42" s="99" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death (lecture topics)</t>
@@ -1946,18 +1942,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B43" s="98" t="inlineStr"/>
-      <c r="C43" s="98" t="inlineStr">
+      <c r="B43" s="136" t="inlineStr"/>
+      <c r="C43" s="136" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D43" s="98" t="inlineStr">
+      <c r="D43" s="136" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E43" s="98" t="inlineStr"/>
+      <c r="E43" s="136" t="inlineStr"/>
       <c r="F43" s="99" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life (lecture topics)</t>
@@ -1970,18 +1966,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B44" s="98" t="inlineStr"/>
-      <c r="C44" s="98" t="inlineStr">
+      <c r="B44" s="136" t="inlineStr"/>
+      <c r="C44" s="136" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D44" s="98" t="inlineStr">
+      <c r="D44" s="136" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E44" s="98" t="inlineStr"/>
+      <c r="E44" s="136" t="inlineStr"/>
       <c r="F44" s="99" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance (lecture topics)</t>
@@ -1994,18 +1990,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B45" s="98" t="inlineStr"/>
-      <c r="C45" s="98" t="inlineStr">
+      <c r="B45" s="136" t="inlineStr"/>
+      <c r="C45" s="136" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D45" s="98" t="inlineStr">
+      <c r="D45" s="136" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E45" s="98" t="inlineStr"/>
+      <c r="E45" s="136" t="inlineStr"/>
       <c r="F45" s="99" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance (lecture topics)</t>
@@ -2018,18 +2014,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B46" s="98" t="inlineStr"/>
-      <c r="C46" s="98" t="inlineStr">
+      <c r="B46" s="136" t="inlineStr"/>
+      <c r="C46" s="136" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D46" s="98" t="inlineStr">
+      <c r="D46" s="136" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E46" s="98" t="inlineStr"/>
+      <c r="E46" s="136" t="inlineStr"/>
       <c r="F46" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion (lecture topics)</t>
@@ -2042,18 +2038,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B47" s="98" t="inlineStr"/>
-      <c r="C47" s="98" t="inlineStr">
+      <c r="B47" s="136" t="inlineStr"/>
+      <c r="C47" s="136" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="D47" s="98" t="inlineStr">
+      <c r="D47" s="136" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E47" s="98" t="inlineStr"/>
+      <c r="E47" s="136" t="inlineStr"/>
       <c r="F47" s="99" t="inlineStr">
         <is>
           <t>Week Oct 6-9: Midterm &amp; Break (lecture topics)</t>
@@ -2066,18 +2062,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B48" s="98" t="inlineStr"/>
-      <c r="C48" s="98" t="inlineStr">
+      <c r="B48" s="136" t="inlineStr"/>
+      <c r="C48" s="136" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="D48" s="98" t="inlineStr">
+      <c r="D48" s="136" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="E48" s="98" t="inlineStr"/>
+      <c r="E48" s="136" t="inlineStr"/>
       <c r="F48" s="99" t="inlineStr">
         <is>
           <t>Week Oct 13-16: The Reformation (lecture topics)</t>
@@ -2090,18 +2086,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B49" s="98" t="inlineStr"/>
-      <c r="C49" s="98" t="inlineStr">
+      <c r="B49" s="136" t="inlineStr"/>
+      <c r="C49" s="136" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="D49" s="98" t="inlineStr">
+      <c r="D49" s="136" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="E49" s="98" t="inlineStr"/>
+      <c r="E49" s="136" t="inlineStr"/>
       <c r="F49" s="99" t="inlineStr">
         <is>
           <t>Week Oct 20-23: The Reformation (lecture topics)</t>
@@ -2114,18 +2110,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B50" s="98" t="inlineStr"/>
-      <c r="C50" s="98" t="inlineStr">
+      <c r="B50" s="136" t="inlineStr"/>
+      <c r="C50" s="136" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D50" s="98" t="inlineStr">
+      <c r="D50" s="136" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E50" s="98" t="inlineStr"/>
+      <c r="E50" s="136" t="inlineStr"/>
       <c r="F50" s="99" t="inlineStr">
         <is>
           <t>Week Oct 27-30: Reformation (lecture topics)</t>
@@ -2138,18 +2134,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B51" s="98" t="inlineStr"/>
-      <c r="C51" s="98" t="inlineStr">
+      <c r="B51" s="136" t="inlineStr"/>
+      <c r="C51" s="136" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D51" s="98" t="inlineStr">
+      <c r="D51" s="136" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E51" s="98" t="inlineStr"/>
+      <c r="E51" s="136" t="inlineStr"/>
       <c r="F51" s="99" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science (lecture topics)</t>
@@ -2162,18 +2158,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B52" s="98" t="inlineStr"/>
-      <c r="C52" s="98" t="inlineStr">
+      <c r="B52" s="136" t="inlineStr"/>
+      <c r="C52" s="136" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D52" s="98" t="inlineStr">
+      <c r="D52" s="136" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E52" s="98" t="inlineStr"/>
+      <c r="E52" s="136" t="inlineStr"/>
       <c r="F52" s="99" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment (lecture topics)</t>
@@ -2186,18 +2182,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B53" s="98" t="inlineStr"/>
-      <c r="C53" s="98" t="inlineStr">
+      <c r="B53" s="136" t="inlineStr"/>
+      <c r="C53" s="136" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D53" s="98" t="inlineStr">
+      <c r="D53" s="136" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E53" s="98" t="inlineStr"/>
+      <c r="E53" s="136" t="inlineStr"/>
       <c r="F53" s="99" t="inlineStr">
         <is>
           <t>Week Nov 17-20: Enlightenment (lecture topics)</t>
@@ -2210,18 +2206,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B54" s="98" t="inlineStr"/>
-      <c r="C54" s="98" t="inlineStr">
+      <c r="B54" s="136" t="inlineStr"/>
+      <c r="C54" s="136" t="inlineStr">
         <is>
           <t>2026-12-01</t>
         </is>
       </c>
-      <c r="D54" s="98" t="inlineStr">
+      <c r="D54" s="136" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E54" s="98" t="inlineStr"/>
+      <c r="E54" s="136" t="inlineStr"/>
       <c r="F54" s="99" t="inlineStr">
         <is>
           <t>Week Dec 1-4: Modern Europe? (lecture topics)</t>
@@ -2234,18 +2230,18 @@
           <t>Extra Credit</t>
         </is>
       </c>
-      <c r="B55" s="94" t="inlineStr">
+      <c r="B55" s="134" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C55" s="95" t="inlineStr"/>
-      <c r="D55" s="95" t="inlineStr">
+      <c r="C55" s="135" t="inlineStr"/>
+      <c r="D55" s="135" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E55" s="95" t="inlineStr">
+      <c r="E55" s="135" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2394,18 +2390,18 @@
           <t>Midterm 1</t>
         </is>
       </c>
-      <c r="B9" s="107" t="inlineStr">
+      <c r="B9" s="138" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C9" s="108" t="inlineStr"/>
-      <c r="D9" s="108" t="inlineStr">
+      <c r="C9" s="139" t="inlineStr"/>
+      <c r="D9" s="139" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="E9" s="108" t="inlineStr">
+      <c r="E9" s="139" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2421,18 +2417,18 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B10" s="111" t="inlineStr"/>
-      <c r="C10" s="111" t="inlineStr">
+      <c r="B10" s="140" t="inlineStr"/>
+      <c r="C10" s="140" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="D10" s="111" t="inlineStr">
+      <c r="D10" s="140" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="E10" s="111" t="inlineStr"/>
+      <c r="E10" s="140" t="inlineStr"/>
       <c r="F10" s="112" t="inlineStr">
         <is>
           <t>9/30 Midterm 1: 250 Points Chapters 1, 2, 3, 4, 5, 8</t>
@@ -2445,18 +2441,18 @@
           <t>Midterm 2</t>
         </is>
       </c>
-      <c r="B11" s="107" t="inlineStr">
+      <c r="B11" s="138" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C11" s="114" t="inlineStr"/>
-      <c r="D11" s="114" t="inlineStr">
+      <c r="C11" s="141" t="inlineStr"/>
+      <c r="D11" s="141" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E11" s="114" t="inlineStr">
+      <c r="E11" s="141" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2472,18 +2468,18 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B12" s="111" t="inlineStr"/>
-      <c r="C12" s="111" t="inlineStr">
+      <c r="B12" s="140" t="inlineStr"/>
+      <c r="C12" s="140" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="D12" s="111" t="inlineStr">
+      <c r="D12" s="140" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E12" s="111" t="inlineStr"/>
+      <c r="E12" s="140" t="inlineStr"/>
       <c r="F12" s="112" t="inlineStr">
         <is>
           <t>10/26 Midterm 2: 250 Points Chapters 6, 7, 9, &amp; 16</t>
@@ -2496,18 +2492,18 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B13" s="107" t="inlineStr">
+      <c r="B13" s="138" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C13" s="108" t="inlineStr"/>
-      <c r="D13" s="108" t="inlineStr">
+      <c r="C13" s="139" t="inlineStr"/>
+      <c r="D13" s="139" t="inlineStr">
         <is>
           <t>2026-12-16</t>
         </is>
       </c>
-      <c r="E13" s="108" t="inlineStr">
+      <c r="E13" s="139" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2523,18 +2519,18 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B14" s="111" t="inlineStr"/>
-      <c r="C14" s="111" t="inlineStr">
+      <c r="B14" s="140" t="inlineStr"/>
+      <c r="C14" s="140" t="inlineStr">
         <is>
           <t>2026-12-16</t>
         </is>
       </c>
-      <c r="D14" s="111" t="inlineStr">
+      <c r="D14" s="140" t="inlineStr">
         <is>
           <t>2026-12-16</t>
         </is>
       </c>
-      <c r="E14" s="111" t="inlineStr"/>
+      <c r="E14" s="140" t="inlineStr"/>
       <c r="F14" s="112" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -2547,22 +2543,22 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B15" s="107" t="inlineStr">
+      <c r="B15" s="138" t="inlineStr">
         <is>
           <t>170 pts</t>
         </is>
       </c>
-      <c r="C15" s="114" t="inlineStr">
+      <c r="C15" s="141" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="D15" s="114" t="inlineStr">
+      <c r="D15" s="141" t="inlineStr">
         <is>
           <t>2026-11-16</t>
         </is>
       </c>
-      <c r="E15" s="114" t="inlineStr">
+      <c r="E15" s="141" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2578,18 +2574,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B16" s="111" t="inlineStr"/>
-      <c r="C16" s="111" t="inlineStr">
+      <c r="B16" s="140" t="inlineStr"/>
+      <c r="C16" s="140" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D16" s="111" t="inlineStr">
+      <c r="D16" s="140" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="E16" s="111" t="inlineStr"/>
+      <c r="E16" s="140" t="inlineStr"/>
       <c r="F16" s="112" t="inlineStr">
         <is>
           <t>Class 1 (8/24) - Course Overview &amp; Introductions</t>
@@ -2602,18 +2598,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B17" s="111" t="inlineStr"/>
-      <c r="C17" s="111" t="inlineStr">
+      <c r="B17" s="140" t="inlineStr"/>
+      <c r="C17" s="140" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D17" s="111" t="inlineStr">
+      <c r="D17" s="140" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="E17" s="111" t="inlineStr"/>
+      <c r="E17" s="140" t="inlineStr"/>
       <c r="F17" s="112" t="inlineStr">
         <is>
           <t>Class 2 (8/26) - Role of Managerial accounting: Chapter 1</t>
@@ -2626,18 +2622,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B18" s="111" t="inlineStr"/>
-      <c r="C18" s="111" t="inlineStr">
+      <c r="B18" s="140" t="inlineStr"/>
+      <c r="C18" s="140" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D18" s="111" t="inlineStr">
+      <c r="D18" s="140" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="E18" s="111" t="inlineStr"/>
+      <c r="E18" s="140" t="inlineStr"/>
       <c r="F18" s="112" t="inlineStr">
         <is>
           <t>Class 3 (8/31) - Basic Cost Mgt Concepts: Chapter 2</t>
@@ -2650,18 +2646,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B19" s="111" t="inlineStr"/>
-      <c r="C19" s="111" t="inlineStr">
+      <c r="B19" s="140" t="inlineStr"/>
+      <c r="C19" s="140" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="D19" s="111" t="inlineStr">
+      <c r="D19" s="140" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="E19" s="111" t="inlineStr"/>
+      <c r="E19" s="140" t="inlineStr"/>
       <c r="F19" s="112" t="inlineStr">
         <is>
           <t>Class 4 (9/2) - Basic Cost Mgt Concepts: Chapter 2</t>
@@ -2674,18 +2670,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B20" s="111" t="inlineStr"/>
-      <c r="C20" s="111" t="inlineStr">
+      <c r="B20" s="140" t="inlineStr"/>
+      <c r="C20" s="140" t="inlineStr">
         <is>
           <t>2026-09-07</t>
         </is>
       </c>
-      <c r="D20" s="111" t="inlineStr">
+      <c r="D20" s="140" t="inlineStr">
         <is>
           <t>2026-09-07</t>
         </is>
       </c>
-      <c r="E20" s="111" t="inlineStr"/>
+      <c r="E20" s="140" t="inlineStr"/>
       <c r="F20" s="112" t="inlineStr">
         <is>
           <t>9/7 - No Class Labor Day Holiday</t>
@@ -2698,18 +2694,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B21" s="111" t="inlineStr"/>
-      <c r="C21" s="111" t="inlineStr">
+      <c r="B21" s="140" t="inlineStr"/>
+      <c r="C21" s="140" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="D21" s="111" t="inlineStr">
+      <c r="D21" s="140" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="E21" s="111" t="inlineStr"/>
+      <c r="E21" s="140" t="inlineStr"/>
       <c r="F21" s="112" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - Product Cost Accumulation: Job; Order Co: Chapter 3</t>
@@ -2722,18 +2718,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B22" s="111" t="inlineStr"/>
-      <c r="C22" s="111" t="inlineStr">
+      <c r="B22" s="140" t="inlineStr"/>
+      <c r="C22" s="140" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="D22" s="111" t="inlineStr">
+      <c r="D22" s="140" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="E22" s="111" t="inlineStr"/>
+      <c r="E22" s="140" t="inlineStr"/>
       <c r="F22" s="112" t="inlineStr">
         <is>
           <t>Class 6 (9/14) - Manufacturing Overhead Normal; Costing: Chapter 3</t>
@@ -2746,18 +2742,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B23" s="111" t="inlineStr"/>
-      <c r="C23" s="111" t="inlineStr">
+      <c r="B23" s="140" t="inlineStr"/>
+      <c r="C23" s="140" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="D23" s="111" t="inlineStr">
+      <c r="D23" s="140" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E23" s="111" t="inlineStr"/>
+      <c r="E23" s="140" t="inlineStr"/>
       <c r="F23" s="112" t="inlineStr">
         <is>
           <t>Class 7 (9/16) - Activity Based Costing: Chapter 5- ONLY; LO 5.1, 2, 4 &amp; 5</t>
@@ -2770,18 +2766,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B24" s="111" t="inlineStr"/>
-      <c r="C24" s="111" t="inlineStr">
+      <c r="B24" s="140" t="inlineStr"/>
+      <c r="C24" s="140" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="D24" s="111" t="inlineStr">
+      <c r="D24" s="140" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="E24" s="111" t="inlineStr"/>
+      <c r="E24" s="140" t="inlineStr"/>
       <c r="F24" s="112" t="inlineStr">
         <is>
           <t>Class 8 (9/21) - Product Cost Accumulation: Pro-; cess Co: Chapter 4- ONLY; LO 4.1, 3, 4, &amp; 5</t>
@@ -2794,18 +2790,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B25" s="111" t="inlineStr"/>
-      <c r="C25" s="111" t="inlineStr">
+      <c r="B25" s="140" t="inlineStr"/>
+      <c r="C25" s="140" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D25" s="111" t="inlineStr">
+      <c r="D25" s="140" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="E25" s="111" t="inlineStr"/>
+      <c r="E25" s="140" t="inlineStr"/>
       <c r="F25" s="112" t="inlineStr">
         <is>
           <t>Class 9 (9/23) - Cost of Quality &amp; ESG &amp;; Overview of; • : Chapter 8 - ONLY; LO 8.7, 8, 9</t>
@@ -2818,18 +2814,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B26" s="111" t="inlineStr"/>
-      <c r="C26" s="111" t="inlineStr">
+      <c r="B26" s="140" t="inlineStr"/>
+      <c r="C26" s="140" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="D26" s="111" t="inlineStr">
+      <c r="D26" s="140" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="E26" s="111" t="inlineStr"/>
+      <c r="E26" s="140" t="inlineStr"/>
       <c r="F26" s="112" t="inlineStr">
         <is>
           <t>Class 11 (10/5) - Cost Estimation: Chapter 6</t>
@@ -2842,18 +2838,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B27" s="111" t="inlineStr"/>
-      <c r="C27" s="111" t="inlineStr">
+      <c r="B27" s="140" t="inlineStr"/>
+      <c r="C27" s="140" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="D27" s="111" t="inlineStr">
+      <c r="D27" s="140" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="E27" s="111" t="inlineStr"/>
+      <c r="E27" s="140" t="inlineStr"/>
       <c r="F27" s="112" t="inlineStr">
         <is>
           <t>Class 12 (10/7) - Cost volume profit analysis: Chapter 7</t>
@@ -2866,18 +2862,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B28" s="111" t="inlineStr"/>
-      <c r="C28" s="111" t="inlineStr">
+      <c r="B28" s="140" t="inlineStr"/>
+      <c r="C28" s="140" t="inlineStr">
         <is>
           <t>2026-10-12</t>
         </is>
       </c>
-      <c r="D28" s="111" t="inlineStr">
+      <c r="D28" s="140" t="inlineStr">
         <is>
           <t>2026-10-12</t>
         </is>
       </c>
-      <c r="E28" s="111" t="inlineStr"/>
+      <c r="E28" s="140" t="inlineStr"/>
       <c r="F28" s="112" t="inlineStr">
         <is>
           <t>Class 13 (10/12) - Cost volume profit analysis &amp;: Chapter 7</t>
@@ -2890,18 +2886,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B29" s="111" t="inlineStr"/>
-      <c r="C29" s="111" t="inlineStr">
+      <c r="B29" s="140" t="inlineStr"/>
+      <c r="C29" s="140" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="D29" s="111" t="inlineStr">
+      <c r="D29" s="140" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E29" s="111" t="inlineStr"/>
+      <c r="E29" s="140" t="inlineStr"/>
       <c r="F29" s="112" t="inlineStr">
         <is>
           <t>Class 14 (10/14) - Financial planning and analysis:; Static: Chapter 9</t>
@@ -2914,18 +2910,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B30" s="111" t="inlineStr"/>
-      <c r="C30" s="111" t="inlineStr">
+      <c r="B30" s="140" t="inlineStr"/>
+      <c r="C30" s="140" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="D30" s="111" t="inlineStr">
+      <c r="D30" s="140" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E30" s="111" t="inlineStr"/>
+      <c r="E30" s="140" t="inlineStr"/>
       <c r="F30" s="112" t="inlineStr">
         <is>
           <t>Class 15 (10/19) - Capital Budgeting; Practice Midterm Ques: Chapter 16- ONLY; LO 16.1, 2, 3</t>
@@ -2938,18 +2934,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B31" s="111" t="inlineStr"/>
-      <c r="C31" s="111" t="inlineStr">
+      <c r="B31" s="140" t="inlineStr"/>
+      <c r="C31" s="140" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
       </c>
-      <c r="D31" s="111" t="inlineStr">
+      <c r="D31" s="140" t="inlineStr">
         <is>
           <t>2026-10-28</t>
         </is>
       </c>
-      <c r="E31" s="111" t="inlineStr"/>
+      <c r="E31" s="140" t="inlineStr"/>
       <c r="F31" s="112" t="inlineStr">
         <is>
           <t>Class 17 (10/28) - Guest Speaker</t>
@@ -2962,18 +2958,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B32" s="111" t="inlineStr"/>
-      <c r="C32" s="111" t="inlineStr">
+      <c r="B32" s="140" t="inlineStr"/>
+      <c r="C32" s="140" t="inlineStr">
         <is>
           <t>2026-11-02</t>
         </is>
       </c>
-      <c r="D32" s="111" t="inlineStr">
+      <c r="D32" s="140" t="inlineStr">
         <is>
           <t>2026-11-02</t>
         </is>
       </c>
-      <c r="E32" s="111" t="inlineStr"/>
+      <c r="E32" s="140" t="inlineStr"/>
       <c r="F32" s="112" t="inlineStr">
         <is>
           <t>Class 19 (11/2) - Standard Costing &amp; Direct Cost; Variance: Chapter 10 – ONLY; LO 10.1 thru 8</t>
@@ -2986,18 +2982,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B33" s="111" t="inlineStr"/>
-      <c r="C33" s="111" t="inlineStr">
+      <c r="B33" s="140" t="inlineStr"/>
+      <c r="C33" s="140" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="D33" s="111" t="inlineStr">
+      <c r="D33" s="140" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="E33" s="111" t="inlineStr"/>
+      <c r="E33" s="140" t="inlineStr"/>
       <c r="F33" s="112" t="inlineStr">
         <is>
           <t>Class 19 (11/4) - Sales Variance Analysis; Flexible Budget: Chapter 11 - ONLY; LO 11.1, 11.2 &amp;; Appendix B</t>
@@ -3010,18 +3006,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B34" s="111" t="inlineStr"/>
-      <c r="C34" s="111" t="inlineStr">
+      <c r="B34" s="140" t="inlineStr"/>
+      <c r="C34" s="140" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="D34" s="111" t="inlineStr">
+      <c r="D34" s="140" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E34" s="111" t="inlineStr"/>
+      <c r="E34" s="140" t="inlineStr"/>
       <c r="F34" s="112" t="inlineStr">
         <is>
           <t>Class 20 (11/9) - Investment Centers: Chapter 13- ONLY; LO 13-1, 2, 3, 4</t>
@@ -3034,18 +3030,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B35" s="111" t="inlineStr"/>
-      <c r="C35" s="111" t="inlineStr">
+      <c r="B35" s="140" t="inlineStr"/>
+      <c r="C35" s="140" t="inlineStr">
         <is>
           <t>2026-11-11</t>
         </is>
       </c>
-      <c r="D35" s="111" t="inlineStr">
+      <c r="D35" s="140" t="inlineStr">
         <is>
           <t>2026-11-11</t>
         </is>
       </c>
-      <c r="E35" s="111" t="inlineStr"/>
+      <c r="E35" s="140" t="inlineStr"/>
       <c r="F35" s="112" t="inlineStr">
         <is>
           <t>11/11 - No Class Veterans Day</t>
@@ -3058,18 +3054,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B36" s="111" t="inlineStr"/>
-      <c r="C36" s="111" t="inlineStr">
+      <c r="B36" s="140" t="inlineStr"/>
+      <c r="C36" s="140" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="D36" s="111" t="inlineStr">
+      <c r="D36" s="140" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E36" s="111" t="inlineStr"/>
+      <c r="E36" s="140" t="inlineStr"/>
       <c r="F36" s="112" t="inlineStr">
         <is>
           <t>Class 22 (11/18) - Decision-making: relevant costs; and ben: Chapter 14; (Part 1 of 3)</t>
@@ -3082,18 +3078,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B37" s="111" t="inlineStr"/>
-      <c r="C37" s="111" t="inlineStr">
+      <c r="B37" s="140" t="inlineStr"/>
+      <c r="C37" s="140" t="inlineStr">
         <is>
           <t>2026-11-23</t>
         </is>
       </c>
-      <c r="D37" s="111" t="inlineStr">
+      <c r="D37" s="140" t="inlineStr">
         <is>
           <t>2026-11-23</t>
         </is>
       </c>
-      <c r="E37" s="111" t="inlineStr"/>
+      <c r="E37" s="140" t="inlineStr"/>
       <c r="F37" s="112" t="inlineStr">
         <is>
           <t>Class 23 (11/23) - Decision-making: relevant costs; and ben: Chapter 14; (Part 2 of 3)</t>
@@ -3106,18 +3102,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B38" s="111" t="inlineStr"/>
-      <c r="C38" s="111" t="inlineStr">
+      <c r="B38" s="140" t="inlineStr"/>
+      <c r="C38" s="140" t="inlineStr">
         <is>
           <t>2026-11-25</t>
         </is>
       </c>
-      <c r="D38" s="111" t="inlineStr">
+      <c r="D38" s="140" t="inlineStr">
         <is>
           <t>2026-11-25</t>
         </is>
       </c>
-      <c r="E38" s="111" t="inlineStr"/>
+      <c r="E38" s="140" t="inlineStr"/>
       <c r="F38" s="112" t="inlineStr">
         <is>
           <t>11/25 - No Class Thanksgiving Holiday</t>
@@ -3130,18 +3126,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B39" s="111" t="inlineStr"/>
-      <c r="C39" s="111" t="inlineStr">
+      <c r="B39" s="140" t="inlineStr"/>
+      <c r="C39" s="140" t="inlineStr">
         <is>
           <t>2026-11-30</t>
         </is>
       </c>
-      <c r="D39" s="111" t="inlineStr">
+      <c r="D39" s="140" t="inlineStr">
         <is>
           <t>2026-11-30</t>
         </is>
       </c>
-      <c r="E39" s="111" t="inlineStr"/>
+      <c r="E39" s="140" t="inlineStr"/>
       <c r="F39" s="112" t="inlineStr">
         <is>
           <t>Class 24 (11/30) - Decision-making: relevant costs; and ben: Chapter 14; (Part 3 of 3)</t>
@@ -3154,18 +3150,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B40" s="111" t="inlineStr"/>
-      <c r="C40" s="111" t="inlineStr">
+      <c r="B40" s="140" t="inlineStr"/>
+      <c r="C40" s="140" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="D40" s="111" t="inlineStr">
+      <c r="D40" s="140" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E40" s="111" t="inlineStr"/>
+      <c r="E40" s="140" t="inlineStr"/>
       <c r="F40" s="112" t="inlineStr">
         <is>
           <t>Class 2 (12/2) - Catchup &amp; Final Review; Practice Final Questions Posted to Brightspace at; 5:00 PM</t>
@@ -3178,18 +3174,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B41" s="111" t="inlineStr"/>
-      <c r="C41" s="111" t="inlineStr">
+      <c r="B41" s="140" t="inlineStr"/>
+      <c r="C41" s="140" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="D41" s="111" t="inlineStr">
+      <c r="D41" s="140" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="E41" s="111" t="inlineStr"/>
+      <c r="E41" s="140" t="inlineStr"/>
       <c r="F41" s="112" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
@@ -3202,18 +3198,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B42" s="111" t="inlineStr"/>
-      <c r="C42" s="111" t="inlineStr">
+      <c r="B42" s="140" t="inlineStr"/>
+      <c r="C42" s="140" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="D42" s="111" t="inlineStr">
+      <c r="D42" s="140" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E42" s="111" t="inlineStr"/>
+      <c r="E42" s="140" t="inlineStr"/>
       <c r="F42" s="112" t="inlineStr">
         <is>
           <t>Class 7 (9/16) - 3-24, 3-28, 3-32; 15 Points</t>
@@ -3226,18 +3222,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B43" s="111" t="inlineStr"/>
-      <c r="C43" s="111" t="inlineStr">
+      <c r="B43" s="140" t="inlineStr"/>
+      <c r="C43" s="140" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="D43" s="111" t="inlineStr">
+      <c r="D43" s="140" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="E43" s="111" t="inlineStr"/>
+      <c r="E43" s="140" t="inlineStr"/>
       <c r="F43" s="112" t="inlineStr">
         <is>
           <t>Class 8 (9/21) - 5-27 5-46; 10 Points</t>
@@ -3250,18 +3246,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B44" s="111" t="inlineStr"/>
-      <c r="C44" s="111" t="inlineStr">
+      <c r="B44" s="140" t="inlineStr"/>
+      <c r="C44" s="140" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D44" s="111" t="inlineStr">
+      <c r="D44" s="140" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="E44" s="111" t="inlineStr"/>
+      <c r="E44" s="140" t="inlineStr"/>
       <c r="F44" s="112" t="inlineStr">
         <is>
           <t>Class 9 (9/23) - 4-21, 4-22; 10 Points</t>
@@ -3274,18 +3270,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B45" s="111" t="inlineStr"/>
-      <c r="C45" s="111" t="inlineStr">
+      <c r="B45" s="140" t="inlineStr"/>
+      <c r="C45" s="140" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="D45" s="111" t="inlineStr">
+      <c r="D45" s="140" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E45" s="111" t="inlineStr"/>
+      <c r="E45" s="140" t="inlineStr"/>
       <c r="F45" s="112" t="inlineStr">
         <is>
           <t>Class 10 (9/28) - 8-28, 8-29; 10 Points</t>
@@ -3298,18 +3294,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B46" s="111" t="inlineStr"/>
-      <c r="C46" s="111" t="inlineStr">
+      <c r="B46" s="140" t="inlineStr"/>
+      <c r="C46" s="140" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="D46" s="111" t="inlineStr">
+      <c r="D46" s="140" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="E46" s="111" t="inlineStr"/>
+      <c r="E46" s="140" t="inlineStr"/>
       <c r="F46" s="112" t="inlineStr">
         <is>
           <t>Class 12 (10/7) - 6-24, 6-25, 6-34; 15 Points</t>
@@ -3322,18 +3318,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B47" s="111" t="inlineStr"/>
-      <c r="C47" s="111" t="inlineStr">
+      <c r="B47" s="140" t="inlineStr"/>
+      <c r="C47" s="140" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="D47" s="111" t="inlineStr">
+      <c r="D47" s="140" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E47" s="111" t="inlineStr"/>
+      <c r="E47" s="140" t="inlineStr"/>
       <c r="F47" s="112" t="inlineStr">
         <is>
           <t>Class 14 (10/14) - 7-29, 7-33, 7-40; 15 Points</t>
@@ -3346,18 +3342,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B48" s="111" t="inlineStr"/>
-      <c r="C48" s="111" t="inlineStr">
+      <c r="B48" s="140" t="inlineStr"/>
+      <c r="C48" s="140" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="D48" s="111" t="inlineStr">
+      <c r="D48" s="140" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E48" s="111" t="inlineStr"/>
+      <c r="E48" s="140" t="inlineStr"/>
       <c r="F48" s="112" t="inlineStr">
         <is>
           <t>Class 15 (10/19) - 9-25, 9-28, 9-37; 15 - Points</t>
@@ -3370,18 +3366,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B49" s="111" t="inlineStr"/>
-      <c r="C49" s="111" t="inlineStr">
+      <c r="B49" s="140" t="inlineStr"/>
+      <c r="C49" s="140" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="D49" s="111" t="inlineStr">
+      <c r="D49" s="140" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E49" s="111" t="inlineStr"/>
+      <c r="E49" s="140" t="inlineStr"/>
       <c r="F49" s="112" t="inlineStr">
         <is>
           <t>Class 16 (10/21) - 16-28, 16-40; 10 Points</t>
@@ -3394,18 +3390,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B50" s="111" t="inlineStr"/>
-      <c r="C50" s="111" t="inlineStr">
+      <c r="B50" s="140" t="inlineStr"/>
+      <c r="C50" s="140" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="D50" s="111" t="inlineStr">
+      <c r="D50" s="140" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="E50" s="111" t="inlineStr"/>
+      <c r="E50" s="140" t="inlineStr"/>
       <c r="F50" s="112" t="inlineStr">
         <is>
           <t>Class 19 (11/4) - 10-26, 10-30; 10 Points</t>
@@ -3418,18 +3414,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B51" s="111" t="inlineStr"/>
-      <c r="C51" s="111" t="inlineStr">
+      <c r="B51" s="140" t="inlineStr"/>
+      <c r="C51" s="140" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="D51" s="111" t="inlineStr">
+      <c r="D51" s="140" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E51" s="111" t="inlineStr"/>
+      <c r="E51" s="140" t="inlineStr"/>
       <c r="F51" s="112" t="inlineStr">
         <is>
           <t>Class 20 (11/9) - 11-31, 11-52; 10 Points</t>
@@ -3442,18 +3438,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B52" s="111" t="inlineStr"/>
-      <c r="C52" s="111" t="inlineStr">
+      <c r="B52" s="140" t="inlineStr"/>
+      <c r="C52" s="140" t="inlineStr">
         <is>
           <t>2026-11-16</t>
         </is>
       </c>
-      <c r="D52" s="111" t="inlineStr">
+      <c r="D52" s="140" t="inlineStr">
         <is>
           <t>2026-11-16</t>
         </is>
       </c>
-      <c r="E52" s="111" t="inlineStr"/>
+      <c r="E52" s="140" t="inlineStr"/>
       <c r="F52" s="112" t="inlineStr">
         <is>
           <t>Class 21 (11/16) - 13-29, 13-33; 10 Points</t>
@@ -3466,22 +3462,22 @@
           <t>LinkedIn Learning Excel Certification</t>
         </is>
       </c>
-      <c r="B53" s="107" t="inlineStr">
+      <c r="B53" s="138" t="inlineStr">
         <is>
           <t>75 pts</t>
         </is>
       </c>
-      <c r="C53" s="108" t="inlineStr">
+      <c r="C53" s="139" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D53" s="108" t="inlineStr">
+      <c r="D53" s="139" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E53" s="108" t="inlineStr">
+      <c r="E53" s="139" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3497,18 +3493,18 @@
           <t>Certification</t>
         </is>
       </c>
-      <c r="B54" s="111" t="inlineStr"/>
-      <c r="C54" s="111" t="inlineStr">
+      <c r="B54" s="140" t="inlineStr"/>
+      <c r="C54" s="140" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D54" s="111" t="inlineStr">
+      <c r="D54" s="140" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E54" s="111" t="inlineStr"/>
+      <c r="E54" s="140" t="inlineStr"/>
       <c r="F54" s="112" t="inlineStr">
         <is>
           <t>LinkedIn Learning Excel Certification</t>
@@ -3521,22 +3517,22 @@
           <t>Stukent Simternship</t>
         </is>
       </c>
-      <c r="B55" s="107" t="inlineStr">
+      <c r="B55" s="138" t="inlineStr">
         <is>
           <t>75 pts</t>
         </is>
       </c>
-      <c r="C55" s="114" t="inlineStr">
+      <c r="C55" s="141" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D55" s="114" t="inlineStr">
+      <c r="D55" s="141" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E55" s="114" t="inlineStr">
+      <c r="E55" s="141" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3552,18 +3548,18 @@
           <t>Certification</t>
         </is>
       </c>
-      <c r="B56" s="111" t="inlineStr"/>
-      <c r="C56" s="111" t="inlineStr">
+      <c r="B56" s="140" t="inlineStr"/>
+      <c r="C56" s="140" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D56" s="111" t="inlineStr">
+      <c r="D56" s="140" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E56" s="111" t="inlineStr"/>
+      <c r="E56" s="140" t="inlineStr"/>
       <c r="F56" s="112" t="inlineStr">
         <is>
           <t>Stukent Simternship</t>
@@ -3709,22 +3705,22 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B9" s="121" t="inlineStr">
+      <c r="B9" s="142" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="C9" s="122" t="inlineStr">
+      <c r="C9" s="143" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D9" s="122" t="inlineStr">
+      <c r="D9" s="143" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E9" s="122" t="inlineStr">
+      <c r="E9" s="143" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3740,18 +3736,18 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B10" s="125" t="inlineStr"/>
-      <c r="C10" s="125" t="inlineStr">
+      <c r="B10" s="144" t="inlineStr"/>
+      <c r="C10" s="144" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D10" s="125" t="inlineStr">
+      <c r="D10" s="144" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E10" s="125" t="inlineStr"/>
+      <c r="E10" s="144" t="inlineStr"/>
       <c r="F10" s="126" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -3764,22 +3760,22 @@
           <t>Participation</t>
         </is>
       </c>
-      <c r="B11" s="121" t="inlineStr">
+      <c r="B11" s="142" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C11" s="128" t="inlineStr">
+      <c r="C11" s="145" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D11" s="128" t="inlineStr">
+      <c r="D11" s="145" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E11" s="128" t="inlineStr">
+      <c r="E11" s="145" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3795,21 +3791,17 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B12" s="125" t="inlineStr"/>
-      <c r="C12" s="125" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D12" s="125" t="inlineStr">
-        <is>
-          <t>2026-12-20</t>
-        </is>
-      </c>
-      <c r="E12" s="125" t="inlineStr"/>
+      <c r="B12" s="144" t="inlineStr"/>
+      <c r="C12" s="144" t="inlineStr"/>
+      <c r="D12" s="144" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="E12" s="144" t="inlineStr"/>
       <c r="F12" s="126" t="inlineStr">
         <is>
-          <t>Connect: Self-Assessment 11.01 - What is my</t>
+          <t>Connect: Sharpen Companion</t>
         </is>
       </c>
     </row>
@@ -3819,21 +3811,21 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B13" s="125" t="inlineStr"/>
-      <c r="C13" s="125" t="inlineStr">
+      <c r="B13" s="144" t="inlineStr"/>
+      <c r="C13" s="144" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D13" s="125" t="inlineStr">
+      <c r="D13" s="144" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E13" s="125" t="inlineStr"/>
+      <c r="E13" s="144" t="inlineStr"/>
       <c r="F13" s="126" t="inlineStr">
         <is>
-          <t>Connect: Self-Assessment 11.02 - What is my</t>
+          <t>Connect: Self-Assessment 11.01 - What is my</t>
         </is>
       </c>
     </row>
@@ -3843,21 +3835,21 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B14" s="125" t="inlineStr"/>
-      <c r="C14" s="125" t="inlineStr">
+      <c r="B14" s="144" t="inlineStr"/>
+      <c r="C14" s="144" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D14" s="125" t="inlineStr">
+      <c r="D14" s="144" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E14" s="125" t="inlineStr"/>
+      <c r="E14" s="144" t="inlineStr"/>
       <c r="F14" s="126" t="inlineStr">
         <is>
-          <t>Connect: Self-Assessment 12.02 - Which influence</t>
+          <t>Connect: Self-Assessment 11.02 - What is my</t>
         </is>
       </c>
     </row>
@@ -3867,21 +3859,21 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B15" s="125" t="inlineStr"/>
-      <c r="C15" s="125" t="inlineStr">
+      <c r="B15" s="144" t="inlineStr"/>
+      <c r="C15" s="144" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D15" s="125" t="inlineStr">
+      <c r="D15" s="144" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E15" s="125" t="inlineStr"/>
+      <c r="E15" s="144" t="inlineStr"/>
       <c r="F15" s="126" t="inlineStr">
         <is>
-          <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
+          <t>Connect: Self-Assessment 12.02 - Which influence</t>
         </is>
       </c>
     </row>
@@ -3891,21 +3883,21 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B16" s="125" t="inlineStr"/>
-      <c r="C16" s="125" t="inlineStr">
+      <c r="B16" s="144" t="inlineStr"/>
+      <c r="C16" s="144" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D16" s="125" t="inlineStr">
+      <c r="D16" s="144" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E16" s="125" t="inlineStr"/>
+      <c r="E16" s="144" t="inlineStr"/>
       <c r="F16" s="126" t="inlineStr">
         <is>
-          <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
+          <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
         </is>
       </c>
     </row>
@@ -3915,21 +3907,21 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B17" s="125" t="inlineStr"/>
-      <c r="C17" s="125" t="inlineStr">
+      <c r="B17" s="144" t="inlineStr"/>
+      <c r="C17" s="144" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D17" s="125" t="inlineStr">
+      <c r="D17" s="144" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E17" s="125" t="inlineStr"/>
+      <c r="E17" s="144" t="inlineStr"/>
       <c r="F17" s="126" t="inlineStr">
         <is>
-          <t>Connect: Self-Assessment 5.01 - Assessing Your</t>
+          <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
         </is>
       </c>
     </row>
@@ -3939,21 +3931,21 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B18" s="125" t="inlineStr"/>
-      <c r="C18" s="125" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D18" s="125" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="E18" s="125" t="inlineStr"/>
+      <c r="B18" s="144" t="inlineStr"/>
+      <c r="C18" s="144" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D18" s="144" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E18" s="144" t="inlineStr"/>
       <c r="F18" s="126" t="inlineStr">
         <is>
-          <t>Connect: Sharpen Companion</t>
+          <t>Connect: Self-Assessment 5.01 - Assessing Your</t>
         </is>
       </c>
     </row>
@@ -3963,14 +3955,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B19" s="125" t="inlineStr"/>
-      <c r="C19" s="125" t="inlineStr"/>
-      <c r="D19" s="125" t="inlineStr">
+      <c r="B19" s="144" t="inlineStr"/>
+      <c r="C19" s="144" t="inlineStr"/>
+      <c r="D19" s="144" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="E19" s="125" t="inlineStr"/>
+      <c r="E19" s="144" t="inlineStr"/>
       <c r="F19" s="126" t="inlineStr">
         <is>
           <t>Research: Setup deadline (registration, prescreening, contacts)</t>
@@ -3983,14 +3975,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B20" s="125" t="inlineStr"/>
-      <c r="C20" s="125" t="inlineStr"/>
-      <c r="D20" s="125" t="inlineStr">
+      <c r="B20" s="144" t="inlineStr"/>
+      <c r="C20" s="144" t="inlineStr"/>
+      <c r="D20" s="144" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E20" s="125" t="inlineStr"/>
+      <c r="E20" s="144" t="inlineStr"/>
       <c r="F20" s="126" t="inlineStr">
         <is>
           <t>Research: Employee contact surveys sent</t>
@@ -4003,14 +3995,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B21" s="125" t="inlineStr"/>
-      <c r="C21" s="125" t="inlineStr"/>
-      <c r="D21" s="125" t="inlineStr">
+      <c r="B21" s="144" t="inlineStr"/>
+      <c r="C21" s="144" t="inlineStr"/>
+      <c r="D21" s="144" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E21" s="125" t="inlineStr"/>
+      <c r="E21" s="144" t="inlineStr"/>
       <c r="F21" s="126" t="inlineStr">
         <is>
           <t>Research: Complete 2.0 research credits</t>
@@ -4023,14 +4015,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B22" s="125" t="inlineStr"/>
-      <c r="C22" s="125" t="inlineStr">
+      <c r="B22" s="144" t="inlineStr"/>
+      <c r="C22" s="144" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D22" s="125" t="inlineStr"/>
-      <c r="E22" s="125" t="inlineStr"/>
+      <c r="D22" s="144" t="inlineStr"/>
+      <c r="E22" s="144" t="inlineStr"/>
       <c r="F22" s="126" t="inlineStr">
         <is>
           <t>Research: SONA registration opens</t>
@@ -4043,14 +4035,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B23" s="125" t="inlineStr"/>
-      <c r="C23" s="125" t="inlineStr">
+      <c r="B23" s="144" t="inlineStr"/>
+      <c r="C23" s="144" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="D23" s="125" t="inlineStr"/>
-      <c r="E23" s="125" t="inlineStr"/>
+      <c r="D23" s="144" t="inlineStr"/>
+      <c r="E23" s="144" t="inlineStr"/>
       <c r="F23" s="126" t="inlineStr">
         <is>
           <t>Research: Prescreening questionnaire opens</t>
@@ -4063,14 +4055,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B24" s="125" t="inlineStr"/>
-      <c r="C24" s="125" t="inlineStr">
+      <c r="B24" s="144" t="inlineStr"/>
+      <c r="C24" s="144" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="D24" s="125" t="inlineStr"/>
-      <c r="E24" s="125" t="inlineStr"/>
+      <c r="D24" s="144" t="inlineStr"/>
+      <c r="E24" s="144" t="inlineStr"/>
       <c r="F24" s="126" t="inlineStr">
         <is>
           <t>Research: Study invitations begin (after setup)</t>
@@ -4083,22 +4075,22 @@
           <t>Midterm Exam</t>
         </is>
       </c>
-      <c r="B25" s="121" t="inlineStr">
+      <c r="B25" s="142" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C25" s="122" t="inlineStr">
+      <c r="C25" s="143" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D25" s="122" t="inlineStr">
+      <c r="D25" s="143" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E25" s="122" t="inlineStr">
+      <c r="E25" s="143" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4114,18 +4106,18 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B26" s="125" t="inlineStr"/>
-      <c r="C26" s="125" t="inlineStr">
+      <c r="B26" s="144" t="inlineStr"/>
+      <c r="C26" s="144" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D26" s="125" t="inlineStr">
+      <c r="D26" s="144" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E26" s="125" t="inlineStr"/>
+      <c r="E26" s="144" t="inlineStr"/>
       <c r="F26" s="126" t="inlineStr">
         <is>
           <t>Midterm Exam</t>
@@ -4138,22 +4130,22 @@
           <t>Team Project Paper</t>
         </is>
       </c>
-      <c r="B27" s="121" t="inlineStr">
+      <c r="B27" s="142" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C27" s="128" t="inlineStr">
+      <c r="C27" s="145" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D27" s="128" t="inlineStr">
+      <c r="D27" s="145" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E27" s="128" t="inlineStr">
+      <c r="E27" s="145" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4169,18 +4161,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B28" s="125" t="inlineStr"/>
-      <c r="C28" s="125" t="inlineStr">
+      <c r="B28" s="144" t="inlineStr"/>
+      <c r="C28" s="144" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D28" s="125" t="inlineStr">
+      <c r="D28" s="144" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E28" s="125" t="inlineStr"/>
+      <c r="E28" s="144" t="inlineStr"/>
       <c r="F28" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 14.02 - What Type of Organizational Culture Do I</t>
@@ -4193,18 +4185,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B29" s="125" t="inlineStr"/>
-      <c r="C29" s="125" t="inlineStr">
+      <c r="B29" s="144" t="inlineStr"/>
+      <c r="C29" s="144" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D29" s="125" t="inlineStr">
+      <c r="D29" s="144" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E29" s="125" t="inlineStr"/>
+      <c r="E29" s="144" t="inlineStr"/>
       <c r="F29" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 8.01 - Group</t>
@@ -4217,18 +4209,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B30" s="125" t="inlineStr"/>
-      <c r="C30" s="125" t="inlineStr">
+      <c r="B30" s="144" t="inlineStr"/>
+      <c r="C30" s="144" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D30" s="125" t="inlineStr">
+      <c r="D30" s="144" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E30" s="125" t="inlineStr"/>
+      <c r="E30" s="144" t="inlineStr"/>
       <c r="F30" s="126" t="inlineStr">
         <is>
           <t>Team project outline</t>
@@ -4241,18 +4233,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B31" s="125" t="inlineStr"/>
-      <c r="C31" s="125" t="inlineStr">
+      <c r="B31" s="144" t="inlineStr"/>
+      <c r="C31" s="144" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D31" s="125" t="inlineStr">
+      <c r="D31" s="144" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E31" s="125" t="inlineStr"/>
+      <c r="E31" s="144" t="inlineStr"/>
       <c r="F31" s="126" t="inlineStr">
         <is>
           <t>Team project paper</t>
@@ -4265,22 +4257,22 @@
           <t>Final Reflection Paper</t>
         </is>
       </c>
-      <c r="B32" s="121" t="inlineStr">
+      <c r="B32" s="142" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C32" s="122" t="inlineStr">
+      <c r="C32" s="143" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D32" s="122" t="inlineStr">
+      <c r="D32" s="143" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E32" s="122" t="inlineStr">
+      <c r="E32" s="143" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4296,18 +4288,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B33" s="125" t="inlineStr"/>
-      <c r="C33" s="125" t="inlineStr">
+      <c r="B33" s="144" t="inlineStr"/>
+      <c r="C33" s="144" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D33" s="125" t="inlineStr">
+      <c r="D33" s="144" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E33" s="125" t="inlineStr"/>
+      <c r="E33" s="144" t="inlineStr"/>
       <c r="F33" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 16.02 - What Is Your</t>
@@ -4320,18 +4312,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B34" s="125" t="inlineStr"/>
-      <c r="C34" s="125" t="inlineStr">
+      <c r="B34" s="144" t="inlineStr"/>
+      <c r="C34" s="144" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D34" s="125" t="inlineStr">
+      <c r="D34" s="144" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E34" s="125" t="inlineStr"/>
+      <c r="E34" s="144" t="inlineStr"/>
       <c r="F34" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 16.03 - Assessing Your</t>
@@ -4344,18 +4336,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B35" s="125" t="inlineStr"/>
-      <c r="C35" s="125" t="inlineStr">
+      <c r="B35" s="144" t="inlineStr"/>
+      <c r="C35" s="144" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D35" s="125" t="inlineStr">
+      <c r="D35" s="144" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E35" s="125" t="inlineStr"/>
+      <c r="E35" s="144" t="inlineStr"/>
       <c r="F35" s="126" t="inlineStr">
         <is>
           <t>Personal Reflection Paper</t>
@@ -4368,22 +4360,22 @@
           <t>Presentation</t>
         </is>
       </c>
-      <c r="B36" s="121" t="inlineStr">
+      <c r="B36" s="142" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C36" s="128" t="inlineStr">
+      <c r="C36" s="145" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D36" s="128" t="inlineStr">
+      <c r="D36" s="145" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E36" s="128" t="inlineStr">
+      <c r="E36" s="145" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4399,18 +4391,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B37" s="125" t="inlineStr"/>
-      <c r="C37" s="125" t="inlineStr">
+      <c r="B37" s="144" t="inlineStr"/>
+      <c r="C37" s="144" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D37" s="125" t="inlineStr">
+      <c r="D37" s="144" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E37" s="125" t="inlineStr"/>
+      <c r="E37" s="144" t="inlineStr"/>
       <c r="F37" s="126" t="inlineStr">
         <is>
           <t>Presentation slides</t>
@@ -4423,22 +4415,22 @@
           <t>Case Analysis Assignments</t>
         </is>
       </c>
-      <c r="B38" s="121" t="inlineStr">
+      <c r="B38" s="142" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C38" s="122" t="inlineStr">
+      <c r="C38" s="143" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D38" s="122" t="inlineStr">
+      <c r="D38" s="143" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E38" s="122" t="inlineStr">
+      <c r="E38" s="143" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4454,18 +4446,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B39" s="125" t="inlineStr"/>
-      <c r="C39" s="125" t="inlineStr">
+      <c r="B39" s="144" t="inlineStr"/>
+      <c r="C39" s="144" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D39" s="125" t="inlineStr">
+      <c r="D39" s="144" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E39" s="125" t="inlineStr"/>
+      <c r="E39" s="144" t="inlineStr"/>
       <c r="F39" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 12.01 - What kind of</t>
@@ -4478,18 +4470,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B40" s="125" t="inlineStr"/>
-      <c r="C40" s="125" t="inlineStr">
+      <c r="B40" s="144" t="inlineStr"/>
+      <c r="C40" s="144" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D40" s="125" t="inlineStr">
+      <c r="D40" s="144" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E40" s="125" t="inlineStr"/>
+      <c r="E40" s="144" t="inlineStr"/>
       <c r="F40" s="126" t="inlineStr">
         <is>
           <t>Thomas Green Case Analysis Memo</t>
@@ -4502,18 +4494,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B41" s="125" t="inlineStr"/>
-      <c r="C41" s="125" t="inlineStr">
+      <c r="B41" s="144" t="inlineStr"/>
+      <c r="C41" s="144" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D41" s="125" t="inlineStr">
+      <c r="D41" s="144" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E41" s="125" t="inlineStr"/>
+      <c r="E41" s="144" t="inlineStr"/>
       <c r="F41" s="126" t="inlineStr">
         <is>
           <t>SkillsForTomorrow Analysis Memo</t>
@@ -4526,22 +4518,22 @@
           <t>Proposal &amp; Team Contract</t>
         </is>
       </c>
-      <c r="B42" s="121" t="inlineStr">
+      <c r="B42" s="142" t="inlineStr">
         <is>
           <t>3%</t>
         </is>
       </c>
-      <c r="C42" s="128" t="inlineStr">
+      <c r="C42" s="145" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D42" s="128" t="inlineStr">
+      <c r="D42" s="145" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E42" s="128" t="inlineStr">
+      <c r="E42" s="145" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4557,18 +4549,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B43" s="125" t="inlineStr"/>
-      <c r="C43" s="125" t="inlineStr">
+      <c r="B43" s="144" t="inlineStr"/>
+      <c r="C43" s="144" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D43" s="125" t="inlineStr">
+      <c r="D43" s="144" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E43" s="125" t="inlineStr"/>
+      <c r="E43" s="144" t="inlineStr"/>
       <c r="F43" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 10.5 - Preferred Conflict</t>
@@ -4581,18 +4573,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B44" s="125" t="inlineStr"/>
-      <c r="C44" s="125" t="inlineStr">
+      <c r="B44" s="144" t="inlineStr"/>
+      <c r="C44" s="144" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D44" s="125" t="inlineStr">
+      <c r="D44" s="144" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E44" s="125" t="inlineStr"/>
+      <c r="E44" s="144" t="inlineStr"/>
       <c r="F44" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 9.01 - Assessing My</t>
@@ -4605,18 +4597,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B45" s="125" t="inlineStr"/>
-      <c r="C45" s="125" t="inlineStr">
+      <c r="B45" s="144" t="inlineStr"/>
+      <c r="C45" s="144" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D45" s="125" t="inlineStr">
+      <c r="D45" s="144" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E45" s="125" t="inlineStr"/>
+      <c r="E45" s="144" t="inlineStr"/>
       <c r="F45" s="126" t="inlineStr">
         <is>
           <t>Team project proposal &amp; team contract</t>
@@ -4629,22 +4621,22 @@
           <t>Self &amp; Peer Evaluation</t>
         </is>
       </c>
-      <c r="B46" s="121" t="inlineStr">
+      <c r="B46" s="142" t="inlineStr">
         <is>
           <t>2%</t>
         </is>
       </c>
-      <c r="C46" s="122" t="inlineStr">
+      <c r="C46" s="143" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D46" s="122" t="inlineStr">
+      <c r="D46" s="143" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E46" s="122" t="inlineStr">
+      <c r="E46" s="143" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4660,18 +4652,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B47" s="125" t="inlineStr"/>
-      <c r="C47" s="125" t="inlineStr">
+      <c r="B47" s="144" t="inlineStr"/>
+      <c r="C47" s="144" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D47" s="125" t="inlineStr">
+      <c r="D47" s="144" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E47" s="125" t="inlineStr"/>
+      <c r="E47" s="144" t="inlineStr"/>
       <c r="F47" s="126" t="inlineStr">
         <is>
           <t>Self &amp; peer evaluation</t>

</xml_diff>

<commit_message>
BUAD-281: due-only calendar dates; Reading+Homework pairs chronological
- Calendar PDF has one class date (due by 8:00 am), no start date - Start Date blank
- Homework category: Reading+Homework pairs on graded problem-set dates only, earliest first
- Fix homework detection when cert footer shares the same table cell (Class 12/2)
- Document chronological pairing standard in skill docs
- Regenerated all three class sheets

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -251,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="161">
+  <cellXfs count="185">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -710,6 +710,78 @@
     </xf>
     <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -1206,18 +1278,18 @@
           <t>Sleep Paper</t>
         </is>
       </c>
-      <c r="B10" s="147" t="inlineStr">
+      <c r="B10" s="173" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C10" s="148" t="inlineStr"/>
-      <c r="D10" s="148" t="inlineStr">
+      <c r="C10" s="174" t="inlineStr"/>
+      <c r="D10" s="174" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="E10" s="148" t="inlineStr">
+      <c r="E10" s="174" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1233,14 +1305,14 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B11" s="149" t="inlineStr"/>
-      <c r="C11" s="149" t="inlineStr"/>
-      <c r="D11" s="149" t="inlineStr">
+      <c r="B11" s="175" t="inlineStr"/>
+      <c r="C11" s="175" t="inlineStr"/>
+      <c r="D11" s="175" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="E11" s="149" t="inlineStr"/>
+      <c r="E11" s="175" t="inlineStr"/>
       <c r="F11" s="99" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
@@ -1253,18 +1325,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B12" s="149" t="inlineStr"/>
-      <c r="C12" s="149" t="inlineStr">
+      <c r="B12" s="175" t="inlineStr"/>
+      <c r="C12" s="175" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D12" s="149" t="inlineStr">
+      <c r="D12" s="175" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E12" s="149" t="inlineStr"/>
+      <c r="E12" s="175" t="inlineStr"/>
       <c r="F12" s="99" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance</t>
@@ -1277,18 +1349,18 @@
           <t>Witchcraft Paper</t>
         </is>
       </c>
-      <c r="B13" s="147" t="inlineStr">
+      <c r="B13" s="173" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C13" s="150" t="inlineStr"/>
-      <c r="D13" s="150" t="inlineStr">
+      <c r="C13" s="176" t="inlineStr"/>
+      <c r="D13" s="176" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="E13" s="150" t="inlineStr">
+      <c r="E13" s="176" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1304,14 +1376,14 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B14" s="149" t="inlineStr"/>
-      <c r="C14" s="149" t="inlineStr"/>
-      <c r="D14" s="149" t="inlineStr">
+      <c r="B14" s="175" t="inlineStr"/>
+      <c r="C14" s="175" t="inlineStr"/>
+      <c r="D14" s="175" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="E14" s="149" t="inlineStr"/>
+      <c r="E14" s="175" t="inlineStr"/>
       <c r="F14" s="99" t="inlineStr">
         <is>
           <t>Witchcraft Paper Due</t>
@@ -1324,18 +1396,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B15" s="149" t="inlineStr"/>
-      <c r="C15" s="149" t="inlineStr">
+      <c r="B15" s="175" t="inlineStr"/>
+      <c r="C15" s="175" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D15" s="149" t="inlineStr">
+      <c r="D15" s="175" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E15" s="149" t="inlineStr"/>
+      <c r="E15" s="175" t="inlineStr"/>
       <c r="F15" s="99" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment</t>
@@ -1348,18 +1420,18 @@
           <t>Mid-term</t>
         </is>
       </c>
-      <c r="B16" s="147" t="inlineStr">
+      <c r="B16" s="173" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C16" s="148" t="inlineStr"/>
-      <c r="D16" s="148" t="inlineStr">
+      <c r="C16" s="174" t="inlineStr"/>
+      <c r="D16" s="174" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E16" s="148" t="inlineStr">
+      <c r="E16" s="174" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1375,14 +1447,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B17" s="149" t="inlineStr"/>
-      <c r="C17" s="149" t="inlineStr"/>
-      <c r="D17" s="149" t="inlineStr">
+      <c r="B17" s="175" t="inlineStr"/>
+      <c r="C17" s="175" t="inlineStr"/>
+      <c r="D17" s="175" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="E17" s="149" t="inlineStr"/>
+      <c r="E17" s="175" t="inlineStr"/>
       <c r="F17" s="99" t="inlineStr">
         <is>
           <t>Midterm Exam</t>
@@ -1395,18 +1467,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B18" s="149" t="inlineStr"/>
-      <c r="C18" s="149" t="inlineStr">
+      <c r="B18" s="175" t="inlineStr"/>
+      <c r="C18" s="175" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="D18" s="149" t="inlineStr">
+      <c r="D18" s="175" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E18" s="149" t="inlineStr"/>
+      <c r="E18" s="175" t="inlineStr"/>
       <c r="F18" s="99" t="inlineStr">
         <is>
           <t>Week Oct 6-9: Midterm &amp; Break</t>
@@ -1419,18 +1491,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B19" s="149" t="inlineStr"/>
-      <c r="C19" s="149" t="inlineStr">
+      <c r="B19" s="175" t="inlineStr"/>
+      <c r="C19" s="175" t="inlineStr">
         <is>
           <t>2026-12-01</t>
         </is>
       </c>
-      <c r="D19" s="149" t="inlineStr">
+      <c r="D19" s="175" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E19" s="149" t="inlineStr"/>
+      <c r="E19" s="175" t="inlineStr"/>
       <c r="F19" s="99" t="inlineStr">
         <is>
           <t>Week Dec 1-4: Modern Europe?</t>
@@ -1443,18 +1515,18 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B20" s="147" t="inlineStr">
+      <c r="B20" s="173" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C20" s="150" t="inlineStr"/>
-      <c r="D20" s="150" t="inlineStr">
+      <c r="C20" s="176" t="inlineStr"/>
+      <c r="D20" s="176" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="E20" s="150" t="inlineStr">
+      <c r="E20" s="176" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1470,14 +1542,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B21" s="149" t="inlineStr"/>
-      <c r="C21" s="149" t="inlineStr"/>
-      <c r="D21" s="149" t="inlineStr">
+      <c r="B21" s="175" t="inlineStr"/>
+      <c r="C21" s="175" t="inlineStr"/>
+      <c r="D21" s="175" t="inlineStr">
         <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="E21" s="149" t="inlineStr"/>
+      <c r="E21" s="175" t="inlineStr"/>
       <c r="F21" s="99" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -1490,18 +1562,18 @@
           <t>Discussion Section</t>
         </is>
       </c>
-      <c r="B22" s="147" t="inlineStr">
+      <c r="B22" s="173" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C22" s="148" t="inlineStr"/>
-      <c r="D22" s="148" t="inlineStr">
+      <c r="C22" s="174" t="inlineStr"/>
+      <c r="D22" s="174" t="inlineStr">
         <is>
           <t>2026-11-12</t>
         </is>
       </c>
-      <c r="E22" s="148" t="inlineStr">
+      <c r="E22" s="174" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1517,18 +1589,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B23" s="149" t="inlineStr"/>
-      <c r="C23" s="149" t="inlineStr">
+      <c r="B23" s="175" t="inlineStr"/>
+      <c r="C23" s="175" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D23" s="149" t="inlineStr">
+      <c r="D23" s="175" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E23" s="149" t="inlineStr"/>
+      <c r="E23" s="175" t="inlineStr"/>
       <c r="F23" s="99" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death</t>
@@ -1541,18 +1613,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B24" s="149" t="inlineStr"/>
-      <c r="C24" s="149" t="inlineStr">
+      <c r="B24" s="175" t="inlineStr"/>
+      <c r="C24" s="175" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D24" s="149" t="inlineStr">
+      <c r="D24" s="175" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E24" s="149" t="inlineStr"/>
+      <c r="E24" s="175" t="inlineStr"/>
       <c r="F24" s="99" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death - Section reading 1: -- 13 of 33 -- Lizzie Wade, “From Black Death to fatal flu, pas</t>
@@ -1565,18 +1637,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B25" s="149" t="inlineStr"/>
-      <c r="C25" s="149" t="inlineStr">
+      <c r="B25" s="175" t="inlineStr"/>
+      <c r="C25" s="175" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D25" s="149" t="inlineStr">
+      <c r="D25" s="175" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E25" s="149" t="inlineStr"/>
+      <c r="E25" s="175" t="inlineStr"/>
       <c r="F25" s="99" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life</t>
@@ -1589,18 +1661,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B26" s="149" t="inlineStr"/>
-      <c r="C26" s="149" t="inlineStr">
+      <c r="B26" s="175" t="inlineStr"/>
+      <c r="C26" s="175" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D26" s="149" t="inlineStr">
+      <c r="D26" s="175" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E26" s="149" t="inlineStr"/>
+      <c r="E26" s="175" t="inlineStr"/>
       <c r="F26" s="99" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life - Section reading 1: A Roger Ekirch, “Sleep we have lost: Pre-Industrial Slumber in the Brit</t>
@@ -1613,18 +1685,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B27" s="149" t="inlineStr"/>
-      <c r="C27" s="149" t="inlineStr">
+      <c r="B27" s="175" t="inlineStr"/>
+      <c r="C27" s="175" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D27" s="149" t="inlineStr">
+      <c r="D27" s="175" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E27" s="149" t="inlineStr"/>
+      <c r="E27" s="175" t="inlineStr"/>
       <c r="F27" s="99" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance</t>
@@ -1637,18 +1709,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B28" s="149" t="inlineStr"/>
-      <c r="C28" s="149" t="inlineStr">
+      <c r="B28" s="175" t="inlineStr"/>
+      <c r="C28" s="175" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D28" s="149" t="inlineStr">
+      <c r="D28" s="175" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E28" s="149" t="inlineStr"/>
+      <c r="E28" s="175" t="inlineStr"/>
       <c r="F28" s="99" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance - Section reading 1: -- 14 of 33 -- Kay Daly, “Diverting the Flood of History: Ada Palmer’s I</t>
@@ -1661,18 +1733,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B29" s="149" t="inlineStr"/>
-      <c r="C29" s="149" t="inlineStr">
+      <c r="B29" s="175" t="inlineStr"/>
+      <c r="C29" s="175" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D29" s="149" t="inlineStr">
+      <c r="D29" s="175" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E29" s="149" t="inlineStr"/>
+      <c r="E29" s="175" t="inlineStr"/>
       <c r="F29" s="99" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance - Section reading 1: Vasari, Lives of the Artists: Leonardo da Vinci &amp; Properzia de’ Rossi V</t>
@@ -1685,18 +1757,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B30" s="149" t="inlineStr"/>
-      <c r="C30" s="149" t="inlineStr">
+      <c r="B30" s="175" t="inlineStr"/>
+      <c r="C30" s="175" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D30" s="149" t="inlineStr">
+      <c r="D30" s="175" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E30" s="149" t="inlineStr"/>
+      <c r="E30" s="175" t="inlineStr"/>
       <c r="F30" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion</t>
@@ -1709,18 +1781,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B31" s="149" t="inlineStr"/>
-      <c r="C31" s="149" t="inlineStr">
+      <c r="B31" s="175" t="inlineStr"/>
+      <c r="C31" s="175" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D31" s="149" t="inlineStr">
+      <c r="D31" s="175" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E31" s="149" t="inlineStr"/>
+      <c r="E31" s="175" t="inlineStr"/>
       <c r="F31" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion - Section reading 1: Jerry Brotton, The Renaissance Bazaar, Chap 1 (15 pgs) Read Colu</t>
@@ -1733,18 +1805,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B32" s="149" t="inlineStr"/>
-      <c r="C32" s="149" t="inlineStr">
+      <c r="B32" s="175" t="inlineStr"/>
+      <c r="C32" s="175" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D32" s="149" t="inlineStr">
+      <c r="D32" s="175" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E32" s="149" t="inlineStr"/>
+      <c r="E32" s="175" t="inlineStr"/>
       <c r="F32" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion - Section reading 2: Bernal Diaz del Castillo, The True History of the Conquest of Ne</t>
@@ -1757,18 +1829,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B33" s="149" t="inlineStr"/>
-      <c r="C33" s="149" t="inlineStr">
+      <c r="B33" s="175" t="inlineStr"/>
+      <c r="C33" s="175" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="D33" s="149" t="inlineStr">
+      <c r="D33" s="175" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="E33" s="149" t="inlineStr"/>
+      <c r="E33" s="175" t="inlineStr"/>
       <c r="F33" s="99" t="inlineStr">
         <is>
           <t>Week Oct 13-16: The Reformation</t>
@@ -1781,18 +1853,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B34" s="149" t="inlineStr"/>
-      <c r="C34" s="149" t="inlineStr">
+      <c r="B34" s="175" t="inlineStr"/>
+      <c r="C34" s="175" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="D34" s="149" t="inlineStr">
+      <c r="D34" s="175" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="E34" s="149" t="inlineStr"/>
+      <c r="E34" s="175" t="inlineStr"/>
       <c r="F34" s="99" t="inlineStr">
         <is>
           <t>Week Oct 20-23: The Reformation</t>
@@ -1805,18 +1877,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B35" s="149" t="inlineStr"/>
-      <c r="C35" s="149" t="inlineStr">
+      <c r="B35" s="175" t="inlineStr"/>
+      <c r="C35" s="175" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D35" s="149" t="inlineStr">
+      <c r="D35" s="175" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E35" s="149" t="inlineStr"/>
+      <c r="E35" s="175" t="inlineStr"/>
       <c r="F35" s="99" t="inlineStr">
         <is>
           <t>Week Oct 27-30: Reformation</t>
@@ -1829,18 +1901,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B36" s="149" t="inlineStr"/>
-      <c r="C36" s="149" t="inlineStr">
+      <c r="B36" s="175" t="inlineStr"/>
+      <c r="C36" s="175" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D36" s="149" t="inlineStr">
+      <c r="D36" s="175" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E36" s="149" t="inlineStr"/>
+      <c r="E36" s="175" t="inlineStr"/>
       <c r="F36" s="99" t="inlineStr">
         <is>
           <t xml:space="preserve">Week Oct 27-30: Reformation - Section reading 1: Barbara Diefendorf, ed., The Saint Bartholomew’s Day Massacre: A Brief </t>
@@ -1853,18 +1925,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B37" s="149" t="inlineStr"/>
-      <c r="C37" s="149" t="inlineStr">
+      <c r="B37" s="175" t="inlineStr"/>
+      <c r="C37" s="175" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D37" s="149" t="inlineStr">
+      <c r="D37" s="175" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E37" s="149" t="inlineStr"/>
+      <c r="E37" s="175" t="inlineStr"/>
       <c r="F37" s="99" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science</t>
@@ -1877,18 +1949,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B38" s="149" t="inlineStr"/>
-      <c r="C38" s="149" t="inlineStr">
+      <c r="B38" s="175" t="inlineStr"/>
+      <c r="C38" s="175" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D38" s="149" t="inlineStr">
+      <c r="D38" s="175" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E38" s="149" t="inlineStr"/>
+      <c r="E38" s="175" t="inlineStr"/>
       <c r="F38" s="99" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science - Section reading 1: Brian Levack, The Witchcraft Sourcebook, Chaps 36-44, 46-47 103.Lev</t>
@@ -1901,18 +1973,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B39" s="149" t="inlineStr"/>
-      <c r="C39" s="149" t="inlineStr">
+      <c r="B39" s="175" t="inlineStr"/>
+      <c r="C39" s="175" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D39" s="149" t="inlineStr">
+      <c r="D39" s="175" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E39" s="149" t="inlineStr"/>
+      <c r="E39" s="175" t="inlineStr"/>
       <c r="F39" s="99" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment - Section reading 1: Excerpt: John Locke, Two Treatises of Government (1689) Excerpt: Rous</t>
@@ -1925,18 +1997,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B40" s="149" t="inlineStr"/>
-      <c r="C40" s="149" t="inlineStr">
+      <c r="B40" s="175" t="inlineStr"/>
+      <c r="C40" s="175" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D40" s="149" t="inlineStr">
+      <c r="D40" s="175" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E40" s="149" t="inlineStr"/>
+      <c r="E40" s="175" t="inlineStr"/>
       <c r="F40" s="99" t="inlineStr">
         <is>
           <t>Week Nov 17-20: Enlightenment</t>
@@ -1949,18 +2021,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B41" s="149" t="inlineStr"/>
-      <c r="C41" s="149" t="inlineStr">
+      <c r="B41" s="175" t="inlineStr"/>
+      <c r="C41" s="175" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D41" s="149" t="inlineStr">
+      <c r="D41" s="175" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E41" s="149" t="inlineStr"/>
+      <c r="E41" s="175" t="inlineStr"/>
       <c r="F41" s="99" t="inlineStr">
         <is>
           <t xml:space="preserve">Week Nov 17-20: Enlightenment - Section reading 1: Video: Africa &amp; Britain, A Forgotten History, Episode 2: Freedom (50 </t>
@@ -1973,18 +2045,18 @@
           <t>Identification Quizzes</t>
         </is>
       </c>
-      <c r="B42" s="147" t="inlineStr">
+      <c r="B42" s="173" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C42" s="150" t="inlineStr"/>
-      <c r="D42" s="150" t="inlineStr">
+      <c r="C42" s="176" t="inlineStr"/>
+      <c r="D42" s="176" t="inlineStr">
         <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="E42" s="150" t="inlineStr">
+      <c r="E42" s="176" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2000,18 +2072,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B43" s="149" t="inlineStr"/>
-      <c r="C43" s="149" t="inlineStr">
+      <c r="B43" s="175" t="inlineStr"/>
+      <c r="C43" s="175" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D43" s="149" t="inlineStr">
+      <c r="D43" s="175" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E43" s="149" t="inlineStr"/>
+      <c r="E43" s="175" t="inlineStr"/>
       <c r="F43" s="99" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death (lecture topics)</t>
@@ -2024,18 +2096,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B44" s="149" t="inlineStr"/>
-      <c r="C44" s="149" t="inlineStr">
+      <c r="B44" s="175" t="inlineStr"/>
+      <c r="C44" s="175" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D44" s="149" t="inlineStr">
+      <c r="D44" s="175" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E44" s="149" t="inlineStr"/>
+      <c r="E44" s="175" t="inlineStr"/>
       <c r="F44" s="99" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life (lecture topics)</t>
@@ -2048,18 +2120,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B45" s="149" t="inlineStr"/>
-      <c r="C45" s="149" t="inlineStr">
+      <c r="B45" s="175" t="inlineStr"/>
+      <c r="C45" s="175" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D45" s="149" t="inlineStr">
+      <c r="D45" s="175" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E45" s="149" t="inlineStr"/>
+      <c r="E45" s="175" t="inlineStr"/>
       <c r="F45" s="99" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance (lecture topics)</t>
@@ -2072,18 +2144,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B46" s="149" t="inlineStr"/>
-      <c r="C46" s="149" t="inlineStr">
+      <c r="B46" s="175" t="inlineStr"/>
+      <c r="C46" s="175" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D46" s="149" t="inlineStr">
+      <c r="D46" s="175" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E46" s="149" t="inlineStr"/>
+      <c r="E46" s="175" t="inlineStr"/>
       <c r="F46" s="99" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance (lecture topics)</t>
@@ -2096,18 +2168,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B47" s="149" t="inlineStr"/>
-      <c r="C47" s="149" t="inlineStr">
+      <c r="B47" s="175" t="inlineStr"/>
+      <c r="C47" s="175" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D47" s="149" t="inlineStr">
+      <c r="D47" s="175" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E47" s="149" t="inlineStr"/>
+      <c r="E47" s="175" t="inlineStr"/>
       <c r="F47" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion (lecture topics)</t>
@@ -2120,18 +2192,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B48" s="149" t="inlineStr"/>
-      <c r="C48" s="149" t="inlineStr">
+      <c r="B48" s="175" t="inlineStr"/>
+      <c r="C48" s="175" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="D48" s="149" t="inlineStr">
+      <c r="D48" s="175" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E48" s="149" t="inlineStr"/>
+      <c r="E48" s="175" t="inlineStr"/>
       <c r="F48" s="99" t="inlineStr">
         <is>
           <t>Week Oct 6-9: Midterm &amp; Break (lecture topics)</t>
@@ -2144,18 +2216,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B49" s="149" t="inlineStr"/>
-      <c r="C49" s="149" t="inlineStr">
+      <c r="B49" s="175" t="inlineStr"/>
+      <c r="C49" s="175" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="D49" s="149" t="inlineStr">
+      <c r="D49" s="175" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="E49" s="149" t="inlineStr"/>
+      <c r="E49" s="175" t="inlineStr"/>
       <c r="F49" s="99" t="inlineStr">
         <is>
           <t>Week Oct 13-16: The Reformation (lecture topics)</t>
@@ -2168,18 +2240,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B50" s="149" t="inlineStr"/>
-      <c r="C50" s="149" t="inlineStr">
+      <c r="B50" s="175" t="inlineStr"/>
+      <c r="C50" s="175" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="D50" s="149" t="inlineStr">
+      <c r="D50" s="175" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="E50" s="149" t="inlineStr"/>
+      <c r="E50" s="175" t="inlineStr"/>
       <c r="F50" s="99" t="inlineStr">
         <is>
           <t>Week Oct 20-23: The Reformation (lecture topics)</t>
@@ -2192,18 +2264,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B51" s="149" t="inlineStr"/>
-      <c r="C51" s="149" t="inlineStr">
+      <c r="B51" s="175" t="inlineStr"/>
+      <c r="C51" s="175" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D51" s="149" t="inlineStr">
+      <c r="D51" s="175" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E51" s="149" t="inlineStr"/>
+      <c r="E51" s="175" t="inlineStr"/>
       <c r="F51" s="99" t="inlineStr">
         <is>
           <t>Week Oct 27-30: Reformation (lecture topics)</t>
@@ -2216,18 +2288,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B52" s="149" t="inlineStr"/>
-      <c r="C52" s="149" t="inlineStr">
+      <c r="B52" s="175" t="inlineStr"/>
+      <c r="C52" s="175" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D52" s="149" t="inlineStr">
+      <c r="D52" s="175" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E52" s="149" t="inlineStr"/>
+      <c r="E52" s="175" t="inlineStr"/>
       <c r="F52" s="99" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science (lecture topics)</t>
@@ -2240,18 +2312,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B53" s="149" t="inlineStr"/>
-      <c r="C53" s="149" t="inlineStr">
+      <c r="B53" s="175" t="inlineStr"/>
+      <c r="C53" s="175" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D53" s="149" t="inlineStr">
+      <c r="D53" s="175" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E53" s="149" t="inlineStr"/>
+      <c r="E53" s="175" t="inlineStr"/>
       <c r="F53" s="99" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment (lecture topics)</t>
@@ -2264,18 +2336,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B54" s="149" t="inlineStr"/>
-      <c r="C54" s="149" t="inlineStr">
+      <c r="B54" s="175" t="inlineStr"/>
+      <c r="C54" s="175" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D54" s="149" t="inlineStr">
+      <c r="D54" s="175" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E54" s="149" t="inlineStr"/>
+      <c r="E54" s="175" t="inlineStr"/>
       <c r="F54" s="99" t="inlineStr">
         <is>
           <t>Week Nov 17-20: Enlightenment (lecture topics)</t>
@@ -2288,18 +2360,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B55" s="149" t="inlineStr"/>
-      <c r="C55" s="149" t="inlineStr">
+      <c r="B55" s="175" t="inlineStr"/>
+      <c r="C55" s="175" t="inlineStr">
         <is>
           <t>2026-12-01</t>
         </is>
       </c>
-      <c r="D55" s="149" t="inlineStr">
+      <c r="D55" s="175" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E55" s="149" t="inlineStr"/>
+      <c r="E55" s="175" t="inlineStr"/>
       <c r="F55" s="99" t="inlineStr">
         <is>
           <t>Week Dec 1-4: Modern Europe? (lecture topics)</t>
@@ -2312,18 +2384,18 @@
           <t>Extra Credit</t>
         </is>
       </c>
-      <c r="B56" s="147" t="inlineStr">
+      <c r="B56" s="173" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C56" s="148" t="inlineStr"/>
-      <c r="D56" s="148" t="inlineStr">
+      <c r="C56" s="174" t="inlineStr"/>
+      <c r="D56" s="174" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E56" s="148" t="inlineStr">
+      <c r="E56" s="174" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2363,7 +2435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2480,18 +2552,18 @@
           <t>Midterm 1</t>
         </is>
       </c>
-      <c r="B10" s="152" t="inlineStr">
+      <c r="B10" s="177" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C10" s="153" t="inlineStr"/>
-      <c r="D10" s="153" t="inlineStr">
+      <c r="C10" s="178" t="inlineStr"/>
+      <c r="D10" s="178" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="E10" s="153" t="inlineStr">
+      <c r="E10" s="178" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2507,18 +2579,18 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B11" s="154" t="inlineStr"/>
-      <c r="C11" s="154" t="inlineStr">
+      <c r="B11" s="179" t="inlineStr"/>
+      <c r="C11" s="179" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="D11" s="154" t="inlineStr">
+      <c r="D11" s="179" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="E11" s="154" t="inlineStr"/>
+      <c r="E11" s="179" t="inlineStr"/>
       <c r="F11" s="112" t="inlineStr">
         <is>
           <t>9/30 Midterm 1: 250 Points Chapters 1, 2, 3, 4, 5, 8</t>
@@ -2531,18 +2603,18 @@
           <t>Midterm 2</t>
         </is>
       </c>
-      <c r="B12" s="152" t="inlineStr">
+      <c r="B12" s="177" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C12" s="155" t="inlineStr"/>
-      <c r="D12" s="155" t="inlineStr">
+      <c r="C12" s="180" t="inlineStr"/>
+      <c r="D12" s="180" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E12" s="155" t="inlineStr">
+      <c r="E12" s="180" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2558,18 +2630,18 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B13" s="154" t="inlineStr"/>
-      <c r="C13" s="154" t="inlineStr">
+      <c r="B13" s="179" t="inlineStr"/>
+      <c r="C13" s="179" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="D13" s="154" t="inlineStr">
+      <c r="D13" s="179" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E13" s="154" t="inlineStr"/>
+      <c r="E13" s="179" t="inlineStr"/>
       <c r="F13" s="112" t="inlineStr">
         <is>
           <t>10/26 Midterm 2: 250 Points Chapters 6, 7, 9, &amp; 16</t>
@@ -2582,18 +2654,18 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B14" s="152" t="inlineStr">
+      <c r="B14" s="177" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C14" s="153" t="inlineStr"/>
-      <c r="D14" s="153" t="inlineStr">
+      <c r="C14" s="178" t="inlineStr"/>
+      <c r="D14" s="178" t="inlineStr">
         <is>
           <t>2026-12-16</t>
         </is>
       </c>
-      <c r="E14" s="153" t="inlineStr">
+      <c r="E14" s="178" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2609,18 +2681,18 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B15" s="154" t="inlineStr"/>
-      <c r="C15" s="154" t="inlineStr">
+      <c r="B15" s="179" t="inlineStr"/>
+      <c r="C15" s="179" t="inlineStr">
         <is>
           <t>2026-12-16</t>
         </is>
       </c>
-      <c r="D15" s="154" t="inlineStr">
+      <c r="D15" s="179" t="inlineStr">
         <is>
           <t>2026-12-16</t>
         </is>
       </c>
-      <c r="E15" s="154" t="inlineStr"/>
+      <c r="E15" s="179" t="inlineStr"/>
       <c r="F15" s="112" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -2633,22 +2705,22 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B16" s="152" t="inlineStr">
+      <c r="B16" s="177" t="inlineStr">
         <is>
           <t>170 pts</t>
         </is>
       </c>
-      <c r="C16" s="155" t="inlineStr">
+      <c r="C16" s="180" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="D16" s="155" t="inlineStr">
-        <is>
-          <t>2026-11-16</t>
-        </is>
-      </c>
-      <c r="E16" s="155" t="inlineStr">
+      <c r="D16" s="180" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E16" s="180" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2664,45 +2736,37 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B17" s="154" t="inlineStr"/>
-      <c r="C17" s="154" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D17" s="154" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="E17" s="154" t="inlineStr"/>
+      <c r="B17" s="179" t="inlineStr"/>
+      <c r="C17" s="179" t="inlineStr"/>
+      <c r="D17" s="179" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="E17" s="179" t="inlineStr"/>
       <c r="F17" s="112" t="inlineStr">
         <is>
-          <t>Class 1 (8/24) - Course Overview &amp; Introductions</t>
+          <t>Class 5 (9/9) - Product Cost Accumulation: Job; Order Co: Chapter 3</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B18" s="154" t="inlineStr"/>
-      <c r="C18" s="154" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="D18" s="154" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="E18" s="154" t="inlineStr"/>
+      <c r="A18" s="117" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B18" s="179" t="inlineStr"/>
+      <c r="C18" s="179" t="inlineStr"/>
+      <c r="D18" s="179" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="E18" s="179" t="inlineStr"/>
       <c r="F18" s="112" t="inlineStr">
         <is>
-          <t>Class 2 (8/26) - Role of Managerial accounting: Chapter 1</t>
+          <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
         </is>
       </c>
     </row>
@@ -2712,45 +2776,37 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B19" s="154" t="inlineStr"/>
-      <c r="C19" s="154" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D19" s="154" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="E19" s="154" t="inlineStr"/>
+      <c r="B19" s="179" t="inlineStr"/>
+      <c r="C19" s="179" t="inlineStr"/>
+      <c r="D19" s="179" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E19" s="179" t="inlineStr"/>
       <c r="F19" s="112" t="inlineStr">
         <is>
-          <t>Class 3 (8/31) - Basic Cost Mgt Concepts: Chapter 2</t>
+          <t>Class 7 (9/16) - Activity Based Costing: Chapter 5- ONLY; LO 5.1, 2, 4 &amp; 5</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B20" s="154" t="inlineStr"/>
-      <c r="C20" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="D20" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="E20" s="154" t="inlineStr"/>
+      <c r="A20" s="117" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B20" s="179" t="inlineStr"/>
+      <c r="C20" s="179" t="inlineStr"/>
+      <c r="D20" s="179" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E20" s="179" t="inlineStr"/>
       <c r="F20" s="112" t="inlineStr">
         <is>
-          <t>Class 4 (9/2) - Basic Cost Mgt Concepts: Chapter 2</t>
+          <t>Class 7 (9/16) - 3-24, 3-28, 3-32; 15 Points</t>
         </is>
       </c>
     </row>
@@ -2760,93 +2816,77 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B21" s="154" t="inlineStr"/>
-      <c r="C21" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="D21" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="E21" s="154" t="inlineStr"/>
+      <c r="B21" s="179" t="inlineStr"/>
+      <c r="C21" s="179" t="inlineStr"/>
+      <c r="D21" s="179" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E21" s="179" t="inlineStr"/>
       <c r="F21" s="112" t="inlineStr">
         <is>
-          <t>9/7 - No Class Labor Day Holiday</t>
+          <t>Class 8 (9/21) - Product Cost Accumulation: Pro-; cess Co: Chapter 4- ONLY; LO 4.1, 3, 4, &amp; 5</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B22" s="154" t="inlineStr"/>
-      <c r="C22" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="D22" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="E22" s="154" t="inlineStr"/>
+      <c r="A22" s="117" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B22" s="179" t="inlineStr"/>
+      <c r="C22" s="179" t="inlineStr"/>
+      <c r="D22" s="179" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E22" s="179" t="inlineStr"/>
       <c r="F22" s="112" t="inlineStr">
         <is>
-          <t>Class 5 (9/9) - Product Cost Accumulation: Job; Order Co: Chapter 3</t>
+          <t>Class 8 (9/21) - 5-27 5-46; 10 Points</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="117" t="inlineStr">
+      <c r="A23" s="116" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B23" s="179" t="inlineStr"/>
+      <c r="C23" s="179" t="inlineStr"/>
+      <c r="D23" s="179" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E23" s="179" t="inlineStr"/>
+      <c r="F23" s="112" t="inlineStr">
+        <is>
+          <t>Class 9 (9/23) - Cost of Quality &amp; ESG &amp;; Overview of; • : Chapter 8 - ONLY; LO 8.7, 8, 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="117" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="B23" s="154" t="inlineStr"/>
-      <c r="C23" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="D23" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="E23" s="154" t="inlineStr"/>
-      <c r="F23" s="112" t="inlineStr">
-        <is>
-          <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B24" s="154" t="inlineStr"/>
-      <c r="C24" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="D24" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="E24" s="154" t="inlineStr"/>
+      <c r="B24" s="179" t="inlineStr"/>
+      <c r="C24" s="179" t="inlineStr"/>
+      <c r="D24" s="179" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E24" s="179" t="inlineStr"/>
       <c r="F24" s="112" t="inlineStr">
         <is>
-          <t>Class 6 (9/14) - Manufacturing Overhead Normal; Costing: Chapter 3</t>
+          <t>Class 9 (9/23) - 4-21, 4-22; 10 Points</t>
         </is>
       </c>
     </row>
@@ -2856,21 +2896,17 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B25" s="154" t="inlineStr"/>
-      <c r="C25" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="D25" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="E25" s="154" t="inlineStr"/>
+      <c r="B25" s="179" t="inlineStr"/>
+      <c r="C25" s="179" t="inlineStr"/>
+      <c r="D25" s="179" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E25" s="179" t="inlineStr"/>
       <c r="F25" s="112" t="inlineStr">
         <is>
-          <t>Class 7 (9/16) - Activity Based Costing: Chapter 5- ONLY; LO 5.1, 2, 4 &amp; 5</t>
+          <t>Class 10 (9/28) - Catchup &amp; Midterm Review</t>
         </is>
       </c>
     </row>
@@ -2880,21 +2916,17 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B26" s="154" t="inlineStr"/>
-      <c r="C26" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="D26" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="E26" s="154" t="inlineStr"/>
+      <c r="B26" s="179" t="inlineStr"/>
+      <c r="C26" s="179" t="inlineStr"/>
+      <c r="D26" s="179" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E26" s="179" t="inlineStr"/>
       <c r="F26" s="112" t="inlineStr">
         <is>
-          <t>Class 7 (9/16) - 3-24, 3-28, 3-32; 15 Points</t>
+          <t>Class 10 (9/28) - 8-28, 8-29; 10 Points</t>
         </is>
       </c>
     </row>
@@ -2904,21 +2936,17 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B27" s="154" t="inlineStr"/>
-      <c r="C27" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="D27" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="E27" s="154" t="inlineStr"/>
+      <c r="B27" s="179" t="inlineStr"/>
+      <c r="C27" s="179" t="inlineStr"/>
+      <c r="D27" s="179" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E27" s="179" t="inlineStr"/>
       <c r="F27" s="112" t="inlineStr">
         <is>
-          <t>Class 8 (9/21) - Product Cost Accumulation: Pro-; cess Co: Chapter 4- ONLY; LO 4.1, 3, 4, &amp; 5</t>
+          <t>Class 12 (10/7) - Cost volume profit analysis: Chapter 7</t>
         </is>
       </c>
     </row>
@@ -2928,21 +2956,17 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B28" s="154" t="inlineStr"/>
-      <c r="C28" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="D28" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="E28" s="154" t="inlineStr"/>
+      <c r="B28" s="179" t="inlineStr"/>
+      <c r="C28" s="179" t="inlineStr"/>
+      <c r="D28" s="179" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E28" s="179" t="inlineStr"/>
       <c r="F28" s="112" t="inlineStr">
         <is>
-          <t>Class 8 (9/21) - 5-27 5-46; 10 Points</t>
+          <t>Class 12 (10/7) - 6-24, 6-25, 6-34; 15 Points</t>
         </is>
       </c>
     </row>
@@ -2952,21 +2976,17 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B29" s="154" t="inlineStr"/>
-      <c r="C29" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="D29" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="E29" s="154" t="inlineStr"/>
+      <c r="B29" s="179" t="inlineStr"/>
+      <c r="C29" s="179" t="inlineStr"/>
+      <c r="D29" s="179" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E29" s="179" t="inlineStr"/>
       <c r="F29" s="112" t="inlineStr">
         <is>
-          <t>Class 9 (9/23) - Cost of Quality &amp; ESG &amp;; Overview of; • : Chapter 8 - ONLY; LO 8.7, 8, 9</t>
+          <t>Class 14 (10/14) - Financial planning and analysis:; Static: Chapter 9</t>
         </is>
       </c>
     </row>
@@ -2976,69 +2996,57 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B30" s="154" t="inlineStr"/>
-      <c r="C30" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="D30" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="E30" s="154" t="inlineStr"/>
+      <c r="B30" s="179" t="inlineStr"/>
+      <c r="C30" s="179" t="inlineStr"/>
+      <c r="D30" s="179" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E30" s="179" t="inlineStr"/>
       <c r="F30" s="112" t="inlineStr">
         <is>
-          <t>Class 9 (9/23) - 4-21, 4-22; 10 Points</t>
+          <t>Class 14 (10/14) - 7-29, 7-33, 7-40; 15 Points</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="117" t="inlineStr">
+      <c r="A31" s="116" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B31" s="179" t="inlineStr"/>
+      <c r="C31" s="179" t="inlineStr"/>
+      <c r="D31" s="179" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E31" s="179" t="inlineStr"/>
+      <c r="F31" s="112" t="inlineStr">
+        <is>
+          <t>Class 15 (10/19) - Capital Budgeting; Practice Midterm Ques: Chapter 16- ONLY; LO 16.1, 2, 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="117" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="B31" s="154" t="inlineStr"/>
-      <c r="C31" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="D31" s="154" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E31" s="154" t="inlineStr"/>
-      <c r="F31" s="112" t="inlineStr">
-        <is>
-          <t>Class 10 (9/28) - 8-28, 8-29; 10 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B32" s="154" t="inlineStr"/>
-      <c r="C32" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="D32" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="E32" s="154" t="inlineStr"/>
+      <c r="B32" s="179" t="inlineStr"/>
+      <c r="C32" s="179" t="inlineStr"/>
+      <c r="D32" s="179" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E32" s="179" t="inlineStr"/>
       <c r="F32" s="112" t="inlineStr">
         <is>
-          <t>Class 11 (10/5) - Cost Estimation: Chapter 6</t>
+          <t>Class 15 (10/19) - 9-25, 9-28, 9-37; 15 - Points</t>
         </is>
       </c>
     </row>
@@ -3048,21 +3056,17 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B33" s="154" t="inlineStr"/>
-      <c r="C33" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="D33" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="E33" s="154" t="inlineStr"/>
+      <c r="B33" s="179" t="inlineStr"/>
+      <c r="C33" s="179" t="inlineStr"/>
+      <c r="D33" s="179" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E33" s="179" t="inlineStr"/>
       <c r="F33" s="112" t="inlineStr">
         <is>
-          <t>Class 12 (10/7) - Cost volume profit analysis: Chapter 7</t>
+          <t>Class 16 (10/21) - Catchup &amp; Midterm Review</t>
         </is>
       </c>
     </row>
@@ -3072,21 +3076,17 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B34" s="154" t="inlineStr"/>
-      <c r="C34" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="D34" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="E34" s="154" t="inlineStr"/>
+      <c r="B34" s="179" t="inlineStr"/>
+      <c r="C34" s="179" t="inlineStr"/>
+      <c r="D34" s="179" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E34" s="179" t="inlineStr"/>
       <c r="F34" s="112" t="inlineStr">
         <is>
-          <t>Class 12 (10/7) - 6-24, 6-25, 6-34; 15 Points</t>
+          <t>Class 16 (10/21) - 16-28, 16-40; 10 Points</t>
         </is>
       </c>
     </row>
@@ -3096,117 +3096,97 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B35" s="154" t="inlineStr"/>
-      <c r="C35" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="D35" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E35" s="154" t="inlineStr"/>
+      <c r="B35" s="179" t="inlineStr"/>
+      <c r="C35" s="179" t="inlineStr"/>
+      <c r="D35" s="179" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="E35" s="179" t="inlineStr"/>
       <c r="F35" s="112" t="inlineStr">
         <is>
-          <t>Class 13 (10/12) - Cost volume profit analysis &amp;: Chapter 7</t>
+          <t>Class 19 (11/4) - Sales Variance Analysis; Flexible Budget: Chapter 11 - ONLY; LO 11.1, 11.2 &amp;; Appendix B</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B36" s="154" t="inlineStr"/>
-      <c r="C36" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="D36" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E36" s="154" t="inlineStr"/>
+      <c r="A36" s="117" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B36" s="179" t="inlineStr"/>
+      <c r="C36" s="179" t="inlineStr"/>
+      <c r="D36" s="179" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="E36" s="179" t="inlineStr"/>
       <c r="F36" s="112" t="inlineStr">
         <is>
-          <t>Class 14 (10/14) - Financial planning and analysis:; Static: Chapter 9</t>
+          <t>Class 19 (11/4) - 10-26, 10-30; 10 Points</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="117" t="inlineStr">
+      <c r="A37" s="116" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B37" s="179" t="inlineStr"/>
+      <c r="C37" s="179" t="inlineStr"/>
+      <c r="D37" s="179" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E37" s="179" t="inlineStr"/>
+      <c r="F37" s="112" t="inlineStr">
+        <is>
+          <t>Class 20 (11/9) - Investment Centers: Chapter 13- ONLY; LO 13-1, 2, 3, 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="117" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="B37" s="154" t="inlineStr"/>
-      <c r="C37" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="D37" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E37" s="154" t="inlineStr"/>
-      <c r="F37" s="112" t="inlineStr">
-        <is>
-          <t>Class 14 (10/14) - 7-29, 7-33, 7-40; 15 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B38" s="154" t="inlineStr"/>
-      <c r="C38" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="D38" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E38" s="154" t="inlineStr"/>
+      <c r="B38" s="179" t="inlineStr"/>
+      <c r="C38" s="179" t="inlineStr"/>
+      <c r="D38" s="179" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E38" s="179" t="inlineStr"/>
       <c r="F38" s="112" t="inlineStr">
         <is>
-          <t>Class 15 (10/19) - Capital Budgeting; Practice Midterm Ques: Chapter 16- ONLY; LO 16.1, 2, 3</t>
+          <t>Class 20 (11/9) - 11-31, 11-52; 10 Points</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="117" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B39" s="154" t="inlineStr"/>
-      <c r="C39" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="D39" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E39" s="154" t="inlineStr"/>
+      <c r="A39" s="116" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B39" s="179" t="inlineStr"/>
+      <c r="C39" s="179" t="inlineStr"/>
+      <c r="D39" s="179" t="inlineStr">
+        <is>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="E39" s="179" t="inlineStr"/>
       <c r="F39" s="112" t="inlineStr">
         <is>
-          <t>Class 15 (10/19) - 9-25, 9-28, 9-37; 15 - Points</t>
+          <t>Class 21 (11/16) - AI &amp; FP&amp;A</t>
         </is>
       </c>
     </row>
@@ -3216,21 +3196,17 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B40" s="154" t="inlineStr"/>
-      <c r="C40" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="D40" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="E40" s="154" t="inlineStr"/>
+      <c r="B40" s="179" t="inlineStr"/>
+      <c r="C40" s="179" t="inlineStr"/>
+      <c r="D40" s="179" t="inlineStr">
+        <is>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="E40" s="179" t="inlineStr"/>
       <c r="F40" s="112" t="inlineStr">
         <is>
-          <t>Class 16 (10/21) - 16-28, 16-40; 10 Points</t>
+          <t>Class 21 (11/16) - 13-29, 13-33; 10 Points</t>
         </is>
       </c>
     </row>
@@ -3240,429 +3216,157 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B41" s="154" t="inlineStr"/>
-      <c r="C41" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-28</t>
-        </is>
-      </c>
-      <c r="D41" s="154" t="inlineStr">
-        <is>
-          <t>2026-10-28</t>
-        </is>
-      </c>
-      <c r="E41" s="154" t="inlineStr"/>
+      <c r="B41" s="179" t="inlineStr"/>
+      <c r="C41" s="179" t="inlineStr"/>
+      <c r="D41" s="179" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E41" s="179" t="inlineStr"/>
       <c r="F41" s="112" t="inlineStr">
         <is>
-          <t>Class 17 (10/28) - Guest Speaker</t>
+          <t>Class 2 (12/2) - Catchup &amp; Final Review; Practice Final Questions Posted to Brightspace at; 5:00 PM</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B42" s="154" t="inlineStr"/>
-      <c r="C42" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-02</t>
-        </is>
-      </c>
-      <c r="D42" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-02</t>
-        </is>
-      </c>
-      <c r="E42" s="154" t="inlineStr"/>
+      <c r="A42" s="117" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B42" s="179" t="inlineStr"/>
+      <c r="C42" s="179" t="inlineStr"/>
+      <c r="D42" s="179" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E42" s="179" t="inlineStr"/>
       <c r="F42" s="112" t="inlineStr">
         <is>
-          <t>Class 19 (11/2) - Standard Costing &amp; Direct Cost; Variance: Chapter 10 – ONLY; LO 10.1 thru 8</t>
+          <t>Class 2 (12/2) - 14-35, 14-41; 10 Points; Assignments listed Be-; low Due by11:59 PM; Linked In Learning; E</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B43" s="154" t="inlineStr"/>
-      <c r="C43" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="D43" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="E43" s="154" t="inlineStr"/>
-      <c r="F43" s="112" t="inlineStr">
-        <is>
-          <t>Class 19 (11/4) - Sales Variance Analysis; Flexible Budget: Chapter 11 - ONLY; LO 11.1, 11.2 &amp;; Appendix B</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="117" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B44" s="154" t="inlineStr"/>
-      <c r="C44" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="D44" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="E44" s="154" t="inlineStr"/>
-      <c r="F44" s="112" t="inlineStr">
-        <is>
-          <t>Class 19 (11/4) - 10-26, 10-30; 10 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B45" s="154" t="inlineStr"/>
-      <c r="C45" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="D45" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="E45" s="154" t="inlineStr"/>
-      <c r="F45" s="112" t="inlineStr">
-        <is>
-          <t>Class 20 (11/9) - Investment Centers: Chapter 13- ONLY; LO 13-1, 2, 3, 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="117" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B46" s="154" t="inlineStr"/>
-      <c r="C46" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="D46" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="E46" s="154" t="inlineStr"/>
-      <c r="F46" s="112" t="inlineStr">
-        <is>
-          <t>Class 20 (11/9) - 11-31, 11-52; 10 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B47" s="154" t="inlineStr"/>
-      <c r="C47" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-11</t>
-        </is>
-      </c>
-      <c r="D47" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-11</t>
-        </is>
-      </c>
-      <c r="E47" s="154" t="inlineStr"/>
-      <c r="F47" s="112" t="inlineStr">
-        <is>
-          <t>11/11 - No Class Veterans Day</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="117" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B48" s="154" t="inlineStr"/>
-      <c r="C48" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-16</t>
-        </is>
-      </c>
-      <c r="D48" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-16</t>
-        </is>
-      </c>
-      <c r="E48" s="154" t="inlineStr"/>
-      <c r="F48" s="112" t="inlineStr">
-        <is>
-          <t>Class 21 (11/16) - 13-29, 13-33; 10 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B49" s="154" t="inlineStr"/>
-      <c r="C49" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-18</t>
-        </is>
-      </c>
-      <c r="D49" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-18</t>
-        </is>
-      </c>
-      <c r="E49" s="154" t="inlineStr"/>
-      <c r="F49" s="112" t="inlineStr">
-        <is>
-          <t>Class 22 (11/18) - Decision-making: relevant costs; and ben: Chapter 14; (Part 1 of 3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B50" s="154" t="inlineStr"/>
-      <c r="C50" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-23</t>
-        </is>
-      </c>
-      <c r="D50" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-23</t>
-        </is>
-      </c>
-      <c r="E50" s="154" t="inlineStr"/>
-      <c r="F50" s="112" t="inlineStr">
-        <is>
-          <t>Class 23 (11/23) - Decision-making: relevant costs; and ben: Chapter 14; (Part 2 of 3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B51" s="154" t="inlineStr"/>
-      <c r="C51" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-25</t>
-        </is>
-      </c>
-      <c r="D51" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-25</t>
-        </is>
-      </c>
-      <c r="E51" s="154" t="inlineStr"/>
-      <c r="F51" s="112" t="inlineStr">
-        <is>
-          <t>11/25 - No Class Thanksgiving Holiday</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B52" s="154" t="inlineStr"/>
-      <c r="C52" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
-      </c>
-      <c r="D52" s="154" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
-      </c>
-      <c r="E52" s="154" t="inlineStr"/>
-      <c r="F52" s="112" t="inlineStr">
-        <is>
-          <t>Class 24 (11/30) - Decision-making: relevant costs; and ben: Chapter 14; (Part 3 of 3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B53" s="154" t="inlineStr"/>
-      <c r="C53" s="154" t="inlineStr">
+      <c r="A43" s="106" t="inlineStr">
+        <is>
+          <t>LinkedIn Learning Excel Certification</t>
+        </is>
+      </c>
+      <c r="B43" s="177" t="inlineStr">
+        <is>
+          <t>75 pts</t>
+        </is>
+      </c>
+      <c r="C43" s="178" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D43" s="178" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="D53" s="154" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E53" s="154" t="inlineStr"/>
-      <c r="F53" s="112" t="inlineStr">
-        <is>
-          <t>Class 2 (12/2) - Catchup &amp; Final Review; Practice Final Questions Posted to Brightspace at; 5:00 PM</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="106" t="inlineStr">
-        <is>
-          <t>LinkedIn Learning Excel Certification</t>
-        </is>
-      </c>
-      <c r="B54" s="152" t="inlineStr">
-        <is>
-          <t>75 pts</t>
-        </is>
-      </c>
-      <c r="C54" s="153" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="D54" s="153" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E54" s="153" t="inlineStr">
+      <c r="E43" s="178" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F54" s="109">
+      <c r="F43" s="109">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-linkedin-learning-excel-certification.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="118" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="118" t="inlineStr">
         <is>
           <t>Certification</t>
         </is>
       </c>
-      <c r="B55" s="154" t="inlineStr"/>
-      <c r="C55" s="154" t="inlineStr">
+      <c r="B44" s="179" t="inlineStr"/>
+      <c r="C44" s="179" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D55" s="154" t="inlineStr">
+      <c r="D44" s="179" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E55" s="154" t="inlineStr"/>
-      <c r="F55" s="112" t="inlineStr">
+      <c r="E44" s="179" t="inlineStr"/>
+      <c r="F44" s="112" t="inlineStr">
         <is>
           <t>LinkedIn Learning Excel Certification</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="113" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="113" t="inlineStr">
         <is>
           <t>Stukent Simternship</t>
         </is>
       </c>
-      <c r="B56" s="152" t="inlineStr">
+      <c r="B45" s="177" t="inlineStr">
         <is>
           <t>75 pts</t>
         </is>
       </c>
-      <c r="C56" s="155" t="inlineStr">
+      <c r="C45" s="180" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D56" s="155" t="inlineStr">
+      <c r="D45" s="180" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E56" s="155" t="inlineStr">
+      <c r="E45" s="180" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F56" s="115">
+      <c r="F45" s="115">
         <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-stukent-simternship.pdf","Open PDF")</f>
         <v/>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="118" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="118" t="inlineStr">
         <is>
           <t>Certification</t>
         </is>
       </c>
-      <c r="B57" s="154" t="inlineStr"/>
-      <c r="C57" s="154" t="inlineStr">
+      <c r="B46" s="179" t="inlineStr"/>
+      <c r="C46" s="179" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D57" s="154" t="inlineStr">
+      <c r="D46" s="179" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E57" s="154" t="inlineStr"/>
-      <c r="F57" s="112" t="inlineStr">
+      <c r="E46" s="179" t="inlineStr"/>
+      <c r="F46" s="112" t="inlineStr">
         <is>
           <t>Stukent Simternship</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B58" s="119" t="inlineStr">
+      <c r="B47" s="119" t="inlineStr">
         <is>
           <t>1070 pts</t>
         </is>
@@ -3803,22 +3507,22 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B10" s="157" t="inlineStr">
+      <c r="B10" s="181" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="C10" s="158" t="inlineStr">
+      <c r="C10" s="182" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D10" s="158" t="inlineStr">
+      <c r="D10" s="182" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E10" s="158" t="inlineStr">
+      <c r="E10" s="182" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3834,18 +3538,18 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B11" s="159" t="inlineStr"/>
-      <c r="C11" s="159" t="inlineStr">
+      <c r="B11" s="183" t="inlineStr"/>
+      <c r="C11" s="183" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D11" s="159" t="inlineStr">
+      <c r="D11" s="183" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E11" s="159" t="inlineStr"/>
+      <c r="E11" s="183" t="inlineStr"/>
       <c r="F11" s="126" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -3858,22 +3562,22 @@
           <t>Participation</t>
         </is>
       </c>
-      <c r="B12" s="157" t="inlineStr">
+      <c r="B12" s="181" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C12" s="160" t="inlineStr">
+      <c r="C12" s="184" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D12" s="160" t="inlineStr">
+      <c r="D12" s="184" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E12" s="160" t="inlineStr">
+      <c r="E12" s="184" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3889,14 +3593,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B13" s="159" t="inlineStr"/>
-      <c r="C13" s="159" t="inlineStr">
+      <c r="B13" s="183" t="inlineStr"/>
+      <c r="C13" s="183" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D13" s="159" t="inlineStr"/>
-      <c r="E13" s="159" t="inlineStr"/>
+      <c r="D13" s="183" t="inlineStr"/>
+      <c r="E13" s="183" t="inlineStr"/>
       <c r="F13" s="126" t="inlineStr">
         <is>
           <t>Research: SONA registration opens</t>
@@ -3909,14 +3613,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B14" s="159" t="inlineStr"/>
-      <c r="C14" s="159" t="inlineStr">
+      <c r="B14" s="183" t="inlineStr"/>
+      <c r="C14" s="183" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="D14" s="159" t="inlineStr"/>
-      <c r="E14" s="159" t="inlineStr"/>
+      <c r="D14" s="183" t="inlineStr"/>
+      <c r="E14" s="183" t="inlineStr"/>
       <c r="F14" s="126" t="inlineStr">
         <is>
           <t>Research: Prescreening questionnaire opens</t>
@@ -3929,14 +3633,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B15" s="159" t="inlineStr"/>
-      <c r="C15" s="159" t="inlineStr"/>
-      <c r="D15" s="159" t="inlineStr">
+      <c r="B15" s="183" t="inlineStr"/>
+      <c r="C15" s="183" t="inlineStr"/>
+      <c r="D15" s="183" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="E15" s="159" t="inlineStr"/>
+      <c r="E15" s="183" t="inlineStr"/>
       <c r="F15" s="126" t="inlineStr">
         <is>
           <t>Research: Setup deadline (registration, prescreening, contacts)</t>
@@ -3949,14 +3653,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B16" s="159" t="inlineStr"/>
-      <c r="C16" s="159" t="inlineStr">
+      <c r="B16" s="183" t="inlineStr"/>
+      <c r="C16" s="183" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="D16" s="159" t="inlineStr"/>
-      <c r="E16" s="159" t="inlineStr"/>
+      <c r="D16" s="183" t="inlineStr"/>
+      <c r="E16" s="183" t="inlineStr"/>
       <c r="F16" s="126" t="inlineStr">
         <is>
           <t>Research: Study invitations begin (after setup)</t>
@@ -3969,14 +3673,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B17" s="159" t="inlineStr"/>
-      <c r="C17" s="159" t="inlineStr"/>
-      <c r="D17" s="159" t="inlineStr">
+      <c r="B17" s="183" t="inlineStr"/>
+      <c r="C17" s="183" t="inlineStr"/>
+      <c r="D17" s="183" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E17" s="159" t="inlineStr"/>
+      <c r="E17" s="183" t="inlineStr"/>
       <c r="F17" s="126" t="inlineStr">
         <is>
           <t>Research: Employee contact surveys sent</t>
@@ -3989,14 +3693,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B18" s="159" t="inlineStr"/>
-      <c r="C18" s="159" t="inlineStr"/>
-      <c r="D18" s="159" t="inlineStr">
+      <c r="B18" s="183" t="inlineStr"/>
+      <c r="C18" s="183" t="inlineStr"/>
+      <c r="D18" s="183" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E18" s="159" t="inlineStr"/>
+      <c r="E18" s="183" t="inlineStr"/>
       <c r="F18" s="126" t="inlineStr">
         <is>
           <t>Research: Complete 2.0 research credits</t>
@@ -4009,22 +3713,22 @@
           <t>Midterm Exam</t>
         </is>
       </c>
-      <c r="B19" s="157" t="inlineStr">
+      <c r="B19" s="181" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C19" s="158" t="inlineStr">
+      <c r="C19" s="182" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D19" s="158" t="inlineStr">
+      <c r="D19" s="182" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E19" s="158" t="inlineStr">
+      <c r="E19" s="182" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4040,18 +3744,18 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B20" s="159" t="inlineStr"/>
-      <c r="C20" s="159" t="inlineStr">
+      <c r="B20" s="183" t="inlineStr"/>
+      <c r="C20" s="183" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D20" s="159" t="inlineStr">
+      <c r="D20" s="183" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E20" s="159" t="inlineStr"/>
+      <c r="E20" s="183" t="inlineStr"/>
       <c r="F20" s="126" t="inlineStr">
         <is>
           <t>Midterm Exam</t>
@@ -4064,22 +3768,22 @@
           <t>Team Project Paper</t>
         </is>
       </c>
-      <c r="B21" s="157" t="inlineStr">
+      <c r="B21" s="181" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C21" s="160" t="inlineStr">
+      <c r="C21" s="184" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D21" s="160" t="inlineStr">
+      <c r="D21" s="184" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E21" s="160" t="inlineStr">
+      <c r="E21" s="184" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4095,18 +3799,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B22" s="159" t="inlineStr"/>
-      <c r="C22" s="159" t="inlineStr">
+      <c r="B22" s="183" t="inlineStr"/>
+      <c r="C22" s="183" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D22" s="159" t="inlineStr">
+      <c r="D22" s="183" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E22" s="159" t="inlineStr"/>
+      <c r="E22" s="183" t="inlineStr"/>
       <c r="F22" s="126" t="inlineStr">
         <is>
           <t>Team project outline</t>
@@ -4119,18 +3823,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B23" s="159" t="inlineStr"/>
-      <c r="C23" s="159" t="inlineStr">
+      <c r="B23" s="183" t="inlineStr"/>
+      <c r="C23" s="183" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D23" s="159" t="inlineStr">
+      <c r="D23" s="183" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E23" s="159" t="inlineStr"/>
+      <c r="E23" s="183" t="inlineStr"/>
       <c r="F23" s="126" t="inlineStr">
         <is>
           <t>Team project paper</t>
@@ -4143,22 +3847,22 @@
           <t>Final Reflection Paper</t>
         </is>
       </c>
-      <c r="B24" s="157" t="inlineStr">
+      <c r="B24" s="181" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C24" s="158" t="inlineStr">
+      <c r="C24" s="182" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D24" s="158" t="inlineStr">
+      <c r="D24" s="182" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E24" s="158" t="inlineStr">
+      <c r="E24" s="182" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4174,18 +3878,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B25" s="159" t="inlineStr"/>
-      <c r="C25" s="159" t="inlineStr">
+      <c r="B25" s="183" t="inlineStr"/>
+      <c r="C25" s="183" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D25" s="159" t="inlineStr">
+      <c r="D25" s="183" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E25" s="159" t="inlineStr"/>
+      <c r="E25" s="183" t="inlineStr"/>
       <c r="F25" s="126" t="inlineStr">
         <is>
           <t>Personal Reflection Paper</t>
@@ -4198,22 +3902,22 @@
           <t>Presentation</t>
         </is>
       </c>
-      <c r="B26" s="157" t="inlineStr">
+      <c r="B26" s="181" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C26" s="160" t="inlineStr">
+      <c r="C26" s="184" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D26" s="160" t="inlineStr">
+      <c r="D26" s="184" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E26" s="160" t="inlineStr">
+      <c r="E26" s="184" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4229,18 +3933,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B27" s="159" t="inlineStr"/>
-      <c r="C27" s="159" t="inlineStr">
+      <c r="B27" s="183" t="inlineStr"/>
+      <c r="C27" s="183" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D27" s="159" t="inlineStr">
+      <c r="D27" s="183" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E27" s="159" t="inlineStr"/>
+      <c r="E27" s="183" t="inlineStr"/>
       <c r="F27" s="126" t="inlineStr">
         <is>
           <t>Presentation slides</t>
@@ -4253,22 +3957,22 @@
           <t>Case Analysis Assignments</t>
         </is>
       </c>
-      <c r="B28" s="157" t="inlineStr">
+      <c r="B28" s="181" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C28" s="158" t="inlineStr">
+      <c r="C28" s="182" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D28" s="158" t="inlineStr">
+      <c r="D28" s="182" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E28" s="158" t="inlineStr">
+      <c r="E28" s="182" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4284,18 +3988,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B29" s="159" t="inlineStr"/>
-      <c r="C29" s="159" t="inlineStr">
+      <c r="B29" s="183" t="inlineStr"/>
+      <c r="C29" s="183" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D29" s="159" t="inlineStr">
+      <c r="D29" s="183" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E29" s="159" t="inlineStr"/>
+      <c r="E29" s="183" t="inlineStr"/>
       <c r="F29" s="126" t="inlineStr">
         <is>
           <t>Thomas Green Case Analysis Memo</t>
@@ -4308,18 +4012,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B30" s="159" t="inlineStr"/>
-      <c r="C30" s="159" t="inlineStr">
+      <c r="B30" s="183" t="inlineStr"/>
+      <c r="C30" s="183" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D30" s="159" t="inlineStr">
+      <c r="D30" s="183" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E30" s="159" t="inlineStr"/>
+      <c r="E30" s="183" t="inlineStr"/>
       <c r="F30" s="126" t="inlineStr">
         <is>
           <t>SkillsForTomorrow Analysis Memo</t>
@@ -4332,22 +4036,22 @@
           <t>Proposal &amp; Team Contract</t>
         </is>
       </c>
-      <c r="B31" s="157" t="inlineStr">
+      <c r="B31" s="181" t="inlineStr">
         <is>
           <t>3%</t>
         </is>
       </c>
-      <c r="C31" s="160" t="inlineStr">
+      <c r="C31" s="184" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D31" s="160" t="inlineStr">
+      <c r="D31" s="184" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E31" s="160" t="inlineStr">
+      <c r="E31" s="184" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4363,18 +4067,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B32" s="159" t="inlineStr"/>
-      <c r="C32" s="159" t="inlineStr">
+      <c r="B32" s="183" t="inlineStr"/>
+      <c r="C32" s="183" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D32" s="159" t="inlineStr">
+      <c r="D32" s="183" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E32" s="159" t="inlineStr"/>
+      <c r="E32" s="183" t="inlineStr"/>
       <c r="F32" s="126" t="inlineStr">
         <is>
           <t>Team project proposal &amp; team contract</t>
@@ -4387,22 +4091,22 @@
           <t>Self &amp; Peer Evaluation</t>
         </is>
       </c>
-      <c r="B33" s="157" t="inlineStr">
+      <c r="B33" s="181" t="inlineStr">
         <is>
           <t>2%</t>
         </is>
       </c>
-      <c r="C33" s="158" t="inlineStr">
+      <c r="C33" s="182" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D33" s="158" t="inlineStr">
+      <c r="D33" s="182" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E33" s="158" t="inlineStr">
+      <c r="E33" s="182" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4418,18 +4122,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B34" s="159" t="inlineStr"/>
-      <c r="C34" s="159" t="inlineStr">
+      <c r="B34" s="183" t="inlineStr"/>
+      <c r="C34" s="183" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D34" s="159" t="inlineStr">
+      <c r="D34" s="183" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E34" s="159" t="inlineStr"/>
+      <c r="E34" s="183" t="inlineStr"/>
       <c r="F34" s="126" t="inlineStr">
         <is>
           <t>Self &amp; peer evaluation</t>
@@ -4442,22 +4146,22 @@
           <t>Personal Assessments (Connect)</t>
         </is>
       </c>
-      <c r="B35" s="157" t="inlineStr">
+      <c r="B35" s="181" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C35" s="160" t="inlineStr">
+      <c r="C35" s="184" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D35" s="160" t="inlineStr">
+      <c r="D35" s="184" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E35" s="160" t="inlineStr">
+      <c r="E35" s="184" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4473,18 +4177,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B36" s="159" t="inlineStr"/>
-      <c r="C36" s="159" t="inlineStr">
+      <c r="B36" s="183" t="inlineStr"/>
+      <c r="C36" s="183" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D36" s="159" t="inlineStr">
+      <c r="D36" s="183" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="E36" s="159" t="inlineStr"/>
+      <c r="E36" s="183" t="inlineStr"/>
       <c r="F36" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
@@ -4497,18 +4201,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B37" s="159" t="inlineStr"/>
-      <c r="C37" s="159" t="inlineStr">
+      <c r="B37" s="183" t="inlineStr"/>
+      <c r="C37" s="183" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D37" s="159" t="inlineStr">
+      <c r="D37" s="183" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="E37" s="159" t="inlineStr"/>
+      <c r="E37" s="183" t="inlineStr"/>
       <c r="F37" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
@@ -4521,18 +4225,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B38" s="159" t="inlineStr"/>
-      <c r="C38" s="159" t="inlineStr">
+      <c r="B38" s="183" t="inlineStr"/>
+      <c r="C38" s="183" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="D38" s="159" t="inlineStr">
+      <c r="D38" s="183" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="E38" s="159" t="inlineStr"/>
+      <c r="E38" s="183" t="inlineStr"/>
       <c r="F38" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 5.01 - Assessing Your</t>
@@ -4545,14 +4249,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B39" s="159" t="inlineStr"/>
-      <c r="C39" s="159" t="inlineStr"/>
-      <c r="D39" s="159" t="inlineStr">
+      <c r="B39" s="183" t="inlineStr"/>
+      <c r="C39" s="183" t="inlineStr"/>
+      <c r="D39" s="183" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E39" s="159" t="inlineStr"/>
+      <c r="E39" s="183" t="inlineStr"/>
       <c r="F39" s="126" t="inlineStr">
         <is>
           <t>Connect: Sharpen Companion</t>
@@ -4565,18 +4269,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B40" s="159" t="inlineStr"/>
-      <c r="C40" s="159" t="inlineStr">
+      <c r="B40" s="183" t="inlineStr"/>
+      <c r="C40" s="183" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="D40" s="159" t="inlineStr">
+      <c r="D40" s="183" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="E40" s="159" t="inlineStr"/>
+      <c r="E40" s="183" t="inlineStr"/>
       <c r="F40" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 11.01 - What is my</t>
@@ -4589,18 +4293,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B41" s="159" t="inlineStr"/>
-      <c r="C41" s="159" t="inlineStr">
+      <c r="B41" s="183" t="inlineStr"/>
+      <c r="C41" s="183" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="D41" s="159" t="inlineStr">
+      <c r="D41" s="183" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="E41" s="159" t="inlineStr"/>
+      <c r="E41" s="183" t="inlineStr"/>
       <c r="F41" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 11.02 - What is my</t>
@@ -4613,18 +4317,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B42" s="159" t="inlineStr"/>
-      <c r="C42" s="159" t="inlineStr">
+      <c r="B42" s="183" t="inlineStr"/>
+      <c r="C42" s="183" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="D42" s="159" t="inlineStr">
+      <c r="D42" s="183" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E42" s="159" t="inlineStr"/>
+      <c r="E42" s="183" t="inlineStr"/>
       <c r="F42" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 12.01 - What kind of</t>
@@ -4637,18 +4341,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B43" s="159" t="inlineStr"/>
-      <c r="C43" s="159" t="inlineStr">
+      <c r="B43" s="183" t="inlineStr"/>
+      <c r="C43" s="183" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="D43" s="159" t="inlineStr">
+      <c r="D43" s="183" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E43" s="159" t="inlineStr"/>
+      <c r="E43" s="183" t="inlineStr"/>
       <c r="F43" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 10.5 - Preferred Conflict</t>
@@ -4661,18 +4365,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B44" s="159" t="inlineStr"/>
-      <c r="C44" s="159" t="inlineStr">
+      <c r="B44" s="183" t="inlineStr"/>
+      <c r="C44" s="183" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="D44" s="159" t="inlineStr">
+      <c r="D44" s="183" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E44" s="159" t="inlineStr"/>
+      <c r="E44" s="183" t="inlineStr"/>
       <c r="F44" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 9.01 - Assessing My</t>
@@ -4685,18 +4389,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B45" s="159" t="inlineStr"/>
-      <c r="C45" s="159" t="inlineStr">
+      <c r="B45" s="183" t="inlineStr"/>
+      <c r="C45" s="183" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="D45" s="159" t="inlineStr">
+      <c r="D45" s="183" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E45" s="159" t="inlineStr"/>
+      <c r="E45" s="183" t="inlineStr"/>
       <c r="F45" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 8.01 - Group</t>
@@ -4709,18 +4413,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B46" s="159" t="inlineStr"/>
-      <c r="C46" s="159" t="inlineStr">
+      <c r="B46" s="183" t="inlineStr"/>
+      <c r="C46" s="183" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="D46" s="159" t="inlineStr">
+      <c r="D46" s="183" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="E46" s="159" t="inlineStr"/>
+      <c r="E46" s="183" t="inlineStr"/>
       <c r="F46" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 14.02 - What Type of Organizational Culture Do I</t>
@@ -4733,18 +4437,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B47" s="159" t="inlineStr"/>
-      <c r="C47" s="159" t="inlineStr">
+      <c r="B47" s="183" t="inlineStr"/>
+      <c r="C47" s="183" t="inlineStr">
         <is>
           <t>2026-11-30</t>
         </is>
       </c>
-      <c r="D47" s="159" t="inlineStr">
+      <c r="D47" s="183" t="inlineStr">
         <is>
           <t>2026-11-30</t>
         </is>
       </c>
-      <c r="E47" s="159" t="inlineStr"/>
+      <c r="E47" s="183" t="inlineStr"/>
       <c r="F47" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 16.02 - What Is Your</t>
@@ -4757,18 +4461,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B48" s="159" t="inlineStr"/>
-      <c r="C48" s="159" t="inlineStr">
+      <c r="B48" s="183" t="inlineStr"/>
+      <c r="C48" s="183" t="inlineStr">
         <is>
           <t>2026-11-30</t>
         </is>
       </c>
-      <c r="D48" s="159" t="inlineStr">
+      <c r="D48" s="183" t="inlineStr">
         <is>
           <t>2026-11-30</t>
         </is>
       </c>
-      <c r="E48" s="159" t="inlineStr"/>
+      <c r="E48" s="183" t="inlineStr"/>
       <c r="F48" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 16.03 - Assessing Your</t>
@@ -4781,14 +4485,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B49" s="159" t="inlineStr"/>
-      <c r="C49" s="159" t="inlineStr"/>
-      <c r="D49" s="159" t="inlineStr">
+      <c r="B49" s="183" t="inlineStr"/>
+      <c r="C49" s="183" t="inlineStr"/>
+      <c r="D49" s="183" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E49" s="159" t="inlineStr"/>
+      <c r="E49" s="183" t="inlineStr"/>
       <c r="F49" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 12.02 - Which influence</t>

</xml_diff>

<commit_message>
BUAD-304 Connect: due date only, blank start date
Connect self-assessments list a class-session due date in the schedule,
not a separate start. Start Date column now blank; Due Date keeps session date.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -251,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="185">
+  <cellXfs count="189">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -781,6 +781,18 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -3507,22 +3519,22 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B10" s="181" t="inlineStr">
+      <c r="B10" s="185" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="C10" s="182" t="inlineStr">
+      <c r="C10" s="186" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D10" s="182" t="inlineStr">
+      <c r="D10" s="186" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E10" s="182" t="inlineStr">
+      <c r="E10" s="186" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3538,18 +3550,18 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B11" s="183" t="inlineStr"/>
-      <c r="C11" s="183" t="inlineStr">
+      <c r="B11" s="187" t="inlineStr"/>
+      <c r="C11" s="187" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D11" s="183" t="inlineStr">
+      <c r="D11" s="187" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E11" s="183" t="inlineStr"/>
+      <c r="E11" s="187" t="inlineStr"/>
       <c r="F11" s="126" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -3562,22 +3574,22 @@
           <t>Participation</t>
         </is>
       </c>
-      <c r="B12" s="181" t="inlineStr">
+      <c r="B12" s="185" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C12" s="184" t="inlineStr">
+      <c r="C12" s="188" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D12" s="184" t="inlineStr">
+      <c r="D12" s="188" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E12" s="184" t="inlineStr">
+      <c r="E12" s="188" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3593,14 +3605,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B13" s="183" t="inlineStr"/>
-      <c r="C13" s="183" t="inlineStr">
+      <c r="B13" s="187" t="inlineStr"/>
+      <c r="C13" s="187" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D13" s="183" t="inlineStr"/>
-      <c r="E13" s="183" t="inlineStr"/>
+      <c r="D13" s="187" t="inlineStr"/>
+      <c r="E13" s="187" t="inlineStr"/>
       <c r="F13" s="126" t="inlineStr">
         <is>
           <t>Research: SONA registration opens</t>
@@ -3613,14 +3625,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B14" s="183" t="inlineStr"/>
-      <c r="C14" s="183" t="inlineStr">
+      <c r="B14" s="187" t="inlineStr"/>
+      <c r="C14" s="187" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="D14" s="183" t="inlineStr"/>
-      <c r="E14" s="183" t="inlineStr"/>
+      <c r="D14" s="187" t="inlineStr"/>
+      <c r="E14" s="187" t="inlineStr"/>
       <c r="F14" s="126" t="inlineStr">
         <is>
           <t>Research: Prescreening questionnaire opens</t>
@@ -3633,14 +3645,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B15" s="183" t="inlineStr"/>
-      <c r="C15" s="183" t="inlineStr"/>
-      <c r="D15" s="183" t="inlineStr">
+      <c r="B15" s="187" t="inlineStr"/>
+      <c r="C15" s="187" t="inlineStr"/>
+      <c r="D15" s="187" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="E15" s="183" t="inlineStr"/>
+      <c r="E15" s="187" t="inlineStr"/>
       <c r="F15" s="126" t="inlineStr">
         <is>
           <t>Research: Setup deadline (registration, prescreening, contacts)</t>
@@ -3653,14 +3665,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B16" s="183" t="inlineStr"/>
-      <c r="C16" s="183" t="inlineStr">
+      <c r="B16" s="187" t="inlineStr"/>
+      <c r="C16" s="187" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="D16" s="183" t="inlineStr"/>
-      <c r="E16" s="183" t="inlineStr"/>
+      <c r="D16" s="187" t="inlineStr"/>
+      <c r="E16" s="187" t="inlineStr"/>
       <c r="F16" s="126" t="inlineStr">
         <is>
           <t>Research: Study invitations begin (after setup)</t>
@@ -3673,14 +3685,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B17" s="183" t="inlineStr"/>
-      <c r="C17" s="183" t="inlineStr"/>
-      <c r="D17" s="183" t="inlineStr">
+      <c r="B17" s="187" t="inlineStr"/>
+      <c r="C17" s="187" t="inlineStr"/>
+      <c r="D17" s="187" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E17" s="183" t="inlineStr"/>
+      <c r="E17" s="187" t="inlineStr"/>
       <c r="F17" s="126" t="inlineStr">
         <is>
           <t>Research: Employee contact surveys sent</t>
@@ -3693,14 +3705,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B18" s="183" t="inlineStr"/>
-      <c r="C18" s="183" t="inlineStr"/>
-      <c r="D18" s="183" t="inlineStr">
+      <c r="B18" s="187" t="inlineStr"/>
+      <c r="C18" s="187" t="inlineStr"/>
+      <c r="D18" s="187" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E18" s="183" t="inlineStr"/>
+      <c r="E18" s="187" t="inlineStr"/>
       <c r="F18" s="126" t="inlineStr">
         <is>
           <t>Research: Complete 2.0 research credits</t>
@@ -3713,22 +3725,22 @@
           <t>Midterm Exam</t>
         </is>
       </c>
-      <c r="B19" s="181" t="inlineStr">
+      <c r="B19" s="185" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C19" s="182" t="inlineStr">
+      <c r="C19" s="186" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D19" s="182" t="inlineStr">
+      <c r="D19" s="186" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E19" s="182" t="inlineStr">
+      <c r="E19" s="186" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3744,18 +3756,18 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B20" s="183" t="inlineStr"/>
-      <c r="C20" s="183" t="inlineStr">
+      <c r="B20" s="187" t="inlineStr"/>
+      <c r="C20" s="187" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D20" s="183" t="inlineStr">
+      <c r="D20" s="187" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E20" s="183" t="inlineStr"/>
+      <c r="E20" s="187" t="inlineStr"/>
       <c r="F20" s="126" t="inlineStr">
         <is>
           <t>Midterm Exam</t>
@@ -3768,22 +3780,22 @@
           <t>Team Project Paper</t>
         </is>
       </c>
-      <c r="B21" s="181" t="inlineStr">
+      <c r="B21" s="185" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C21" s="184" t="inlineStr">
+      <c r="C21" s="188" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D21" s="184" t="inlineStr">
+      <c r="D21" s="188" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E21" s="184" t="inlineStr">
+      <c r="E21" s="188" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3799,18 +3811,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B22" s="183" t="inlineStr"/>
-      <c r="C22" s="183" t="inlineStr">
+      <c r="B22" s="187" t="inlineStr"/>
+      <c r="C22" s="187" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D22" s="183" t="inlineStr">
+      <c r="D22" s="187" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E22" s="183" t="inlineStr"/>
+      <c r="E22" s="187" t="inlineStr"/>
       <c r="F22" s="126" t="inlineStr">
         <is>
           <t>Team project outline</t>
@@ -3823,18 +3835,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B23" s="183" t="inlineStr"/>
-      <c r="C23" s="183" t="inlineStr">
+      <c r="B23" s="187" t="inlineStr"/>
+      <c r="C23" s="187" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D23" s="183" t="inlineStr">
+      <c r="D23" s="187" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E23" s="183" t="inlineStr"/>
+      <c r="E23" s="187" t="inlineStr"/>
       <c r="F23" s="126" t="inlineStr">
         <is>
           <t>Team project paper</t>
@@ -3847,22 +3859,22 @@
           <t>Final Reflection Paper</t>
         </is>
       </c>
-      <c r="B24" s="181" t="inlineStr">
+      <c r="B24" s="185" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C24" s="182" t="inlineStr">
+      <c r="C24" s="186" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D24" s="182" t="inlineStr">
+      <c r="D24" s="186" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E24" s="182" t="inlineStr">
+      <c r="E24" s="186" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3878,18 +3890,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B25" s="183" t="inlineStr"/>
-      <c r="C25" s="183" t="inlineStr">
+      <c r="B25" s="187" t="inlineStr"/>
+      <c r="C25" s="187" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D25" s="183" t="inlineStr">
+      <c r="D25" s="187" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E25" s="183" t="inlineStr"/>
+      <c r="E25" s="187" t="inlineStr"/>
       <c r="F25" s="126" t="inlineStr">
         <is>
           <t>Personal Reflection Paper</t>
@@ -3902,22 +3914,22 @@
           <t>Presentation</t>
         </is>
       </c>
-      <c r="B26" s="181" t="inlineStr">
+      <c r="B26" s="185" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C26" s="184" t="inlineStr">
+      <c r="C26" s="188" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D26" s="184" t="inlineStr">
+      <c r="D26" s="188" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E26" s="184" t="inlineStr">
+      <c r="E26" s="188" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3933,18 +3945,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B27" s="183" t="inlineStr"/>
-      <c r="C27" s="183" t="inlineStr">
+      <c r="B27" s="187" t="inlineStr"/>
+      <c r="C27" s="187" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D27" s="183" t="inlineStr">
+      <c r="D27" s="187" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E27" s="183" t="inlineStr"/>
+      <c r="E27" s="187" t="inlineStr"/>
       <c r="F27" s="126" t="inlineStr">
         <is>
           <t>Presentation slides</t>
@@ -3957,22 +3969,22 @@
           <t>Case Analysis Assignments</t>
         </is>
       </c>
-      <c r="B28" s="181" t="inlineStr">
+      <c r="B28" s="185" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C28" s="182" t="inlineStr">
+      <c r="C28" s="186" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D28" s="182" t="inlineStr">
+      <c r="D28" s="186" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E28" s="182" t="inlineStr">
+      <c r="E28" s="186" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3988,18 +4000,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B29" s="183" t="inlineStr"/>
-      <c r="C29" s="183" t="inlineStr">
+      <c r="B29" s="187" t="inlineStr"/>
+      <c r="C29" s="187" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D29" s="183" t="inlineStr">
+      <c r="D29" s="187" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E29" s="183" t="inlineStr"/>
+      <c r="E29" s="187" t="inlineStr"/>
       <c r="F29" s="126" t="inlineStr">
         <is>
           <t>Thomas Green Case Analysis Memo</t>
@@ -4012,18 +4024,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B30" s="183" t="inlineStr"/>
-      <c r="C30" s="183" t="inlineStr">
+      <c r="B30" s="187" t="inlineStr"/>
+      <c r="C30" s="187" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D30" s="183" t="inlineStr">
+      <c r="D30" s="187" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E30" s="183" t="inlineStr"/>
+      <c r="E30" s="187" t="inlineStr"/>
       <c r="F30" s="126" t="inlineStr">
         <is>
           <t>SkillsForTomorrow Analysis Memo</t>
@@ -4036,22 +4048,22 @@
           <t>Proposal &amp; Team Contract</t>
         </is>
       </c>
-      <c r="B31" s="181" t="inlineStr">
+      <c r="B31" s="185" t="inlineStr">
         <is>
           <t>3%</t>
         </is>
       </c>
-      <c r="C31" s="184" t="inlineStr">
+      <c r="C31" s="188" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D31" s="184" t="inlineStr">
+      <c r="D31" s="188" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E31" s="184" t="inlineStr">
+      <c r="E31" s="188" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4067,18 +4079,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B32" s="183" t="inlineStr"/>
-      <c r="C32" s="183" t="inlineStr">
+      <c r="B32" s="187" t="inlineStr"/>
+      <c r="C32" s="187" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D32" s="183" t="inlineStr">
+      <c r="D32" s="187" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E32" s="183" t="inlineStr"/>
+      <c r="E32" s="187" t="inlineStr"/>
       <c r="F32" s="126" t="inlineStr">
         <is>
           <t>Team project proposal &amp; team contract</t>
@@ -4091,22 +4103,22 @@
           <t>Self &amp; Peer Evaluation</t>
         </is>
       </c>
-      <c r="B33" s="181" t="inlineStr">
+      <c r="B33" s="185" t="inlineStr">
         <is>
           <t>2%</t>
         </is>
       </c>
-      <c r="C33" s="182" t="inlineStr">
+      <c r="C33" s="186" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D33" s="182" t="inlineStr">
+      <c r="D33" s="186" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E33" s="182" t="inlineStr">
+      <c r="E33" s="186" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4122,18 +4134,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B34" s="183" t="inlineStr"/>
-      <c r="C34" s="183" t="inlineStr">
+      <c r="B34" s="187" t="inlineStr"/>
+      <c r="C34" s="187" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D34" s="183" t="inlineStr">
+      <c r="D34" s="187" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E34" s="183" t="inlineStr"/>
+      <c r="E34" s="187" t="inlineStr"/>
       <c r="F34" s="126" t="inlineStr">
         <is>
           <t>Self &amp; peer evaluation</t>
@@ -4146,22 +4158,22 @@
           <t>Personal Assessments (Connect)</t>
         </is>
       </c>
-      <c r="B35" s="181" t="inlineStr">
+      <c r="B35" s="185" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C35" s="184" t="inlineStr">
+      <c r="C35" s="188" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D35" s="184" t="inlineStr">
+      <c r="D35" s="188" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E35" s="184" t="inlineStr">
+      <c r="E35" s="188" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4177,18 +4189,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B36" s="183" t="inlineStr"/>
-      <c r="C36" s="183" t="inlineStr">
+      <c r="B36" s="187" t="inlineStr"/>
+      <c r="C36" s="187" t="inlineStr"/>
+      <c r="D36" s="187" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D36" s="183" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="E36" s="183" t="inlineStr"/>
+      <c r="E36" s="187" t="inlineStr"/>
       <c r="F36" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
@@ -4201,18 +4209,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B37" s="183" t="inlineStr"/>
-      <c r="C37" s="183" t="inlineStr">
+      <c r="B37" s="187" t="inlineStr"/>
+      <c r="C37" s="187" t="inlineStr"/>
+      <c r="D37" s="187" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D37" s="183" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="E37" s="183" t="inlineStr"/>
+      <c r="E37" s="187" t="inlineStr"/>
       <c r="F37" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
@@ -4225,18 +4229,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B38" s="183" t="inlineStr"/>
-      <c r="C38" s="183" t="inlineStr">
+      <c r="B38" s="187" t="inlineStr"/>
+      <c r="C38" s="187" t="inlineStr"/>
+      <c r="D38" s="187" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="D38" s="183" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="E38" s="183" t="inlineStr"/>
+      <c r="E38" s="187" t="inlineStr"/>
       <c r="F38" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 5.01 - Assessing Your</t>
@@ -4249,14 +4249,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B39" s="183" t="inlineStr"/>
-      <c r="C39" s="183" t="inlineStr"/>
-      <c r="D39" s="183" t="inlineStr">
+      <c r="B39" s="187" t="inlineStr"/>
+      <c r="C39" s="187" t="inlineStr"/>
+      <c r="D39" s="187" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E39" s="183" t="inlineStr"/>
+      <c r="E39" s="187" t="inlineStr"/>
       <c r="F39" s="126" t="inlineStr">
         <is>
           <t>Connect: Sharpen Companion</t>
@@ -4269,18 +4269,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B40" s="183" t="inlineStr"/>
-      <c r="C40" s="183" t="inlineStr">
+      <c r="B40" s="187" t="inlineStr"/>
+      <c r="C40" s="187" t="inlineStr"/>
+      <c r="D40" s="187" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="D40" s="183" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="E40" s="183" t="inlineStr"/>
+      <c r="E40" s="187" t="inlineStr"/>
       <c r="F40" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 11.01 - What is my</t>
@@ -4293,18 +4289,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B41" s="183" t="inlineStr"/>
-      <c r="C41" s="183" t="inlineStr">
+      <c r="B41" s="187" t="inlineStr"/>
+      <c r="C41" s="187" t="inlineStr"/>
+      <c r="D41" s="187" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="D41" s="183" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="E41" s="183" t="inlineStr"/>
+      <c r="E41" s="187" t="inlineStr"/>
       <c r="F41" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 11.02 - What is my</t>
@@ -4317,18 +4309,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B42" s="183" t="inlineStr"/>
-      <c r="C42" s="183" t="inlineStr">
+      <c r="B42" s="187" t="inlineStr"/>
+      <c r="C42" s="187" t="inlineStr"/>
+      <c r="D42" s="187" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="D42" s="183" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="E42" s="183" t="inlineStr"/>
+      <c r="E42" s="187" t="inlineStr"/>
       <c r="F42" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 12.01 - What kind of</t>
@@ -4341,18 +4329,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B43" s="183" t="inlineStr"/>
-      <c r="C43" s="183" t="inlineStr">
+      <c r="B43" s="187" t="inlineStr"/>
+      <c r="C43" s="187" t="inlineStr"/>
+      <c r="D43" s="187" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="D43" s="183" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E43" s="183" t="inlineStr"/>
+      <c r="E43" s="187" t="inlineStr"/>
       <c r="F43" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 10.5 - Preferred Conflict</t>
@@ -4365,18 +4349,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B44" s="183" t="inlineStr"/>
-      <c r="C44" s="183" t="inlineStr">
+      <c r="B44" s="187" t="inlineStr"/>
+      <c r="C44" s="187" t="inlineStr"/>
+      <c r="D44" s="187" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="D44" s="183" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E44" s="183" t="inlineStr"/>
+      <c r="E44" s="187" t="inlineStr"/>
       <c r="F44" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 9.01 - Assessing My</t>
@@ -4389,18 +4369,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B45" s="183" t="inlineStr"/>
-      <c r="C45" s="183" t="inlineStr">
+      <c r="B45" s="187" t="inlineStr"/>
+      <c r="C45" s="187" t="inlineStr"/>
+      <c r="D45" s="187" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="D45" s="183" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E45" s="183" t="inlineStr"/>
+      <c r="E45" s="187" t="inlineStr"/>
       <c r="F45" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 8.01 - Group</t>
@@ -4413,18 +4389,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B46" s="183" t="inlineStr"/>
-      <c r="C46" s="183" t="inlineStr">
+      <c r="B46" s="187" t="inlineStr"/>
+      <c r="C46" s="187" t="inlineStr"/>
+      <c r="D46" s="187" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="D46" s="183" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="E46" s="183" t="inlineStr"/>
+      <c r="E46" s="187" t="inlineStr"/>
       <c r="F46" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 14.02 - What Type of Organizational Culture Do I</t>
@@ -4437,18 +4409,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B47" s="183" t="inlineStr"/>
-      <c r="C47" s="183" t="inlineStr">
+      <c r="B47" s="187" t="inlineStr"/>
+      <c r="C47" s="187" t="inlineStr"/>
+      <c r="D47" s="187" t="inlineStr">
         <is>
           <t>2026-11-30</t>
         </is>
       </c>
-      <c r="D47" s="183" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
-      </c>
-      <c r="E47" s="183" t="inlineStr"/>
+      <c r="E47" s="187" t="inlineStr"/>
       <c r="F47" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 16.02 - What Is Your</t>
@@ -4461,18 +4429,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B48" s="183" t="inlineStr"/>
-      <c r="C48" s="183" t="inlineStr">
+      <c r="B48" s="187" t="inlineStr"/>
+      <c r="C48" s="187" t="inlineStr"/>
+      <c r="D48" s="187" t="inlineStr">
         <is>
           <t>2026-11-30</t>
         </is>
       </c>
-      <c r="D48" s="183" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
-      </c>
-      <c r="E48" s="183" t="inlineStr"/>
+      <c r="E48" s="187" t="inlineStr"/>
       <c r="F48" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 16.03 - Assessing Your</t>
@@ -4485,14 +4449,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B49" s="183" t="inlineStr"/>
-      <c r="C49" s="183" t="inlineStr"/>
-      <c r="D49" s="183" t="inlineStr">
+      <c r="B49" s="187" t="inlineStr"/>
+      <c r="C49" s="187" t="inlineStr"/>
+      <c r="D49" s="187" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E49" s="183" t="inlineStr"/>
+      <c r="E49" s="187" t="inlineStr"/>
       <c r="F49" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 12.02 - Which influence</t>

</xml_diff>

<commit_message>
Retrain: block start==due false detection across all parsers
- Add strip_false_start_when_same_as_due() in apply_start_date_cutoff()
- Calendar exam sub-rows: due only, blank start
- SKILL.md: corrected verified-start rules, Step 2 sanity check script
- reference.md: past error for start=due on calendar/Connect rows
- Regenerated all three class sheets; validation passes

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -251,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="189">
+  <cellXfs count="213">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -793,6 +793,78 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1290,18 +1362,18 @@
           <t>Sleep Paper</t>
         </is>
       </c>
-      <c r="B10" s="173" t="inlineStr">
+      <c r="B10" s="201" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C10" s="174" t="inlineStr"/>
-      <c r="D10" s="174" t="inlineStr">
+      <c r="C10" s="202" t="inlineStr"/>
+      <c r="D10" s="202" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="E10" s="174" t="inlineStr">
+      <c r="E10" s="202" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1317,14 +1389,14 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B11" s="175" t="inlineStr"/>
-      <c r="C11" s="175" t="inlineStr"/>
-      <c r="D11" s="175" t="inlineStr">
+      <c r="B11" s="203" t="inlineStr"/>
+      <c r="C11" s="203" t="inlineStr"/>
+      <c r="D11" s="203" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="E11" s="175" t="inlineStr"/>
+      <c r="E11" s="203" t="inlineStr"/>
       <c r="F11" s="99" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
@@ -1337,18 +1409,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B12" s="175" t="inlineStr"/>
-      <c r="C12" s="175" t="inlineStr">
+      <c r="B12" s="203" t="inlineStr"/>
+      <c r="C12" s="203" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D12" s="175" t="inlineStr">
+      <c r="D12" s="203" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E12" s="175" t="inlineStr"/>
+      <c r="E12" s="203" t="inlineStr"/>
       <c r="F12" s="99" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance</t>
@@ -1361,18 +1433,18 @@
           <t>Witchcraft Paper</t>
         </is>
       </c>
-      <c r="B13" s="173" t="inlineStr">
+      <c r="B13" s="201" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C13" s="176" t="inlineStr"/>
-      <c r="D13" s="176" t="inlineStr">
+      <c r="C13" s="204" t="inlineStr"/>
+      <c r="D13" s="204" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="E13" s="176" t="inlineStr">
+      <c r="E13" s="204" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1388,14 +1460,14 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B14" s="175" t="inlineStr"/>
-      <c r="C14" s="175" t="inlineStr"/>
-      <c r="D14" s="175" t="inlineStr">
+      <c r="B14" s="203" t="inlineStr"/>
+      <c r="C14" s="203" t="inlineStr"/>
+      <c r="D14" s="203" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="E14" s="175" t="inlineStr"/>
+      <c r="E14" s="203" t="inlineStr"/>
       <c r="F14" s="99" t="inlineStr">
         <is>
           <t>Witchcraft Paper Due</t>
@@ -1408,18 +1480,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B15" s="175" t="inlineStr"/>
-      <c r="C15" s="175" t="inlineStr">
+      <c r="B15" s="203" t="inlineStr"/>
+      <c r="C15" s="203" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D15" s="175" t="inlineStr">
+      <c r="D15" s="203" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E15" s="175" t="inlineStr"/>
+      <c r="E15" s="203" t="inlineStr"/>
       <c r="F15" s="99" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment</t>
@@ -1432,18 +1504,18 @@
           <t>Mid-term</t>
         </is>
       </c>
-      <c r="B16" s="173" t="inlineStr">
+      <c r="B16" s="201" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C16" s="174" t="inlineStr"/>
-      <c r="D16" s="174" t="inlineStr">
+      <c r="C16" s="202" t="inlineStr"/>
+      <c r="D16" s="202" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E16" s="174" t="inlineStr">
+      <c r="E16" s="202" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1459,14 +1531,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B17" s="175" t="inlineStr"/>
-      <c r="C17" s="175" t="inlineStr"/>
-      <c r="D17" s="175" t="inlineStr">
+      <c r="B17" s="203" t="inlineStr"/>
+      <c r="C17" s="203" t="inlineStr"/>
+      <c r="D17" s="203" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="E17" s="175" t="inlineStr"/>
+      <c r="E17" s="203" t="inlineStr"/>
       <c r="F17" s="99" t="inlineStr">
         <is>
           <t>Midterm Exam</t>
@@ -1479,18 +1551,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B18" s="175" t="inlineStr"/>
-      <c r="C18" s="175" t="inlineStr">
+      <c r="B18" s="203" t="inlineStr"/>
+      <c r="C18" s="203" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="D18" s="175" t="inlineStr">
+      <c r="D18" s="203" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E18" s="175" t="inlineStr"/>
+      <c r="E18" s="203" t="inlineStr"/>
       <c r="F18" s="99" t="inlineStr">
         <is>
           <t>Week Oct 6-9: Midterm &amp; Break</t>
@@ -1503,18 +1575,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B19" s="175" t="inlineStr"/>
-      <c r="C19" s="175" t="inlineStr">
+      <c r="B19" s="203" t="inlineStr"/>
+      <c r="C19" s="203" t="inlineStr">
         <is>
           <t>2026-12-01</t>
         </is>
       </c>
-      <c r="D19" s="175" t="inlineStr">
+      <c r="D19" s="203" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E19" s="175" t="inlineStr"/>
+      <c r="E19" s="203" t="inlineStr"/>
       <c r="F19" s="99" t="inlineStr">
         <is>
           <t>Week Dec 1-4: Modern Europe?</t>
@@ -1527,18 +1599,18 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B20" s="173" t="inlineStr">
+      <c r="B20" s="201" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C20" s="176" t="inlineStr"/>
-      <c r="D20" s="176" t="inlineStr">
+      <c r="C20" s="204" t="inlineStr"/>
+      <c r="D20" s="204" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="E20" s="176" t="inlineStr">
+      <c r="E20" s="204" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1554,14 +1626,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B21" s="175" t="inlineStr"/>
-      <c r="C21" s="175" t="inlineStr"/>
-      <c r="D21" s="175" t="inlineStr">
+      <c r="B21" s="203" t="inlineStr"/>
+      <c r="C21" s="203" t="inlineStr"/>
+      <c r="D21" s="203" t="inlineStr">
         <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="E21" s="175" t="inlineStr"/>
+      <c r="E21" s="203" t="inlineStr"/>
       <c r="F21" s="99" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -1574,18 +1646,18 @@
           <t>Discussion Section</t>
         </is>
       </c>
-      <c r="B22" s="173" t="inlineStr">
+      <c r="B22" s="201" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C22" s="174" t="inlineStr"/>
-      <c r="D22" s="174" t="inlineStr">
+      <c r="C22" s="202" t="inlineStr"/>
+      <c r="D22" s="202" t="inlineStr">
         <is>
           <t>2026-11-12</t>
         </is>
       </c>
-      <c r="E22" s="174" t="inlineStr">
+      <c r="E22" s="202" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1601,18 +1673,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B23" s="175" t="inlineStr"/>
-      <c r="C23" s="175" t="inlineStr">
+      <c r="B23" s="203" t="inlineStr"/>
+      <c r="C23" s="203" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D23" s="175" t="inlineStr">
+      <c r="D23" s="203" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E23" s="175" t="inlineStr"/>
+      <c r="E23" s="203" t="inlineStr"/>
       <c r="F23" s="99" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death</t>
@@ -1625,18 +1697,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B24" s="175" t="inlineStr"/>
-      <c r="C24" s="175" t="inlineStr">
+      <c r="B24" s="203" t="inlineStr"/>
+      <c r="C24" s="203" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D24" s="175" t="inlineStr">
+      <c r="D24" s="203" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E24" s="175" t="inlineStr"/>
+      <c r="E24" s="203" t="inlineStr"/>
       <c r="F24" s="99" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death - Section reading 1: -- 13 of 33 -- Lizzie Wade, “From Black Death to fatal flu, pas</t>
@@ -1649,18 +1721,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B25" s="175" t="inlineStr"/>
-      <c r="C25" s="175" t="inlineStr">
+      <c r="B25" s="203" t="inlineStr"/>
+      <c r="C25" s="203" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D25" s="175" t="inlineStr">
+      <c r="D25" s="203" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E25" s="175" t="inlineStr"/>
+      <c r="E25" s="203" t="inlineStr"/>
       <c r="F25" s="99" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life</t>
@@ -1673,18 +1745,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B26" s="175" t="inlineStr"/>
-      <c r="C26" s="175" t="inlineStr">
+      <c r="B26" s="203" t="inlineStr"/>
+      <c r="C26" s="203" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D26" s="175" t="inlineStr">
+      <c r="D26" s="203" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E26" s="175" t="inlineStr"/>
+      <c r="E26" s="203" t="inlineStr"/>
       <c r="F26" s="99" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life - Section reading 1: A Roger Ekirch, “Sleep we have lost: Pre-Industrial Slumber in the Brit</t>
@@ -1697,18 +1769,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B27" s="175" t="inlineStr"/>
-      <c r="C27" s="175" t="inlineStr">
+      <c r="B27" s="203" t="inlineStr"/>
+      <c r="C27" s="203" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D27" s="175" t="inlineStr">
+      <c r="D27" s="203" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E27" s="175" t="inlineStr"/>
+      <c r="E27" s="203" t="inlineStr"/>
       <c r="F27" s="99" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance</t>
@@ -1721,18 +1793,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B28" s="175" t="inlineStr"/>
-      <c r="C28" s="175" t="inlineStr">
+      <c r="B28" s="203" t="inlineStr"/>
+      <c r="C28" s="203" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D28" s="175" t="inlineStr">
+      <c r="D28" s="203" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E28" s="175" t="inlineStr"/>
+      <c r="E28" s="203" t="inlineStr"/>
       <c r="F28" s="99" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance - Section reading 1: -- 14 of 33 -- Kay Daly, “Diverting the Flood of History: Ada Palmer’s I</t>
@@ -1745,18 +1817,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B29" s="175" t="inlineStr"/>
-      <c r="C29" s="175" t="inlineStr">
+      <c r="B29" s="203" t="inlineStr"/>
+      <c r="C29" s="203" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D29" s="175" t="inlineStr">
+      <c r="D29" s="203" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E29" s="175" t="inlineStr"/>
+      <c r="E29" s="203" t="inlineStr"/>
       <c r="F29" s="99" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance - Section reading 1: Vasari, Lives of the Artists: Leonardo da Vinci &amp; Properzia de’ Rossi V</t>
@@ -1769,18 +1841,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B30" s="175" t="inlineStr"/>
-      <c r="C30" s="175" t="inlineStr">
+      <c r="B30" s="203" t="inlineStr"/>
+      <c r="C30" s="203" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D30" s="175" t="inlineStr">
+      <c r="D30" s="203" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E30" s="175" t="inlineStr"/>
+      <c r="E30" s="203" t="inlineStr"/>
       <c r="F30" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion</t>
@@ -1793,18 +1865,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B31" s="175" t="inlineStr"/>
-      <c r="C31" s="175" t="inlineStr">
+      <c r="B31" s="203" t="inlineStr"/>
+      <c r="C31" s="203" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D31" s="175" t="inlineStr">
+      <c r="D31" s="203" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E31" s="175" t="inlineStr"/>
+      <c r="E31" s="203" t="inlineStr"/>
       <c r="F31" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion - Section reading 1: Jerry Brotton, The Renaissance Bazaar, Chap 1 (15 pgs) Read Colu</t>
@@ -1817,18 +1889,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B32" s="175" t="inlineStr"/>
-      <c r="C32" s="175" t="inlineStr">
+      <c r="B32" s="203" t="inlineStr"/>
+      <c r="C32" s="203" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D32" s="175" t="inlineStr">
+      <c r="D32" s="203" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E32" s="175" t="inlineStr"/>
+      <c r="E32" s="203" t="inlineStr"/>
       <c r="F32" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion - Section reading 2: Bernal Diaz del Castillo, The True History of the Conquest of Ne</t>
@@ -1841,18 +1913,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B33" s="175" t="inlineStr"/>
-      <c r="C33" s="175" t="inlineStr">
+      <c r="B33" s="203" t="inlineStr"/>
+      <c r="C33" s="203" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="D33" s="175" t="inlineStr">
+      <c r="D33" s="203" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="E33" s="175" t="inlineStr"/>
+      <c r="E33" s="203" t="inlineStr"/>
       <c r="F33" s="99" t="inlineStr">
         <is>
           <t>Week Oct 13-16: The Reformation</t>
@@ -1865,18 +1937,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B34" s="175" t="inlineStr"/>
-      <c r="C34" s="175" t="inlineStr">
+      <c r="B34" s="203" t="inlineStr"/>
+      <c r="C34" s="203" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="D34" s="175" t="inlineStr">
+      <c r="D34" s="203" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="E34" s="175" t="inlineStr"/>
+      <c r="E34" s="203" t="inlineStr"/>
       <c r="F34" s="99" t="inlineStr">
         <is>
           <t>Week Oct 20-23: The Reformation</t>
@@ -1889,18 +1961,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B35" s="175" t="inlineStr"/>
-      <c r="C35" s="175" t="inlineStr">
+      <c r="B35" s="203" t="inlineStr"/>
+      <c r="C35" s="203" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D35" s="175" t="inlineStr">
+      <c r="D35" s="203" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E35" s="175" t="inlineStr"/>
+      <c r="E35" s="203" t="inlineStr"/>
       <c r="F35" s="99" t="inlineStr">
         <is>
           <t>Week Oct 27-30: Reformation</t>
@@ -1913,18 +1985,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B36" s="175" t="inlineStr"/>
-      <c r="C36" s="175" t="inlineStr">
+      <c r="B36" s="203" t="inlineStr"/>
+      <c r="C36" s="203" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D36" s="175" t="inlineStr">
+      <c r="D36" s="203" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E36" s="175" t="inlineStr"/>
+      <c r="E36" s="203" t="inlineStr"/>
       <c r="F36" s="99" t="inlineStr">
         <is>
           <t xml:space="preserve">Week Oct 27-30: Reformation - Section reading 1: Barbara Diefendorf, ed., The Saint Bartholomew’s Day Massacre: A Brief </t>
@@ -1937,18 +2009,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B37" s="175" t="inlineStr"/>
-      <c r="C37" s="175" t="inlineStr">
+      <c r="B37" s="203" t="inlineStr"/>
+      <c r="C37" s="203" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D37" s="175" t="inlineStr">
+      <c r="D37" s="203" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E37" s="175" t="inlineStr"/>
+      <c r="E37" s="203" t="inlineStr"/>
       <c r="F37" s="99" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science</t>
@@ -1961,18 +2033,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B38" s="175" t="inlineStr"/>
-      <c r="C38" s="175" t="inlineStr">
+      <c r="B38" s="203" t="inlineStr"/>
+      <c r="C38" s="203" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D38" s="175" t="inlineStr">
+      <c r="D38" s="203" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E38" s="175" t="inlineStr"/>
+      <c r="E38" s="203" t="inlineStr"/>
       <c r="F38" s="99" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science - Section reading 1: Brian Levack, The Witchcraft Sourcebook, Chaps 36-44, 46-47 103.Lev</t>
@@ -1985,18 +2057,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B39" s="175" t="inlineStr"/>
-      <c r="C39" s="175" t="inlineStr">
+      <c r="B39" s="203" t="inlineStr"/>
+      <c r="C39" s="203" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D39" s="175" t="inlineStr">
+      <c r="D39" s="203" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E39" s="175" t="inlineStr"/>
+      <c r="E39" s="203" t="inlineStr"/>
       <c r="F39" s="99" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment - Section reading 1: Excerpt: John Locke, Two Treatises of Government (1689) Excerpt: Rous</t>
@@ -2009,18 +2081,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B40" s="175" t="inlineStr"/>
-      <c r="C40" s="175" t="inlineStr">
+      <c r="B40" s="203" t="inlineStr"/>
+      <c r="C40" s="203" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D40" s="175" t="inlineStr">
+      <c r="D40" s="203" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E40" s="175" t="inlineStr"/>
+      <c r="E40" s="203" t="inlineStr"/>
       <c r="F40" s="99" t="inlineStr">
         <is>
           <t>Week Nov 17-20: Enlightenment</t>
@@ -2033,18 +2105,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B41" s="175" t="inlineStr"/>
-      <c r="C41" s="175" t="inlineStr">
+      <c r="B41" s="203" t="inlineStr"/>
+      <c r="C41" s="203" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D41" s="175" t="inlineStr">
+      <c r="D41" s="203" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E41" s="175" t="inlineStr"/>
+      <c r="E41" s="203" t="inlineStr"/>
       <c r="F41" s="99" t="inlineStr">
         <is>
           <t xml:space="preserve">Week Nov 17-20: Enlightenment - Section reading 1: Video: Africa &amp; Britain, A Forgotten History, Episode 2: Freedom (50 </t>
@@ -2057,18 +2129,18 @@
           <t>Identification Quizzes</t>
         </is>
       </c>
-      <c r="B42" s="173" t="inlineStr">
+      <c r="B42" s="201" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C42" s="176" t="inlineStr"/>
-      <c r="D42" s="176" t="inlineStr">
+      <c r="C42" s="204" t="inlineStr"/>
+      <c r="D42" s="204" t="inlineStr">
         <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="E42" s="176" t="inlineStr">
+      <c r="E42" s="204" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2084,18 +2156,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B43" s="175" t="inlineStr"/>
-      <c r="C43" s="175" t="inlineStr">
+      <c r="B43" s="203" t="inlineStr"/>
+      <c r="C43" s="203" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D43" s="175" t="inlineStr">
+      <c r="D43" s="203" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E43" s="175" t="inlineStr"/>
+      <c r="E43" s="203" t="inlineStr"/>
       <c r="F43" s="99" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death (lecture topics)</t>
@@ -2108,18 +2180,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B44" s="175" t="inlineStr"/>
-      <c r="C44" s="175" t="inlineStr">
+      <c r="B44" s="203" t="inlineStr"/>
+      <c r="C44" s="203" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D44" s="175" t="inlineStr">
+      <c r="D44" s="203" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E44" s="175" t="inlineStr"/>
+      <c r="E44" s="203" t="inlineStr"/>
       <c r="F44" s="99" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life (lecture topics)</t>
@@ -2132,18 +2204,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B45" s="175" t="inlineStr"/>
-      <c r="C45" s="175" t="inlineStr">
+      <c r="B45" s="203" t="inlineStr"/>
+      <c r="C45" s="203" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D45" s="175" t="inlineStr">
+      <c r="D45" s="203" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E45" s="175" t="inlineStr"/>
+      <c r="E45" s="203" t="inlineStr"/>
       <c r="F45" s="99" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance (lecture topics)</t>
@@ -2156,18 +2228,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B46" s="175" t="inlineStr"/>
-      <c r="C46" s="175" t="inlineStr">
+      <c r="B46" s="203" t="inlineStr"/>
+      <c r="C46" s="203" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D46" s="175" t="inlineStr">
+      <c r="D46" s="203" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E46" s="175" t="inlineStr"/>
+      <c r="E46" s="203" t="inlineStr"/>
       <c r="F46" s="99" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance (lecture topics)</t>
@@ -2180,18 +2252,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B47" s="175" t="inlineStr"/>
-      <c r="C47" s="175" t="inlineStr">
+      <c r="B47" s="203" t="inlineStr"/>
+      <c r="C47" s="203" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D47" s="175" t="inlineStr">
+      <c r="D47" s="203" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E47" s="175" t="inlineStr"/>
+      <c r="E47" s="203" t="inlineStr"/>
       <c r="F47" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion (lecture topics)</t>
@@ -2204,18 +2276,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B48" s="175" t="inlineStr"/>
-      <c r="C48" s="175" t="inlineStr">
+      <c r="B48" s="203" t="inlineStr"/>
+      <c r="C48" s="203" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="D48" s="175" t="inlineStr">
+      <c r="D48" s="203" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E48" s="175" t="inlineStr"/>
+      <c r="E48" s="203" t="inlineStr"/>
       <c r="F48" s="99" t="inlineStr">
         <is>
           <t>Week Oct 6-9: Midterm &amp; Break (lecture topics)</t>
@@ -2228,18 +2300,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B49" s="175" t="inlineStr"/>
-      <c r="C49" s="175" t="inlineStr">
+      <c r="B49" s="203" t="inlineStr"/>
+      <c r="C49" s="203" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="D49" s="175" t="inlineStr">
+      <c r="D49" s="203" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="E49" s="175" t="inlineStr"/>
+      <c r="E49" s="203" t="inlineStr"/>
       <c r="F49" s="99" t="inlineStr">
         <is>
           <t>Week Oct 13-16: The Reformation (lecture topics)</t>
@@ -2252,18 +2324,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B50" s="175" t="inlineStr"/>
-      <c r="C50" s="175" t="inlineStr">
+      <c r="B50" s="203" t="inlineStr"/>
+      <c r="C50" s="203" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="D50" s="175" t="inlineStr">
+      <c r="D50" s="203" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="E50" s="175" t="inlineStr"/>
+      <c r="E50" s="203" t="inlineStr"/>
       <c r="F50" s="99" t="inlineStr">
         <is>
           <t>Week Oct 20-23: The Reformation (lecture topics)</t>
@@ -2276,18 +2348,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B51" s="175" t="inlineStr"/>
-      <c r="C51" s="175" t="inlineStr">
+      <c r="B51" s="203" t="inlineStr"/>
+      <c r="C51" s="203" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D51" s="175" t="inlineStr">
+      <c r="D51" s="203" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E51" s="175" t="inlineStr"/>
+      <c r="E51" s="203" t="inlineStr"/>
       <c r="F51" s="99" t="inlineStr">
         <is>
           <t>Week Oct 27-30: Reformation (lecture topics)</t>
@@ -2300,18 +2372,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B52" s="175" t="inlineStr"/>
-      <c r="C52" s="175" t="inlineStr">
+      <c r="B52" s="203" t="inlineStr"/>
+      <c r="C52" s="203" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D52" s="175" t="inlineStr">
+      <c r="D52" s="203" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E52" s="175" t="inlineStr"/>
+      <c r="E52" s="203" t="inlineStr"/>
       <c r="F52" s="99" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science (lecture topics)</t>
@@ -2324,18 +2396,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B53" s="175" t="inlineStr"/>
-      <c r="C53" s="175" t="inlineStr">
+      <c r="B53" s="203" t="inlineStr"/>
+      <c r="C53" s="203" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D53" s="175" t="inlineStr">
+      <c r="D53" s="203" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E53" s="175" t="inlineStr"/>
+      <c r="E53" s="203" t="inlineStr"/>
       <c r="F53" s="99" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment (lecture topics)</t>
@@ -2348,18 +2420,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B54" s="175" t="inlineStr"/>
-      <c r="C54" s="175" t="inlineStr">
+      <c r="B54" s="203" t="inlineStr"/>
+      <c r="C54" s="203" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D54" s="175" t="inlineStr">
+      <c r="D54" s="203" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E54" s="175" t="inlineStr"/>
+      <c r="E54" s="203" t="inlineStr"/>
       <c r="F54" s="99" t="inlineStr">
         <is>
           <t>Week Nov 17-20: Enlightenment (lecture topics)</t>
@@ -2372,18 +2444,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B55" s="175" t="inlineStr"/>
-      <c r="C55" s="175" t="inlineStr">
+      <c r="B55" s="203" t="inlineStr"/>
+      <c r="C55" s="203" t="inlineStr">
         <is>
           <t>2026-12-01</t>
         </is>
       </c>
-      <c r="D55" s="175" t="inlineStr">
+      <c r="D55" s="203" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E55" s="175" t="inlineStr"/>
+      <c r="E55" s="203" t="inlineStr"/>
       <c r="F55" s="99" t="inlineStr">
         <is>
           <t>Week Dec 1-4: Modern Europe? (lecture topics)</t>
@@ -2396,18 +2468,18 @@
           <t>Extra Credit</t>
         </is>
       </c>
-      <c r="B56" s="173" t="inlineStr">
+      <c r="B56" s="201" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C56" s="174" t="inlineStr"/>
-      <c r="D56" s="174" t="inlineStr">
+      <c r="C56" s="202" t="inlineStr"/>
+      <c r="D56" s="202" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E56" s="174" t="inlineStr">
+      <c r="E56" s="202" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2564,18 +2636,18 @@
           <t>Midterm 1</t>
         </is>
       </c>
-      <c r="B10" s="177" t="inlineStr">
+      <c r="B10" s="205" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C10" s="178" t="inlineStr"/>
-      <c r="D10" s="178" t="inlineStr">
+      <c r="C10" s="206" t="inlineStr"/>
+      <c r="D10" s="206" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="E10" s="178" t="inlineStr">
+      <c r="E10" s="206" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2591,18 +2663,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B11" s="179" t="inlineStr"/>
-      <c r="C11" s="179" t="inlineStr">
+      <c r="B11" s="207" t="inlineStr"/>
+      <c r="C11" s="207" t="inlineStr"/>
+      <c r="D11" s="207" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="D11" s="179" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="E11" s="179" t="inlineStr"/>
+      <c r="E11" s="207" t="inlineStr"/>
       <c r="F11" s="112" t="inlineStr">
         <is>
           <t>9/30 Midterm 1: 250 Points Chapters 1, 2, 3, 4, 5, 8</t>
@@ -2615,18 +2683,18 @@
           <t>Midterm 2</t>
         </is>
       </c>
-      <c r="B12" s="177" t="inlineStr">
+      <c r="B12" s="205" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C12" s="180" t="inlineStr"/>
-      <c r="D12" s="180" t="inlineStr">
+      <c r="C12" s="208" t="inlineStr"/>
+      <c r="D12" s="208" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E12" s="180" t="inlineStr">
+      <c r="E12" s="208" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2642,18 +2710,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B13" s="179" t="inlineStr"/>
-      <c r="C13" s="179" t="inlineStr">
+      <c r="B13" s="207" t="inlineStr"/>
+      <c r="C13" s="207" t="inlineStr"/>
+      <c r="D13" s="207" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="D13" s="179" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="E13" s="179" t="inlineStr"/>
+      <c r="E13" s="207" t="inlineStr"/>
       <c r="F13" s="112" t="inlineStr">
         <is>
           <t>10/26 Midterm 2: 250 Points Chapters 6, 7, 9, &amp; 16</t>
@@ -2666,18 +2730,18 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B14" s="177" t="inlineStr">
+      <c r="B14" s="205" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C14" s="178" t="inlineStr"/>
-      <c r="D14" s="178" t="inlineStr">
+      <c r="C14" s="206" t="inlineStr"/>
+      <c r="D14" s="206" t="inlineStr">
         <is>
           <t>2026-12-16</t>
         </is>
       </c>
-      <c r="E14" s="178" t="inlineStr">
+      <c r="E14" s="206" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2693,18 +2757,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B15" s="179" t="inlineStr"/>
-      <c r="C15" s="179" t="inlineStr">
+      <c r="B15" s="207" t="inlineStr"/>
+      <c r="C15" s="207" t="inlineStr"/>
+      <c r="D15" s="207" t="inlineStr">
         <is>
           <t>2026-12-16</t>
         </is>
       </c>
-      <c r="D15" s="179" t="inlineStr">
-        <is>
-          <t>2026-12-16</t>
-        </is>
-      </c>
-      <c r="E15" s="179" t="inlineStr"/>
+      <c r="E15" s="207" t="inlineStr"/>
       <c r="F15" s="112" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -2717,22 +2777,22 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B16" s="177" t="inlineStr">
+      <c r="B16" s="205" t="inlineStr">
         <is>
           <t>170 pts</t>
         </is>
       </c>
-      <c r="C16" s="180" t="inlineStr">
+      <c r="C16" s="208" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="D16" s="180" t="inlineStr">
+      <c r="D16" s="208" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E16" s="180" t="inlineStr">
+      <c r="E16" s="208" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2748,14 +2808,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B17" s="179" t="inlineStr"/>
-      <c r="C17" s="179" t="inlineStr"/>
-      <c r="D17" s="179" t="inlineStr">
+      <c r="B17" s="207" t="inlineStr"/>
+      <c r="C17" s="207" t="inlineStr"/>
+      <c r="D17" s="207" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="E17" s="179" t="inlineStr"/>
+      <c r="E17" s="207" t="inlineStr"/>
       <c r="F17" s="112" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - Product Cost Accumulation: Job; Order Co: Chapter 3</t>
@@ -2768,14 +2828,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B18" s="179" t="inlineStr"/>
-      <c r="C18" s="179" t="inlineStr"/>
-      <c r="D18" s="179" t="inlineStr">
+      <c r="B18" s="207" t="inlineStr"/>
+      <c r="C18" s="207" t="inlineStr"/>
+      <c r="D18" s="207" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="E18" s="179" t="inlineStr"/>
+      <c r="E18" s="207" t="inlineStr"/>
       <c r="F18" s="112" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
@@ -2788,14 +2848,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B19" s="179" t="inlineStr"/>
-      <c r="C19" s="179" t="inlineStr"/>
-      <c r="D19" s="179" t="inlineStr">
+      <c r="B19" s="207" t="inlineStr"/>
+      <c r="C19" s="207" t="inlineStr"/>
+      <c r="D19" s="207" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E19" s="179" t="inlineStr"/>
+      <c r="E19" s="207" t="inlineStr"/>
       <c r="F19" s="112" t="inlineStr">
         <is>
           <t>Class 7 (9/16) - Activity Based Costing: Chapter 5- ONLY; LO 5.1, 2, 4 &amp; 5</t>
@@ -2808,14 +2868,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B20" s="179" t="inlineStr"/>
-      <c r="C20" s="179" t="inlineStr"/>
-      <c r="D20" s="179" t="inlineStr">
+      <c r="B20" s="207" t="inlineStr"/>
+      <c r="C20" s="207" t="inlineStr"/>
+      <c r="D20" s="207" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E20" s="179" t="inlineStr"/>
+      <c r="E20" s="207" t="inlineStr"/>
       <c r="F20" s="112" t="inlineStr">
         <is>
           <t>Class 7 (9/16) - 3-24, 3-28, 3-32; 15 Points</t>
@@ -2828,14 +2888,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B21" s="179" t="inlineStr"/>
-      <c r="C21" s="179" t="inlineStr"/>
-      <c r="D21" s="179" t="inlineStr">
+      <c r="B21" s="207" t="inlineStr"/>
+      <c r="C21" s="207" t="inlineStr"/>
+      <c r="D21" s="207" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="E21" s="179" t="inlineStr"/>
+      <c r="E21" s="207" t="inlineStr"/>
       <c r="F21" s="112" t="inlineStr">
         <is>
           <t>Class 8 (9/21) - Product Cost Accumulation: Pro-; cess Co: Chapter 4- ONLY; LO 4.1, 3, 4, &amp; 5</t>
@@ -2848,14 +2908,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B22" s="179" t="inlineStr"/>
-      <c r="C22" s="179" t="inlineStr"/>
-      <c r="D22" s="179" t="inlineStr">
+      <c r="B22" s="207" t="inlineStr"/>
+      <c r="C22" s="207" t="inlineStr"/>
+      <c r="D22" s="207" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="E22" s="179" t="inlineStr"/>
+      <c r="E22" s="207" t="inlineStr"/>
       <c r="F22" s="112" t="inlineStr">
         <is>
           <t>Class 8 (9/21) - 5-27 5-46; 10 Points</t>
@@ -2868,14 +2928,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B23" s="179" t="inlineStr"/>
-      <c r="C23" s="179" t="inlineStr"/>
-      <c r="D23" s="179" t="inlineStr">
+      <c r="B23" s="207" t="inlineStr"/>
+      <c r="C23" s="207" t="inlineStr"/>
+      <c r="D23" s="207" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="E23" s="179" t="inlineStr"/>
+      <c r="E23" s="207" t="inlineStr"/>
       <c r="F23" s="112" t="inlineStr">
         <is>
           <t>Class 9 (9/23) - Cost of Quality &amp; ESG &amp;; Overview of; • : Chapter 8 - ONLY; LO 8.7, 8, 9</t>
@@ -2888,14 +2948,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B24" s="179" t="inlineStr"/>
-      <c r="C24" s="179" t="inlineStr"/>
-      <c r="D24" s="179" t="inlineStr">
+      <c r="B24" s="207" t="inlineStr"/>
+      <c r="C24" s="207" t="inlineStr"/>
+      <c r="D24" s="207" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="E24" s="179" t="inlineStr"/>
+      <c r="E24" s="207" t="inlineStr"/>
       <c r="F24" s="112" t="inlineStr">
         <is>
           <t>Class 9 (9/23) - 4-21, 4-22; 10 Points</t>
@@ -2908,14 +2968,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B25" s="179" t="inlineStr"/>
-      <c r="C25" s="179" t="inlineStr"/>
-      <c r="D25" s="179" t="inlineStr">
+      <c r="B25" s="207" t="inlineStr"/>
+      <c r="C25" s="207" t="inlineStr"/>
+      <c r="D25" s="207" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E25" s="179" t="inlineStr"/>
+      <c r="E25" s="207" t="inlineStr"/>
       <c r="F25" s="112" t="inlineStr">
         <is>
           <t>Class 10 (9/28) - Catchup &amp; Midterm Review</t>
@@ -2928,14 +2988,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B26" s="179" t="inlineStr"/>
-      <c r="C26" s="179" t="inlineStr"/>
-      <c r="D26" s="179" t="inlineStr">
+      <c r="B26" s="207" t="inlineStr"/>
+      <c r="C26" s="207" t="inlineStr"/>
+      <c r="D26" s="207" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E26" s="179" t="inlineStr"/>
+      <c r="E26" s="207" t="inlineStr"/>
       <c r="F26" s="112" t="inlineStr">
         <is>
           <t>Class 10 (9/28) - 8-28, 8-29; 10 Points</t>
@@ -2948,14 +3008,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B27" s="179" t="inlineStr"/>
-      <c r="C27" s="179" t="inlineStr"/>
-      <c r="D27" s="179" t="inlineStr">
+      <c r="B27" s="207" t="inlineStr"/>
+      <c r="C27" s="207" t="inlineStr"/>
+      <c r="D27" s="207" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="E27" s="179" t="inlineStr"/>
+      <c r="E27" s="207" t="inlineStr"/>
       <c r="F27" s="112" t="inlineStr">
         <is>
           <t>Class 12 (10/7) - Cost volume profit analysis: Chapter 7</t>
@@ -2968,14 +3028,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B28" s="179" t="inlineStr"/>
-      <c r="C28" s="179" t="inlineStr"/>
-      <c r="D28" s="179" t="inlineStr">
+      <c r="B28" s="207" t="inlineStr"/>
+      <c r="C28" s="207" t="inlineStr"/>
+      <c r="D28" s="207" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="E28" s="179" t="inlineStr"/>
+      <c r="E28" s="207" t="inlineStr"/>
       <c r="F28" s="112" t="inlineStr">
         <is>
           <t>Class 12 (10/7) - 6-24, 6-25, 6-34; 15 Points</t>
@@ -2988,14 +3048,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B29" s="179" t="inlineStr"/>
-      <c r="C29" s="179" t="inlineStr"/>
-      <c r="D29" s="179" t="inlineStr">
+      <c r="B29" s="207" t="inlineStr"/>
+      <c r="C29" s="207" t="inlineStr"/>
+      <c r="D29" s="207" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E29" s="179" t="inlineStr"/>
+      <c r="E29" s="207" t="inlineStr"/>
       <c r="F29" s="112" t="inlineStr">
         <is>
           <t>Class 14 (10/14) - Financial planning and analysis:; Static: Chapter 9</t>
@@ -3008,14 +3068,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B30" s="179" t="inlineStr"/>
-      <c r="C30" s="179" t="inlineStr"/>
-      <c r="D30" s="179" t="inlineStr">
+      <c r="B30" s="207" t="inlineStr"/>
+      <c r="C30" s="207" t="inlineStr"/>
+      <c r="D30" s="207" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E30" s="179" t="inlineStr"/>
+      <c r="E30" s="207" t="inlineStr"/>
       <c r="F30" s="112" t="inlineStr">
         <is>
           <t>Class 14 (10/14) - 7-29, 7-33, 7-40; 15 Points</t>
@@ -3028,14 +3088,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B31" s="179" t="inlineStr"/>
-      <c r="C31" s="179" t="inlineStr"/>
-      <c r="D31" s="179" t="inlineStr">
+      <c r="B31" s="207" t="inlineStr"/>
+      <c r="C31" s="207" t="inlineStr"/>
+      <c r="D31" s="207" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E31" s="179" t="inlineStr"/>
+      <c r="E31" s="207" t="inlineStr"/>
       <c r="F31" s="112" t="inlineStr">
         <is>
           <t>Class 15 (10/19) - Capital Budgeting; Practice Midterm Ques: Chapter 16- ONLY; LO 16.1, 2, 3</t>
@@ -3048,14 +3108,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B32" s="179" t="inlineStr"/>
-      <c r="C32" s="179" t="inlineStr"/>
-      <c r="D32" s="179" t="inlineStr">
+      <c r="B32" s="207" t="inlineStr"/>
+      <c r="C32" s="207" t="inlineStr"/>
+      <c r="D32" s="207" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E32" s="179" t="inlineStr"/>
+      <c r="E32" s="207" t="inlineStr"/>
       <c r="F32" s="112" t="inlineStr">
         <is>
           <t>Class 15 (10/19) - 9-25, 9-28, 9-37; 15 - Points</t>
@@ -3068,14 +3128,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B33" s="179" t="inlineStr"/>
-      <c r="C33" s="179" t="inlineStr"/>
-      <c r="D33" s="179" t="inlineStr">
+      <c r="B33" s="207" t="inlineStr"/>
+      <c r="C33" s="207" t="inlineStr"/>
+      <c r="D33" s="207" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E33" s="179" t="inlineStr"/>
+      <c r="E33" s="207" t="inlineStr"/>
       <c r="F33" s="112" t="inlineStr">
         <is>
           <t>Class 16 (10/21) - Catchup &amp; Midterm Review</t>
@@ -3088,14 +3148,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B34" s="179" t="inlineStr"/>
-      <c r="C34" s="179" t="inlineStr"/>
-      <c r="D34" s="179" t="inlineStr">
+      <c r="B34" s="207" t="inlineStr"/>
+      <c r="C34" s="207" t="inlineStr"/>
+      <c r="D34" s="207" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E34" s="179" t="inlineStr"/>
+      <c r="E34" s="207" t="inlineStr"/>
       <c r="F34" s="112" t="inlineStr">
         <is>
           <t>Class 16 (10/21) - 16-28, 16-40; 10 Points</t>
@@ -3108,14 +3168,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B35" s="179" t="inlineStr"/>
-      <c r="C35" s="179" t="inlineStr"/>
-      <c r="D35" s="179" t="inlineStr">
+      <c r="B35" s="207" t="inlineStr"/>
+      <c r="C35" s="207" t="inlineStr"/>
+      <c r="D35" s="207" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="E35" s="179" t="inlineStr"/>
+      <c r="E35" s="207" t="inlineStr"/>
       <c r="F35" s="112" t="inlineStr">
         <is>
           <t>Class 19 (11/4) - Sales Variance Analysis; Flexible Budget: Chapter 11 - ONLY; LO 11.1, 11.2 &amp;; Appendix B</t>
@@ -3128,14 +3188,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B36" s="179" t="inlineStr"/>
-      <c r="C36" s="179" t="inlineStr"/>
-      <c r="D36" s="179" t="inlineStr">
+      <c r="B36" s="207" t="inlineStr"/>
+      <c r="C36" s="207" t="inlineStr"/>
+      <c r="D36" s="207" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="E36" s="179" t="inlineStr"/>
+      <c r="E36" s="207" t="inlineStr"/>
       <c r="F36" s="112" t="inlineStr">
         <is>
           <t>Class 19 (11/4) - 10-26, 10-30; 10 Points</t>
@@ -3148,14 +3208,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B37" s="179" t="inlineStr"/>
-      <c r="C37" s="179" t="inlineStr"/>
-      <c r="D37" s="179" t="inlineStr">
+      <c r="B37" s="207" t="inlineStr"/>
+      <c r="C37" s="207" t="inlineStr"/>
+      <c r="D37" s="207" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E37" s="179" t="inlineStr"/>
+      <c r="E37" s="207" t="inlineStr"/>
       <c r="F37" s="112" t="inlineStr">
         <is>
           <t>Class 20 (11/9) - Investment Centers: Chapter 13- ONLY; LO 13-1, 2, 3, 4</t>
@@ -3168,14 +3228,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B38" s="179" t="inlineStr"/>
-      <c r="C38" s="179" t="inlineStr"/>
-      <c r="D38" s="179" t="inlineStr">
+      <c r="B38" s="207" t="inlineStr"/>
+      <c r="C38" s="207" t="inlineStr"/>
+      <c r="D38" s="207" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E38" s="179" t="inlineStr"/>
+      <c r="E38" s="207" t="inlineStr"/>
       <c r="F38" s="112" t="inlineStr">
         <is>
           <t>Class 20 (11/9) - 11-31, 11-52; 10 Points</t>
@@ -3188,14 +3248,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B39" s="179" t="inlineStr"/>
-      <c r="C39" s="179" t="inlineStr"/>
-      <c r="D39" s="179" t="inlineStr">
+      <c r="B39" s="207" t="inlineStr"/>
+      <c r="C39" s="207" t="inlineStr"/>
+      <c r="D39" s="207" t="inlineStr">
         <is>
           <t>2026-11-16</t>
         </is>
       </c>
-      <c r="E39" s="179" t="inlineStr"/>
+      <c r="E39" s="207" t="inlineStr"/>
       <c r="F39" s="112" t="inlineStr">
         <is>
           <t>Class 21 (11/16) - AI &amp; FP&amp;A</t>
@@ -3208,14 +3268,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B40" s="179" t="inlineStr"/>
-      <c r="C40" s="179" t="inlineStr"/>
-      <c r="D40" s="179" t="inlineStr">
+      <c r="B40" s="207" t="inlineStr"/>
+      <c r="C40" s="207" t="inlineStr"/>
+      <c r="D40" s="207" t="inlineStr">
         <is>
           <t>2026-11-16</t>
         </is>
       </c>
-      <c r="E40" s="179" t="inlineStr"/>
+      <c r="E40" s="207" t="inlineStr"/>
       <c r="F40" s="112" t="inlineStr">
         <is>
           <t>Class 21 (11/16) - 13-29, 13-33; 10 Points</t>
@@ -3228,14 +3288,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B41" s="179" t="inlineStr"/>
-      <c r="C41" s="179" t="inlineStr"/>
-      <c r="D41" s="179" t="inlineStr">
+      <c r="B41" s="207" t="inlineStr"/>
+      <c r="C41" s="207" t="inlineStr"/>
+      <c r="D41" s="207" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E41" s="179" t="inlineStr"/>
+      <c r="E41" s="207" t="inlineStr"/>
       <c r="F41" s="112" t="inlineStr">
         <is>
           <t>Class 2 (12/2) - Catchup &amp; Final Review; Practice Final Questions Posted to Brightspace at; 5:00 PM</t>
@@ -3248,14 +3308,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B42" s="179" t="inlineStr"/>
-      <c r="C42" s="179" t="inlineStr"/>
-      <c r="D42" s="179" t="inlineStr">
+      <c r="B42" s="207" t="inlineStr"/>
+      <c r="C42" s="207" t="inlineStr"/>
+      <c r="D42" s="207" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E42" s="179" t="inlineStr"/>
+      <c r="E42" s="207" t="inlineStr"/>
       <c r="F42" s="112" t="inlineStr">
         <is>
           <t>Class 2 (12/2) - 14-35, 14-41; 10 Points; Assignments listed Be-; low Due by11:59 PM; Linked In Learning; E</t>
@@ -3268,22 +3328,22 @@
           <t>LinkedIn Learning Excel Certification</t>
         </is>
       </c>
-      <c r="B43" s="177" t="inlineStr">
+      <c r="B43" s="205" t="inlineStr">
         <is>
           <t>75 pts</t>
         </is>
       </c>
-      <c r="C43" s="178" t="inlineStr">
+      <c r="C43" s="206" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D43" s="178" t="inlineStr">
+      <c r="D43" s="206" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E43" s="178" t="inlineStr">
+      <c r="E43" s="206" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3299,18 +3359,18 @@
           <t>Certification</t>
         </is>
       </c>
-      <c r="B44" s="179" t="inlineStr"/>
-      <c r="C44" s="179" t="inlineStr">
+      <c r="B44" s="207" t="inlineStr"/>
+      <c r="C44" s="207" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D44" s="179" t="inlineStr">
+      <c r="D44" s="207" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E44" s="179" t="inlineStr"/>
+      <c r="E44" s="207" t="inlineStr"/>
       <c r="F44" s="112" t="inlineStr">
         <is>
           <t>LinkedIn Learning Excel Certification</t>
@@ -3323,22 +3383,22 @@
           <t>Stukent Simternship</t>
         </is>
       </c>
-      <c r="B45" s="177" t="inlineStr">
+      <c r="B45" s="205" t="inlineStr">
         <is>
           <t>75 pts</t>
         </is>
       </c>
-      <c r="C45" s="180" t="inlineStr">
+      <c r="C45" s="208" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D45" s="180" t="inlineStr">
+      <c r="D45" s="208" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E45" s="180" t="inlineStr">
+      <c r="E45" s="208" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3354,18 +3414,18 @@
           <t>Certification</t>
         </is>
       </c>
-      <c r="B46" s="179" t="inlineStr"/>
-      <c r="C46" s="179" t="inlineStr">
+      <c r="B46" s="207" t="inlineStr"/>
+      <c r="C46" s="207" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D46" s="179" t="inlineStr">
+      <c r="D46" s="207" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E46" s="179" t="inlineStr"/>
+      <c r="E46" s="207" t="inlineStr"/>
       <c r="F46" s="112" t="inlineStr">
         <is>
           <t>Stukent Simternship</t>
@@ -3519,22 +3579,22 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B10" s="185" t="inlineStr">
+      <c r="B10" s="209" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="C10" s="186" t="inlineStr">
+      <c r="C10" s="210" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D10" s="186" t="inlineStr">
+      <c r="D10" s="210" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E10" s="186" t="inlineStr">
+      <c r="E10" s="210" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3550,18 +3610,18 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B11" s="187" t="inlineStr"/>
-      <c r="C11" s="187" t="inlineStr">
+      <c r="B11" s="211" t="inlineStr"/>
+      <c r="C11" s="211" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D11" s="187" t="inlineStr">
+      <c r="D11" s="211" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E11" s="187" t="inlineStr"/>
+      <c r="E11" s="211" t="inlineStr"/>
       <c r="F11" s="126" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -3574,22 +3634,22 @@
           <t>Participation</t>
         </is>
       </c>
-      <c r="B12" s="185" t="inlineStr">
+      <c r="B12" s="209" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C12" s="188" t="inlineStr">
+      <c r="C12" s="212" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D12" s="188" t="inlineStr">
+      <c r="D12" s="212" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E12" s="188" t="inlineStr">
+      <c r="E12" s="212" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3605,14 +3665,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B13" s="187" t="inlineStr"/>
-      <c r="C13" s="187" t="inlineStr">
+      <c r="B13" s="211" t="inlineStr"/>
+      <c r="C13" s="211" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D13" s="187" t="inlineStr"/>
-      <c r="E13" s="187" t="inlineStr"/>
+      <c r="D13" s="211" t="inlineStr"/>
+      <c r="E13" s="211" t="inlineStr"/>
       <c r="F13" s="126" t="inlineStr">
         <is>
           <t>Research: SONA registration opens</t>
@@ -3625,14 +3685,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B14" s="187" t="inlineStr"/>
-      <c r="C14" s="187" t="inlineStr">
+      <c r="B14" s="211" t="inlineStr"/>
+      <c r="C14" s="211" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="D14" s="187" t="inlineStr"/>
-      <c r="E14" s="187" t="inlineStr"/>
+      <c r="D14" s="211" t="inlineStr"/>
+      <c r="E14" s="211" t="inlineStr"/>
       <c r="F14" s="126" t="inlineStr">
         <is>
           <t>Research: Prescreening questionnaire opens</t>
@@ -3645,14 +3705,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B15" s="187" t="inlineStr"/>
-      <c r="C15" s="187" t="inlineStr"/>
-      <c r="D15" s="187" t="inlineStr">
+      <c r="B15" s="211" t="inlineStr"/>
+      <c r="C15" s="211" t="inlineStr"/>
+      <c r="D15" s="211" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="E15" s="187" t="inlineStr"/>
+      <c r="E15" s="211" t="inlineStr"/>
       <c r="F15" s="126" t="inlineStr">
         <is>
           <t>Research: Setup deadline (registration, prescreening, contacts)</t>
@@ -3665,14 +3725,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B16" s="187" t="inlineStr"/>
-      <c r="C16" s="187" t="inlineStr">
+      <c r="B16" s="211" t="inlineStr"/>
+      <c r="C16" s="211" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="D16" s="187" t="inlineStr"/>
-      <c r="E16" s="187" t="inlineStr"/>
+      <c r="D16" s="211" t="inlineStr"/>
+      <c r="E16" s="211" t="inlineStr"/>
       <c r="F16" s="126" t="inlineStr">
         <is>
           <t>Research: Study invitations begin (after setup)</t>
@@ -3685,14 +3745,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B17" s="187" t="inlineStr"/>
-      <c r="C17" s="187" t="inlineStr"/>
-      <c r="D17" s="187" t="inlineStr">
+      <c r="B17" s="211" t="inlineStr"/>
+      <c r="C17" s="211" t="inlineStr"/>
+      <c r="D17" s="211" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E17" s="187" t="inlineStr"/>
+      <c r="E17" s="211" t="inlineStr"/>
       <c r="F17" s="126" t="inlineStr">
         <is>
           <t>Research: Employee contact surveys sent</t>
@@ -3705,14 +3765,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B18" s="187" t="inlineStr"/>
-      <c r="C18" s="187" t="inlineStr"/>
-      <c r="D18" s="187" t="inlineStr">
+      <c r="B18" s="211" t="inlineStr"/>
+      <c r="C18" s="211" t="inlineStr"/>
+      <c r="D18" s="211" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E18" s="187" t="inlineStr"/>
+      <c r="E18" s="211" t="inlineStr"/>
       <c r="F18" s="126" t="inlineStr">
         <is>
           <t>Research: Complete 2.0 research credits</t>
@@ -3725,22 +3785,22 @@
           <t>Midterm Exam</t>
         </is>
       </c>
-      <c r="B19" s="185" t="inlineStr">
+      <c r="B19" s="209" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C19" s="186" t="inlineStr">
+      <c r="C19" s="210" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D19" s="186" t="inlineStr">
+      <c r="D19" s="210" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E19" s="186" t="inlineStr">
+      <c r="E19" s="210" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3756,18 +3816,18 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B20" s="187" t="inlineStr"/>
-      <c r="C20" s="187" t="inlineStr">
+      <c r="B20" s="211" t="inlineStr"/>
+      <c r="C20" s="211" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D20" s="187" t="inlineStr">
+      <c r="D20" s="211" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E20" s="187" t="inlineStr"/>
+      <c r="E20" s="211" t="inlineStr"/>
       <c r="F20" s="126" t="inlineStr">
         <is>
           <t>Midterm Exam</t>
@@ -3780,22 +3840,22 @@
           <t>Team Project Paper</t>
         </is>
       </c>
-      <c r="B21" s="185" t="inlineStr">
+      <c r="B21" s="209" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C21" s="188" t="inlineStr">
+      <c r="C21" s="212" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D21" s="188" t="inlineStr">
+      <c r="D21" s="212" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E21" s="188" t="inlineStr">
+      <c r="E21" s="212" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3811,18 +3871,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B22" s="187" t="inlineStr"/>
-      <c r="C22" s="187" t="inlineStr">
+      <c r="B22" s="211" t="inlineStr"/>
+      <c r="C22" s="211" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D22" s="187" t="inlineStr">
+      <c r="D22" s="211" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E22" s="187" t="inlineStr"/>
+      <c r="E22" s="211" t="inlineStr"/>
       <c r="F22" s="126" t="inlineStr">
         <is>
           <t>Team project outline</t>
@@ -3835,18 +3895,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B23" s="187" t="inlineStr"/>
-      <c r="C23" s="187" t="inlineStr">
+      <c r="B23" s="211" t="inlineStr"/>
+      <c r="C23" s="211" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D23" s="187" t="inlineStr">
+      <c r="D23" s="211" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E23" s="187" t="inlineStr"/>
+      <c r="E23" s="211" t="inlineStr"/>
       <c r="F23" s="126" t="inlineStr">
         <is>
           <t>Team project paper</t>
@@ -3859,22 +3919,22 @@
           <t>Final Reflection Paper</t>
         </is>
       </c>
-      <c r="B24" s="185" t="inlineStr">
+      <c r="B24" s="209" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C24" s="186" t="inlineStr">
+      <c r="C24" s="210" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D24" s="186" t="inlineStr">
+      <c r="D24" s="210" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E24" s="186" t="inlineStr">
+      <c r="E24" s="210" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3890,18 +3950,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B25" s="187" t="inlineStr"/>
-      <c r="C25" s="187" t="inlineStr">
+      <c r="B25" s="211" t="inlineStr"/>
+      <c r="C25" s="211" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D25" s="187" t="inlineStr">
+      <c r="D25" s="211" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E25" s="187" t="inlineStr"/>
+      <c r="E25" s="211" t="inlineStr"/>
       <c r="F25" s="126" t="inlineStr">
         <is>
           <t>Personal Reflection Paper</t>
@@ -3914,22 +3974,22 @@
           <t>Presentation</t>
         </is>
       </c>
-      <c r="B26" s="185" t="inlineStr">
+      <c r="B26" s="209" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C26" s="188" t="inlineStr">
+      <c r="C26" s="212" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D26" s="188" t="inlineStr">
+      <c r="D26" s="212" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E26" s="188" t="inlineStr">
+      <c r="E26" s="212" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3945,18 +4005,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B27" s="187" t="inlineStr"/>
-      <c r="C27" s="187" t="inlineStr">
+      <c r="B27" s="211" t="inlineStr"/>
+      <c r="C27" s="211" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D27" s="187" t="inlineStr">
+      <c r="D27" s="211" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E27" s="187" t="inlineStr"/>
+      <c r="E27" s="211" t="inlineStr"/>
       <c r="F27" s="126" t="inlineStr">
         <is>
           <t>Presentation slides</t>
@@ -3969,22 +4029,22 @@
           <t>Case Analysis Assignments</t>
         </is>
       </c>
-      <c r="B28" s="185" t="inlineStr">
+      <c r="B28" s="209" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C28" s="186" t="inlineStr">
+      <c r="C28" s="210" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D28" s="186" t="inlineStr">
+      <c r="D28" s="210" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E28" s="186" t="inlineStr">
+      <c r="E28" s="210" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4000,18 +4060,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B29" s="187" t="inlineStr"/>
-      <c r="C29" s="187" t="inlineStr">
+      <c r="B29" s="211" t="inlineStr"/>
+      <c r="C29" s="211" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D29" s="187" t="inlineStr">
+      <c r="D29" s="211" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E29" s="187" t="inlineStr"/>
+      <c r="E29" s="211" t="inlineStr"/>
       <c r="F29" s="126" t="inlineStr">
         <is>
           <t>Thomas Green Case Analysis Memo</t>
@@ -4024,18 +4084,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B30" s="187" t="inlineStr"/>
-      <c r="C30" s="187" t="inlineStr">
+      <c r="B30" s="211" t="inlineStr"/>
+      <c r="C30" s="211" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D30" s="187" t="inlineStr">
+      <c r="D30" s="211" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E30" s="187" t="inlineStr"/>
+      <c r="E30" s="211" t="inlineStr"/>
       <c r="F30" s="126" t="inlineStr">
         <is>
           <t>SkillsForTomorrow Analysis Memo</t>
@@ -4048,22 +4108,22 @@
           <t>Proposal &amp; Team Contract</t>
         </is>
       </c>
-      <c r="B31" s="185" t="inlineStr">
+      <c r="B31" s="209" t="inlineStr">
         <is>
           <t>3%</t>
         </is>
       </c>
-      <c r="C31" s="188" t="inlineStr">
+      <c r="C31" s="212" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D31" s="188" t="inlineStr">
+      <c r="D31" s="212" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E31" s="188" t="inlineStr">
+      <c r="E31" s="212" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4079,18 +4139,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B32" s="187" t="inlineStr"/>
-      <c r="C32" s="187" t="inlineStr">
+      <c r="B32" s="211" t="inlineStr"/>
+      <c r="C32" s="211" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D32" s="187" t="inlineStr">
+      <c r="D32" s="211" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E32" s="187" t="inlineStr"/>
+      <c r="E32" s="211" t="inlineStr"/>
       <c r="F32" s="126" t="inlineStr">
         <is>
           <t>Team project proposal &amp; team contract</t>
@@ -4103,22 +4163,22 @@
           <t>Self &amp; Peer Evaluation</t>
         </is>
       </c>
-      <c r="B33" s="185" t="inlineStr">
+      <c r="B33" s="209" t="inlineStr">
         <is>
           <t>2%</t>
         </is>
       </c>
-      <c r="C33" s="186" t="inlineStr">
+      <c r="C33" s="210" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D33" s="186" t="inlineStr">
+      <c r="D33" s="210" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E33" s="186" t="inlineStr">
+      <c r="E33" s="210" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4134,18 +4194,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B34" s="187" t="inlineStr"/>
-      <c r="C34" s="187" t="inlineStr">
+      <c r="B34" s="211" t="inlineStr"/>
+      <c r="C34" s="211" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D34" s="187" t="inlineStr">
+      <c r="D34" s="211" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E34" s="187" t="inlineStr"/>
+      <c r="E34" s="211" t="inlineStr"/>
       <c r="F34" s="126" t="inlineStr">
         <is>
           <t>Self &amp; peer evaluation</t>
@@ -4158,22 +4218,22 @@
           <t>Personal Assessments (Connect)</t>
         </is>
       </c>
-      <c r="B35" s="185" t="inlineStr">
+      <c r="B35" s="209" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C35" s="188" t="inlineStr">
+      <c r="C35" s="212" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D35" s="188" t="inlineStr">
+      <c r="D35" s="212" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E35" s="188" t="inlineStr">
+      <c r="E35" s="212" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4189,14 +4249,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B36" s="187" t="inlineStr"/>
-      <c r="C36" s="187" t="inlineStr"/>
-      <c r="D36" s="187" t="inlineStr">
+      <c r="B36" s="211" t="inlineStr"/>
+      <c r="C36" s="211" t="inlineStr"/>
+      <c r="D36" s="211" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="E36" s="187" t="inlineStr"/>
+      <c r="E36" s="211" t="inlineStr"/>
       <c r="F36" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
@@ -4209,14 +4269,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B37" s="187" t="inlineStr"/>
-      <c r="C37" s="187" t="inlineStr"/>
-      <c r="D37" s="187" t="inlineStr">
+      <c r="B37" s="211" t="inlineStr"/>
+      <c r="C37" s="211" t="inlineStr"/>
+      <c r="D37" s="211" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="E37" s="187" t="inlineStr"/>
+      <c r="E37" s="211" t="inlineStr"/>
       <c r="F37" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
@@ -4229,14 +4289,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B38" s="187" t="inlineStr"/>
-      <c r="C38" s="187" t="inlineStr"/>
-      <c r="D38" s="187" t="inlineStr">
+      <c r="B38" s="211" t="inlineStr"/>
+      <c r="C38" s="211" t="inlineStr"/>
+      <c r="D38" s="211" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="E38" s="187" t="inlineStr"/>
+      <c r="E38" s="211" t="inlineStr"/>
       <c r="F38" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 5.01 - Assessing Your</t>
@@ -4249,14 +4309,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B39" s="187" t="inlineStr"/>
-      <c r="C39" s="187" t="inlineStr"/>
-      <c r="D39" s="187" t="inlineStr">
+      <c r="B39" s="211" t="inlineStr"/>
+      <c r="C39" s="211" t="inlineStr"/>
+      <c r="D39" s="211" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E39" s="187" t="inlineStr"/>
+      <c r="E39" s="211" t="inlineStr"/>
       <c r="F39" s="126" t="inlineStr">
         <is>
           <t>Connect: Sharpen Companion</t>
@@ -4269,14 +4329,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B40" s="187" t="inlineStr"/>
-      <c r="C40" s="187" t="inlineStr"/>
-      <c r="D40" s="187" t="inlineStr">
+      <c r="B40" s="211" t="inlineStr"/>
+      <c r="C40" s="211" t="inlineStr"/>
+      <c r="D40" s="211" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="E40" s="187" t="inlineStr"/>
+      <c r="E40" s="211" t="inlineStr"/>
       <c r="F40" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 11.01 - What is my</t>
@@ -4289,14 +4349,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B41" s="187" t="inlineStr"/>
-      <c r="C41" s="187" t="inlineStr"/>
-      <c r="D41" s="187" t="inlineStr">
+      <c r="B41" s="211" t="inlineStr"/>
+      <c r="C41" s="211" t="inlineStr"/>
+      <c r="D41" s="211" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="E41" s="187" t="inlineStr"/>
+      <c r="E41" s="211" t="inlineStr"/>
       <c r="F41" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 11.02 - What is my</t>
@@ -4309,14 +4369,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B42" s="187" t="inlineStr"/>
-      <c r="C42" s="187" t="inlineStr"/>
-      <c r="D42" s="187" t="inlineStr">
+      <c r="B42" s="211" t="inlineStr"/>
+      <c r="C42" s="211" t="inlineStr"/>
+      <c r="D42" s="211" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E42" s="187" t="inlineStr"/>
+      <c r="E42" s="211" t="inlineStr"/>
       <c r="F42" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 12.01 - What kind of</t>
@@ -4329,14 +4389,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B43" s="187" t="inlineStr"/>
-      <c r="C43" s="187" t="inlineStr"/>
-      <c r="D43" s="187" t="inlineStr">
+      <c r="B43" s="211" t="inlineStr"/>
+      <c r="C43" s="211" t="inlineStr"/>
+      <c r="D43" s="211" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E43" s="187" t="inlineStr"/>
+      <c r="E43" s="211" t="inlineStr"/>
       <c r="F43" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 10.5 - Preferred Conflict</t>
@@ -4349,14 +4409,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B44" s="187" t="inlineStr"/>
-      <c r="C44" s="187" t="inlineStr"/>
-      <c r="D44" s="187" t="inlineStr">
+      <c r="B44" s="211" t="inlineStr"/>
+      <c r="C44" s="211" t="inlineStr"/>
+      <c r="D44" s="211" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E44" s="187" t="inlineStr"/>
+      <c r="E44" s="211" t="inlineStr"/>
       <c r="F44" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 9.01 - Assessing My</t>
@@ -4369,14 +4429,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B45" s="187" t="inlineStr"/>
-      <c r="C45" s="187" t="inlineStr"/>
-      <c r="D45" s="187" t="inlineStr">
+      <c r="B45" s="211" t="inlineStr"/>
+      <c r="C45" s="211" t="inlineStr"/>
+      <c r="D45" s="211" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E45" s="187" t="inlineStr"/>
+      <c r="E45" s="211" t="inlineStr"/>
       <c r="F45" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 8.01 - Group</t>
@@ -4389,14 +4449,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B46" s="187" t="inlineStr"/>
-      <c r="C46" s="187" t="inlineStr"/>
-      <c r="D46" s="187" t="inlineStr">
+      <c r="B46" s="211" t="inlineStr"/>
+      <c r="C46" s="211" t="inlineStr"/>
+      <c r="D46" s="211" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="E46" s="187" t="inlineStr"/>
+      <c r="E46" s="211" t="inlineStr"/>
       <c r="F46" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 14.02 - What Type of Organizational Culture Do I</t>
@@ -4409,14 +4469,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B47" s="187" t="inlineStr"/>
-      <c r="C47" s="187" t="inlineStr"/>
-      <c r="D47" s="187" t="inlineStr">
+      <c r="B47" s="211" t="inlineStr"/>
+      <c r="C47" s="211" t="inlineStr"/>
+      <c r="D47" s="211" t="inlineStr">
         <is>
           <t>2026-11-30</t>
         </is>
       </c>
-      <c r="E47" s="187" t="inlineStr"/>
+      <c r="E47" s="211" t="inlineStr"/>
       <c r="F47" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 16.02 - What Is Your</t>
@@ -4429,14 +4489,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B48" s="187" t="inlineStr"/>
-      <c r="C48" s="187" t="inlineStr"/>
-      <c r="D48" s="187" t="inlineStr">
+      <c r="B48" s="211" t="inlineStr"/>
+      <c r="C48" s="211" t="inlineStr"/>
+      <c r="D48" s="211" t="inlineStr">
         <is>
           <t>2026-11-30</t>
         </is>
       </c>
-      <c r="E48" s="187" t="inlineStr"/>
+      <c r="E48" s="211" t="inlineStr"/>
       <c r="F48" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 16.03 - Assessing Your</t>
@@ -4449,14 +4509,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B49" s="187" t="inlineStr"/>
-      <c r="C49" s="187" t="inlineStr"/>
-      <c r="D49" s="187" t="inlineStr">
+      <c r="B49" s="211" t="inlineStr"/>
+      <c r="C49" s="211" t="inlineStr"/>
+      <c r="D49" s="211" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E49" s="187" t="inlineStr"/>
+      <c r="E49" s="211" t="inlineStr"/>
       <c r="F49" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 12.02 - Which influence</t>

</xml_diff>

<commit_message>
Retrain: blank homework starts unless rubric explicitly states one
Add strip_unverified_homework_starts() to check raw category rubrics
(extracted_text + sections) for opens/assigned/mentioned language before
keeping Start Date on Homework sub-rows or Homework/Connect categories.

- calendar_homework_dates: due span only (no earliest session as start)
- Personal Assessments (Connect): category start blank
- Sharpen: parse explicit prose only; no hardcoded start
- SKILL.md + reference.md: homework start rules and sanity check
- Regenerated syllabi.xlsx and all JSON/PDF outputs

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -251,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="213">
+  <cellXfs count="225">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -793,6 +793,42 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1362,18 +1398,18 @@
           <t>Sleep Paper</t>
         </is>
       </c>
-      <c r="B10" s="201" t="inlineStr">
+      <c r="B10" s="213" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C10" s="202" t="inlineStr"/>
-      <c r="D10" s="202" t="inlineStr">
+      <c r="C10" s="214" t="inlineStr"/>
+      <c r="D10" s="214" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="E10" s="202" t="inlineStr">
+      <c r="E10" s="214" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1389,14 +1425,14 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B11" s="203" t="inlineStr"/>
-      <c r="C11" s="203" t="inlineStr"/>
-      <c r="D11" s="203" t="inlineStr">
+      <c r="B11" s="215" t="inlineStr"/>
+      <c r="C11" s="215" t="inlineStr"/>
+      <c r="D11" s="215" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="E11" s="203" t="inlineStr"/>
+      <c r="E11" s="215" t="inlineStr"/>
       <c r="F11" s="99" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
@@ -1409,18 +1445,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B12" s="203" t="inlineStr"/>
-      <c r="C12" s="203" t="inlineStr">
+      <c r="B12" s="215" t="inlineStr"/>
+      <c r="C12" s="215" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D12" s="203" t="inlineStr">
+      <c r="D12" s="215" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E12" s="203" t="inlineStr"/>
+      <c r="E12" s="215" t="inlineStr"/>
       <c r="F12" s="99" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance</t>
@@ -1433,18 +1469,18 @@
           <t>Witchcraft Paper</t>
         </is>
       </c>
-      <c r="B13" s="201" t="inlineStr">
+      <c r="B13" s="213" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C13" s="204" t="inlineStr"/>
-      <c r="D13" s="204" t="inlineStr">
+      <c r="C13" s="216" t="inlineStr"/>
+      <c r="D13" s="216" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="E13" s="204" t="inlineStr">
+      <c r="E13" s="216" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1460,14 +1496,14 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B14" s="203" t="inlineStr"/>
-      <c r="C14" s="203" t="inlineStr"/>
-      <c r="D14" s="203" t="inlineStr">
+      <c r="B14" s="215" t="inlineStr"/>
+      <c r="C14" s="215" t="inlineStr"/>
+      <c r="D14" s="215" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="E14" s="203" t="inlineStr"/>
+      <c r="E14" s="215" t="inlineStr"/>
       <c r="F14" s="99" t="inlineStr">
         <is>
           <t>Witchcraft Paper Due</t>
@@ -1480,18 +1516,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B15" s="203" t="inlineStr"/>
-      <c r="C15" s="203" t="inlineStr">
+      <c r="B15" s="215" t="inlineStr"/>
+      <c r="C15" s="215" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D15" s="203" t="inlineStr">
+      <c r="D15" s="215" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E15" s="203" t="inlineStr"/>
+      <c r="E15" s="215" t="inlineStr"/>
       <c r="F15" s="99" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment</t>
@@ -1504,18 +1540,18 @@
           <t>Mid-term</t>
         </is>
       </c>
-      <c r="B16" s="201" t="inlineStr">
+      <c r="B16" s="213" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C16" s="202" t="inlineStr"/>
-      <c r="D16" s="202" t="inlineStr">
+      <c r="C16" s="214" t="inlineStr"/>
+      <c r="D16" s="214" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E16" s="202" t="inlineStr">
+      <c r="E16" s="214" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1531,14 +1567,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B17" s="203" t="inlineStr"/>
-      <c r="C17" s="203" t="inlineStr"/>
-      <c r="D17" s="203" t="inlineStr">
+      <c r="B17" s="215" t="inlineStr"/>
+      <c r="C17" s="215" t="inlineStr"/>
+      <c r="D17" s="215" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="E17" s="203" t="inlineStr"/>
+      <c r="E17" s="215" t="inlineStr"/>
       <c r="F17" s="99" t="inlineStr">
         <is>
           <t>Midterm Exam</t>
@@ -1551,18 +1587,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B18" s="203" t="inlineStr"/>
-      <c r="C18" s="203" t="inlineStr">
+      <c r="B18" s="215" t="inlineStr"/>
+      <c r="C18" s="215" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="D18" s="203" t="inlineStr">
+      <c r="D18" s="215" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E18" s="203" t="inlineStr"/>
+      <c r="E18" s="215" t="inlineStr"/>
       <c r="F18" s="99" t="inlineStr">
         <is>
           <t>Week Oct 6-9: Midterm &amp; Break</t>
@@ -1575,18 +1611,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B19" s="203" t="inlineStr"/>
-      <c r="C19" s="203" t="inlineStr">
+      <c r="B19" s="215" t="inlineStr"/>
+      <c r="C19" s="215" t="inlineStr">
         <is>
           <t>2026-12-01</t>
         </is>
       </c>
-      <c r="D19" s="203" t="inlineStr">
+      <c r="D19" s="215" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E19" s="203" t="inlineStr"/>
+      <c r="E19" s="215" t="inlineStr"/>
       <c r="F19" s="99" t="inlineStr">
         <is>
           <t>Week Dec 1-4: Modern Europe?</t>
@@ -1599,18 +1635,18 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B20" s="201" t="inlineStr">
+      <c r="B20" s="213" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C20" s="204" t="inlineStr"/>
-      <c r="D20" s="204" t="inlineStr">
+      <c r="C20" s="216" t="inlineStr"/>
+      <c r="D20" s="216" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="E20" s="204" t="inlineStr">
+      <c r="E20" s="216" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1626,14 +1662,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B21" s="203" t="inlineStr"/>
-      <c r="C21" s="203" t="inlineStr"/>
-      <c r="D21" s="203" t="inlineStr">
+      <c r="B21" s="215" t="inlineStr"/>
+      <c r="C21" s="215" t="inlineStr"/>
+      <c r="D21" s="215" t="inlineStr">
         <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="E21" s="203" t="inlineStr"/>
+      <c r="E21" s="215" t="inlineStr"/>
       <c r="F21" s="99" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -1646,18 +1682,18 @@
           <t>Discussion Section</t>
         </is>
       </c>
-      <c r="B22" s="201" t="inlineStr">
+      <c r="B22" s="213" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C22" s="202" t="inlineStr"/>
-      <c r="D22" s="202" t="inlineStr">
+      <c r="C22" s="214" t="inlineStr"/>
+      <c r="D22" s="214" t="inlineStr">
         <is>
           <t>2026-11-12</t>
         </is>
       </c>
-      <c r="E22" s="202" t="inlineStr">
+      <c r="E22" s="214" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1673,18 +1709,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B23" s="203" t="inlineStr"/>
-      <c r="C23" s="203" t="inlineStr">
+      <c r="B23" s="215" t="inlineStr"/>
+      <c r="C23" s="215" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D23" s="203" t="inlineStr">
+      <c r="D23" s="215" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E23" s="203" t="inlineStr"/>
+      <c r="E23" s="215" t="inlineStr"/>
       <c r="F23" s="99" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death</t>
@@ -1697,18 +1733,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B24" s="203" t="inlineStr"/>
-      <c r="C24" s="203" t="inlineStr">
+      <c r="B24" s="215" t="inlineStr"/>
+      <c r="C24" s="215" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D24" s="203" t="inlineStr">
+      <c r="D24" s="215" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E24" s="203" t="inlineStr"/>
+      <c r="E24" s="215" t="inlineStr"/>
       <c r="F24" s="99" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death - Section reading 1: -- 13 of 33 -- Lizzie Wade, “From Black Death to fatal flu, pas</t>
@@ -1721,18 +1757,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B25" s="203" t="inlineStr"/>
-      <c r="C25" s="203" t="inlineStr">
+      <c r="B25" s="215" t="inlineStr"/>
+      <c r="C25" s="215" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D25" s="203" t="inlineStr">
+      <c r="D25" s="215" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E25" s="203" t="inlineStr"/>
+      <c r="E25" s="215" t="inlineStr"/>
       <c r="F25" s="99" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life</t>
@@ -1745,18 +1781,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B26" s="203" t="inlineStr"/>
-      <c r="C26" s="203" t="inlineStr">
+      <c r="B26" s="215" t="inlineStr"/>
+      <c r="C26" s="215" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D26" s="203" t="inlineStr">
+      <c r="D26" s="215" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E26" s="203" t="inlineStr"/>
+      <c r="E26" s="215" t="inlineStr"/>
       <c r="F26" s="99" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life - Section reading 1: A Roger Ekirch, “Sleep we have lost: Pre-Industrial Slumber in the Brit</t>
@@ -1769,18 +1805,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B27" s="203" t="inlineStr"/>
-      <c r="C27" s="203" t="inlineStr">
+      <c r="B27" s="215" t="inlineStr"/>
+      <c r="C27" s="215" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D27" s="203" t="inlineStr">
+      <c r="D27" s="215" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E27" s="203" t="inlineStr"/>
+      <c r="E27" s="215" t="inlineStr"/>
       <c r="F27" s="99" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance</t>
@@ -1793,18 +1829,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B28" s="203" t="inlineStr"/>
-      <c r="C28" s="203" t="inlineStr">
+      <c r="B28" s="215" t="inlineStr"/>
+      <c r="C28" s="215" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D28" s="203" t="inlineStr">
+      <c r="D28" s="215" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E28" s="203" t="inlineStr"/>
+      <c r="E28" s="215" t="inlineStr"/>
       <c r="F28" s="99" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance - Section reading 1: -- 14 of 33 -- Kay Daly, “Diverting the Flood of History: Ada Palmer’s I</t>
@@ -1817,18 +1853,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B29" s="203" t="inlineStr"/>
-      <c r="C29" s="203" t="inlineStr">
+      <c r="B29" s="215" t="inlineStr"/>
+      <c r="C29" s="215" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D29" s="203" t="inlineStr">
+      <c r="D29" s="215" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E29" s="203" t="inlineStr"/>
+      <c r="E29" s="215" t="inlineStr"/>
       <c r="F29" s="99" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance - Section reading 1: Vasari, Lives of the Artists: Leonardo da Vinci &amp; Properzia de’ Rossi V</t>
@@ -1841,18 +1877,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B30" s="203" t="inlineStr"/>
-      <c r="C30" s="203" t="inlineStr">
+      <c r="B30" s="215" t="inlineStr"/>
+      <c r="C30" s="215" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D30" s="203" t="inlineStr">
+      <c r="D30" s="215" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E30" s="203" t="inlineStr"/>
+      <c r="E30" s="215" t="inlineStr"/>
       <c r="F30" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion</t>
@@ -1865,18 +1901,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B31" s="203" t="inlineStr"/>
-      <c r="C31" s="203" t="inlineStr">
+      <c r="B31" s="215" t="inlineStr"/>
+      <c r="C31" s="215" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D31" s="203" t="inlineStr">
+      <c r="D31" s="215" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E31" s="203" t="inlineStr"/>
+      <c r="E31" s="215" t="inlineStr"/>
       <c r="F31" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion - Section reading 1: Jerry Brotton, The Renaissance Bazaar, Chap 1 (15 pgs) Read Colu</t>
@@ -1889,18 +1925,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B32" s="203" t="inlineStr"/>
-      <c r="C32" s="203" t="inlineStr">
+      <c r="B32" s="215" t="inlineStr"/>
+      <c r="C32" s="215" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D32" s="203" t="inlineStr">
+      <c r="D32" s="215" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E32" s="203" t="inlineStr"/>
+      <c r="E32" s="215" t="inlineStr"/>
       <c r="F32" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion - Section reading 2: Bernal Diaz del Castillo, The True History of the Conquest of Ne</t>
@@ -1913,18 +1949,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B33" s="203" t="inlineStr"/>
-      <c r="C33" s="203" t="inlineStr">
+      <c r="B33" s="215" t="inlineStr"/>
+      <c r="C33" s="215" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="D33" s="203" t="inlineStr">
+      <c r="D33" s="215" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="E33" s="203" t="inlineStr"/>
+      <c r="E33" s="215" t="inlineStr"/>
       <c r="F33" s="99" t="inlineStr">
         <is>
           <t>Week Oct 13-16: The Reformation</t>
@@ -1937,18 +1973,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B34" s="203" t="inlineStr"/>
-      <c r="C34" s="203" t="inlineStr">
+      <c r="B34" s="215" t="inlineStr"/>
+      <c r="C34" s="215" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="D34" s="203" t="inlineStr">
+      <c r="D34" s="215" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="E34" s="203" t="inlineStr"/>
+      <c r="E34" s="215" t="inlineStr"/>
       <c r="F34" s="99" t="inlineStr">
         <is>
           <t>Week Oct 20-23: The Reformation</t>
@@ -1961,18 +1997,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B35" s="203" t="inlineStr"/>
-      <c r="C35" s="203" t="inlineStr">
+      <c r="B35" s="215" t="inlineStr"/>
+      <c r="C35" s="215" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D35" s="203" t="inlineStr">
+      <c r="D35" s="215" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E35" s="203" t="inlineStr"/>
+      <c r="E35" s="215" t="inlineStr"/>
       <c r="F35" s="99" t="inlineStr">
         <is>
           <t>Week Oct 27-30: Reformation</t>
@@ -1985,18 +2021,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B36" s="203" t="inlineStr"/>
-      <c r="C36" s="203" t="inlineStr">
+      <c r="B36" s="215" t="inlineStr"/>
+      <c r="C36" s="215" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D36" s="203" t="inlineStr">
+      <c r="D36" s="215" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E36" s="203" t="inlineStr"/>
+      <c r="E36" s="215" t="inlineStr"/>
       <c r="F36" s="99" t="inlineStr">
         <is>
           <t xml:space="preserve">Week Oct 27-30: Reformation - Section reading 1: Barbara Diefendorf, ed., The Saint Bartholomew’s Day Massacre: A Brief </t>
@@ -2009,18 +2045,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B37" s="203" t="inlineStr"/>
-      <c r="C37" s="203" t="inlineStr">
+      <c r="B37" s="215" t="inlineStr"/>
+      <c r="C37" s="215" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D37" s="203" t="inlineStr">
+      <c r="D37" s="215" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E37" s="203" t="inlineStr"/>
+      <c r="E37" s="215" t="inlineStr"/>
       <c r="F37" s="99" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science</t>
@@ -2033,18 +2069,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B38" s="203" t="inlineStr"/>
-      <c r="C38" s="203" t="inlineStr">
+      <c r="B38" s="215" t="inlineStr"/>
+      <c r="C38" s="215" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D38" s="203" t="inlineStr">
+      <c r="D38" s="215" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E38" s="203" t="inlineStr"/>
+      <c r="E38" s="215" t="inlineStr"/>
       <c r="F38" s="99" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science - Section reading 1: Brian Levack, The Witchcraft Sourcebook, Chaps 36-44, 46-47 103.Lev</t>
@@ -2057,18 +2093,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B39" s="203" t="inlineStr"/>
-      <c r="C39" s="203" t="inlineStr">
+      <c r="B39" s="215" t="inlineStr"/>
+      <c r="C39" s="215" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D39" s="203" t="inlineStr">
+      <c r="D39" s="215" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E39" s="203" t="inlineStr"/>
+      <c r="E39" s="215" t="inlineStr"/>
       <c r="F39" s="99" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment - Section reading 1: Excerpt: John Locke, Two Treatises of Government (1689) Excerpt: Rous</t>
@@ -2081,18 +2117,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B40" s="203" t="inlineStr"/>
-      <c r="C40" s="203" t="inlineStr">
+      <c r="B40" s="215" t="inlineStr"/>
+      <c r="C40" s="215" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D40" s="203" t="inlineStr">
+      <c r="D40" s="215" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E40" s="203" t="inlineStr"/>
+      <c r="E40" s="215" t="inlineStr"/>
       <c r="F40" s="99" t="inlineStr">
         <is>
           <t>Week Nov 17-20: Enlightenment</t>
@@ -2105,18 +2141,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B41" s="203" t="inlineStr"/>
-      <c r="C41" s="203" t="inlineStr">
+      <c r="B41" s="215" t="inlineStr"/>
+      <c r="C41" s="215" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D41" s="203" t="inlineStr">
+      <c r="D41" s="215" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E41" s="203" t="inlineStr"/>
+      <c r="E41" s="215" t="inlineStr"/>
       <c r="F41" s="99" t="inlineStr">
         <is>
           <t xml:space="preserve">Week Nov 17-20: Enlightenment - Section reading 1: Video: Africa &amp; Britain, A Forgotten History, Episode 2: Freedom (50 </t>
@@ -2129,18 +2165,18 @@
           <t>Identification Quizzes</t>
         </is>
       </c>
-      <c r="B42" s="201" t="inlineStr">
+      <c r="B42" s="213" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C42" s="204" t="inlineStr"/>
-      <c r="D42" s="204" t="inlineStr">
+      <c r="C42" s="216" t="inlineStr"/>
+      <c r="D42" s="216" t="inlineStr">
         <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="E42" s="204" t="inlineStr">
+      <c r="E42" s="216" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2156,18 +2192,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B43" s="203" t="inlineStr"/>
-      <c r="C43" s="203" t="inlineStr">
+      <c r="B43" s="215" t="inlineStr"/>
+      <c r="C43" s="215" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D43" s="203" t="inlineStr">
+      <c r="D43" s="215" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E43" s="203" t="inlineStr"/>
+      <c r="E43" s="215" t="inlineStr"/>
       <c r="F43" s="99" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death (lecture topics)</t>
@@ -2180,18 +2216,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B44" s="203" t="inlineStr"/>
-      <c r="C44" s="203" t="inlineStr">
+      <c r="B44" s="215" t="inlineStr"/>
+      <c r="C44" s="215" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D44" s="203" t="inlineStr">
+      <c r="D44" s="215" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E44" s="203" t="inlineStr"/>
+      <c r="E44" s="215" t="inlineStr"/>
       <c r="F44" s="99" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life (lecture topics)</t>
@@ -2204,18 +2240,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B45" s="203" t="inlineStr"/>
-      <c r="C45" s="203" t="inlineStr">
+      <c r="B45" s="215" t="inlineStr"/>
+      <c r="C45" s="215" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D45" s="203" t="inlineStr">
+      <c r="D45" s="215" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E45" s="203" t="inlineStr"/>
+      <c r="E45" s="215" t="inlineStr"/>
       <c r="F45" s="99" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance (lecture topics)</t>
@@ -2228,18 +2264,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B46" s="203" t="inlineStr"/>
-      <c r="C46" s="203" t="inlineStr">
+      <c r="B46" s="215" t="inlineStr"/>
+      <c r="C46" s="215" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D46" s="203" t="inlineStr">
+      <c r="D46" s="215" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E46" s="203" t="inlineStr"/>
+      <c r="E46" s="215" t="inlineStr"/>
       <c r="F46" s="99" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance (lecture topics)</t>
@@ -2252,18 +2288,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B47" s="203" t="inlineStr"/>
-      <c r="C47" s="203" t="inlineStr">
+      <c r="B47" s="215" t="inlineStr"/>
+      <c r="C47" s="215" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D47" s="203" t="inlineStr">
+      <c r="D47" s="215" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E47" s="203" t="inlineStr"/>
+      <c r="E47" s="215" t="inlineStr"/>
       <c r="F47" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion (lecture topics)</t>
@@ -2276,18 +2312,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B48" s="203" t="inlineStr"/>
-      <c r="C48" s="203" t="inlineStr">
+      <c r="B48" s="215" t="inlineStr"/>
+      <c r="C48" s="215" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="D48" s="203" t="inlineStr">
+      <c r="D48" s="215" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E48" s="203" t="inlineStr"/>
+      <c r="E48" s="215" t="inlineStr"/>
       <c r="F48" s="99" t="inlineStr">
         <is>
           <t>Week Oct 6-9: Midterm &amp; Break (lecture topics)</t>
@@ -2300,18 +2336,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B49" s="203" t="inlineStr"/>
-      <c r="C49" s="203" t="inlineStr">
+      <c r="B49" s="215" t="inlineStr"/>
+      <c r="C49" s="215" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="D49" s="203" t="inlineStr">
+      <c r="D49" s="215" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="E49" s="203" t="inlineStr"/>
+      <c r="E49" s="215" t="inlineStr"/>
       <c r="F49" s="99" t="inlineStr">
         <is>
           <t>Week Oct 13-16: The Reformation (lecture topics)</t>
@@ -2324,18 +2360,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B50" s="203" t="inlineStr"/>
-      <c r="C50" s="203" t="inlineStr">
+      <c r="B50" s="215" t="inlineStr"/>
+      <c r="C50" s="215" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="D50" s="203" t="inlineStr">
+      <c r="D50" s="215" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="E50" s="203" t="inlineStr"/>
+      <c r="E50" s="215" t="inlineStr"/>
       <c r="F50" s="99" t="inlineStr">
         <is>
           <t>Week Oct 20-23: The Reformation (lecture topics)</t>
@@ -2348,18 +2384,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B51" s="203" t="inlineStr"/>
-      <c r="C51" s="203" t="inlineStr">
+      <c r="B51" s="215" t="inlineStr"/>
+      <c r="C51" s="215" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D51" s="203" t="inlineStr">
+      <c r="D51" s="215" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E51" s="203" t="inlineStr"/>
+      <c r="E51" s="215" t="inlineStr"/>
       <c r="F51" s="99" t="inlineStr">
         <is>
           <t>Week Oct 27-30: Reformation (lecture topics)</t>
@@ -2372,18 +2408,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B52" s="203" t="inlineStr"/>
-      <c r="C52" s="203" t="inlineStr">
+      <c r="B52" s="215" t="inlineStr"/>
+      <c r="C52" s="215" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D52" s="203" t="inlineStr">
+      <c r="D52" s="215" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E52" s="203" t="inlineStr"/>
+      <c r="E52" s="215" t="inlineStr"/>
       <c r="F52" s="99" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science (lecture topics)</t>
@@ -2396,18 +2432,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B53" s="203" t="inlineStr"/>
-      <c r="C53" s="203" t="inlineStr">
+      <c r="B53" s="215" t="inlineStr"/>
+      <c r="C53" s="215" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D53" s="203" t="inlineStr">
+      <c r="D53" s="215" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E53" s="203" t="inlineStr"/>
+      <c r="E53" s="215" t="inlineStr"/>
       <c r="F53" s="99" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment (lecture topics)</t>
@@ -2420,18 +2456,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B54" s="203" t="inlineStr"/>
-      <c r="C54" s="203" t="inlineStr">
+      <c r="B54" s="215" t="inlineStr"/>
+      <c r="C54" s="215" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D54" s="203" t="inlineStr">
+      <c r="D54" s="215" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E54" s="203" t="inlineStr"/>
+      <c r="E54" s="215" t="inlineStr"/>
       <c r="F54" s="99" t="inlineStr">
         <is>
           <t>Week Nov 17-20: Enlightenment (lecture topics)</t>
@@ -2444,18 +2480,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B55" s="203" t="inlineStr"/>
-      <c r="C55" s="203" t="inlineStr">
+      <c r="B55" s="215" t="inlineStr"/>
+      <c r="C55" s="215" t="inlineStr">
         <is>
           <t>2026-12-01</t>
         </is>
       </c>
-      <c r="D55" s="203" t="inlineStr">
+      <c r="D55" s="215" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E55" s="203" t="inlineStr"/>
+      <c r="E55" s="215" t="inlineStr"/>
       <c r="F55" s="99" t="inlineStr">
         <is>
           <t>Week Dec 1-4: Modern Europe? (lecture topics)</t>
@@ -2468,18 +2504,18 @@
           <t>Extra Credit</t>
         </is>
       </c>
-      <c r="B56" s="201" t="inlineStr">
+      <c r="B56" s="213" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C56" s="202" t="inlineStr"/>
-      <c r="D56" s="202" t="inlineStr">
+      <c r="C56" s="214" t="inlineStr"/>
+      <c r="D56" s="214" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E56" s="202" t="inlineStr">
+      <c r="E56" s="214" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2636,18 +2672,18 @@
           <t>Midterm 1</t>
         </is>
       </c>
-      <c r="B10" s="205" t="inlineStr">
+      <c r="B10" s="217" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C10" s="206" t="inlineStr"/>
-      <c r="D10" s="206" t="inlineStr">
+      <c r="C10" s="218" t="inlineStr"/>
+      <c r="D10" s="218" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="E10" s="206" t="inlineStr">
+      <c r="E10" s="218" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2663,14 +2699,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B11" s="207" t="inlineStr"/>
-      <c r="C11" s="207" t="inlineStr"/>
-      <c r="D11" s="207" t="inlineStr">
+      <c r="B11" s="219" t="inlineStr"/>
+      <c r="C11" s="219" t="inlineStr"/>
+      <c r="D11" s="219" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="E11" s="207" t="inlineStr"/>
+      <c r="E11" s="219" t="inlineStr"/>
       <c r="F11" s="112" t="inlineStr">
         <is>
           <t>9/30 Midterm 1: 250 Points Chapters 1, 2, 3, 4, 5, 8</t>
@@ -2683,18 +2719,18 @@
           <t>Midterm 2</t>
         </is>
       </c>
-      <c r="B12" s="205" t="inlineStr">
+      <c r="B12" s="217" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C12" s="208" t="inlineStr"/>
-      <c r="D12" s="208" t="inlineStr">
+      <c r="C12" s="220" t="inlineStr"/>
+      <c r="D12" s="220" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E12" s="208" t="inlineStr">
+      <c r="E12" s="220" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2710,14 +2746,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B13" s="207" t="inlineStr"/>
-      <c r="C13" s="207" t="inlineStr"/>
-      <c r="D13" s="207" t="inlineStr">
+      <c r="B13" s="219" t="inlineStr"/>
+      <c r="C13" s="219" t="inlineStr"/>
+      <c r="D13" s="219" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E13" s="207" t="inlineStr"/>
+      <c r="E13" s="219" t="inlineStr"/>
       <c r="F13" s="112" t="inlineStr">
         <is>
           <t>10/26 Midterm 2: 250 Points Chapters 6, 7, 9, &amp; 16</t>
@@ -2730,18 +2766,18 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B14" s="205" t="inlineStr">
+      <c r="B14" s="217" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C14" s="206" t="inlineStr"/>
-      <c r="D14" s="206" t="inlineStr">
+      <c r="C14" s="218" t="inlineStr"/>
+      <c r="D14" s="218" t="inlineStr">
         <is>
           <t>2026-12-16</t>
         </is>
       </c>
-      <c r="E14" s="206" t="inlineStr">
+      <c r="E14" s="218" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2757,14 +2793,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B15" s="207" t="inlineStr"/>
-      <c r="C15" s="207" t="inlineStr"/>
-      <c r="D15" s="207" t="inlineStr">
+      <c r="B15" s="219" t="inlineStr"/>
+      <c r="C15" s="219" t="inlineStr"/>
+      <c r="D15" s="219" t="inlineStr">
         <is>
           <t>2026-12-16</t>
         </is>
       </c>
-      <c r="E15" s="207" t="inlineStr"/>
+      <c r="E15" s="219" t="inlineStr"/>
       <c r="F15" s="112" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -2777,22 +2813,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B16" s="205" t="inlineStr">
+      <c r="B16" s="217" t="inlineStr">
         <is>
           <t>170 pts</t>
         </is>
       </c>
-      <c r="C16" s="208" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="D16" s="208" t="inlineStr">
+      <c r="C16" s="220" t="inlineStr"/>
+      <c r="D16" s="220" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E16" s="208" t="inlineStr">
+      <c r="E16" s="220" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2808,14 +2840,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B17" s="207" t="inlineStr"/>
-      <c r="C17" s="207" t="inlineStr"/>
-      <c r="D17" s="207" t="inlineStr">
+      <c r="B17" s="219" t="inlineStr"/>
+      <c r="C17" s="219" t="inlineStr"/>
+      <c r="D17" s="219" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="E17" s="207" t="inlineStr"/>
+      <c r="E17" s="219" t="inlineStr"/>
       <c r="F17" s="112" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - Product Cost Accumulation: Job; Order Co: Chapter 3</t>
@@ -2828,14 +2860,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B18" s="207" t="inlineStr"/>
-      <c r="C18" s="207" t="inlineStr"/>
-      <c r="D18" s="207" t="inlineStr">
+      <c r="B18" s="219" t="inlineStr"/>
+      <c r="C18" s="219" t="inlineStr"/>
+      <c r="D18" s="219" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="E18" s="207" t="inlineStr"/>
+      <c r="E18" s="219" t="inlineStr"/>
       <c r="F18" s="112" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
@@ -2848,14 +2880,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B19" s="207" t="inlineStr"/>
-      <c r="C19" s="207" t="inlineStr"/>
-      <c r="D19" s="207" t="inlineStr">
+      <c r="B19" s="219" t="inlineStr"/>
+      <c r="C19" s="219" t="inlineStr"/>
+      <c r="D19" s="219" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E19" s="207" t="inlineStr"/>
+      <c r="E19" s="219" t="inlineStr"/>
       <c r="F19" s="112" t="inlineStr">
         <is>
           <t>Class 7 (9/16) - Activity Based Costing: Chapter 5- ONLY; LO 5.1, 2, 4 &amp; 5</t>
@@ -2868,14 +2900,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B20" s="207" t="inlineStr"/>
-      <c r="C20" s="207" t="inlineStr"/>
-      <c r="D20" s="207" t="inlineStr">
+      <c r="B20" s="219" t="inlineStr"/>
+      <c r="C20" s="219" t="inlineStr"/>
+      <c r="D20" s="219" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E20" s="207" t="inlineStr"/>
+      <c r="E20" s="219" t="inlineStr"/>
       <c r="F20" s="112" t="inlineStr">
         <is>
           <t>Class 7 (9/16) - 3-24, 3-28, 3-32; 15 Points</t>
@@ -2888,14 +2920,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B21" s="207" t="inlineStr"/>
-      <c r="C21" s="207" t="inlineStr"/>
-      <c r="D21" s="207" t="inlineStr">
+      <c r="B21" s="219" t="inlineStr"/>
+      <c r="C21" s="219" t="inlineStr"/>
+      <c r="D21" s="219" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="E21" s="207" t="inlineStr"/>
+      <c r="E21" s="219" t="inlineStr"/>
       <c r="F21" s="112" t="inlineStr">
         <is>
           <t>Class 8 (9/21) - Product Cost Accumulation: Pro-; cess Co: Chapter 4- ONLY; LO 4.1, 3, 4, &amp; 5</t>
@@ -2908,14 +2940,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B22" s="207" t="inlineStr"/>
-      <c r="C22" s="207" t="inlineStr"/>
-      <c r="D22" s="207" t="inlineStr">
+      <c r="B22" s="219" t="inlineStr"/>
+      <c r="C22" s="219" t="inlineStr"/>
+      <c r="D22" s="219" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="E22" s="207" t="inlineStr"/>
+      <c r="E22" s="219" t="inlineStr"/>
       <c r="F22" s="112" t="inlineStr">
         <is>
           <t>Class 8 (9/21) - 5-27 5-46; 10 Points</t>
@@ -2928,14 +2960,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B23" s="207" t="inlineStr"/>
-      <c r="C23" s="207" t="inlineStr"/>
-      <c r="D23" s="207" t="inlineStr">
+      <c r="B23" s="219" t="inlineStr"/>
+      <c r="C23" s="219" t="inlineStr"/>
+      <c r="D23" s="219" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="E23" s="207" t="inlineStr"/>
+      <c r="E23" s="219" t="inlineStr"/>
       <c r="F23" s="112" t="inlineStr">
         <is>
           <t>Class 9 (9/23) - Cost of Quality &amp; ESG &amp;; Overview of; • : Chapter 8 - ONLY; LO 8.7, 8, 9</t>
@@ -2948,14 +2980,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B24" s="207" t="inlineStr"/>
-      <c r="C24" s="207" t="inlineStr"/>
-      <c r="D24" s="207" t="inlineStr">
+      <c r="B24" s="219" t="inlineStr"/>
+      <c r="C24" s="219" t="inlineStr"/>
+      <c r="D24" s="219" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="E24" s="207" t="inlineStr"/>
+      <c r="E24" s="219" t="inlineStr"/>
       <c r="F24" s="112" t="inlineStr">
         <is>
           <t>Class 9 (9/23) - 4-21, 4-22; 10 Points</t>
@@ -2968,14 +3000,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B25" s="207" t="inlineStr"/>
-      <c r="C25" s="207" t="inlineStr"/>
-      <c r="D25" s="207" t="inlineStr">
+      <c r="B25" s="219" t="inlineStr"/>
+      <c r="C25" s="219" t="inlineStr"/>
+      <c r="D25" s="219" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E25" s="207" t="inlineStr"/>
+      <c r="E25" s="219" t="inlineStr"/>
       <c r="F25" s="112" t="inlineStr">
         <is>
           <t>Class 10 (9/28) - Catchup &amp; Midterm Review</t>
@@ -2988,14 +3020,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B26" s="207" t="inlineStr"/>
-      <c r="C26" s="207" t="inlineStr"/>
-      <c r="D26" s="207" t="inlineStr">
+      <c r="B26" s="219" t="inlineStr"/>
+      <c r="C26" s="219" t="inlineStr"/>
+      <c r="D26" s="219" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E26" s="207" t="inlineStr"/>
+      <c r="E26" s="219" t="inlineStr"/>
       <c r="F26" s="112" t="inlineStr">
         <is>
           <t>Class 10 (9/28) - 8-28, 8-29; 10 Points</t>
@@ -3008,14 +3040,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B27" s="207" t="inlineStr"/>
-      <c r="C27" s="207" t="inlineStr"/>
-      <c r="D27" s="207" t="inlineStr">
+      <c r="B27" s="219" t="inlineStr"/>
+      <c r="C27" s="219" t="inlineStr"/>
+      <c r="D27" s="219" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="E27" s="207" t="inlineStr"/>
+      <c r="E27" s="219" t="inlineStr"/>
       <c r="F27" s="112" t="inlineStr">
         <is>
           <t>Class 12 (10/7) - Cost volume profit analysis: Chapter 7</t>
@@ -3028,14 +3060,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B28" s="207" t="inlineStr"/>
-      <c r="C28" s="207" t="inlineStr"/>
-      <c r="D28" s="207" t="inlineStr">
+      <c r="B28" s="219" t="inlineStr"/>
+      <c r="C28" s="219" t="inlineStr"/>
+      <c r="D28" s="219" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="E28" s="207" t="inlineStr"/>
+      <c r="E28" s="219" t="inlineStr"/>
       <c r="F28" s="112" t="inlineStr">
         <is>
           <t>Class 12 (10/7) - 6-24, 6-25, 6-34; 15 Points</t>
@@ -3048,14 +3080,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B29" s="207" t="inlineStr"/>
-      <c r="C29" s="207" t="inlineStr"/>
-      <c r="D29" s="207" t="inlineStr">
+      <c r="B29" s="219" t="inlineStr"/>
+      <c r="C29" s="219" t="inlineStr"/>
+      <c r="D29" s="219" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E29" s="207" t="inlineStr"/>
+      <c r="E29" s="219" t="inlineStr"/>
       <c r="F29" s="112" t="inlineStr">
         <is>
           <t>Class 14 (10/14) - Financial planning and analysis:; Static: Chapter 9</t>
@@ -3068,14 +3100,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B30" s="207" t="inlineStr"/>
-      <c r="C30" s="207" t="inlineStr"/>
-      <c r="D30" s="207" t="inlineStr">
+      <c r="B30" s="219" t="inlineStr"/>
+      <c r="C30" s="219" t="inlineStr"/>
+      <c r="D30" s="219" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E30" s="207" t="inlineStr"/>
+      <c r="E30" s="219" t="inlineStr"/>
       <c r="F30" s="112" t="inlineStr">
         <is>
           <t>Class 14 (10/14) - 7-29, 7-33, 7-40; 15 Points</t>
@@ -3088,14 +3120,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B31" s="207" t="inlineStr"/>
-      <c r="C31" s="207" t="inlineStr"/>
-      <c r="D31" s="207" t="inlineStr">
+      <c r="B31" s="219" t="inlineStr"/>
+      <c r="C31" s="219" t="inlineStr"/>
+      <c r="D31" s="219" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E31" s="207" t="inlineStr"/>
+      <c r="E31" s="219" t="inlineStr"/>
       <c r="F31" s="112" t="inlineStr">
         <is>
           <t>Class 15 (10/19) - Capital Budgeting; Practice Midterm Ques: Chapter 16- ONLY; LO 16.1, 2, 3</t>
@@ -3108,14 +3140,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B32" s="207" t="inlineStr"/>
-      <c r="C32" s="207" t="inlineStr"/>
-      <c r="D32" s="207" t="inlineStr">
+      <c r="B32" s="219" t="inlineStr"/>
+      <c r="C32" s="219" t="inlineStr"/>
+      <c r="D32" s="219" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E32" s="207" t="inlineStr"/>
+      <c r="E32" s="219" t="inlineStr"/>
       <c r="F32" s="112" t="inlineStr">
         <is>
           <t>Class 15 (10/19) - 9-25, 9-28, 9-37; 15 - Points</t>
@@ -3128,14 +3160,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B33" s="207" t="inlineStr"/>
-      <c r="C33" s="207" t="inlineStr"/>
-      <c r="D33" s="207" t="inlineStr">
+      <c r="B33" s="219" t="inlineStr"/>
+      <c r="C33" s="219" t="inlineStr"/>
+      <c r="D33" s="219" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E33" s="207" t="inlineStr"/>
+      <c r="E33" s="219" t="inlineStr"/>
       <c r="F33" s="112" t="inlineStr">
         <is>
           <t>Class 16 (10/21) - Catchup &amp; Midterm Review</t>
@@ -3148,14 +3180,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B34" s="207" t="inlineStr"/>
-      <c r="C34" s="207" t="inlineStr"/>
-      <c r="D34" s="207" t="inlineStr">
+      <c r="B34" s="219" t="inlineStr"/>
+      <c r="C34" s="219" t="inlineStr"/>
+      <c r="D34" s="219" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E34" s="207" t="inlineStr"/>
+      <c r="E34" s="219" t="inlineStr"/>
       <c r="F34" s="112" t="inlineStr">
         <is>
           <t>Class 16 (10/21) - 16-28, 16-40; 10 Points</t>
@@ -3168,14 +3200,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B35" s="207" t="inlineStr"/>
-      <c r="C35" s="207" t="inlineStr"/>
-      <c r="D35" s="207" t="inlineStr">
+      <c r="B35" s="219" t="inlineStr"/>
+      <c r="C35" s="219" t="inlineStr"/>
+      <c r="D35" s="219" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="E35" s="207" t="inlineStr"/>
+      <c r="E35" s="219" t="inlineStr"/>
       <c r="F35" s="112" t="inlineStr">
         <is>
           <t>Class 19 (11/4) - Sales Variance Analysis; Flexible Budget: Chapter 11 - ONLY; LO 11.1, 11.2 &amp;; Appendix B</t>
@@ -3188,14 +3220,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B36" s="207" t="inlineStr"/>
-      <c r="C36" s="207" t="inlineStr"/>
-      <c r="D36" s="207" t="inlineStr">
+      <c r="B36" s="219" t="inlineStr"/>
+      <c r="C36" s="219" t="inlineStr"/>
+      <c r="D36" s="219" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="E36" s="207" t="inlineStr"/>
+      <c r="E36" s="219" t="inlineStr"/>
       <c r="F36" s="112" t="inlineStr">
         <is>
           <t>Class 19 (11/4) - 10-26, 10-30; 10 Points</t>
@@ -3208,14 +3240,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B37" s="207" t="inlineStr"/>
-      <c r="C37" s="207" t="inlineStr"/>
-      <c r="D37" s="207" t="inlineStr">
+      <c r="B37" s="219" t="inlineStr"/>
+      <c r="C37" s="219" t="inlineStr"/>
+      <c r="D37" s="219" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E37" s="207" t="inlineStr"/>
+      <c r="E37" s="219" t="inlineStr"/>
       <c r="F37" s="112" t="inlineStr">
         <is>
           <t>Class 20 (11/9) - Investment Centers: Chapter 13- ONLY; LO 13-1, 2, 3, 4</t>
@@ -3228,14 +3260,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B38" s="207" t="inlineStr"/>
-      <c r="C38" s="207" t="inlineStr"/>
-      <c r="D38" s="207" t="inlineStr">
+      <c r="B38" s="219" t="inlineStr"/>
+      <c r="C38" s="219" t="inlineStr"/>
+      <c r="D38" s="219" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E38" s="207" t="inlineStr"/>
+      <c r="E38" s="219" t="inlineStr"/>
       <c r="F38" s="112" t="inlineStr">
         <is>
           <t>Class 20 (11/9) - 11-31, 11-52; 10 Points</t>
@@ -3248,14 +3280,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B39" s="207" t="inlineStr"/>
-      <c r="C39" s="207" t="inlineStr"/>
-      <c r="D39" s="207" t="inlineStr">
+      <c r="B39" s="219" t="inlineStr"/>
+      <c r="C39" s="219" t="inlineStr"/>
+      <c r="D39" s="219" t="inlineStr">
         <is>
           <t>2026-11-16</t>
         </is>
       </c>
-      <c r="E39" s="207" t="inlineStr"/>
+      <c r="E39" s="219" t="inlineStr"/>
       <c r="F39" s="112" t="inlineStr">
         <is>
           <t>Class 21 (11/16) - AI &amp; FP&amp;A</t>
@@ -3268,14 +3300,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B40" s="207" t="inlineStr"/>
-      <c r="C40" s="207" t="inlineStr"/>
-      <c r="D40" s="207" t="inlineStr">
+      <c r="B40" s="219" t="inlineStr"/>
+      <c r="C40" s="219" t="inlineStr"/>
+      <c r="D40" s="219" t="inlineStr">
         <is>
           <t>2026-11-16</t>
         </is>
       </c>
-      <c r="E40" s="207" t="inlineStr"/>
+      <c r="E40" s="219" t="inlineStr"/>
       <c r="F40" s="112" t="inlineStr">
         <is>
           <t>Class 21 (11/16) - 13-29, 13-33; 10 Points</t>
@@ -3288,14 +3320,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B41" s="207" t="inlineStr"/>
-      <c r="C41" s="207" t="inlineStr"/>
-      <c r="D41" s="207" t="inlineStr">
+      <c r="B41" s="219" t="inlineStr"/>
+      <c r="C41" s="219" t="inlineStr"/>
+      <c r="D41" s="219" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E41" s="207" t="inlineStr"/>
+      <c r="E41" s="219" t="inlineStr"/>
       <c r="F41" s="112" t="inlineStr">
         <is>
           <t>Class 2 (12/2) - Catchup &amp; Final Review; Practice Final Questions Posted to Brightspace at; 5:00 PM</t>
@@ -3308,14 +3340,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B42" s="207" t="inlineStr"/>
-      <c r="C42" s="207" t="inlineStr"/>
-      <c r="D42" s="207" t="inlineStr">
+      <c r="B42" s="219" t="inlineStr"/>
+      <c r="C42" s="219" t="inlineStr"/>
+      <c r="D42" s="219" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E42" s="207" t="inlineStr"/>
+      <c r="E42" s="219" t="inlineStr"/>
       <c r="F42" s="112" t="inlineStr">
         <is>
           <t>Class 2 (12/2) - 14-35, 14-41; 10 Points; Assignments listed Be-; low Due by11:59 PM; Linked In Learning; E</t>
@@ -3328,22 +3360,22 @@
           <t>LinkedIn Learning Excel Certification</t>
         </is>
       </c>
-      <c r="B43" s="205" t="inlineStr">
+      <c r="B43" s="217" t="inlineStr">
         <is>
           <t>75 pts</t>
         </is>
       </c>
-      <c r="C43" s="206" t="inlineStr">
+      <c r="C43" s="218" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D43" s="206" t="inlineStr">
+      <c r="D43" s="218" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E43" s="206" t="inlineStr">
+      <c r="E43" s="218" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3359,18 +3391,18 @@
           <t>Certification</t>
         </is>
       </c>
-      <c r="B44" s="207" t="inlineStr"/>
-      <c r="C44" s="207" t="inlineStr">
+      <c r="B44" s="219" t="inlineStr"/>
+      <c r="C44" s="219" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D44" s="207" t="inlineStr">
+      <c r="D44" s="219" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E44" s="207" t="inlineStr"/>
+      <c r="E44" s="219" t="inlineStr"/>
       <c r="F44" s="112" t="inlineStr">
         <is>
           <t>LinkedIn Learning Excel Certification</t>
@@ -3383,22 +3415,22 @@
           <t>Stukent Simternship</t>
         </is>
       </c>
-      <c r="B45" s="205" t="inlineStr">
+      <c r="B45" s="217" t="inlineStr">
         <is>
           <t>75 pts</t>
         </is>
       </c>
-      <c r="C45" s="208" t="inlineStr">
+      <c r="C45" s="220" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D45" s="208" t="inlineStr">
+      <c r="D45" s="220" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E45" s="208" t="inlineStr">
+      <c r="E45" s="220" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3414,18 +3446,18 @@
           <t>Certification</t>
         </is>
       </c>
-      <c r="B46" s="207" t="inlineStr"/>
-      <c r="C46" s="207" t="inlineStr">
+      <c r="B46" s="219" t="inlineStr"/>
+      <c r="C46" s="219" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D46" s="207" t="inlineStr">
+      <c r="D46" s="219" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E46" s="207" t="inlineStr"/>
+      <c r="E46" s="219" t="inlineStr"/>
       <c r="F46" s="112" t="inlineStr">
         <is>
           <t>Stukent Simternship</t>
@@ -3579,22 +3611,22 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B10" s="209" t="inlineStr">
+      <c r="B10" s="221" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="C10" s="210" t="inlineStr">
+      <c r="C10" s="222" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D10" s="210" t="inlineStr">
+      <c r="D10" s="222" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E10" s="210" t="inlineStr">
+      <c r="E10" s="222" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3610,18 +3642,18 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B11" s="211" t="inlineStr"/>
-      <c r="C11" s="211" t="inlineStr">
+      <c r="B11" s="223" t="inlineStr"/>
+      <c r="C11" s="223" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D11" s="211" t="inlineStr">
+      <c r="D11" s="223" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E11" s="211" t="inlineStr"/>
+      <c r="E11" s="223" t="inlineStr"/>
       <c r="F11" s="126" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -3634,22 +3666,22 @@
           <t>Participation</t>
         </is>
       </c>
-      <c r="B12" s="209" t="inlineStr">
+      <c r="B12" s="221" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C12" s="212" t="inlineStr">
+      <c r="C12" s="224" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D12" s="212" t="inlineStr">
+      <c r="D12" s="224" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E12" s="212" t="inlineStr">
+      <c r="E12" s="224" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3665,14 +3697,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B13" s="211" t="inlineStr"/>
-      <c r="C13" s="211" t="inlineStr">
+      <c r="B13" s="223" t="inlineStr"/>
+      <c r="C13" s="223" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D13" s="211" t="inlineStr"/>
-      <c r="E13" s="211" t="inlineStr"/>
+      <c r="D13" s="223" t="inlineStr"/>
+      <c r="E13" s="223" t="inlineStr"/>
       <c r="F13" s="126" t="inlineStr">
         <is>
           <t>Research: SONA registration opens</t>
@@ -3685,14 +3717,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B14" s="211" t="inlineStr"/>
-      <c r="C14" s="211" t="inlineStr">
+      <c r="B14" s="223" t="inlineStr"/>
+      <c r="C14" s="223" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="D14" s="211" t="inlineStr"/>
-      <c r="E14" s="211" t="inlineStr"/>
+      <c r="D14" s="223" t="inlineStr"/>
+      <c r="E14" s="223" t="inlineStr"/>
       <c r="F14" s="126" t="inlineStr">
         <is>
           <t>Research: Prescreening questionnaire opens</t>
@@ -3705,14 +3737,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B15" s="211" t="inlineStr"/>
-      <c r="C15" s="211" t="inlineStr"/>
-      <c r="D15" s="211" t="inlineStr">
+      <c r="B15" s="223" t="inlineStr"/>
+      <c r="C15" s="223" t="inlineStr"/>
+      <c r="D15" s="223" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="E15" s="211" t="inlineStr"/>
+      <c r="E15" s="223" t="inlineStr"/>
       <c r="F15" s="126" t="inlineStr">
         <is>
           <t>Research: Setup deadline (registration, prescreening, contacts)</t>
@@ -3725,14 +3757,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B16" s="211" t="inlineStr"/>
-      <c r="C16" s="211" t="inlineStr">
+      <c r="B16" s="223" t="inlineStr"/>
+      <c r="C16" s="223" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="D16" s="211" t="inlineStr"/>
-      <c r="E16" s="211" t="inlineStr"/>
+      <c r="D16" s="223" t="inlineStr"/>
+      <c r="E16" s="223" t="inlineStr"/>
       <c r="F16" s="126" t="inlineStr">
         <is>
           <t>Research: Study invitations begin (after setup)</t>
@@ -3745,14 +3777,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B17" s="211" t="inlineStr"/>
-      <c r="C17" s="211" t="inlineStr"/>
-      <c r="D17" s="211" t="inlineStr">
+      <c r="B17" s="223" t="inlineStr"/>
+      <c r="C17" s="223" t="inlineStr"/>
+      <c r="D17" s="223" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E17" s="211" t="inlineStr"/>
+      <c r="E17" s="223" t="inlineStr"/>
       <c r="F17" s="126" t="inlineStr">
         <is>
           <t>Research: Employee contact surveys sent</t>
@@ -3765,14 +3797,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B18" s="211" t="inlineStr"/>
-      <c r="C18" s="211" t="inlineStr"/>
-      <c r="D18" s="211" t="inlineStr">
+      <c r="B18" s="223" t="inlineStr"/>
+      <c r="C18" s="223" t="inlineStr"/>
+      <c r="D18" s="223" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E18" s="211" t="inlineStr"/>
+      <c r="E18" s="223" t="inlineStr"/>
       <c r="F18" s="126" t="inlineStr">
         <is>
           <t>Research: Complete 2.0 research credits</t>
@@ -3785,22 +3817,22 @@
           <t>Midterm Exam</t>
         </is>
       </c>
-      <c r="B19" s="209" t="inlineStr">
+      <c r="B19" s="221" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C19" s="210" t="inlineStr">
+      <c r="C19" s="222" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D19" s="210" t="inlineStr">
+      <c r="D19" s="222" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E19" s="210" t="inlineStr">
+      <c r="E19" s="222" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3816,18 +3848,18 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B20" s="211" t="inlineStr"/>
-      <c r="C20" s="211" t="inlineStr">
+      <c r="B20" s="223" t="inlineStr"/>
+      <c r="C20" s="223" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D20" s="211" t="inlineStr">
+      <c r="D20" s="223" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E20" s="211" t="inlineStr"/>
+      <c r="E20" s="223" t="inlineStr"/>
       <c r="F20" s="126" t="inlineStr">
         <is>
           <t>Midterm Exam</t>
@@ -3840,22 +3872,22 @@
           <t>Team Project Paper</t>
         </is>
       </c>
-      <c r="B21" s="209" t="inlineStr">
+      <c r="B21" s="221" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C21" s="212" t="inlineStr">
+      <c r="C21" s="224" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D21" s="212" t="inlineStr">
+      <c r="D21" s="224" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E21" s="212" t="inlineStr">
+      <c r="E21" s="224" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3871,18 +3903,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B22" s="211" t="inlineStr"/>
-      <c r="C22" s="211" t="inlineStr">
+      <c r="B22" s="223" t="inlineStr"/>
+      <c r="C22" s="223" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D22" s="211" t="inlineStr">
+      <c r="D22" s="223" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E22" s="211" t="inlineStr"/>
+      <c r="E22" s="223" t="inlineStr"/>
       <c r="F22" s="126" t="inlineStr">
         <is>
           <t>Team project outline</t>
@@ -3895,18 +3927,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B23" s="211" t="inlineStr"/>
-      <c r="C23" s="211" t="inlineStr">
+      <c r="B23" s="223" t="inlineStr"/>
+      <c r="C23" s="223" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D23" s="211" t="inlineStr">
+      <c r="D23" s="223" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E23" s="211" t="inlineStr"/>
+      <c r="E23" s="223" t="inlineStr"/>
       <c r="F23" s="126" t="inlineStr">
         <is>
           <t>Team project paper</t>
@@ -3919,22 +3951,22 @@
           <t>Final Reflection Paper</t>
         </is>
       </c>
-      <c r="B24" s="209" t="inlineStr">
+      <c r="B24" s="221" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C24" s="210" t="inlineStr">
+      <c r="C24" s="222" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D24" s="210" t="inlineStr">
+      <c r="D24" s="222" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E24" s="210" t="inlineStr">
+      <c r="E24" s="222" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3950,18 +3982,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B25" s="211" t="inlineStr"/>
-      <c r="C25" s="211" t="inlineStr">
+      <c r="B25" s="223" t="inlineStr"/>
+      <c r="C25" s="223" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D25" s="211" t="inlineStr">
+      <c r="D25" s="223" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E25" s="211" t="inlineStr"/>
+      <c r="E25" s="223" t="inlineStr"/>
       <c r="F25" s="126" t="inlineStr">
         <is>
           <t>Personal Reflection Paper</t>
@@ -3974,22 +4006,22 @@
           <t>Presentation</t>
         </is>
       </c>
-      <c r="B26" s="209" t="inlineStr">
+      <c r="B26" s="221" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C26" s="212" t="inlineStr">
+      <c r="C26" s="224" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D26" s="212" t="inlineStr">
+      <c r="D26" s="224" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E26" s="212" t="inlineStr">
+      <c r="E26" s="224" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4005,18 +4037,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B27" s="211" t="inlineStr"/>
-      <c r="C27" s="211" t="inlineStr">
+      <c r="B27" s="223" t="inlineStr"/>
+      <c r="C27" s="223" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D27" s="211" t="inlineStr">
+      <c r="D27" s="223" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E27" s="211" t="inlineStr"/>
+      <c r="E27" s="223" t="inlineStr"/>
       <c r="F27" s="126" t="inlineStr">
         <is>
           <t>Presentation slides</t>
@@ -4029,22 +4061,22 @@
           <t>Case Analysis Assignments</t>
         </is>
       </c>
-      <c r="B28" s="209" t="inlineStr">
+      <c r="B28" s="221" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C28" s="210" t="inlineStr">
+      <c r="C28" s="222" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D28" s="210" t="inlineStr">
+      <c r="D28" s="222" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E28" s="210" t="inlineStr">
+      <c r="E28" s="222" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4060,18 +4092,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B29" s="211" t="inlineStr"/>
-      <c r="C29" s="211" t="inlineStr">
+      <c r="B29" s="223" t="inlineStr"/>
+      <c r="C29" s="223" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D29" s="211" t="inlineStr">
+      <c r="D29" s="223" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E29" s="211" t="inlineStr"/>
+      <c r="E29" s="223" t="inlineStr"/>
       <c r="F29" s="126" t="inlineStr">
         <is>
           <t>Thomas Green Case Analysis Memo</t>
@@ -4084,18 +4116,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B30" s="211" t="inlineStr"/>
-      <c r="C30" s="211" t="inlineStr">
+      <c r="B30" s="223" t="inlineStr"/>
+      <c r="C30" s="223" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D30" s="211" t="inlineStr">
+      <c r="D30" s="223" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E30" s="211" t="inlineStr"/>
+      <c r="E30" s="223" t="inlineStr"/>
       <c r="F30" s="126" t="inlineStr">
         <is>
           <t>SkillsForTomorrow Analysis Memo</t>
@@ -4108,22 +4140,22 @@
           <t>Proposal &amp; Team Contract</t>
         </is>
       </c>
-      <c r="B31" s="209" t="inlineStr">
+      <c r="B31" s="221" t="inlineStr">
         <is>
           <t>3%</t>
         </is>
       </c>
-      <c r="C31" s="212" t="inlineStr">
+      <c r="C31" s="224" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D31" s="212" t="inlineStr">
+      <c r="D31" s="224" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E31" s="212" t="inlineStr">
+      <c r="E31" s="224" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4139,18 +4171,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B32" s="211" t="inlineStr"/>
-      <c r="C32" s="211" t="inlineStr">
+      <c r="B32" s="223" t="inlineStr"/>
+      <c r="C32" s="223" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D32" s="211" t="inlineStr">
+      <c r="D32" s="223" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E32" s="211" t="inlineStr"/>
+      <c r="E32" s="223" t="inlineStr"/>
       <c r="F32" s="126" t="inlineStr">
         <is>
           <t>Team project proposal &amp; team contract</t>
@@ -4163,22 +4195,22 @@
           <t>Self &amp; Peer Evaluation</t>
         </is>
       </c>
-      <c r="B33" s="209" t="inlineStr">
+      <c r="B33" s="221" t="inlineStr">
         <is>
           <t>2%</t>
         </is>
       </c>
-      <c r="C33" s="210" t="inlineStr">
+      <c r="C33" s="222" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D33" s="210" t="inlineStr">
+      <c r="D33" s="222" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E33" s="210" t="inlineStr">
+      <c r="E33" s="222" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4194,18 +4226,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B34" s="211" t="inlineStr"/>
-      <c r="C34" s="211" t="inlineStr">
+      <c r="B34" s="223" t="inlineStr"/>
+      <c r="C34" s="223" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D34" s="211" t="inlineStr">
+      <c r="D34" s="223" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E34" s="211" t="inlineStr"/>
+      <c r="E34" s="223" t="inlineStr"/>
       <c r="F34" s="126" t="inlineStr">
         <is>
           <t>Self &amp; peer evaluation</t>
@@ -4218,22 +4250,18 @@
           <t>Personal Assessments (Connect)</t>
         </is>
       </c>
-      <c r="B35" s="209" t="inlineStr">
+      <c r="B35" s="221" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C35" s="212" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D35" s="212" t="inlineStr">
+      <c r="C35" s="224" t="inlineStr"/>
+      <c r="D35" s="224" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E35" s="212" t="inlineStr">
+      <c r="E35" s="224" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4249,14 +4277,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B36" s="211" t="inlineStr"/>
-      <c r="C36" s="211" t="inlineStr"/>
-      <c r="D36" s="211" t="inlineStr">
+      <c r="B36" s="223" t="inlineStr"/>
+      <c r="C36" s="223" t="inlineStr"/>
+      <c r="D36" s="223" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="E36" s="211" t="inlineStr"/>
+      <c r="E36" s="223" t="inlineStr"/>
       <c r="F36" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
@@ -4269,14 +4297,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B37" s="211" t="inlineStr"/>
-      <c r="C37" s="211" t="inlineStr"/>
-      <c r="D37" s="211" t="inlineStr">
+      <c r="B37" s="223" t="inlineStr"/>
+      <c r="C37" s="223" t="inlineStr"/>
+      <c r="D37" s="223" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="E37" s="211" t="inlineStr"/>
+      <c r="E37" s="223" t="inlineStr"/>
       <c r="F37" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
@@ -4289,14 +4317,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B38" s="211" t="inlineStr"/>
-      <c r="C38" s="211" t="inlineStr"/>
-      <c r="D38" s="211" t="inlineStr">
+      <c r="B38" s="223" t="inlineStr"/>
+      <c r="C38" s="223" t="inlineStr"/>
+      <c r="D38" s="223" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="E38" s="211" t="inlineStr"/>
+      <c r="E38" s="223" t="inlineStr"/>
       <c r="F38" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 5.01 - Assessing Your</t>
@@ -4309,14 +4337,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B39" s="211" t="inlineStr"/>
-      <c r="C39" s="211" t="inlineStr"/>
-      <c r="D39" s="211" t="inlineStr">
+      <c r="B39" s="223" t="inlineStr"/>
+      <c r="C39" s="223" t="inlineStr"/>
+      <c r="D39" s="223" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E39" s="211" t="inlineStr"/>
+      <c r="E39" s="223" t="inlineStr"/>
       <c r="F39" s="126" t="inlineStr">
         <is>
           <t>Connect: Sharpen Companion</t>
@@ -4329,14 +4357,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B40" s="211" t="inlineStr"/>
-      <c r="C40" s="211" t="inlineStr"/>
-      <c r="D40" s="211" t="inlineStr">
+      <c r="B40" s="223" t="inlineStr"/>
+      <c r="C40" s="223" t="inlineStr"/>
+      <c r="D40" s="223" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="E40" s="211" t="inlineStr"/>
+      <c r="E40" s="223" t="inlineStr"/>
       <c r="F40" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 11.01 - What is my</t>
@@ -4349,14 +4377,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B41" s="211" t="inlineStr"/>
-      <c r="C41" s="211" t="inlineStr"/>
-      <c r="D41" s="211" t="inlineStr">
+      <c r="B41" s="223" t="inlineStr"/>
+      <c r="C41" s="223" t="inlineStr"/>
+      <c r="D41" s="223" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="E41" s="211" t="inlineStr"/>
+      <c r="E41" s="223" t="inlineStr"/>
       <c r="F41" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 11.02 - What is my</t>
@@ -4369,14 +4397,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B42" s="211" t="inlineStr"/>
-      <c r="C42" s="211" t="inlineStr"/>
-      <c r="D42" s="211" t="inlineStr">
+      <c r="B42" s="223" t="inlineStr"/>
+      <c r="C42" s="223" t="inlineStr"/>
+      <c r="D42" s="223" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E42" s="211" t="inlineStr"/>
+      <c r="E42" s="223" t="inlineStr"/>
       <c r="F42" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 12.01 - What kind of</t>
@@ -4389,14 +4417,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B43" s="211" t="inlineStr"/>
-      <c r="C43" s="211" t="inlineStr"/>
-      <c r="D43" s="211" t="inlineStr">
+      <c r="B43" s="223" t="inlineStr"/>
+      <c r="C43" s="223" t="inlineStr"/>
+      <c r="D43" s="223" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E43" s="211" t="inlineStr"/>
+      <c r="E43" s="223" t="inlineStr"/>
       <c r="F43" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 10.5 - Preferred Conflict</t>
@@ -4409,14 +4437,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B44" s="211" t="inlineStr"/>
-      <c r="C44" s="211" t="inlineStr"/>
-      <c r="D44" s="211" t="inlineStr">
+      <c r="B44" s="223" t="inlineStr"/>
+      <c r="C44" s="223" t="inlineStr"/>
+      <c r="D44" s="223" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E44" s="211" t="inlineStr"/>
+      <c r="E44" s="223" t="inlineStr"/>
       <c r="F44" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 9.01 - Assessing My</t>
@@ -4429,14 +4457,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B45" s="211" t="inlineStr"/>
-      <c r="C45" s="211" t="inlineStr"/>
-      <c r="D45" s="211" t="inlineStr">
+      <c r="B45" s="223" t="inlineStr"/>
+      <c r="C45" s="223" t="inlineStr"/>
+      <c r="D45" s="223" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E45" s="211" t="inlineStr"/>
+      <c r="E45" s="223" t="inlineStr"/>
       <c r="F45" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 8.01 - Group</t>
@@ -4449,14 +4477,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B46" s="211" t="inlineStr"/>
-      <c r="C46" s="211" t="inlineStr"/>
-      <c r="D46" s="211" t="inlineStr">
+      <c r="B46" s="223" t="inlineStr"/>
+      <c r="C46" s="223" t="inlineStr"/>
+      <c r="D46" s="223" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="E46" s="211" t="inlineStr"/>
+      <c r="E46" s="223" t="inlineStr"/>
       <c r="F46" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 14.02 - What Type of Organizational Culture Do I</t>
@@ -4469,14 +4497,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B47" s="211" t="inlineStr"/>
-      <c r="C47" s="211" t="inlineStr"/>
-      <c r="D47" s="211" t="inlineStr">
+      <c r="B47" s="223" t="inlineStr"/>
+      <c r="C47" s="223" t="inlineStr"/>
+      <c r="D47" s="223" t="inlineStr">
         <is>
           <t>2026-11-30</t>
         </is>
       </c>
-      <c r="E47" s="211" t="inlineStr"/>
+      <c r="E47" s="223" t="inlineStr"/>
       <c r="F47" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 16.02 - What Is Your</t>
@@ -4489,14 +4517,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B48" s="211" t="inlineStr"/>
-      <c r="C48" s="211" t="inlineStr"/>
-      <c r="D48" s="211" t="inlineStr">
+      <c r="B48" s="223" t="inlineStr"/>
+      <c r="C48" s="223" t="inlineStr"/>
+      <c r="D48" s="223" t="inlineStr">
         <is>
           <t>2026-11-30</t>
         </is>
       </c>
-      <c r="E48" s="211" t="inlineStr"/>
+      <c r="E48" s="223" t="inlineStr"/>
       <c r="F48" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 16.03 - Assessing Your</t>
@@ -4509,14 +4537,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B49" s="211" t="inlineStr"/>
-      <c r="C49" s="211" t="inlineStr"/>
-      <c r="D49" s="211" t="inlineStr">
+      <c r="B49" s="223" t="inlineStr"/>
+      <c r="C49" s="223" t="inlineStr"/>
+      <c r="D49" s="223" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E49" s="211" t="inlineStr"/>
+      <c r="E49" s="223" t="inlineStr"/>
       <c r="F49" s="126" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 12.02 - Which influence</t>

</xml_diff>

<commit_message>
Add BUAD-281 Strategy section for homework-bank study approach
Inject optional strategy text into BUAD-281 calendar JSON and render
a green Strategy row on the Excel sheet between the weight bar and
assignment table. Documents the AI homework-bank mechanics approach.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-281" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-304" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-304" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-281" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -122,7 +122,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -224,6 +224,11 @@
         <fgColor rgb="00CDE1EE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -251,7 +256,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="225">
+  <cellXfs count="230">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -913,6 +918,21 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2551,945 +2571,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00FF7F0E"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F47"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
-        <is>
-          <t>BUAD-281 — Managerial Accounting</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="2">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/sources/buad-281-source.pdf","SEE HERE")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Instructor</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Braunegg</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Term</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Fall 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Required for an A</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Grading scale</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Total graded points in calendar: 1070 (letter scale not in document)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="151" t="inlineStr">
-        <is>
-          <t>Midterm 1 250 pts  |  Midterm 2 250 pts  |  Final Exam 250 pts  |  Homework 170 pts  |  LinkedIn Learning Excel Certification 75 pts  |  Stukent Simternship 75 pts</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>Weight</t>
-        </is>
-      </c>
-      <c r="C9" s="13" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>Due Date</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="inlineStr">
-        <is>
-          <t>Group Project</t>
-        </is>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="106" t="inlineStr">
-        <is>
-          <t>Midterm 1</t>
-        </is>
-      </c>
-      <c r="B10" s="217" t="inlineStr">
-        <is>
-          <t>250 pts</t>
-        </is>
-      </c>
-      <c r="C10" s="218" t="inlineStr"/>
-      <c r="D10" s="218" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="E10" s="218" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F10" s="109">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-midterm-1.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="110" t="inlineStr">
-        <is>
-          <t>Exam</t>
-        </is>
-      </c>
-      <c r="B11" s="219" t="inlineStr"/>
-      <c r="C11" s="219" t="inlineStr"/>
-      <c r="D11" s="219" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="E11" s="219" t="inlineStr"/>
-      <c r="F11" s="112" t="inlineStr">
-        <is>
-          <t>9/30 Midterm 1: 250 Points Chapters 1, 2, 3, 4, 5, 8</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="113" t="inlineStr">
-        <is>
-          <t>Midterm 2</t>
-        </is>
-      </c>
-      <c r="B12" s="217" t="inlineStr">
-        <is>
-          <t>250 pts</t>
-        </is>
-      </c>
-      <c r="C12" s="220" t="inlineStr"/>
-      <c r="D12" s="220" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="E12" s="220" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F12" s="115">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-midterm-2.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="110" t="inlineStr">
-        <is>
-          <t>Exam</t>
-        </is>
-      </c>
-      <c r="B13" s="219" t="inlineStr"/>
-      <c r="C13" s="219" t="inlineStr"/>
-      <c r="D13" s="219" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="E13" s="219" t="inlineStr"/>
-      <c r="F13" s="112" t="inlineStr">
-        <is>
-          <t>10/26 Midterm 2: 250 Points Chapters 6, 7, 9, &amp; 16</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="106" t="inlineStr">
-        <is>
-          <t>Final Exam</t>
-        </is>
-      </c>
-      <c r="B14" s="217" t="inlineStr">
-        <is>
-          <t>250 pts</t>
-        </is>
-      </c>
-      <c r="C14" s="218" t="inlineStr"/>
-      <c r="D14" s="218" t="inlineStr">
-        <is>
-          <t>2026-12-16</t>
-        </is>
-      </c>
-      <c r="E14" s="218" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F14" s="109">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-final-exam.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="110" t="inlineStr">
-        <is>
-          <t>Exam</t>
-        </is>
-      </c>
-      <c r="B15" s="219" t="inlineStr"/>
-      <c r="C15" s="219" t="inlineStr"/>
-      <c r="D15" s="219" t="inlineStr">
-        <is>
-          <t>2026-12-16</t>
-        </is>
-      </c>
-      <c r="E15" s="219" t="inlineStr"/>
-      <c r="F15" s="112" t="inlineStr">
-        <is>
-          <t>Final Exam</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="113" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B16" s="217" t="inlineStr">
-        <is>
-          <t>170 pts</t>
-        </is>
-      </c>
-      <c r="C16" s="220" t="inlineStr"/>
-      <c r="D16" s="220" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E16" s="220" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F16" s="115">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-homework.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B17" s="219" t="inlineStr"/>
-      <c r="C17" s="219" t="inlineStr"/>
-      <c r="D17" s="219" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="E17" s="219" t="inlineStr"/>
-      <c r="F17" s="112" t="inlineStr">
-        <is>
-          <t>Class 5 (9/9) - Product Cost Accumulation: Job; Order Co: Chapter 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="117" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B18" s="219" t="inlineStr"/>
-      <c r="C18" s="219" t="inlineStr"/>
-      <c r="D18" s="219" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="E18" s="219" t="inlineStr"/>
-      <c r="F18" s="112" t="inlineStr">
-        <is>
-          <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B19" s="219" t="inlineStr"/>
-      <c r="C19" s="219" t="inlineStr"/>
-      <c r="D19" s="219" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="E19" s="219" t="inlineStr"/>
-      <c r="F19" s="112" t="inlineStr">
-        <is>
-          <t>Class 7 (9/16) - Activity Based Costing: Chapter 5- ONLY; LO 5.1, 2, 4 &amp; 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="117" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B20" s="219" t="inlineStr"/>
-      <c r="C20" s="219" t="inlineStr"/>
-      <c r="D20" s="219" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="E20" s="219" t="inlineStr"/>
-      <c r="F20" s="112" t="inlineStr">
-        <is>
-          <t>Class 7 (9/16) - 3-24, 3-28, 3-32; 15 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B21" s="219" t="inlineStr"/>
-      <c r="C21" s="219" t="inlineStr"/>
-      <c r="D21" s="219" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="E21" s="219" t="inlineStr"/>
-      <c r="F21" s="112" t="inlineStr">
-        <is>
-          <t>Class 8 (9/21) - Product Cost Accumulation: Pro-; cess Co: Chapter 4- ONLY; LO 4.1, 3, 4, &amp; 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="117" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B22" s="219" t="inlineStr"/>
-      <c r="C22" s="219" t="inlineStr"/>
-      <c r="D22" s="219" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="E22" s="219" t="inlineStr"/>
-      <c r="F22" s="112" t="inlineStr">
-        <is>
-          <t>Class 8 (9/21) - 5-27 5-46; 10 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B23" s="219" t="inlineStr"/>
-      <c r="C23" s="219" t="inlineStr"/>
-      <c r="D23" s="219" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="E23" s="219" t="inlineStr"/>
-      <c r="F23" s="112" t="inlineStr">
-        <is>
-          <t>Class 9 (9/23) - Cost of Quality &amp; ESG &amp;; Overview of; • : Chapter 8 - ONLY; LO 8.7, 8, 9</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="117" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B24" s="219" t="inlineStr"/>
-      <c r="C24" s="219" t="inlineStr"/>
-      <c r="D24" s="219" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="E24" s="219" t="inlineStr"/>
-      <c r="F24" s="112" t="inlineStr">
-        <is>
-          <t>Class 9 (9/23) - 4-21, 4-22; 10 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B25" s="219" t="inlineStr"/>
-      <c r="C25" s="219" t="inlineStr"/>
-      <c r="D25" s="219" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E25" s="219" t="inlineStr"/>
-      <c r="F25" s="112" t="inlineStr">
-        <is>
-          <t>Class 10 (9/28) - Catchup &amp; Midterm Review</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="117" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B26" s="219" t="inlineStr"/>
-      <c r="C26" s="219" t="inlineStr"/>
-      <c r="D26" s="219" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E26" s="219" t="inlineStr"/>
-      <c r="F26" s="112" t="inlineStr">
-        <is>
-          <t>Class 10 (9/28) - 8-28, 8-29; 10 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B27" s="219" t="inlineStr"/>
-      <c r="C27" s="219" t="inlineStr"/>
-      <c r="D27" s="219" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="E27" s="219" t="inlineStr"/>
-      <c r="F27" s="112" t="inlineStr">
-        <is>
-          <t>Class 12 (10/7) - Cost volume profit analysis: Chapter 7</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="117" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B28" s="219" t="inlineStr"/>
-      <c r="C28" s="219" t="inlineStr"/>
-      <c r="D28" s="219" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="E28" s="219" t="inlineStr"/>
-      <c r="F28" s="112" t="inlineStr">
-        <is>
-          <t>Class 12 (10/7) - 6-24, 6-25, 6-34; 15 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B29" s="219" t="inlineStr"/>
-      <c r="C29" s="219" t="inlineStr"/>
-      <c r="D29" s="219" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E29" s="219" t="inlineStr"/>
-      <c r="F29" s="112" t="inlineStr">
-        <is>
-          <t>Class 14 (10/14) - Financial planning and analysis:; Static: Chapter 9</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="117" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B30" s="219" t="inlineStr"/>
-      <c r="C30" s="219" t="inlineStr"/>
-      <c r="D30" s="219" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E30" s="219" t="inlineStr"/>
-      <c r="F30" s="112" t="inlineStr">
-        <is>
-          <t>Class 14 (10/14) - 7-29, 7-33, 7-40; 15 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B31" s="219" t="inlineStr"/>
-      <c r="C31" s="219" t="inlineStr"/>
-      <c r="D31" s="219" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E31" s="219" t="inlineStr"/>
-      <c r="F31" s="112" t="inlineStr">
-        <is>
-          <t>Class 15 (10/19) - Capital Budgeting; Practice Midterm Ques: Chapter 16- ONLY; LO 16.1, 2, 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="117" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B32" s="219" t="inlineStr"/>
-      <c r="C32" s="219" t="inlineStr"/>
-      <c r="D32" s="219" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E32" s="219" t="inlineStr"/>
-      <c r="F32" s="112" t="inlineStr">
-        <is>
-          <t>Class 15 (10/19) - 9-25, 9-28, 9-37; 15 - Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B33" s="219" t="inlineStr"/>
-      <c r="C33" s="219" t="inlineStr"/>
-      <c r="D33" s="219" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="E33" s="219" t="inlineStr"/>
-      <c r="F33" s="112" t="inlineStr">
-        <is>
-          <t>Class 16 (10/21) - Catchup &amp; Midterm Review</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="117" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B34" s="219" t="inlineStr"/>
-      <c r="C34" s="219" t="inlineStr"/>
-      <c r="D34" s="219" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="E34" s="219" t="inlineStr"/>
-      <c r="F34" s="112" t="inlineStr">
-        <is>
-          <t>Class 16 (10/21) - 16-28, 16-40; 10 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B35" s="219" t="inlineStr"/>
-      <c r="C35" s="219" t="inlineStr"/>
-      <c r="D35" s="219" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="E35" s="219" t="inlineStr"/>
-      <c r="F35" s="112" t="inlineStr">
-        <is>
-          <t>Class 19 (11/4) - Sales Variance Analysis; Flexible Budget: Chapter 11 - ONLY; LO 11.1, 11.2 &amp;; Appendix B</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="117" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B36" s="219" t="inlineStr"/>
-      <c r="C36" s="219" t="inlineStr"/>
-      <c r="D36" s="219" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="E36" s="219" t="inlineStr"/>
-      <c r="F36" s="112" t="inlineStr">
-        <is>
-          <t>Class 19 (11/4) - 10-26, 10-30; 10 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B37" s="219" t="inlineStr"/>
-      <c r="C37" s="219" t="inlineStr"/>
-      <c r="D37" s="219" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="E37" s="219" t="inlineStr"/>
-      <c r="F37" s="112" t="inlineStr">
-        <is>
-          <t>Class 20 (11/9) - Investment Centers: Chapter 13- ONLY; LO 13-1, 2, 3, 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="117" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B38" s="219" t="inlineStr"/>
-      <c r="C38" s="219" t="inlineStr"/>
-      <c r="D38" s="219" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="E38" s="219" t="inlineStr"/>
-      <c r="F38" s="112" t="inlineStr">
-        <is>
-          <t>Class 20 (11/9) - 11-31, 11-52; 10 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B39" s="219" t="inlineStr"/>
-      <c r="C39" s="219" t="inlineStr"/>
-      <c r="D39" s="219" t="inlineStr">
-        <is>
-          <t>2026-11-16</t>
-        </is>
-      </c>
-      <c r="E39" s="219" t="inlineStr"/>
-      <c r="F39" s="112" t="inlineStr">
-        <is>
-          <t>Class 21 (11/16) - AI &amp; FP&amp;A</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="117" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B40" s="219" t="inlineStr"/>
-      <c r="C40" s="219" t="inlineStr"/>
-      <c r="D40" s="219" t="inlineStr">
-        <is>
-          <t>2026-11-16</t>
-        </is>
-      </c>
-      <c r="E40" s="219" t="inlineStr"/>
-      <c r="F40" s="112" t="inlineStr">
-        <is>
-          <t>Class 21 (11/16) - 13-29, 13-33; 10 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="116" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B41" s="219" t="inlineStr"/>
-      <c r="C41" s="219" t="inlineStr"/>
-      <c r="D41" s="219" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E41" s="219" t="inlineStr"/>
-      <c r="F41" s="112" t="inlineStr">
-        <is>
-          <t>Class 2 (12/2) - Catchup &amp; Final Review; Practice Final Questions Posted to Brightspace at; 5:00 PM</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="117" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B42" s="219" t="inlineStr"/>
-      <c r="C42" s="219" t="inlineStr"/>
-      <c r="D42" s="219" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E42" s="219" t="inlineStr"/>
-      <c r="F42" s="112" t="inlineStr">
-        <is>
-          <t>Class 2 (12/2) - 14-35, 14-41; 10 Points; Assignments listed Be-; low Due by11:59 PM; Linked In Learning; E</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="106" t="inlineStr">
-        <is>
-          <t>LinkedIn Learning Excel Certification</t>
-        </is>
-      </c>
-      <c r="B43" s="217" t="inlineStr">
-        <is>
-          <t>75 pts</t>
-        </is>
-      </c>
-      <c r="C43" s="218" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="D43" s="218" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E43" s="218" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F43" s="109">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-linkedin-learning-excel-certification.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="118" t="inlineStr">
-        <is>
-          <t>Certification</t>
-        </is>
-      </c>
-      <c r="B44" s="219" t="inlineStr"/>
-      <c r="C44" s="219" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="D44" s="219" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E44" s="219" t="inlineStr"/>
-      <c r="F44" s="112" t="inlineStr">
-        <is>
-          <t>LinkedIn Learning Excel Certification</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="113" t="inlineStr">
-        <is>
-          <t>Stukent Simternship</t>
-        </is>
-      </c>
-      <c r="B45" s="217" t="inlineStr">
-        <is>
-          <t>75 pts</t>
-        </is>
-      </c>
-      <c r="C45" s="220" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="D45" s="220" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E45" s="220" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F45" s="115">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-stukent-simternship.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="118" t="inlineStr">
-        <is>
-          <t>Certification</t>
-        </is>
-      </c>
-      <c r="B46" s="219" t="inlineStr"/>
-      <c r="C46" s="219" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="D46" s="219" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E46" s="219" t="inlineStr"/>
-      <c r="F46" s="112" t="inlineStr">
-        <is>
-          <t>Stukent Simternship</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B47" s="119" t="inlineStr">
-        <is>
-          <t>1070 pts</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="B6:F6"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
     <tabColor rgb="001F77B4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -4572,4 +3653,956 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FF7F0E"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>BUAD-281 — Managerial Accounting</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="2">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/sources/buad-281-source.pdf","SEE HERE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Instructor</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Braunegg</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fall 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Required for an A</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Grading scale</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Total graded points in calendar: 1070 (letter scale not in document)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="151" t="inlineStr">
+        <is>
+          <t>Midterm 1 250 pts  |  Midterm 2 250 pts  |  Final Exam 250 pts  |  Homework 170 pts  |  LinkedIn Learning Excel Certification 75 pts  |  Stukent Simternship 75 pts</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="B8" s="225" t="inlineStr">
+        <is>
+          <t>If your AI tool breaks down and solves the homework bank problems - extracting step-by-step mechanics from the textbook - mastering those exact mechanics is all you need to get an A without reading prose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>Group Project</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="106" t="inlineStr">
+        <is>
+          <t>Midterm 1</t>
+        </is>
+      </c>
+      <c r="B11" s="226" t="inlineStr">
+        <is>
+          <t>250 pts</t>
+        </is>
+      </c>
+      <c r="C11" s="227" t="inlineStr"/>
+      <c r="D11" s="227" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E11" s="227" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" s="109">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-midterm-1.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="110" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="B12" s="228" t="inlineStr"/>
+      <c r="C12" s="228" t="inlineStr"/>
+      <c r="D12" s="228" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E12" s="228" t="inlineStr"/>
+      <c r="F12" s="112" t="inlineStr">
+        <is>
+          <t>9/30 Midterm 1: 250 Points Chapters 1, 2, 3, 4, 5, 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="113" t="inlineStr">
+        <is>
+          <t>Midterm 2</t>
+        </is>
+      </c>
+      <c r="B13" s="226" t="inlineStr">
+        <is>
+          <t>250 pts</t>
+        </is>
+      </c>
+      <c r="C13" s="229" t="inlineStr"/>
+      <c r="D13" s="229" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="E13" s="229" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" s="115">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-midterm-2.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="110" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="B14" s="228" t="inlineStr"/>
+      <c r="C14" s="228" t="inlineStr"/>
+      <c r="D14" s="228" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="E14" s="228" t="inlineStr"/>
+      <c r="F14" s="112" t="inlineStr">
+        <is>
+          <t>10/26 Midterm 2: 250 Points Chapters 6, 7, 9, &amp; 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="106" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+      <c r="B15" s="226" t="inlineStr">
+        <is>
+          <t>250 pts</t>
+        </is>
+      </c>
+      <c r="C15" s="227" t="inlineStr"/>
+      <c r="D15" s="227" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="E15" s="227" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F15" s="109">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-final-exam.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="110" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="B16" s="228" t="inlineStr"/>
+      <c r="C16" s="228" t="inlineStr"/>
+      <c r="D16" s="228" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="E16" s="228" t="inlineStr"/>
+      <c r="F16" s="112" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="113" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B17" s="226" t="inlineStr">
+        <is>
+          <t>170 pts</t>
+        </is>
+      </c>
+      <c r="C17" s="229" t="inlineStr"/>
+      <c r="D17" s="229" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E17" s="229" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F17" s="115">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-homework.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="116" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B18" s="228" t="inlineStr"/>
+      <c r="C18" s="228" t="inlineStr"/>
+      <c r="D18" s="228" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="E18" s="228" t="inlineStr"/>
+      <c r="F18" s="112" t="inlineStr">
+        <is>
+          <t>Class 5 (9/9) - Product Cost Accumulation: Job; Order Co: Chapter 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="117" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B19" s="228" t="inlineStr"/>
+      <c r="C19" s="228" t="inlineStr"/>
+      <c r="D19" s="228" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="E19" s="228" t="inlineStr"/>
+      <c r="F19" s="112" t="inlineStr">
+        <is>
+          <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="116" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B20" s="228" t="inlineStr"/>
+      <c r="C20" s="228" t="inlineStr"/>
+      <c r="D20" s="228" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E20" s="228" t="inlineStr"/>
+      <c r="F20" s="112" t="inlineStr">
+        <is>
+          <t>Class 7 (9/16) - Activity Based Costing: Chapter 5- ONLY; LO 5.1, 2, 4 &amp; 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="117" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B21" s="228" t="inlineStr"/>
+      <c r="C21" s="228" t="inlineStr"/>
+      <c r="D21" s="228" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E21" s="228" t="inlineStr"/>
+      <c r="F21" s="112" t="inlineStr">
+        <is>
+          <t>Class 7 (9/16) - 3-24, 3-28, 3-32; 15 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="116" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B22" s="228" t="inlineStr"/>
+      <c r="C22" s="228" t="inlineStr"/>
+      <c r="D22" s="228" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E22" s="228" t="inlineStr"/>
+      <c r="F22" s="112" t="inlineStr">
+        <is>
+          <t>Class 8 (9/21) - Product Cost Accumulation: Pro-; cess Co: Chapter 4- ONLY; LO 4.1, 3, 4, &amp; 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="117" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B23" s="228" t="inlineStr"/>
+      <c r="C23" s="228" t="inlineStr"/>
+      <c r="D23" s="228" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E23" s="228" t="inlineStr"/>
+      <c r="F23" s="112" t="inlineStr">
+        <is>
+          <t>Class 8 (9/21) - 5-27 5-46; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="116" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B24" s="228" t="inlineStr"/>
+      <c r="C24" s="228" t="inlineStr"/>
+      <c r="D24" s="228" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E24" s="228" t="inlineStr"/>
+      <c r="F24" s="112" t="inlineStr">
+        <is>
+          <t>Class 9 (9/23) - Cost of Quality &amp; ESG &amp;; Overview of; • : Chapter 8 - ONLY; LO 8.7, 8, 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="117" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B25" s="228" t="inlineStr"/>
+      <c r="C25" s="228" t="inlineStr"/>
+      <c r="D25" s="228" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E25" s="228" t="inlineStr"/>
+      <c r="F25" s="112" t="inlineStr">
+        <is>
+          <t>Class 9 (9/23) - 4-21, 4-22; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="116" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B26" s="228" t="inlineStr"/>
+      <c r="C26" s="228" t="inlineStr"/>
+      <c r="D26" s="228" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E26" s="228" t="inlineStr"/>
+      <c r="F26" s="112" t="inlineStr">
+        <is>
+          <t>Class 10 (9/28) - Catchup &amp; Midterm Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="117" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B27" s="228" t="inlineStr"/>
+      <c r="C27" s="228" t="inlineStr"/>
+      <c r="D27" s="228" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E27" s="228" t="inlineStr"/>
+      <c r="F27" s="112" t="inlineStr">
+        <is>
+          <t>Class 10 (9/28) - 8-28, 8-29; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="116" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B28" s="228" t="inlineStr"/>
+      <c r="C28" s="228" t="inlineStr"/>
+      <c r="D28" s="228" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E28" s="228" t="inlineStr"/>
+      <c r="F28" s="112" t="inlineStr">
+        <is>
+          <t>Class 12 (10/7) - Cost volume profit analysis: Chapter 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="117" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B29" s="228" t="inlineStr"/>
+      <c r="C29" s="228" t="inlineStr"/>
+      <c r="D29" s="228" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E29" s="228" t="inlineStr"/>
+      <c r="F29" s="112" t="inlineStr">
+        <is>
+          <t>Class 12 (10/7) - 6-24, 6-25, 6-34; 15 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="116" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B30" s="228" t="inlineStr"/>
+      <c r="C30" s="228" t="inlineStr"/>
+      <c r="D30" s="228" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E30" s="228" t="inlineStr"/>
+      <c r="F30" s="112" t="inlineStr">
+        <is>
+          <t>Class 14 (10/14) - Financial planning and analysis:; Static: Chapter 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="117" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B31" s="228" t="inlineStr"/>
+      <c r="C31" s="228" t="inlineStr"/>
+      <c r="D31" s="228" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E31" s="228" t="inlineStr"/>
+      <c r="F31" s="112" t="inlineStr">
+        <is>
+          <t>Class 14 (10/14) - 7-29, 7-33, 7-40; 15 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="116" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B32" s="228" t="inlineStr"/>
+      <c r="C32" s="228" t="inlineStr"/>
+      <c r="D32" s="228" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E32" s="228" t="inlineStr"/>
+      <c r="F32" s="112" t="inlineStr">
+        <is>
+          <t>Class 15 (10/19) - Capital Budgeting; Practice Midterm Ques: Chapter 16- ONLY; LO 16.1, 2, 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="117" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B33" s="228" t="inlineStr"/>
+      <c r="C33" s="228" t="inlineStr"/>
+      <c r="D33" s="228" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E33" s="228" t="inlineStr"/>
+      <c r="F33" s="112" t="inlineStr">
+        <is>
+          <t>Class 15 (10/19) - 9-25, 9-28, 9-37; 15 - Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="116" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B34" s="228" t="inlineStr"/>
+      <c r="C34" s="228" t="inlineStr"/>
+      <c r="D34" s="228" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E34" s="228" t="inlineStr"/>
+      <c r="F34" s="112" t="inlineStr">
+        <is>
+          <t>Class 16 (10/21) - Catchup &amp; Midterm Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="117" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B35" s="228" t="inlineStr"/>
+      <c r="C35" s="228" t="inlineStr"/>
+      <c r="D35" s="228" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E35" s="228" t="inlineStr"/>
+      <c r="F35" s="112" t="inlineStr">
+        <is>
+          <t>Class 16 (10/21) - 16-28, 16-40; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="116" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B36" s="228" t="inlineStr"/>
+      <c r="C36" s="228" t="inlineStr"/>
+      <c r="D36" s="228" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="E36" s="228" t="inlineStr"/>
+      <c r="F36" s="112" t="inlineStr">
+        <is>
+          <t>Class 19 (11/4) - Sales Variance Analysis; Flexible Budget: Chapter 11 - ONLY; LO 11.1, 11.2 &amp;; Appendix B</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="117" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B37" s="228" t="inlineStr"/>
+      <c r="C37" s="228" t="inlineStr"/>
+      <c r="D37" s="228" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="E37" s="228" t="inlineStr"/>
+      <c r="F37" s="112" t="inlineStr">
+        <is>
+          <t>Class 19 (11/4) - 10-26, 10-30; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="116" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B38" s="228" t="inlineStr"/>
+      <c r="C38" s="228" t="inlineStr"/>
+      <c r="D38" s="228" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E38" s="228" t="inlineStr"/>
+      <c r="F38" s="112" t="inlineStr">
+        <is>
+          <t>Class 20 (11/9) - Investment Centers: Chapter 13- ONLY; LO 13-1, 2, 3, 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="117" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B39" s="228" t="inlineStr"/>
+      <c r="C39" s="228" t="inlineStr"/>
+      <c r="D39" s="228" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E39" s="228" t="inlineStr"/>
+      <c r="F39" s="112" t="inlineStr">
+        <is>
+          <t>Class 20 (11/9) - 11-31, 11-52; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="116" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B40" s="228" t="inlineStr"/>
+      <c r="C40" s="228" t="inlineStr"/>
+      <c r="D40" s="228" t="inlineStr">
+        <is>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="E40" s="228" t="inlineStr"/>
+      <c r="F40" s="112" t="inlineStr">
+        <is>
+          <t>Class 21 (11/16) - AI &amp; FP&amp;A</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="117" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B41" s="228" t="inlineStr"/>
+      <c r="C41" s="228" t="inlineStr"/>
+      <c r="D41" s="228" t="inlineStr">
+        <is>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="E41" s="228" t="inlineStr"/>
+      <c r="F41" s="112" t="inlineStr">
+        <is>
+          <t>Class 21 (11/16) - 13-29, 13-33; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="116" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B42" s="228" t="inlineStr"/>
+      <c r="C42" s="228" t="inlineStr"/>
+      <c r="D42" s="228" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E42" s="228" t="inlineStr"/>
+      <c r="F42" s="112" t="inlineStr">
+        <is>
+          <t>Class 2 (12/2) - Catchup &amp; Final Review; Practice Final Questions Posted to Brightspace at; 5:00 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="117" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B43" s="228" t="inlineStr"/>
+      <c r="C43" s="228" t="inlineStr"/>
+      <c r="D43" s="228" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E43" s="228" t="inlineStr"/>
+      <c r="F43" s="112" t="inlineStr">
+        <is>
+          <t>Class 2 (12/2) - 14-35, 14-41; 10 Points; Assignments listed Be-; low Due by11:59 PM; Linked In Learning; E</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="106" t="inlineStr">
+        <is>
+          <t>LinkedIn Learning Excel Certification</t>
+        </is>
+      </c>
+      <c r="B44" s="226" t="inlineStr">
+        <is>
+          <t>75 pts</t>
+        </is>
+      </c>
+      <c r="C44" s="227" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D44" s="227" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E44" s="227" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F44" s="109">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-linkedin-learning-excel-certification.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="118" t="inlineStr">
+        <is>
+          <t>Certification</t>
+        </is>
+      </c>
+      <c r="B45" s="228" t="inlineStr"/>
+      <c r="C45" s="228" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D45" s="228" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E45" s="228" t="inlineStr"/>
+      <c r="F45" s="112" t="inlineStr">
+        <is>
+          <t>LinkedIn Learning Excel Certification</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="113" t="inlineStr">
+        <is>
+          <t>Stukent Simternship</t>
+        </is>
+      </c>
+      <c r="B46" s="226" t="inlineStr">
+        <is>
+          <t>75 pts</t>
+        </is>
+      </c>
+      <c r="C46" s="229" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D46" s="229" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E46" s="229" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F46" s="115">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-stukent-simternship.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="118" t="inlineStr">
+        <is>
+          <t>Certification</t>
+        </is>
+      </c>
+      <c r="B47" s="228" t="inlineStr"/>
+      <c r="C47" s="228" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D47" s="228" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E47" s="228" t="inlineStr"/>
+      <c r="F47" s="112" t="inlineStr">
+        <is>
+          <t>Stukent Simternship</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B48" s="119" t="inlineStr">
+        <is>
+          <t>1070 pts</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="A7:F7"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Overview: assignments-only to-dos, first assignment per class
Exclude Reading from Start here, First assignment column, and Do First
list. Always include each class's earliest assignment even when due after
other classes' month items. Rename First on list to First assignment.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-281" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-304" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-304" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-281" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="26">
+  <fonts count="28">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -142,6 +142,14 @@
     <font>
       <b val="1"/>
       <color rgb="00C65911"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000070C0"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007030A0"/>
     </font>
   </fonts>
   <fills count="27">
@@ -303,7 +311,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="264">
+  <cellXfs count="278">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1065,6 +1073,48 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="25" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -1444,18 +1494,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1475,7 +1526,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="232" t="inlineStr">
         <is>
-          <t>Start here: 2026-08-29 - HIST-103 - Reading: Week Aug 25-29: Intro &amp; Black Death</t>
+          <t>Start here: 2026-08-31 - BUAD-304 - Homework: Connect: Self-Assessment 3.01 - What is my Big thinking about your top</t>
         </is>
       </c>
     </row>
@@ -1507,20 +1558,25 @@
       </c>
       <c r="F5" s="233" t="inlineStr">
         <is>
-          <t>First on list</t>
+          <t>External certs</t>
         </is>
       </c>
       <c r="G5" s="233" t="inlineStr">
         <is>
-          <t>List due</t>
+          <t>First assignment</t>
         </is>
       </c>
       <c r="H5" s="233" t="inlineStr">
         <is>
+          <t>Assign due</t>
+        </is>
+      </c>
+      <c r="I5" s="233" t="inlineStr">
+        <is>
           <t>First major</t>
         </is>
       </c>
-      <c r="I5" s="233" t="inlineStr">
+      <c r="J5" s="233" t="inlineStr">
         <is>
           <t>Major due</t>
         </is>
@@ -1551,22 +1607,27 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F6" s="235" t="inlineStr">
-        <is>
-          <t>Class 5 (9/9) - Product Cost Accumulation: Job; Order C</t>
+      <c r="F6" s="264" t="inlineStr">
+        <is>
+          <t>LinkedIn Learning Excel Certification, Stukent Simternship</t>
         </is>
       </c>
       <c r="G6" s="235" t="inlineStr">
         <is>
+          <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
+        </is>
+      </c>
+      <c r="H6" s="235" t="inlineStr">
+        <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="H6" s="235" t="inlineStr">
+      <c r="I6" s="235" t="inlineStr">
         <is>
           <t>Midterm 1</t>
         </is>
       </c>
-      <c r="I6" s="235" t="inlineStr">
+      <c r="J6" s="235" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
@@ -1599,20 +1660,25 @@
       </c>
       <c r="F7" s="237" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="237" t="inlineStr">
+        <is>
           <t>Connect: Self-Assessment 3.01 - What is my Big thinking</t>
         </is>
       </c>
-      <c r="G7" s="237" t="inlineStr">
+      <c r="H7" s="237" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="H7" s="237" t="inlineStr">
+      <c r="I7" s="237" t="inlineStr">
         <is>
           <t>Thomas Green Case Analysis Memo</t>
         </is>
       </c>
-      <c r="I7" s="237" t="inlineStr">
+      <c r="J7" s="237" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
@@ -1645,20 +1711,25 @@
       </c>
       <c r="F8" s="235" t="inlineStr">
         <is>
-          <t>Week Aug 25-29: Intro &amp; Black Death</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G8" s="235" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>Sleep Paper Due</t>
         </is>
       </c>
       <c r="H8" s="235" t="inlineStr">
         <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="I8" s="235" t="inlineStr">
+        <is>
           <t>Sleep Paper</t>
         </is>
       </c>
-      <c r="I8" s="235" t="inlineStr">
+      <c r="J8" s="235" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
@@ -1667,7 +1738,7 @@
     <row r="10">
       <c r="A10" s="238" t="inlineStr">
         <is>
-          <t>Do First - August 2026</t>
+          <t>Do First - August 2026 (assignments only; first per class included)</t>
         </is>
       </c>
     </row>
@@ -1696,125 +1767,1190 @@
     <row r="12">
       <c r="A12" s="235" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B12" s="235" t="inlineStr">
         <is>
-          <t>HIST-103</t>
-        </is>
-      </c>
-      <c r="C12" s="240" t="inlineStr">
-        <is>
-          <t>Reading</t>
+          <t>BUAD-304</t>
+        </is>
+      </c>
+      <c r="C12" s="243" t="inlineStr">
+        <is>
+          <t>Homework</t>
         </is>
       </c>
       <c r="D12" s="235" t="inlineStr">
         <is>
-          <t>Week Aug 25-29: Intro &amp; Black Death</t>
+          <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="237" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B13" s="237" t="inlineStr">
         <is>
-          <t>HIST-103</t>
-        </is>
-      </c>
-      <c r="C13" s="241" t="inlineStr">
-        <is>
-          <t>Reading</t>
+          <t>BUAD-304</t>
+        </is>
+      </c>
+      <c r="C13" s="242" t="inlineStr">
+        <is>
+          <t>Homework</t>
         </is>
       </c>
       <c r="D13" s="237" t="inlineStr">
         <is>
-          <t>Week Aug 25-29: Intro &amp; Black Death (lecture topics)</t>
+          <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="235" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B14" s="235" t="inlineStr">
         <is>
-          <t>HIST-103</t>
-        </is>
-      </c>
-      <c r="C14" s="240" t="inlineStr">
-        <is>
-          <t>Reading</t>
+          <t>BUAD-281</t>
+        </is>
+      </c>
+      <c r="C14" s="243" t="inlineStr">
+        <is>
+          <t>Homework</t>
         </is>
       </c>
       <c r="D14" s="235" t="inlineStr">
         <is>
-          <t>Week Aug 25-29: Intro &amp; Black Death - Section reading 1: -- 13 of 33 -- Lizzie W</t>
+          <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="237" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B15" s="237" t="inlineStr">
         <is>
-          <t>BUAD-304</t>
-        </is>
-      </c>
-      <c r="C15" s="242" t="inlineStr">
-        <is>
-          <t>Homework</t>
+          <t>HIST-103</t>
+        </is>
+      </c>
+      <c r="C15" s="273" t="inlineStr">
+        <is>
+          <t>Assignment</t>
         </is>
       </c>
       <c r="D15" s="237" t="inlineStr">
         <is>
-          <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="235" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="B16" s="235" t="inlineStr">
-        <is>
-          <t>BUAD-304</t>
-        </is>
-      </c>
-      <c r="C16" s="243" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="D16" s="235" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
+          <t>Sleep Paper Due</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A10:I10"/>
+    <mergeCell ref="A10:J10"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001F77B4"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>BUAD-304 — Organizational Behavior and Leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="2">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/sources/buad-304-source.pdf","SEE HERE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Instructor</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Christine El Haddad</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fall 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Required for an A</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Curved (class rank)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Grading scale</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Weighted score (% of points earned) + class average + student ranking (relative grading - no fixed A threshold in syllabus)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="156" t="inlineStr">
+        <is>
+          <t>Final Exam 25%  |  Participation 15%  |  Midterm Exam 15%  |  Team Project Paper 15%  |  Final Reflection Paper 10%  |  Presentation 10%  |  Case Analysis Assignments 5%  |  Proposal &amp; Team Contract 3%  |  Self &amp; Peer Evaluation 2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="E9" s="21" t="inlineStr">
+        <is>
+          <t>Group Project</t>
+        </is>
+      </c>
+      <c r="F9" s="21" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="120" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+      <c r="B10" s="256" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="C10" s="257" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D10" s="257" t="inlineStr">
+        <is>
+          <t>2026-12-09</t>
+        </is>
+      </c>
+      <c r="E10" s="257" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" s="123">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-final-exam.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="124" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="B11" s="258" t="inlineStr"/>
+      <c r="C11" s="258" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D11" s="258" t="inlineStr">
+        <is>
+          <t>2026-12-09</t>
+        </is>
+      </c>
+      <c r="E11" s="258" t="inlineStr"/>
+      <c r="F11" s="126" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="127" t="inlineStr">
+        <is>
+          <t>Participation</t>
+        </is>
+      </c>
+      <c r="B12" s="256" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="C12" s="259" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D12" s="259" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E12" s="259" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F12" s="129">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-participation.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="131" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B13" s="258" t="inlineStr"/>
+      <c r="C13" s="258" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D13" s="258" t="inlineStr"/>
+      <c r="E13" s="258" t="inlineStr"/>
+      <c r="F13" s="126" t="inlineStr">
+        <is>
+          <t>Research: SONA registration opens</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="131" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B14" s="258" t="inlineStr"/>
+      <c r="C14" s="258" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="D14" s="258" t="inlineStr"/>
+      <c r="E14" s="258" t="inlineStr"/>
+      <c r="F14" s="126" t="inlineStr">
+        <is>
+          <t>Research: Prescreening questionnaire opens</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="131" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B15" s="258" t="inlineStr"/>
+      <c r="C15" s="258" t="inlineStr"/>
+      <c r="D15" s="258" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E15" s="258" t="inlineStr"/>
+      <c r="F15" s="126" t="inlineStr">
+        <is>
+          <t>Research: Setup deadline (registration, prescreening, contacts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="131" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B16" s="258" t="inlineStr"/>
+      <c r="C16" s="258" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="D16" s="258" t="inlineStr"/>
+      <c r="E16" s="258" t="inlineStr"/>
+      <c r="F16" s="126" t="inlineStr">
+        <is>
+          <t>Research: Study invitations begin (after setup)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="131" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B17" s="258" t="inlineStr"/>
+      <c r="C17" s="258" t="inlineStr"/>
+      <c r="D17" s="258" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="E17" s="258" t="inlineStr"/>
+      <c r="F17" s="126" t="inlineStr">
+        <is>
+          <t>Research: Employee contact surveys sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="131" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B18" s="258" t="inlineStr"/>
+      <c r="C18" s="258" t="inlineStr"/>
+      <c r="D18" s="258" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E18" s="258" t="inlineStr"/>
+      <c r="F18" s="126" t="inlineStr">
+        <is>
+          <t>Research: Complete 2.0 research credits</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="120" t="inlineStr">
+        <is>
+          <t>Midterm Exam</t>
+        </is>
+      </c>
+      <c r="B19" s="256" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="C19" s="257" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D19" s="257" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E19" s="257" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F19" s="123">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-midterm-exam.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="124" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="B20" s="258" t="inlineStr"/>
+      <c r="C20" s="258" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D20" s="258" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E20" s="258" t="inlineStr"/>
+      <c r="F20" s="126" t="inlineStr">
+        <is>
+          <t>Midterm Exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="127" t="inlineStr">
+        <is>
+          <t>Team Project Paper</t>
+        </is>
+      </c>
+      <c r="B21" s="256" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="C21" s="259" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D21" s="259" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E21" s="259" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F21" s="129">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-team-project-paper.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="132" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B22" s="258" t="inlineStr"/>
+      <c r="C22" s="258" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D22" s="258" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E22" s="258" t="inlineStr"/>
+      <c r="F22" s="126" t="inlineStr">
+        <is>
+          <t>Team project outline</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="132" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B23" s="258" t="inlineStr"/>
+      <c r="C23" s="258" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D23" s="258" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E23" s="258" t="inlineStr"/>
+      <c r="F23" s="126" t="inlineStr">
+        <is>
+          <t>Team project paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="120" t="inlineStr">
+        <is>
+          <t>Final Reflection Paper</t>
+        </is>
+      </c>
+      <c r="B24" s="256" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C24" s="257" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D24" s="257" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E24" s="257" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F24" s="123">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-final-reflection-paper.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="132" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B25" s="258" t="inlineStr"/>
+      <c r="C25" s="258" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D25" s="258" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E25" s="258" t="inlineStr"/>
+      <c r="F25" s="126" t="inlineStr">
+        <is>
+          <t>Personal Reflection Paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="127" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="B26" s="256" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C26" s="259" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D26" s="259" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E26" s="259" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F26" s="129">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-presentation.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="132" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B27" s="258" t="inlineStr"/>
+      <c r="C27" s="258" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D27" s="258" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E27" s="258" t="inlineStr"/>
+      <c r="F27" s="126" t="inlineStr">
+        <is>
+          <t>Presentation slides</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="120" t="inlineStr">
+        <is>
+          <t>Case Analysis Assignments</t>
+        </is>
+      </c>
+      <c r="B28" s="256" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="C28" s="257" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D28" s="257" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E28" s="257" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F28" s="123">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-case-analysis-assignments.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="132" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B29" s="258" t="inlineStr"/>
+      <c r="C29" s="258" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D29" s="258" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E29" s="258" t="inlineStr"/>
+      <c r="F29" s="126" t="inlineStr">
+        <is>
+          <t>Thomas Green Case Analysis Memo</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="132" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B30" s="258" t="inlineStr"/>
+      <c r="C30" s="258" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D30" s="258" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E30" s="258" t="inlineStr"/>
+      <c r="F30" s="126" t="inlineStr">
+        <is>
+          <t>SkillsForTomorrow Analysis Memo</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="127" t="inlineStr">
+        <is>
+          <t>Proposal &amp; Team Contract</t>
+        </is>
+      </c>
+      <c r="B31" s="256" t="inlineStr">
+        <is>
+          <t>3%</t>
+        </is>
+      </c>
+      <c r="C31" s="259" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D31" s="259" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E31" s="259" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F31" s="129">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-proposal-team-contract.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="132" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B32" s="258" t="inlineStr"/>
+      <c r="C32" s="258" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D32" s="258" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E32" s="258" t="inlineStr"/>
+      <c r="F32" s="126" t="inlineStr">
+        <is>
+          <t>Team project proposal &amp; team contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="120" t="inlineStr">
+        <is>
+          <t>Self &amp; Peer Evaluation</t>
+        </is>
+      </c>
+      <c r="B33" s="256" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="C33" s="257" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D33" s="257" t="inlineStr">
+        <is>
+          <t>2026-11-18</t>
+        </is>
+      </c>
+      <c r="E33" s="257" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F33" s="123">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-self-peer-evaluation.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="132" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B34" s="258" t="inlineStr"/>
+      <c r="C34" s="258" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D34" s="258" t="inlineStr">
+        <is>
+          <t>2026-11-18</t>
+        </is>
+      </c>
+      <c r="E34" s="258" t="inlineStr"/>
+      <c r="F34" s="126" t="inlineStr">
+        <is>
+          <t>Self &amp; peer evaluation</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="127" t="inlineStr">
+        <is>
+          <t>Personal Assessments (Connect)</t>
+        </is>
+      </c>
+      <c r="B35" s="256" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C35" s="259" t="inlineStr"/>
+      <c r="D35" s="259" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E35" s="259" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F35" s="129">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-personal-assessments-connect.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="130" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B36" s="258" t="inlineStr"/>
+      <c r="C36" s="258" t="inlineStr"/>
+      <c r="D36" s="258" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E36" s="258" t="inlineStr"/>
+      <c r="F36" s="126" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="130" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B37" s="258" t="inlineStr"/>
+      <c r="C37" s="258" t="inlineStr"/>
+      <c r="D37" s="258" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E37" s="258" t="inlineStr"/>
+      <c r="F37" s="126" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="130" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B38" s="258" t="inlineStr"/>
+      <c r="C38" s="258" t="inlineStr"/>
+      <c r="D38" s="258" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E38" s="258" t="inlineStr"/>
+      <c r="F38" s="126" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 5.01 - Assessing Your</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="130" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B39" s="258" t="inlineStr"/>
+      <c r="C39" s="258" t="inlineStr"/>
+      <c r="D39" s="258" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="E39" s="258" t="inlineStr"/>
+      <c r="F39" s="126" t="inlineStr">
+        <is>
+          <t>Connect: Sharpen Companion</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="130" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B40" s="258" t="inlineStr"/>
+      <c r="C40" s="258" t="inlineStr"/>
+      <c r="D40" s="258" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="E40" s="258" t="inlineStr"/>
+      <c r="F40" s="126" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 11.01 - What is my</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="130" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B41" s="258" t="inlineStr"/>
+      <c r="C41" s="258" t="inlineStr"/>
+      <c r="D41" s="258" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="E41" s="258" t="inlineStr"/>
+      <c r="F41" s="126" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 11.02 - What is my</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="130" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B42" s="258" t="inlineStr"/>
+      <c r="C42" s="258" t="inlineStr"/>
+      <c r="D42" s="258" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E42" s="258" t="inlineStr"/>
+      <c r="F42" s="126" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 12.01 - What kind of</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="130" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B43" s="258" t="inlineStr"/>
+      <c r="C43" s="258" t="inlineStr"/>
+      <c r="D43" s="258" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E43" s="258" t="inlineStr"/>
+      <c r="F43" s="126" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 10.5 - Preferred Conflict</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="130" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B44" s="258" t="inlineStr"/>
+      <c r="C44" s="258" t="inlineStr"/>
+      <c r="D44" s="258" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E44" s="258" t="inlineStr"/>
+      <c r="F44" s="126" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 9.01 - Assessing My</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="130" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B45" s="258" t="inlineStr"/>
+      <c r="C45" s="258" t="inlineStr"/>
+      <c r="D45" s="258" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E45" s="258" t="inlineStr"/>
+      <c r="F45" s="126" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 8.01 - Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="130" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B46" s="258" t="inlineStr"/>
+      <c r="C46" s="258" t="inlineStr"/>
+      <c r="D46" s="258" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="E46" s="258" t="inlineStr"/>
+      <c r="F46" s="126" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 14.02 - What Type of Organizational Culture Do I</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="130" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B47" s="258" t="inlineStr"/>
+      <c r="C47" s="258" t="inlineStr"/>
+      <c r="D47" s="258" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="E47" s="258" t="inlineStr"/>
+      <c r="F47" s="126" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 16.02 - What Is Your</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="130" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B48" s="258" t="inlineStr"/>
+      <c r="C48" s="258" t="inlineStr"/>
+      <c r="D48" s="258" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="E48" s="258" t="inlineStr"/>
+      <c r="F48" s="126" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 16.03 - Assessing Your</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="130" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B49" s="258" t="inlineStr"/>
+      <c r="C49" s="258" t="inlineStr"/>
+      <c r="D49" s="258" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E49" s="258" t="inlineStr"/>
+      <c r="F49" s="126" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 12.02 - Which influence</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B50" s="133" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="B6:F6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00FF7F0E"/>
@@ -1950,18 +3086,18 @@
           <t>Midterm 1</t>
         </is>
       </c>
-      <c r="B11" s="248" t="inlineStr">
+      <c r="B11" s="269" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C11" s="249" t="inlineStr"/>
-      <c r="D11" s="249" t="inlineStr">
+      <c r="C11" s="270" t="inlineStr"/>
+      <c r="D11" s="270" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="E11" s="249" t="inlineStr">
+      <c r="E11" s="270" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1977,14 +3113,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B12" s="250" t="inlineStr"/>
-      <c r="C12" s="250" t="inlineStr"/>
-      <c r="D12" s="250" t="inlineStr">
+      <c r="B12" s="271" t="inlineStr"/>
+      <c r="C12" s="271" t="inlineStr"/>
+      <c r="D12" s="271" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="E12" s="250" t="inlineStr"/>
+      <c r="E12" s="271" t="inlineStr"/>
       <c r="F12" s="112" t="inlineStr">
         <is>
           <t>9/30 Midterm 1: 250 Points Chapters 1, 2, 3, 4, 5, 8</t>
@@ -1997,18 +3133,18 @@
           <t>Midterm 2</t>
         </is>
       </c>
-      <c r="B13" s="248" t="inlineStr">
+      <c r="B13" s="269" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C13" s="251" t="inlineStr"/>
-      <c r="D13" s="251" t="inlineStr">
+      <c r="C13" s="272" t="inlineStr"/>
+      <c r="D13" s="272" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E13" s="251" t="inlineStr">
+      <c r="E13" s="272" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2024,14 +3160,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B14" s="250" t="inlineStr"/>
-      <c r="C14" s="250" t="inlineStr"/>
-      <c r="D14" s="250" t="inlineStr">
+      <c r="B14" s="271" t="inlineStr"/>
+      <c r="C14" s="271" t="inlineStr"/>
+      <c r="D14" s="271" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E14" s="250" t="inlineStr"/>
+      <c r="E14" s="271" t="inlineStr"/>
       <c r="F14" s="112" t="inlineStr">
         <is>
           <t>10/26 Midterm 2: 250 Points Chapters 6, 7, 9, &amp; 16</t>
@@ -2044,18 +3180,18 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B15" s="248" t="inlineStr">
+      <c r="B15" s="269" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C15" s="249" t="inlineStr"/>
-      <c r="D15" s="249" t="inlineStr">
+      <c r="C15" s="270" t="inlineStr"/>
+      <c r="D15" s="270" t="inlineStr">
         <is>
           <t>2026-12-16</t>
         </is>
       </c>
-      <c r="E15" s="249" t="inlineStr">
+      <c r="E15" s="270" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2071,14 +3207,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B16" s="250" t="inlineStr"/>
-      <c r="C16" s="250" t="inlineStr"/>
-      <c r="D16" s="250" t="inlineStr">
+      <c r="B16" s="271" t="inlineStr"/>
+      <c r="C16" s="271" t="inlineStr"/>
+      <c r="D16" s="271" t="inlineStr">
         <is>
           <t>2026-12-16</t>
         </is>
       </c>
-      <c r="E16" s="250" t="inlineStr"/>
+      <c r="E16" s="271" t="inlineStr"/>
       <c r="F16" s="112" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -2091,18 +3227,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B17" s="248" t="inlineStr">
+      <c r="B17" s="269" t="inlineStr">
         <is>
           <t>170 pts</t>
         </is>
       </c>
-      <c r="C17" s="251" t="inlineStr"/>
-      <c r="D17" s="251" t="inlineStr">
+      <c r="C17" s="272" t="inlineStr"/>
+      <c r="D17" s="272" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E17" s="251" t="inlineStr">
+      <c r="E17" s="272" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2118,14 +3254,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B18" s="250" t="inlineStr"/>
-      <c r="C18" s="250" t="inlineStr"/>
-      <c r="D18" s="250" t="inlineStr">
+      <c r="B18" s="271" t="inlineStr"/>
+      <c r="C18" s="271" t="inlineStr"/>
+      <c r="D18" s="271" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="E18" s="250" t="inlineStr"/>
+      <c r="E18" s="271" t="inlineStr"/>
       <c r="F18" s="112" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - Product Cost Accumulation: Job; Order Co: Chapter 3</t>
@@ -2138,14 +3274,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B19" s="250" t="inlineStr"/>
-      <c r="C19" s="250" t="inlineStr"/>
-      <c r="D19" s="250" t="inlineStr">
+      <c r="B19" s="271" t="inlineStr"/>
+      <c r="C19" s="271" t="inlineStr"/>
+      <c r="D19" s="271" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="E19" s="250" t="inlineStr"/>
+      <c r="E19" s="271" t="inlineStr"/>
       <c r="F19" s="112" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
@@ -2158,14 +3294,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B20" s="250" t="inlineStr"/>
-      <c r="C20" s="250" t="inlineStr"/>
-      <c r="D20" s="250" t="inlineStr">
+      <c r="B20" s="271" t="inlineStr"/>
+      <c r="C20" s="271" t="inlineStr"/>
+      <c r="D20" s="271" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E20" s="250" t="inlineStr"/>
+      <c r="E20" s="271" t="inlineStr"/>
       <c r="F20" s="112" t="inlineStr">
         <is>
           <t>Class 7 (9/16) - Activity Based Costing: Chapter 5- ONLY; LO 5.1, 2, 4 &amp; 5</t>
@@ -2178,14 +3314,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B21" s="250" t="inlineStr"/>
-      <c r="C21" s="250" t="inlineStr"/>
-      <c r="D21" s="250" t="inlineStr">
+      <c r="B21" s="271" t="inlineStr"/>
+      <c r="C21" s="271" t="inlineStr"/>
+      <c r="D21" s="271" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E21" s="250" t="inlineStr"/>
+      <c r="E21" s="271" t="inlineStr"/>
       <c r="F21" s="112" t="inlineStr">
         <is>
           <t>Class 7 (9/16) - 3-24, 3-28, 3-32; 15 Points</t>
@@ -2198,14 +3334,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B22" s="250" t="inlineStr"/>
-      <c r="C22" s="250" t="inlineStr"/>
-      <c r="D22" s="250" t="inlineStr">
+      <c r="B22" s="271" t="inlineStr"/>
+      <c r="C22" s="271" t="inlineStr"/>
+      <c r="D22" s="271" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="E22" s="250" t="inlineStr"/>
+      <c r="E22" s="271" t="inlineStr"/>
       <c r="F22" s="112" t="inlineStr">
         <is>
           <t>Class 8 (9/21) - Product Cost Accumulation: Pro-; cess Co: Chapter 4- ONLY; LO 4.1, 3, 4, &amp; 5</t>
@@ -2218,14 +3354,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B23" s="250" t="inlineStr"/>
-      <c r="C23" s="250" t="inlineStr"/>
-      <c r="D23" s="250" t="inlineStr">
+      <c r="B23" s="271" t="inlineStr"/>
+      <c r="C23" s="271" t="inlineStr"/>
+      <c r="D23" s="271" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="E23" s="250" t="inlineStr"/>
+      <c r="E23" s="271" t="inlineStr"/>
       <c r="F23" s="112" t="inlineStr">
         <is>
           <t>Class 8 (9/21) - 5-27 5-46; 10 Points</t>
@@ -2238,14 +3374,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B24" s="250" t="inlineStr"/>
-      <c r="C24" s="250" t="inlineStr"/>
-      <c r="D24" s="250" t="inlineStr">
+      <c r="B24" s="271" t="inlineStr"/>
+      <c r="C24" s="271" t="inlineStr"/>
+      <c r="D24" s="271" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="E24" s="250" t="inlineStr"/>
+      <c r="E24" s="271" t="inlineStr"/>
       <c r="F24" s="112" t="inlineStr">
         <is>
           <t>Class 9 (9/23) - Cost of Quality &amp; ESG &amp;; Overview of; • : Chapter 8 - ONLY; LO 8.7, 8, 9</t>
@@ -2258,14 +3394,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B25" s="250" t="inlineStr"/>
-      <c r="C25" s="250" t="inlineStr"/>
-      <c r="D25" s="250" t="inlineStr">
+      <c r="B25" s="271" t="inlineStr"/>
+      <c r="C25" s="271" t="inlineStr"/>
+      <c r="D25" s="271" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="E25" s="250" t="inlineStr"/>
+      <c r="E25" s="271" t="inlineStr"/>
       <c r="F25" s="112" t="inlineStr">
         <is>
           <t>Class 9 (9/23) - 4-21, 4-22; 10 Points</t>
@@ -2278,14 +3414,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B26" s="250" t="inlineStr"/>
-      <c r="C26" s="250" t="inlineStr"/>
-      <c r="D26" s="250" t="inlineStr">
+      <c r="B26" s="271" t="inlineStr"/>
+      <c r="C26" s="271" t="inlineStr"/>
+      <c r="D26" s="271" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E26" s="250" t="inlineStr"/>
+      <c r="E26" s="271" t="inlineStr"/>
       <c r="F26" s="112" t="inlineStr">
         <is>
           <t>Class 10 (9/28) - Catchup &amp; Midterm Review</t>
@@ -2298,14 +3434,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B27" s="250" t="inlineStr"/>
-      <c r="C27" s="250" t="inlineStr"/>
-      <c r="D27" s="250" t="inlineStr">
+      <c r="B27" s="271" t="inlineStr"/>
+      <c r="C27" s="271" t="inlineStr"/>
+      <c r="D27" s="271" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E27" s="250" t="inlineStr"/>
+      <c r="E27" s="271" t="inlineStr"/>
       <c r="F27" s="112" t="inlineStr">
         <is>
           <t>Class 10 (9/28) - 8-28, 8-29; 10 Points</t>
@@ -2318,14 +3454,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B28" s="250" t="inlineStr"/>
-      <c r="C28" s="250" t="inlineStr"/>
-      <c r="D28" s="250" t="inlineStr">
+      <c r="B28" s="271" t="inlineStr"/>
+      <c r="C28" s="271" t="inlineStr"/>
+      <c r="D28" s="271" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="E28" s="250" t="inlineStr"/>
+      <c r="E28" s="271" t="inlineStr"/>
       <c r="F28" s="112" t="inlineStr">
         <is>
           <t>Class 12 (10/7) - Cost volume profit analysis: Chapter 7</t>
@@ -2338,14 +3474,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B29" s="250" t="inlineStr"/>
-      <c r="C29" s="250" t="inlineStr"/>
-      <c r="D29" s="250" t="inlineStr">
+      <c r="B29" s="271" t="inlineStr"/>
+      <c r="C29" s="271" t="inlineStr"/>
+      <c r="D29" s="271" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="E29" s="250" t="inlineStr"/>
+      <c r="E29" s="271" t="inlineStr"/>
       <c r="F29" s="112" t="inlineStr">
         <is>
           <t>Class 12 (10/7) - 6-24, 6-25, 6-34; 15 Points</t>
@@ -2358,14 +3494,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B30" s="250" t="inlineStr"/>
-      <c r="C30" s="250" t="inlineStr"/>
-      <c r="D30" s="250" t="inlineStr">
+      <c r="B30" s="271" t="inlineStr"/>
+      <c r="C30" s="271" t="inlineStr"/>
+      <c r="D30" s="271" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E30" s="250" t="inlineStr"/>
+      <c r="E30" s="271" t="inlineStr"/>
       <c r="F30" s="112" t="inlineStr">
         <is>
           <t>Class 14 (10/14) - Financial planning and analysis:; Static: Chapter 9</t>
@@ -2378,14 +3514,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B31" s="250" t="inlineStr"/>
-      <c r="C31" s="250" t="inlineStr"/>
-      <c r="D31" s="250" t="inlineStr">
+      <c r="B31" s="271" t="inlineStr"/>
+      <c r="C31" s="271" t="inlineStr"/>
+      <c r="D31" s="271" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E31" s="250" t="inlineStr"/>
+      <c r="E31" s="271" t="inlineStr"/>
       <c r="F31" s="112" t="inlineStr">
         <is>
           <t>Class 14 (10/14) - 7-29, 7-33, 7-40; 15 Points</t>
@@ -2398,14 +3534,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B32" s="250" t="inlineStr"/>
-      <c r="C32" s="250" t="inlineStr"/>
-      <c r="D32" s="250" t="inlineStr">
+      <c r="B32" s="271" t="inlineStr"/>
+      <c r="C32" s="271" t="inlineStr"/>
+      <c r="D32" s="271" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E32" s="250" t="inlineStr"/>
+      <c r="E32" s="271" t="inlineStr"/>
       <c r="F32" s="112" t="inlineStr">
         <is>
           <t>Class 15 (10/19) - Capital Budgeting; Practice Midterm Ques: Chapter 16- ONLY; LO 16.1, 2, 3</t>
@@ -2418,14 +3554,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B33" s="250" t="inlineStr"/>
-      <c r="C33" s="250" t="inlineStr"/>
-      <c r="D33" s="250" t="inlineStr">
+      <c r="B33" s="271" t="inlineStr"/>
+      <c r="C33" s="271" t="inlineStr"/>
+      <c r="D33" s="271" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E33" s="250" t="inlineStr"/>
+      <c r="E33" s="271" t="inlineStr"/>
       <c r="F33" s="112" t="inlineStr">
         <is>
           <t>Class 15 (10/19) - 9-25, 9-28, 9-37; 15 - Points</t>
@@ -2438,14 +3574,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B34" s="250" t="inlineStr"/>
-      <c r="C34" s="250" t="inlineStr"/>
-      <c r="D34" s="250" t="inlineStr">
+      <c r="B34" s="271" t="inlineStr"/>
+      <c r="C34" s="271" t="inlineStr"/>
+      <c r="D34" s="271" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E34" s="250" t="inlineStr"/>
+      <c r="E34" s="271" t="inlineStr"/>
       <c r="F34" s="112" t="inlineStr">
         <is>
           <t>Class 16 (10/21) - Catchup &amp; Midterm Review</t>
@@ -2458,14 +3594,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B35" s="250" t="inlineStr"/>
-      <c r="C35" s="250" t="inlineStr"/>
-      <c r="D35" s="250" t="inlineStr">
+      <c r="B35" s="271" t="inlineStr"/>
+      <c r="C35" s="271" t="inlineStr"/>
+      <c r="D35" s="271" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E35" s="250" t="inlineStr"/>
+      <c r="E35" s="271" t="inlineStr"/>
       <c r="F35" s="112" t="inlineStr">
         <is>
           <t>Class 16 (10/21) - 16-28, 16-40; 10 Points</t>
@@ -2478,14 +3614,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B36" s="250" t="inlineStr"/>
-      <c r="C36" s="250" t="inlineStr"/>
-      <c r="D36" s="250" t="inlineStr">
+      <c r="B36" s="271" t="inlineStr"/>
+      <c r="C36" s="271" t="inlineStr"/>
+      <c r="D36" s="271" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="E36" s="250" t="inlineStr"/>
+      <c r="E36" s="271" t="inlineStr"/>
       <c r="F36" s="112" t="inlineStr">
         <is>
           <t>Class 19 (11/4) - Sales Variance Analysis; Flexible Budget: Chapter 11 - ONLY; LO 11.1, 11.2 &amp;; Appendix B</t>
@@ -2498,14 +3634,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B37" s="250" t="inlineStr"/>
-      <c r="C37" s="250" t="inlineStr"/>
-      <c r="D37" s="250" t="inlineStr">
+      <c r="B37" s="271" t="inlineStr"/>
+      <c r="C37" s="271" t="inlineStr"/>
+      <c r="D37" s="271" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="E37" s="250" t="inlineStr"/>
+      <c r="E37" s="271" t="inlineStr"/>
       <c r="F37" s="112" t="inlineStr">
         <is>
           <t>Class 19 (11/4) - 10-26, 10-30; 10 Points</t>
@@ -2518,14 +3654,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B38" s="250" t="inlineStr"/>
-      <c r="C38" s="250" t="inlineStr"/>
-      <c r="D38" s="250" t="inlineStr">
+      <c r="B38" s="271" t="inlineStr"/>
+      <c r="C38" s="271" t="inlineStr"/>
+      <c r="D38" s="271" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E38" s="250" t="inlineStr"/>
+      <c r="E38" s="271" t="inlineStr"/>
       <c r="F38" s="112" t="inlineStr">
         <is>
           <t>Class 20 (11/9) - Investment Centers: Chapter 13- ONLY; LO 13-1, 2, 3, 4</t>
@@ -2538,14 +3674,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B39" s="250" t="inlineStr"/>
-      <c r="C39" s="250" t="inlineStr"/>
-      <c r="D39" s="250" t="inlineStr">
+      <c r="B39" s="271" t="inlineStr"/>
+      <c r="C39" s="271" t="inlineStr"/>
+      <c r="D39" s="271" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E39" s="250" t="inlineStr"/>
+      <c r="E39" s="271" t="inlineStr"/>
       <c r="F39" s="112" t="inlineStr">
         <is>
           <t>Class 20 (11/9) - 11-31, 11-52; 10 Points</t>
@@ -2558,14 +3694,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B40" s="250" t="inlineStr"/>
-      <c r="C40" s="250" t="inlineStr"/>
-      <c r="D40" s="250" t="inlineStr">
+      <c r="B40" s="271" t="inlineStr"/>
+      <c r="C40" s="271" t="inlineStr"/>
+      <c r="D40" s="271" t="inlineStr">
         <is>
           <t>2026-11-16</t>
         </is>
       </c>
-      <c r="E40" s="250" t="inlineStr"/>
+      <c r="E40" s="271" t="inlineStr"/>
       <c r="F40" s="112" t="inlineStr">
         <is>
           <t>Class 21 (11/16) - AI &amp; FP&amp;A</t>
@@ -2578,14 +3714,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B41" s="250" t="inlineStr"/>
-      <c r="C41" s="250" t="inlineStr"/>
-      <c r="D41" s="250" t="inlineStr">
+      <c r="B41" s="271" t="inlineStr"/>
+      <c r="C41" s="271" t="inlineStr"/>
+      <c r="D41" s="271" t="inlineStr">
         <is>
           <t>2026-11-16</t>
         </is>
       </c>
-      <c r="E41" s="250" t="inlineStr"/>
+      <c r="E41" s="271" t="inlineStr"/>
       <c r="F41" s="112" t="inlineStr">
         <is>
           <t>Class 21 (11/16) - 13-29, 13-33; 10 Points</t>
@@ -2598,14 +3734,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B42" s="250" t="inlineStr"/>
-      <c r="C42" s="250" t="inlineStr"/>
-      <c r="D42" s="250" t="inlineStr">
+      <c r="B42" s="271" t="inlineStr"/>
+      <c r="C42" s="271" t="inlineStr"/>
+      <c r="D42" s="271" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E42" s="250" t="inlineStr"/>
+      <c r="E42" s="271" t="inlineStr"/>
       <c r="F42" s="112" t="inlineStr">
         <is>
           <t>Class 2 (12/2) - Catchup &amp; Final Review; Practice Final Questions Posted to Brightspace at; 5:00 PM</t>
@@ -2618,14 +3754,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B43" s="250" t="inlineStr"/>
-      <c r="C43" s="250" t="inlineStr"/>
-      <c r="D43" s="250" t="inlineStr">
+      <c r="B43" s="271" t="inlineStr"/>
+      <c r="C43" s="271" t="inlineStr"/>
+      <c r="D43" s="271" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E43" s="250" t="inlineStr"/>
+      <c r="E43" s="271" t="inlineStr"/>
       <c r="F43" s="112" t="inlineStr">
         <is>
           <t>Class 2 (12/2) - 14-35, 14-41; 10 Points; Assignments listed Be-; low Due by11:59 PM; Linked In Learning; E</t>
@@ -2638,22 +3774,22 @@
           <t>LinkedIn Learning Excel Certification</t>
         </is>
       </c>
-      <c r="B44" s="248" t="inlineStr">
+      <c r="B44" s="269" t="inlineStr">
         <is>
           <t>75 pts</t>
         </is>
       </c>
-      <c r="C44" s="249" t="inlineStr">
+      <c r="C44" s="270" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D44" s="249" t="inlineStr">
+      <c r="D44" s="270" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E44" s="249" t="inlineStr">
+      <c r="E44" s="270" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2669,18 +3805,18 @@
           <t>Certification</t>
         </is>
       </c>
-      <c r="B45" s="250" t="inlineStr"/>
-      <c r="C45" s="250" t="inlineStr">
+      <c r="B45" s="271" t="inlineStr"/>
+      <c r="C45" s="271" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D45" s="250" t="inlineStr">
+      <c r="D45" s="271" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E45" s="250" t="inlineStr"/>
+      <c r="E45" s="271" t="inlineStr"/>
       <c r="F45" s="112" t="inlineStr">
         <is>
           <t>LinkedIn Learning Excel Certification</t>
@@ -2693,22 +3829,22 @@
           <t>Stukent Simternship</t>
         </is>
       </c>
-      <c r="B46" s="248" t="inlineStr">
+      <c r="B46" s="269" t="inlineStr">
         <is>
           <t>75 pts</t>
         </is>
       </c>
-      <c r="C46" s="251" t="inlineStr">
+      <c r="C46" s="272" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D46" s="251" t="inlineStr">
+      <c r="D46" s="272" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E46" s="251" t="inlineStr">
+      <c r="E46" s="272" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -2724,18 +3860,18 @@
           <t>Certification</t>
         </is>
       </c>
-      <c r="B47" s="250" t="inlineStr"/>
-      <c r="C47" s="250" t="inlineStr">
+      <c r="B47" s="271" t="inlineStr"/>
+      <c r="C47" s="271" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D47" s="250" t="inlineStr">
+      <c r="D47" s="271" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E47" s="250" t="inlineStr"/>
+      <c r="E47" s="271" t="inlineStr"/>
       <c r="F47" s="112" t="inlineStr">
         <is>
           <t>Stukent Simternship</t>
@@ -2761,1093 +3897,6 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="A7:F7"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="001F77B4"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F50"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="20" t="inlineStr">
-        <is>
-          <t>BUAD-304 — Organizational Behavior and Leadership</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="2">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/sources/buad-304-source.pdf","SEE HERE")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Instructor</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Christine El Haddad</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Term</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Fall 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Required for an A</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Curved (class rank)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Grading scale</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Weighted score (% of points earned) + class average + student ranking (relative grading - no fixed A threshold in syllabus)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="156" t="inlineStr">
-        <is>
-          <t>Final Exam 25%  |  Participation 15%  |  Midterm Exam 15%  |  Team Project Paper 15%  |  Final Reflection Paper 10%  |  Presentation 10%  |  Case Analysis Assignments 5%  |  Proposal &amp; Team Contract 3%  |  Self &amp; Peer Evaluation 2%</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="21" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B9" s="21" t="inlineStr">
-        <is>
-          <t>Weight</t>
-        </is>
-      </c>
-      <c r="C9" s="21" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="D9" s="21" t="inlineStr">
-        <is>
-          <t>Due Date</t>
-        </is>
-      </c>
-      <c r="E9" s="21" t="inlineStr">
-        <is>
-          <t>Group Project</t>
-        </is>
-      </c>
-      <c r="F9" s="21" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="120" t="inlineStr">
-        <is>
-          <t>Final Exam</t>
-        </is>
-      </c>
-      <c r="B10" s="256" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="C10" s="257" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D10" s="257" t="inlineStr">
-        <is>
-          <t>2026-12-09</t>
-        </is>
-      </c>
-      <c r="E10" s="257" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F10" s="123">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-final-exam.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="124" t="inlineStr">
-        <is>
-          <t>Exam</t>
-        </is>
-      </c>
-      <c r="B11" s="258" t="inlineStr"/>
-      <c r="C11" s="258" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D11" s="258" t="inlineStr">
-        <is>
-          <t>2026-12-09</t>
-        </is>
-      </c>
-      <c r="E11" s="258" t="inlineStr"/>
-      <c r="F11" s="126" t="inlineStr">
-        <is>
-          <t>Final Exam</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="127" t="inlineStr">
-        <is>
-          <t>Participation</t>
-        </is>
-      </c>
-      <c r="B12" s="256" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="C12" s="259" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D12" s="259" t="inlineStr">
-        <is>
-          <t>2026-12-04</t>
-        </is>
-      </c>
-      <c r="E12" s="259" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F12" s="129">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-participation.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="131" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B13" s="258" t="inlineStr"/>
-      <c r="C13" s="258" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D13" s="258" t="inlineStr"/>
-      <c r="E13" s="258" t="inlineStr"/>
-      <c r="F13" s="126" t="inlineStr">
-        <is>
-          <t>Research: SONA registration opens</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="131" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B14" s="258" t="inlineStr"/>
-      <c r="C14" s="258" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="D14" s="258" t="inlineStr"/>
-      <c r="E14" s="258" t="inlineStr"/>
-      <c r="F14" s="126" t="inlineStr">
-        <is>
-          <t>Research: Prescreening questionnaire opens</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="131" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B15" s="258" t="inlineStr"/>
-      <c r="C15" s="258" t="inlineStr"/>
-      <c r="D15" s="258" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="E15" s="258" t="inlineStr"/>
-      <c r="F15" s="126" t="inlineStr">
-        <is>
-          <t>Research: Setup deadline (registration, prescreening, contacts)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="131" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B16" s="258" t="inlineStr"/>
-      <c r="C16" s="258" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="D16" s="258" t="inlineStr"/>
-      <c r="E16" s="258" t="inlineStr"/>
-      <c r="F16" s="126" t="inlineStr">
-        <is>
-          <t>Research: Study invitations begin (after setup)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="131" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B17" s="258" t="inlineStr"/>
-      <c r="C17" s="258" t="inlineStr"/>
-      <c r="D17" s="258" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="E17" s="258" t="inlineStr"/>
-      <c r="F17" s="126" t="inlineStr">
-        <is>
-          <t>Research: Employee contact surveys sent</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="131" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B18" s="258" t="inlineStr"/>
-      <c r="C18" s="258" t="inlineStr"/>
-      <c r="D18" s="258" t="inlineStr">
-        <is>
-          <t>2026-12-04</t>
-        </is>
-      </c>
-      <c r="E18" s="258" t="inlineStr"/>
-      <c r="F18" s="126" t="inlineStr">
-        <is>
-          <t>Research: Complete 2.0 research credits</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="120" t="inlineStr">
-        <is>
-          <t>Midterm Exam</t>
-        </is>
-      </c>
-      <c r="B19" s="256" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="C19" s="257" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D19" s="257" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E19" s="257" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F19" s="123">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-midterm-exam.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="124" t="inlineStr">
-        <is>
-          <t>Exam</t>
-        </is>
-      </c>
-      <c r="B20" s="258" t="inlineStr"/>
-      <c r="C20" s="258" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D20" s="258" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E20" s="258" t="inlineStr"/>
-      <c r="F20" s="126" t="inlineStr">
-        <is>
-          <t>Midterm Exam</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="127" t="inlineStr">
-        <is>
-          <t>Team Project Paper</t>
-        </is>
-      </c>
-      <c r="B21" s="256" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="C21" s="259" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D21" s="259" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="E21" s="259" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F21" s="129">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-team-project-paper.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="132" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B22" s="258" t="inlineStr"/>
-      <c r="C22" s="258" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D22" s="258" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E22" s="258" t="inlineStr"/>
-      <c r="F22" s="126" t="inlineStr">
-        <is>
-          <t>Team project outline</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="132" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B23" s="258" t="inlineStr"/>
-      <c r="C23" s="258" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D23" s="258" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="E23" s="258" t="inlineStr"/>
-      <c r="F23" s="126" t="inlineStr">
-        <is>
-          <t>Team project paper</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="120" t="inlineStr">
-        <is>
-          <t>Final Reflection Paper</t>
-        </is>
-      </c>
-      <c r="B24" s="256" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="C24" s="257" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D24" s="257" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E24" s="257" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F24" s="123">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-final-reflection-paper.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="132" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B25" s="258" t="inlineStr"/>
-      <c r="C25" s="258" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D25" s="258" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E25" s="258" t="inlineStr"/>
-      <c r="F25" s="126" t="inlineStr">
-        <is>
-          <t>Personal Reflection Paper</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="127" t="inlineStr">
-        <is>
-          <t>Presentation</t>
-        </is>
-      </c>
-      <c r="B26" s="256" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="C26" s="259" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D26" s="259" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="E26" s="259" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F26" s="129">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-presentation.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="132" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B27" s="258" t="inlineStr"/>
-      <c r="C27" s="258" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D27" s="258" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="E27" s="258" t="inlineStr"/>
-      <c r="F27" s="126" t="inlineStr">
-        <is>
-          <t>Presentation slides</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="120" t="inlineStr">
-        <is>
-          <t>Case Analysis Assignments</t>
-        </is>
-      </c>
-      <c r="B28" s="256" t="inlineStr">
-        <is>
-          <t>5%</t>
-        </is>
-      </c>
-      <c r="C28" s="257" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="D28" s="257" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="E28" s="257" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F28" s="123">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-case-analysis-assignments.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="132" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B29" s="258" t="inlineStr"/>
-      <c r="C29" s="258" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="D29" s="258" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="E29" s="258" t="inlineStr"/>
-      <c r="F29" s="126" t="inlineStr">
-        <is>
-          <t>Thomas Green Case Analysis Memo</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="132" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B30" s="258" t="inlineStr"/>
-      <c r="C30" s="258" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="D30" s="258" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="E30" s="258" t="inlineStr"/>
-      <c r="F30" s="126" t="inlineStr">
-        <is>
-          <t>SkillsForTomorrow Analysis Memo</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="127" t="inlineStr">
-        <is>
-          <t>Proposal &amp; Team Contract</t>
-        </is>
-      </c>
-      <c r="B31" s="256" t="inlineStr">
-        <is>
-          <t>3%</t>
-        </is>
-      </c>
-      <c r="C31" s="259" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D31" s="259" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E31" s="259" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F31" s="129">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-proposal-team-contract.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="132" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B32" s="258" t="inlineStr"/>
-      <c r="C32" s="258" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D32" s="258" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E32" s="258" t="inlineStr"/>
-      <c r="F32" s="126" t="inlineStr">
-        <is>
-          <t>Team project proposal &amp; team contract</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="120" t="inlineStr">
-        <is>
-          <t>Self &amp; Peer Evaluation</t>
-        </is>
-      </c>
-      <c r="B33" s="256" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="C33" s="257" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D33" s="257" t="inlineStr">
-        <is>
-          <t>2026-11-18</t>
-        </is>
-      </c>
-      <c r="E33" s="257" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F33" s="123">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-self-peer-evaluation.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="132" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B34" s="258" t="inlineStr"/>
-      <c r="C34" s="258" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D34" s="258" t="inlineStr">
-        <is>
-          <t>2026-11-18</t>
-        </is>
-      </c>
-      <c r="E34" s="258" t="inlineStr"/>
-      <c r="F34" s="126" t="inlineStr">
-        <is>
-          <t>Self &amp; peer evaluation</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="127" t="inlineStr">
-        <is>
-          <t>Personal Assessments (Connect)</t>
-        </is>
-      </c>
-      <c r="B35" s="256" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C35" s="259" t="inlineStr"/>
-      <c r="D35" s="259" t="inlineStr">
-        <is>
-          <t>2026-12-20</t>
-        </is>
-      </c>
-      <c r="E35" s="259" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F35" s="129">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-personal-assessments-connect.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="130" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B36" s="258" t="inlineStr"/>
-      <c r="C36" s="258" t="inlineStr"/>
-      <c r="D36" s="258" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="E36" s="258" t="inlineStr"/>
-      <c r="F36" s="126" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="130" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B37" s="258" t="inlineStr"/>
-      <c r="C37" s="258" t="inlineStr"/>
-      <c r="D37" s="258" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="E37" s="258" t="inlineStr"/>
-      <c r="F37" s="126" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="130" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B38" s="258" t="inlineStr"/>
-      <c r="C38" s="258" t="inlineStr"/>
-      <c r="D38" s="258" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="E38" s="258" t="inlineStr"/>
-      <c r="F38" s="126" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 5.01 - Assessing Your</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="130" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B39" s="258" t="inlineStr"/>
-      <c r="C39" s="258" t="inlineStr"/>
-      <c r="D39" s="258" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="E39" s="258" t="inlineStr"/>
-      <c r="F39" s="126" t="inlineStr">
-        <is>
-          <t>Connect: Sharpen Companion</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="130" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B40" s="258" t="inlineStr"/>
-      <c r="C40" s="258" t="inlineStr"/>
-      <c r="D40" s="258" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="E40" s="258" t="inlineStr"/>
-      <c r="F40" s="126" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 11.01 - What is my</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="130" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B41" s="258" t="inlineStr"/>
-      <c r="C41" s="258" t="inlineStr"/>
-      <c r="D41" s="258" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="E41" s="258" t="inlineStr"/>
-      <c r="F41" s="126" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 11.02 - What is my</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="130" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B42" s="258" t="inlineStr"/>
-      <c r="C42" s="258" t="inlineStr"/>
-      <c r="D42" s="258" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="E42" s="258" t="inlineStr"/>
-      <c r="F42" s="126" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 12.01 - What kind of</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="130" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B43" s="258" t="inlineStr"/>
-      <c r="C43" s="258" t="inlineStr"/>
-      <c r="D43" s="258" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E43" s="258" t="inlineStr"/>
-      <c r="F43" s="126" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 10.5 - Preferred Conflict</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="130" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B44" s="258" t="inlineStr"/>
-      <c r="C44" s="258" t="inlineStr"/>
-      <c r="D44" s="258" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E44" s="258" t="inlineStr"/>
-      <c r="F44" s="126" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 9.01 - Assessing My</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="130" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B45" s="258" t="inlineStr"/>
-      <c r="C45" s="258" t="inlineStr"/>
-      <c r="D45" s="258" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E45" s="258" t="inlineStr"/>
-      <c r="F45" s="126" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 8.01 - Group</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="130" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B46" s="258" t="inlineStr"/>
-      <c r="C46" s="258" t="inlineStr"/>
-      <c r="D46" s="258" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="E46" s="258" t="inlineStr"/>
-      <c r="F46" s="126" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 14.02 - What Type of Organizational Culture Do I</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="130" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B47" s="258" t="inlineStr"/>
-      <c r="C47" s="258" t="inlineStr"/>
-      <c r="D47" s="258" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
-      </c>
-      <c r="E47" s="258" t="inlineStr"/>
-      <c r="F47" s="126" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 16.02 - What Is Your</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="130" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B48" s="258" t="inlineStr"/>
-      <c r="C48" s="258" t="inlineStr"/>
-      <c r="D48" s="258" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
-      </c>
-      <c r="E48" s="258" t="inlineStr"/>
-      <c r="F48" s="126" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 16.03 - Assessing Your</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="130" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B49" s="258" t="inlineStr"/>
-      <c r="C49" s="258" t="inlineStr"/>
-      <c r="D49" s="258" t="inlineStr">
-        <is>
-          <t>2026-12-20</t>
-        </is>
-      </c>
-      <c r="E49" s="258" t="inlineStr"/>
-      <c r="F49" s="126" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 12.02 - Which influence</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B50" s="133" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="B6:F6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3977,18 +4026,18 @@
           <t>Sleep Paper</t>
         </is>
       </c>
-      <c r="B10" s="260" t="inlineStr">
+      <c r="B10" s="274" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C10" s="261" t="inlineStr"/>
-      <c r="D10" s="261" t="inlineStr">
+      <c r="C10" s="275" t="inlineStr"/>
+      <c r="D10" s="275" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="E10" s="261" t="inlineStr">
+      <c r="E10" s="275" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4004,14 +4053,14 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B11" s="262" t="inlineStr"/>
-      <c r="C11" s="262" t="inlineStr"/>
-      <c r="D11" s="262" t="inlineStr">
+      <c r="B11" s="276" t="inlineStr"/>
+      <c r="C11" s="276" t="inlineStr"/>
+      <c r="D11" s="276" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="E11" s="262" t="inlineStr"/>
+      <c r="E11" s="276" t="inlineStr"/>
       <c r="F11" s="99" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
@@ -4024,18 +4073,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B12" s="262" t="inlineStr"/>
-      <c r="C12" s="262" t="inlineStr">
+      <c r="B12" s="276" t="inlineStr"/>
+      <c r="C12" s="276" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D12" s="262" t="inlineStr">
+      <c r="D12" s="276" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E12" s="262" t="inlineStr"/>
+      <c r="E12" s="276" t="inlineStr"/>
       <c r="F12" s="99" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance</t>
@@ -4048,18 +4097,18 @@
           <t>Witchcraft Paper</t>
         </is>
       </c>
-      <c r="B13" s="260" t="inlineStr">
+      <c r="B13" s="274" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C13" s="263" t="inlineStr"/>
-      <c r="D13" s="263" t="inlineStr">
+      <c r="C13" s="277" t="inlineStr"/>
+      <c r="D13" s="277" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="E13" s="263" t="inlineStr">
+      <c r="E13" s="277" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4075,14 +4124,14 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B14" s="262" t="inlineStr"/>
-      <c r="C14" s="262" t="inlineStr"/>
-      <c r="D14" s="262" t="inlineStr">
+      <c r="B14" s="276" t="inlineStr"/>
+      <c r="C14" s="276" t="inlineStr"/>
+      <c r="D14" s="276" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="E14" s="262" t="inlineStr"/>
+      <c r="E14" s="276" t="inlineStr"/>
       <c r="F14" s="99" t="inlineStr">
         <is>
           <t>Witchcraft Paper Due</t>
@@ -4095,18 +4144,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B15" s="262" t="inlineStr"/>
-      <c r="C15" s="262" t="inlineStr">
+      <c r="B15" s="276" t="inlineStr"/>
+      <c r="C15" s="276" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D15" s="262" t="inlineStr">
+      <c r="D15" s="276" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E15" s="262" t="inlineStr"/>
+      <c r="E15" s="276" t="inlineStr"/>
       <c r="F15" s="99" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment</t>
@@ -4119,18 +4168,18 @@
           <t>Mid-term</t>
         </is>
       </c>
-      <c r="B16" s="260" t="inlineStr">
+      <c r="B16" s="274" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C16" s="261" t="inlineStr"/>
-      <c r="D16" s="261" t="inlineStr">
+      <c r="C16" s="275" t="inlineStr"/>
+      <c r="D16" s="275" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E16" s="261" t="inlineStr">
+      <c r="E16" s="275" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4146,14 +4195,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B17" s="262" t="inlineStr"/>
-      <c r="C17" s="262" t="inlineStr"/>
-      <c r="D17" s="262" t="inlineStr">
+      <c r="B17" s="276" t="inlineStr"/>
+      <c r="C17" s="276" t="inlineStr"/>
+      <c r="D17" s="276" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="E17" s="262" t="inlineStr"/>
+      <c r="E17" s="276" t="inlineStr"/>
       <c r="F17" s="99" t="inlineStr">
         <is>
           <t>Midterm Exam</t>
@@ -4166,18 +4215,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B18" s="262" t="inlineStr"/>
-      <c r="C18" s="262" t="inlineStr">
+      <c r="B18" s="276" t="inlineStr"/>
+      <c r="C18" s="276" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="D18" s="262" t="inlineStr">
+      <c r="D18" s="276" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E18" s="262" t="inlineStr"/>
+      <c r="E18" s="276" t="inlineStr"/>
       <c r="F18" s="99" t="inlineStr">
         <is>
           <t>Week Oct 6-9: Midterm &amp; Break</t>
@@ -4190,18 +4239,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B19" s="262" t="inlineStr"/>
-      <c r="C19" s="262" t="inlineStr">
+      <c r="B19" s="276" t="inlineStr"/>
+      <c r="C19" s="276" t="inlineStr">
         <is>
           <t>2026-12-01</t>
         </is>
       </c>
-      <c r="D19" s="262" t="inlineStr">
+      <c r="D19" s="276" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E19" s="262" t="inlineStr"/>
+      <c r="E19" s="276" t="inlineStr"/>
       <c r="F19" s="99" t="inlineStr">
         <is>
           <t>Week Dec 1-4: Modern Europe?</t>
@@ -4214,18 +4263,18 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B20" s="260" t="inlineStr">
+      <c r="B20" s="274" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C20" s="263" t="inlineStr"/>
-      <c r="D20" s="263" t="inlineStr">
+      <c r="C20" s="277" t="inlineStr"/>
+      <c r="D20" s="277" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="E20" s="263" t="inlineStr">
+      <c r="E20" s="277" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4241,14 +4290,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B21" s="262" t="inlineStr"/>
-      <c r="C21" s="262" t="inlineStr"/>
-      <c r="D21" s="262" t="inlineStr">
+      <c r="B21" s="276" t="inlineStr"/>
+      <c r="C21" s="276" t="inlineStr"/>
+      <c r="D21" s="276" t="inlineStr">
         <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="E21" s="262" t="inlineStr"/>
+      <c r="E21" s="276" t="inlineStr"/>
       <c r="F21" s="99" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -4261,18 +4310,18 @@
           <t>Discussion Section</t>
         </is>
       </c>
-      <c r="B22" s="260" t="inlineStr">
+      <c r="B22" s="274" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C22" s="261" t="inlineStr"/>
-      <c r="D22" s="261" t="inlineStr">
+      <c r="C22" s="275" t="inlineStr"/>
+      <c r="D22" s="275" t="inlineStr">
         <is>
           <t>2026-11-12</t>
         </is>
       </c>
-      <c r="E22" s="261" t="inlineStr">
+      <c r="E22" s="275" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4288,18 +4337,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B23" s="262" t="inlineStr"/>
-      <c r="C23" s="262" t="inlineStr">
+      <c r="B23" s="276" t="inlineStr"/>
+      <c r="C23" s="276" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D23" s="262" t="inlineStr">
+      <c r="D23" s="276" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E23" s="262" t="inlineStr"/>
+      <c r="E23" s="276" t="inlineStr"/>
       <c r="F23" s="99" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death</t>
@@ -4312,18 +4361,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B24" s="262" t="inlineStr"/>
-      <c r="C24" s="262" t="inlineStr">
+      <c r="B24" s="276" t="inlineStr"/>
+      <c r="C24" s="276" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D24" s="262" t="inlineStr">
+      <c r="D24" s="276" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E24" s="262" t="inlineStr"/>
+      <c r="E24" s="276" t="inlineStr"/>
       <c r="F24" s="99" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death - Section reading 1: -- 13 of 33 -- Lizzie Wade, “From Black Death to fatal flu, pas</t>
@@ -4336,18 +4385,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B25" s="262" t="inlineStr"/>
-      <c r="C25" s="262" t="inlineStr">
+      <c r="B25" s="276" t="inlineStr"/>
+      <c r="C25" s="276" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D25" s="262" t="inlineStr">
+      <c r="D25" s="276" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E25" s="262" t="inlineStr"/>
+      <c r="E25" s="276" t="inlineStr"/>
       <c r="F25" s="99" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life</t>
@@ -4360,18 +4409,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B26" s="262" t="inlineStr"/>
-      <c r="C26" s="262" t="inlineStr">
+      <c r="B26" s="276" t="inlineStr"/>
+      <c r="C26" s="276" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D26" s="262" t="inlineStr">
+      <c r="D26" s="276" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E26" s="262" t="inlineStr"/>
+      <c r="E26" s="276" t="inlineStr"/>
       <c r="F26" s="99" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life - Section reading 1: A Roger Ekirch, “Sleep we have lost: Pre-Industrial Slumber in the Brit</t>
@@ -4384,18 +4433,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B27" s="262" t="inlineStr"/>
-      <c r="C27" s="262" t="inlineStr">
+      <c r="B27" s="276" t="inlineStr"/>
+      <c r="C27" s="276" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D27" s="262" t="inlineStr">
+      <c r="D27" s="276" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E27" s="262" t="inlineStr"/>
+      <c r="E27" s="276" t="inlineStr"/>
       <c r="F27" s="99" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance</t>
@@ -4408,18 +4457,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B28" s="262" t="inlineStr"/>
-      <c r="C28" s="262" t="inlineStr">
+      <c r="B28" s="276" t="inlineStr"/>
+      <c r="C28" s="276" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D28" s="262" t="inlineStr">
+      <c r="D28" s="276" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E28" s="262" t="inlineStr"/>
+      <c r="E28" s="276" t="inlineStr"/>
       <c r="F28" s="99" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance - Section reading 1: -- 14 of 33 -- Kay Daly, “Diverting the Flood of History: Ada Palmer’s I</t>
@@ -4432,18 +4481,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B29" s="262" t="inlineStr"/>
-      <c r="C29" s="262" t="inlineStr">
+      <c r="B29" s="276" t="inlineStr"/>
+      <c r="C29" s="276" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D29" s="262" t="inlineStr">
+      <c r="D29" s="276" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E29" s="262" t="inlineStr"/>
+      <c r="E29" s="276" t="inlineStr"/>
       <c r="F29" s="99" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance - Section reading 1: Vasari, Lives of the Artists: Leonardo da Vinci &amp; Properzia de’ Rossi V</t>
@@ -4456,18 +4505,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B30" s="262" t="inlineStr"/>
-      <c r="C30" s="262" t="inlineStr">
+      <c r="B30" s="276" t="inlineStr"/>
+      <c r="C30" s="276" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D30" s="262" t="inlineStr">
+      <c r="D30" s="276" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E30" s="262" t="inlineStr"/>
+      <c r="E30" s="276" t="inlineStr"/>
       <c r="F30" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion</t>
@@ -4480,18 +4529,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B31" s="262" t="inlineStr"/>
-      <c r="C31" s="262" t="inlineStr">
+      <c r="B31" s="276" t="inlineStr"/>
+      <c r="C31" s="276" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D31" s="262" t="inlineStr">
+      <c r="D31" s="276" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E31" s="262" t="inlineStr"/>
+      <c r="E31" s="276" t="inlineStr"/>
       <c r="F31" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion - Section reading 1: Jerry Brotton, The Renaissance Bazaar, Chap 1 (15 pgs) Read Colu</t>
@@ -4504,18 +4553,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B32" s="262" t="inlineStr"/>
-      <c r="C32" s="262" t="inlineStr">
+      <c r="B32" s="276" t="inlineStr"/>
+      <c r="C32" s="276" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D32" s="262" t="inlineStr">
+      <c r="D32" s="276" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E32" s="262" t="inlineStr"/>
+      <c r="E32" s="276" t="inlineStr"/>
       <c r="F32" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion - Section reading 2: Bernal Diaz del Castillo, The True History of the Conquest of Ne</t>
@@ -4528,18 +4577,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B33" s="262" t="inlineStr"/>
-      <c r="C33" s="262" t="inlineStr">
+      <c r="B33" s="276" t="inlineStr"/>
+      <c r="C33" s="276" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="D33" s="262" t="inlineStr">
+      <c r="D33" s="276" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="E33" s="262" t="inlineStr"/>
+      <c r="E33" s="276" t="inlineStr"/>
       <c r="F33" s="99" t="inlineStr">
         <is>
           <t>Week Oct 13-16: The Reformation</t>
@@ -4552,18 +4601,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B34" s="262" t="inlineStr"/>
-      <c r="C34" s="262" t="inlineStr">
+      <c r="B34" s="276" t="inlineStr"/>
+      <c r="C34" s="276" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="D34" s="262" t="inlineStr">
+      <c r="D34" s="276" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="E34" s="262" t="inlineStr"/>
+      <c r="E34" s="276" t="inlineStr"/>
       <c r="F34" s="99" t="inlineStr">
         <is>
           <t>Week Oct 20-23: The Reformation</t>
@@ -4576,18 +4625,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B35" s="262" t="inlineStr"/>
-      <c r="C35" s="262" t="inlineStr">
+      <c r="B35" s="276" t="inlineStr"/>
+      <c r="C35" s="276" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D35" s="262" t="inlineStr">
+      <c r="D35" s="276" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E35" s="262" t="inlineStr"/>
+      <c r="E35" s="276" t="inlineStr"/>
       <c r="F35" s="99" t="inlineStr">
         <is>
           <t>Week Oct 27-30: Reformation</t>
@@ -4600,18 +4649,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B36" s="262" t="inlineStr"/>
-      <c r="C36" s="262" t="inlineStr">
+      <c r="B36" s="276" t="inlineStr"/>
+      <c r="C36" s="276" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D36" s="262" t="inlineStr">
+      <c r="D36" s="276" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E36" s="262" t="inlineStr"/>
+      <c r="E36" s="276" t="inlineStr"/>
       <c r="F36" s="99" t="inlineStr">
         <is>
           <t xml:space="preserve">Week Oct 27-30: Reformation - Section reading 1: Barbara Diefendorf, ed., The Saint Bartholomew’s Day Massacre: A Brief </t>
@@ -4624,18 +4673,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B37" s="262" t="inlineStr"/>
-      <c r="C37" s="262" t="inlineStr">
+      <c r="B37" s="276" t="inlineStr"/>
+      <c r="C37" s="276" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D37" s="262" t="inlineStr">
+      <c r="D37" s="276" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E37" s="262" t="inlineStr"/>
+      <c r="E37" s="276" t="inlineStr"/>
       <c r="F37" s="99" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science</t>
@@ -4648,18 +4697,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B38" s="262" t="inlineStr"/>
-      <c r="C38" s="262" t="inlineStr">
+      <c r="B38" s="276" t="inlineStr"/>
+      <c r="C38" s="276" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D38" s="262" t="inlineStr">
+      <c r="D38" s="276" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E38" s="262" t="inlineStr"/>
+      <c r="E38" s="276" t="inlineStr"/>
       <c r="F38" s="99" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science - Section reading 1: Brian Levack, The Witchcraft Sourcebook, Chaps 36-44, 46-47 103.Lev</t>
@@ -4672,18 +4721,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B39" s="262" t="inlineStr"/>
-      <c r="C39" s="262" t="inlineStr">
+      <c r="B39" s="276" t="inlineStr"/>
+      <c r="C39" s="276" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D39" s="262" t="inlineStr">
+      <c r="D39" s="276" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E39" s="262" t="inlineStr"/>
+      <c r="E39" s="276" t="inlineStr"/>
       <c r="F39" s="99" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment - Section reading 1: Excerpt: John Locke, Two Treatises of Government (1689) Excerpt: Rous</t>
@@ -4696,18 +4745,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B40" s="262" t="inlineStr"/>
-      <c r="C40" s="262" t="inlineStr">
+      <c r="B40" s="276" t="inlineStr"/>
+      <c r="C40" s="276" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D40" s="262" t="inlineStr">
+      <c r="D40" s="276" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E40" s="262" t="inlineStr"/>
+      <c r="E40" s="276" t="inlineStr"/>
       <c r="F40" s="99" t="inlineStr">
         <is>
           <t>Week Nov 17-20: Enlightenment</t>
@@ -4720,18 +4769,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B41" s="262" t="inlineStr"/>
-      <c r="C41" s="262" t="inlineStr">
+      <c r="B41" s="276" t="inlineStr"/>
+      <c r="C41" s="276" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D41" s="262" t="inlineStr">
+      <c r="D41" s="276" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E41" s="262" t="inlineStr"/>
+      <c r="E41" s="276" t="inlineStr"/>
       <c r="F41" s="99" t="inlineStr">
         <is>
           <t xml:space="preserve">Week Nov 17-20: Enlightenment - Section reading 1: Video: Africa &amp; Britain, A Forgotten History, Episode 2: Freedom (50 </t>
@@ -4744,18 +4793,18 @@
           <t>Identification Quizzes</t>
         </is>
       </c>
-      <c r="B42" s="260" t="inlineStr">
+      <c r="B42" s="274" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C42" s="263" t="inlineStr"/>
-      <c r="D42" s="263" t="inlineStr">
+      <c r="C42" s="277" t="inlineStr"/>
+      <c r="D42" s="277" t="inlineStr">
         <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="E42" s="263" t="inlineStr">
+      <c r="E42" s="277" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4771,18 +4820,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B43" s="262" t="inlineStr"/>
-      <c r="C43" s="262" t="inlineStr">
+      <c r="B43" s="276" t="inlineStr"/>
+      <c r="C43" s="276" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D43" s="262" t="inlineStr">
+      <c r="D43" s="276" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E43" s="262" t="inlineStr"/>
+      <c r="E43" s="276" t="inlineStr"/>
       <c r="F43" s="99" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death (lecture topics)</t>
@@ -4795,18 +4844,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B44" s="262" t="inlineStr"/>
-      <c r="C44" s="262" t="inlineStr">
+      <c r="B44" s="276" t="inlineStr"/>
+      <c r="C44" s="276" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D44" s="262" t="inlineStr">
+      <c r="D44" s="276" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E44" s="262" t="inlineStr"/>
+      <c r="E44" s="276" t="inlineStr"/>
       <c r="F44" s="99" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life (lecture topics)</t>
@@ -4819,18 +4868,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B45" s="262" t="inlineStr"/>
-      <c r="C45" s="262" t="inlineStr">
+      <c r="B45" s="276" t="inlineStr"/>
+      <c r="C45" s="276" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D45" s="262" t="inlineStr">
+      <c r="D45" s="276" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E45" s="262" t="inlineStr"/>
+      <c r="E45" s="276" t="inlineStr"/>
       <c r="F45" s="99" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance (lecture topics)</t>
@@ -4843,18 +4892,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B46" s="262" t="inlineStr"/>
-      <c r="C46" s="262" t="inlineStr">
+      <c r="B46" s="276" t="inlineStr"/>
+      <c r="C46" s="276" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D46" s="262" t="inlineStr">
+      <c r="D46" s="276" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E46" s="262" t="inlineStr"/>
+      <c r="E46" s="276" t="inlineStr"/>
       <c r="F46" s="99" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance (lecture topics)</t>
@@ -4867,18 +4916,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B47" s="262" t="inlineStr"/>
-      <c r="C47" s="262" t="inlineStr">
+      <c r="B47" s="276" t="inlineStr"/>
+      <c r="C47" s="276" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D47" s="262" t="inlineStr">
+      <c r="D47" s="276" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E47" s="262" t="inlineStr"/>
+      <c r="E47" s="276" t="inlineStr"/>
       <c r="F47" s="99" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion (lecture topics)</t>
@@ -4891,18 +4940,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B48" s="262" t="inlineStr"/>
-      <c r="C48" s="262" t="inlineStr">
+      <c r="B48" s="276" t="inlineStr"/>
+      <c r="C48" s="276" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="D48" s="262" t="inlineStr">
+      <c r="D48" s="276" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E48" s="262" t="inlineStr"/>
+      <c r="E48" s="276" t="inlineStr"/>
       <c r="F48" s="99" t="inlineStr">
         <is>
           <t>Week Oct 6-9: Midterm &amp; Break (lecture topics)</t>
@@ -4915,18 +4964,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B49" s="262" t="inlineStr"/>
-      <c r="C49" s="262" t="inlineStr">
+      <c r="B49" s="276" t="inlineStr"/>
+      <c r="C49" s="276" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="D49" s="262" t="inlineStr">
+      <c r="D49" s="276" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="E49" s="262" t="inlineStr"/>
+      <c r="E49" s="276" t="inlineStr"/>
       <c r="F49" s="99" t="inlineStr">
         <is>
           <t>Week Oct 13-16: The Reformation (lecture topics)</t>
@@ -4939,18 +4988,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B50" s="262" t="inlineStr"/>
-      <c r="C50" s="262" t="inlineStr">
+      <c r="B50" s="276" t="inlineStr"/>
+      <c r="C50" s="276" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="D50" s="262" t="inlineStr">
+      <c r="D50" s="276" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="E50" s="262" t="inlineStr"/>
+      <c r="E50" s="276" t="inlineStr"/>
       <c r="F50" s="99" t="inlineStr">
         <is>
           <t>Week Oct 20-23: The Reformation (lecture topics)</t>
@@ -4963,18 +5012,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B51" s="262" t="inlineStr"/>
-      <c r="C51" s="262" t="inlineStr">
+      <c r="B51" s="276" t="inlineStr"/>
+      <c r="C51" s="276" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D51" s="262" t="inlineStr">
+      <c r="D51" s="276" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E51" s="262" t="inlineStr"/>
+      <c r="E51" s="276" t="inlineStr"/>
       <c r="F51" s="99" t="inlineStr">
         <is>
           <t>Week Oct 27-30: Reformation (lecture topics)</t>
@@ -4987,18 +5036,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B52" s="262" t="inlineStr"/>
-      <c r="C52" s="262" t="inlineStr">
+      <c r="B52" s="276" t="inlineStr"/>
+      <c r="C52" s="276" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D52" s="262" t="inlineStr">
+      <c r="D52" s="276" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E52" s="262" t="inlineStr"/>
+      <c r="E52" s="276" t="inlineStr"/>
       <c r="F52" s="99" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science (lecture topics)</t>
@@ -5011,18 +5060,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B53" s="262" t="inlineStr"/>
-      <c r="C53" s="262" t="inlineStr">
+      <c r="B53" s="276" t="inlineStr"/>
+      <c r="C53" s="276" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D53" s="262" t="inlineStr">
+      <c r="D53" s="276" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E53" s="262" t="inlineStr"/>
+      <c r="E53" s="276" t="inlineStr"/>
       <c r="F53" s="99" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment (lecture topics)</t>
@@ -5035,18 +5084,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B54" s="262" t="inlineStr"/>
-      <c r="C54" s="262" t="inlineStr">
+      <c r="B54" s="276" t="inlineStr"/>
+      <c r="C54" s="276" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D54" s="262" t="inlineStr">
+      <c r="D54" s="276" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E54" s="262" t="inlineStr"/>
+      <c r="E54" s="276" t="inlineStr"/>
       <c r="F54" s="99" t="inlineStr">
         <is>
           <t>Week Nov 17-20: Enlightenment (lecture topics)</t>
@@ -5059,18 +5108,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B55" s="262" t="inlineStr"/>
-      <c r="C55" s="262" t="inlineStr">
+      <c r="B55" s="276" t="inlineStr"/>
+      <c r="C55" s="276" t="inlineStr">
         <is>
           <t>2026-12-01</t>
         </is>
       </c>
-      <c r="D55" s="262" t="inlineStr">
+      <c r="D55" s="276" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E55" s="262" t="inlineStr"/>
+      <c r="E55" s="276" t="inlineStr"/>
       <c r="F55" s="99" t="inlineStr">
         <is>
           <t>Week Dec 1-4: Modern Europe? (lecture topics)</t>
@@ -5083,18 +5132,18 @@
           <t>Extra Credit</t>
         </is>
       </c>
-      <c r="B56" s="260" t="inlineStr">
+      <c r="B56" s="274" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C56" s="261" t="inlineStr"/>
-      <c r="D56" s="261" t="inlineStr">
+      <c r="C56" s="275" t="inlineStr"/>
+      <c r="D56" s="275" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E56" s="261" t="inlineStr">
+      <c r="E56" s="275" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Fix Overview scroll freeze and expand RMP consensus detail
- Remove freeze_panes on Overview so professor stats no longer lock the sheet
- Split RMP into compact stats table plus full consensus paragraphs below
- Expand rmp.json consensus with STRENGTHS / workload / bottom-line themes

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -9,8 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-304" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-281" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-281" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -345,7 +345,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -630,6 +630,22 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -998,12 +1014,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
@@ -1073,11 +1089,6 @@
           <t># Ratings</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Consensus</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="7">
@@ -1109,11 +1120,6 @@
           <t>255</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>Warm, funny, and supportive outside class; strong career advice. Lectures and exams are polarizing—some find exams misal</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="10">
@@ -1145,11 +1151,6 @@
           <t>50</t>
         </is>
       </c>
-      <c r="G7" s="11" t="inlineStr">
-        <is>
-          <t>Highly supportive and organized; standout Marshall teacher (negotiations, OB). Caring environment with group work and ge</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="7">
@@ -1181,858 +1182,921 @@
           <t>53</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>Passionate, engaging lectures (multimedia, humor); discussion- and reading-heavy. Mixed on grading strictness; occasiona</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="91" t="inlineStr">
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Consensus - recurring student review themes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="135" customHeight="1">
+      <c r="A11" s="104" t="inlineStr">
+        <is>
+          <t>BUAD-281</t>
+        </is>
+      </c>
+      <c r="B11" s="105" t="inlineStr">
+        <is>
+          <t>George Braunegg</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>STRENGTHS: Very high marks for personality and support — students call Prof. Braunegg kind, funny, caring, and responsive by email. Daily accounting facts/jokes are a recurring positive. Many praise his career advice and willingness to help outside class; several credit him with influencing their major choice.
+TEACHING &amp; EXAMS: More divided on in-class instruction — some say he struggles to work through problems live or that lectures don't always align with exams. Course draws on Prof. Layton's materials but sections may not match perfectly. Textbook gets criticism.
+BOTTOM LINE: Strong human connection and mentorship; be prepared to self-study or use tutors if lecture pace doesn't click. High would-take-again despite polarized exam/lecture comments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="135" customHeight="1">
+      <c r="A12" s="106" t="inlineStr">
+        <is>
+          <t>BUAD-304</t>
+        </is>
+      </c>
+      <c r="B12" s="107" t="inlineStr">
+        <is>
+          <t>Christine El Haddad</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>STRENGTHS: Among the most praised Marshall professors on RMP — repeatedly called the 'best' or 'sweetest' instructor students have had. Negotiation and OB classes get standout reviews: supportive classroom culture, clear and organized Brightspace, strong lectures, and generous extra credit. Weekly in-class negotiations are a highlight for many.
+WORKLOAD: Group projects and class participation carry real weight; some find readings or lecture content repetitive. A few note group work can feel heavy even when the professor is beloved.
+BOTTOM LINE: Take her if you can — especially for negotiation-heavy offerings. Show up, participate, and lean into the structured group work; exams reward attentive note-taking on lecture and slide content.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="135" customHeight="1">
+      <c r="A13" s="104" t="inlineStr">
+        <is>
+          <t>HIST-103</t>
+        </is>
+      </c>
+      <c r="B13" s="105" t="inlineStr">
+        <is>
+          <t>Lindsay O'Neill</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>STRENGTHS: Students consistently describe Dr. O'Neill as passionate and engaging — lectures use multimedia (Monty Python clips, movie trailers, humor) that make a GE history class feel lively rather than dry. Many say the content is genuinely interesting if you show up and pay attention.
+GRADING &amp; WORKLOAD: Mixed reviews on grading — several note she can be a harsh essay grader and that strong discussion participation matters. Expect substantial section readings; essays benefit from office-hours or TA help. Low-weight pop quizzes (~5% total) sometimes used to track attendance.
+BOTTOM LINE: Solid pick for students who engage in class and discussion; less ideal if you want a low-effort GE or struggle with writing-heavy assessments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="91" t="inlineStr">
         <is>
           <t>RMP data as of 2026-08-21. Source: ratemyprofessors.com</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Connect prep (e.g. BUAD-304 Personal Assessments) is ungraded class prep - not part of Participation or other graded categories.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Start here (graded): 2026-09-09 - BUAD-281 - Homework: Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Reading</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>Papers</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>Group Project</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>External certs</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>Connect prep</t>
         </is>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>First assignment</t>
         </is>
       </c>
-      <c r="I14" s="6" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>Assign due</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr">
+      <c r="J19" s="6" t="inlineStr">
         <is>
           <t>First major</t>
         </is>
       </c>
-      <c r="K14" s="6" t="inlineStr">
+      <c r="K19" s="6" t="inlineStr">
         <is>
           <t>Major due</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="7">
+    <row r="20">
+      <c r="A20" s="7">
         <f>HYPERLINK("#'BUAD-281'!A1","BUAD-281")</f>
         <v/>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="F20" s="9" t="inlineStr">
         <is>
           <t>LinkedIn Learning Excel Certification, Stukent Simternship</t>
         </is>
       </c>
-      <c r="G15" s="8" t="inlineStr">
+      <c r="G20" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H15" s="8" t="inlineStr">
+      <c r="H20" s="8" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
         </is>
       </c>
-      <c r="I15" s="8" t="inlineStr">
+      <c r="I20" s="8" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="J15" s="8" t="inlineStr">
+      <c r="J20" s="8" t="inlineStr">
         <is>
           <t>Midterm 1</t>
         </is>
       </c>
-      <c r="K15" s="8" t="inlineStr">
+      <c r="K20" s="8" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="10">
+    <row r="21">
+      <c r="A21" s="10">
         <f>HYPERLINK("#'BUAD-304'!A1","BUAD-304")</f>
         <v/>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>Final Reflection Paper, Team Project Paper</t>
         </is>
       </c>
-      <c r="E16" s="11" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F16" s="11" t="inlineStr">
+      <c r="F21" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G16" s="12" t="inlineStr">
+      <c r="G21" s="12" t="inlineStr">
         <is>
           <t>Ungraded prep</t>
         </is>
       </c>
-      <c r="H16" s="11" t="inlineStr">
+      <c r="H21" s="11" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.01 - What is my Big thinking</t>
         </is>
       </c>
-      <c r="I16" s="11" t="inlineStr">
+      <c r="I21" s="11" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="J16" s="11" t="inlineStr">
+      <c r="J21" s="11" t="inlineStr">
         <is>
           <t>Thomas Green Case Analysis Memo</t>
         </is>
       </c>
-      <c r="K16" s="11" t="inlineStr">
+      <c r="K21" s="11" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="7">
+    <row r="22">
+      <c r="A22" s="7">
         <f>HYPERLINK("#'HIST-103'!A1","HIST-103")</f>
         <v/>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>Sleep Paper, Witchcraft Paper</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="F22" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="8" t="inlineStr">
+      <c r="G22" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H17" s="8" t="inlineStr">
+      <c r="H22" s="8" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
         </is>
       </c>
-      <c r="I17" s="8" t="inlineStr">
+      <c r="I22" s="8" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="J17" s="8" t="inlineStr">
+      <c r="J22" s="8" t="inlineStr">
         <is>
           <t>Sleep Paper</t>
         </is>
       </c>
-      <c r="K17" s="8" t="inlineStr">
+      <c r="K22" s="8" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>Do First - August 2026 - graded assignments (first per class always listed)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="B20" s="14" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="C20" s="14" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr">
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>Graded?</t>
         </is>
       </c>
-      <c r="E20" s="14" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="C26" s="15" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="D26" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="E26" s="8" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>HIST-103</t>
         </is>
       </c>
-      <c r="C22" s="16" t="inlineStr">
+      <c r="C27" s="16" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D22" s="11" t="inlineStr">
+      <c r="D27" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E22" s="11" t="inlineStr">
+      <c r="E27" s="11" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="17" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>Do First - August 2026 - Connect prep only (ungraded, not Participation)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="18" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="18" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="B25" s="18" t="inlineStr">
+      <c r="B30" s="18" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="C25" s="18" t="inlineStr">
+      <c r="C30" s="18" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D25" s="18" t="inlineStr">
+      <c r="D30" s="18" t="inlineStr">
         <is>
           <t>Graded?</t>
         </is>
       </c>
-      <c r="E25" s="18" t="inlineStr">
+      <c r="E30" s="18" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="19" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="19" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B26" s="19" t="inlineStr">
+      <c r="B31" s="19" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C26" s="20" t="inlineStr">
+      <c r="C31" s="20" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D26" s="21" t="inlineStr">
+      <c r="D31" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E26" s="19" t="inlineStr">
+      <c r="E31" s="19" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="22" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="22" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B27" s="22" t="inlineStr">
+      <c r="B32" s="22" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C27" s="23" t="inlineStr">
+      <c r="C32" s="23" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D27" s="24" t="inlineStr">
+      <c r="D32" s="24" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E27" s="22" t="inlineStr">
+      <c r="E32" s="22" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="13" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
         <is>
           <t>Upcoming graded assignments (next 45 days)</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="14" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="B30" s="14" t="inlineStr">
+      <c r="B35" s="14" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="C30" s="14" t="inlineStr">
+      <c r="C35" s="14" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D30" s="14" t="inlineStr">
+      <c r="D35" s="14" t="inlineStr">
         <is>
           <t>Graded?</t>
         </is>
       </c>
-      <c r="E30" s="14" t="inlineStr">
+      <c r="E35" s="14" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="B31" s="8" t="inlineStr">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C31" s="15" t="inlineStr">
+      <c r="C36" s="15" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D31" s="8" t="inlineStr">
+      <c r="D36" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E31" s="8" t="inlineStr">
+      <c r="E36" s="8" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="11" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="B32" s="11" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
         <is>
           <t>HIST-103</t>
         </is>
       </c>
-      <c r="C32" s="16" t="inlineStr">
+      <c r="C37" s="16" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D32" s="11" t="inlineStr">
+      <c r="D37" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E32" s="11" t="inlineStr">
+      <c r="E37" s="11" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B38" s="8" t="inlineStr">
         <is>
           <t>HIST-103</t>
         </is>
       </c>
-      <c r="C33" s="25" t="inlineStr">
+      <c r="C38" s="25" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D33" s="8" t="inlineStr">
+      <c r="D38" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E33" s="8" t="inlineStr">
+      <c r="E38" s="8" t="inlineStr">
         <is>
           <t>Sleep Paper</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="11" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="B34" s="11" t="inlineStr">
+      <c r="B39" s="11" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C34" s="46" t="inlineStr">
+      <c r="C39" s="46" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D34" s="11" t="inlineStr">
+      <c r="D39" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E34" s="11" t="inlineStr">
+      <c r="E39" s="11" t="inlineStr">
         <is>
           <t>Class 7 (9/16) - 3-24, 3-28, 3-32; 15 Points</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B40" s="8" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C35" s="25" t="inlineStr">
+      <c r="C40" s="25" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D35" s="8" t="inlineStr">
+      <c r="D40" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E35" s="8" t="inlineStr">
+      <c r="E40" s="8" t="inlineStr">
         <is>
           <t>Thomas Green Case Analysis Memo</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="11" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="B36" s="11" t="inlineStr">
+      <c r="B41" s="11" t="inlineStr">
         <is>
           <t>HIST-103</t>
         </is>
       </c>
-      <c r="C36" s="16" t="inlineStr">
+      <c r="C41" s="16" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D36" s="11" t="inlineStr">
+      <c r="D41" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E36" s="11" t="inlineStr">
+      <c r="E41" s="11" t="inlineStr">
         <is>
           <t>Final Exam</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="B37" s="8" t="inlineStr">
+      <c r="B42" s="8" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C37" s="15" t="inlineStr">
+      <c r="C42" s="15" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D37" s="8" t="inlineStr">
+      <c r="D42" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E37" s="8" t="inlineStr">
+      <c r="E42" s="8" t="inlineStr">
         <is>
           <t>Class 8 (9/21) - 5-27 5-46; 10 Points</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="11" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="11" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="B38" s="11" t="inlineStr">
+      <c r="B43" s="11" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C38" s="46" t="inlineStr">
+      <c r="C43" s="46" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D38" s="11" t="inlineStr">
+      <c r="D43" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E38" s="11" t="inlineStr">
+      <c r="E43" s="11" t="inlineStr">
         <is>
           <t>Class 9 (9/23) - 4-21, 4-22; 10 Points</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="B39" s="8" t="inlineStr">
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C39" s="26" t="inlineStr">
+      <c r="C44" s="26" t="inlineStr">
         <is>
           <t>Research</t>
         </is>
       </c>
-      <c r="D39" s="8" t="inlineStr">
+      <c r="D44" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E39" s="8" t="inlineStr">
+      <c r="E44" s="8" t="inlineStr">
         <is>
           <t>Research: Setup deadline (registration, prescreening, contacts)</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="11" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="11" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="B40" s="11" t="inlineStr">
+      <c r="B45" s="11" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C40" s="46" t="inlineStr">
+      <c r="C45" s="46" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D40" s="11" t="inlineStr">
+      <c r="D45" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E40" s="11" t="inlineStr">
+      <c r="E45" s="11" t="inlineStr">
         <is>
           <t>Class 10 (9/28) - 8-28, 8-29; 10 Points</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="B41" s="8" t="inlineStr">
+      <c r="B46" s="8" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C41" s="25" t="inlineStr">
+      <c r="C46" s="25" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D41" s="8" t="inlineStr">
+      <c r="D46" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E41" s="8" t="inlineStr">
+      <c r="E46" s="8" t="inlineStr">
         <is>
           <t>Team project proposal &amp; team contract</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="11" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="11" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="B42" s="11" t="inlineStr">
+      <c r="B47" s="11" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C42" s="16" t="inlineStr">
+      <c r="C47" s="16" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D42" s="11" t="inlineStr">
+      <c r="D47" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E42" s="11" t="inlineStr">
+      <c r="E47" s="11" t="inlineStr">
         <is>
           <t>Proposal &amp; Team Contract</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B43" s="8" t="inlineStr">
+      <c r="B48" s="8" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C43" s="47" t="inlineStr">
+      <c r="C48" s="47" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="D43" s="8" t="inlineStr">
+      <c r="D48" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E43" s="8" t="inlineStr">
+      <c r="E48" s="8" t="inlineStr">
         <is>
           <t>9/30 Midterm 1: 250 Points Chapters 1, 2, 3, 4, 5, 8</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="11" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="11" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B44" s="11" t="inlineStr">
+      <c r="B49" s="11" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C44" s="16" t="inlineStr">
+      <c r="C49" s="16" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D44" s="11" t="inlineStr">
+      <c r="D49" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E44" s="11" t="inlineStr">
+      <c r="E49" s="11" t="inlineStr">
         <is>
           <t>Midterm 1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A12:K12"/>
+  <mergeCells count="14">
+    <mergeCell ref="A34:K34"/>
     <mergeCell ref="A4:K4"/>
+    <mergeCell ref="C11:K11"/>
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A29:K29"/>
+    <mergeCell ref="C13:K13"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A16:K16"/>
+    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="A10:K10"/>
     <mergeCell ref="A24:K24"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A11:K11"/>
-    <mergeCell ref="A19:K19"/>
+    <mergeCell ref="A14:K14"/>
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A9:K9"/>
+    <mergeCell ref="C12:K12"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId1"/>
@@ -3146,6 +3210,958 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FF7F0E"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="48" t="inlineStr">
+        <is>
+          <t>BUAD-281 — Managerial Accounting</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="28">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/sources/buad-281-source.pdf","SEE HERE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="29" t="inlineStr">
+        <is>
+          <t>Instructor</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>George Braunegg</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fall 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>Required for an A</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>Grading scale</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Total graded points in calendar: 1070 (letter scale not in document)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="49" t="inlineStr">
+        <is>
+          <t>Midterm 1 250 pts  |  Midterm 2 250 pts  |  Final Exam 250 pts  |  Homework 170 pts  |  LinkedIn Learning Excel Certification 75 pts  |  Stukent Simternship 75 pts</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="B8" s="50" t="inlineStr">
+        <is>
+          <t>If your AI tool breaks down and solves the homework bank problems - extracting step-by-step mechanics from the textbook - mastering those exact mechanics is all you need to get an A without reading prose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="51" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B10" s="51" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="C10" s="51" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="D10" s="51" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="E10" s="51" t="inlineStr">
+        <is>
+          <t>Group Project</t>
+        </is>
+      </c>
+      <c r="F10" s="51" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="52" t="inlineStr">
+        <is>
+          <t>Midterm 1</t>
+        </is>
+      </c>
+      <c r="B11" s="100" t="inlineStr">
+        <is>
+          <t>250 pts</t>
+        </is>
+      </c>
+      <c r="C11" s="101" t="inlineStr"/>
+      <c r="D11" s="101" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E11" s="101" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" s="55">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-midterm-1.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="56" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="B12" s="102" t="inlineStr"/>
+      <c r="C12" s="102" t="inlineStr"/>
+      <c r="D12" s="102" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E12" s="102" t="inlineStr"/>
+      <c r="F12" s="58" t="inlineStr">
+        <is>
+          <t>9/30 Midterm 1: 250 Points Chapters 1, 2, 3, 4, 5, 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="59" t="inlineStr">
+        <is>
+          <t>Midterm 2</t>
+        </is>
+      </c>
+      <c r="B13" s="100" t="inlineStr">
+        <is>
+          <t>250 pts</t>
+        </is>
+      </c>
+      <c r="C13" s="103" t="inlineStr"/>
+      <c r="D13" s="103" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="E13" s="103" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" s="61">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-midterm-2.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="56" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="B14" s="102" t="inlineStr"/>
+      <c r="C14" s="102" t="inlineStr"/>
+      <c r="D14" s="102" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="E14" s="102" t="inlineStr"/>
+      <c r="F14" s="58" t="inlineStr">
+        <is>
+          <t>10/26 Midterm 2: 250 Points Chapters 6, 7, 9, &amp; 16</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="52" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+      <c r="B15" s="100" t="inlineStr">
+        <is>
+          <t>250 pts</t>
+        </is>
+      </c>
+      <c r="C15" s="101" t="inlineStr"/>
+      <c r="D15" s="101" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="E15" s="101" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F15" s="55">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-final-exam.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="56" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="B16" s="102" t="inlineStr"/>
+      <c r="C16" s="102" t="inlineStr"/>
+      <c r="D16" s="102" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="E16" s="102" t="inlineStr"/>
+      <c r="F16" s="58" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="59" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B17" s="100" t="inlineStr">
+        <is>
+          <t>170 pts</t>
+        </is>
+      </c>
+      <c r="C17" s="103" t="inlineStr"/>
+      <c r="D17" s="103" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E17" s="103" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F17" s="61">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-homework.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="62" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B18" s="102" t="inlineStr"/>
+      <c r="C18" s="102" t="inlineStr"/>
+      <c r="D18" s="102" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="E18" s="102" t="inlineStr"/>
+      <c r="F18" s="58" t="inlineStr">
+        <is>
+          <t>Class 5 (9/9) - Product Cost Accumulation: Job; Order Co: Chapter 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="63" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B19" s="102" t="inlineStr"/>
+      <c r="C19" s="102" t="inlineStr"/>
+      <c r="D19" s="102" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="E19" s="102" t="inlineStr"/>
+      <c r="F19" s="58" t="inlineStr">
+        <is>
+          <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="62" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B20" s="102" t="inlineStr"/>
+      <c r="C20" s="102" t="inlineStr"/>
+      <c r="D20" s="102" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E20" s="102" t="inlineStr"/>
+      <c r="F20" s="58" t="inlineStr">
+        <is>
+          <t>Class 7 (9/16) - Activity Based Costing: Chapter 5- ONLY; LO 5.1, 2, 4 &amp; 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="63" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B21" s="102" t="inlineStr"/>
+      <c r="C21" s="102" t="inlineStr"/>
+      <c r="D21" s="102" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E21" s="102" t="inlineStr"/>
+      <c r="F21" s="58" t="inlineStr">
+        <is>
+          <t>Class 7 (9/16) - 3-24, 3-28, 3-32; 15 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="62" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B22" s="102" t="inlineStr"/>
+      <c r="C22" s="102" t="inlineStr"/>
+      <c r="D22" s="102" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E22" s="102" t="inlineStr"/>
+      <c r="F22" s="58" t="inlineStr">
+        <is>
+          <t>Class 8 (9/21) - Product Cost Accumulation: Pro-; cess Co: Chapter 4- ONLY; LO 4.1, 3, 4, &amp; 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="63" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B23" s="102" t="inlineStr"/>
+      <c r="C23" s="102" t="inlineStr"/>
+      <c r="D23" s="102" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="E23" s="102" t="inlineStr"/>
+      <c r="F23" s="58" t="inlineStr">
+        <is>
+          <t>Class 8 (9/21) - 5-27 5-46; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="62" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B24" s="102" t="inlineStr"/>
+      <c r="C24" s="102" t="inlineStr"/>
+      <c r="D24" s="102" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E24" s="102" t="inlineStr"/>
+      <c r="F24" s="58" t="inlineStr">
+        <is>
+          <t>Class 9 (9/23) - Cost of Quality &amp; ESG &amp;; Overview of; • : Chapter 8 - ONLY; LO 8.7, 8, 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="63" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B25" s="102" t="inlineStr"/>
+      <c r="C25" s="102" t="inlineStr"/>
+      <c r="D25" s="102" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E25" s="102" t="inlineStr"/>
+      <c r="F25" s="58" t="inlineStr">
+        <is>
+          <t>Class 9 (9/23) - 4-21, 4-22; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="62" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B26" s="102" t="inlineStr"/>
+      <c r="C26" s="102" t="inlineStr"/>
+      <c r="D26" s="102" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E26" s="102" t="inlineStr"/>
+      <c r="F26" s="58" t="inlineStr">
+        <is>
+          <t>Class 10 (9/28) - Catchup &amp; Midterm Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="63" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B27" s="102" t="inlineStr"/>
+      <c r="C27" s="102" t="inlineStr"/>
+      <c r="D27" s="102" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E27" s="102" t="inlineStr"/>
+      <c r="F27" s="58" t="inlineStr">
+        <is>
+          <t>Class 10 (9/28) - 8-28, 8-29; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="62" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B28" s="102" t="inlineStr"/>
+      <c r="C28" s="102" t="inlineStr"/>
+      <c r="D28" s="102" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E28" s="102" t="inlineStr"/>
+      <c r="F28" s="58" t="inlineStr">
+        <is>
+          <t>Class 12 (10/7) - Cost volume profit analysis: Chapter 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="63" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B29" s="102" t="inlineStr"/>
+      <c r="C29" s="102" t="inlineStr"/>
+      <c r="D29" s="102" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="E29" s="102" t="inlineStr"/>
+      <c r="F29" s="58" t="inlineStr">
+        <is>
+          <t>Class 12 (10/7) - 6-24, 6-25, 6-34; 15 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="62" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B30" s="102" t="inlineStr"/>
+      <c r="C30" s="102" t="inlineStr"/>
+      <c r="D30" s="102" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E30" s="102" t="inlineStr"/>
+      <c r="F30" s="58" t="inlineStr">
+        <is>
+          <t>Class 14 (10/14) - Financial planning and analysis:; Static: Chapter 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="63" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B31" s="102" t="inlineStr"/>
+      <c r="C31" s="102" t="inlineStr"/>
+      <c r="D31" s="102" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E31" s="102" t="inlineStr"/>
+      <c r="F31" s="58" t="inlineStr">
+        <is>
+          <t>Class 14 (10/14) - 7-29, 7-33, 7-40; 15 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="62" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B32" s="102" t="inlineStr"/>
+      <c r="C32" s="102" t="inlineStr"/>
+      <c r="D32" s="102" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E32" s="102" t="inlineStr"/>
+      <c r="F32" s="58" t="inlineStr">
+        <is>
+          <t>Class 15 (10/19) - Capital Budgeting; Practice Midterm Ques: Chapter 16- ONLY; LO 16.1, 2, 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="63" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B33" s="102" t="inlineStr"/>
+      <c r="C33" s="102" t="inlineStr"/>
+      <c r="D33" s="102" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E33" s="102" t="inlineStr"/>
+      <c r="F33" s="58" t="inlineStr">
+        <is>
+          <t>Class 15 (10/19) - 9-25, 9-28, 9-37; 15 - Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="62" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B34" s="102" t="inlineStr"/>
+      <c r="C34" s="102" t="inlineStr"/>
+      <c r="D34" s="102" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E34" s="102" t="inlineStr"/>
+      <c r="F34" s="58" t="inlineStr">
+        <is>
+          <t>Class 16 (10/21) - Catchup &amp; Midterm Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="63" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B35" s="102" t="inlineStr"/>
+      <c r="C35" s="102" t="inlineStr"/>
+      <c r="D35" s="102" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E35" s="102" t="inlineStr"/>
+      <c r="F35" s="58" t="inlineStr">
+        <is>
+          <t>Class 16 (10/21) - 16-28, 16-40; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="62" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B36" s="102" t="inlineStr"/>
+      <c r="C36" s="102" t="inlineStr"/>
+      <c r="D36" s="102" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="E36" s="102" t="inlineStr"/>
+      <c r="F36" s="58" t="inlineStr">
+        <is>
+          <t>Class 19 (11/4) - Sales Variance Analysis; Flexible Budget: Chapter 11 - ONLY; LO 11.1, 11.2 &amp;; Appendix B</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="63" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B37" s="102" t="inlineStr"/>
+      <c r="C37" s="102" t="inlineStr"/>
+      <c r="D37" s="102" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="E37" s="102" t="inlineStr"/>
+      <c r="F37" s="58" t="inlineStr">
+        <is>
+          <t>Class 19 (11/4) - 10-26, 10-30; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="62" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B38" s="102" t="inlineStr"/>
+      <c r="C38" s="102" t="inlineStr"/>
+      <c r="D38" s="102" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E38" s="102" t="inlineStr"/>
+      <c r="F38" s="58" t="inlineStr">
+        <is>
+          <t>Class 20 (11/9) - Investment Centers: Chapter 13- ONLY; LO 13-1, 2, 3, 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="63" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B39" s="102" t="inlineStr"/>
+      <c r="C39" s="102" t="inlineStr"/>
+      <c r="D39" s="102" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E39" s="102" t="inlineStr"/>
+      <c r="F39" s="58" t="inlineStr">
+        <is>
+          <t>Class 20 (11/9) - 11-31, 11-52; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="62" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B40" s="102" t="inlineStr"/>
+      <c r="C40" s="102" t="inlineStr"/>
+      <c r="D40" s="102" t="inlineStr">
+        <is>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="E40" s="102" t="inlineStr"/>
+      <c r="F40" s="58" t="inlineStr">
+        <is>
+          <t>Class 21 (11/16) - AI &amp; FP&amp;A</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="63" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B41" s="102" t="inlineStr"/>
+      <c r="C41" s="102" t="inlineStr"/>
+      <c r="D41" s="102" t="inlineStr">
+        <is>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="E41" s="102" t="inlineStr"/>
+      <c r="F41" s="58" t="inlineStr">
+        <is>
+          <t>Class 21 (11/16) - 13-29, 13-33; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="62" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B42" s="102" t="inlineStr"/>
+      <c r="C42" s="102" t="inlineStr"/>
+      <c r="D42" s="102" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E42" s="102" t="inlineStr"/>
+      <c r="F42" s="58" t="inlineStr">
+        <is>
+          <t>Class 2 (12/2) - Catchup &amp; Final Review; Practice Final Questions Posted to Brightspace at; 5:00 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="63" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B43" s="102" t="inlineStr"/>
+      <c r="C43" s="102" t="inlineStr"/>
+      <c r="D43" s="102" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E43" s="102" t="inlineStr"/>
+      <c r="F43" s="58" t="inlineStr">
+        <is>
+          <t>Class 2 (12/2) - 14-35, 14-41; 10 Points; Assignments listed Be-; low Due by11:59 PM; Linked In Learning; E</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="52" t="inlineStr">
+        <is>
+          <t>LinkedIn Learning Excel Certification</t>
+        </is>
+      </c>
+      <c r="B44" s="100" t="inlineStr">
+        <is>
+          <t>75 pts</t>
+        </is>
+      </c>
+      <c r="C44" s="101" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D44" s="101" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E44" s="101" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F44" s="55">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-linkedin-learning-excel-certification.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="64" t="inlineStr">
+        <is>
+          <t>Certification</t>
+        </is>
+      </c>
+      <c r="B45" s="102" t="inlineStr"/>
+      <c r="C45" s="102" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D45" s="102" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E45" s="102" t="inlineStr"/>
+      <c r="F45" s="58" t="inlineStr">
+        <is>
+          <t>LinkedIn Learning Excel Certification</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="59" t="inlineStr">
+        <is>
+          <t>Stukent Simternship</t>
+        </is>
+      </c>
+      <c r="B46" s="100" t="inlineStr">
+        <is>
+          <t>75 pts</t>
+        </is>
+      </c>
+      <c r="C46" s="103" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D46" s="103" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E46" s="103" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F46" s="61">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-stukent-simternship.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="64" t="inlineStr">
+        <is>
+          <t>Certification</t>
+        </is>
+      </c>
+      <c r="B47" s="102" t="inlineStr"/>
+      <c r="C47" s="102" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="D47" s="102" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E47" s="102" t="inlineStr"/>
+      <c r="F47" s="58" t="inlineStr">
+        <is>
+          <t>Stukent Simternship</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="29" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B48" s="65" t="inlineStr">
+        <is>
+          <t>1070 pts</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="A7:F7"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00D62728"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -3267,18 +4283,18 @@
           <t>Sleep Paper</t>
         </is>
       </c>
-      <c r="B10" s="96" t="inlineStr">
+      <c r="B10" s="108" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C10" s="97" t="inlineStr"/>
-      <c r="D10" s="97" t="inlineStr">
+      <c r="C10" s="109" t="inlineStr"/>
+      <c r="D10" s="109" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="E10" s="97" t="inlineStr">
+      <c r="E10" s="109" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3294,14 +4310,14 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B11" s="98" t="inlineStr"/>
-      <c r="C11" s="98" t="inlineStr"/>
-      <c r="D11" s="98" t="inlineStr">
+      <c r="B11" s="110" t="inlineStr"/>
+      <c r="C11" s="110" t="inlineStr"/>
+      <c r="D11" s="110" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="E11" s="98" t="inlineStr"/>
+      <c r="E11" s="110" t="inlineStr"/>
       <c r="F11" s="39" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
@@ -3314,18 +4330,18 @@
           <t>Witchcraft Paper</t>
         </is>
       </c>
-      <c r="B12" s="96" t="inlineStr">
+      <c r="B12" s="108" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C12" s="99" t="inlineStr"/>
-      <c r="D12" s="99" t="inlineStr">
+      <c r="C12" s="111" t="inlineStr"/>
+      <c r="D12" s="111" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="E12" s="99" t="inlineStr">
+      <c r="E12" s="111" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3341,14 +4357,14 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B13" s="98" t="inlineStr"/>
-      <c r="C13" s="98" t="inlineStr"/>
-      <c r="D13" s="98" t="inlineStr">
+      <c r="B13" s="110" t="inlineStr"/>
+      <c r="C13" s="110" t="inlineStr"/>
+      <c r="D13" s="110" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="E13" s="98" t="inlineStr"/>
+      <c r="E13" s="110" t="inlineStr"/>
       <c r="F13" s="39" t="inlineStr">
         <is>
           <t>Witchcraft Paper Due</t>
@@ -3361,18 +4377,18 @@
           <t>Mid-term</t>
         </is>
       </c>
-      <c r="B14" s="96" t="inlineStr">
+      <c r="B14" s="108" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C14" s="97" t="inlineStr"/>
-      <c r="D14" s="97" t="inlineStr">
+      <c r="C14" s="109" t="inlineStr"/>
+      <c r="D14" s="109" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E14" s="97" t="inlineStr">
+      <c r="E14" s="109" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3388,14 +4404,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B15" s="98" t="inlineStr"/>
-      <c r="C15" s="98" t="inlineStr"/>
-      <c r="D15" s="98" t="inlineStr">
+      <c r="B15" s="110" t="inlineStr"/>
+      <c r="C15" s="110" t="inlineStr"/>
+      <c r="D15" s="110" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="E15" s="98" t="inlineStr"/>
+      <c r="E15" s="110" t="inlineStr"/>
       <c r="F15" s="39" t="inlineStr">
         <is>
           <t>Midterm Exam</t>
@@ -3408,18 +4424,18 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B16" s="96" t="inlineStr">
+      <c r="B16" s="108" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C16" s="99" t="inlineStr"/>
-      <c r="D16" s="99" t="inlineStr">
+      <c r="C16" s="111" t="inlineStr"/>
+      <c r="D16" s="111" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="E16" s="99" t="inlineStr">
+      <c r="E16" s="111" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -3435,14 +4451,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B17" s="98" t="inlineStr"/>
-      <c r="C17" s="98" t="inlineStr"/>
-      <c r="D17" s="98" t="inlineStr">
+      <c r="B17" s="110" t="inlineStr"/>
+      <c r="C17" s="110" t="inlineStr"/>
+      <c r="D17" s="110" t="inlineStr">
         <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="E17" s="98" t="inlineStr"/>
+      <c r="E17" s="110" t="inlineStr"/>
       <c r="F17" s="39" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -3455,18 +4471,18 @@
           <t>Discussion Section</t>
         </is>
       </c>
-      <c r="B18" s="96" t="inlineStr">
+      <c r="B18" s="108" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C18" s="97" t="inlineStr"/>
-      <c r="D18" s="97" t="inlineStr">
+      <c r="C18" s="109" t="inlineStr"/>
+      <c r="D18" s="109" t="inlineStr">
         <is>
           <t>2026-11-12</t>
         </is>
       </c>
-      <c r="E18" s="97" t="inlineStr">
+      <c r="E18" s="109" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -3482,18 +4498,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B19" s="98" t="inlineStr"/>
-      <c r="C19" s="98" t="inlineStr">
+      <c r="B19" s="110" t="inlineStr"/>
+      <c r="C19" s="110" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D19" s="98" t="inlineStr">
+      <c r="D19" s="110" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E19" s="98" t="inlineStr"/>
+      <c r="E19" s="110" t="inlineStr"/>
       <c r="F19" s="39" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death</t>
@@ -3506,18 +4522,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B20" s="98" t="inlineStr"/>
-      <c r="C20" s="98" t="inlineStr">
+      <c r="B20" s="110" t="inlineStr"/>
+      <c r="C20" s="110" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D20" s="98" t="inlineStr">
+      <c r="D20" s="110" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E20" s="98" t="inlineStr"/>
+      <c r="E20" s="110" t="inlineStr"/>
       <c r="F20" s="39" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death - Section reading 1: Lizzie Wade, “From Black Death to fatal flu, past pandemics sho</t>
@@ -3530,18 +4546,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B21" s="98" t="inlineStr"/>
-      <c r="C21" s="98" t="inlineStr">
+      <c r="B21" s="110" t="inlineStr"/>
+      <c r="C21" s="110" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D21" s="98" t="inlineStr">
+      <c r="D21" s="110" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E21" s="98" t="inlineStr"/>
+      <c r="E21" s="110" t="inlineStr"/>
       <c r="F21" s="39" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life</t>
@@ -3554,18 +4570,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B22" s="98" t="inlineStr"/>
-      <c r="C22" s="98" t="inlineStr">
+      <c r="B22" s="110" t="inlineStr"/>
+      <c r="C22" s="110" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D22" s="98" t="inlineStr">
+      <c r="D22" s="110" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E22" s="98" t="inlineStr"/>
+      <c r="E22" s="110" t="inlineStr"/>
       <c r="F22" s="39" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life - Section reading 1: A Roger Ekirch, “Sleep we have lost: Pre-Industrial Slumber in the Brit</t>
@@ -3578,18 +4594,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B23" s="98" t="inlineStr"/>
-      <c r="C23" s="98" t="inlineStr">
+      <c r="B23" s="110" t="inlineStr"/>
+      <c r="C23" s="110" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D23" s="98" t="inlineStr">
+      <c r="D23" s="110" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E23" s="98" t="inlineStr"/>
+      <c r="E23" s="110" t="inlineStr"/>
       <c r="F23" s="39" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance</t>
@@ -3602,18 +4618,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B24" s="98" t="inlineStr"/>
-      <c r="C24" s="98" t="inlineStr">
+      <c r="B24" s="110" t="inlineStr"/>
+      <c r="C24" s="110" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D24" s="98" t="inlineStr">
+      <c r="D24" s="110" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E24" s="98" t="inlineStr"/>
+      <c r="E24" s="110" t="inlineStr"/>
       <c r="F24" s="39" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance - Section reading 1: Kay Daly, “Diverting the Flood of History: Ada Palmer’s Inventing the Re</t>
@@ -3626,18 +4642,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B25" s="98" t="inlineStr"/>
-      <c r="C25" s="98" t="inlineStr">
+      <c r="B25" s="110" t="inlineStr"/>
+      <c r="C25" s="110" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D25" s="98" t="inlineStr">
+      <c r="D25" s="110" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E25" s="98" t="inlineStr"/>
+      <c r="E25" s="110" t="inlineStr"/>
       <c r="F25" s="39" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance</t>
@@ -3650,18 +4666,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B26" s="98" t="inlineStr"/>
-      <c r="C26" s="98" t="inlineStr">
+      <c r="B26" s="110" t="inlineStr"/>
+      <c r="C26" s="110" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D26" s="98" t="inlineStr">
+      <c r="D26" s="110" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E26" s="98" t="inlineStr"/>
+      <c r="E26" s="110" t="inlineStr"/>
       <c r="F26" s="39" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance - Section reading 1: Vasari, Lives of the Artists: Leonardo da Vinci &amp; Properzia de’ Rossi V</t>
@@ -3674,18 +4690,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B27" s="98" t="inlineStr"/>
-      <c r="C27" s="98" t="inlineStr">
+      <c r="B27" s="110" t="inlineStr"/>
+      <c r="C27" s="110" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D27" s="98" t="inlineStr">
+      <c r="D27" s="110" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E27" s="98" t="inlineStr"/>
+      <c r="E27" s="110" t="inlineStr"/>
       <c r="F27" s="39" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion</t>
@@ -3698,18 +4714,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B28" s="98" t="inlineStr"/>
-      <c r="C28" s="98" t="inlineStr">
+      <c r="B28" s="110" t="inlineStr"/>
+      <c r="C28" s="110" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D28" s="98" t="inlineStr">
+      <c r="D28" s="110" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E28" s="98" t="inlineStr"/>
+      <c r="E28" s="110" t="inlineStr"/>
       <c r="F28" s="39" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion - Section reading 1: Jerry Brotton, The Renaissance Bazaar, Chap 1 (15 pgs) Read Colu</t>
@@ -3722,18 +4738,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B29" s="98" t="inlineStr"/>
-      <c r="C29" s="98" t="inlineStr">
+      <c r="B29" s="110" t="inlineStr"/>
+      <c r="C29" s="110" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D29" s="98" t="inlineStr">
+      <c r="D29" s="110" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E29" s="98" t="inlineStr"/>
+      <c r="E29" s="110" t="inlineStr"/>
       <c r="F29" s="39" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion - Section reading 2: Bernal Diaz del Castillo, The True History of the Conquest of Ne</t>
@@ -3746,18 +4762,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B30" s="98" t="inlineStr"/>
-      <c r="C30" s="98" t="inlineStr">
+      <c r="B30" s="110" t="inlineStr"/>
+      <c r="C30" s="110" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="D30" s="98" t="inlineStr">
+      <c r="D30" s="110" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E30" s="98" t="inlineStr"/>
+      <c r="E30" s="110" t="inlineStr"/>
       <c r="F30" s="39" t="inlineStr">
         <is>
           <t>Week Oct 6-9: Midterm &amp; Break</t>
@@ -3770,18 +4786,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B31" s="98" t="inlineStr"/>
-      <c r="C31" s="98" t="inlineStr">
+      <c r="B31" s="110" t="inlineStr"/>
+      <c r="C31" s="110" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="D31" s="98" t="inlineStr">
+      <c r="D31" s="110" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="E31" s="98" t="inlineStr"/>
+      <c r="E31" s="110" t="inlineStr"/>
       <c r="F31" s="39" t="inlineStr">
         <is>
           <t>Week Oct 13-16: The Reformation</t>
@@ -3794,18 +4810,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B32" s="98" t="inlineStr"/>
-      <c r="C32" s="98" t="inlineStr">
+      <c r="B32" s="110" t="inlineStr"/>
+      <c r="C32" s="110" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="D32" s="98" t="inlineStr">
+      <c r="D32" s="110" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="E32" s="98" t="inlineStr"/>
+      <c r="E32" s="110" t="inlineStr"/>
       <c r="F32" s="39" t="inlineStr">
         <is>
           <t>Week Oct 20-23: The Reformation</t>
@@ -3818,18 +4834,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B33" s="98" t="inlineStr"/>
-      <c r="C33" s="98" t="inlineStr">
+      <c r="B33" s="110" t="inlineStr"/>
+      <c r="C33" s="110" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D33" s="98" t="inlineStr">
+      <c r="D33" s="110" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E33" s="98" t="inlineStr"/>
+      <c r="E33" s="110" t="inlineStr"/>
       <c r="F33" s="39" t="inlineStr">
         <is>
           <t>Week Oct 27-30: Reformation</t>
@@ -3842,18 +4858,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B34" s="98" t="inlineStr"/>
-      <c r="C34" s="98" t="inlineStr">
+      <c r="B34" s="110" t="inlineStr"/>
+      <c r="C34" s="110" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D34" s="98" t="inlineStr">
+      <c r="D34" s="110" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E34" s="98" t="inlineStr"/>
+      <c r="E34" s="110" t="inlineStr"/>
       <c r="F34" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Week Oct 27-30: Reformation - Section reading 1: Barbara Diefendorf, ed., The Saint Bartholomew’s Day Massacre: A Brief </t>
@@ -3866,18 +4882,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B35" s="98" t="inlineStr"/>
-      <c r="C35" s="98" t="inlineStr">
+      <c r="B35" s="110" t="inlineStr"/>
+      <c r="C35" s="110" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D35" s="98" t="inlineStr">
+      <c r="D35" s="110" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E35" s="98" t="inlineStr"/>
+      <c r="E35" s="110" t="inlineStr"/>
       <c r="F35" s="39" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science</t>
@@ -3890,18 +4906,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B36" s="98" t="inlineStr"/>
-      <c r="C36" s="98" t="inlineStr">
+      <c r="B36" s="110" t="inlineStr"/>
+      <c r="C36" s="110" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D36" s="98" t="inlineStr">
+      <c r="D36" s="110" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E36" s="98" t="inlineStr"/>
+      <c r="E36" s="110" t="inlineStr"/>
       <c r="F36" s="39" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science - Section reading 1: Brian Levack, The Witchcraft Sourcebook, Chaps 36-44, 46-47</t>
@@ -3914,18 +4930,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B37" s="98" t="inlineStr"/>
-      <c r="C37" s="98" t="inlineStr">
+      <c r="B37" s="110" t="inlineStr"/>
+      <c r="C37" s="110" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D37" s="98" t="inlineStr">
+      <c r="D37" s="110" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E37" s="98" t="inlineStr"/>
+      <c r="E37" s="110" t="inlineStr"/>
       <c r="F37" s="39" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment</t>
@@ -3938,18 +4954,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B38" s="98" t="inlineStr"/>
-      <c r="C38" s="98" t="inlineStr">
+      <c r="B38" s="110" t="inlineStr"/>
+      <c r="C38" s="110" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D38" s="98" t="inlineStr">
+      <c r="D38" s="110" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E38" s="98" t="inlineStr"/>
+      <c r="E38" s="110" t="inlineStr"/>
       <c r="F38" s="39" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment - Section reading 1: Excerpt: John Locke, Two Treatises of Government (1689) Excerpt: Rous</t>
@@ -3962,18 +4978,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B39" s="98" t="inlineStr"/>
-      <c r="C39" s="98" t="inlineStr">
+      <c r="B39" s="110" t="inlineStr"/>
+      <c r="C39" s="110" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D39" s="98" t="inlineStr">
+      <c r="D39" s="110" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E39" s="98" t="inlineStr"/>
+      <c r="E39" s="110" t="inlineStr"/>
       <c r="F39" s="39" t="inlineStr">
         <is>
           <t>Week Nov 17-20: Enlightenment</t>
@@ -3986,18 +5002,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B40" s="98" t="inlineStr"/>
-      <c r="C40" s="98" t="inlineStr">
+      <c r="B40" s="110" t="inlineStr"/>
+      <c r="C40" s="110" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D40" s="98" t="inlineStr">
+      <c r="D40" s="110" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E40" s="98" t="inlineStr"/>
+      <c r="E40" s="110" t="inlineStr"/>
       <c r="F40" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Week Nov 17-20: Enlightenment - Section reading 1: Video: Africa &amp; Britain, A Forgotten History, Episode 2: Freedom (50 </t>
@@ -4010,18 +5026,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B41" s="98" t="inlineStr"/>
-      <c r="C41" s="98" t="inlineStr">
+      <c r="B41" s="110" t="inlineStr"/>
+      <c r="C41" s="110" t="inlineStr">
         <is>
           <t>2026-12-01</t>
         </is>
       </c>
-      <c r="D41" s="98" t="inlineStr">
+      <c r="D41" s="110" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E41" s="98" t="inlineStr"/>
+      <c r="E41" s="110" t="inlineStr"/>
       <c r="F41" s="39" t="inlineStr">
         <is>
           <t>Week Dec 1-4: Modern Europe?</t>
@@ -4034,18 +5050,18 @@
           <t>Identification Quizzes</t>
         </is>
       </c>
-      <c r="B42" s="96" t="inlineStr">
+      <c r="B42" s="108" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C42" s="99" t="inlineStr"/>
-      <c r="D42" s="99" t="inlineStr">
+      <c r="C42" s="111" t="inlineStr"/>
+      <c r="D42" s="111" t="inlineStr">
         <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="E42" s="99" t="inlineStr">
+      <c r="E42" s="111" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4061,18 +5077,18 @@
           <t>Extra Credit</t>
         </is>
       </c>
-      <c r="B43" s="96" t="inlineStr">
+      <c r="B43" s="108" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C43" s="97" t="inlineStr"/>
-      <c r="D43" s="97" t="inlineStr">
+      <c r="C43" s="109" t="inlineStr"/>
+      <c r="D43" s="109" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E43" s="97" t="inlineStr">
+      <c r="E43" s="109" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4103,956 +5119,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00FF7F0E"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F48"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="48" t="inlineStr">
-        <is>
-          <t>BUAD-281 — Managerial Accounting</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="28">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/sources/buad-281-source.pdf","SEE HERE")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="29" t="inlineStr">
-        <is>
-          <t>Instructor</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>George Braunegg</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="29" t="inlineStr">
-        <is>
-          <t>Term</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Fall 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="29" t="inlineStr">
-        <is>
-          <t>Required for an A</t>
-        </is>
-      </c>
-      <c r="B5" s="30" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="29" t="inlineStr">
-        <is>
-          <t>Grading scale</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Total graded points in calendar: 1070 (letter scale not in document)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="49" t="inlineStr">
-        <is>
-          <t>Midterm 1 250 pts  |  Midterm 2 250 pts  |  Final Exam 250 pts  |  Homework 170 pts  |  LinkedIn Learning Excel Certification 75 pts  |  Stukent Simternship 75 pts</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="29" t="inlineStr">
-        <is>
-          <t>Strategy</t>
-        </is>
-      </c>
-      <c r="B8" s="50" t="inlineStr">
-        <is>
-          <t>If your AI tool breaks down and solves the homework bank problems - extracting step-by-step mechanics from the textbook - mastering those exact mechanics is all you need to get an A without reading prose.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="51" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B10" s="51" t="inlineStr">
-        <is>
-          <t>Weight</t>
-        </is>
-      </c>
-      <c r="C10" s="51" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="D10" s="51" t="inlineStr">
-        <is>
-          <t>Due Date</t>
-        </is>
-      </c>
-      <c r="E10" s="51" t="inlineStr">
-        <is>
-          <t>Group Project</t>
-        </is>
-      </c>
-      <c r="F10" s="51" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="52" t="inlineStr">
-        <is>
-          <t>Midterm 1</t>
-        </is>
-      </c>
-      <c r="B11" s="100" t="inlineStr">
-        <is>
-          <t>250 pts</t>
-        </is>
-      </c>
-      <c r="C11" s="101" t="inlineStr"/>
-      <c r="D11" s="101" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="E11" s="101" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F11" s="55">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-midterm-1.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="56" t="inlineStr">
-        <is>
-          <t>Exam</t>
-        </is>
-      </c>
-      <c r="B12" s="102" t="inlineStr"/>
-      <c r="C12" s="102" t="inlineStr"/>
-      <c r="D12" s="102" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="E12" s="102" t="inlineStr"/>
-      <c r="F12" s="58" t="inlineStr">
-        <is>
-          <t>9/30 Midterm 1: 250 Points Chapters 1, 2, 3, 4, 5, 8</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="59" t="inlineStr">
-        <is>
-          <t>Midterm 2</t>
-        </is>
-      </c>
-      <c r="B13" s="100" t="inlineStr">
-        <is>
-          <t>250 pts</t>
-        </is>
-      </c>
-      <c r="C13" s="103" t="inlineStr"/>
-      <c r="D13" s="103" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="E13" s="103" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F13" s="61">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-midterm-2.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="56" t="inlineStr">
-        <is>
-          <t>Exam</t>
-        </is>
-      </c>
-      <c r="B14" s="102" t="inlineStr"/>
-      <c r="C14" s="102" t="inlineStr"/>
-      <c r="D14" s="102" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="E14" s="102" t="inlineStr"/>
-      <c r="F14" s="58" t="inlineStr">
-        <is>
-          <t>10/26 Midterm 2: 250 Points Chapters 6, 7, 9, &amp; 16</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="52" t="inlineStr">
-        <is>
-          <t>Final Exam</t>
-        </is>
-      </c>
-      <c r="B15" s="100" t="inlineStr">
-        <is>
-          <t>250 pts</t>
-        </is>
-      </c>
-      <c r="C15" s="101" t="inlineStr"/>
-      <c r="D15" s="101" t="inlineStr">
-        <is>
-          <t>2026-12-16</t>
-        </is>
-      </c>
-      <c r="E15" s="101" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F15" s="55">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-final-exam.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="56" t="inlineStr">
-        <is>
-          <t>Exam</t>
-        </is>
-      </c>
-      <c r="B16" s="102" t="inlineStr"/>
-      <c r="C16" s="102" t="inlineStr"/>
-      <c r="D16" s="102" t="inlineStr">
-        <is>
-          <t>2026-12-16</t>
-        </is>
-      </c>
-      <c r="E16" s="102" t="inlineStr"/>
-      <c r="F16" s="58" t="inlineStr">
-        <is>
-          <t>Final Exam</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="59" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B17" s="100" t="inlineStr">
-        <is>
-          <t>170 pts</t>
-        </is>
-      </c>
-      <c r="C17" s="103" t="inlineStr"/>
-      <c r="D17" s="103" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E17" s="103" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F17" s="61">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-homework.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="62" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B18" s="102" t="inlineStr"/>
-      <c r="C18" s="102" t="inlineStr"/>
-      <c r="D18" s="102" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="E18" s="102" t="inlineStr"/>
-      <c r="F18" s="58" t="inlineStr">
-        <is>
-          <t>Class 5 (9/9) - Product Cost Accumulation: Job; Order Co: Chapter 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="63" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B19" s="102" t="inlineStr"/>
-      <c r="C19" s="102" t="inlineStr"/>
-      <c r="D19" s="102" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="E19" s="102" t="inlineStr"/>
-      <c r="F19" s="58" t="inlineStr">
-        <is>
-          <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="62" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B20" s="102" t="inlineStr"/>
-      <c r="C20" s="102" t="inlineStr"/>
-      <c r="D20" s="102" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="E20" s="102" t="inlineStr"/>
-      <c r="F20" s="58" t="inlineStr">
-        <is>
-          <t>Class 7 (9/16) - Activity Based Costing: Chapter 5- ONLY; LO 5.1, 2, 4 &amp; 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="63" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B21" s="102" t="inlineStr"/>
-      <c r="C21" s="102" t="inlineStr"/>
-      <c r="D21" s="102" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="E21" s="102" t="inlineStr"/>
-      <c r="F21" s="58" t="inlineStr">
-        <is>
-          <t>Class 7 (9/16) - 3-24, 3-28, 3-32; 15 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="62" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B22" s="102" t="inlineStr"/>
-      <c r="C22" s="102" t="inlineStr"/>
-      <c r="D22" s="102" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="E22" s="102" t="inlineStr"/>
-      <c r="F22" s="58" t="inlineStr">
-        <is>
-          <t>Class 8 (9/21) - Product Cost Accumulation: Pro-; cess Co: Chapter 4- ONLY; LO 4.1, 3, 4, &amp; 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="63" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B23" s="102" t="inlineStr"/>
-      <c r="C23" s="102" t="inlineStr"/>
-      <c r="D23" s="102" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="E23" s="102" t="inlineStr"/>
-      <c r="F23" s="58" t="inlineStr">
-        <is>
-          <t>Class 8 (9/21) - 5-27 5-46; 10 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="62" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B24" s="102" t="inlineStr"/>
-      <c r="C24" s="102" t="inlineStr"/>
-      <c r="D24" s="102" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="E24" s="102" t="inlineStr"/>
-      <c r="F24" s="58" t="inlineStr">
-        <is>
-          <t>Class 9 (9/23) - Cost of Quality &amp; ESG &amp;; Overview of; • : Chapter 8 - ONLY; LO 8.7, 8, 9</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="63" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B25" s="102" t="inlineStr"/>
-      <c r="C25" s="102" t="inlineStr"/>
-      <c r="D25" s="102" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="E25" s="102" t="inlineStr"/>
-      <c r="F25" s="58" t="inlineStr">
-        <is>
-          <t>Class 9 (9/23) - 4-21, 4-22; 10 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="62" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B26" s="102" t="inlineStr"/>
-      <c r="C26" s="102" t="inlineStr"/>
-      <c r="D26" s="102" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E26" s="102" t="inlineStr"/>
-      <c r="F26" s="58" t="inlineStr">
-        <is>
-          <t>Class 10 (9/28) - Catchup &amp; Midterm Review</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="63" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B27" s="102" t="inlineStr"/>
-      <c r="C27" s="102" t="inlineStr"/>
-      <c r="D27" s="102" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E27" s="102" t="inlineStr"/>
-      <c r="F27" s="58" t="inlineStr">
-        <is>
-          <t>Class 10 (9/28) - 8-28, 8-29; 10 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="62" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B28" s="102" t="inlineStr"/>
-      <c r="C28" s="102" t="inlineStr"/>
-      <c r="D28" s="102" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="E28" s="102" t="inlineStr"/>
-      <c r="F28" s="58" t="inlineStr">
-        <is>
-          <t>Class 12 (10/7) - Cost volume profit analysis: Chapter 7</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="63" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B29" s="102" t="inlineStr"/>
-      <c r="C29" s="102" t="inlineStr"/>
-      <c r="D29" s="102" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="E29" s="102" t="inlineStr"/>
-      <c r="F29" s="58" t="inlineStr">
-        <is>
-          <t>Class 12 (10/7) - 6-24, 6-25, 6-34; 15 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="62" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B30" s="102" t="inlineStr"/>
-      <c r="C30" s="102" t="inlineStr"/>
-      <c r="D30" s="102" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E30" s="102" t="inlineStr"/>
-      <c r="F30" s="58" t="inlineStr">
-        <is>
-          <t>Class 14 (10/14) - Financial planning and analysis:; Static: Chapter 9</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="63" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B31" s="102" t="inlineStr"/>
-      <c r="C31" s="102" t="inlineStr"/>
-      <c r="D31" s="102" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E31" s="102" t="inlineStr"/>
-      <c r="F31" s="58" t="inlineStr">
-        <is>
-          <t>Class 14 (10/14) - 7-29, 7-33, 7-40; 15 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="62" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B32" s="102" t="inlineStr"/>
-      <c r="C32" s="102" t="inlineStr"/>
-      <c r="D32" s="102" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E32" s="102" t="inlineStr"/>
-      <c r="F32" s="58" t="inlineStr">
-        <is>
-          <t>Class 15 (10/19) - Capital Budgeting; Practice Midterm Ques: Chapter 16- ONLY; LO 16.1, 2, 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="63" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B33" s="102" t="inlineStr"/>
-      <c r="C33" s="102" t="inlineStr"/>
-      <c r="D33" s="102" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E33" s="102" t="inlineStr"/>
-      <c r="F33" s="58" t="inlineStr">
-        <is>
-          <t>Class 15 (10/19) - 9-25, 9-28, 9-37; 15 - Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="62" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B34" s="102" t="inlineStr"/>
-      <c r="C34" s="102" t="inlineStr"/>
-      <c r="D34" s="102" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="E34" s="102" t="inlineStr"/>
-      <c r="F34" s="58" t="inlineStr">
-        <is>
-          <t>Class 16 (10/21) - Catchup &amp; Midterm Review</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="63" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B35" s="102" t="inlineStr"/>
-      <c r="C35" s="102" t="inlineStr"/>
-      <c r="D35" s="102" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="E35" s="102" t="inlineStr"/>
-      <c r="F35" s="58" t="inlineStr">
-        <is>
-          <t>Class 16 (10/21) - 16-28, 16-40; 10 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="62" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B36" s="102" t="inlineStr"/>
-      <c r="C36" s="102" t="inlineStr"/>
-      <c r="D36" s="102" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="E36" s="102" t="inlineStr"/>
-      <c r="F36" s="58" t="inlineStr">
-        <is>
-          <t>Class 19 (11/4) - Sales Variance Analysis; Flexible Budget: Chapter 11 - ONLY; LO 11.1, 11.2 &amp;; Appendix B</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="63" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B37" s="102" t="inlineStr"/>
-      <c r="C37" s="102" t="inlineStr"/>
-      <c r="D37" s="102" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="E37" s="102" t="inlineStr"/>
-      <c r="F37" s="58" t="inlineStr">
-        <is>
-          <t>Class 19 (11/4) - 10-26, 10-30; 10 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="62" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B38" s="102" t="inlineStr"/>
-      <c r="C38" s="102" t="inlineStr"/>
-      <c r="D38" s="102" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="E38" s="102" t="inlineStr"/>
-      <c r="F38" s="58" t="inlineStr">
-        <is>
-          <t>Class 20 (11/9) - Investment Centers: Chapter 13- ONLY; LO 13-1, 2, 3, 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="63" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B39" s="102" t="inlineStr"/>
-      <c r="C39" s="102" t="inlineStr"/>
-      <c r="D39" s="102" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="E39" s="102" t="inlineStr"/>
-      <c r="F39" s="58" t="inlineStr">
-        <is>
-          <t>Class 20 (11/9) - 11-31, 11-52; 10 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="62" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B40" s="102" t="inlineStr"/>
-      <c r="C40" s="102" t="inlineStr"/>
-      <c r="D40" s="102" t="inlineStr">
-        <is>
-          <t>2026-11-16</t>
-        </is>
-      </c>
-      <c r="E40" s="102" t="inlineStr"/>
-      <c r="F40" s="58" t="inlineStr">
-        <is>
-          <t>Class 21 (11/16) - AI &amp; FP&amp;A</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="63" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B41" s="102" t="inlineStr"/>
-      <c r="C41" s="102" t="inlineStr"/>
-      <c r="D41" s="102" t="inlineStr">
-        <is>
-          <t>2026-11-16</t>
-        </is>
-      </c>
-      <c r="E41" s="102" t="inlineStr"/>
-      <c r="F41" s="58" t="inlineStr">
-        <is>
-          <t>Class 21 (11/16) - 13-29, 13-33; 10 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="62" t="inlineStr">
-        <is>
-          <t>Reading</t>
-        </is>
-      </c>
-      <c r="B42" s="102" t="inlineStr"/>
-      <c r="C42" s="102" t="inlineStr"/>
-      <c r="D42" s="102" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E42" s="102" t="inlineStr"/>
-      <c r="F42" s="58" t="inlineStr">
-        <is>
-          <t>Class 2 (12/2) - Catchup &amp; Final Review; Practice Final Questions Posted to Brightspace at; 5:00 PM</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="63" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B43" s="102" t="inlineStr"/>
-      <c r="C43" s="102" t="inlineStr"/>
-      <c r="D43" s="102" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E43" s="102" t="inlineStr"/>
-      <c r="F43" s="58" t="inlineStr">
-        <is>
-          <t>Class 2 (12/2) - 14-35, 14-41; 10 Points; Assignments listed Be-; low Due by11:59 PM; Linked In Learning; E</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="52" t="inlineStr">
-        <is>
-          <t>LinkedIn Learning Excel Certification</t>
-        </is>
-      </c>
-      <c r="B44" s="100" t="inlineStr">
-        <is>
-          <t>75 pts</t>
-        </is>
-      </c>
-      <c r="C44" s="101" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="D44" s="101" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E44" s="101" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F44" s="55">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-linkedin-learning-excel-certification.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="64" t="inlineStr">
-        <is>
-          <t>Certification</t>
-        </is>
-      </c>
-      <c r="B45" s="102" t="inlineStr"/>
-      <c r="C45" s="102" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="D45" s="102" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E45" s="102" t="inlineStr"/>
-      <c r="F45" s="58" t="inlineStr">
-        <is>
-          <t>LinkedIn Learning Excel Certification</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="59" t="inlineStr">
-        <is>
-          <t>Stukent Simternship</t>
-        </is>
-      </c>
-      <c r="B46" s="100" t="inlineStr">
-        <is>
-          <t>75 pts</t>
-        </is>
-      </c>
-      <c r="C46" s="103" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="D46" s="103" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E46" s="103" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F46" s="61">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-281-stukent-simternship.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="64" t="inlineStr">
-        <is>
-          <t>Certification</t>
-        </is>
-      </c>
-      <c r="B47" s="102" t="inlineStr"/>
-      <c r="C47" s="102" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="D47" s="102" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E47" s="102" t="inlineStr"/>
-      <c r="F47" s="58" t="inlineStr">
-        <is>
-          <t>Stukent Simternship</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="29" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B48" s="65" t="inlineStr">
-        <is>
-          <t>1070 pts</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="A7:F7"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Make Overview professor ratings collapsible with Excel row grouping
- Group stats and consensus rows under the RMP title with +/- controls
- Start collapsed by default so assignments stay visible on open
- Document grouping behavior in reference.md

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -319,7 +319,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -341,11 +341,55 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -636,6 +680,18 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1011,7 +1067,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00203764"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K49"/>
@@ -1054,11 +1110,11 @@
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>Professor Ratings (Rate My Professors)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>Professor Ratings (Rate My Professors) — click +/- at left to expand/collapse</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" hidden="1" outlineLevel="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Class</t>
@@ -1090,7 +1146,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" hidden="1" outlineLevel="1">
       <c r="A6" s="7">
         <f>HYPERLINK("#'BUAD-281'!A1","BUAD-281")</f>
         <v/>
@@ -1121,7 +1177,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" hidden="1" outlineLevel="1">
       <c r="A7" s="10">
         <f>HYPERLINK("#'BUAD-304'!A1","BUAD-304")</f>
         <v/>
@@ -1152,7 +1208,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" hidden="1" outlineLevel="1">
       <c r="A8" s="7">
         <f>HYPERLINK("#'HIST-103'!A1","HIST-103")</f>
         <v/>
@@ -1183,14 +1239,15 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="9" hidden="1" outlineLevel="1"/>
+    <row r="10" hidden="1" outlineLevel="1">
       <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Consensus - recurring student review themes</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="135" customHeight="1">
+    <row r="11" hidden="1" outlineLevel="1" ht="135" customHeight="1">
       <c r="A11" s="104" t="inlineStr">
         <is>
           <t>BUAD-281</t>
@@ -1209,7 +1266,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="135" customHeight="1">
+    <row r="12" hidden="1" outlineLevel="1" ht="135" customHeight="1">
       <c r="A12" s="106" t="inlineStr">
         <is>
           <t>BUAD-304</t>
@@ -1228,7 +1285,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="135" customHeight="1">
+    <row r="13" hidden="1" outlineLevel="1" ht="135" customHeight="1">
       <c r="A13" s="104" t="inlineStr">
         <is>
           <t>HIST-103</t>
@@ -1247,7 +1304,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" hidden="1" outlineLevel="1">
       <c r="A14" s="91" t="inlineStr">
         <is>
           <t>RMP data as of 2026-08-21. Source: ratemyprofessors.com</t>
@@ -4283,18 +4340,18 @@
           <t>Sleep Paper</t>
         </is>
       </c>
-      <c r="B10" s="108" t="inlineStr">
+      <c r="B10" s="112" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C10" s="109" t="inlineStr"/>
-      <c r="D10" s="109" t="inlineStr">
+      <c r="C10" s="113" t="inlineStr"/>
+      <c r="D10" s="113" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="E10" s="109" t="inlineStr">
+      <c r="E10" s="113" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4310,14 +4367,14 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B11" s="110" t="inlineStr"/>
-      <c r="C11" s="110" t="inlineStr"/>
-      <c r="D11" s="110" t="inlineStr">
+      <c r="B11" s="114" t="inlineStr"/>
+      <c r="C11" s="114" t="inlineStr"/>
+      <c r="D11" s="114" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="E11" s="110" t="inlineStr"/>
+      <c r="E11" s="114" t="inlineStr"/>
       <c r="F11" s="39" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
@@ -4330,18 +4387,18 @@
           <t>Witchcraft Paper</t>
         </is>
       </c>
-      <c r="B12" s="108" t="inlineStr">
+      <c r="B12" s="112" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C12" s="111" t="inlineStr"/>
-      <c r="D12" s="111" t="inlineStr">
+      <c r="C12" s="115" t="inlineStr"/>
+      <c r="D12" s="115" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="E12" s="111" t="inlineStr">
+      <c r="E12" s="115" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4357,14 +4414,14 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B13" s="110" t="inlineStr"/>
-      <c r="C13" s="110" t="inlineStr"/>
-      <c r="D13" s="110" t="inlineStr">
+      <c r="B13" s="114" t="inlineStr"/>
+      <c r="C13" s="114" t="inlineStr"/>
+      <c r="D13" s="114" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="E13" s="110" t="inlineStr"/>
+      <c r="E13" s="114" t="inlineStr"/>
       <c r="F13" s="39" t="inlineStr">
         <is>
           <t>Witchcraft Paper Due</t>
@@ -4377,18 +4434,18 @@
           <t>Mid-term</t>
         </is>
       </c>
-      <c r="B14" s="108" t="inlineStr">
+      <c r="B14" s="112" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C14" s="109" t="inlineStr"/>
-      <c r="D14" s="109" t="inlineStr">
+      <c r="C14" s="113" t="inlineStr"/>
+      <c r="D14" s="113" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E14" s="109" t="inlineStr">
+      <c r="E14" s="113" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4404,14 +4461,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B15" s="110" t="inlineStr"/>
-      <c r="C15" s="110" t="inlineStr"/>
-      <c r="D15" s="110" t="inlineStr">
+      <c r="B15" s="114" t="inlineStr"/>
+      <c r="C15" s="114" t="inlineStr"/>
+      <c r="D15" s="114" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="E15" s="110" t="inlineStr"/>
+      <c r="E15" s="114" t="inlineStr"/>
       <c r="F15" s="39" t="inlineStr">
         <is>
           <t>Midterm Exam</t>
@@ -4424,18 +4481,18 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B16" s="108" t="inlineStr">
+      <c r="B16" s="112" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C16" s="111" t="inlineStr"/>
-      <c r="D16" s="111" t="inlineStr">
+      <c r="C16" s="115" t="inlineStr"/>
+      <c r="D16" s="115" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="E16" s="111" t="inlineStr">
+      <c r="E16" s="115" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4451,14 +4508,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B17" s="110" t="inlineStr"/>
-      <c r="C17" s="110" t="inlineStr"/>
-      <c r="D17" s="110" t="inlineStr">
+      <c r="B17" s="114" t="inlineStr"/>
+      <c r="C17" s="114" t="inlineStr"/>
+      <c r="D17" s="114" t="inlineStr">
         <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="E17" s="110" t="inlineStr"/>
+      <c r="E17" s="114" t="inlineStr"/>
       <c r="F17" s="39" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -4471,18 +4528,18 @@
           <t>Discussion Section</t>
         </is>
       </c>
-      <c r="B18" s="108" t="inlineStr">
+      <c r="B18" s="112" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C18" s="109" t="inlineStr"/>
-      <c r="D18" s="109" t="inlineStr">
+      <c r="C18" s="113" t="inlineStr"/>
+      <c r="D18" s="113" t="inlineStr">
         <is>
           <t>2026-11-12</t>
         </is>
       </c>
-      <c r="E18" s="109" t="inlineStr">
+      <c r="E18" s="113" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4498,18 +4555,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B19" s="110" t="inlineStr"/>
-      <c r="C19" s="110" t="inlineStr">
+      <c r="B19" s="114" t="inlineStr"/>
+      <c r="C19" s="114" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D19" s="110" t="inlineStr">
+      <c r="D19" s="114" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E19" s="110" t="inlineStr"/>
+      <c r="E19" s="114" t="inlineStr"/>
       <c r="F19" s="39" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death</t>
@@ -4522,18 +4579,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B20" s="110" t="inlineStr"/>
-      <c r="C20" s="110" t="inlineStr">
+      <c r="B20" s="114" t="inlineStr"/>
+      <c r="C20" s="114" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D20" s="110" t="inlineStr">
+      <c r="D20" s="114" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E20" s="110" t="inlineStr"/>
+      <c r="E20" s="114" t="inlineStr"/>
       <c r="F20" s="39" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death - Section reading 1: Lizzie Wade, “From Black Death to fatal flu, past pandemics sho</t>
@@ -4546,18 +4603,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B21" s="110" t="inlineStr"/>
-      <c r="C21" s="110" t="inlineStr">
+      <c r="B21" s="114" t="inlineStr"/>
+      <c r="C21" s="114" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D21" s="110" t="inlineStr">
+      <c r="D21" s="114" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E21" s="110" t="inlineStr"/>
+      <c r="E21" s="114" t="inlineStr"/>
       <c r="F21" s="39" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life</t>
@@ -4570,18 +4627,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B22" s="110" t="inlineStr"/>
-      <c r="C22" s="110" t="inlineStr">
+      <c r="B22" s="114" t="inlineStr"/>
+      <c r="C22" s="114" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D22" s="110" t="inlineStr">
+      <c r="D22" s="114" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E22" s="110" t="inlineStr"/>
+      <c r="E22" s="114" t="inlineStr"/>
       <c r="F22" s="39" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life - Section reading 1: A Roger Ekirch, “Sleep we have lost: Pre-Industrial Slumber in the Brit</t>
@@ -4594,18 +4651,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B23" s="110" t="inlineStr"/>
-      <c r="C23" s="110" t="inlineStr">
+      <c r="B23" s="114" t="inlineStr"/>
+      <c r="C23" s="114" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D23" s="110" t="inlineStr">
+      <c r="D23" s="114" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E23" s="110" t="inlineStr"/>
+      <c r="E23" s="114" t="inlineStr"/>
       <c r="F23" s="39" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance</t>
@@ -4618,18 +4675,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B24" s="110" t="inlineStr"/>
-      <c r="C24" s="110" t="inlineStr">
+      <c r="B24" s="114" t="inlineStr"/>
+      <c r="C24" s="114" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D24" s="110" t="inlineStr">
+      <c r="D24" s="114" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E24" s="110" t="inlineStr"/>
+      <c r="E24" s="114" t="inlineStr"/>
       <c r="F24" s="39" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance - Section reading 1: Kay Daly, “Diverting the Flood of History: Ada Palmer’s Inventing the Re</t>
@@ -4642,18 +4699,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B25" s="110" t="inlineStr"/>
-      <c r="C25" s="110" t="inlineStr">
+      <c r="B25" s="114" t="inlineStr"/>
+      <c r="C25" s="114" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D25" s="110" t="inlineStr">
+      <c r="D25" s="114" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E25" s="110" t="inlineStr"/>
+      <c r="E25" s="114" t="inlineStr"/>
       <c r="F25" s="39" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance</t>
@@ -4666,18 +4723,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B26" s="110" t="inlineStr"/>
-      <c r="C26" s="110" t="inlineStr">
+      <c r="B26" s="114" t="inlineStr"/>
+      <c r="C26" s="114" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D26" s="110" t="inlineStr">
+      <c r="D26" s="114" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E26" s="110" t="inlineStr"/>
+      <c r="E26" s="114" t="inlineStr"/>
       <c r="F26" s="39" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance - Section reading 1: Vasari, Lives of the Artists: Leonardo da Vinci &amp; Properzia de’ Rossi V</t>
@@ -4690,18 +4747,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B27" s="110" t="inlineStr"/>
-      <c r="C27" s="110" t="inlineStr">
+      <c r="B27" s="114" t="inlineStr"/>
+      <c r="C27" s="114" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D27" s="110" t="inlineStr">
+      <c r="D27" s="114" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E27" s="110" t="inlineStr"/>
+      <c r="E27" s="114" t="inlineStr"/>
       <c r="F27" s="39" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion</t>
@@ -4714,18 +4771,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B28" s="110" t="inlineStr"/>
-      <c r="C28" s="110" t="inlineStr">
+      <c r="B28" s="114" t="inlineStr"/>
+      <c r="C28" s="114" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D28" s="110" t="inlineStr">
+      <c r="D28" s="114" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E28" s="110" t="inlineStr"/>
+      <c r="E28" s="114" t="inlineStr"/>
       <c r="F28" s="39" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion - Section reading 1: Jerry Brotton, The Renaissance Bazaar, Chap 1 (15 pgs) Read Colu</t>
@@ -4738,18 +4795,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B29" s="110" t="inlineStr"/>
-      <c r="C29" s="110" t="inlineStr">
+      <c r="B29" s="114" t="inlineStr"/>
+      <c r="C29" s="114" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D29" s="110" t="inlineStr">
+      <c r="D29" s="114" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E29" s="110" t="inlineStr"/>
+      <c r="E29" s="114" t="inlineStr"/>
       <c r="F29" s="39" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion - Section reading 2: Bernal Diaz del Castillo, The True History of the Conquest of Ne</t>
@@ -4762,18 +4819,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B30" s="110" t="inlineStr"/>
-      <c r="C30" s="110" t="inlineStr">
+      <c r="B30" s="114" t="inlineStr"/>
+      <c r="C30" s="114" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="D30" s="110" t="inlineStr">
+      <c r="D30" s="114" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E30" s="110" t="inlineStr"/>
+      <c r="E30" s="114" t="inlineStr"/>
       <c r="F30" s="39" t="inlineStr">
         <is>
           <t>Week Oct 6-9: Midterm &amp; Break</t>
@@ -4786,18 +4843,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B31" s="110" t="inlineStr"/>
-      <c r="C31" s="110" t="inlineStr">
+      <c r="B31" s="114" t="inlineStr"/>
+      <c r="C31" s="114" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="D31" s="110" t="inlineStr">
+      <c r="D31" s="114" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="E31" s="110" t="inlineStr"/>
+      <c r="E31" s="114" t="inlineStr"/>
       <c r="F31" s="39" t="inlineStr">
         <is>
           <t>Week Oct 13-16: The Reformation</t>
@@ -4810,18 +4867,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B32" s="110" t="inlineStr"/>
-      <c r="C32" s="110" t="inlineStr">
+      <c r="B32" s="114" t="inlineStr"/>
+      <c r="C32" s="114" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="D32" s="110" t="inlineStr">
+      <c r="D32" s="114" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="E32" s="110" t="inlineStr"/>
+      <c r="E32" s="114" t="inlineStr"/>
       <c r="F32" s="39" t="inlineStr">
         <is>
           <t>Week Oct 20-23: The Reformation</t>
@@ -4834,18 +4891,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B33" s="110" t="inlineStr"/>
-      <c r="C33" s="110" t="inlineStr">
+      <c r="B33" s="114" t="inlineStr"/>
+      <c r="C33" s="114" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D33" s="110" t="inlineStr">
+      <c r="D33" s="114" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E33" s="110" t="inlineStr"/>
+      <c r="E33" s="114" t="inlineStr"/>
       <c r="F33" s="39" t="inlineStr">
         <is>
           <t>Week Oct 27-30: Reformation</t>
@@ -4858,18 +4915,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B34" s="110" t="inlineStr"/>
-      <c r="C34" s="110" t="inlineStr">
+      <c r="B34" s="114" t="inlineStr"/>
+      <c r="C34" s="114" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D34" s="110" t="inlineStr">
+      <c r="D34" s="114" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E34" s="110" t="inlineStr"/>
+      <c r="E34" s="114" t="inlineStr"/>
       <c r="F34" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Week Oct 27-30: Reformation - Section reading 1: Barbara Diefendorf, ed., The Saint Bartholomew’s Day Massacre: A Brief </t>
@@ -4882,18 +4939,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B35" s="110" t="inlineStr"/>
-      <c r="C35" s="110" t="inlineStr">
+      <c r="B35" s="114" t="inlineStr"/>
+      <c r="C35" s="114" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D35" s="110" t="inlineStr">
+      <c r="D35" s="114" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E35" s="110" t="inlineStr"/>
+      <c r="E35" s="114" t="inlineStr"/>
       <c r="F35" s="39" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science</t>
@@ -4906,18 +4963,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B36" s="110" t="inlineStr"/>
-      <c r="C36" s="110" t="inlineStr">
+      <c r="B36" s="114" t="inlineStr"/>
+      <c r="C36" s="114" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D36" s="110" t="inlineStr">
+      <c r="D36" s="114" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E36" s="110" t="inlineStr"/>
+      <c r="E36" s="114" t="inlineStr"/>
       <c r="F36" s="39" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science - Section reading 1: Brian Levack, The Witchcraft Sourcebook, Chaps 36-44, 46-47</t>
@@ -4930,18 +4987,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B37" s="110" t="inlineStr"/>
-      <c r="C37" s="110" t="inlineStr">
+      <c r="B37" s="114" t="inlineStr"/>
+      <c r="C37" s="114" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D37" s="110" t="inlineStr">
+      <c r="D37" s="114" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E37" s="110" t="inlineStr"/>
+      <c r="E37" s="114" t="inlineStr"/>
       <c r="F37" s="39" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment</t>
@@ -4954,18 +5011,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B38" s="110" t="inlineStr"/>
-      <c r="C38" s="110" t="inlineStr">
+      <c r="B38" s="114" t="inlineStr"/>
+      <c r="C38" s="114" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D38" s="110" t="inlineStr">
+      <c r="D38" s="114" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E38" s="110" t="inlineStr"/>
+      <c r="E38" s="114" t="inlineStr"/>
       <c r="F38" s="39" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment - Section reading 1: Excerpt: John Locke, Two Treatises of Government (1689) Excerpt: Rous</t>
@@ -4978,18 +5035,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B39" s="110" t="inlineStr"/>
-      <c r="C39" s="110" t="inlineStr">
+      <c r="B39" s="114" t="inlineStr"/>
+      <c r="C39" s="114" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D39" s="110" t="inlineStr">
+      <c r="D39" s="114" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E39" s="110" t="inlineStr"/>
+      <c r="E39" s="114" t="inlineStr"/>
       <c r="F39" s="39" t="inlineStr">
         <is>
           <t>Week Nov 17-20: Enlightenment</t>
@@ -5002,18 +5059,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B40" s="110" t="inlineStr"/>
-      <c r="C40" s="110" t="inlineStr">
+      <c r="B40" s="114" t="inlineStr"/>
+      <c r="C40" s="114" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D40" s="110" t="inlineStr">
+      <c r="D40" s="114" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E40" s="110" t="inlineStr"/>
+      <c r="E40" s="114" t="inlineStr"/>
       <c r="F40" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Week Nov 17-20: Enlightenment - Section reading 1: Video: Africa &amp; Britain, A Forgotten History, Episode 2: Freedom (50 </t>
@@ -5026,18 +5083,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B41" s="110" t="inlineStr"/>
-      <c r="C41" s="110" t="inlineStr">
+      <c r="B41" s="114" t="inlineStr"/>
+      <c r="C41" s="114" t="inlineStr">
         <is>
           <t>2026-12-01</t>
         </is>
       </c>
-      <c r="D41" s="110" t="inlineStr">
+      <c r="D41" s="114" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E41" s="110" t="inlineStr"/>
+      <c r="E41" s="114" t="inlineStr"/>
       <c r="F41" s="39" t="inlineStr">
         <is>
           <t>Week Dec 1-4: Modern Europe?</t>
@@ -5050,18 +5107,18 @@
           <t>Identification Quizzes</t>
         </is>
       </c>
-      <c r="B42" s="108" t="inlineStr">
+      <c r="B42" s="112" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C42" s="111" t="inlineStr"/>
-      <c r="D42" s="111" t="inlineStr">
+      <c r="C42" s="115" t="inlineStr"/>
+      <c r="D42" s="115" t="inlineStr">
         <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="E42" s="111" t="inlineStr">
+      <c r="E42" s="115" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5077,18 +5134,18 @@
           <t>Extra Credit</t>
         </is>
       </c>
-      <c r="B43" s="108" t="inlineStr">
+      <c r="B43" s="112" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C43" s="109" t="inlineStr"/>
-      <c r="D43" s="109" t="inlineStr">
+      <c r="C43" s="113" t="inlineStr"/>
+      <c r="D43" s="113" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E43" s="109" t="inlineStr">
+      <c r="E43" s="113" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Add average reviewer grade to RMP Overview stats
- Fetch letter grades via RMP GraphQL and compute avg GPA + letter
- Show Avg Reviewer Grade column with reported-grade count
- Rewrite fetch_rmp.py to use GraphQL instead of HTML scraping

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -389,7 +389,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="116">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -680,6 +680,18 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1110,7 +1122,7 @@
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>Professor Ratings (Rate My Professors) — click +/- at left to expand/collapse</t>
+          <t>Professor Ratings (Rate My Professors) - click +/- at left to expand/collapse</t>
         </is>
       </c>
     </row>
@@ -1137,10 +1149,15 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
+          <t>Avg Reviewer Grade</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
           <t>Would Take Again</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t># Ratings</t>
         </is>
@@ -1168,10 +1185,15 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>81%</t>
+          <t>A- (3.69) [177/255 reported]</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>80.9%</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
         <is>
           <t>255</t>
         </is>
@@ -1199,10 +1221,15 @@
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>79%</t>
+          <t>A- (3.71) [29/50 reported]</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>78.9%</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -1225,17 +1252,22 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>2.6</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>78.6%</t>
+          <t>A- (3.77) [27/54 reported]</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>79.3%</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>54</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1339,7 @@
     <row r="14" hidden="1" outlineLevel="1">
       <c r="A14" s="91" t="inlineStr">
         <is>
-          <t>RMP data as of 2026-08-21. Source: ratemyprofessors.com</t>
+          <t>RMP data as of 2026-08-21. Source: ratemyprofessors.com. Avg reviewer grade = mean of self-reported letter grades (4.0 scale); not all reviewers report a grade.</t>
         </is>
       </c>
     </row>
@@ -4340,18 +4372,18 @@
           <t>Sleep Paper</t>
         </is>
       </c>
-      <c r="B10" s="112" t="inlineStr">
+      <c r="B10" s="116" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C10" s="113" t="inlineStr"/>
-      <c r="D10" s="113" t="inlineStr">
+      <c r="C10" s="117" t="inlineStr"/>
+      <c r="D10" s="117" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="E10" s="113" t="inlineStr">
+      <c r="E10" s="117" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4367,14 +4399,14 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B11" s="114" t="inlineStr"/>
-      <c r="C11" s="114" t="inlineStr"/>
-      <c r="D11" s="114" t="inlineStr">
+      <c r="B11" s="118" t="inlineStr"/>
+      <c r="C11" s="118" t="inlineStr"/>
+      <c r="D11" s="118" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="E11" s="114" t="inlineStr"/>
+      <c r="E11" s="118" t="inlineStr"/>
       <c r="F11" s="39" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
@@ -4387,18 +4419,18 @@
           <t>Witchcraft Paper</t>
         </is>
       </c>
-      <c r="B12" s="112" t="inlineStr">
+      <c r="B12" s="116" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C12" s="115" t="inlineStr"/>
-      <c r="D12" s="115" t="inlineStr">
+      <c r="C12" s="119" t="inlineStr"/>
+      <c r="D12" s="119" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="E12" s="115" t="inlineStr">
+      <c r="E12" s="119" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4414,14 +4446,14 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B13" s="114" t="inlineStr"/>
-      <c r="C13" s="114" t="inlineStr"/>
-      <c r="D13" s="114" t="inlineStr">
+      <c r="B13" s="118" t="inlineStr"/>
+      <c r="C13" s="118" t="inlineStr"/>
+      <c r="D13" s="118" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="E13" s="114" t="inlineStr"/>
+      <c r="E13" s="118" t="inlineStr"/>
       <c r="F13" s="39" t="inlineStr">
         <is>
           <t>Witchcraft Paper Due</t>
@@ -4434,18 +4466,18 @@
           <t>Mid-term</t>
         </is>
       </c>
-      <c r="B14" s="112" t="inlineStr">
+      <c r="B14" s="116" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C14" s="113" t="inlineStr"/>
-      <c r="D14" s="113" t="inlineStr">
+      <c r="C14" s="117" t="inlineStr"/>
+      <c r="D14" s="117" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E14" s="113" t="inlineStr">
+      <c r="E14" s="117" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4461,14 +4493,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B15" s="114" t="inlineStr"/>
-      <c r="C15" s="114" t="inlineStr"/>
-      <c r="D15" s="114" t="inlineStr">
+      <c r="B15" s="118" t="inlineStr"/>
+      <c r="C15" s="118" t="inlineStr"/>
+      <c r="D15" s="118" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="E15" s="114" t="inlineStr"/>
+      <c r="E15" s="118" t="inlineStr"/>
       <c r="F15" s="39" t="inlineStr">
         <is>
           <t>Midterm Exam</t>
@@ -4481,18 +4513,18 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B16" s="112" t="inlineStr">
+      <c r="B16" s="116" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C16" s="115" t="inlineStr"/>
-      <c r="D16" s="115" t="inlineStr">
+      <c r="C16" s="119" t="inlineStr"/>
+      <c r="D16" s="119" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="E16" s="115" t="inlineStr">
+      <c r="E16" s="119" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -4508,14 +4540,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B17" s="114" t="inlineStr"/>
-      <c r="C17" s="114" t="inlineStr"/>
-      <c r="D17" s="114" t="inlineStr">
+      <c r="B17" s="118" t="inlineStr"/>
+      <c r="C17" s="118" t="inlineStr"/>
+      <c r="D17" s="118" t="inlineStr">
         <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="E17" s="114" t="inlineStr"/>
+      <c r="E17" s="118" t="inlineStr"/>
       <c r="F17" s="39" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -4528,18 +4560,18 @@
           <t>Discussion Section</t>
         </is>
       </c>
-      <c r="B18" s="112" t="inlineStr">
+      <c r="B18" s="116" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C18" s="113" t="inlineStr"/>
-      <c r="D18" s="113" t="inlineStr">
+      <c r="C18" s="117" t="inlineStr"/>
+      <c r="D18" s="117" t="inlineStr">
         <is>
           <t>2026-11-12</t>
         </is>
       </c>
-      <c r="E18" s="113" t="inlineStr">
+      <c r="E18" s="117" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -4555,18 +4587,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B19" s="114" t="inlineStr"/>
-      <c r="C19" s="114" t="inlineStr">
+      <c r="B19" s="118" t="inlineStr"/>
+      <c r="C19" s="118" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D19" s="114" t="inlineStr">
+      <c r="D19" s="118" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E19" s="114" t="inlineStr"/>
+      <c r="E19" s="118" t="inlineStr"/>
       <c r="F19" s="39" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death</t>
@@ -4579,18 +4611,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B20" s="114" t="inlineStr"/>
-      <c r="C20" s="114" t="inlineStr">
+      <c r="B20" s="118" t="inlineStr"/>
+      <c r="C20" s="118" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="D20" s="114" t="inlineStr">
+      <c r="D20" s="118" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="E20" s="114" t="inlineStr"/>
+      <c r="E20" s="118" t="inlineStr"/>
       <c r="F20" s="39" t="inlineStr">
         <is>
           <t>Week Aug 25-29: Intro &amp; Black Death - Section reading 1: Lizzie Wade, “From Black Death to fatal flu, past pandemics sho</t>
@@ -4603,18 +4635,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B21" s="114" t="inlineStr"/>
-      <c r="C21" s="114" t="inlineStr">
+      <c r="B21" s="118" t="inlineStr"/>
+      <c r="C21" s="118" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D21" s="114" t="inlineStr">
+      <c r="D21" s="118" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E21" s="114" t="inlineStr"/>
+      <c r="E21" s="118" t="inlineStr"/>
       <c r="F21" s="39" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life</t>
@@ -4627,18 +4659,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B22" s="114" t="inlineStr"/>
-      <c r="C22" s="114" t="inlineStr">
+      <c r="B22" s="118" t="inlineStr"/>
+      <c r="C22" s="118" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="D22" s="114" t="inlineStr">
+      <c r="D22" s="118" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E22" s="114" t="inlineStr"/>
+      <c r="E22" s="118" t="inlineStr"/>
       <c r="F22" s="39" t="inlineStr">
         <is>
           <t>Week Sep 1-4: Everyday Life - Section reading 1: A Roger Ekirch, “Sleep we have lost: Pre-Industrial Slumber in the Brit</t>
@@ -4651,18 +4683,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B23" s="114" t="inlineStr"/>
-      <c r="C23" s="114" t="inlineStr">
+      <c r="B23" s="118" t="inlineStr"/>
+      <c r="C23" s="118" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D23" s="114" t="inlineStr">
+      <c r="D23" s="118" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E23" s="114" t="inlineStr"/>
+      <c r="E23" s="118" t="inlineStr"/>
       <c r="F23" s="39" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance</t>
@@ -4675,18 +4707,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B24" s="114" t="inlineStr"/>
-      <c r="C24" s="114" t="inlineStr">
+      <c r="B24" s="118" t="inlineStr"/>
+      <c r="C24" s="118" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="D24" s="114" t="inlineStr">
+      <c r="D24" s="118" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E24" s="114" t="inlineStr"/>
+      <c r="E24" s="118" t="inlineStr"/>
       <c r="F24" s="39" t="inlineStr">
         <is>
           <t>Week Sep 8-11: Renaissance - Section reading 1: Kay Daly, “Diverting the Flood of History: Ada Palmer’s Inventing the Re</t>
@@ -4699,18 +4731,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B25" s="114" t="inlineStr"/>
-      <c r="C25" s="114" t="inlineStr">
+      <c r="B25" s="118" t="inlineStr"/>
+      <c r="C25" s="118" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D25" s="114" t="inlineStr">
+      <c r="D25" s="118" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E25" s="114" t="inlineStr"/>
+      <c r="E25" s="118" t="inlineStr"/>
       <c r="F25" s="39" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance</t>
@@ -4723,18 +4755,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B26" s="114" t="inlineStr"/>
-      <c r="C26" s="114" t="inlineStr">
+      <c r="B26" s="118" t="inlineStr"/>
+      <c r="C26" s="118" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="D26" s="114" t="inlineStr">
+      <c r="D26" s="118" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E26" s="114" t="inlineStr"/>
+      <c r="E26" s="118" t="inlineStr"/>
       <c r="F26" s="39" t="inlineStr">
         <is>
           <t>Week Sep 15-18: Renaissance - Section reading 1: Vasari, Lives of the Artists: Leonardo da Vinci &amp; Properzia de’ Rossi V</t>
@@ -4747,18 +4779,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B27" s="114" t="inlineStr"/>
-      <c r="C27" s="114" t="inlineStr">
+      <c r="B27" s="118" t="inlineStr"/>
+      <c r="C27" s="118" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D27" s="114" t="inlineStr">
+      <c r="D27" s="118" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E27" s="114" t="inlineStr"/>
+      <c r="E27" s="118" t="inlineStr"/>
       <c r="F27" s="39" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion</t>
@@ -4771,18 +4803,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B28" s="114" t="inlineStr"/>
-      <c r="C28" s="114" t="inlineStr">
+      <c r="B28" s="118" t="inlineStr"/>
+      <c r="C28" s="118" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D28" s="114" t="inlineStr">
+      <c r="D28" s="118" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E28" s="114" t="inlineStr"/>
+      <c r="E28" s="118" t="inlineStr"/>
       <c r="F28" s="39" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion - Section reading 1: Jerry Brotton, The Renaissance Bazaar, Chap 1 (15 pgs) Read Colu</t>
@@ -4795,18 +4827,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B29" s="114" t="inlineStr"/>
-      <c r="C29" s="114" t="inlineStr">
+      <c r="B29" s="118" t="inlineStr"/>
+      <c r="C29" s="118" t="inlineStr">
         <is>
           <t>2026-09-20</t>
         </is>
       </c>
-      <c r="D29" s="114" t="inlineStr">
+      <c r="D29" s="118" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E29" s="114" t="inlineStr"/>
+      <c r="E29" s="118" t="inlineStr"/>
       <c r="F29" s="39" t="inlineStr">
         <is>
           <t>Week Sep 20-24: European Expansion - Section reading 2: Bernal Diaz del Castillo, The True History of the Conquest of Ne</t>
@@ -4819,18 +4851,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B30" s="114" t="inlineStr"/>
-      <c r="C30" s="114" t="inlineStr">
+      <c r="B30" s="118" t="inlineStr"/>
+      <c r="C30" s="118" t="inlineStr">
         <is>
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="D30" s="114" t="inlineStr">
+      <c r="D30" s="118" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E30" s="114" t="inlineStr"/>
+      <c r="E30" s="118" t="inlineStr"/>
       <c r="F30" s="39" t="inlineStr">
         <is>
           <t>Week Oct 6-9: Midterm &amp; Break</t>
@@ -4843,18 +4875,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B31" s="114" t="inlineStr"/>
-      <c r="C31" s="114" t="inlineStr">
+      <c r="B31" s="118" t="inlineStr"/>
+      <c r="C31" s="118" t="inlineStr">
         <is>
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="D31" s="114" t="inlineStr">
+      <c r="D31" s="118" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="E31" s="114" t="inlineStr"/>
+      <c r="E31" s="118" t="inlineStr"/>
       <c r="F31" s="39" t="inlineStr">
         <is>
           <t>Week Oct 13-16: The Reformation</t>
@@ -4867,18 +4899,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B32" s="114" t="inlineStr"/>
-      <c r="C32" s="114" t="inlineStr">
+      <c r="B32" s="118" t="inlineStr"/>
+      <c r="C32" s="118" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>
       </c>
-      <c r="D32" s="114" t="inlineStr">
+      <c r="D32" s="118" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="E32" s="114" t="inlineStr"/>
+      <c r="E32" s="118" t="inlineStr"/>
       <c r="F32" s="39" t="inlineStr">
         <is>
           <t>Week Oct 20-23: The Reformation</t>
@@ -4891,18 +4923,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B33" s="114" t="inlineStr"/>
-      <c r="C33" s="114" t="inlineStr">
+      <c r="B33" s="118" t="inlineStr"/>
+      <c r="C33" s="118" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D33" s="114" t="inlineStr">
+      <c r="D33" s="118" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E33" s="114" t="inlineStr"/>
+      <c r="E33" s="118" t="inlineStr"/>
       <c r="F33" s="39" t="inlineStr">
         <is>
           <t>Week Oct 27-30: Reformation</t>
@@ -4915,18 +4947,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B34" s="114" t="inlineStr"/>
-      <c r="C34" s="114" t="inlineStr">
+      <c r="B34" s="118" t="inlineStr"/>
+      <c r="C34" s="118" t="inlineStr">
         <is>
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="D34" s="114" t="inlineStr">
+      <c r="D34" s="118" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E34" s="114" t="inlineStr"/>
+      <c r="E34" s="118" t="inlineStr"/>
       <c r="F34" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Week Oct 27-30: Reformation - Section reading 1: Barbara Diefendorf, ed., The Saint Bartholomew’s Day Massacre: A Brief </t>
@@ -4939,18 +4971,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B35" s="114" t="inlineStr"/>
-      <c r="C35" s="114" t="inlineStr">
+      <c r="B35" s="118" t="inlineStr"/>
+      <c r="C35" s="118" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D35" s="114" t="inlineStr">
+      <c r="D35" s="118" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E35" s="114" t="inlineStr"/>
+      <c r="E35" s="118" t="inlineStr"/>
       <c r="F35" s="39" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science</t>
@@ -4963,18 +4995,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B36" s="114" t="inlineStr"/>
-      <c r="C36" s="114" t="inlineStr">
+      <c r="B36" s="118" t="inlineStr"/>
+      <c r="C36" s="118" t="inlineStr">
         <is>
           <t>2026-11-03</t>
         </is>
       </c>
-      <c r="D36" s="114" t="inlineStr">
+      <c r="D36" s="118" t="inlineStr">
         <is>
           <t>2026-11-06</t>
         </is>
       </c>
-      <c r="E36" s="114" t="inlineStr"/>
+      <c r="E36" s="118" t="inlineStr"/>
       <c r="F36" s="39" t="inlineStr">
         <is>
           <t>Week Nov 3-6: Witches &amp; Science - Section reading 1: Brian Levack, The Witchcraft Sourcebook, Chaps 36-44, 46-47</t>
@@ -4987,18 +5019,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B37" s="114" t="inlineStr"/>
-      <c r="C37" s="114" t="inlineStr">
+      <c r="B37" s="118" t="inlineStr"/>
+      <c r="C37" s="118" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D37" s="114" t="inlineStr">
+      <c r="D37" s="118" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E37" s="114" t="inlineStr"/>
+      <c r="E37" s="118" t="inlineStr"/>
       <c r="F37" s="39" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment</t>
@@ -5011,18 +5043,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B38" s="114" t="inlineStr"/>
-      <c r="C38" s="114" t="inlineStr">
+      <c r="B38" s="118" t="inlineStr"/>
+      <c r="C38" s="118" t="inlineStr">
         <is>
           <t>2026-11-10</t>
         </is>
       </c>
-      <c r="D38" s="114" t="inlineStr">
+      <c r="D38" s="118" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E38" s="114" t="inlineStr"/>
+      <c r="E38" s="118" t="inlineStr"/>
       <c r="F38" s="39" t="inlineStr">
         <is>
           <t>Week Nov 10-13: Enlightenment - Section reading 1: Excerpt: John Locke, Two Treatises of Government (1689) Excerpt: Rous</t>
@@ -5035,18 +5067,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B39" s="114" t="inlineStr"/>
-      <c r="C39" s="114" t="inlineStr">
+      <c r="B39" s="118" t="inlineStr"/>
+      <c r="C39" s="118" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D39" s="114" t="inlineStr">
+      <c r="D39" s="118" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E39" s="114" t="inlineStr"/>
+      <c r="E39" s="118" t="inlineStr"/>
       <c r="F39" s="39" t="inlineStr">
         <is>
           <t>Week Nov 17-20: Enlightenment</t>
@@ -5059,18 +5091,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B40" s="114" t="inlineStr"/>
-      <c r="C40" s="114" t="inlineStr">
+      <c r="B40" s="118" t="inlineStr"/>
+      <c r="C40" s="118" t="inlineStr">
         <is>
           <t>2026-11-17</t>
         </is>
       </c>
-      <c r="D40" s="114" t="inlineStr">
+      <c r="D40" s="118" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E40" s="114" t="inlineStr"/>
+      <c r="E40" s="118" t="inlineStr"/>
       <c r="F40" s="39" t="inlineStr">
         <is>
           <t xml:space="preserve">Week Nov 17-20: Enlightenment - Section reading 1: Video: Africa &amp; Britain, A Forgotten History, Episode 2: Freedom (50 </t>
@@ -5083,18 +5115,18 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B41" s="114" t="inlineStr"/>
-      <c r="C41" s="114" t="inlineStr">
+      <c r="B41" s="118" t="inlineStr"/>
+      <c r="C41" s="118" t="inlineStr">
         <is>
           <t>2026-12-01</t>
         </is>
       </c>
-      <c r="D41" s="114" t="inlineStr">
+      <c r="D41" s="118" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E41" s="114" t="inlineStr"/>
+      <c r="E41" s="118" t="inlineStr"/>
       <c r="F41" s="39" t="inlineStr">
         <is>
           <t>Week Dec 1-4: Modern Europe?</t>
@@ -5107,18 +5139,18 @@
           <t>Identification Quizzes</t>
         </is>
       </c>
-      <c r="B42" s="112" t="inlineStr">
+      <c r="B42" s="116" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C42" s="115" t="inlineStr"/>
-      <c r="D42" s="115" t="inlineStr">
+      <c r="C42" s="119" t="inlineStr"/>
+      <c r="D42" s="119" t="inlineStr">
         <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="E42" s="115" t="inlineStr">
+      <c r="E42" s="119" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5134,18 +5166,18 @@
           <t>Extra Credit</t>
         </is>
       </c>
-      <c r="B43" s="112" t="inlineStr">
+      <c r="B43" s="116" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C43" s="113" t="inlineStr"/>
-      <c r="D43" s="113" t="inlineStr">
+      <c r="C43" s="117" t="inlineStr"/>
+      <c r="D43" s="117" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E43" s="113" t="inlineStr">
+      <c r="E43" s="117" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Add ECON-351 Marshall grading-policies syllabus parser
Parse Grading Policies percentage table and embedded COURSE CALENDAR
for ECON-351: four midterms, homework sub-rows, AI project parts,
and WSJ extra credit. Distinguish point calendars (BUAD-281) from
full syllabi with schedule tables. Add RMP entry for Martínez-Marquina.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-304" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-281" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ECON-351" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="31">
+  <fonts count="33">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -165,8 +166,18 @@
       <color rgb="00808080"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009467BD"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009467BD"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="31">
+  <fills count="37">
     <fill>
       <patternFill/>
     </fill>
@@ -318,6 +329,36 @@
         <fgColor rgb="00EFF5F9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="009467BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7DDF0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEE8F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E1D4EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FAF8FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F4FA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -389,7 +430,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="120">
+  <cellXfs count="146">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -714,6 +755,82 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="31" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="33" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="34" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="33" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="36" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="36" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="34" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="34" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1082,7 +1199,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1237,60 +1354,96 @@
     </row>
     <row r="8" hidden="1" outlineLevel="1">
       <c r="A8" s="7">
+        <f>HYPERLINK("#'ECON-351'!A1","ECON-351")</f>
+        <v/>
+      </c>
+      <c r="B8" s="88" t="inlineStr">
+        <is>
+          <t>Alejandro Martínez-Marquina / João Ramos</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>A- (3.76) [39/62 reported]</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>85.2%</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" hidden="1" outlineLevel="1">
+      <c r="A9" s="10">
         <f>HYPERLINK("#'HIST-103'!A1","HIST-103")</f>
         <v/>
       </c>
-      <c r="B8" s="88" t="inlineStr">
+      <c r="B9" s="89" t="inlineStr">
         <is>
           <t>Lindsay O'Neill</t>
         </is>
       </c>
-      <c r="C8" s="26" t="inlineStr">
+      <c r="C9" s="90" t="inlineStr">
         <is>
           <t>4.3</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E9" s="11" t="inlineStr">
         <is>
           <t>A- (3.77) [27/54 reported]</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F9" s="11" t="inlineStr">
         <is>
           <t>79.3%</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="G9" s="11" t="inlineStr">
         <is>
           <t>54</t>
         </is>
       </c>
     </row>
-    <row r="9" hidden="1" outlineLevel="1"/>
-    <row r="10" hidden="1" outlineLevel="1">
-      <c r="A10" s="13" t="inlineStr">
+    <row r="10" hidden="1" outlineLevel="1"/>
+    <row r="11" hidden="1" outlineLevel="1">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>Consensus - recurring student review themes</t>
         </is>
       </c>
     </row>
-    <row r="11" hidden="1" outlineLevel="1" ht="135" customHeight="1">
-      <c r="A11" s="104" t="inlineStr">
+    <row r="12" hidden="1" outlineLevel="1" ht="135" customHeight="1">
+      <c r="A12" s="104" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="B11" s="105" t="inlineStr">
+      <c r="B12" s="105" t="inlineStr">
         <is>
           <t>George Braunegg</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>STRENGTHS: Very high marks for personality and support — students call Prof. Braunegg kind, funny, caring, and responsive by email. Daily accounting facts/jokes are a recurring positive. Many praise his career advice and willingness to help outside class; several credit him with influencing their major choice.
 TEACHING &amp; EXAMS: More divided on in-class instruction — some say he struggles to work through problems live or that lectures don't always align with exams. Course draws on Prof. Layton's materials but sections may not match perfectly. Textbook gets criticism.
@@ -1298,18 +1451,18 @@
         </is>
       </c>
     </row>
-    <row r="12" hidden="1" outlineLevel="1" ht="135" customHeight="1">
-      <c r="A12" s="106" t="inlineStr">
+    <row r="13" hidden="1" outlineLevel="1" ht="135" customHeight="1">
+      <c r="A13" s="106" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="B12" s="107" t="inlineStr">
+      <c r="B13" s="107" t="inlineStr">
         <is>
           <t>Christine El Haddad</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>STRENGTHS: Among the most praised Marshall professors on RMP — repeatedly called the 'best' or 'sweetest' instructor students have had. Negotiation and OB classes get standout reviews: supportive classroom culture, clear and organized Brightspace, strong lectures, and generous extra credit. Weekly in-class negotiations are a highlight for many.
 WORKLOAD: Group projects and class participation carry real weight; some find readings or lecture content repetitive. A few note group work can feel heavy even when the professor is beloved.
@@ -1317,18 +1470,37 @@
         </is>
       </c>
     </row>
-    <row r="13" hidden="1" outlineLevel="1" ht="135" customHeight="1">
-      <c r="A13" s="104" t="inlineStr">
+    <row r="14" hidden="1" outlineLevel="1" ht="120" customHeight="1">
+      <c r="A14" s="104" t="inlineStr">
+        <is>
+          <t>ECON-351</t>
+        </is>
+      </c>
+      <c r="B14" s="105" t="inlineStr">
+        <is>
+          <t>Alejandro Martínez-Marquina / João Ramos</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>STRENGTHS: Martínez-Marquina earns strong marks for clear board work, practice problems, and supportive TAs; students say concepts click when you attend and use office hours. Ramos sections get mixed reviews — some praise exam alignment with practice problems, others find lectures hard to follow due to pace/accent.
+GRADING &amp; WORKLOAD: Four non-cumulative midterms (20% each) plus weekly Brightspace homework (best 10 of 12 count). AI Forecast Project is individual. Letter grades follow Marshall guidelines with rough bands (A above ~85%, B 70–85%, C 60–70%).
+BOTTOM LINE: Engage with practice problems and TAs; homework drops give flexibility. WSJ Future View offers optional +10% extra credit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" hidden="1" outlineLevel="1" ht="135" customHeight="1">
+      <c r="A15" s="106" t="inlineStr">
         <is>
           <t>HIST-103</t>
         </is>
       </c>
-      <c r="B13" s="105" t="inlineStr">
+      <c r="B15" s="107" t="inlineStr">
         <is>
           <t>Lindsay O'Neill</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>STRENGTHS: Students consistently describe Dr. O'Neill as passionate and engaging — lectures use multimedia (Monty Python clips, movie trailers, humor) that make a GE history class feel lively rather than dry. Many say the content is genuinely interesting if you show up and pay attention.
 GRADING &amp; WORKLOAD: Mixed reviews on grading — several note she can be a harsh essay grader and that strong discussion participation matters. Expect substantial section readings; essays benefit from office-hours or TA help. Low-weight pop quizzes (~5% total) sometimes used to track attendance.
@@ -1336,584 +1508,559 @@
         </is>
       </c>
     </row>
-    <row r="14" hidden="1" outlineLevel="1">
-      <c r="A14" s="91" t="inlineStr">
+    <row r="16" hidden="1" outlineLevel="1">
+      <c r="A16" s="91" t="inlineStr">
         <is>
           <t>RMP data as of 2026-08-21. Source: ratemyprofessors.com. Avg reviewer grade = mean of self-reported letter grades (4.0 scale); not all reviewers report a grade.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Connect prep (e.g. BUAD-304 Personal Assessments) is ungraded class prep - not part of Participation or other graded categories.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="32" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Start here (graded): 2026-09-09 - BUAD-281 - Homework: Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Start here (graded): 2026-09-04 - ECON-351 - Homework: Homework 1 (Chapter 4) — Brightspace, due 11:59 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Reading</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>Papers</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>Group Project</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>External certs</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>Connect prep</t>
         </is>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>First assignment</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="I21" s="6" t="inlineStr">
         <is>
           <t>Assign due</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr">
+      <c r="J21" s="6" t="inlineStr">
         <is>
           <t>First major</t>
         </is>
       </c>
-      <c r="K19" s="6" t="inlineStr">
+      <c r="K21" s="6" t="inlineStr">
         <is>
           <t>Major due</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="7">
+    <row r="22">
+      <c r="A22" s="7">
         <f>HYPERLINK("#'BUAD-281'!A1","BUAD-281")</f>
         <v/>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>LinkedIn Learning Excel Certification, Stukent Simternship</t>
         </is>
       </c>
-      <c r="G20" s="8" t="inlineStr">
+      <c r="G22" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H20" s="8" t="inlineStr">
+      <c r="H22" s="8" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
         </is>
       </c>
-      <c r="I20" s="8" t="inlineStr">
+      <c r="I22" s="8" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="J20" s="8" t="inlineStr">
+      <c r="J22" s="8" t="inlineStr">
         <is>
           <t>Midterm 1</t>
         </is>
       </c>
-      <c r="K20" s="8" t="inlineStr">
+      <c r="K22" s="8" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="10">
+    <row r="23">
+      <c r="A23" s="10">
         <f>HYPERLINK("#'BUAD-304'!A1","BUAD-304")</f>
         <v/>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D21" s="11" t="inlineStr">
+      <c r="D23" s="11" t="inlineStr">
         <is>
           <t>Final Reflection Paper, Team Project Paper</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E23" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F21" s="11" t="inlineStr">
+      <c r="F23" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G21" s="12" t="inlineStr">
+      <c r="G23" s="12" t="inlineStr">
         <is>
           <t>Ungraded prep</t>
         </is>
       </c>
-      <c r="H21" s="11" t="inlineStr">
+      <c r="H23" s="11" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.01 - What is my Big thinking</t>
         </is>
       </c>
-      <c r="I21" s="11" t="inlineStr">
+      <c r="I23" s="11" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="J21" s="11" t="inlineStr">
+      <c r="J23" s="11" t="inlineStr">
         <is>
           <t>Thomas Green Case Analysis Memo</t>
         </is>
       </c>
-      <c r="K21" s="11" t="inlineStr">
+      <c r="K23" s="11" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="7">
+    <row r="24">
+      <c r="A24" s="7">
+        <f>HYPERLINK("#'ECON-351'!A1","ECON-351")</f>
+        <v/>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>Homework 1 (Chapter 4) — Brightspace, due 11:59 pm</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>First midterm exam</t>
+        </is>
+      </c>
+      <c r="K24" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10">
         <f>HYPERLINK("#'HIST-103'!A1","HIST-103")</f>
         <v/>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>Sleep Paper, Witchcraft Paper</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F25" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G22" s="8" t="inlineStr">
+      <c r="G25" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H22" s="8" t="inlineStr">
+      <c r="H25" s="11" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
         </is>
       </c>
-      <c r="I22" s="8" t="inlineStr">
+      <c r="I25" s="11" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="J22" s="8" t="inlineStr">
+      <c r="J25" s="11" t="inlineStr">
         <is>
           <t>Sleep Paper</t>
         </is>
       </c>
-      <c r="K22" s="8" t="inlineStr">
+      <c r="K25" s="11" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="13" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>Do First - August 2026 - graded assignments (first per class always listed)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="14" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="C25" s="14" t="inlineStr">
+      <c r="C28" s="14" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr">
+      <c r="D28" s="14" t="inlineStr">
         <is>
           <t>Graded?</t>
         </is>
       </c>
-      <c r="E25" s="14" t="inlineStr">
+      <c r="E28" s="14" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>ECON-351</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Homework 1 (Chapter 4) — Brightspace, due 11:59 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C26" s="15" t="inlineStr">
+      <c r="C30" s="46" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
+      <c r="D30" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="11" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>HIST-103</t>
         </is>
       </c>
-      <c r="C27" s="16" t="inlineStr">
+      <c r="C31" s="25" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D27" s="11" t="inlineStr">
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="E31" s="8" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="17" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>Do First - August 2026 - Connect prep only (ungraded, not Participation)</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="18" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="B30" s="18" t="inlineStr">
+      <c r="B34" s="18" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="C30" s="18" t="inlineStr">
+      <c r="C34" s="18" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D30" s="18" t="inlineStr">
+      <c r="D34" s="18" t="inlineStr">
         <is>
           <t>Graded?</t>
         </is>
       </c>
-      <c r="E30" s="18" t="inlineStr">
+      <c r="E34" s="18" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="19" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B31" s="19" t="inlineStr">
+      <c r="B35" s="19" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C31" s="20" t="inlineStr">
+      <c r="C35" s="20" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D31" s="21" t="inlineStr">
+      <c r="D35" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E31" s="19" t="inlineStr">
+      <c r="E35" s="19" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="22" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="22" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B32" s="22" t="inlineStr">
+      <c r="B36" s="22" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C32" s="23" t="inlineStr">
+      <c r="C36" s="23" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D32" s="24" t="inlineStr">
+      <c r="D36" s="24" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E32" s="22" t="inlineStr">
+      <c r="E36" s="22" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="13" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
         <is>
           <t>Upcoming graded assignments (next 45 days)</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="14" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="B35" s="14" t="inlineStr">
+      <c r="B39" s="14" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="C35" s="14" t="inlineStr">
+      <c r="C39" s="14" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D35" s="14" t="inlineStr">
+      <c r="D39" s="14" t="inlineStr">
         <is>
           <t>Graded?</t>
         </is>
       </c>
-      <c r="E35" s="14" t="inlineStr">
+      <c r="E39" s="14" t="inlineStr">
         <is>
           <t>Item</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>BUAD-281</t>
-        </is>
-      </c>
-      <c r="C36" s="15" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="B37" s="11" t="inlineStr">
-        <is>
-          <t>HIST-103</t>
-        </is>
-      </c>
-      <c r="C37" s="16" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="D37" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E37" s="11" t="inlineStr">
-        <is>
-          <t>Sleep Paper Due</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>HIST-103</t>
-        </is>
-      </c>
-      <c r="C38" s="25" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>Sleep Paper</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="B39" s="11" t="inlineStr">
-        <is>
-          <t>BUAD-281</t>
-        </is>
-      </c>
-      <c r="C39" s="46" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="D39" s="11" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E39" s="11" t="inlineStr">
-        <is>
-          <t>Class 7 (9/16) - 3-24, 3-28, 3-32; 15 Points</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>BUAD-304</t>
-        </is>
-      </c>
-      <c r="C40" s="25" t="inlineStr">
-        <is>
-          <t>Assignment</t>
+          <t>ECON-351</t>
+        </is>
+      </c>
+      <c r="C40" s="15" t="inlineStr">
+        <is>
+          <t>Homework</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
@@ -1923,24 +2070,24 @@
       </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t>Thomas Green Case Analysis Memo</t>
+          <t>Homework 1 (Chapter 4) — Brightspace, due 11:59 pm</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="11" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
-          <t>HIST-103</t>
-        </is>
-      </c>
-      <c r="C41" s="16" t="inlineStr">
-        <is>
-          <t>Assignment</t>
+          <t>BUAD-281</t>
+        </is>
+      </c>
+      <c r="C41" s="46" t="inlineStr">
+        <is>
+          <t>Homework</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
@@ -1950,19 +2097,19 @@
       </c>
       <c r="E41" s="11" t="inlineStr">
         <is>
-          <t>Final Exam</t>
+          <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>BUAD-281</t>
+          <t>ECON-351</t>
         </is>
       </c>
       <c r="C42" s="15" t="inlineStr">
@@ -1977,24 +2124,24 @@
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>Class 8 (9/21) - 5-27 5-46; 10 Points</t>
+          <t>Homework 2 (Chapter 9) — Brightspace, due 11:59 pm</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="11" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B43" s="11" t="inlineStr">
         <is>
-          <t>BUAD-281</t>
-        </is>
-      </c>
-      <c r="C43" s="46" t="inlineStr">
-        <is>
-          <t>Homework</t>
+          <t>ECON-351</t>
+        </is>
+      </c>
+      <c r="C43" s="120" t="inlineStr">
+        <is>
+          <t>Exam</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
@@ -2004,24 +2151,24 @@
       </c>
       <c r="E43" s="11" t="inlineStr">
         <is>
-          <t>Class 9 (9/23) - 4-21, 4-22; 10 Points</t>
+          <t>Midterm 1 — covers Chapters 4 and 9</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>BUAD-304</t>
-        </is>
-      </c>
-      <c r="C44" s="26" t="inlineStr">
-        <is>
-          <t>Research</t>
+          <t>ECON-351</t>
+        </is>
+      </c>
+      <c r="C44" s="25" t="inlineStr">
+        <is>
+          <t>Assignment</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
@@ -2031,24 +2178,24 @@
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t>Research: Setup deadline (registration, prescreening, contacts)</t>
+          <t>First midterm exam</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="11" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B45" s="11" t="inlineStr">
         <is>
-          <t>BUAD-281</t>
-        </is>
-      </c>
-      <c r="C45" s="46" t="inlineStr">
-        <is>
-          <t>Homework</t>
+          <t>HIST-103</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>Assignment</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr">
@@ -2058,19 +2205,19 @@
       </c>
       <c r="E45" s="11" t="inlineStr">
         <is>
-          <t>Class 10 (9/28) - 8-28, 8-29; 10 Points</t>
+          <t>Sleep Paper Due</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>BUAD-304</t>
+          <t>HIST-103</t>
         </is>
       </c>
       <c r="C46" s="25" t="inlineStr">
@@ -2085,24 +2232,24 @@
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>Team project proposal &amp; team contract</t>
+          <t>Sleep Paper</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="11" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B47" s="11" t="inlineStr">
         <is>
-          <t>BUAD-304</t>
-        </is>
-      </c>
-      <c r="C47" s="16" t="inlineStr">
-        <is>
-          <t>Assignment</t>
+          <t>BUAD-281</t>
+        </is>
+      </c>
+      <c r="C47" s="46" t="inlineStr">
+        <is>
+          <t>Homework</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr">
@@ -2112,24 +2259,24 @@
       </c>
       <c r="E47" s="11" t="inlineStr">
         <is>
-          <t>Proposal &amp; Team Contract</t>
+          <t>Class 7 (9/16) - 3-24, 3-28, 3-32; 15 Points</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>BUAD-281</t>
-        </is>
-      </c>
-      <c r="C48" s="47" t="inlineStr">
-        <is>
-          <t>Exam</t>
+          <t>BUAD-304</t>
+        </is>
+      </c>
+      <c r="C48" s="25" t="inlineStr">
+        <is>
+          <t>Assignment</t>
         </is>
       </c>
       <c r="D48" s="8" t="inlineStr">
@@ -2139,58 +2286,384 @@
       </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t>9/30 Midterm 1: 250 Points Chapters 1, 2, 3, 4, 5, 8</t>
+          <t>Thomas Green Case Analysis Memo</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="11" t="inlineStr">
         <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>HIST-103</t>
+        </is>
+      </c>
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E49" s="11" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>ECON-351</t>
+        </is>
+      </c>
+      <c r="C50" s="15" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Homework 3 — Brightspace, due 11:59 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>BUAD-281</t>
+        </is>
+      </c>
+      <c r="C51" s="46" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="D51" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E51" s="11" t="inlineStr">
+        <is>
+          <t>Class 8 (9/21) - 5-27 5-46; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>BUAD-281</t>
+        </is>
+      </c>
+      <c r="C52" s="15" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Class 9 (9/23) - 4-21, 4-22; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B53" s="11" t="inlineStr">
+        <is>
+          <t>ECON-351</t>
+        </is>
+      </c>
+      <c r="C53" s="46" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="D53" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E53" s="11" t="inlineStr">
+        <is>
+          <t>Homework 4 (Chapter 3) — Brightspace, due 11:59 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>BUAD-304</t>
+        </is>
+      </c>
+      <c r="C54" s="26" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>Research: Setup deadline (registration, prescreening, contacts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B55" s="11" t="inlineStr">
+        <is>
+          <t>BUAD-281</t>
+        </is>
+      </c>
+      <c r="C55" s="46" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="D55" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E55" s="11" t="inlineStr">
+        <is>
+          <t>Class 10 (9/28) - 8-28, 8-29; 10 Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>BUAD-304</t>
+        </is>
+      </c>
+      <c r="C56" s="25" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>Team project proposal &amp; team contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B57" s="11" t="inlineStr">
+        <is>
+          <t>BUAD-304</t>
+        </is>
+      </c>
+      <c r="C57" s="16" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="D57" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E57" s="11" t="inlineStr">
+        <is>
+          <t>Proposal &amp; Team Contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
+        <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B49" s="11" t="inlineStr">
+      <c r="B58" s="8" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C49" s="16" t="inlineStr">
+      <c r="C58" s="47" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>9/30 Midterm 1: 250 Points Chapters 1, 2, 3, 4, 5, 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B59" s="11" t="inlineStr">
+        <is>
+          <t>BUAD-281</t>
+        </is>
+      </c>
+      <c r="C59" s="16" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D49" s="11" t="inlineStr">
+      <c r="D59" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E49" s="11" t="inlineStr">
+      <c r="E59" s="11" t="inlineStr">
         <is>
           <t>Midterm 1</t>
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>ECON-351</t>
+        </is>
+      </c>
+      <c r="C60" s="15" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>Homework 5 (Chapter 5) — Brightspace, due 11:59 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B61" s="11" t="inlineStr">
+        <is>
+          <t>ECON-351</t>
+        </is>
+      </c>
+      <c r="C61" s="16" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="D61" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E61" s="11" t="inlineStr">
+        <is>
+          <t>AI Forecast Project — Part I</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="A34:K34"/>
+  <mergeCells count="15">
+    <mergeCell ref="C15:K15"/>
+    <mergeCell ref="A18:K18"/>
     <mergeCell ref="A4:K4"/>
-    <mergeCell ref="C11:K11"/>
     <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A29:K29"/>
+    <mergeCell ref="C14:K14"/>
     <mergeCell ref="C13:K13"/>
     <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A11:K11"/>
     <mergeCell ref="A16:K16"/>
-    <mergeCell ref="A17:K17"/>
-    <mergeCell ref="A10:K10"/>
-    <mergeCell ref="A24:K24"/>
-    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="A19:K19"/>
+    <mergeCell ref="A33:K33"/>
+    <mergeCell ref="A38:K38"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="C12:K12"/>
+    <mergeCell ref="A27:K27"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5208,4 +5681,1166 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="009467BD"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="121" t="inlineStr">
+        <is>
+          <t>ECON-351 — Microeconomics for Business</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="28">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/sources/econ-351-source.pdf","SEE HERE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="29" t="inlineStr">
+        <is>
+          <t>Instructor</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Alejandro Martínez-Marquina / João Ramos</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fall 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>Required for an A</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>85%+ (rough guideline)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>Grading scale</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Each course requirement receives a numerical score but not a letter grade. The overall numerical score in the course is converted into a letter grade at the end of the semester in accordance with the Marshall School guidelines. The instructor’s evaluation of the performance of each individual student is the final basis for assigning grades. Each student will be given a grade based on the student's performance in class and demonstrated mastery of the course learning objectives. In the past, students with grades below 60% received either a D or an F (below 50%) in the course. Students with grades between 60% and 70% received a C, 70% and 85% a B, and above 85% an A. However, I emphasize again that these are only rough guidelines – grades will be determined as specified above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="122" t="inlineStr">
+        <is>
+          <t>First midterm exam 20%  |  Second midterm exam 20%  |  Third midterm exam 20%  |  Fourth midterm exam 20%  |  AI Forecast Project 10%  |  Homework 10%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="123" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B9" s="123" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="C9" s="123" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="D9" s="123" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="E9" s="123" t="inlineStr">
+        <is>
+          <t>Group Project</t>
+        </is>
+      </c>
+      <c r="F9" s="123" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="124" t="inlineStr">
+        <is>
+          <t>First midterm exam</t>
+        </is>
+      </c>
+      <c r="B10" s="142" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="C10" s="143" t="inlineStr"/>
+      <c r="D10" s="143" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="E10" s="143" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" s="127">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/econ-351-first-midterm-exam.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="128" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="B11" s="144" t="inlineStr"/>
+      <c r="C11" s="144" t="inlineStr"/>
+      <c r="D11" s="144" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="E11" s="144" t="inlineStr"/>
+      <c r="F11" s="130" t="inlineStr">
+        <is>
+          <t>Midterm 1 — covers Chapters 4 and 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="131" t="inlineStr">
+        <is>
+          <t>Second midterm exam</t>
+        </is>
+      </c>
+      <c r="B12" s="142" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="C12" s="145" t="inlineStr"/>
+      <c r="D12" s="145" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E12" s="145" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F12" s="133">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/econ-351-second-midterm-exam.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="128" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="B13" s="144" t="inlineStr"/>
+      <c r="C13" s="144" t="inlineStr"/>
+      <c r="D13" s="144" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E13" s="144" t="inlineStr"/>
+      <c r="F13" s="130" t="inlineStr">
+        <is>
+          <t>Midterm 2 — covers Chapters 3, 5, and 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="124" t="inlineStr">
+        <is>
+          <t>Third midterm exam</t>
+        </is>
+      </c>
+      <c r="B14" s="142" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="C14" s="143" t="inlineStr"/>
+      <c r="D14" s="143" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="E14" s="143" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F14" s="127">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/econ-351-third-midterm-exam.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="128" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="B15" s="144" t="inlineStr"/>
+      <c r="C15" s="144" t="inlineStr"/>
+      <c r="D15" s="144" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="E15" s="144" t="inlineStr"/>
+      <c r="F15" s="130" t="inlineStr">
+        <is>
+          <t>Midterm 3 — covers Chapters 7, 8, and 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="131" t="inlineStr">
+        <is>
+          <t>Fourth midterm exam</t>
+        </is>
+      </c>
+      <c r="B16" s="142" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="C16" s="145" t="inlineStr"/>
+      <c r="D16" s="145" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E16" s="145" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F16" s="133">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/econ-351-fourth-midterm-exam.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="128" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="B17" s="144" t="inlineStr"/>
+      <c r="C17" s="144" t="inlineStr"/>
+      <c r="D17" s="144" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E17" s="144" t="inlineStr"/>
+      <c r="F17" s="130" t="inlineStr">
+        <is>
+          <t>Midterm 4 — covers Chapters 11, 12, and 13</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="124" t="inlineStr">
+        <is>
+          <t>AI Forecast Project</t>
+        </is>
+      </c>
+      <c r="B18" s="142" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C18" s="143" t="inlineStr"/>
+      <c r="D18" s="143" t="inlineStr">
+        <is>
+          <t>2026-12-11</t>
+        </is>
+      </c>
+      <c r="E18" s="143" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F18" s="127">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/econ-351-ai-forecast-project.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="134" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B19" s="144" t="inlineStr"/>
+      <c r="C19" s="144" t="inlineStr"/>
+      <c r="D19" s="144" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="E19" s="144" t="inlineStr"/>
+      <c r="F19" s="130" t="inlineStr">
+        <is>
+          <t>AI Forecast Project — Part I</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="134" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B20" s="144" t="inlineStr"/>
+      <c r="C20" s="144" t="inlineStr"/>
+      <c r="D20" s="144" t="inlineStr">
+        <is>
+          <t>2026-12-11</t>
+        </is>
+      </c>
+      <c r="E20" s="144" t="inlineStr"/>
+      <c r="F20" s="130" t="inlineStr">
+        <is>
+          <t>AI Forecast Project — Part II</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="131" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B21" s="142" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C21" s="145" t="inlineStr"/>
+      <c r="D21" s="145" t="inlineStr">
+        <is>
+          <t>2026-11-27</t>
+        </is>
+      </c>
+      <c r="E21" s="145" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F21" s="133">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/econ-351-homework.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B22" s="144" t="inlineStr"/>
+      <c r="C22" s="144" t="inlineStr"/>
+      <c r="D22" s="144" t="inlineStr"/>
+      <c r="E22" s="144" t="inlineStr"/>
+      <c r="F22" s="130" t="inlineStr">
+        <is>
+          <t>Finals Week: - AI Project – Part II due December 11</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B23" s="144" t="inlineStr"/>
+      <c r="C23" s="144" t="inlineStr"/>
+      <c r="D23" s="144" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="E23" s="144" t="inlineStr"/>
+      <c r="F23" s="130" t="inlineStr">
+        <is>
+          <t>Week 1: Aug.24/26 - Complete the math self-assessment on Brightspace</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B24" s="144" t="inlineStr"/>
+      <c r="C24" s="144" t="inlineStr"/>
+      <c r="D24" s="144" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="E24" s="144" t="inlineStr"/>
+      <c r="F24" s="130" t="inlineStr">
+        <is>
+          <t>Week 1: Aug.24/26 - Read Chapters 2 and 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B25" s="144" t="inlineStr"/>
+      <c r="C25" s="144" t="inlineStr"/>
+      <c r="D25" s="144" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="E25" s="144" t="inlineStr"/>
+      <c r="F25" s="130" t="inlineStr">
+        <is>
+          <t>Week 1: Aug.24/26 - Read the syllabus</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B26" s="144" t="inlineStr"/>
+      <c r="C26" s="144" t="inlineStr"/>
+      <c r="D26" s="144" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="E26" s="144" t="inlineStr"/>
+      <c r="F26" s="130" t="inlineStr">
+        <is>
+          <t>Week 2: Aug.31/Sep.2 - Begin Chapter 9: Uncertainty</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B27" s="144" t="inlineStr"/>
+      <c r="C27" s="144" t="inlineStr"/>
+      <c r="D27" s="144" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="E27" s="144" t="inlineStr"/>
+      <c r="F27" s="130" t="inlineStr">
+        <is>
+          <t>Week 2: Aug.31/Sep.2 - Finish reading Chapter 4 (in-class dis- cussion)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="136" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B28" s="144" t="inlineStr"/>
+      <c r="C28" s="144" t="inlineStr"/>
+      <c r="D28" s="144" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="E28" s="144" t="inlineStr"/>
+      <c r="F28" s="130" t="inlineStr">
+        <is>
+          <t>Homework 1 (Chapter 4) — Brightspace, due 11:59 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B29" s="144" t="inlineStr"/>
+      <c r="C29" s="144" t="inlineStr"/>
+      <c r="D29" s="144" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E29" s="144" t="inlineStr"/>
+      <c r="F29" s="130" t="inlineStr">
+        <is>
+          <t>Week 3: Sep.7/9 - Discussion of Chapter 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B30" s="144" t="inlineStr"/>
+      <c r="C30" s="144" t="inlineStr"/>
+      <c r="D30" s="144" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E30" s="144" t="inlineStr"/>
+      <c r="F30" s="130" t="inlineStr">
+        <is>
+          <t>Week 3: Sep.7/9 - No class Monday Sep.7 (Labor Day)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="136" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B31" s="144" t="inlineStr"/>
+      <c r="C31" s="144" t="inlineStr"/>
+      <c r="D31" s="144" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E31" s="144" t="inlineStr"/>
+      <c r="F31" s="130" t="inlineStr">
+        <is>
+          <t>Homework 2 (Chapter 9) — Brightspace, due 11:59 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="136" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B32" s="144" t="inlineStr"/>
+      <c r="C32" s="144" t="inlineStr"/>
+      <c r="D32" s="144" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="E32" s="144" t="inlineStr"/>
+      <c r="F32" s="130" t="inlineStr">
+        <is>
+          <t>Homework 3 — Brightspace, due 11:59 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B33" s="144" t="inlineStr"/>
+      <c r="C33" s="144" t="inlineStr"/>
+      <c r="D33" s="144" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E33" s="144" t="inlineStr"/>
+      <c r="F33" s="130" t="inlineStr">
+        <is>
+          <t>Week 5: Sep.21/23 - Complete the Chapter 3 - Part II home- work on Brightspace (due Sep.25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B34" s="144" t="inlineStr"/>
+      <c r="C34" s="144" t="inlineStr"/>
+      <c r="D34" s="144" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E34" s="144" t="inlineStr"/>
+      <c r="F34" s="130" t="inlineStr">
+        <is>
+          <t>Week 5: Sep.21/23 - Discussion of Chapter 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B35" s="144" t="inlineStr"/>
+      <c r="C35" s="144" t="inlineStr"/>
+      <c r="D35" s="144" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E35" s="144" t="inlineStr"/>
+      <c r="F35" s="130" t="inlineStr">
+        <is>
+          <t>Week 5: Sep.21/23 - Finish reading Chapter 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="136" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B36" s="144" t="inlineStr"/>
+      <c r="C36" s="144" t="inlineStr"/>
+      <c r="D36" s="144" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E36" s="144" t="inlineStr"/>
+      <c r="F36" s="130" t="inlineStr">
+        <is>
+          <t>Homework 4 (Chapter 3) — Brightspace, due 11:59 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B37" s="144" t="inlineStr"/>
+      <c r="C37" s="144" t="inlineStr"/>
+      <c r="D37" s="144" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="E37" s="144" t="inlineStr"/>
+      <c r="F37" s="130" t="inlineStr">
+        <is>
+          <t>Week 6: Sep.28/30 - AI Project – Part I due October 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B38" s="144" t="inlineStr"/>
+      <c r="C38" s="144" t="inlineStr"/>
+      <c r="D38" s="144" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="E38" s="144" t="inlineStr"/>
+      <c r="F38" s="130" t="inlineStr">
+        <is>
+          <t>Week 6: Sep.28/30 - Discussion of Chapter 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B39" s="144" t="inlineStr"/>
+      <c r="C39" s="144" t="inlineStr"/>
+      <c r="D39" s="144" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="E39" s="144" t="inlineStr"/>
+      <c r="F39" s="130" t="inlineStr">
+        <is>
+          <t>Week 6: Sep.28/30 - Read Chapter 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="136" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B40" s="144" t="inlineStr"/>
+      <c r="C40" s="144" t="inlineStr"/>
+      <c r="D40" s="144" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="E40" s="144" t="inlineStr"/>
+      <c r="F40" s="130" t="inlineStr">
+        <is>
+          <t>Homework 5 (Chapter 5) — Brightspace, due 11:59 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B41" s="144" t="inlineStr"/>
+      <c r="C41" s="144" t="inlineStr"/>
+      <c r="D41" s="144" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E41" s="144" t="inlineStr"/>
+      <c r="F41" s="130" t="inlineStr">
+        <is>
+          <t>Week 7: Oct.5/7 - Midterm review on Oct.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B42" s="144" t="inlineStr"/>
+      <c r="C42" s="144" t="inlineStr"/>
+      <c r="D42" s="144" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E42" s="144" t="inlineStr"/>
+      <c r="F42" s="130" t="inlineStr">
+        <is>
+          <t>Week 7: Oct.5/7 - Read Chapter 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="136" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B43" s="144" t="inlineStr"/>
+      <c r="C43" s="144" t="inlineStr"/>
+      <c r="D43" s="144" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="E43" s="144" t="inlineStr"/>
+      <c r="F43" s="130" t="inlineStr">
+        <is>
+          <t>Homework 6 (Chapter 6) — Brightspace, due 11:59 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="136" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B44" s="144" t="inlineStr"/>
+      <c r="C44" s="144" t="inlineStr"/>
+      <c r="D44" s="144" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="E44" s="144" t="inlineStr"/>
+      <c r="F44" s="130" t="inlineStr">
+        <is>
+          <t>Homework 7 — Brightspace, due 11:59 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B45" s="144" t="inlineStr"/>
+      <c r="C45" s="144" t="inlineStr"/>
+      <c r="D45" s="144" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="E45" s="144" t="inlineStr"/>
+      <c r="F45" s="130" t="inlineStr">
+        <is>
+          <t>Week 9: Oct.19/21 - Read Chapter 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="136" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B46" s="144" t="inlineStr"/>
+      <c r="C46" s="144" t="inlineStr"/>
+      <c r="D46" s="144" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="E46" s="144" t="inlineStr"/>
+      <c r="F46" s="130" t="inlineStr">
+        <is>
+          <t>Homework 8 (Chapter 8) — Brightspace, due 11:59 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B47" s="144" t="inlineStr"/>
+      <c r="C47" s="144" t="inlineStr"/>
+      <c r="D47" s="144" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="E47" s="144" t="inlineStr"/>
+      <c r="F47" s="130" t="inlineStr">
+        <is>
+          <t>Week 10: Oct.26/28 - Read Chapter 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="136" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B48" s="144" t="inlineStr"/>
+      <c r="C48" s="144" t="inlineStr"/>
+      <c r="D48" s="144" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="E48" s="144" t="inlineStr"/>
+      <c r="F48" s="130" t="inlineStr">
+        <is>
+          <t>Homework 9 (Chapter 10) — Brightspace, due 11:59 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B49" s="144" t="inlineStr"/>
+      <c r="C49" s="144" t="inlineStr"/>
+      <c r="D49" s="144" t="inlineStr">
+        <is>
+          <t>2026-11-13</t>
+        </is>
+      </c>
+      <c r="E49" s="144" t="inlineStr"/>
+      <c r="F49" s="130" t="inlineStr">
+        <is>
+          <t>Week 12: Nov.9/11 - No class Wednesday Nov.11 (Veterans Day)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B50" s="144" t="inlineStr"/>
+      <c r="C50" s="144" t="inlineStr"/>
+      <c r="D50" s="144" t="inlineStr">
+        <is>
+          <t>2026-11-13</t>
+        </is>
+      </c>
+      <c r="E50" s="144" t="inlineStr"/>
+      <c r="F50" s="130" t="inlineStr">
+        <is>
+          <t>Week 12: Nov.9/11 - Read Chapter 11</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="136" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B51" s="144" t="inlineStr"/>
+      <c r="C51" s="144" t="inlineStr"/>
+      <c r="D51" s="144" t="inlineStr">
+        <is>
+          <t>2026-11-13</t>
+        </is>
+      </c>
+      <c r="E51" s="144" t="inlineStr"/>
+      <c r="F51" s="130" t="inlineStr">
+        <is>
+          <t>Homework 10 (Chapter 11) — Brightspace, due 11:59 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B52" s="144" t="inlineStr"/>
+      <c r="C52" s="144" t="inlineStr"/>
+      <c r="D52" s="144" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="E52" s="144" t="inlineStr"/>
+      <c r="F52" s="130" t="inlineStr">
+        <is>
+          <t>Week 13: Nov.16/18 - Read Chapter 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="136" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B53" s="144" t="inlineStr"/>
+      <c r="C53" s="144" t="inlineStr"/>
+      <c r="D53" s="144" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="E53" s="144" t="inlineStr"/>
+      <c r="F53" s="130" t="inlineStr">
+        <is>
+          <t>Homework 11 (Chapter 12) — Brightspace, due 11:59 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B54" s="144" t="inlineStr"/>
+      <c r="C54" s="144" t="inlineStr"/>
+      <c r="D54" s="144" t="inlineStr">
+        <is>
+          <t>2026-11-27</t>
+        </is>
+      </c>
+      <c r="E54" s="144" t="inlineStr"/>
+      <c r="F54" s="130" t="inlineStr">
+        <is>
+          <t>Week 14: Nov.23 - Complete the Chapter 12+13 home- work on Brightspace (due Nov.27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B55" s="144" t="inlineStr"/>
+      <c r="C55" s="144" t="inlineStr"/>
+      <c r="D55" s="144" t="inlineStr">
+        <is>
+          <t>2026-11-27</t>
+        </is>
+      </c>
+      <c r="E55" s="144" t="inlineStr"/>
+      <c r="F55" s="130" t="inlineStr">
+        <is>
+          <t>Week 14: Nov.23 - No class Wednesday Nov.25 (Thanks- giving)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="135" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="B56" s="144" t="inlineStr"/>
+      <c r="C56" s="144" t="inlineStr"/>
+      <c r="D56" s="144" t="inlineStr">
+        <is>
+          <t>2026-11-27</t>
+        </is>
+      </c>
+      <c r="E56" s="144" t="inlineStr"/>
+      <c r="F56" s="130" t="inlineStr">
+        <is>
+          <t>Week 14: Nov.23 - Read Chapter 13</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="136" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B57" s="144" t="inlineStr"/>
+      <c r="C57" s="144" t="inlineStr"/>
+      <c r="D57" s="144" t="inlineStr">
+        <is>
+          <t>2026-11-27</t>
+        </is>
+      </c>
+      <c r="E57" s="144" t="inlineStr"/>
+      <c r="F57" s="130" t="inlineStr">
+        <is>
+          <t>Homework 12 (Chapter 13) — Brightspace, due 11:59 pm</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="124" t="inlineStr">
+        <is>
+          <t>Extra Credit</t>
+        </is>
+      </c>
+      <c r="B58" s="142" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C58" s="143" t="inlineStr"/>
+      <c r="D58" s="143" t="inlineStr"/>
+      <c r="E58" s="143" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F58" s="127">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/econ-351-extra-credit.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="29" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B59" s="137" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="B6:F6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add full RMP review text for Martínez-Marquina (ECON-351)
Fetch all 61 student comments from professor 2880539 via GraphQL,
store in rmp.json, and show them on the Overview tab in a collapsible
reviews block. RMP profile name is labeled separately from co-instructor.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -430,7 +430,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="146">
+  <cellXfs count="150">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -809,6 +809,18 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="34" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="32" fillId="34" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1199,7 +1211,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:K126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1359,7 +1371,7 @@
       </c>
       <c r="B8" s="88" t="inlineStr">
         <is>
-          <t>Alejandro Martínez-Marquina / João Ramos</t>
+          <t>Alejandro Martínez-Marquina / João Ramos (RMP: Alejandro Martínez-Marquina)</t>
         </is>
       </c>
       <c r="C8" s="26" t="inlineStr">
@@ -1470,7 +1482,7 @@
         </is>
       </c>
     </row>
-    <row r="14" hidden="1" outlineLevel="1" ht="120" customHeight="1">
+    <row r="14" hidden="1" outlineLevel="1" ht="165" customHeight="1">
       <c r="A14" s="104" t="inlineStr">
         <is>
           <t>ECON-351</t>
@@ -1478,14 +1490,15 @@
       </c>
       <c r="B14" s="105" t="inlineStr">
         <is>
-          <t>Alejandro Martínez-Marquina / João Ramos</t>
+          <t>Alejandro Martínez-Marquina / João Ramos (RMP: Alejandro Martínez-Marquina)</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>STRENGTHS: Martínez-Marquina earns strong marks for clear board work, practice problems, and supportive TAs; students say concepts click when you attend and use office hours. Ramos sections get mixed reviews — some praise exam alignment with practice problems, others find lectures hard to follow due to pace/accent.
-GRADING &amp; WORKLOAD: Four non-cumulative midterms (20% each) plus weekly Brightspace homework (best 10 of 12 count). AI Forecast Project is individual. Letter grades follow Marshall guidelines with rough bands (A above ~85%, B 70–85%, C 60–70%).
-BOTTOM LINE: Engage with practice problems and TAs; homework drops give flexibility. WSJ Future View offers optional +10% extra credit.</t>
+          <t>STRENGTHS: Reviewers repeatedly praise board work, step-by-step problem breakdowns, and practice sets that mirror exams. Many call him kind, funny, and responsive by email; office hours and TAs get strong mentions. Several note you can succeed without mandatory attendance if you self-study from the textbook.
+COMMON CAVEATS: Spanish accent and fast lecture pace come up often — sit near the front. Some say lectures/textbook do not fully prepare you unless you drill mock exams and homework. Content volume is high; procrastination hurts.
+EXAMS &amp; GRADING: Midterms align with practice problems and mock exams; homework is described as easy/lenient (best-of policy). Grades span A to C- depending on effort. AI/group project mentioned as straightforward when you keep up.
+BOTTOM LINE: Do the practice sets, use TAs/office hours, and do not fall behind — accent and pace are manageable with front-row seating and self-study.</t>
         </is>
       </c>
     </row>
@@ -1508,1156 +1521,2661 @@
         </is>
       </c>
     </row>
-    <row r="16" hidden="1" outlineLevel="1">
-      <c r="A16" s="91" t="inlineStr">
+    <row r="16" hidden="1" outlineLevel="1"/>
+    <row r="17" hidden="1" outlineLevel="1">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>Student reviews (Rate My Professors) - newest first</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" hidden="1" outlineLevel="1">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Q/D</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" hidden="1" outlineLevel="1" ht="30" customHeight="1">
+      <c r="A19" s="104" t="inlineStr">
+        <is>
+          <t>ECON-351</t>
+        </is>
+      </c>
+      <c r="B19" s="105" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="C19" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D19" s="105" t="inlineStr">
+        <is>
+          <t>5/1</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>The tests are easy if you just do the practice sets. He's great at explanations. [Amazing lectures, So many papers, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A20" s="107" t="inlineStr"/>
+      <c r="B20" s="107" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="C20" s="107" t="inlineStr">
+        <is>
+          <t>C-</t>
+        </is>
+      </c>
+      <c r="D20" s="107" t="inlineStr">
+        <is>
+          <t>5/4</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>personally the class is hard, because there is a lot of content. do not procrastinate it will be your downfall. midterms are the same as mock exams and homework, so just practice that. group project at end is straightforward, homework is easy. ultimately your grade depends on your own effort so try!! [Get ready to read, Lecture heavy, Test heavy]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="A21" s="105" t="inlineStr"/>
+      <c r="B21" s="105" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="C21" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D21" s="105" t="inlineStr">
+        <is>
+          <t>4/3</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Alejandro is very nice and sometimes his accent is hard to understand in lecture but overall you understand what he is saying. The tests are exactly like the practice problems and he's very funny. Do the practice and you will do well in class! [Respected, Test heavy]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A22" s="107" t="inlineStr"/>
+      <c r="B22" s="107" t="inlineStr">
+        <is>
+          <t>2026-01-06</t>
+        </is>
+      </c>
+      <c r="C22" s="107" t="inlineStr">
+        <is>
+          <t>C-</t>
+        </is>
+      </c>
+      <c r="D22" s="107" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>His lectures are enjoyable and structures the class to be very flexible with no required attendance and lenient homework policies. He does however have a spanish accent which makes understading lecture difficult sometimes. Additonally, I felt the lectures and textbook do not adequately prepare you for exams. [Amazing lectures, Respected, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" hidden="1" outlineLevel="1" ht="90" customHeight="1">
+      <c r="A23" s="105" t="inlineStr"/>
+      <c r="B23" s="105" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="C23" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D23" s="105" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Really great professor, he writes on the board with practice questions, so concepts are easier to follow. He has an excellent TA who goes through all the questions, is super understanding and helpful, and she explains concepts really well. He has an accent, but it did not hinder my ability to learn. Definitely self-study as well, with the textbook! [Lecture heavy, Test heavy, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A24" s="107" t="inlineStr"/>
+      <c r="B24" s="107" t="inlineStr">
+        <is>
+          <t>2025-12-24</t>
+        </is>
+      </c>
+      <c r="C24" s="107" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D24" s="107" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Amazing professor. Has an accent but you get used to it. Can go through material pretty quickly, but he writes on board and explains while demonstrating, which helps a lot. He also goes back to explain if students are still confused. Exams are relatively the same as practice problems he gives. [Lecture heavy, Test heavy, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="A25" s="105" t="inlineStr"/>
+      <c r="B25" s="105" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="C25" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D25" s="105" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>GREAT PROFESSOR. He breaks down the steps of each problem amazingly, accent is a little thick (sit in the front it helps a lot), His office hours are worth it, he will make sure you understand!! Work hard from the beginning and do ALL practice problems (repeats in test). [Hilarious, Respected, Test heavy]</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A26" s="107" t="inlineStr"/>
+      <c r="B26" s="107" t="inlineStr">
+        <is>
+          <t>2025-12-11</t>
+        </is>
+      </c>
+      <c r="C26" s="107" t="inlineStr">
+        <is>
+          <t>Not sure yet</t>
+        </is>
+      </c>
+      <c r="D26" s="107" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>Its a hard class and his lectures go by quick. With that being said he is really good at teaching and also really accessible outside of class. Answers emails extremely quickly and grades test within a few days of the test date. Exams are hard, but if you study and go to an office hour before the test your fine. [Amazing lectures, Test heavy, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A27" s="105" t="inlineStr"/>
+      <c r="B27" s="105" t="inlineStr">
+        <is>
+          <t>2025-12-05</t>
+        </is>
+      </c>
+      <c r="C27" s="105" t="inlineStr">
+        <is>
+          <t>Drop/Withdrawal</t>
+        </is>
+      </c>
+      <c r="D27" s="105" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>Professor flies through the lectures and his accent makes it difficult to understand and keep up. The course is already known for being a tough course. When questions are asked he sort of laughs and makes you feel bad before explaining. He has really good TAs though that help you step by step. I would definitely go to office hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="A28" s="107" t="inlineStr"/>
+      <c r="B28" s="107" t="inlineStr">
+        <is>
+          <t>2025-12-04</t>
+        </is>
+      </c>
+      <c r="C28" s="107" t="inlineStr">
+        <is>
+          <t>Not sure yet</t>
+        </is>
+      </c>
+      <c r="D28" s="107" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>- Genuinely moves at the speed of light - Is accessible outside of class, but truly have to grind for an A - Exams are super hard, homeworks are free - Professor is a bit condescending but means well [Lecture heavy, Test heavy, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" hidden="1" outlineLevel="1" ht="45" customHeight="1">
+      <c r="A29" s="105" t="inlineStr"/>
+      <c r="B29" s="105" t="inlineStr">
+        <is>
+          <t>2025-11-17</t>
+        </is>
+      </c>
+      <c r="C29" s="105" t="inlineStr">
+        <is>
+          <t>Not sure yet</t>
+        </is>
+      </c>
+      <c r="D29" s="105" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>His accent and super fast pace of the class/lecture make it so hard to understand. The class is already hard and the speed of the lectures make this so hard [Lecture heavy, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A30" s="107" t="inlineStr"/>
+      <c r="B30" s="107" t="inlineStr">
+        <is>
+          <t>2025-10-16</t>
+        </is>
+      </c>
+      <c r="C30" s="107" t="inlineStr">
+        <is>
+          <t>Not sure yet</t>
+        </is>
+      </c>
+      <c r="D30" s="107" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>He does talk fast but if you don't understand or need to hear concept again he will gladly explain it to you until you get it. Very nice wants you to get an A but Econ isn't an easy class. Office hours are great way to prepare for test. Study guides very similar to exams. [Amazing lectures, Clear grading criteria, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" hidden="1" outlineLevel="1" ht="30" customHeight="1">
+      <c r="A31" s="105" t="inlineStr"/>
+      <c r="B31" s="105" t="inlineStr">
+        <is>
+          <t>2025-10-15</t>
+        </is>
+      </c>
+      <c r="C31" s="105" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D31" s="105" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>Fantastic Professor. Easy looking at. Funny guy. Muy bien</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" hidden="1" outlineLevel="1" ht="45" customHeight="1">
+      <c r="A32" s="107" t="inlineStr"/>
+      <c r="B32" s="107" t="inlineStr">
+        <is>
+          <t>2025-10-06</t>
+        </is>
+      </c>
+      <c r="C32" s="107" t="inlineStr">
+        <is>
+          <t>Not sure yet</t>
+        </is>
+      </c>
+      <c r="D32" s="107" t="inlineStr">
+        <is>
+          <t>4/2</t>
+        </is>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>Talks too fast and is hard to understand because of his accent. He mostly reads off the slides. But fun classes and passionate lecturer who encourages questions. He also uses real life examples which is useful.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="A33" s="105" t="inlineStr"/>
+      <c r="B33" s="105" t="inlineStr">
+        <is>
+          <t>2025-10-06</t>
+        </is>
+      </c>
+      <c r="C33" s="105" t="inlineStr">
+        <is>
+          <t>Not sure yet</t>
+        </is>
+      </c>
+      <c r="D33" s="105" t="inlineStr">
+        <is>
+          <t>1/4</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Bro talks so fast, literally I was better off teaching it to myself outside of class. EXTREMELY condescending. I would go to his office hours and he would laugh at certain students questions and belittle them. Idk how his rating is so high, I'd drop if it weren't already to late in the semester. [Test heavy]</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" hidden="1" outlineLevel="1" ht="45" customHeight="1">
+      <c r="A34" s="107" t="inlineStr"/>
+      <c r="B34" s="107" t="inlineStr">
+        <is>
+          <t>2025-10-06</t>
+        </is>
+      </c>
+      <c r="C34" s="107" t="inlineStr">
+        <is>
+          <t>Not sure yet</t>
+        </is>
+      </c>
+      <c r="D34" s="107" t="inlineStr">
+        <is>
+          <t>5/4</t>
+        </is>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>no glaze, he's a really good professor and explained concepts very well. Would take him again every single time if I could choose. [Amazing lectures, Inspirational, Caring]</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" hidden="1" outlineLevel="1" ht="45" customHeight="1">
+      <c r="A35" s="105" t="inlineStr"/>
+      <c r="B35" s="105" t="inlineStr">
+        <is>
+          <t>2025-06-25</t>
+        </is>
+      </c>
+      <c r="C35" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D35" s="105" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Best professor I've had at USC. Took his econ351 class in fall 2024 and learned so much. Class is on Marshall curve so its competitive to get an A, but it wasn't that hard. [Inspirational, Lecture heavy, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A36" s="107" t="inlineStr"/>
+      <c r="B36" s="107" t="inlineStr">
+        <is>
+          <t>2025-05-30</t>
+        </is>
+      </c>
+      <c r="C36" s="107" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D36" s="107" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>ECON 351 is a hard class no matter what, but if you have to take it def take Professor Martinez. Funny guy, doesn't mind explaining over and over again and has great lecture slides. Great TAs and curve. Tests are hard but they are no matter who you take. Hosts lots of reviews and genuinely cares and wants to hear our perspectives. Miss him!</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="A37" s="105" t="inlineStr"/>
+      <c r="B37" s="105" t="inlineStr">
+        <is>
+          <t>2025-05-17</t>
+        </is>
+      </c>
+      <c r="C37" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D37" s="105" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>This was my favorite professor of all time. In fact, the best professor I have ever had in my academic career. I highly recommend him. He makes lectures so fun. The class is hard, but if you understand calculus then you will ace the course. Highly recommend. [Amazing lectures, Inspirational, Caring]</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A38" s="107" t="inlineStr"/>
+      <c r="B38" s="107" t="inlineStr">
+        <is>
+          <t>2025-05-01</t>
+        </is>
+      </c>
+      <c r="C38" s="107" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="D38" s="107" t="inlineStr">
+        <is>
+          <t>2/5</t>
+        </is>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>I am not sure why his reviews are so high... I was barely able to get a B- in this class after studying over 10 hours for each test. The practice tests were only somewhat similar and the homework took a lot of time. I would not recommend this teacher unless you want to go to office hours every week and try to get him to like you. [Lecture heavy, Test heavy, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" hidden="1" outlineLevel="1" ht="30" customHeight="1">
+      <c r="A39" s="105" t="inlineStr"/>
+      <c r="B39" s="105" t="inlineStr">
+        <is>
+          <t>2025-01-29</t>
+        </is>
+      </c>
+      <c r="C39" s="105" t="inlineStr">
+        <is>
+          <t>Not sure yet</t>
+        </is>
+      </c>
+      <c r="D39" s="105" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>He's so easy to look at&amp;#8230; take him [Tough grader, EXTRA CREDIT, Amazing lectures]</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A40" s="107" t="inlineStr"/>
+      <c r="B40" s="107" t="inlineStr">
+        <is>
+          <t>2025-01-18</t>
+        </is>
+      </c>
+      <c r="C40" s="107" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D40" s="107" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>He is amazing. Went into 351 being really scared but honestly this class was way easier than I thought it would be. As long as you do all the practice problems and homework, there's no reason why you shouldn't get an A as tests are 95% similar to what you've seen before. For those complaining, they were just lazy and didn't do the work. [Amazing lectures, Hilarious, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="A41" s="105" t="inlineStr"/>
+      <c r="B41" s="105" t="inlineStr">
+        <is>
+          <t>2025-01-10</t>
+        </is>
+      </c>
+      <c r="C41" s="105" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D41" s="105" t="inlineStr">
+        <is>
+          <t>2/4</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>office hours with the TA saved me as his were completely full all the time. lectures were organized but he went so fast with explanations and skipped many steps making it confusing. only graded on 3 tests no curve and they are very difficult and only 24 points so very hard to get a good grade [Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="A42" s="107" t="inlineStr"/>
+      <c r="B42" s="107" t="inlineStr">
+        <is>
+          <t>2025-01-02</t>
+        </is>
+      </c>
+      <c r="C42" s="107" t="inlineStr">
+        <is>
+          <t>Not sure yet</t>
+        </is>
+      </c>
+      <c r="D42" s="107" t="inlineStr">
+        <is>
+          <t>3/5</t>
+        </is>
+      </c>
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>His lectures were very confusing, and he taught so quickly. If you go to HIS office hours, he'll give you all the answers to homework and practice tests, which was nice, but his tests were very hard. He does not curve at all, so expect your grade to be heavily based on how you perform on the tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A43" s="105" t="inlineStr"/>
+      <c r="B43" s="105" t="inlineStr">
+        <is>
+          <t>2024-12-28</t>
+        </is>
+      </c>
+      <c r="C43" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D43" s="105" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>BEST PROF FOR ECON351. Tests are exactly what's on hw &amp; practice sets. Lots of office hours. He let us go to any of his lectures (no attendance taken) + recordings posted online. He's great at explaining and his class makes econ fun/interesting. No complaints at all, very fair/interesting/funny guy. He wants you to get an A! TAKE HIM, TRUST. [Hilarious, Respected, Lecture heavy]</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" hidden="1" outlineLevel="1" ht="30" customHeight="1">
+      <c r="A44" s="107" t="inlineStr"/>
+      <c r="B44" s="107" t="inlineStr">
+        <is>
+          <t>2024-12-21</t>
+        </is>
+      </c>
+      <c r="C44" s="107" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D44" s="107" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E44" s="11" t="inlineStr">
+        <is>
+          <t>Awesome professor. Lectures are interesting and exams are very similar to practice tests. [Amazing lectures, Clear grading criteria, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A45" s="105" t="inlineStr"/>
+      <c r="B45" s="105" t="inlineStr">
+        <is>
+          <t>2024-12-21</t>
+        </is>
+      </c>
+      <c r="C45" s="105" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D45" s="105" t="inlineStr">
+        <is>
+          <t>4/5</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Good professor, but I would not take him again. he puts "trick questions" on exams so no one ends up getting them right. He switches up the questions on exams and they are way harder. I never put so much work into a class and I only got a B+ and thats with a 10 point curve so in reality my grade should be lower. [Tough grader, Amazing lectures, Test heavy]</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A46" s="107" t="inlineStr"/>
+      <c r="B46" s="107" t="inlineStr">
+        <is>
+          <t>2024-12-20</t>
+        </is>
+      </c>
+      <c r="C46" s="107" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D46" s="107" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E46" s="11" t="inlineStr">
+        <is>
+          <t>goat. 351 is hard but he makes it interesting and manageable. 3 exams each worth 30% and the other 10% is homework. go to lecture, do the practice problems and if you're still struggling read the textbook or go to office hours. take his class to get an A in econ and to laugh because he's hilarious. [Amazing lectures, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" hidden="1" outlineLevel="1" ht="45" customHeight="1">
+      <c r="A47" s="105" t="inlineStr"/>
+      <c r="B47" s="105" t="inlineStr">
+        <is>
+          <t>2024-12-20</t>
+        </is>
+      </c>
+      <c r="C47" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D47" s="105" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Amazing professor! He includes real-world applications, which helps with understanding. And, I thought the class aligned with what he shared on the first day. Overall could not recommend more! [Amazing lectures, Caring]</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="A48" s="107" t="inlineStr"/>
+      <c r="B48" s="107" t="inlineStr">
+        <is>
+          <t>2024-12-19</t>
+        </is>
+      </c>
+      <c r="C48" s="107" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D48" s="107" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E48" s="11" t="inlineStr">
+        <is>
+          <t>Goat. Simple as that. Gives plenty of practice tests/problems that are identical in concept and form to the actual tests. Just be aware that the bar for an A-range grade may change throughout the semester (i.e. A-range = &gt;80 to A-range = &gt;85). [Caring, Test heavy, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A49" s="105" t="inlineStr"/>
+      <c r="B49" s="105" t="inlineStr">
+        <is>
+          <t>2024-12-05</t>
+        </is>
+      </c>
+      <c r="C49" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D49" s="105" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Best teacher for microeconomics. Explains concepts well and is very clear about what will be on exams. Practice exams and chapter questions are identical to what will be on the tests. He's also super caring and will take the time to help you out and answer questions. By far my favorite professor this semester! [Caring]</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A50" s="107" t="inlineStr"/>
+      <c r="B50" s="107" t="inlineStr">
+        <is>
+          <t>2024-12-05</t>
+        </is>
+      </c>
+      <c r="C50" s="107" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D50" s="107" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E50" s="11" t="inlineStr">
+        <is>
+          <t>Professor Alejandro is one of my favorite and best professors in Marshall! He is so engaging and incorporated lots of humor into his lectures (which attendance was not mandatory for). It's also evident that he wants his students to do well and holds many office hours for studnets. Would totally take him again. THE GOAT &amp;#128016; [Amazing lectures, Lecture heavy, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="A51" s="105" t="inlineStr"/>
+      <c r="B51" s="105" t="inlineStr">
+        <is>
+          <t>2024-12-04</t>
+        </is>
+      </c>
+      <c r="C51" s="105" t="inlineStr">
+        <is>
+          <t>Not sure yet</t>
+        </is>
+      </c>
+      <c r="D51" s="105" t="inlineStr">
+        <is>
+          <t>5/1</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Professor Alejandro is awesome. His lecture is inspirational and well-explained. I love the vibe of his class, and the tests are always easy as long as you finish the sample problems. [Amazing lectures, Inspirational, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A52" s="107" t="inlineStr"/>
+      <c r="B52" s="107" t="inlineStr">
+        <is>
+          <t>2024-12-03</t>
+        </is>
+      </c>
+      <c r="C52" s="107" t="inlineStr">
+        <is>
+          <t>Not sure yet</t>
+        </is>
+      </c>
+      <c r="D52" s="107" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E52" s="11" t="inlineStr">
+        <is>
+          <t>If you attend classes and office hours, you will understand all concepts. The class isn't too bad especially if you did IB Econ. Just do the homework and practice tests, and you're good. His papers are also not too bad so if you practice well you will do well. [Clear grading criteria, Lots of homework, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A53" s="105" t="inlineStr"/>
+      <c r="B53" s="105" t="inlineStr">
+        <is>
+          <t>2024-11-13</t>
+        </is>
+      </c>
+      <c r="C53" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D53" s="105" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Best 351 prof he's so nice!!! Midterms are exactly like practice tests given. Homework is completion as long as you get half right and he gives you answers in office hours. Don't need to go to class-- he posts lectures and doesn't take attendance. Do the practice problems twice before the 3 tests and you can get an A. 80 or above overall is an A. [Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" hidden="1" outlineLevel="1" ht="45" customHeight="1">
+      <c r="A54" s="107" t="inlineStr"/>
+      <c r="B54" s="107" t="inlineStr">
+        <is>
+          <t>2024-11-13</t>
+        </is>
+      </c>
+      <c r="C54" s="107" t="inlineStr">
+        <is>
+          <t>Not sure yet</t>
+        </is>
+      </c>
+      <c r="D54" s="107" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E54" s="11" t="inlineStr">
+        <is>
+          <t>&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" hidden="1" outlineLevel="1" ht="90" customHeight="1">
+      <c r="A55" s="105" t="inlineStr"/>
+      <c r="B55" s="105" t="inlineStr">
+        <is>
+          <t>2024-11-11</t>
+        </is>
+      </c>
+      <c r="C55" s="105" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D55" s="105" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>It's definitely a difficult class and you have to study A LOT for tests, but he holds office hours every day for the entire semester and gives a bunch of practice problems prior to midterms. The homework isn't too bad, but the difficulty of the class is dependent on whether or not you go to lectures. He overall made a difficult class digestible. [Amazing lectures, Lecture heavy, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" hidden="1" outlineLevel="1" ht="30" customHeight="1">
+      <c r="A56" s="107" t="inlineStr"/>
+      <c r="B56" s="107" t="inlineStr">
+        <is>
+          <t>2024-10-22</t>
+        </is>
+      </c>
+      <c r="C56" s="107" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D56" s="107" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E56" s="11" t="inlineStr">
+        <is>
+          <t>Exam questions are very similar to the practice sets he provides. Wants you to do well. [Caring, Test heavy, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A57" s="105" t="inlineStr"/>
+      <c r="B57" s="105" t="inlineStr">
+        <is>
+          <t>2024-08-01</t>
+        </is>
+      </c>
+      <c r="C57" s="105" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="D57" s="105" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>Such a great professor his class is so manageable. I barely went to lecture and never went to office hours and did perfectly fine. Homework is graded very easily and basically every single possible midterm question is provided to you between all the practice sets. Do all the questions and you'll be fine. By far the best choice for 351.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="A58" s="107" t="inlineStr"/>
+      <c r="B58" s="107" t="inlineStr">
+        <is>
+          <t>2024-06-22</t>
+        </is>
+      </c>
+      <c r="C58" s="107" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D58" s="107" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E58" s="11" t="inlineStr">
+        <is>
+          <t>Great course if you show up to every lecture and pay attention. Taking notes, reviewing practice problems, and going to office hours when I needed help with certain problems made the class not overly difficult. Great lecturer and cares about his students. Would take him again if I could. [Respected, Lecture heavy]</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" hidden="1" outlineLevel="1" ht="45" customHeight="1">
+      <c r="A59" s="105" t="inlineStr"/>
+      <c r="B59" s="105" t="inlineStr">
+        <is>
+          <t>2024-06-19</t>
+        </is>
+      </c>
+      <c r="C59" s="105" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="D59" s="105" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>I never went to his office hours and skipped around 70% of classes and still got a decent grade. He is a good lecturer and grades aren't hard to get. PLEASE do practice questions because exam questions are 80% based on them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A60" s="107" t="inlineStr"/>
+      <c r="B60" s="107" t="inlineStr">
+        <is>
+          <t>2024-05-28</t>
+        </is>
+      </c>
+      <c r="C60" s="107" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D60" s="107" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E60" s="11" t="inlineStr">
+        <is>
+          <t>Marquina made ECON351 a breeze. His lectures are straightforward, engaging, and explain the material well. Your grade is determined by 3 tests spaced out throughout the semester. They're non-cumulative which is nice. Do the homework and the exam practice sets and you'll get a top grade. [Amazing lectures, Clear grading criteria, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A61" s="105" t="inlineStr"/>
+      <c r="B61" s="105" t="inlineStr">
+        <is>
+          <t>2024-05-19</t>
+        </is>
+      </c>
+      <c r="C61" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D61" s="105" t="inlineStr">
+        <is>
+          <t>5/1</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>Makes microeconomics easy and provides fun examples for students to engage with. Do the homework and the practice midterms/final he provides to study and you will get an A in this class. Provides really, really helpful office hours for questions on homework and allows test revision. GOATED Marshall professor. [Lots of homework, Test heavy]</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A62" s="107" t="inlineStr"/>
+      <c r="B62" s="107" t="inlineStr">
+        <is>
+          <t>2024-05-10</t>
+        </is>
+      </c>
+      <c r="C62" s="107" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D62" s="107" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E62" s="11" t="inlineStr">
+        <is>
+          <t>Great professor, but a fast lecturer. Overall would highly recommend him for Econ 351. The course is graded on only 3 written exams and weekly homework assignments, and as long as you do the practice questions he posts before each exam, they should be quite easy. [Inspirational, Graded by few things, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" hidden="1" outlineLevel="1" ht="90" customHeight="1">
+      <c r="A63" s="105" t="inlineStr"/>
+      <c r="B63" s="105" t="inlineStr">
+        <is>
+          <t>2024-05-02</t>
+        </is>
+      </c>
+      <c r="C63" s="105" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="D63" s="105" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>Despite being a new prof, Alejandro is a really engaging and fun lecturer. He's accessible and will help you perform your best in class as long as you put in the work. I love him and would take his classes again. Looking forward to taking his class in my upperclassmen years. Go to office hours before a midterm/final and I guarantee you'll ace them. [Gives good feedback, Caring, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" hidden="1" outlineLevel="1" ht="30" customHeight="1">
+      <c r="A64" s="107" t="inlineStr"/>
+      <c r="B64" s="107" t="inlineStr">
+        <is>
+          <t>2024-05-02</t>
+        </is>
+      </c>
+      <c r="C64" s="107" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="D64" s="107" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E64" s="11" t="inlineStr">
+        <is>
+          <t>351 is a hard class and he's easily the best teacher for it. [Caring, Test heavy, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A65" s="105" t="inlineStr"/>
+      <c r="B65" s="105" t="inlineStr">
+        <is>
+          <t>2024-05-02</t>
+        </is>
+      </c>
+      <c r="C65" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D65" s="105" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>Professor Martinez-Marquina was hands-down awesome! He's so caring and easy to talk to if you had concerns about your grade or the course content. Lectures are fast-paced for sure, but his office hours are SO worth it! Overall such an amazing professor! He's super accommodating and wants you to succeed in and out of class. [Amazing lectures, Respected, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" hidden="1" outlineLevel="1" ht="45" customHeight="1">
+      <c r="A66" s="107" t="inlineStr"/>
+      <c r="B66" s="107" t="inlineStr">
+        <is>
+          <t>2024-04-25</t>
+        </is>
+      </c>
+      <c r="C66" s="107" t="inlineStr">
+        <is>
+          <t>Not sure yet</t>
+        </is>
+      </c>
+      <c r="D66" s="107" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E66" s="11" t="inlineStr">
+        <is>
+          <t>Tests are very similar to practice problems, and lectures are easy to follow. If you show up to class it is very manageable! [Amazing lectures, Clear grading criteria, Gives good feedback]</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A67" s="105" t="inlineStr"/>
+      <c r="B67" s="105" t="inlineStr">
+        <is>
+          <t>2024-04-16</t>
+        </is>
+      </c>
+      <c r="C67" s="105" t="inlineStr">
+        <is>
+          <t>Not sure yet</t>
+        </is>
+      </c>
+      <c r="D67" s="105" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>Econ 351 is probably one of the hardest classes in Marshall. However, Marquina makes the content very much digestable. He's a very caring professor and wants you to understand the topic, and the lengths that he goes to to do so is very respectable. Genuine guy, very fun to talk to and honestly an amazing professor. [Inspirational, Caring, Respected]</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="A68" s="107" t="inlineStr"/>
+      <c r="B68" s="107" t="inlineStr">
+        <is>
+          <t>2024-04-15</t>
+        </is>
+      </c>
+      <c r="C68" s="107" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D68" s="107" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E68" s="11" t="inlineStr">
+        <is>
+          <t>Literally my favorite professor I've taken so far. I would take ANY class he teaches! He was super accessible and reasonable. He genuinely cared for you to grasp the material, and would often stay late after class or office hours if you needed his help. [Amazing lectures, Respected, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A69" s="105" t="inlineStr"/>
+      <c r="B69" s="105" t="inlineStr">
+        <is>
+          <t>2024-04-02</t>
+        </is>
+      </c>
+      <c r="C69" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D69" s="105" t="inlineStr">
+        <is>
+          <t>5/4</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>Yes, lectures are fast paced &amp; the material is difficult. However, Alejandro makes everything manageable. Coming in with no econ experience, I was still able to succeed. To succeed: go to class, read the textbook (its free &amp; really helpful), go to office hours, &amp; do the practice problems (all 3 tests resemble practice problems VERY closely). [Amazing lectures, Gives good feedback, Test heavy]</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" hidden="1" outlineLevel="1" ht="30" customHeight="1">
+      <c r="A70" s="107" t="inlineStr"/>
+      <c r="B70" s="107" t="inlineStr">
+        <is>
+          <t>2023-10-25</t>
+        </is>
+      </c>
+      <c r="C70" s="107" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D70" s="107" t="inlineStr">
+        <is>
+          <t>5/1</t>
+        </is>
+      </c>
+      <c r="E70" s="11" t="inlineStr">
+        <is>
+          <t>great professor with clear lectures, easy homework and tests [Amazing lectures, Caring, Respected]</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A71" s="105" t="inlineStr"/>
+      <c r="B71" s="105" t="inlineStr">
+        <is>
+          <t>2023-06-21</t>
+        </is>
+      </c>
+      <c r="C71" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D71" s="105" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>Take this class +1 !! Prof. Martinez explains the lectures thoroughly, provides real-world examples, and his pace is perfect. He is determined to help students succeed by going above and beyond to provide office hours (especially before exams) and exam review/revision afterward. Test-heavy, but the content is relevant to lectures and homework. [Amazing lectures, Caring, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A72" s="107" t="inlineStr"/>
+      <c r="B72" s="107" t="inlineStr">
+        <is>
+          <t>2023-05-26</t>
+        </is>
+      </c>
+      <c r="C72" s="107" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D72" s="107" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E72" s="11" t="inlineStr">
+        <is>
+          <t>Amazing professor who truly wants his students to learn and succeed. Grading: 90% from 3 exams, 10% from HW. Thought this course was a very quantitative, fast-paced, and difficult class to get adjusted to. I struggling at first as I failed (D+) both midterm 1 and midterm 2 (post-curve). Got an A on the final exam (post-curve). Ended with a B. [Clear grading criteria, Caring, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="A73" s="105" t="inlineStr"/>
+      <c r="B73" s="105" t="inlineStr">
+        <is>
+          <t>2023-05-09</t>
+        </is>
+      </c>
+      <c r="C73" s="105" t="inlineStr">
+        <is>
+          <t>Not sure yet</t>
+        </is>
+      </c>
+      <c r="D73" s="105" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>He's a really caring and understanding professor. Although Econ 351 itself can be tough, he makes the lectures engaging and tries his best to help us understand. Doing the homework and practice chapter samples are really helpful for the tests! [Clear grading criteria, Gives good feedback, Caring]</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" hidden="1" outlineLevel="1" ht="90" customHeight="1">
+      <c r="A74" s="107" t="inlineStr"/>
+      <c r="B74" s="107" t="inlineStr">
+        <is>
+          <t>2023-05-06</t>
+        </is>
+      </c>
+      <c r="C74" s="107" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D74" s="107" t="inlineStr">
+        <is>
+          <t>5/4</t>
+        </is>
+      </c>
+      <c r="E74" s="11" t="inlineStr">
+        <is>
+          <t>Professor Marquina is a very kind and sweet guy. You can tell he genuinely cares for his students, he consistently gave extra office hours and met with me 1-on-1 after my poor 2nd midterm performance, encouraged and strategized with me on how I could improve. 2 midterms &amp; 1 final, very challenging course content. Get ready to put in the work [Caring, Graded by few things, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A75" s="105" t="inlineStr"/>
+      <c r="B75" s="105" t="inlineStr">
+        <is>
+          <t>2023-04-26</t>
+        </is>
+      </c>
+      <c r="C75" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D75" s="105" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>Take this class!!!!!!! He is such a nice guy and is always willing to meet with students, whether that means just re explaining something after class, holding office hours, or scheduling 1 on 1 time to meet with you and talk through questions or go over tests. If you pay any attention in the lectures you won't have any trouble.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A76" s="107" t="inlineStr"/>
+      <c r="B76" s="107" t="inlineStr">
+        <is>
+          <t>2023-04-26</t>
+        </is>
+      </c>
+      <c r="C76" s="107" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D76" s="107" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E76" s="11" t="inlineStr">
+        <is>
+          <t>Prof. Martinez is a fairly new professor, but he's one of the best I've had. Although the course is decently tough, if you took AP Econ in Highschool, you'll be fine. Otherwise, he provides very good lectures and is very accessible if you have questions. The hw is harder than the tests, and the practice problems are identical/very similar to tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A77" s="105" t="inlineStr"/>
+      <c r="B77" s="105" t="inlineStr">
+        <is>
+          <t>2023-04-06</t>
+        </is>
+      </c>
+      <c r="C77" s="105" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D77" s="105" t="inlineStr">
+        <is>
+          <t>5/3</t>
+        </is>
+      </c>
+      <c r="E77" s="8" t="inlineStr">
+        <is>
+          <t>Despite the difficulty of Micro, Professor Martinez-Marquina's lectures are engaging, practical, and interactive. He emphasizes building intuition to see the world from a different perspective and is readily available for support outside of class. Professor Martinez-Marquina's passion and expertise in the subject matter further enrich his lectures. [Amazing lectures, Inspirational, Respected]</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="A78" s="107" t="inlineStr"/>
+      <c r="B78" s="107" t="inlineStr">
+        <is>
+          <t>2023-04-06</t>
+        </is>
+      </c>
+      <c r="C78" s="107" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D78" s="107" t="inlineStr">
+        <is>
+          <t>5/4</t>
+        </is>
+      </c>
+      <c r="E78" s="11" t="inlineStr">
+        <is>
+          <t>Thought he was going to be hard since he was new, but ended up being one of the most chill professors I've had. Makes homework harder than the exams, but uses examples similar to slides. Keeps lectures entertaining. [Amazing lectures, Caring]</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A79" s="105" t="inlineStr"/>
+      <c r="B79" s="105" t="inlineStr">
+        <is>
+          <t>2023-04-05</t>
+        </is>
+      </c>
+      <c r="C79" s="105" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="D79" s="105" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E79" s="8" t="inlineStr">
+        <is>
+          <t>The hardest class at usc, but he makes it worth it. Great professor overall - willing to work with students to help with exams and understanding the material. His lectures go by very fast, and his accent can be hard to understand at first. Go to office hours, read the textbook, pay attention and go to every single class...and maybe you'll pass. [Caring, Test heavy, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" hidden="1" outlineLevel="1"/>
+    <row r="81" hidden="1" outlineLevel="1">
+      <c r="A81" s="91" t="inlineStr">
         <is>
           <t>RMP data as of 2026-08-21. Source: ratemyprofessors.com. Avg reviewer grade = mean of self-reported letter grades (4.0 scale); not all reviewers report a grade.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="83" ht="28" customHeight="1">
+      <c r="A83" s="4" t="inlineStr">
         <is>
           <t>Connect prep (e.g. BUAD-304 Personal Assessments) is ungraded class prep - not part of Participation or other graded categories.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
+    <row r="84" ht="32" customHeight="1">
+      <c r="A84" s="5" t="inlineStr">
         <is>
           <t>Start here (graded): 2026-09-04 - ECON-351 - Homework: Homework 1 (Chapter 4) — Brightspace, due 11:59 pm</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B86" s="6" t="inlineStr">
         <is>
           <t>Reading</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C86" s="6" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D86" s="6" t="inlineStr">
         <is>
           <t>Papers</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="E86" s="6" t="inlineStr">
         <is>
           <t>Group Project</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F86" s="6" t="inlineStr">
         <is>
           <t>External certs</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="G86" s="6" t="inlineStr">
         <is>
           <t>Connect prep</t>
         </is>
       </c>
-      <c r="H21" s="6" t="inlineStr">
+      <c r="H86" s="6" t="inlineStr">
         <is>
           <t>First assignment</t>
         </is>
       </c>
-      <c r="I21" s="6" t="inlineStr">
+      <c r="I86" s="6" t="inlineStr">
         <is>
           <t>Assign due</t>
         </is>
       </c>
-      <c r="J21" s="6" t="inlineStr">
+      <c r="J86" s="6" t="inlineStr">
         <is>
           <t>First major</t>
         </is>
       </c>
-      <c r="K21" s="6" t="inlineStr">
+      <c r="K86" s="6" t="inlineStr">
         <is>
           <t>Major due</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="7">
+    <row r="87">
+      <c r="A87" s="7">
         <f>HYPERLINK("#'BUAD-281'!A1","BUAD-281")</f>
         <v/>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B87" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C87" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D87" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E87" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="F87" s="9" t="inlineStr">
         <is>
           <t>LinkedIn Learning Excel Certification, Stukent Simternship</t>
         </is>
       </c>
-      <c r="G22" s="8" t="inlineStr">
+      <c r="G87" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H22" s="8" t="inlineStr">
+      <c r="H87" s="8" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
         </is>
       </c>
-      <c r="I22" s="8" t="inlineStr">
+      <c r="I87" s="8" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="J22" s="8" t="inlineStr">
+      <c r="J87" s="8" t="inlineStr">
         <is>
           <t>Midterm 1</t>
         </is>
       </c>
-      <c r="K22" s="8" t="inlineStr">
+      <c r="K87" s="8" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="10">
+    <row r="88">
+      <c r="A88" s="10">
         <f>HYPERLINK("#'BUAD-304'!A1","BUAD-304")</f>
         <v/>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B88" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
+      <c r="C88" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D23" s="11" t="inlineStr">
+      <c r="D88" s="11" t="inlineStr">
         <is>
           <t>Final Reflection Paper, Team Project Paper</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="E88" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F23" s="11" t="inlineStr">
+      <c r="F88" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G23" s="12" t="inlineStr">
+      <c r="G88" s="12" t="inlineStr">
         <is>
           <t>Ungraded prep</t>
         </is>
       </c>
-      <c r="H23" s="11" t="inlineStr">
+      <c r="H88" s="11" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.01 - What is my Big thinking</t>
         </is>
       </c>
-      <c r="I23" s="11" t="inlineStr">
+      <c r="I88" s="11" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="J23" s="11" t="inlineStr">
+      <c r="J88" s="11" t="inlineStr">
         <is>
           <t>Thomas Green Case Analysis Memo</t>
         </is>
       </c>
-      <c r="K23" s="11" t="inlineStr">
+      <c r="K88" s="11" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="7">
+    <row r="89">
+      <c r="A89" s="7">
         <f>HYPERLINK("#'ECON-351'!A1","ECON-351")</f>
         <v/>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B89" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C89" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D89" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E89" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F24" s="8" t="inlineStr">
+      <c r="F89" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G24" s="8" t="inlineStr">
+      <c r="G89" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H24" s="8" t="inlineStr">
+      <c r="H89" s="8" t="inlineStr">
         <is>
           <t>Homework 1 (Chapter 4) — Brightspace, due 11:59 pm</t>
         </is>
       </c>
-      <c r="I24" s="8" t="inlineStr">
+      <c r="I89" s="8" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="J24" s="8" t="inlineStr">
+      <c r="J89" s="8" t="inlineStr">
         <is>
           <t>First midterm exam</t>
         </is>
       </c>
-      <c r="K24" s="8" t="inlineStr">
+      <c r="K89" s="8" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="10">
+    <row r="90">
+      <c r="A90" s="10">
         <f>HYPERLINK("#'HIST-103'!A1","HIST-103")</f>
         <v/>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B90" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C25" s="11" t="inlineStr">
+      <c r="C90" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D25" s="11" t="inlineStr">
+      <c r="D90" s="11" t="inlineStr">
         <is>
           <t>Sleep Paper, Witchcraft Paper</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E90" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F25" s="11" t="inlineStr">
+      <c r="F90" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G25" s="11" t="inlineStr">
+      <c r="G90" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H25" s="11" t="inlineStr">
+      <c r="H90" s="11" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
         </is>
       </c>
-      <c r="I25" s="11" t="inlineStr">
+      <c r="I90" s="11" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="J25" s="11" t="inlineStr">
+      <c r="J90" s="11" t="inlineStr">
         <is>
           <t>Sleep Paper</t>
         </is>
       </c>
-      <c r="K25" s="11" t="inlineStr">
+      <c r="K90" s="11" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="13" t="inlineStr">
         <is>
           <t>Do First - August 2026 - graded assignments (first per class always listed)</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="14" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="14" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="B28" s="14" t="inlineStr">
+      <c r="B93" s="14" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="C28" s="14" t="inlineStr">
+      <c r="C93" s="14" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D28" s="14" t="inlineStr">
+      <c r="D93" s="14" t="inlineStr">
         <is>
           <t>Graded?</t>
         </is>
       </c>
-      <c r="E28" s="14" t="inlineStr">
+      <c r="E93" s="14" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="8" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="B29" s="8" t="inlineStr">
+      <c r="B94" s="8" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="C29" s="15" t="inlineStr">
+      <c r="C94" s="15" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D29" s="8" t="inlineStr">
+      <c r="D94" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E29" s="8" t="inlineStr">
+      <c r="E94" s="8" t="inlineStr">
         <is>
           <t>Homework 1 (Chapter 4) — Brightspace, due 11:59 pm</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="11" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="11" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="B30" s="11" t="inlineStr">
+      <c r="B95" s="11" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C30" s="46" t="inlineStr">
+      <c r="C95" s="46" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D30" s="11" t="inlineStr">
+      <c r="D95" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E30" s="11" t="inlineStr">
+      <c r="E95" s="11" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="8" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="B31" s="8" t="inlineStr">
+      <c r="B96" s="8" t="inlineStr">
         <is>
           <t>HIST-103</t>
         </is>
       </c>
-      <c r="C31" s="25" t="inlineStr">
+      <c r="C96" s="25" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D31" s="8" t="inlineStr">
+      <c r="D96" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E31" s="8" t="inlineStr">
+      <c r="E96" s="8" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="17" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="17" t="inlineStr">
         <is>
           <t>Do First - August 2026 - Connect prep only (ungraded, not Participation)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="18" t="inlineStr">
+    <row r="99">
+      <c r="A99" s="18" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="B34" s="18" t="inlineStr">
+      <c r="B99" s="18" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="C34" s="18" t="inlineStr">
+      <c r="C99" s="18" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D34" s="18" t="inlineStr">
+      <c r="D99" s="18" t="inlineStr">
         <is>
           <t>Graded?</t>
         </is>
       </c>
-      <c r="E34" s="18" t="inlineStr">
+      <c r="E99" s="18" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="19" t="inlineStr">
+    <row r="100">
+      <c r="A100" s="19" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B35" s="19" t="inlineStr">
+      <c r="B100" s="19" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C35" s="20" t="inlineStr">
+      <c r="C100" s="20" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D35" s="21" t="inlineStr">
+      <c r="D100" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E35" s="19" t="inlineStr">
+      <c r="E100" s="19" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="22" t="inlineStr">
+    <row r="101">
+      <c r="A101" s="22" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B36" s="22" t="inlineStr">
+      <c r="B101" s="22" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C36" s="23" t="inlineStr">
+      <c r="C101" s="23" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D36" s="24" t="inlineStr">
+      <c r="D101" s="24" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E36" s="22" t="inlineStr">
+      <c r="E101" s="22" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="13" t="inlineStr">
+    <row r="103">
+      <c r="A103" s="13" t="inlineStr">
         <is>
           <t>Upcoming graded assignments (next 45 days)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="14" t="inlineStr">
+    <row r="104">
+      <c r="A104" s="14" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="B39" s="14" t="inlineStr">
+      <c r="B104" s="14" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="C39" s="14" t="inlineStr">
+      <c r="C104" s="14" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D39" s="14" t="inlineStr">
+      <c r="D104" s="14" t="inlineStr">
         <is>
           <t>Graded?</t>
         </is>
       </c>
-      <c r="E39" s="14" t="inlineStr">
+      <c r="E104" s="14" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="8" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B105" s="8" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="C40" s="15" t="inlineStr">
+      <c r="C105" s="15" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D40" s="8" t="inlineStr">
+      <c r="D105" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E40" s="8" t="inlineStr">
+      <c r="E105" s="8" t="inlineStr">
         <is>
           <t>Homework 1 (Chapter 4) — Brightspace, due 11:59 pm</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="11" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="11" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="B41" s="11" t="inlineStr">
+      <c r="B106" s="11" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C41" s="46" t="inlineStr">
+      <c r="C106" s="46" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D41" s="11" t="inlineStr">
+      <c r="D106" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E41" s="11" t="inlineStr">
+      <c r="E106" s="11" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+    <row r="107">
+      <c r="A107" s="8" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B107" s="8" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="C42" s="15" t="inlineStr">
+      <c r="C107" s="15" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D42" s="8" t="inlineStr">
+      <c r="D107" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E42" s="8" t="inlineStr">
+      <c r="E107" s="8" t="inlineStr">
         <is>
           <t>Homework 2 (Chapter 9) — Brightspace, due 11:59 pm</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="11" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="11" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="B43" s="11" t="inlineStr">
+      <c r="B108" s="11" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="C43" s="120" t="inlineStr">
+      <c r="C108" s="120" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="D43" s="11" t="inlineStr">
+      <c r="D108" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E43" s="11" t="inlineStr">
+      <c r="E108" s="11" t="inlineStr">
         <is>
           <t>Midterm 1 — covers Chapters 4 and 9</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+    <row r="109">
+      <c r="A109" s="8" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="B44" s="8" t="inlineStr">
+      <c r="B109" s="8" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="C44" s="25" t="inlineStr">
+      <c r="C109" s="25" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D44" s="8" t="inlineStr">
+      <c r="D109" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E44" s="8" t="inlineStr">
+      <c r="E109" s="8" t="inlineStr">
         <is>
           <t>First midterm exam</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="11" t="inlineStr">
+    <row r="110">
+      <c r="A110" s="11" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="B45" s="11" t="inlineStr">
+      <c r="B110" s="11" t="inlineStr">
         <is>
           <t>HIST-103</t>
         </is>
       </c>
-      <c r="C45" s="16" t="inlineStr">
+      <c r="C110" s="16" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D45" s="11" t="inlineStr">
+      <c r="D110" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E45" s="11" t="inlineStr">
+      <c r="E110" s="11" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+    <row r="111">
+      <c r="A111" s="8" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="B46" s="8" t="inlineStr">
+      <c r="B111" s="8" t="inlineStr">
         <is>
           <t>HIST-103</t>
         </is>
       </c>
-      <c r="C46" s="25" t="inlineStr">
+      <c r="C111" s="25" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D46" s="8" t="inlineStr">
+      <c r="D111" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E46" s="8" t="inlineStr">
+      <c r="E111" s="8" t="inlineStr">
         <is>
           <t>Sleep Paper</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="11" t="inlineStr">
+    <row r="112">
+      <c r="A112" s="11" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="B47" s="11" t="inlineStr">
+      <c r="B112" s="11" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C47" s="46" t="inlineStr">
+      <c r="C112" s="46" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D47" s="11" t="inlineStr">
+      <c r="D112" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E47" s="11" t="inlineStr">
+      <c r="E112" s="11" t="inlineStr">
         <is>
           <t>Class 7 (9/16) - 3-24, 3-28, 3-32; 15 Points</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+    <row r="113">
+      <c r="A113" s="8" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B113" s="8" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C48" s="25" t="inlineStr">
+      <c r="C113" s="25" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D48" s="8" t="inlineStr">
+      <c r="D113" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E48" s="8" t="inlineStr">
+      <c r="E113" s="8" t="inlineStr">
         <is>
           <t>Thomas Green Case Analysis Memo</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="11" t="inlineStr">
+    <row r="114">
+      <c r="A114" s="11" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="B49" s="11" t="inlineStr">
+      <c r="B114" s="11" t="inlineStr">
         <is>
           <t>HIST-103</t>
         </is>
       </c>
-      <c r="C49" s="16" t="inlineStr">
+      <c r="C114" s="16" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D49" s="11" t="inlineStr">
+      <c r="D114" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E49" s="11" t="inlineStr">
+      <c r="E114" s="11" t="inlineStr">
         <is>
           <t>Final Exam</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="8" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B115" s="8" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="C50" s="15" t="inlineStr">
+      <c r="C115" s="15" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D50" s="8" t="inlineStr">
+      <c r="D115" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E50" s="8" t="inlineStr">
+      <c r="E115" s="8" t="inlineStr">
         <is>
           <t>Homework 3 — Brightspace, due 11:59 pm</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="11" t="inlineStr">
+    <row r="116">
+      <c r="A116" s="11" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="B51" s="11" t="inlineStr">
+      <c r="B116" s="11" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C51" s="46" t="inlineStr">
+      <c r="C116" s="46" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D51" s="11" t="inlineStr">
+      <c r="D116" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E51" s="11" t="inlineStr">
+      <c r="E116" s="11" t="inlineStr">
         <is>
           <t>Class 8 (9/21) - 5-27 5-46; 10 Points</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="8" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="B52" s="8" t="inlineStr">
+      <c r="B117" s="8" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C52" s="15" t="inlineStr">
+      <c r="C117" s="15" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D52" s="8" t="inlineStr">
+      <c r="D117" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E52" s="8" t="inlineStr">
+      <c r="E117" s="8" t="inlineStr">
         <is>
           <t>Class 9 (9/23) - 4-21, 4-22; 10 Points</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="11" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="11" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="B53" s="11" t="inlineStr">
+      <c r="B118" s="11" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="C53" s="46" t="inlineStr">
+      <c r="C118" s="46" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D53" s="11" t="inlineStr">
+      <c r="D118" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E53" s="11" t="inlineStr">
+      <c r="E118" s="11" t="inlineStr">
         <is>
           <t>Homework 4 (Chapter 3) — Brightspace, due 11:59 pm</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="8" t="inlineStr">
+    <row r="119">
+      <c r="A119" s="8" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="B54" s="8" t="inlineStr">
+      <c r="B119" s="8" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C54" s="26" t="inlineStr">
+      <c r="C119" s="26" t="inlineStr">
         <is>
           <t>Research</t>
         </is>
       </c>
-      <c r="D54" s="8" t="inlineStr">
+      <c r="D119" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E54" s="8" t="inlineStr">
+      <c r="E119" s="8" t="inlineStr">
         <is>
           <t>Research: Setup deadline (registration, prescreening, contacts)</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="11" t="inlineStr">
+    <row r="120">
+      <c r="A120" s="11" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="B55" s="11" t="inlineStr">
+      <c r="B120" s="11" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C55" s="46" t="inlineStr">
+      <c r="C120" s="46" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D55" s="11" t="inlineStr">
+      <c r="D120" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E55" s="11" t="inlineStr">
+      <c r="E120" s="11" t="inlineStr">
         <is>
           <t>Class 10 (9/28) - 8-28, 8-29; 10 Points</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="8" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="B56" s="8" t="inlineStr">
+      <c r="B121" s="8" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C56" s="25" t="inlineStr">
+      <c r="C121" s="25" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D56" s="8" t="inlineStr">
+      <c r="D121" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E56" s="8" t="inlineStr">
+      <c r="E121" s="8" t="inlineStr">
         <is>
           <t>Team project proposal &amp; team contract</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="11" t="inlineStr">
+    <row r="122">
+      <c r="A122" s="11" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="B57" s="11" t="inlineStr">
+      <c r="B122" s="11" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C57" s="16" t="inlineStr">
+      <c r="C122" s="16" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D57" s="11" t="inlineStr">
+      <c r="D122" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E57" s="11" t="inlineStr">
+      <c r="E122" s="11" t="inlineStr">
         <is>
           <t>Proposal &amp; Team Contract</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="8" t="inlineStr">
+    <row r="123">
+      <c r="A123" s="8" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B58" s="8" t="inlineStr">
+      <c r="B123" s="8" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C58" s="47" t="inlineStr">
+      <c r="C123" s="47" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="D58" s="8" t="inlineStr">
+      <c r="D123" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E58" s="8" t="inlineStr">
+      <c r="E123" s="8" t="inlineStr">
         <is>
           <t>9/30 Midterm 1: 250 Points Chapters 1, 2, 3, 4, 5, 8</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="11" t="inlineStr">
+    <row r="124">
+      <c r="A124" s="11" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B59" s="11" t="inlineStr">
+      <c r="B124" s="11" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C59" s="16" t="inlineStr">
+      <c r="C124" s="16" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D59" s="11" t="inlineStr">
+      <c r="D124" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E59" s="11" t="inlineStr">
+      <c r="E124" s="11" t="inlineStr">
         <is>
           <t>Midterm 1</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="8" t="inlineStr">
+    <row r="125">
+      <c r="A125" s="8" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B60" s="8" t="inlineStr">
+      <c r="B125" s="8" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="C60" s="15" t="inlineStr">
+      <c r="C125" s="15" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D60" s="8" t="inlineStr">
+      <c r="D125" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E60" s="8" t="inlineStr">
+      <c r="E125" s="8" t="inlineStr">
         <is>
           <t>Homework 5 (Chapter 5) — Brightspace, due 11:59 pm</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="11" t="inlineStr">
+    <row r="126">
+      <c r="A126" s="11" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B61" s="11" t="inlineStr">
+      <c r="B126" s="11" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="C61" s="16" t="inlineStr">
+      <c r="C126" s="16" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D61" s="11" t="inlineStr">
+      <c r="D126" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E61" s="11" t="inlineStr">
+      <c r="E126" s="11" t="inlineStr">
         <is>
           <t>AI Forecast Project — Part I</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="C15:K15"/>
-    <mergeCell ref="A18:K18"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A3:K3"/>
+  <mergeCells count="77">
+    <mergeCell ref="E36:K36"/>
+    <mergeCell ref="E75:K75"/>
+    <mergeCell ref="E22:K22"/>
+    <mergeCell ref="E53:K53"/>
+    <mergeCell ref="E55:K55"/>
+    <mergeCell ref="E67:K67"/>
+    <mergeCell ref="E39:K39"/>
+    <mergeCell ref="E48:K48"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="E29:K29"/>
+    <mergeCell ref="E38:K38"/>
+    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="E31:K31"/>
+    <mergeCell ref="E40:K40"/>
     <mergeCell ref="C14:K14"/>
-    <mergeCell ref="C13:K13"/>
-    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="E26:K26"/>
     <mergeCell ref="A11:K11"/>
-    <mergeCell ref="A16:K16"/>
-    <mergeCell ref="A19:K19"/>
-    <mergeCell ref="A33:K33"/>
-    <mergeCell ref="A38:K38"/>
+    <mergeCell ref="A98:K98"/>
+    <mergeCell ref="E76:K76"/>
+    <mergeCell ref="E25:K25"/>
+    <mergeCell ref="E66:K66"/>
+    <mergeCell ref="E58:K58"/>
+    <mergeCell ref="E50:K50"/>
+    <mergeCell ref="E68:K68"/>
+    <mergeCell ref="E42:K42"/>
+    <mergeCell ref="E52:K52"/>
+    <mergeCell ref="E44:K44"/>
+    <mergeCell ref="E20:K20"/>
+    <mergeCell ref="E69:K69"/>
+    <mergeCell ref="E78:K78"/>
+    <mergeCell ref="E30:K30"/>
+    <mergeCell ref="E59:K59"/>
+    <mergeCell ref="E77:K77"/>
+    <mergeCell ref="E46:K46"/>
+    <mergeCell ref="A83:K83"/>
+    <mergeCell ref="E61:K61"/>
+    <mergeCell ref="A92:K92"/>
+    <mergeCell ref="E70:K70"/>
+    <mergeCell ref="E57:K57"/>
+    <mergeCell ref="E54:K54"/>
+    <mergeCell ref="E32:K32"/>
+    <mergeCell ref="E72:K72"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="C12:K12"/>
-    <mergeCell ref="A27:K27"/>
+    <mergeCell ref="E41:K41"/>
+    <mergeCell ref="A103:K103"/>
+    <mergeCell ref="E47:K47"/>
+    <mergeCell ref="E56:K56"/>
+    <mergeCell ref="E43:K43"/>
+    <mergeCell ref="E24:K24"/>
+    <mergeCell ref="E33:K33"/>
+    <mergeCell ref="E35:K35"/>
+    <mergeCell ref="E19:K19"/>
+    <mergeCell ref="E28:K28"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="E60:K60"/>
+    <mergeCell ref="E74:K74"/>
+    <mergeCell ref="E45:K45"/>
+    <mergeCell ref="E37:K37"/>
+    <mergeCell ref="E21:K21"/>
+    <mergeCell ref="A84:K84"/>
+    <mergeCell ref="E62:K62"/>
+    <mergeCell ref="E71:K71"/>
+    <mergeCell ref="E23:K23"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="E64:K64"/>
+    <mergeCell ref="E79:K79"/>
+    <mergeCell ref="C13:K13"/>
+    <mergeCell ref="E73:K73"/>
+    <mergeCell ref="E51:K51"/>
+    <mergeCell ref="E63:K63"/>
+    <mergeCell ref="C15:K15"/>
+    <mergeCell ref="E65:K65"/>
+    <mergeCell ref="A81:K81"/>
+    <mergeCell ref="E34:K34"/>
+    <mergeCell ref="E49:K49"/>
+    <mergeCell ref="E27:K27"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId1"/>
@@ -5807,18 +7325,18 @@
           <t>First midterm exam</t>
         </is>
       </c>
-      <c r="B10" s="142" t="inlineStr">
+      <c r="B10" s="146" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C10" s="143" t="inlineStr"/>
-      <c r="D10" s="143" t="inlineStr">
+      <c r="C10" s="147" t="inlineStr"/>
+      <c r="D10" s="147" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="E10" s="143" t="inlineStr">
+      <c r="E10" s="147" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5834,14 +7352,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B11" s="144" t="inlineStr"/>
-      <c r="C11" s="144" t="inlineStr"/>
-      <c r="D11" s="144" t="inlineStr">
+      <c r="B11" s="148" t="inlineStr"/>
+      <c r="C11" s="148" t="inlineStr"/>
+      <c r="D11" s="148" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="E11" s="144" t="inlineStr"/>
+      <c r="E11" s="148" t="inlineStr"/>
       <c r="F11" s="130" t="inlineStr">
         <is>
           <t>Midterm 1 — covers Chapters 4 and 9</t>
@@ -5854,18 +7372,18 @@
           <t>Second midterm exam</t>
         </is>
       </c>
-      <c r="B12" s="142" t="inlineStr">
+      <c r="B12" s="146" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C12" s="145" t="inlineStr"/>
-      <c r="D12" s="145" t="inlineStr">
+      <c r="C12" s="149" t="inlineStr"/>
+      <c r="D12" s="149" t="inlineStr">
         <is>
           <t>2026-10-12</t>
         </is>
       </c>
-      <c r="E12" s="145" t="inlineStr">
+      <c r="E12" s="149" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5881,14 +7399,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B13" s="144" t="inlineStr"/>
-      <c r="C13" s="144" t="inlineStr"/>
-      <c r="D13" s="144" t="inlineStr">
+      <c r="B13" s="148" t="inlineStr"/>
+      <c r="C13" s="148" t="inlineStr"/>
+      <c r="D13" s="148" t="inlineStr">
         <is>
           <t>2026-10-12</t>
         </is>
       </c>
-      <c r="E13" s="144" t="inlineStr"/>
+      <c r="E13" s="148" t="inlineStr"/>
       <c r="F13" s="130" t="inlineStr">
         <is>
           <t>Midterm 2 — covers Chapters 3, 5, and 6</t>
@@ -5901,18 +7419,18 @@
           <t>Third midterm exam</t>
         </is>
       </c>
-      <c r="B14" s="142" t="inlineStr">
+      <c r="B14" s="146" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C14" s="143" t="inlineStr"/>
-      <c r="D14" s="143" t="inlineStr">
+      <c r="C14" s="147" t="inlineStr"/>
+      <c r="D14" s="147" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="E14" s="143" t="inlineStr">
+      <c r="E14" s="147" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5928,14 +7446,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B15" s="144" t="inlineStr"/>
-      <c r="C15" s="144" t="inlineStr"/>
-      <c r="D15" s="144" t="inlineStr">
+      <c r="B15" s="148" t="inlineStr"/>
+      <c r="C15" s="148" t="inlineStr"/>
+      <c r="D15" s="148" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="E15" s="144" t="inlineStr"/>
+      <c r="E15" s="148" t="inlineStr"/>
       <c r="F15" s="130" t="inlineStr">
         <is>
           <t>Midterm 3 — covers Chapters 7, 8, and 10</t>
@@ -5948,18 +7466,18 @@
           <t>Fourth midterm exam</t>
         </is>
       </c>
-      <c r="B16" s="142" t="inlineStr">
+      <c r="B16" s="146" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C16" s="145" t="inlineStr"/>
-      <c r="D16" s="145" t="inlineStr">
+      <c r="C16" s="149" t="inlineStr"/>
+      <c r="D16" s="149" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E16" s="145" t="inlineStr">
+      <c r="E16" s="149" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -5975,14 +7493,14 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B17" s="144" t="inlineStr"/>
-      <c r="C17" s="144" t="inlineStr"/>
-      <c r="D17" s="144" t="inlineStr">
+      <c r="B17" s="148" t="inlineStr"/>
+      <c r="C17" s="148" t="inlineStr"/>
+      <c r="D17" s="148" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E17" s="144" t="inlineStr"/>
+      <c r="E17" s="148" t="inlineStr"/>
       <c r="F17" s="130" t="inlineStr">
         <is>
           <t>Midterm 4 — covers Chapters 11, 12, and 13</t>
@@ -5995,18 +7513,18 @@
           <t>AI Forecast Project</t>
         </is>
       </c>
-      <c r="B18" s="142" t="inlineStr">
+      <c r="B18" s="146" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C18" s="143" t="inlineStr"/>
-      <c r="D18" s="143" t="inlineStr">
+      <c r="C18" s="147" t="inlineStr"/>
+      <c r="D18" s="147" t="inlineStr">
         <is>
           <t>2026-12-11</t>
         </is>
       </c>
-      <c r="E18" s="143" t="inlineStr">
+      <c r="E18" s="147" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -6022,14 +7540,14 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B19" s="144" t="inlineStr"/>
-      <c r="C19" s="144" t="inlineStr"/>
-      <c r="D19" s="144" t="inlineStr">
+      <c r="B19" s="148" t="inlineStr"/>
+      <c r="C19" s="148" t="inlineStr"/>
+      <c r="D19" s="148" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="E19" s="144" t="inlineStr"/>
+      <c r="E19" s="148" t="inlineStr"/>
       <c r="F19" s="130" t="inlineStr">
         <is>
           <t>AI Forecast Project — Part I</t>
@@ -6042,14 +7560,14 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B20" s="144" t="inlineStr"/>
-      <c r="C20" s="144" t="inlineStr"/>
-      <c r="D20" s="144" t="inlineStr">
+      <c r="B20" s="148" t="inlineStr"/>
+      <c r="C20" s="148" t="inlineStr"/>
+      <c r="D20" s="148" t="inlineStr">
         <is>
           <t>2026-12-11</t>
         </is>
       </c>
-      <c r="E20" s="144" t="inlineStr"/>
+      <c r="E20" s="148" t="inlineStr"/>
       <c r="F20" s="130" t="inlineStr">
         <is>
           <t>AI Forecast Project — Part II</t>
@@ -6062,18 +7580,18 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B21" s="142" t="inlineStr">
+      <c r="B21" s="146" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C21" s="145" t="inlineStr"/>
-      <c r="D21" s="145" t="inlineStr">
+      <c r="C21" s="149" t="inlineStr"/>
+      <c r="D21" s="149" t="inlineStr">
         <is>
           <t>2026-11-27</t>
         </is>
       </c>
-      <c r="E21" s="145" t="inlineStr">
+      <c r="E21" s="149" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -6089,10 +7607,10 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B22" s="144" t="inlineStr"/>
-      <c r="C22" s="144" t="inlineStr"/>
-      <c r="D22" s="144" t="inlineStr"/>
-      <c r="E22" s="144" t="inlineStr"/>
+      <c r="B22" s="148" t="inlineStr"/>
+      <c r="C22" s="148" t="inlineStr"/>
+      <c r="D22" s="148" t="inlineStr"/>
+      <c r="E22" s="148" t="inlineStr"/>
       <c r="F22" s="130" t="inlineStr">
         <is>
           <t>Finals Week: - AI Project – Part II due December 11</t>
@@ -6105,14 +7623,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B23" s="144" t="inlineStr"/>
-      <c r="C23" s="144" t="inlineStr"/>
-      <c r="D23" s="144" t="inlineStr">
+      <c r="B23" s="148" t="inlineStr"/>
+      <c r="C23" s="148" t="inlineStr"/>
+      <c r="D23" s="148" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="E23" s="144" t="inlineStr"/>
+      <c r="E23" s="148" t="inlineStr"/>
       <c r="F23" s="130" t="inlineStr">
         <is>
           <t>Week 1: Aug.24/26 - Complete the math self-assessment on Brightspace</t>
@@ -6125,14 +7643,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B24" s="144" t="inlineStr"/>
-      <c r="C24" s="144" t="inlineStr"/>
-      <c r="D24" s="144" t="inlineStr">
+      <c r="B24" s="148" t="inlineStr"/>
+      <c r="C24" s="148" t="inlineStr"/>
+      <c r="D24" s="148" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="E24" s="144" t="inlineStr"/>
+      <c r="E24" s="148" t="inlineStr"/>
       <c r="F24" s="130" t="inlineStr">
         <is>
           <t>Week 1: Aug.24/26 - Read Chapters 2 and 4</t>
@@ -6145,14 +7663,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B25" s="144" t="inlineStr"/>
-      <c r="C25" s="144" t="inlineStr"/>
-      <c r="D25" s="144" t="inlineStr">
+      <c r="B25" s="148" t="inlineStr"/>
+      <c r="C25" s="148" t="inlineStr"/>
+      <c r="D25" s="148" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="E25" s="144" t="inlineStr"/>
+      <c r="E25" s="148" t="inlineStr"/>
       <c r="F25" s="130" t="inlineStr">
         <is>
           <t>Week 1: Aug.24/26 - Read the syllabus</t>
@@ -6165,14 +7683,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B26" s="144" t="inlineStr"/>
-      <c r="C26" s="144" t="inlineStr"/>
-      <c r="D26" s="144" t="inlineStr">
+      <c r="B26" s="148" t="inlineStr"/>
+      <c r="C26" s="148" t="inlineStr"/>
+      <c r="D26" s="148" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E26" s="144" t="inlineStr"/>
+      <c r="E26" s="148" t="inlineStr"/>
       <c r="F26" s="130" t="inlineStr">
         <is>
           <t>Week 2: Aug.31/Sep.2 - Begin Chapter 9: Uncertainty</t>
@@ -6185,14 +7703,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B27" s="144" t="inlineStr"/>
-      <c r="C27" s="144" t="inlineStr"/>
-      <c r="D27" s="144" t="inlineStr">
+      <c r="B27" s="148" t="inlineStr"/>
+      <c r="C27" s="148" t="inlineStr"/>
+      <c r="D27" s="148" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E27" s="144" t="inlineStr"/>
+      <c r="E27" s="148" t="inlineStr"/>
       <c r="F27" s="130" t="inlineStr">
         <is>
           <t>Week 2: Aug.31/Sep.2 - Finish reading Chapter 4 (in-class dis- cussion)</t>
@@ -6205,14 +7723,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B28" s="144" t="inlineStr"/>
-      <c r="C28" s="144" t="inlineStr"/>
-      <c r="D28" s="144" t="inlineStr">
+      <c r="B28" s="148" t="inlineStr"/>
+      <c r="C28" s="148" t="inlineStr"/>
+      <c r="D28" s="148" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E28" s="144" t="inlineStr"/>
+      <c r="E28" s="148" t="inlineStr"/>
       <c r="F28" s="130" t="inlineStr">
         <is>
           <t>Homework 1 (Chapter 4) — Brightspace, due 11:59 pm</t>
@@ -6225,14 +7743,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B29" s="144" t="inlineStr"/>
-      <c r="C29" s="144" t="inlineStr"/>
-      <c r="D29" s="144" t="inlineStr">
+      <c r="B29" s="148" t="inlineStr"/>
+      <c r="C29" s="148" t="inlineStr"/>
+      <c r="D29" s="148" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E29" s="144" t="inlineStr"/>
+      <c r="E29" s="148" t="inlineStr"/>
       <c r="F29" s="130" t="inlineStr">
         <is>
           <t>Week 3: Sep.7/9 - Discussion of Chapter 9</t>
@@ -6245,14 +7763,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B30" s="144" t="inlineStr"/>
-      <c r="C30" s="144" t="inlineStr"/>
-      <c r="D30" s="144" t="inlineStr">
+      <c r="B30" s="148" t="inlineStr"/>
+      <c r="C30" s="148" t="inlineStr"/>
+      <c r="D30" s="148" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E30" s="144" t="inlineStr"/>
+      <c r="E30" s="148" t="inlineStr"/>
       <c r="F30" s="130" t="inlineStr">
         <is>
           <t>Week 3: Sep.7/9 - No class Monday Sep.7 (Labor Day)</t>
@@ -6265,14 +7783,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B31" s="144" t="inlineStr"/>
-      <c r="C31" s="144" t="inlineStr"/>
-      <c r="D31" s="144" t="inlineStr">
+      <c r="B31" s="148" t="inlineStr"/>
+      <c r="C31" s="148" t="inlineStr"/>
+      <c r="D31" s="148" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="E31" s="144" t="inlineStr"/>
+      <c r="E31" s="148" t="inlineStr"/>
       <c r="F31" s="130" t="inlineStr">
         <is>
           <t>Homework 2 (Chapter 9) — Brightspace, due 11:59 pm</t>
@@ -6285,14 +7803,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B32" s="144" t="inlineStr"/>
-      <c r="C32" s="144" t="inlineStr"/>
-      <c r="D32" s="144" t="inlineStr">
+      <c r="B32" s="148" t="inlineStr"/>
+      <c r="C32" s="148" t="inlineStr"/>
+      <c r="D32" s="148" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="E32" s="144" t="inlineStr"/>
+      <c r="E32" s="148" t="inlineStr"/>
       <c r="F32" s="130" t="inlineStr">
         <is>
           <t>Homework 3 — Brightspace, due 11:59 pm</t>
@@ -6305,14 +7823,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B33" s="144" t="inlineStr"/>
-      <c r="C33" s="144" t="inlineStr"/>
-      <c r="D33" s="144" t="inlineStr">
+      <c r="B33" s="148" t="inlineStr"/>
+      <c r="C33" s="148" t="inlineStr"/>
+      <c r="D33" s="148" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="E33" s="144" t="inlineStr"/>
+      <c r="E33" s="148" t="inlineStr"/>
       <c r="F33" s="130" t="inlineStr">
         <is>
           <t>Week 5: Sep.21/23 - Complete the Chapter 3 - Part II home- work on Brightspace (due Sep.25)</t>
@@ -6325,14 +7843,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B34" s="144" t="inlineStr"/>
-      <c r="C34" s="144" t="inlineStr"/>
-      <c r="D34" s="144" t="inlineStr">
+      <c r="B34" s="148" t="inlineStr"/>
+      <c r="C34" s="148" t="inlineStr"/>
+      <c r="D34" s="148" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="E34" s="144" t="inlineStr"/>
+      <c r="E34" s="148" t="inlineStr"/>
       <c r="F34" s="130" t="inlineStr">
         <is>
           <t>Week 5: Sep.21/23 - Discussion of Chapter 3</t>
@@ -6345,14 +7863,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B35" s="144" t="inlineStr"/>
-      <c r="C35" s="144" t="inlineStr"/>
-      <c r="D35" s="144" t="inlineStr">
+      <c r="B35" s="148" t="inlineStr"/>
+      <c r="C35" s="148" t="inlineStr"/>
+      <c r="D35" s="148" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="E35" s="144" t="inlineStr"/>
+      <c r="E35" s="148" t="inlineStr"/>
       <c r="F35" s="130" t="inlineStr">
         <is>
           <t>Week 5: Sep.21/23 - Finish reading Chapter 3</t>
@@ -6365,14 +7883,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B36" s="144" t="inlineStr"/>
-      <c r="C36" s="144" t="inlineStr"/>
-      <c r="D36" s="144" t="inlineStr">
+      <c r="B36" s="148" t="inlineStr"/>
+      <c r="C36" s="148" t="inlineStr"/>
+      <c r="D36" s="148" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="E36" s="144" t="inlineStr"/>
+      <c r="E36" s="148" t="inlineStr"/>
       <c r="F36" s="130" t="inlineStr">
         <is>
           <t>Homework 4 (Chapter 3) — Brightspace, due 11:59 pm</t>
@@ -6385,14 +7903,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B37" s="144" t="inlineStr"/>
-      <c r="C37" s="144" t="inlineStr"/>
-      <c r="D37" s="144" t="inlineStr">
+      <c r="B37" s="148" t="inlineStr"/>
+      <c r="C37" s="148" t="inlineStr"/>
+      <c r="D37" s="148" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="E37" s="144" t="inlineStr"/>
+      <c r="E37" s="148" t="inlineStr"/>
       <c r="F37" s="130" t="inlineStr">
         <is>
           <t>Week 6: Sep.28/30 - AI Project – Part I due October 2</t>
@@ -6405,14 +7923,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B38" s="144" t="inlineStr"/>
-      <c r="C38" s="144" t="inlineStr"/>
-      <c r="D38" s="144" t="inlineStr">
+      <c r="B38" s="148" t="inlineStr"/>
+      <c r="C38" s="148" t="inlineStr"/>
+      <c r="D38" s="148" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="E38" s="144" t="inlineStr"/>
+      <c r="E38" s="148" t="inlineStr"/>
       <c r="F38" s="130" t="inlineStr">
         <is>
           <t>Week 6: Sep.28/30 - Discussion of Chapter 5</t>
@@ -6425,14 +7943,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B39" s="144" t="inlineStr"/>
-      <c r="C39" s="144" t="inlineStr"/>
-      <c r="D39" s="144" t="inlineStr">
+      <c r="B39" s="148" t="inlineStr"/>
+      <c r="C39" s="148" t="inlineStr"/>
+      <c r="D39" s="148" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="E39" s="144" t="inlineStr"/>
+      <c r="E39" s="148" t="inlineStr"/>
       <c r="F39" s="130" t="inlineStr">
         <is>
           <t>Week 6: Sep.28/30 - Read Chapter 5</t>
@@ -6445,14 +7963,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B40" s="144" t="inlineStr"/>
-      <c r="C40" s="144" t="inlineStr"/>
-      <c r="D40" s="144" t="inlineStr">
+      <c r="B40" s="148" t="inlineStr"/>
+      <c r="C40" s="148" t="inlineStr"/>
+      <c r="D40" s="148" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="E40" s="144" t="inlineStr"/>
+      <c r="E40" s="148" t="inlineStr"/>
       <c r="F40" s="130" t="inlineStr">
         <is>
           <t>Homework 5 (Chapter 5) — Brightspace, due 11:59 pm</t>
@@ -6465,14 +7983,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B41" s="144" t="inlineStr"/>
-      <c r="C41" s="144" t="inlineStr"/>
-      <c r="D41" s="144" t="inlineStr">
+      <c r="B41" s="148" t="inlineStr"/>
+      <c r="C41" s="148" t="inlineStr"/>
+      <c r="D41" s="148" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E41" s="144" t="inlineStr"/>
+      <c r="E41" s="148" t="inlineStr"/>
       <c r="F41" s="130" t="inlineStr">
         <is>
           <t>Week 7: Oct.5/7 - Midterm review on Oct.7</t>
@@ -6485,14 +8003,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B42" s="144" t="inlineStr"/>
-      <c r="C42" s="144" t="inlineStr"/>
-      <c r="D42" s="144" t="inlineStr">
+      <c r="B42" s="148" t="inlineStr"/>
+      <c r="C42" s="148" t="inlineStr"/>
+      <c r="D42" s="148" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E42" s="144" t="inlineStr"/>
+      <c r="E42" s="148" t="inlineStr"/>
       <c r="F42" s="130" t="inlineStr">
         <is>
           <t>Week 7: Oct.5/7 - Read Chapter 6</t>
@@ -6505,14 +8023,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B43" s="144" t="inlineStr"/>
-      <c r="C43" s="144" t="inlineStr"/>
-      <c r="D43" s="144" t="inlineStr">
+      <c r="B43" s="148" t="inlineStr"/>
+      <c r="C43" s="148" t="inlineStr"/>
+      <c r="D43" s="148" t="inlineStr">
         <is>
           <t>2026-10-09</t>
         </is>
       </c>
-      <c r="E43" s="144" t="inlineStr"/>
+      <c r="E43" s="148" t="inlineStr"/>
       <c r="F43" s="130" t="inlineStr">
         <is>
           <t>Homework 6 (Chapter 6) — Brightspace, due 11:59 pm</t>
@@ -6525,14 +8043,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B44" s="144" t="inlineStr"/>
-      <c r="C44" s="144" t="inlineStr"/>
-      <c r="D44" s="144" t="inlineStr">
+      <c r="B44" s="148" t="inlineStr"/>
+      <c r="C44" s="148" t="inlineStr"/>
+      <c r="D44" s="148" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="E44" s="144" t="inlineStr"/>
+      <c r="E44" s="148" t="inlineStr"/>
       <c r="F44" s="130" t="inlineStr">
         <is>
           <t>Homework 7 — Brightspace, due 11:59 pm</t>
@@ -6545,14 +8063,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B45" s="144" t="inlineStr"/>
-      <c r="C45" s="144" t="inlineStr"/>
-      <c r="D45" s="144" t="inlineStr">
+      <c r="B45" s="148" t="inlineStr"/>
+      <c r="C45" s="148" t="inlineStr"/>
+      <c r="D45" s="148" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="E45" s="144" t="inlineStr"/>
+      <c r="E45" s="148" t="inlineStr"/>
       <c r="F45" s="130" t="inlineStr">
         <is>
           <t>Week 9: Oct.19/21 - Read Chapter 8</t>
@@ -6565,14 +8083,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B46" s="144" t="inlineStr"/>
-      <c r="C46" s="144" t="inlineStr"/>
-      <c r="D46" s="144" t="inlineStr">
+      <c r="B46" s="148" t="inlineStr"/>
+      <c r="C46" s="148" t="inlineStr"/>
+      <c r="D46" s="148" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="E46" s="144" t="inlineStr"/>
+      <c r="E46" s="148" t="inlineStr"/>
       <c r="F46" s="130" t="inlineStr">
         <is>
           <t>Homework 8 (Chapter 8) — Brightspace, due 11:59 pm</t>
@@ -6585,14 +8103,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B47" s="144" t="inlineStr"/>
-      <c r="C47" s="144" t="inlineStr"/>
-      <c r="D47" s="144" t="inlineStr">
+      <c r="B47" s="148" t="inlineStr"/>
+      <c r="C47" s="148" t="inlineStr"/>
+      <c r="D47" s="148" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E47" s="144" t="inlineStr"/>
+      <c r="E47" s="148" t="inlineStr"/>
       <c r="F47" s="130" t="inlineStr">
         <is>
           <t>Week 10: Oct.26/28 - Read Chapter 10</t>
@@ -6605,14 +8123,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B48" s="144" t="inlineStr"/>
-      <c r="C48" s="144" t="inlineStr"/>
-      <c r="D48" s="144" t="inlineStr">
+      <c r="B48" s="148" t="inlineStr"/>
+      <c r="C48" s="148" t="inlineStr"/>
+      <c r="D48" s="148" t="inlineStr">
         <is>
           <t>2026-10-30</t>
         </is>
       </c>
-      <c r="E48" s="144" t="inlineStr"/>
+      <c r="E48" s="148" t="inlineStr"/>
       <c r="F48" s="130" t="inlineStr">
         <is>
           <t>Homework 9 (Chapter 10) — Brightspace, due 11:59 pm</t>
@@ -6625,14 +8143,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B49" s="144" t="inlineStr"/>
-      <c r="C49" s="144" t="inlineStr"/>
-      <c r="D49" s="144" t="inlineStr">
+      <c r="B49" s="148" t="inlineStr"/>
+      <c r="C49" s="148" t="inlineStr"/>
+      <c r="D49" s="148" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E49" s="144" t="inlineStr"/>
+      <c r="E49" s="148" t="inlineStr"/>
       <c r="F49" s="130" t="inlineStr">
         <is>
           <t>Week 12: Nov.9/11 - No class Wednesday Nov.11 (Veterans Day)</t>
@@ -6645,14 +8163,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B50" s="144" t="inlineStr"/>
-      <c r="C50" s="144" t="inlineStr"/>
-      <c r="D50" s="144" t="inlineStr">
+      <c r="B50" s="148" t="inlineStr"/>
+      <c r="C50" s="148" t="inlineStr"/>
+      <c r="D50" s="148" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E50" s="144" t="inlineStr"/>
+      <c r="E50" s="148" t="inlineStr"/>
       <c r="F50" s="130" t="inlineStr">
         <is>
           <t>Week 12: Nov.9/11 - Read Chapter 11</t>
@@ -6665,14 +8183,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B51" s="144" t="inlineStr"/>
-      <c r="C51" s="144" t="inlineStr"/>
-      <c r="D51" s="144" t="inlineStr">
+      <c r="B51" s="148" t="inlineStr"/>
+      <c r="C51" s="148" t="inlineStr"/>
+      <c r="D51" s="148" t="inlineStr">
         <is>
           <t>2026-11-13</t>
         </is>
       </c>
-      <c r="E51" s="144" t="inlineStr"/>
+      <c r="E51" s="148" t="inlineStr"/>
       <c r="F51" s="130" t="inlineStr">
         <is>
           <t>Homework 10 (Chapter 11) — Brightspace, due 11:59 pm</t>
@@ -6685,14 +8203,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B52" s="144" t="inlineStr"/>
-      <c r="C52" s="144" t="inlineStr"/>
-      <c r="D52" s="144" t="inlineStr">
+      <c r="B52" s="148" t="inlineStr"/>
+      <c r="C52" s="148" t="inlineStr"/>
+      <c r="D52" s="148" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E52" s="144" t="inlineStr"/>
+      <c r="E52" s="148" t="inlineStr"/>
       <c r="F52" s="130" t="inlineStr">
         <is>
           <t>Week 13: Nov.16/18 - Read Chapter 12</t>
@@ -6705,14 +8223,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B53" s="144" t="inlineStr"/>
-      <c r="C53" s="144" t="inlineStr"/>
-      <c r="D53" s="144" t="inlineStr">
+      <c r="B53" s="148" t="inlineStr"/>
+      <c r="C53" s="148" t="inlineStr"/>
+      <c r="D53" s="148" t="inlineStr">
         <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="E53" s="144" t="inlineStr"/>
+      <c r="E53" s="148" t="inlineStr"/>
       <c r="F53" s="130" t="inlineStr">
         <is>
           <t>Homework 11 (Chapter 12) — Brightspace, due 11:59 pm</t>
@@ -6725,14 +8243,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B54" s="144" t="inlineStr"/>
-      <c r="C54" s="144" t="inlineStr"/>
-      <c r="D54" s="144" t="inlineStr">
+      <c r="B54" s="148" t="inlineStr"/>
+      <c r="C54" s="148" t="inlineStr"/>
+      <c r="D54" s="148" t="inlineStr">
         <is>
           <t>2026-11-27</t>
         </is>
       </c>
-      <c r="E54" s="144" t="inlineStr"/>
+      <c r="E54" s="148" t="inlineStr"/>
       <c r="F54" s="130" t="inlineStr">
         <is>
           <t>Week 14: Nov.23 - Complete the Chapter 12+13 home- work on Brightspace (due Nov.27)</t>
@@ -6745,14 +8263,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B55" s="144" t="inlineStr"/>
-      <c r="C55" s="144" t="inlineStr"/>
-      <c r="D55" s="144" t="inlineStr">
+      <c r="B55" s="148" t="inlineStr"/>
+      <c r="C55" s="148" t="inlineStr"/>
+      <c r="D55" s="148" t="inlineStr">
         <is>
           <t>2026-11-27</t>
         </is>
       </c>
-      <c r="E55" s="144" t="inlineStr"/>
+      <c r="E55" s="148" t="inlineStr"/>
       <c r="F55" s="130" t="inlineStr">
         <is>
           <t>Week 14: Nov.23 - No class Wednesday Nov.25 (Thanks- giving)</t>
@@ -6765,14 +8283,14 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B56" s="144" t="inlineStr"/>
-      <c r="C56" s="144" t="inlineStr"/>
-      <c r="D56" s="144" t="inlineStr">
+      <c r="B56" s="148" t="inlineStr"/>
+      <c r="C56" s="148" t="inlineStr"/>
+      <c r="D56" s="148" t="inlineStr">
         <is>
           <t>2026-11-27</t>
         </is>
       </c>
-      <c r="E56" s="144" t="inlineStr"/>
+      <c r="E56" s="148" t="inlineStr"/>
       <c r="F56" s="130" t="inlineStr">
         <is>
           <t>Week 14: Nov.23 - Read Chapter 13</t>
@@ -6785,14 +8303,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B57" s="144" t="inlineStr"/>
-      <c r="C57" s="144" t="inlineStr"/>
-      <c r="D57" s="144" t="inlineStr">
+      <c r="B57" s="148" t="inlineStr"/>
+      <c r="C57" s="148" t="inlineStr"/>
+      <c r="D57" s="148" t="inlineStr">
         <is>
           <t>2026-11-27</t>
         </is>
       </c>
-      <c r="E57" s="144" t="inlineStr"/>
+      <c r="E57" s="148" t="inlineStr"/>
       <c r="F57" s="130" t="inlineStr">
         <is>
           <t>Homework 12 (Chapter 13) — Brightspace, due 11:59 pm</t>
@@ -6805,14 +8323,14 @@
           <t>Extra Credit</t>
         </is>
       </c>
-      <c r="B58" s="142" t="inlineStr">
+      <c r="B58" s="146" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C58" s="143" t="inlineStr"/>
-      <c r="D58" s="143" t="inlineStr"/>
-      <c r="E58" s="143" t="inlineStr">
+      <c r="C58" s="147" t="inlineStr"/>
+      <c r="D58" s="147" t="inlineStr"/>
+      <c r="E58" s="147" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Organize BUAD-304 Participation 15% with sub-components
Add Active Class Participation, Team Engagement, and Research Studies
sub-rows in Excel; dedicated gather_marshall_participation_content() for
clean PDF sections (attendance, quality criteria, SONA 3-step process).
Remove grep noise, schedule snippets, and duplicate verbatim dump.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -8,10 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-304" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-281" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ECON-351" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-281" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ECON-351" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-304" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -430,7 +430,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="150">
+  <cellXfs count="158">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -843,6 +843,30 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4190,1106 +4214,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001F77B4"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F51"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="66" t="inlineStr">
-        <is>
-          <t>BUAD-304 — Organizational Behavior and Leadership</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="28">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/sources/buad-304-source.pdf","SEE HERE")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="29" t="inlineStr">
-        <is>
-          <t>Instructor</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Christine El Haddad</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="29" t="inlineStr">
-        <is>
-          <t>Term</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Fall 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="29" t="inlineStr">
-        <is>
-          <t>Required for an A</t>
-        </is>
-      </c>
-      <c r="B5" s="30" t="inlineStr">
-        <is>
-          <t>Curved (class rank)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="29" t="inlineStr">
-        <is>
-          <t>Grading scale</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Weighted score (% of points earned) + class average + student ranking (relative grading - no fixed A threshold in syllabus)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="67" t="inlineStr">
-        <is>
-          <t>Final Exam 25%  |  Participation 15%  |  Midterm Exam 15%  |  Team Project Paper 15%  |  Final Reflection Paper 10%  |  Presentation 10%  |  Case Analysis Assignments 5%  |  Proposal &amp; Team Contract 3%  |  Self &amp; Peer Evaluation 2%</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="29" t="inlineStr">
-        <is>
-          <t>Connect prep</t>
-        </is>
-      </c>
-      <c r="B8" s="68" t="inlineStr">
-        <is>
-          <t>Ungraded - Connect self-assessments are class prep, not part of Participation or other grades.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="69" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B10" s="69" t="inlineStr">
-        <is>
-          <t>Weight</t>
-        </is>
-      </c>
-      <c r="C10" s="69" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="D10" s="69" t="inlineStr">
-        <is>
-          <t>Due Date</t>
-        </is>
-      </c>
-      <c r="E10" s="69" t="inlineStr">
-        <is>
-          <t>Group Project</t>
-        </is>
-      </c>
-      <c r="F10" s="69" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="70" t="inlineStr">
-        <is>
-          <t>Final Exam</t>
-        </is>
-      </c>
-      <c r="B11" s="71" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="C11" s="72" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D11" s="72" t="inlineStr">
-        <is>
-          <t>2026-12-09</t>
-        </is>
-      </c>
-      <c r="E11" s="72" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F11" s="73">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-final-exam.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="74" t="inlineStr">
-        <is>
-          <t>Exam</t>
-        </is>
-      </c>
-      <c r="B12" s="75" t="inlineStr"/>
-      <c r="C12" s="75" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D12" s="75" t="inlineStr">
-        <is>
-          <t>2026-12-09</t>
-        </is>
-      </c>
-      <c r="E12" s="75" t="inlineStr"/>
-      <c r="F12" s="76" t="inlineStr">
-        <is>
-          <t>Final Exam</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="77" t="inlineStr">
-        <is>
-          <t>Participation</t>
-        </is>
-      </c>
-      <c r="B13" s="71" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="C13" s="78" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D13" s="78" t="inlineStr">
-        <is>
-          <t>2026-12-04</t>
-        </is>
-      </c>
-      <c r="E13" s="78" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F13" s="79">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-participation.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="80" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B14" s="75" t="inlineStr"/>
-      <c r="C14" s="75" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D14" s="75" t="inlineStr"/>
-      <c r="E14" s="75" t="inlineStr"/>
-      <c r="F14" s="76" t="inlineStr">
-        <is>
-          <t>Research: SONA registration opens</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="80" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B15" s="75" t="inlineStr"/>
-      <c r="C15" s="75" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="D15" s="75" t="inlineStr"/>
-      <c r="E15" s="75" t="inlineStr"/>
-      <c r="F15" s="76" t="inlineStr">
-        <is>
-          <t>Research: Prescreening questionnaire opens</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="80" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B16" s="75" t="inlineStr"/>
-      <c r="C16" s="75" t="inlineStr"/>
-      <c r="D16" s="75" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="E16" s="75" t="inlineStr"/>
-      <c r="F16" s="76" t="inlineStr">
-        <is>
-          <t>Research: Setup deadline (registration, prescreening, contacts)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="80" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B17" s="75" t="inlineStr"/>
-      <c r="C17" s="75" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="D17" s="75" t="inlineStr"/>
-      <c r="E17" s="75" t="inlineStr"/>
-      <c r="F17" s="76" t="inlineStr">
-        <is>
-          <t>Research: Study invitations begin (after setup)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="80" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B18" s="75" t="inlineStr"/>
-      <c r="C18" s="75" t="inlineStr"/>
-      <c r="D18" s="75" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="E18" s="75" t="inlineStr"/>
-      <c r="F18" s="76" t="inlineStr">
-        <is>
-          <t>Research: Employee contact surveys sent</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="80" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B19" s="75" t="inlineStr"/>
-      <c r="C19" s="75" t="inlineStr"/>
-      <c r="D19" s="75" t="inlineStr">
-        <is>
-          <t>2026-12-04</t>
-        </is>
-      </c>
-      <c r="E19" s="75" t="inlineStr"/>
-      <c r="F19" s="76" t="inlineStr">
-        <is>
-          <t>Research: Complete 2.0 research credits</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="70" t="inlineStr">
-        <is>
-          <t>Midterm Exam</t>
-        </is>
-      </c>
-      <c r="B20" s="71" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="C20" s="72" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D20" s="72" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E20" s="72" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F20" s="73">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-midterm-exam.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="74" t="inlineStr">
-        <is>
-          <t>Exam</t>
-        </is>
-      </c>
-      <c r="B21" s="75" t="inlineStr"/>
-      <c r="C21" s="75" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D21" s="75" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E21" s="75" t="inlineStr"/>
-      <c r="F21" s="76" t="inlineStr">
-        <is>
-          <t>Midterm Exam</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="77" t="inlineStr">
-        <is>
-          <t>Team Project Paper</t>
-        </is>
-      </c>
-      <c r="B22" s="71" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="C22" s="78" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D22" s="78" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="E22" s="78" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F22" s="79">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-team-project-paper.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="81" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B23" s="75" t="inlineStr"/>
-      <c r="C23" s="75" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D23" s="75" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E23" s="75" t="inlineStr"/>
-      <c r="F23" s="76" t="inlineStr">
-        <is>
-          <t>Team project outline</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="81" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B24" s="75" t="inlineStr"/>
-      <c r="C24" s="75" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D24" s="75" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="E24" s="75" t="inlineStr"/>
-      <c r="F24" s="76" t="inlineStr">
-        <is>
-          <t>Team project paper</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="70" t="inlineStr">
-        <is>
-          <t>Final Reflection Paper</t>
-        </is>
-      </c>
-      <c r="B25" s="71" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="C25" s="72" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D25" s="72" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E25" s="72" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F25" s="73">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-final-reflection-paper.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="81" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B26" s="75" t="inlineStr"/>
-      <c r="C26" s="75" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D26" s="75" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E26" s="75" t="inlineStr"/>
-      <c r="F26" s="76" t="inlineStr">
-        <is>
-          <t>Personal Reflection Paper</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="77" t="inlineStr">
-        <is>
-          <t>Presentation</t>
-        </is>
-      </c>
-      <c r="B27" s="71" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="C27" s="78" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D27" s="78" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="E27" s="78" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F27" s="79">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-presentation.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="81" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B28" s="75" t="inlineStr"/>
-      <c r="C28" s="75" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D28" s="75" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="E28" s="75" t="inlineStr"/>
-      <c r="F28" s="76" t="inlineStr">
-        <is>
-          <t>Presentation slides</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="70" t="inlineStr">
-        <is>
-          <t>Case Analysis Assignments</t>
-        </is>
-      </c>
-      <c r="B29" s="71" t="inlineStr">
-        <is>
-          <t>5%</t>
-        </is>
-      </c>
-      <c r="C29" s="72" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="D29" s="72" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="E29" s="72" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F29" s="73">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-case-analysis-assignments.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="81" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B30" s="75" t="inlineStr"/>
-      <c r="C30" s="75" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="D30" s="75" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="E30" s="75" t="inlineStr"/>
-      <c r="F30" s="76" t="inlineStr">
-        <is>
-          <t>Thomas Green Case Analysis Memo</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="81" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B31" s="75" t="inlineStr"/>
-      <c r="C31" s="75" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="D31" s="75" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="E31" s="75" t="inlineStr"/>
-      <c r="F31" s="76" t="inlineStr">
-        <is>
-          <t>SkillsForTomorrow Analysis Memo</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="77" t="inlineStr">
-        <is>
-          <t>Proposal &amp; Team Contract</t>
-        </is>
-      </c>
-      <c r="B32" s="71" t="inlineStr">
-        <is>
-          <t>3%</t>
-        </is>
-      </c>
-      <c r="C32" s="78" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D32" s="78" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E32" s="78" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F32" s="79">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-proposal-team-contract.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="81" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B33" s="75" t="inlineStr"/>
-      <c r="C33" s="75" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D33" s="75" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E33" s="75" t="inlineStr"/>
-      <c r="F33" s="76" t="inlineStr">
-        <is>
-          <t>Team project proposal &amp; team contract</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="70" t="inlineStr">
-        <is>
-          <t>Self &amp; Peer Evaluation</t>
-        </is>
-      </c>
-      <c r="B34" s="71" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="C34" s="72" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D34" s="72" t="inlineStr">
-        <is>
-          <t>2026-11-18</t>
-        </is>
-      </c>
-      <c r="E34" s="72" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F34" s="73">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-self-peer-evaluation.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="81" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B35" s="75" t="inlineStr"/>
-      <c r="C35" s="75" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D35" s="75" t="inlineStr">
-        <is>
-          <t>2026-11-18</t>
-        </is>
-      </c>
-      <c r="E35" s="75" t="inlineStr"/>
-      <c r="F35" s="76" t="inlineStr">
-        <is>
-          <t>Self &amp; peer evaluation</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="77" t="inlineStr">
-        <is>
-          <t>Personal Assessments (Connect)</t>
-        </is>
-      </c>
-      <c r="B36" s="71" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C36" s="78" t="inlineStr"/>
-      <c r="D36" s="78" t="inlineStr">
-        <is>
-          <t>2026-12-20</t>
-        </is>
-      </c>
-      <c r="E36" s="78" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F36" s="79">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-personal-assessments-connect.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B37" s="75" t="inlineStr"/>
-      <c r="C37" s="75" t="inlineStr"/>
-      <c r="D37" s="75" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="E37" s="75" t="inlineStr"/>
-      <c r="F37" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B38" s="75" t="inlineStr"/>
-      <c r="C38" s="75" t="inlineStr"/>
-      <c r="D38" s="75" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="E38" s="75" t="inlineStr"/>
-      <c r="F38" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B39" s="75" t="inlineStr"/>
-      <c r="C39" s="75" t="inlineStr"/>
-      <c r="D39" s="75" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="E39" s="75" t="inlineStr"/>
-      <c r="F39" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 5.01 - Assessing Your</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B40" s="75" t="inlineStr"/>
-      <c r="C40" s="75" t="inlineStr"/>
-      <c r="D40" s="75" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="E40" s="75" t="inlineStr"/>
-      <c r="F40" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Sharpen Companion</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B41" s="75" t="inlineStr"/>
-      <c r="C41" s="75" t="inlineStr"/>
-      <c r="D41" s="75" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="E41" s="75" t="inlineStr"/>
-      <c r="F41" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 11.01 - What is my</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B42" s="75" t="inlineStr"/>
-      <c r="C42" s="75" t="inlineStr"/>
-      <c r="D42" s="75" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="E42" s="75" t="inlineStr"/>
-      <c r="F42" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 11.02 - What is my</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B43" s="75" t="inlineStr"/>
-      <c r="C43" s="75" t="inlineStr"/>
-      <c r="D43" s="75" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="E43" s="75" t="inlineStr"/>
-      <c r="F43" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 12.01 - What kind of</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B44" s="75" t="inlineStr"/>
-      <c r="C44" s="75" t="inlineStr"/>
-      <c r="D44" s="75" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E44" s="75" t="inlineStr"/>
-      <c r="F44" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 10.5 - Preferred Conflict</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B45" s="75" t="inlineStr"/>
-      <c r="C45" s="75" t="inlineStr"/>
-      <c r="D45" s="75" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E45" s="75" t="inlineStr"/>
-      <c r="F45" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 9.01 - Assessing My</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B46" s="75" t="inlineStr"/>
-      <c r="C46" s="75" t="inlineStr"/>
-      <c r="D46" s="75" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E46" s="75" t="inlineStr"/>
-      <c r="F46" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 8.01 - Group</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B47" s="75" t="inlineStr"/>
-      <c r="C47" s="75" t="inlineStr"/>
-      <c r="D47" s="75" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="E47" s="75" t="inlineStr"/>
-      <c r="F47" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 14.02 - What Type of Organizational Culture Do I</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B48" s="75" t="inlineStr"/>
-      <c r="C48" s="75" t="inlineStr"/>
-      <c r="D48" s="75" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
-      </c>
-      <c r="E48" s="75" t="inlineStr"/>
-      <c r="F48" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 16.02 - What Is Your</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B49" s="75" t="inlineStr"/>
-      <c r="C49" s="75" t="inlineStr"/>
-      <c r="D49" s="75" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
-      </c>
-      <c r="E49" s="75" t="inlineStr"/>
-      <c r="F49" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 16.03 - Assessing Your</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B50" s="75" t="inlineStr"/>
-      <c r="C50" s="75" t="inlineStr"/>
-      <c r="D50" s="75" t="inlineStr">
-        <is>
-          <t>2026-12-20</t>
-        </is>
-      </c>
-      <c r="E50" s="75" t="inlineStr"/>
-      <c r="F50" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 12.02 - Which influence</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="29" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B51" s="83" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="A7:F7"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
     <tabColor rgb="00FF7F0E"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -6239,7 +5163,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00D62728"/>
@@ -7201,7 +6125,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="009467BD"/>
@@ -8361,4 +7285,1176 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001F77B4"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="66" t="inlineStr">
+        <is>
+          <t>BUAD-304 — Organizational Behavior and Leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="28">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/sources/buad-304-source.pdf","SEE HERE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="29" t="inlineStr">
+        <is>
+          <t>Instructor</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Christine El Haddad</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fall 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>Required for an A</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>Curved (class rank)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>Grading scale</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Weighted score (% of points earned) + class average + student ranking (relative grading - no fixed A threshold in syllabus)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="67" t="inlineStr">
+        <is>
+          <t>Final Exam 25%  |  Participation 15%  |  Midterm Exam 15%  |  Team Project Paper 15%  |  Final Reflection Paper 10%  |  Presentation 10%  |  Case Analysis Assignments 5%  |  Proposal &amp; Team Contract 3%  |  Self &amp; Peer Evaluation 2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>Connect prep</t>
+        </is>
+      </c>
+      <c r="B8" s="68" t="inlineStr">
+        <is>
+          <t>Ungraded - Connect self-assessments are class prep, not part of Participation or other grades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="69" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B10" s="69" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="C10" s="69" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="D10" s="69" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="E10" s="69" t="inlineStr">
+        <is>
+          <t>Group Project</t>
+        </is>
+      </c>
+      <c r="F10" s="69" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="70" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+      <c r="B11" s="154" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="C11" s="155" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D11" s="155" t="inlineStr">
+        <is>
+          <t>2026-12-09</t>
+        </is>
+      </c>
+      <c r="E11" s="155" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" s="73">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-final-exam.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="74" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="B12" s="156" t="inlineStr"/>
+      <c r="C12" s="156" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D12" s="156" t="inlineStr">
+        <is>
+          <t>2026-12-09</t>
+        </is>
+      </c>
+      <c r="E12" s="156" t="inlineStr"/>
+      <c r="F12" s="76" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="77" t="inlineStr">
+        <is>
+          <t>Participation</t>
+        </is>
+      </c>
+      <c r="B13" s="154" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="C13" s="157" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D13" s="157" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E13" s="157" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" s="79">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-participation.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="80" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B14" s="156" t="inlineStr"/>
+      <c r="C14" s="156" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D14" s="156" t="inlineStr"/>
+      <c r="E14" s="156" t="inlineStr"/>
+      <c r="F14" s="76" t="inlineStr">
+        <is>
+          <t>Research: SONA registration opens</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="80" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B15" s="156" t="inlineStr"/>
+      <c r="C15" s="156" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="D15" s="156" t="inlineStr"/>
+      <c r="E15" s="156" t="inlineStr"/>
+      <c r="F15" s="76" t="inlineStr">
+        <is>
+          <t>Research: Prescreening questionnaire opens</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="80" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B16" s="156" t="inlineStr"/>
+      <c r="C16" s="156" t="inlineStr"/>
+      <c r="D16" s="156" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E16" s="156" t="inlineStr"/>
+      <c r="F16" s="76" t="inlineStr">
+        <is>
+          <t>Research: Setup deadline (registration, prescreening, contacts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="80" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B17" s="156" t="inlineStr"/>
+      <c r="C17" s="156" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="D17" s="156" t="inlineStr"/>
+      <c r="E17" s="156" t="inlineStr"/>
+      <c r="F17" s="76" t="inlineStr">
+        <is>
+          <t>Research: Study invitations begin (after setup)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="80" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B18" s="156" t="inlineStr"/>
+      <c r="C18" s="156" t="inlineStr"/>
+      <c r="D18" s="156" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="E18" s="156" t="inlineStr"/>
+      <c r="F18" s="76" t="inlineStr">
+        <is>
+          <t>Research: Employee contact surveys sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B19" s="156" t="inlineStr"/>
+      <c r="C19" s="156" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D19" s="156" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E19" s="156" t="inlineStr"/>
+      <c r="F19" s="76" t="inlineStr">
+        <is>
+          <t>Active Class Participation — attend MW sessions prepared; contribute to discussions and in-class activities (2 free abse</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B20" s="156" t="inlineStr"/>
+      <c r="C20" s="156" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="D20" s="156" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E20" s="156" t="inlineStr"/>
+      <c r="F20" s="76" t="inlineStr">
+        <is>
+          <t>Team Engagement — effective engagement with project team throughout semester</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="80" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B21" s="156" t="inlineStr"/>
+      <c r="C21" s="156" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D21" s="156" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E21" s="156" t="inlineStr"/>
+      <c r="F21" s="76" t="inlineStr">
+        <is>
+          <t>Research Studies — complete 2.0 credits via SONA (register, setup, lab studies)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="80" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B22" s="156" t="inlineStr"/>
+      <c r="C22" s="156" t="inlineStr"/>
+      <c r="D22" s="156" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E22" s="156" t="inlineStr"/>
+      <c r="F22" s="76" t="inlineStr">
+        <is>
+          <t>Research: Complete 2.0 research credits</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="70" t="inlineStr">
+        <is>
+          <t>Midterm Exam</t>
+        </is>
+      </c>
+      <c r="B23" s="154" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="C23" s="155" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D23" s="155" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E23" s="155" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F23" s="73">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-midterm-exam.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="74" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="B24" s="156" t="inlineStr"/>
+      <c r="C24" s="156" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D24" s="156" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E24" s="156" t="inlineStr"/>
+      <c r="F24" s="76" t="inlineStr">
+        <is>
+          <t>Midterm Exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="77" t="inlineStr">
+        <is>
+          <t>Team Project Paper</t>
+        </is>
+      </c>
+      <c r="B25" s="154" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="C25" s="157" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D25" s="157" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E25" s="157" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F25" s="79">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-team-project-paper.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B26" s="156" t="inlineStr"/>
+      <c r="C26" s="156" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D26" s="156" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E26" s="156" t="inlineStr"/>
+      <c r="F26" s="76" t="inlineStr">
+        <is>
+          <t>Team project outline</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B27" s="156" t="inlineStr"/>
+      <c r="C27" s="156" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D27" s="156" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E27" s="156" t="inlineStr"/>
+      <c r="F27" s="76" t="inlineStr">
+        <is>
+          <t>Team project paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="70" t="inlineStr">
+        <is>
+          <t>Final Reflection Paper</t>
+        </is>
+      </c>
+      <c r="B28" s="154" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C28" s="155" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D28" s="155" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E28" s="155" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F28" s="73">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-final-reflection-paper.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B29" s="156" t="inlineStr"/>
+      <c r="C29" s="156" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D29" s="156" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E29" s="156" t="inlineStr"/>
+      <c r="F29" s="76" t="inlineStr">
+        <is>
+          <t>Personal Reflection Paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="77" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="B30" s="154" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C30" s="157" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D30" s="157" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E30" s="157" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F30" s="79">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-presentation.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B31" s="156" t="inlineStr"/>
+      <c r="C31" s="156" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D31" s="156" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E31" s="156" t="inlineStr"/>
+      <c r="F31" s="76" t="inlineStr">
+        <is>
+          <t>Presentation slides</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="70" t="inlineStr">
+        <is>
+          <t>Case Analysis Assignments</t>
+        </is>
+      </c>
+      <c r="B32" s="154" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="C32" s="155" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D32" s="155" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E32" s="155" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F32" s="73">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-case-analysis-assignments.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B33" s="156" t="inlineStr"/>
+      <c r="C33" s="156" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D33" s="156" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E33" s="156" t="inlineStr"/>
+      <c r="F33" s="76" t="inlineStr">
+        <is>
+          <t>Thomas Green Case Analysis Memo</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B34" s="156" t="inlineStr"/>
+      <c r="C34" s="156" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D34" s="156" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E34" s="156" t="inlineStr"/>
+      <c r="F34" s="76" t="inlineStr">
+        <is>
+          <t>SkillsForTomorrow Analysis Memo</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="77" t="inlineStr">
+        <is>
+          <t>Proposal &amp; Team Contract</t>
+        </is>
+      </c>
+      <c r="B35" s="154" t="inlineStr">
+        <is>
+          <t>3%</t>
+        </is>
+      </c>
+      <c r="C35" s="157" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D35" s="157" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E35" s="157" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F35" s="79">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-proposal-team-contract.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B36" s="156" t="inlineStr"/>
+      <c r="C36" s="156" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D36" s="156" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E36" s="156" t="inlineStr"/>
+      <c r="F36" s="76" t="inlineStr">
+        <is>
+          <t>Team project proposal &amp; team contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="70" t="inlineStr">
+        <is>
+          <t>Self &amp; Peer Evaluation</t>
+        </is>
+      </c>
+      <c r="B37" s="154" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="C37" s="155" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D37" s="155" t="inlineStr">
+        <is>
+          <t>2026-11-18</t>
+        </is>
+      </c>
+      <c r="E37" s="155" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F37" s="73">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-self-peer-evaluation.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B38" s="156" t="inlineStr"/>
+      <c r="C38" s="156" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D38" s="156" t="inlineStr">
+        <is>
+          <t>2026-11-18</t>
+        </is>
+      </c>
+      <c r="E38" s="156" t="inlineStr"/>
+      <c r="F38" s="76" t="inlineStr">
+        <is>
+          <t>Self &amp; peer evaluation</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="77" t="inlineStr">
+        <is>
+          <t>Personal Assessments (Connect)</t>
+        </is>
+      </c>
+      <c r="B39" s="154" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C39" s="157" t="inlineStr"/>
+      <c r="D39" s="157" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E39" s="157" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F39" s="79">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/buad-304-personal-assessments-connect.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B40" s="156" t="inlineStr"/>
+      <c r="C40" s="156" t="inlineStr"/>
+      <c r="D40" s="156" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E40" s="156" t="inlineStr"/>
+      <c r="F40" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B41" s="156" t="inlineStr"/>
+      <c r="C41" s="156" t="inlineStr"/>
+      <c r="D41" s="156" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E41" s="156" t="inlineStr"/>
+      <c r="F41" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B42" s="156" t="inlineStr"/>
+      <c r="C42" s="156" t="inlineStr"/>
+      <c r="D42" s="156" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E42" s="156" t="inlineStr"/>
+      <c r="F42" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 5.01 - Assessing Your</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B43" s="156" t="inlineStr"/>
+      <c r="C43" s="156" t="inlineStr"/>
+      <c r="D43" s="156" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="E43" s="156" t="inlineStr"/>
+      <c r="F43" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Sharpen Companion</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B44" s="156" t="inlineStr"/>
+      <c r="C44" s="156" t="inlineStr"/>
+      <c r="D44" s="156" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="E44" s="156" t="inlineStr"/>
+      <c r="F44" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 11.01 - What is my</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B45" s="156" t="inlineStr"/>
+      <c r="C45" s="156" t="inlineStr"/>
+      <c r="D45" s="156" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="E45" s="156" t="inlineStr"/>
+      <c r="F45" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 11.02 - What is my</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B46" s="156" t="inlineStr"/>
+      <c r="C46" s="156" t="inlineStr"/>
+      <c r="D46" s="156" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E46" s="156" t="inlineStr"/>
+      <c r="F46" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 12.01 - What kind of</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B47" s="156" t="inlineStr"/>
+      <c r="C47" s="156" t="inlineStr"/>
+      <c r="D47" s="156" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E47" s="156" t="inlineStr"/>
+      <c r="F47" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 10.5 - Preferred Conflict</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B48" s="156" t="inlineStr"/>
+      <c r="C48" s="156" t="inlineStr"/>
+      <c r="D48" s="156" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E48" s="156" t="inlineStr"/>
+      <c r="F48" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 9.01 - Assessing My</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B49" s="156" t="inlineStr"/>
+      <c r="C49" s="156" t="inlineStr"/>
+      <c r="D49" s="156" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E49" s="156" t="inlineStr"/>
+      <c r="F49" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 8.01 - Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B50" s="156" t="inlineStr"/>
+      <c r="C50" s="156" t="inlineStr"/>
+      <c r="D50" s="156" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="E50" s="156" t="inlineStr"/>
+      <c r="F50" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 14.02 - What Type of Organizational Culture Do I</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B51" s="156" t="inlineStr"/>
+      <c r="C51" s="156" t="inlineStr"/>
+      <c r="D51" s="156" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="E51" s="156" t="inlineStr"/>
+      <c r="F51" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 16.02 - What Is Your</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B52" s="156" t="inlineStr"/>
+      <c r="C52" s="156" t="inlineStr"/>
+      <c r="D52" s="156" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="E52" s="156" t="inlineStr"/>
+      <c r="F52" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 16.03 - Assessing Your</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B53" s="156" t="inlineStr"/>
+      <c r="C53" s="156" t="inlineStr"/>
+      <c r="D53" s="156" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E53" s="156" t="inlineStr"/>
+      <c r="F53" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 12.02 - Which influence</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="29" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B54" s="83" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="A7:F7"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Document Participation 15% sub-weights: not specified in syllabus
Add Weight Breakdown section and Excel weight_note column. Research
guide credit scale (2.0=100% of research component) documented separately.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -430,7 +430,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="158">
+  <cellXfs count="162">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -843,6 +843,18 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -7423,22 +7435,22 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B11" s="154" t="inlineStr">
+      <c r="B11" s="158" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="C11" s="155" t="inlineStr">
+      <c r="C11" s="159" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D11" s="155" t="inlineStr">
+      <c r="D11" s="159" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E11" s="155" t="inlineStr">
+      <c r="E11" s="159" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -7454,18 +7466,18 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B12" s="156" t="inlineStr"/>
-      <c r="C12" s="156" t="inlineStr">
+      <c r="B12" s="160" t="inlineStr"/>
+      <c r="C12" s="160" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D12" s="156" t="inlineStr">
+      <c r="D12" s="160" t="inlineStr">
         <is>
           <t>2026-12-09</t>
         </is>
       </c>
-      <c r="E12" s="156" t="inlineStr"/>
+      <c r="E12" s="160" t="inlineStr"/>
       <c r="F12" s="76" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -7478,22 +7490,22 @@
           <t>Participation</t>
         </is>
       </c>
-      <c r="B13" s="154" t="inlineStr">
+      <c r="B13" s="158" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C13" s="157" t="inlineStr">
+      <c r="C13" s="161" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D13" s="157" t="inlineStr">
+      <c r="D13" s="161" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E13" s="157" t="inlineStr">
+      <c r="E13" s="161" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -7509,14 +7521,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B14" s="156" t="inlineStr"/>
-      <c r="C14" s="156" t="inlineStr">
+      <c r="B14" s="160" t="inlineStr"/>
+      <c r="C14" s="160" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D14" s="156" t="inlineStr"/>
-      <c r="E14" s="156" t="inlineStr"/>
+      <c r="D14" s="160" t="inlineStr"/>
+      <c r="E14" s="160" t="inlineStr"/>
       <c r="F14" s="76" t="inlineStr">
         <is>
           <t>Research: SONA registration opens</t>
@@ -7529,14 +7541,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B15" s="156" t="inlineStr"/>
-      <c r="C15" s="156" t="inlineStr">
+      <c r="B15" s="160" t="inlineStr"/>
+      <c r="C15" s="160" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="D15" s="156" t="inlineStr"/>
-      <c r="E15" s="156" t="inlineStr"/>
+      <c r="D15" s="160" t="inlineStr"/>
+      <c r="E15" s="160" t="inlineStr"/>
       <c r="F15" s="76" t="inlineStr">
         <is>
           <t>Research: Prescreening questionnaire opens</t>
@@ -7549,14 +7561,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B16" s="156" t="inlineStr"/>
-      <c r="C16" s="156" t="inlineStr"/>
-      <c r="D16" s="156" t="inlineStr">
+      <c r="B16" s="160" t="inlineStr"/>
+      <c r="C16" s="160" t="inlineStr"/>
+      <c r="D16" s="160" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="E16" s="156" t="inlineStr"/>
+      <c r="E16" s="160" t="inlineStr"/>
       <c r="F16" s="76" t="inlineStr">
         <is>
           <t>Research: Setup deadline (registration, prescreening, contacts)</t>
@@ -7569,14 +7581,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B17" s="156" t="inlineStr"/>
-      <c r="C17" s="156" t="inlineStr">
+      <c r="B17" s="160" t="inlineStr"/>
+      <c r="C17" s="160" t="inlineStr">
         <is>
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="D17" s="156" t="inlineStr"/>
-      <c r="E17" s="156" t="inlineStr"/>
+      <c r="D17" s="160" t="inlineStr"/>
+      <c r="E17" s="160" t="inlineStr"/>
       <c r="F17" s="76" t="inlineStr">
         <is>
           <t>Research: Study invitations begin (after setup)</t>
@@ -7589,14 +7601,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B18" s="156" t="inlineStr"/>
-      <c r="C18" s="156" t="inlineStr"/>
-      <c r="D18" s="156" t="inlineStr">
+      <c r="B18" s="160" t="inlineStr"/>
+      <c r="C18" s="160" t="inlineStr"/>
+      <c r="D18" s="160" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E18" s="156" t="inlineStr"/>
+      <c r="E18" s="160" t="inlineStr"/>
       <c r="F18" s="76" t="inlineStr">
         <is>
           <t>Research: Employee contact surveys sent</t>
@@ -7609,18 +7621,22 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B19" s="156" t="inlineStr"/>
-      <c r="C19" s="156" t="inlineStr">
+      <c r="B19" s="160" t="inlineStr">
+        <is>
+          <t>Not in syllabus (% of 15%)</t>
+        </is>
+      </c>
+      <c r="C19" s="160" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D19" s="156" t="inlineStr">
+      <c r="D19" s="160" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E19" s="156" t="inlineStr"/>
+      <c r="E19" s="160" t="inlineStr"/>
       <c r="F19" s="76" t="inlineStr">
         <is>
           <t>Active Class Participation — attend MW sessions prepared; contribute to discussions and in-class activities (2 free abse</t>
@@ -7633,18 +7649,22 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B20" s="156" t="inlineStr"/>
-      <c r="C20" s="156" t="inlineStr">
+      <c r="B20" s="160" t="inlineStr">
+        <is>
+          <t>Not in syllabus (% of 15%)</t>
+        </is>
+      </c>
+      <c r="C20" s="160" t="inlineStr">
         <is>
           <t>2026-09-07</t>
         </is>
       </c>
-      <c r="D20" s="156" t="inlineStr">
+      <c r="D20" s="160" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E20" s="156" t="inlineStr"/>
+      <c r="E20" s="160" t="inlineStr"/>
       <c r="F20" s="76" t="inlineStr">
         <is>
           <t>Team Engagement — effective engagement with project team throughout semester</t>
@@ -7657,18 +7677,22 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B21" s="156" t="inlineStr"/>
-      <c r="C21" s="156" t="inlineStr">
+      <c r="B21" s="160" t="inlineStr">
+        <is>
+          <t>Not in syllabus (% of 15%)</t>
+        </is>
+      </c>
+      <c r="C21" s="160" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D21" s="156" t="inlineStr">
+      <c r="D21" s="160" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E21" s="156" t="inlineStr"/>
+      <c r="E21" s="160" t="inlineStr"/>
       <c r="F21" s="76" t="inlineStr">
         <is>
           <t>Research Studies — complete 2.0 credits via SONA (register, setup, lab studies)</t>
@@ -7681,14 +7705,14 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="B22" s="156" t="inlineStr"/>
-      <c r="C22" s="156" t="inlineStr"/>
-      <c r="D22" s="156" t="inlineStr">
+      <c r="B22" s="160" t="inlineStr"/>
+      <c r="C22" s="160" t="inlineStr"/>
+      <c r="D22" s="160" t="inlineStr">
         <is>
           <t>2026-12-04</t>
         </is>
       </c>
-      <c r="E22" s="156" t="inlineStr"/>
+      <c r="E22" s="160" t="inlineStr"/>
       <c r="F22" s="76" t="inlineStr">
         <is>
           <t>Research: Complete 2.0 research credits</t>
@@ -7701,22 +7725,22 @@
           <t>Midterm Exam</t>
         </is>
       </c>
-      <c r="B23" s="154" t="inlineStr">
+      <c r="B23" s="158" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C23" s="155" t="inlineStr">
+      <c r="C23" s="159" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D23" s="155" t="inlineStr">
+      <c r="D23" s="159" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E23" s="155" t="inlineStr">
+      <c r="E23" s="159" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -7732,18 +7756,18 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B24" s="156" t="inlineStr"/>
-      <c r="C24" s="156" t="inlineStr">
+      <c r="B24" s="160" t="inlineStr"/>
+      <c r="C24" s="160" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="D24" s="156" t="inlineStr">
+      <c r="D24" s="160" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E24" s="156" t="inlineStr"/>
+      <c r="E24" s="160" t="inlineStr"/>
       <c r="F24" s="76" t="inlineStr">
         <is>
           <t>Midterm Exam</t>
@@ -7756,22 +7780,22 @@
           <t>Team Project Paper</t>
         </is>
       </c>
-      <c r="B25" s="154" t="inlineStr">
+      <c r="B25" s="158" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C25" s="157" t="inlineStr">
+      <c r="C25" s="161" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D25" s="157" t="inlineStr">
+      <c r="D25" s="161" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E25" s="157" t="inlineStr">
+      <c r="E25" s="161" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -7787,18 +7811,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B26" s="156" t="inlineStr"/>
-      <c r="C26" s="156" t="inlineStr">
+      <c r="B26" s="160" t="inlineStr"/>
+      <c r="C26" s="160" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D26" s="156" t="inlineStr">
+      <c r="D26" s="160" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E26" s="156" t="inlineStr"/>
+      <c r="E26" s="160" t="inlineStr"/>
       <c r="F26" s="76" t="inlineStr">
         <is>
           <t>Team project outline</t>
@@ -7811,18 +7835,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B27" s="156" t="inlineStr"/>
-      <c r="C27" s="156" t="inlineStr">
+      <c r="B27" s="160" t="inlineStr"/>
+      <c r="C27" s="160" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D27" s="156" t="inlineStr">
+      <c r="D27" s="160" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E27" s="156" t="inlineStr"/>
+      <c r="E27" s="160" t="inlineStr"/>
       <c r="F27" s="76" t="inlineStr">
         <is>
           <t>Team project paper</t>
@@ -7835,22 +7859,22 @@
           <t>Final Reflection Paper</t>
         </is>
       </c>
-      <c r="B28" s="154" t="inlineStr">
+      <c r="B28" s="158" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C28" s="155" t="inlineStr">
+      <c r="C28" s="159" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D28" s="155" t="inlineStr">
+      <c r="D28" s="159" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E28" s="155" t="inlineStr">
+      <c r="E28" s="159" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -7866,18 +7890,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B29" s="156" t="inlineStr"/>
-      <c r="C29" s="156" t="inlineStr">
+      <c r="B29" s="160" t="inlineStr"/>
+      <c r="C29" s="160" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D29" s="156" t="inlineStr">
+      <c r="D29" s="160" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E29" s="156" t="inlineStr"/>
+      <c r="E29" s="160" t="inlineStr"/>
       <c r="F29" s="76" t="inlineStr">
         <is>
           <t>Personal Reflection Paper</t>
@@ -7890,22 +7914,22 @@
           <t>Presentation</t>
         </is>
       </c>
-      <c r="B30" s="154" t="inlineStr">
+      <c r="B30" s="158" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C30" s="157" t="inlineStr">
+      <c r="C30" s="161" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D30" s="157" t="inlineStr">
+      <c r="D30" s="161" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E30" s="157" t="inlineStr">
+      <c r="E30" s="161" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -7921,18 +7945,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B31" s="156" t="inlineStr"/>
-      <c r="C31" s="156" t="inlineStr">
+      <c r="B31" s="160" t="inlineStr"/>
+      <c r="C31" s="160" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D31" s="156" t="inlineStr">
+      <c r="D31" s="160" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E31" s="156" t="inlineStr"/>
+      <c r="E31" s="160" t="inlineStr"/>
       <c r="F31" s="76" t="inlineStr">
         <is>
           <t>Presentation slides</t>
@@ -7945,22 +7969,22 @@
           <t>Case Analysis Assignments</t>
         </is>
       </c>
-      <c r="B32" s="154" t="inlineStr">
+      <c r="B32" s="158" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C32" s="155" t="inlineStr">
+      <c r="C32" s="159" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D32" s="155" t="inlineStr">
+      <c r="D32" s="159" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E32" s="155" t="inlineStr">
+      <c r="E32" s="159" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -7976,18 +8000,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B33" s="156" t="inlineStr"/>
-      <c r="C33" s="156" t="inlineStr">
+      <c r="B33" s="160" t="inlineStr"/>
+      <c r="C33" s="160" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D33" s="156" t="inlineStr">
+      <c r="D33" s="160" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E33" s="156" t="inlineStr"/>
+      <c r="E33" s="160" t="inlineStr"/>
       <c r="F33" s="76" t="inlineStr">
         <is>
           <t>Thomas Green Case Analysis Memo</t>
@@ -8000,18 +8024,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B34" s="156" t="inlineStr"/>
-      <c r="C34" s="156" t="inlineStr">
+      <c r="B34" s="160" t="inlineStr"/>
+      <c r="C34" s="160" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="D34" s="156" t="inlineStr">
+      <c r="D34" s="160" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E34" s="156" t="inlineStr"/>
+      <c r="E34" s="160" t="inlineStr"/>
       <c r="F34" s="76" t="inlineStr">
         <is>
           <t>SkillsForTomorrow Analysis Memo</t>
@@ -8024,22 +8048,22 @@
           <t>Proposal &amp; Team Contract</t>
         </is>
       </c>
-      <c r="B35" s="154" t="inlineStr">
+      <c r="B35" s="158" t="inlineStr">
         <is>
           <t>3%</t>
         </is>
       </c>
-      <c r="C35" s="157" t="inlineStr">
+      <c r="C35" s="161" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D35" s="157" t="inlineStr">
+      <c r="D35" s="161" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E35" s="157" t="inlineStr">
+      <c r="E35" s="161" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -8055,18 +8079,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B36" s="156" t="inlineStr"/>
-      <c r="C36" s="156" t="inlineStr">
+      <c r="B36" s="160" t="inlineStr"/>
+      <c r="C36" s="160" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D36" s="156" t="inlineStr">
+      <c r="D36" s="160" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E36" s="156" t="inlineStr"/>
+      <c r="E36" s="160" t="inlineStr"/>
       <c r="F36" s="76" t="inlineStr">
         <is>
           <t>Team project proposal &amp; team contract</t>
@@ -8079,22 +8103,22 @@
           <t>Self &amp; Peer Evaluation</t>
         </is>
       </c>
-      <c r="B37" s="154" t="inlineStr">
+      <c r="B37" s="158" t="inlineStr">
         <is>
           <t>2%</t>
         </is>
       </c>
-      <c r="C37" s="155" t="inlineStr">
+      <c r="C37" s="159" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D37" s="155" t="inlineStr">
+      <c r="D37" s="159" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E37" s="155" t="inlineStr">
+      <c r="E37" s="159" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -8110,18 +8134,18 @@
           <t>Assignment</t>
         </is>
       </c>
-      <c r="B38" s="156" t="inlineStr"/>
-      <c r="C38" s="156" t="inlineStr">
+      <c r="B38" s="160" t="inlineStr"/>
+      <c r="C38" s="160" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="D38" s="156" t="inlineStr">
+      <c r="D38" s="160" t="inlineStr">
         <is>
           <t>2026-11-18</t>
         </is>
       </c>
-      <c r="E38" s="156" t="inlineStr"/>
+      <c r="E38" s="160" t="inlineStr"/>
       <c r="F38" s="76" t="inlineStr">
         <is>
           <t>Self &amp; peer evaluation</t>
@@ -8134,18 +8158,18 @@
           <t>Personal Assessments (Connect)</t>
         </is>
       </c>
-      <c r="B39" s="154" t="inlineStr">
+      <c r="B39" s="158" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C39" s="157" t="inlineStr"/>
-      <c r="D39" s="157" t="inlineStr">
+      <c r="C39" s="161" t="inlineStr"/>
+      <c r="D39" s="161" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E39" s="157" t="inlineStr">
+      <c r="E39" s="161" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -8161,14 +8185,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B40" s="156" t="inlineStr"/>
-      <c r="C40" s="156" t="inlineStr"/>
-      <c r="D40" s="156" t="inlineStr">
+      <c r="B40" s="160" t="inlineStr"/>
+      <c r="C40" s="160" t="inlineStr"/>
+      <c r="D40" s="160" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="E40" s="156" t="inlineStr"/>
+      <c r="E40" s="160" t="inlineStr"/>
       <c r="F40" s="76" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
@@ -8181,14 +8205,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B41" s="156" t="inlineStr"/>
-      <c r="C41" s="156" t="inlineStr"/>
-      <c r="D41" s="156" t="inlineStr">
+      <c r="B41" s="160" t="inlineStr"/>
+      <c r="C41" s="160" t="inlineStr"/>
+      <c r="D41" s="160" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="E41" s="156" t="inlineStr"/>
+      <c r="E41" s="160" t="inlineStr"/>
       <c r="F41" s="76" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
@@ -8201,14 +8225,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B42" s="156" t="inlineStr"/>
-      <c r="C42" s="156" t="inlineStr"/>
-      <c r="D42" s="156" t="inlineStr">
+      <c r="B42" s="160" t="inlineStr"/>
+      <c r="C42" s="160" t="inlineStr"/>
+      <c r="D42" s="160" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="E42" s="156" t="inlineStr"/>
+      <c r="E42" s="160" t="inlineStr"/>
       <c r="F42" s="76" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 5.01 - Assessing Your</t>
@@ -8221,14 +8245,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B43" s="156" t="inlineStr"/>
-      <c r="C43" s="156" t="inlineStr"/>
-      <c r="D43" s="156" t="inlineStr">
+      <c r="B43" s="160" t="inlineStr"/>
+      <c r="C43" s="160" t="inlineStr"/>
+      <c r="D43" s="160" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="E43" s="156" t="inlineStr"/>
+      <c r="E43" s="160" t="inlineStr"/>
       <c r="F43" s="76" t="inlineStr">
         <is>
           <t>Connect: Sharpen Companion</t>
@@ -8241,14 +8265,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B44" s="156" t="inlineStr"/>
-      <c r="C44" s="156" t="inlineStr"/>
-      <c r="D44" s="156" t="inlineStr">
+      <c r="B44" s="160" t="inlineStr"/>
+      <c r="C44" s="160" t="inlineStr"/>
+      <c r="D44" s="160" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="E44" s="156" t="inlineStr"/>
+      <c r="E44" s="160" t="inlineStr"/>
       <c r="F44" s="76" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 11.01 - What is my</t>
@@ -8261,14 +8285,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B45" s="156" t="inlineStr"/>
-      <c r="C45" s="156" t="inlineStr"/>
-      <c r="D45" s="156" t="inlineStr">
+      <c r="B45" s="160" t="inlineStr"/>
+      <c r="C45" s="160" t="inlineStr"/>
+      <c r="D45" s="160" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="E45" s="156" t="inlineStr"/>
+      <c r="E45" s="160" t="inlineStr"/>
       <c r="F45" s="76" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 11.02 - What is my</t>
@@ -8281,14 +8305,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B46" s="156" t="inlineStr"/>
-      <c r="C46" s="156" t="inlineStr"/>
-      <c r="D46" s="156" t="inlineStr">
+      <c r="B46" s="160" t="inlineStr"/>
+      <c r="C46" s="160" t="inlineStr"/>
+      <c r="D46" s="160" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E46" s="156" t="inlineStr"/>
+      <c r="E46" s="160" t="inlineStr"/>
       <c r="F46" s="76" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 12.01 - What kind of</t>
@@ -8301,14 +8325,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B47" s="156" t="inlineStr"/>
-      <c r="C47" s="156" t="inlineStr"/>
-      <c r="D47" s="156" t="inlineStr">
+      <c r="B47" s="160" t="inlineStr"/>
+      <c r="C47" s="160" t="inlineStr"/>
+      <c r="D47" s="160" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E47" s="156" t="inlineStr"/>
+      <c r="E47" s="160" t="inlineStr"/>
       <c r="F47" s="76" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 10.5 - Preferred Conflict</t>
@@ -8321,14 +8345,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B48" s="156" t="inlineStr"/>
-      <c r="C48" s="156" t="inlineStr"/>
-      <c r="D48" s="156" t="inlineStr">
+      <c r="B48" s="160" t="inlineStr"/>
+      <c r="C48" s="160" t="inlineStr"/>
+      <c r="D48" s="160" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E48" s="156" t="inlineStr"/>
+      <c r="E48" s="160" t="inlineStr"/>
       <c r="F48" s="76" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 9.01 - Assessing My</t>
@@ -8341,14 +8365,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B49" s="156" t="inlineStr"/>
-      <c r="C49" s="156" t="inlineStr"/>
-      <c r="D49" s="156" t="inlineStr">
+      <c r="B49" s="160" t="inlineStr"/>
+      <c r="C49" s="160" t="inlineStr"/>
+      <c r="D49" s="160" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E49" s="156" t="inlineStr"/>
+      <c r="E49" s="160" t="inlineStr"/>
       <c r="F49" s="76" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 8.01 - Group</t>
@@ -8361,14 +8385,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B50" s="156" t="inlineStr"/>
-      <c r="C50" s="156" t="inlineStr"/>
-      <c r="D50" s="156" t="inlineStr">
+      <c r="B50" s="160" t="inlineStr"/>
+      <c r="C50" s="160" t="inlineStr"/>
+      <c r="D50" s="160" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="E50" s="156" t="inlineStr"/>
+      <c r="E50" s="160" t="inlineStr"/>
       <c r="F50" s="76" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 14.02 - What Type of Organizational Culture Do I</t>
@@ -8381,14 +8405,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B51" s="156" t="inlineStr"/>
-      <c r="C51" s="156" t="inlineStr"/>
-      <c r="D51" s="156" t="inlineStr">
+      <c r="B51" s="160" t="inlineStr"/>
+      <c r="C51" s="160" t="inlineStr"/>
+      <c r="D51" s="160" t="inlineStr">
         <is>
           <t>2026-11-30</t>
         </is>
       </c>
-      <c r="E51" s="156" t="inlineStr"/>
+      <c r="E51" s="160" t="inlineStr"/>
       <c r="F51" s="76" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 16.02 - What Is Your</t>
@@ -8401,14 +8425,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B52" s="156" t="inlineStr"/>
-      <c r="C52" s="156" t="inlineStr"/>
-      <c r="D52" s="156" t="inlineStr">
+      <c r="B52" s="160" t="inlineStr"/>
+      <c r="C52" s="160" t="inlineStr"/>
+      <c r="D52" s="160" t="inlineStr">
         <is>
           <t>2026-11-30</t>
         </is>
       </c>
-      <c r="E52" s="156" t="inlineStr"/>
+      <c r="E52" s="160" t="inlineStr"/>
       <c r="F52" s="76" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 16.03 - Assessing Your</t>
@@ -8421,14 +8445,14 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B53" s="156" t="inlineStr"/>
-      <c r="C53" s="156" t="inlineStr"/>
-      <c r="D53" s="156" t="inlineStr">
+      <c r="B53" s="160" t="inlineStr"/>
+      <c r="C53" s="160" t="inlineStr"/>
+      <c r="D53" s="160" t="inlineStr">
         <is>
           <t>2026-12-20</t>
         </is>
       </c>
-      <c r="E53" s="156" t="inlineStr"/>
+      <c r="E53" s="160" t="inlineStr"/>
       <c r="F53" s="76" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 12.02 - Which influence</t>

</xml_diff>

<commit_message>
Add JS-310 (Brylak) Eastern European Jewish Experience syllabus
Implement assessment-breakdown parser for Description and Assessment of
Assignments + grading table syllabi. Extracts weekly quiz readings (15 weeks),
midterm/final quizzes, and oral exam rubrics. Add RMP data for Andrzej Brylak
(professor 2745347, includes SLL/JS 310 reviews).

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ECON-351" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-304" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SPAN-290" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JS-310" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="35">
+  <fonts count="37">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -187,8 +188,18 @@
       <color rgb="002CA02C"/>
       <sz val="13"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="008C564B"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="008C564B"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="43">
+  <fills count="49">
     <fill>
       <patternFill/>
     </fill>
@@ -400,6 +411,36 @@
         <fgColor rgb="00F0F8F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008C564B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E5D9D7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDE5E4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DECFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FAF8F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F6F3F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -471,7 +512,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="194">
+  <cellXfs count="218">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1014,6 +1055,76 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="42" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="43" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="44" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="43" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="45" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="46" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="45" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="45" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="47" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="47" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="47" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="48" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="48" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="48" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="47" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="47" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="46" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="45" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="47" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="48" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="46" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="45" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="47" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="48" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1382,7 +1493,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K139"/>
+  <dimension ref="A1:K154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1609,60 +1720,96 @@
     </row>
     <row r="10" hidden="1" outlineLevel="1">
       <c r="A10" s="7">
+        <f>HYPERLINK("#'JS-310'!A1","JS-310")</f>
+        <v/>
+      </c>
+      <c r="B10" s="88" t="inlineStr">
+        <is>
+          <t>Andrzej Brylak / Yulia Dubasova (RMP: Andrzej Brylak)</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>A+ (4) [11/12 reported]</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" hidden="1" outlineLevel="1">
+      <c r="A11" s="10">
         <f>HYPERLINK("#'SPAN-290'!A1","SPAN-290")</f>
         <v/>
       </c>
-      <c r="B10" s="88" t="inlineStr">
+      <c r="B11" s="89" t="inlineStr">
         <is>
           <t>Samuel Steinberg</t>
         </is>
       </c>
-      <c r="C10" s="26" t="inlineStr">
+      <c r="C11" s="90" t="inlineStr">
         <is>
           <t>4.5</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E11" s="11" t="inlineStr">
         <is>
           <t>A- (3.74) [5/5 reported]</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F11" s="11" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="G11" s="11" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
     </row>
-    <row r="11" hidden="1" outlineLevel="1"/>
-    <row r="12" hidden="1" outlineLevel="1">
-      <c r="A12" s="13" t="inlineStr">
+    <row r="12" hidden="1" outlineLevel="1"/>
+    <row r="13" hidden="1" outlineLevel="1">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Consensus - recurring student review themes</t>
         </is>
       </c>
     </row>
-    <row r="13" hidden="1" outlineLevel="1" ht="135" customHeight="1">
-      <c r="A13" s="104" t="inlineStr">
+    <row r="14" hidden="1" outlineLevel="1" ht="135" customHeight="1">
+      <c r="A14" s="104" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="B13" s="105" t="inlineStr">
+      <c r="B14" s="105" t="inlineStr">
         <is>
           <t>George Braunegg</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>STRENGTHS: Very high marks for personality and support — students call Prof. Braunegg kind, funny, caring, and responsive by email. Daily accounting facts/jokes are a recurring positive. Many praise his career advice and willingness to help outside class; several credit him with influencing their major choice.
 TEACHING &amp; EXAMS: More divided on in-class instruction — some say he struggles to work through problems live or that lectures don't always align with exams. Course draws on Prof. Layton's materials but sections may not match perfectly. Textbook gets criticism.
@@ -1670,18 +1817,18 @@
         </is>
       </c>
     </row>
-    <row r="14" hidden="1" outlineLevel="1" ht="135" customHeight="1">
-      <c r="A14" s="106" t="inlineStr">
+    <row r="15" hidden="1" outlineLevel="1" ht="135" customHeight="1">
+      <c r="A15" s="106" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="B14" s="107" t="inlineStr">
+      <c r="B15" s="107" t="inlineStr">
         <is>
           <t>Christine El Haddad</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>STRENGTHS: Among the most praised Marshall professors on RMP — repeatedly called the 'best' or 'sweetest' instructor students have had. Negotiation and OB classes get standout reviews: supportive classroom culture, clear and organized Brightspace, strong lectures, and generous extra credit. Weekly in-class negotiations are a highlight for many.
 WORKLOAD: Group projects and class participation carry real weight; some find readings or lecture content repetitive. A few note group work can feel heavy even when the professor is beloved.
@@ -1689,18 +1836,18 @@
         </is>
       </c>
     </row>
-    <row r="15" hidden="1" outlineLevel="1" ht="165" customHeight="1">
-      <c r="A15" s="104" t="inlineStr">
+    <row r="16" hidden="1" outlineLevel="1" ht="165" customHeight="1">
+      <c r="A16" s="104" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="B15" s="105" t="inlineStr">
+      <c r="B16" s="105" t="inlineStr">
         <is>
           <t>Alejandro Martínez-Marquina / João Ramos (RMP: Alejandro Martínez-Marquina)</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>STRENGTHS: Reviewers repeatedly praise board work, step-by-step problem breakdowns, and practice sets that mirror exams. Many call him kind, funny, and responsive by email; office hours and TAs get strong mentions. Several note you can succeed without mandatory attendance if you self-study from the textbook.
 COMMON CAVEATS: Spanish accent and fast lecture pace come up often — sit near the front. Some say lectures/textbook do not fully prepare you unless you drill mock exams and homework. Content volume is high; procrastination hurts.
@@ -1709,18 +1856,18 @@
         </is>
       </c>
     </row>
-    <row r="16" hidden="1" outlineLevel="1" ht="135" customHeight="1">
-      <c r="A16" s="106" t="inlineStr">
+    <row r="17" hidden="1" outlineLevel="1" ht="135" customHeight="1">
+      <c r="A17" s="106" t="inlineStr">
         <is>
           <t>HIST-103</t>
         </is>
       </c>
-      <c r="B16" s="107" t="inlineStr">
+      <c r="B17" s="107" t="inlineStr">
         <is>
           <t>Lindsay O'Neill</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>STRENGTHS: Students consistently describe Dr. O'Neill as passionate and engaging — lectures use multimedia (Monty Python clips, movie trailers, humor) that make a GE history class feel lively rather than dry. Many say the content is genuinely interesting if you show up and pay attention.
 GRADING &amp; WORKLOAD: Mixed reviews on grading — several note she can be a harsh essay grader and that strong discussion participation matters. Expect substantial section readings; essays benefit from office-hours or TA help. Low-weight pop quizzes (~5% total) sometimes used to track attendance.
@@ -1728,128 +1875,99 @@
         </is>
       </c>
     </row>
-    <row r="17" hidden="1" outlineLevel="1" ht="120" customHeight="1">
-      <c r="A17" s="104" t="inlineStr">
+    <row r="18" hidden="1" outlineLevel="1" ht="165" customHeight="1">
+      <c r="A18" s="104" t="inlineStr">
+        <is>
+          <t>JS-310</t>
+        </is>
+      </c>
+      <c r="B18" s="105" t="inlineStr">
+        <is>
+          <t>Andrzej Brylak / Yulia Dubasova (RMP: Andrzej Brylak)</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>STRENGTHS: Very strong RMP profile (4.9 quality, 1.6 difficulty, 100% would take again). Students call Brylak passionate, hilarious, knowledgeable, and caring — one of the best GE picks at USC. Several reviews are explicitly for SLL/JS 310.\n\nWORKLOAD: Heavy reading (~75–100 pp/week per reviews). Weekly reading quizzes (10 questions) are described as easy if you attend lecture; midterm/final quizzes plus two oral presentations (quote analysis + thematic comparison across 3 readings). Physical book required in class; no laptops except for quizzes.\n\nCAVEATS: Oral exams graded on public-speaking standards with follow-up questions. Assignment instructions sometimes vague (older reviews mention papers; current syllabus uses oral exams). Strict attendance — 2 unexcused absences risks failure.\n\nBOTTOM LINE: Engaging instructor and manageable grading if you do the reading and show up; not a phone/laptop class.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" hidden="1" outlineLevel="1" ht="120" customHeight="1">
+      <c r="A19" s="106" t="inlineStr">
         <is>
           <t>SPAN-290</t>
         </is>
       </c>
-      <c r="B17" s="105" t="inlineStr">
+      <c r="B19" s="107" t="inlineStr">
         <is>
           <t>Samuel Steinberg</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>STRENGTHS: Small sample but uniformly positive — 4.5 quality, 2.2 difficulty, 100% would take again. Students describe Prof. Steinberg as passionate, knowledgeable, and fair; essays and reading notes reward engagement with the material.\n\nWORKLOAD: Reading-heavy with regular reading notes plus two essays and two in-class exams (500-point scale). Provisional schedule packs film screenings and primary sources; BrightSpace distributes readings.\n\nBOTTOM LINE: Strong pick for Latin American/Iberian cultural studies if you keep up with readings and take essays seriously. AI use is prohibited — all written work must be your own.</t>
         </is>
       </c>
     </row>
-    <row r="18" hidden="1" outlineLevel="1"/>
-    <row r="19" hidden="1" outlineLevel="1">
-      <c r="A19" s="13" t="inlineStr">
+    <row r="20" hidden="1" outlineLevel="1"/>
+    <row r="21" hidden="1" outlineLevel="1">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>Student reviews (Rate My Professors) - newest first</t>
         </is>
       </c>
     </row>
-    <row r="20" hidden="1" outlineLevel="1">
-      <c r="A20" s="6" t="inlineStr">
+    <row r="22" hidden="1" outlineLevel="1">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>Grade</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>Q/D</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>Review</t>
         </is>
       </c>
     </row>
-    <row r="21" hidden="1" outlineLevel="1" ht="30" customHeight="1">
-      <c r="A21" s="104" t="inlineStr">
+    <row r="23" hidden="1" outlineLevel="1" ht="30" customHeight="1">
+      <c r="A23" s="104" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="B21" s="105" t="inlineStr">
+      <c r="B23" s="105" t="inlineStr">
         <is>
           <t>2026-02-25</t>
         </is>
       </c>
-      <c r="C21" s="105" t="inlineStr">
+      <c r="C23" s="105" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D21" s="105" t="inlineStr">
+      <c r="D23" s="105" t="inlineStr">
         <is>
           <t>5/1</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>The tests are easy if you just do the practice sets. He's great at explanations. [Amazing lectures, So many papers, Graded by few things]</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" hidden="1" outlineLevel="1" ht="75" customHeight="1">
-      <c r="A22" s="107" t="inlineStr"/>
-      <c r="B22" s="107" t="inlineStr">
-        <is>
-          <t>2026-01-27</t>
-        </is>
-      </c>
-      <c r="C22" s="107" t="inlineStr">
-        <is>
-          <t>C-</t>
-        </is>
-      </c>
-      <c r="D22" s="107" t="inlineStr">
-        <is>
-          <t>5/4</t>
-        </is>
-      </c>
-      <c r="E22" s="11" t="inlineStr">
-        <is>
-          <t>personally the class is hard, because there is a lot of content. do not procrastinate it will be your downfall. midterms are the same as mock exams and homework, so just practice that. group project at end is straightforward, homework is easy. ultimately your grade depends on your own effort so try!! [Get ready to read, Lecture heavy, Test heavy]</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" hidden="1" outlineLevel="1" ht="60" customHeight="1">
-      <c r="A23" s="105" t="inlineStr"/>
-      <c r="B23" s="105" t="inlineStr">
-        <is>
-          <t>2026-01-07</t>
-        </is>
-      </c>
-      <c r="C23" s="105" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D23" s="105" t="inlineStr">
-        <is>
-          <t>4/3</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>Alejandro is very nice and sometimes his accent is hard to understand in lecture but overall you understand what he is saying. The tests are exactly like the practice problems and he's very funny. Do the practice and you will do well in class! [Respected, Test heavy]</t>
         </is>
       </c>
     </row>
@@ -1857,7 +1975,7 @@
       <c r="A24" s="107" t="inlineStr"/>
       <c r="B24" s="107" t="inlineStr">
         <is>
-          <t>2026-01-06</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="C24" s="107" t="inlineStr">
@@ -1867,20 +1985,20 @@
       </c>
       <c r="D24" s="107" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>5/4</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>His lectures are enjoyable and structures the class to be very flexible with no required attendance and lenient homework policies. He does however have a spanish accent which makes understading lecture difficult sometimes. Additonally, I felt the lectures and textbook do not adequately prepare you for exams. [Amazing lectures, Respected, Graded by few things]</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" hidden="1" outlineLevel="1" ht="90" customHeight="1">
+          <t>personally the class is hard, because there is a lot of content. do not procrastinate it will be your downfall. midterms are the same as mock exams and homework, so just practice that. group project at end is straightforward, homework is easy. ultimately your grade depends on your own effort so try!! [Get ready to read, Lecture heavy, Test heavy]</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" hidden="1" outlineLevel="1" ht="60" customHeight="1">
       <c r="A25" s="105" t="inlineStr"/>
       <c r="B25" s="105" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2026-01-07</t>
         </is>
       </c>
       <c r="C25" s="105" t="inlineStr">
@@ -1890,12 +2008,12 @@
       </c>
       <c r="D25" s="105" t="inlineStr">
         <is>
-          <t>4/4</t>
+          <t>4/3</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>Really great professor, he writes on the board with practice questions, so concepts are easier to follow. He has an excellent TA who goes through all the questions, is super understanding and helpful, and she explains concepts really well. He has an accent, but it did not hinder my ability to learn. Definitely self-study as well, with the textbook! [Lecture heavy, Test heavy, Graded by few things]</t>
+          <t>Alejandro is very nice and sometimes his accent is hard to understand in lecture but overall you understand what he is saying. The tests are exactly like the practice problems and he's very funny. Do the practice and you will do well in class! [Respected, Test heavy]</t>
         </is>
       </c>
     </row>
@@ -1903,30 +2021,30 @@
       <c r="A26" s="107" t="inlineStr"/>
       <c r="B26" s="107" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2026-01-06</t>
         </is>
       </c>
       <c r="C26" s="107" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C-</t>
         </is>
       </c>
       <c r="D26" s="107" t="inlineStr">
         <is>
-          <t>5/3</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>Amazing professor. Has an accent but you get used to it. Can go through material pretty quickly, but he writes on board and explains while demonstrating, which helps a lot. He also goes back to explain if students are still confused. Exams are relatively the same as practice problems he gives. [Lecture heavy, Test heavy, Graded by few things]</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+          <t>His lectures are enjoyable and structures the class to be very flexible with no required attendance and lenient homework policies. He does however have a spanish accent which makes understading lecture difficult sometimes. Additonally, I felt the lectures and textbook do not adequately prepare you for exams. [Amazing lectures, Respected, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" hidden="1" outlineLevel="1" ht="90" customHeight="1">
       <c r="A27" s="105" t="inlineStr"/>
       <c r="B27" s="105" t="inlineStr">
         <is>
-          <t>2025-12-16</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="C27" s="105" t="inlineStr">
@@ -1936,12 +2054,12 @@
       </c>
       <c r="D27" s="105" t="inlineStr">
         <is>
-          <t>5/3</t>
+          <t>4/4</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>GREAT PROFESSOR. He breaks down the steps of each problem amazingly, accent is a little thick (sit in the front it helps a lot), His office hours are worth it, he will make sure you understand!! Work hard from the beginning and do ALL practice problems (repeats in test). [Hilarious, Respected, Test heavy]</t>
+          <t>Really great professor, he writes on the board with practice questions, so concepts are easier to follow. He has an excellent TA who goes through all the questions, is super understanding and helpful, and she explains concepts really well. He has an accent, but it did not hinder my ability to learn. Definitely self-study as well, with the textbook! [Lecture heavy, Test heavy, Graded by few things]</t>
         </is>
       </c>
     </row>
@@ -1949,12 +2067,12 @@
       <c r="A28" s="107" t="inlineStr"/>
       <c r="B28" s="107" t="inlineStr">
         <is>
-          <t>2025-12-11</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="C28" s="107" t="inlineStr">
         <is>
-          <t>Not sure yet</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D28" s="107" t="inlineStr">
@@ -1964,38 +2082,38 @@
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>Its a hard class and his lectures go by quick. With that being said he is really good at teaching and also really accessible outside of class. Answers emails extremely quickly and grades test within a few days of the test date. Exams are hard, but if you study and go to an office hour before the test your fine. [Amazing lectures, Test heavy, Accessible outside class]</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+          <t>Amazing professor. Has an accent but you get used to it. Can go through material pretty quickly, but he writes on board and explains while demonstrating, which helps a lot. He also goes back to explain if students are still confused. Exams are relatively the same as practice problems he gives. [Lecture heavy, Test heavy, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" hidden="1" outlineLevel="1" ht="60" customHeight="1">
       <c r="A29" s="105" t="inlineStr"/>
       <c r="B29" s="105" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
+          <t>2025-12-16</t>
         </is>
       </c>
       <c r="C29" s="105" t="inlineStr">
         <is>
-          <t>Drop/Withdrawal</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D29" s="105" t="inlineStr">
         <is>
-          <t>1/5</t>
+          <t>5/3</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>Professor flies through the lectures and his accent makes it difficult to understand and keep up. The course is already known for being a tough course. When questions are asked he sort of laughs and makes you feel bad before explaining. He has really good TAs though that help you step by step. I would definitely go to office hours.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+          <t>GREAT PROFESSOR. He breaks down the steps of each problem amazingly, accent is a little thick (sit in the front it helps a lot), His office hours are worth it, he will make sure you understand!! Work hard from the beginning and do ALL practice problems (repeats in test). [Hilarious, Respected, Test heavy]</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" hidden="1" outlineLevel="1" ht="75" customHeight="1">
       <c r="A30" s="107" t="inlineStr"/>
       <c r="B30" s="107" t="inlineStr">
         <is>
-          <t>2025-12-04</t>
+          <t>2025-12-11</t>
         </is>
       </c>
       <c r="C30" s="107" t="inlineStr">
@@ -2005,43 +2123,43 @@
       </c>
       <c r="D30" s="107" t="inlineStr">
         <is>
-          <t>1/5</t>
+          <t>5/3</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>- Genuinely moves at the speed of light - Is accessible outside of class, but truly have to grind for an A - Exams are super hard, homeworks are free - Professor is a bit condescending but means well [Lecture heavy, Test heavy, Graded by few things]</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" hidden="1" outlineLevel="1" ht="45" customHeight="1">
+          <t>Its a hard class and his lectures go by quick. With that being said he is really good at teaching and also really accessible outside of class. Answers emails extremely quickly and grades test within a few days of the test date. Exams are hard, but if you study and go to an office hour before the test your fine. [Amazing lectures, Test heavy, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" hidden="1" outlineLevel="1" ht="75" customHeight="1">
       <c r="A31" s="105" t="inlineStr"/>
       <c r="B31" s="105" t="inlineStr">
         <is>
-          <t>2025-11-17</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="C31" s="105" t="inlineStr">
         <is>
-          <t>Not sure yet</t>
+          <t>Drop/Withdrawal</t>
         </is>
       </c>
       <c r="D31" s="105" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>1/5</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>His accent and super fast pace of the class/lecture make it so hard to understand. The class is already hard and the speed of the lectures make this so hard [Lecture heavy, Graded by few things]</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+          <t>Professor flies through the lectures and his accent makes it difficult to understand and keep up. The course is already known for being a tough course. When questions are asked he sort of laughs and makes you feel bad before explaining. He has really good TAs though that help you step by step. I would definitely go to office hours.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" hidden="1" outlineLevel="1" ht="60" customHeight="1">
       <c r="A32" s="107" t="inlineStr"/>
       <c r="B32" s="107" t="inlineStr">
         <is>
-          <t>2025-10-16</t>
+          <t>2025-12-04</t>
         </is>
       </c>
       <c r="C32" s="107" t="inlineStr">
@@ -2051,43 +2169,43 @@
       </c>
       <c r="D32" s="107" t="inlineStr">
         <is>
-          <t>5/3</t>
+          <t>1/5</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>He does talk fast but if you don't understand or need to hear concept again he will gladly explain it to you until you get it. Very nice wants you to get an A but Econ isn't an easy class. Office hours are great way to prepare for test. Study guides very similar to exams. [Amazing lectures, Clear grading criteria, Accessible outside class]</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" hidden="1" outlineLevel="1" ht="30" customHeight="1">
+          <t>- Genuinely moves at the speed of light - Is accessible outside of class, but truly have to grind for an A - Exams are super hard, homeworks are free - Professor is a bit condescending but means well [Lecture heavy, Test heavy, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" hidden="1" outlineLevel="1" ht="45" customHeight="1">
       <c r="A33" s="105" t="inlineStr"/>
       <c r="B33" s="105" t="inlineStr">
         <is>
-          <t>2025-10-15</t>
+          <t>2025-11-17</t>
         </is>
       </c>
       <c r="C33" s="105" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Not sure yet</t>
         </is>
       </c>
       <c r="D33" s="105" t="inlineStr">
         <is>
-          <t>5/2</t>
+          <t>3/4</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>Fantastic Professor. Easy looking at. Funny guy. Muy bien</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" hidden="1" outlineLevel="1" ht="45" customHeight="1">
+          <t>His accent and super fast pace of the class/lecture make it so hard to understand. The class is already hard and the speed of the lectures make this so hard [Lecture heavy, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" hidden="1" outlineLevel="1" ht="75" customHeight="1">
       <c r="A34" s="107" t="inlineStr"/>
       <c r="B34" s="107" t="inlineStr">
         <is>
-          <t>2025-10-06</t>
+          <t>2025-10-16</t>
         </is>
       </c>
       <c r="C34" s="107" t="inlineStr">
@@ -2097,35 +2215,35 @@
       </c>
       <c r="D34" s="107" t="inlineStr">
         <is>
-          <t>4/2</t>
+          <t>5/3</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>Talks too fast and is hard to understand because of his accent. He mostly reads off the slides. But fun classes and passionate lecturer who encourages questions. He also uses real life examples which is useful.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+          <t>He does talk fast but if you don't understand or need to hear concept again he will gladly explain it to you until you get it. Very nice wants you to get an A but Econ isn't an easy class. Office hours are great way to prepare for test. Study guides very similar to exams. [Amazing lectures, Clear grading criteria, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" hidden="1" outlineLevel="1" ht="30" customHeight="1">
       <c r="A35" s="105" t="inlineStr"/>
       <c r="B35" s="105" t="inlineStr">
         <is>
-          <t>2025-10-06</t>
+          <t>2025-10-15</t>
         </is>
       </c>
       <c r="C35" s="105" t="inlineStr">
         <is>
-          <t>Not sure yet</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D35" s="105" t="inlineStr">
         <is>
-          <t>1/4</t>
+          <t>5/2</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>Bro talks so fast, literally I was better off teaching it to myself outside of class. EXTREMELY condescending. I would go to his office hours and he would laugh at certain students questions and belittle them. Idk how his rating is so high, I'd drop if it weren't already to late in the semester. [Test heavy]</t>
+          <t>Fantastic Professor. Easy looking at. Funny guy. Muy bien</t>
         </is>
       </c>
     </row>
@@ -2143,66 +2261,66 @@
       </c>
       <c r="D36" s="107" t="inlineStr">
         <is>
-          <t>5/4</t>
+          <t>4/2</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>no glaze, he's a really good professor and explained concepts very well. Would take him again every single time if I could choose. [Amazing lectures, Inspirational, Caring]</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" hidden="1" outlineLevel="1" ht="45" customHeight="1">
+          <t>Talks too fast and is hard to understand because of his accent. He mostly reads off the slides. But fun classes and passionate lecturer who encourages questions. He also uses real life examples which is useful.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" hidden="1" outlineLevel="1" ht="60" customHeight="1">
       <c r="A37" s="105" t="inlineStr"/>
       <c r="B37" s="105" t="inlineStr">
         <is>
-          <t>2025-06-25</t>
+          <t>2025-10-06</t>
         </is>
       </c>
       <c r="C37" s="105" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Not sure yet</t>
         </is>
       </c>
       <c r="D37" s="105" t="inlineStr">
         <is>
-          <t>5/2</t>
+          <t>1/4</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
-          <t>Best professor I've had at USC. Took his econ351 class in fall 2024 and learned so much. Class is on Marshall curve so its competitive to get an A, but it wasn't that hard. [Inspirational, Lecture heavy, Graded by few things]</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+          <t>Bro talks so fast, literally I was better off teaching it to myself outside of class. EXTREMELY condescending. I would go to his office hours and he would laugh at certain students questions and belittle them. Idk how his rating is so high, I'd drop if it weren't already to late in the semester. [Test heavy]</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" hidden="1" outlineLevel="1" ht="45" customHeight="1">
       <c r="A38" s="107" t="inlineStr"/>
       <c r="B38" s="107" t="inlineStr">
         <is>
-          <t>2025-05-30</t>
+          <t>2025-10-06</t>
         </is>
       </c>
       <c r="C38" s="107" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Not sure yet</t>
         </is>
       </c>
       <c r="D38" s="107" t="inlineStr">
         <is>
-          <t>5/2</t>
+          <t>5/4</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>ECON 351 is a hard class no matter what, but if you have to take it def take Professor Martinez. Funny guy, doesn't mind explaining over and over again and has great lecture slides. Great TAs and curve. Tests are hard but they are no matter who you take. Hosts lots of reviews and genuinely cares and wants to hear our perspectives. Miss him!</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+          <t>no glaze, he's a really good professor and explained concepts very well. Would take him again every single time if I could choose. [Amazing lectures, Inspirational, Caring]</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" hidden="1" outlineLevel="1" ht="45" customHeight="1">
       <c r="A39" s="105" t="inlineStr"/>
       <c r="B39" s="105" t="inlineStr">
         <is>
-          <t>2025-05-17</t>
+          <t>2025-06-25</t>
         </is>
       </c>
       <c r="C39" s="105" t="inlineStr">
@@ -2217,7 +2335,7 @@
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>This was my favorite professor of all time. In fact, the best professor I have ever had in my academic career. I highly recommend him. He makes lectures so fun. The class is hard, but if you understand calculus then you will ace the course. Highly recommend. [Amazing lectures, Inspirational, Caring]</t>
+          <t>Best professor I've had at USC. Took his econ351 class in fall 2024 and learned so much. Class is on Marshall curve so its competitive to get an A, but it wasn't that hard. [Inspirational, Lecture heavy, Graded by few things]</t>
         </is>
       </c>
     </row>
@@ -2225,45 +2343,45 @@
       <c r="A40" s="107" t="inlineStr"/>
       <c r="B40" s="107" t="inlineStr">
         <is>
-          <t>2025-05-01</t>
+          <t>2025-05-30</t>
         </is>
       </c>
       <c r="C40" s="107" t="inlineStr">
         <is>
-          <t>B-</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D40" s="107" t="inlineStr">
         <is>
-          <t>2/5</t>
+          <t>5/2</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
-          <t>I am not sure why his reviews are so high... I was barely able to get a B- in this class after studying over 10 hours for each test. The practice tests were only somewhat similar and the homework took a lot of time. I would not recommend this teacher unless you want to go to office hours every week and try to get him to like you. [Lecture heavy, Test heavy, Graded by few things]</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" hidden="1" outlineLevel="1" ht="30" customHeight="1">
+          <t>ECON 351 is a hard class no matter what, but if you have to take it def take Professor Martinez. Funny guy, doesn't mind explaining over and over again and has great lecture slides. Great TAs and curve. Tests are hard but they are no matter who you take. Hosts lots of reviews and genuinely cares and wants to hear our perspectives. Miss him!</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" hidden="1" outlineLevel="1" ht="60" customHeight="1">
       <c r="A41" s="105" t="inlineStr"/>
       <c r="B41" s="105" t="inlineStr">
         <is>
-          <t>2025-01-29</t>
+          <t>2025-05-17</t>
         </is>
       </c>
       <c r="C41" s="105" t="inlineStr">
         <is>
-          <t>Not sure yet</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D41" s="105" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>5/2</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>He's so easy to look at&amp;#8230; take him [Tough grader, EXTRA CREDIT, Amazing lectures]</t>
+          <t>This was my favorite professor of all time. In fact, the best professor I have ever had in my academic career. I highly recommend him. He makes lectures so fun. The class is hard, but if you understand calculus then you will ace the course. Highly recommend. [Amazing lectures, Inspirational, Caring]</t>
         </is>
       </c>
     </row>
@@ -2271,114 +2389,114 @@
       <c r="A42" s="107" t="inlineStr"/>
       <c r="B42" s="107" t="inlineStr">
         <is>
-          <t>2025-01-18</t>
+          <t>2025-05-01</t>
         </is>
       </c>
       <c r="C42" s="107" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="D42" s="107" t="inlineStr">
         <is>
-          <t>5/2</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
         <is>
-          <t>He is amazing. Went into 351 being really scared but honestly this class was way easier than I thought it would be. As long as you do all the practice problems and homework, there's no reason why you shouldn't get an A as tests are 95% similar to what you've seen before. For those complaining, they were just lazy and didn't do the work. [Amazing lectures, Hilarious, Graded by few things]</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+          <t>I am not sure why his reviews are so high... I was barely able to get a B- in this class after studying over 10 hours for each test. The practice tests were only somewhat similar and the homework took a lot of time. I would not recommend this teacher unless you want to go to office hours every week and try to get him to like you. [Lecture heavy, Test heavy, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" hidden="1" outlineLevel="1" ht="30" customHeight="1">
       <c r="A43" s="105" t="inlineStr"/>
       <c r="B43" s="105" t="inlineStr">
         <is>
-          <t>2025-01-10</t>
+          <t>2025-01-29</t>
         </is>
       </c>
       <c r="C43" s="105" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>Not sure yet</t>
         </is>
       </c>
       <c r="D43" s="105" t="inlineStr">
         <is>
-          <t>2/4</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t>office hours with the TA saved me as his were completely full all the time. lectures were organized but he went so fast with explanations and skipped many steps making it confusing. only graded on 3 tests no curve and they are very difficult and only 24 points so very hard to get a good grade [Graded by few things]</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+          <t>He's so easy to look at&amp;#8230; take him [Tough grader, EXTRA CREDIT, Amazing lectures]</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" hidden="1" outlineLevel="1" ht="75" customHeight="1">
       <c r="A44" s="107" t="inlineStr"/>
       <c r="B44" s="107" t="inlineStr">
         <is>
-          <t>2025-01-02</t>
+          <t>2025-01-18</t>
         </is>
       </c>
       <c r="C44" s="107" t="inlineStr">
         <is>
-          <t>Not sure yet</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D44" s="107" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>5/2</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
         <is>
-          <t>His lectures were very confusing, and he taught so quickly. If you go to HIS office hours, he'll give you all the answers to homework and practice tests, which was nice, but his tests were very hard. He does not curve at all, so expect your grade to be heavily based on how you perform on the tests.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+          <t>He is amazing. Went into 351 being really scared but honestly this class was way easier than I thought it would be. As long as you do all the practice problems and homework, there's no reason why you shouldn't get an A as tests are 95% similar to what you've seen before. For those complaining, they were just lazy and didn't do the work. [Amazing lectures, Hilarious, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" hidden="1" outlineLevel="1" ht="60" customHeight="1">
       <c r="A45" s="105" t="inlineStr"/>
       <c r="B45" s="105" t="inlineStr">
         <is>
-          <t>2024-12-28</t>
+          <t>2025-01-10</t>
         </is>
       </c>
       <c r="C45" s="105" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D45" s="105" t="inlineStr">
         <is>
-          <t>5/3</t>
+          <t>2/4</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>BEST PROF FOR ECON351. Tests are exactly what's on hw &amp; practice sets. Lots of office hours. He let us go to any of his lectures (no attendance taken) + recordings posted online. He's great at explaining and his class makes econ fun/interesting. No complaints at all, very fair/interesting/funny guy. He wants you to get an A! TAKE HIM, TRUST. [Hilarious, Respected, Lecture heavy]</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" hidden="1" outlineLevel="1" ht="30" customHeight="1">
+          <t>office hours with the TA saved me as his were completely full all the time. lectures were organized but he went so fast with explanations and skipped many steps making it confusing. only graded on 3 tests no curve and they are very difficult and only 24 points so very hard to get a good grade [Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" hidden="1" outlineLevel="1" ht="60" customHeight="1">
       <c r="A46" s="107" t="inlineStr"/>
       <c r="B46" s="107" t="inlineStr">
         <is>
-          <t>2024-12-21</t>
+          <t>2025-01-02</t>
         </is>
       </c>
       <c r="C46" s="107" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Not sure yet</t>
         </is>
       </c>
       <c r="D46" s="107" t="inlineStr">
         <is>
-          <t>5/3</t>
+          <t>3/5</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
         <is>
-          <t>Awesome professor. Lectures are interesting and exams are very similar to practice tests. [Amazing lectures, Clear grading criteria, Graded by few things]</t>
+          <t>His lectures were very confusing, and he taught so quickly. If you go to HIS office hours, he'll give you all the answers to homework and practice tests, which was nice, but his tests were very hard. He does not curve at all, so expect your grade to be heavily based on how you perform on the tests.</t>
         </is>
       </c>
     </row>
@@ -2386,30 +2504,30 @@
       <c r="A47" s="105" t="inlineStr"/>
       <c r="B47" s="105" t="inlineStr">
         <is>
-          <t>2024-12-21</t>
+          <t>2024-12-28</t>
         </is>
       </c>
       <c r="C47" s="105" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D47" s="105" t="inlineStr">
         <is>
-          <t>4/5</t>
+          <t>5/3</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>Good professor, but I would not take him again. he puts "trick questions" on exams so no one ends up getting them right. He switches up the questions on exams and they are way harder. I never put so much work into a class and I only got a B+ and thats with a 10 point curve so in reality my grade should be lower. [Tough grader, Amazing lectures, Test heavy]</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+          <t>BEST PROF FOR ECON351. Tests are exactly what's on hw &amp; practice sets. Lots of office hours. He let us go to any of his lectures (no attendance taken) + recordings posted online. He's great at explaining and his class makes econ fun/interesting. No complaints at all, very fair/interesting/funny guy. He wants you to get an A! TAKE HIM, TRUST. [Hilarious, Respected, Lecture heavy]</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" hidden="1" outlineLevel="1" ht="30" customHeight="1">
       <c r="A48" s="107" t="inlineStr"/>
       <c r="B48" s="107" t="inlineStr">
         <is>
-          <t>2024-12-20</t>
+          <t>2024-12-21</t>
         </is>
       </c>
       <c r="C48" s="107" t="inlineStr">
@@ -2424,38 +2542,38 @@
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>goat. 351 is hard but he makes it interesting and manageable. 3 exams each worth 30% and the other 10% is homework. go to lecture, do the practice problems and if you're still struggling read the textbook or go to office hours. take his class to get an A in econ and to laugh because he's hilarious. [Amazing lectures, Graded by few things]</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" hidden="1" outlineLevel="1" ht="45" customHeight="1">
+          <t>Awesome professor. Lectures are interesting and exams are very similar to practice tests. [Amazing lectures, Clear grading criteria, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" hidden="1" outlineLevel="1" ht="75" customHeight="1">
       <c r="A49" s="105" t="inlineStr"/>
       <c r="B49" s="105" t="inlineStr">
         <is>
-          <t>2024-12-20</t>
+          <t>2024-12-21</t>
         </is>
       </c>
       <c r="C49" s="105" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="D49" s="105" t="inlineStr">
         <is>
-          <t>5/3</t>
+          <t>4/5</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>Amazing professor! He includes real-world applications, which helps with understanding. And, I thought the class aligned with what he shared on the first day. Overall could not recommend more! [Amazing lectures, Caring]</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+          <t>Good professor, but I would not take him again. he puts "trick questions" on exams so no one ends up getting them right. He switches up the questions on exams and they are way harder. I never put so much work into a class and I only got a B+ and thats with a 10 point curve so in reality my grade should be lower. [Tough grader, Amazing lectures, Test heavy]</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" hidden="1" outlineLevel="1" ht="75" customHeight="1">
       <c r="A50" s="107" t="inlineStr"/>
       <c r="B50" s="107" t="inlineStr">
         <is>
-          <t>2024-12-19</t>
+          <t>2024-12-20</t>
         </is>
       </c>
       <c r="C50" s="107" t="inlineStr">
@@ -2465,20 +2583,20 @@
       </c>
       <c r="D50" s="107" t="inlineStr">
         <is>
-          <t>5/2</t>
+          <t>5/3</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>Goat. Simple as that. Gives plenty of practice tests/problems that are identical in concept and form to the actual tests. Just be aware that the bar for an A-range grade may change throughout the semester (i.e. A-range = &gt;80 to A-range = &gt;85). [Caring, Test heavy, Accessible outside class]</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+          <t>goat. 351 is hard but he makes it interesting and manageable. 3 exams each worth 30% and the other 10% is homework. go to lecture, do the practice problems and if you're still struggling read the textbook or go to office hours. take his class to get an A in econ and to laugh because he's hilarious. [Amazing lectures, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" hidden="1" outlineLevel="1" ht="45" customHeight="1">
       <c r="A51" s="105" t="inlineStr"/>
       <c r="B51" s="105" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
+          <t>2024-12-20</t>
         </is>
       </c>
       <c r="C51" s="105" t="inlineStr">
@@ -2493,20 +2611,20 @@
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
-          <t>Best teacher for microeconomics. Explains concepts well and is very clear about what will be on exams. Practice exams and chapter questions are identical to what will be on the tests. He's also super caring and will take the time to help you out and answer questions. By far my favorite professor this semester! [Caring]</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+          <t>Amazing professor! He includes real-world applications, which helps with understanding. And, I thought the class aligned with what he shared on the first day. Overall could not recommend more! [Amazing lectures, Caring]</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" hidden="1" outlineLevel="1" ht="60" customHeight="1">
       <c r="A52" s="107" t="inlineStr"/>
       <c r="B52" s="107" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
+          <t>2024-12-19</t>
         </is>
       </c>
       <c r="C52" s="107" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D52" s="107" t="inlineStr">
@@ -2516,30 +2634,30 @@
       </c>
       <c r="E52" s="11" t="inlineStr">
         <is>
-          <t>Professor Alejandro is one of my favorite and best professors in Marshall! He is so engaging and incorporated lots of humor into his lectures (which attendance was not mandatory for). It's also evident that he wants his students to do well and holds many office hours for studnets. Would totally take him again. THE GOAT &amp;#128016; [Amazing lectures, Lecture heavy, Accessible outside class]</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+          <t>Goat. Simple as that. Gives plenty of practice tests/problems that are identical in concept and form to the actual tests. Just be aware that the bar for an A-range grade may change throughout the semester (i.e. A-range = &gt;80 to A-range = &gt;85). [Caring, Test heavy, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" hidden="1" outlineLevel="1" ht="75" customHeight="1">
       <c r="A53" s="105" t="inlineStr"/>
       <c r="B53" s="105" t="inlineStr">
         <is>
-          <t>2024-12-04</t>
+          <t>2024-12-05</t>
         </is>
       </c>
       <c r="C53" s="105" t="inlineStr">
         <is>
-          <t>Not sure yet</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D53" s="105" t="inlineStr">
         <is>
-          <t>5/1</t>
+          <t>5/3</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
-          <t>Professor Alejandro is awesome. His lecture is inspirational and well-explained. I love the vibe of his class, and the tests are always easy as long as you finish the sample problems. [Amazing lectures, Inspirational, Accessible outside class]</t>
+          <t>Best teacher for microeconomics. Explains concepts well and is very clear about what will be on exams. Practice exams and chapter questions are identical to what will be on the tests. He's also super caring and will take the time to help you out and answer questions. By far my favorite professor this semester! [Caring]</t>
         </is>
       </c>
     </row>
@@ -2547,53 +2665,53 @@
       <c r="A54" s="107" t="inlineStr"/>
       <c r="B54" s="107" t="inlineStr">
         <is>
-          <t>2024-12-03</t>
+          <t>2024-12-05</t>
         </is>
       </c>
       <c r="C54" s="107" t="inlineStr">
         <is>
-          <t>Not sure yet</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D54" s="107" t="inlineStr">
         <is>
-          <t>5/3</t>
+          <t>5/2</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>If you attend classes and office hours, you will understand all concepts. The class isn't too bad especially if you did IB Econ. Just do the homework and practice tests, and you're good. His papers are also not too bad so if you practice well you will do well. [Clear grading criteria, Lots of homework, Accessible outside class]</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+          <t>Professor Alejandro is one of my favorite and best professors in Marshall! He is so engaging and incorporated lots of humor into his lectures (which attendance was not mandatory for). It's also evident that he wants his students to do well and holds many office hours for studnets. Would totally take him again. THE GOAT &amp;#128016; [Amazing lectures, Lecture heavy, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" hidden="1" outlineLevel="1" ht="60" customHeight="1">
       <c r="A55" s="105" t="inlineStr"/>
       <c r="B55" s="105" t="inlineStr">
         <is>
-          <t>2024-11-13</t>
+          <t>2024-12-04</t>
         </is>
       </c>
       <c r="C55" s="105" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Not sure yet</t>
         </is>
       </c>
       <c r="D55" s="105" t="inlineStr">
         <is>
-          <t>5/3</t>
+          <t>5/1</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t>Best 351 prof he's so nice!!! Midterms are exactly like practice tests given. Homework is completion as long as you get half right and he gives you answers in office hours. Don't need to go to class-- he posts lectures and doesn't take attendance. Do the practice problems twice before the 3 tests and you can get an A. 80 or above overall is an A. [Accessible outside class]</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" hidden="1" outlineLevel="1" ht="45" customHeight="1">
+          <t>Professor Alejandro is awesome. His lecture is inspirational and well-explained. I love the vibe of his class, and the tests are always easy as long as you finish the sample problems. [Amazing lectures, Inspirational, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" hidden="1" outlineLevel="1" ht="75" customHeight="1">
       <c r="A56" s="107" t="inlineStr"/>
       <c r="B56" s="107" t="inlineStr">
         <is>
-          <t>2024-11-13</t>
+          <t>2024-12-03</t>
         </is>
       </c>
       <c r="C56" s="107" t="inlineStr">
@@ -2603,25 +2721,25 @@
       </c>
       <c r="D56" s="107" t="inlineStr">
         <is>
-          <t>5/2</t>
+          <t>5/3</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" hidden="1" outlineLevel="1" ht="90" customHeight="1">
+          <t>If you attend classes and office hours, you will understand all concepts. The class isn't too bad especially if you did IB Econ. Just do the homework and practice tests, and you're good. His papers are also not too bad so if you practice well you will do well. [Clear grading criteria, Lots of homework, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" hidden="1" outlineLevel="1" ht="75" customHeight="1">
       <c r="A57" s="105" t="inlineStr"/>
       <c r="B57" s="105" t="inlineStr">
         <is>
-          <t>2024-11-11</t>
+          <t>2024-11-13</t>
         </is>
       </c>
       <c r="C57" s="105" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D57" s="105" t="inlineStr">
@@ -2631,61 +2749,61 @@
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t>It's definitely a difficult class and you have to study A LOT for tests, but he holds office hours every day for the entire semester and gives a bunch of practice problems prior to midterms. The homework isn't too bad, but the difficulty of the class is dependent on whether or not you go to lectures. He overall made a difficult class digestible. [Amazing lectures, Lecture heavy, Accessible outside class]</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" hidden="1" outlineLevel="1" ht="30" customHeight="1">
+          <t>Best 351 prof he's so nice!!! Midterms are exactly like practice tests given. Homework is completion as long as you get half right and he gives you answers in office hours. Don't need to go to class-- he posts lectures and doesn't take attendance. Do the practice problems twice before the 3 tests and you can get an A. 80 or above overall is an A. [Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" hidden="1" outlineLevel="1" ht="45" customHeight="1">
       <c r="A58" s="107" t="inlineStr"/>
       <c r="B58" s="107" t="inlineStr">
         <is>
-          <t>2024-10-22</t>
+          <t>2024-11-13</t>
         </is>
       </c>
       <c r="C58" s="107" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Not sure yet</t>
         </is>
       </c>
       <c r="D58" s="107" t="inlineStr">
         <is>
-          <t>5/3</t>
+          <t>5/2</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>Exam questions are very similar to the practice sets he provides. Wants you to do well. [Caring, Test heavy, Graded by few things]</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+          <t>&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;&amp;#128016;</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" hidden="1" outlineLevel="1" ht="90" customHeight="1">
       <c r="A59" s="105" t="inlineStr"/>
       <c r="B59" s="105" t="inlineStr">
         <is>
-          <t>2024-08-01</t>
+          <t>2024-11-11</t>
         </is>
       </c>
       <c r="C59" s="105" t="inlineStr">
         <is>
-          <t>A-</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D59" s="105" t="inlineStr">
         <is>
-          <t>5/2</t>
+          <t>5/3</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t>Such a great professor his class is so manageable. I barely went to lecture and never went to office hours and did perfectly fine. Homework is graded very easily and basically every single possible midterm question is provided to you between all the practice sets. Do all the questions and you'll be fine. By far the best choice for 351.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+          <t>It's definitely a difficult class and you have to study A LOT for tests, but he holds office hours every day for the entire semester and gives a bunch of practice problems prior to midterms. The homework isn't too bad, but the difficulty of the class is dependent on whether or not you go to lectures. He overall made a difficult class digestible. [Amazing lectures, Lecture heavy, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" hidden="1" outlineLevel="1" ht="30" customHeight="1">
       <c r="A60" s="107" t="inlineStr"/>
       <c r="B60" s="107" t="inlineStr">
         <is>
-          <t>2024-06-22</t>
+          <t>2024-10-22</t>
         </is>
       </c>
       <c r="C60" s="107" t="inlineStr">
@@ -2700,15 +2818,15 @@
       </c>
       <c r="E60" s="11" t="inlineStr">
         <is>
-          <t>Great course if you show up to every lecture and pay attention. Taking notes, reviewing practice problems, and going to office hours when I needed help with certain problems made the class not overly difficult. Great lecturer and cares about his students. Would take him again if I could. [Respected, Lecture heavy]</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" hidden="1" outlineLevel="1" ht="45" customHeight="1">
+          <t>Exam questions are very similar to the practice sets he provides. Wants you to do well. [Caring, Test heavy, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" hidden="1" outlineLevel="1" ht="75" customHeight="1">
       <c r="A61" s="105" t="inlineStr"/>
       <c r="B61" s="105" t="inlineStr">
         <is>
-          <t>2024-06-19</t>
+          <t>2024-08-01</t>
         </is>
       </c>
       <c r="C61" s="105" t="inlineStr">
@@ -2718,20 +2836,20 @@
       </c>
       <c r="D61" s="105" t="inlineStr">
         <is>
-          <t>5/3</t>
+          <t>5/2</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t>I never went to his office hours and skipped around 70% of classes and still got a decent grade. He is a good lecturer and grades aren't hard to get. PLEASE do practice questions because exam questions are 80% based on them.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+          <t>Such a great professor his class is so manageable. I barely went to lecture and never went to office hours and did perfectly fine. Homework is graded very easily and basically every single possible midterm question is provided to you between all the practice sets. Do all the questions and you'll be fine. By far the best choice for 351.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" hidden="1" outlineLevel="1" ht="60" customHeight="1">
       <c r="A62" s="107" t="inlineStr"/>
       <c r="B62" s="107" t="inlineStr">
         <is>
-          <t>2024-05-28</t>
+          <t>2024-06-22</t>
         </is>
       </c>
       <c r="C62" s="107" t="inlineStr">
@@ -2741,35 +2859,35 @@
       </c>
       <c r="D62" s="107" t="inlineStr">
         <is>
-          <t>5/2</t>
+          <t>5/3</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
         <is>
-          <t>Marquina made ECON351 a breeze. His lectures are straightforward, engaging, and explain the material well. Your grade is determined by 3 tests spaced out throughout the semester. They're non-cumulative which is nice. Do the homework and the exam practice sets and you'll get a top grade. [Amazing lectures, Clear grading criteria, Graded by few things]</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+          <t>Great course if you show up to every lecture and pay attention. Taking notes, reviewing practice problems, and going to office hours when I needed help with certain problems made the class not overly difficult. Great lecturer and cares about his students. Would take him again if I could. [Respected, Lecture heavy]</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" hidden="1" outlineLevel="1" ht="45" customHeight="1">
       <c r="A63" s="105" t="inlineStr"/>
       <c r="B63" s="105" t="inlineStr">
         <is>
-          <t>2024-05-19</t>
+          <t>2024-06-19</t>
         </is>
       </c>
       <c r="C63" s="105" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>A-</t>
         </is>
       </c>
       <c r="D63" s="105" t="inlineStr">
         <is>
-          <t>5/1</t>
+          <t>5/3</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t>Makes microeconomics easy and provides fun examples for students to engage with. Do the homework and the practice midterms/final he provides to study and you will get an A in this class. Provides really, really helpful office hours for questions on homework and allows test revision. GOATED Marshall professor. [Lots of homework, Test heavy]</t>
+          <t>I never went to his office hours and skipped around 70% of classes and still got a decent grade. He is a good lecturer and grades aren't hard to get. PLEASE do practice questions because exam questions are 80% based on them.</t>
         </is>
       </c>
     </row>
@@ -2777,7 +2895,7 @@
       <c r="A64" s="107" t="inlineStr"/>
       <c r="B64" s="107" t="inlineStr">
         <is>
-          <t>2024-05-10</t>
+          <t>2024-05-28</t>
         </is>
       </c>
       <c r="C64" s="107" t="inlineStr">
@@ -2787,48 +2905,48 @@
       </c>
       <c r="D64" s="107" t="inlineStr">
         <is>
-          <t>5/3</t>
+          <t>5/2</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
         <is>
-          <t>Great professor, but a fast lecturer. Overall would highly recommend him for Econ 351. The course is graded on only 3 written exams and weekly homework assignments, and as long as you do the practice questions he posts before each exam, they should be quite easy. [Inspirational, Graded by few things, Accessible outside class]</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" hidden="1" outlineLevel="1" ht="90" customHeight="1">
+          <t>Marquina made ECON351 a breeze. His lectures are straightforward, engaging, and explain the material well. Your grade is determined by 3 tests spaced out throughout the semester. They're non-cumulative which is nice. Do the homework and the exam practice sets and you'll get a top grade. [Amazing lectures, Clear grading criteria, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" hidden="1" outlineLevel="1" ht="75" customHeight="1">
       <c r="A65" s="105" t="inlineStr"/>
       <c r="B65" s="105" t="inlineStr">
         <is>
-          <t>2024-05-02</t>
+          <t>2024-05-19</t>
         </is>
       </c>
       <c r="C65" s="105" t="inlineStr">
         <is>
-          <t>A+</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D65" s="105" t="inlineStr">
         <is>
-          <t>5/2</t>
+          <t>5/1</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>Despite being a new prof, Alejandro is a really engaging and fun lecturer. He's accessible and will help you perform your best in class as long as you put in the work. I love him and would take his classes again. Looking forward to taking his class in my upperclassmen years. Go to office hours before a midterm/final and I guarantee you'll ace them. [Gives good feedback, Caring, Accessible outside class]</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" hidden="1" outlineLevel="1" ht="30" customHeight="1">
+          <t>Makes microeconomics easy and provides fun examples for students to engage with. Do the homework and the practice midterms/final he provides to study and you will get an A in this class. Provides really, really helpful office hours for questions on homework and allows test revision. GOATED Marshall professor. [Lots of homework, Test heavy]</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" hidden="1" outlineLevel="1" ht="75" customHeight="1">
       <c r="A66" s="107" t="inlineStr"/>
       <c r="B66" s="107" t="inlineStr">
         <is>
-          <t>2024-05-02</t>
+          <t>2024-05-10</t>
         </is>
       </c>
       <c r="C66" s="107" t="inlineStr">
         <is>
-          <t>A+</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D66" s="107" t="inlineStr">
@@ -2838,11 +2956,11 @@
       </c>
       <c r="E66" s="11" t="inlineStr">
         <is>
-          <t>351 is a hard class and he's easily the best teacher for it. [Caring, Test heavy, Accessible outside class]</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+          <t>Great professor, but a fast lecturer. Overall would highly recommend him for Econ 351. The course is graded on only 3 written exams and weekly homework assignments, and as long as you do the practice questions he posts before each exam, they should be quite easy. [Inspirational, Graded by few things, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" hidden="1" outlineLevel="1" ht="90" customHeight="1">
       <c r="A67" s="105" t="inlineStr"/>
       <c r="B67" s="105" t="inlineStr">
         <is>
@@ -2851,30 +2969,30 @@
       </c>
       <c r="C67" s="105" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="D67" s="105" t="inlineStr">
         <is>
-          <t>5/3</t>
+          <t>5/2</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>Professor Martinez-Marquina was hands-down awesome! He's so caring and easy to talk to if you had concerns about your grade or the course content. Lectures are fast-paced for sure, but his office hours are SO worth it! Overall such an amazing professor! He's super accommodating and wants you to succeed in and out of class. [Amazing lectures, Respected, Accessible outside class]</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" hidden="1" outlineLevel="1" ht="45" customHeight="1">
+          <t>Despite being a new prof, Alejandro is a really engaging and fun lecturer. He's accessible and will help you perform your best in class as long as you put in the work. I love him and would take his classes again. Looking forward to taking his class in my upperclassmen years. Go to office hours before a midterm/final and I guarantee you'll ace them. [Gives good feedback, Caring, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" hidden="1" outlineLevel="1" ht="30" customHeight="1">
       <c r="A68" s="107" t="inlineStr"/>
       <c r="B68" s="107" t="inlineStr">
         <is>
-          <t>2024-04-25</t>
+          <t>2024-05-02</t>
         </is>
       </c>
       <c r="C68" s="107" t="inlineStr">
         <is>
-          <t>Not sure yet</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="D68" s="107" t="inlineStr">
@@ -2884,7 +3002,7 @@
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>Tests are very similar to practice problems, and lectures are easy to follow. If you show up to class it is very manageable! [Amazing lectures, Clear grading criteria, Gives good feedback]</t>
+          <t>351 is a hard class and he's easily the best teacher for it. [Caring, Test heavy, Accessible outside class]</t>
         </is>
       </c>
     </row>
@@ -2892,12 +3010,12 @@
       <c r="A69" s="105" t="inlineStr"/>
       <c r="B69" s="105" t="inlineStr">
         <is>
-          <t>2024-04-16</t>
+          <t>2024-05-02</t>
         </is>
       </c>
       <c r="C69" s="105" t="inlineStr">
         <is>
-          <t>Not sure yet</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D69" s="105" t="inlineStr">
@@ -2907,30 +3025,30 @@
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>Econ 351 is probably one of the hardest classes in Marshall. However, Marquina makes the content very much digestable. He's a very caring professor and wants you to understand the topic, and the lengths that he goes to to do so is very respectable. Genuine guy, very fun to talk to and honestly an amazing professor. [Inspirational, Caring, Respected]</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+          <t>Professor Martinez-Marquina was hands-down awesome! He's so caring and easy to talk to if you had concerns about your grade or the course content. Lectures are fast-paced for sure, but his office hours are SO worth it! Overall such an amazing professor! He's super accommodating and wants you to succeed in and out of class. [Amazing lectures, Respected, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" hidden="1" outlineLevel="1" ht="45" customHeight="1">
       <c r="A70" s="107" t="inlineStr"/>
       <c r="B70" s="107" t="inlineStr">
         <is>
-          <t>2024-04-15</t>
+          <t>2024-04-25</t>
         </is>
       </c>
       <c r="C70" s="107" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Not sure yet</t>
         </is>
       </c>
       <c r="D70" s="107" t="inlineStr">
         <is>
-          <t>5/2</t>
+          <t>5/3</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
-          <t>Literally my favorite professor I've taken so far. I would take ANY class he teaches! He was super accessible and reasonable. He genuinely cared for you to grasp the material, and would often stay late after class or office hours if you needed his help. [Amazing lectures, Respected, Accessible outside class]</t>
+          <t>Tests are very similar to practice problems, and lectures are easy to follow. If you show up to class it is very manageable! [Amazing lectures, Clear grading criteria, Gives good feedback]</t>
         </is>
       </c>
     </row>
@@ -2938,30 +3056,30 @@
       <c r="A71" s="105" t="inlineStr"/>
       <c r="B71" s="105" t="inlineStr">
         <is>
-          <t>2024-04-02</t>
+          <t>2024-04-16</t>
         </is>
       </c>
       <c r="C71" s="105" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Not sure yet</t>
         </is>
       </c>
       <c r="D71" s="105" t="inlineStr">
         <is>
-          <t>5/4</t>
+          <t>5/3</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
-          <t>Yes, lectures are fast paced &amp; the material is difficult. However, Alejandro makes everything manageable. Coming in with no econ experience, I was still able to succeed. To succeed: go to class, read the textbook (its free &amp; really helpful), go to office hours, &amp; do the practice problems (all 3 tests resemble practice problems VERY closely). [Amazing lectures, Gives good feedback, Test heavy]</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" hidden="1" outlineLevel="1" ht="30" customHeight="1">
+          <t>Econ 351 is probably one of the hardest classes in Marshall. However, Marquina makes the content very much digestable. He's a very caring professor and wants you to understand the topic, and the lengths that he goes to to do so is very respectable. Genuine guy, very fun to talk to and honestly an amazing professor. [Inspirational, Caring, Respected]</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" hidden="1" outlineLevel="1" ht="60" customHeight="1">
       <c r="A72" s="107" t="inlineStr"/>
       <c r="B72" s="107" t="inlineStr">
         <is>
-          <t>2023-10-25</t>
+          <t>2024-04-15</t>
         </is>
       </c>
       <c r="C72" s="107" t="inlineStr">
@@ -2971,12 +3089,12 @@
       </c>
       <c r="D72" s="107" t="inlineStr">
         <is>
-          <t>5/1</t>
+          <t>5/2</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>great professor with clear lectures, easy homework and tests [Amazing lectures, Caring, Respected]</t>
+          <t>Literally my favorite professor I've taken so far. I would take ANY class he teaches! He was super accessible and reasonable. He genuinely cared for you to grasp the material, and would often stay late after class or office hours if you needed his help. [Amazing lectures, Respected, Accessible outside class]</t>
         </is>
       </c>
     </row>
@@ -2984,7 +3102,7 @@
       <c r="A73" s="105" t="inlineStr"/>
       <c r="B73" s="105" t="inlineStr">
         <is>
-          <t>2023-06-21</t>
+          <t>2024-04-02</t>
         </is>
       </c>
       <c r="C73" s="105" t="inlineStr">
@@ -2994,48 +3112,48 @@
       </c>
       <c r="D73" s="105" t="inlineStr">
         <is>
-          <t>5/3</t>
+          <t>5/4</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
-          <t>Take this class +1 !! Prof. Martinez explains the lectures thoroughly, provides real-world examples, and his pace is perfect. He is determined to help students succeed by going above and beyond to provide office hours (especially before exams) and exam review/revision afterward. Test-heavy, but the content is relevant to lectures and homework. [Amazing lectures, Caring, Accessible outside class]</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+          <t>Yes, lectures are fast paced &amp; the material is difficult. However, Alejandro makes everything manageable. Coming in with no econ experience, I was still able to succeed. To succeed: go to class, read the textbook (its free &amp; really helpful), go to office hours, &amp; do the practice problems (all 3 tests resemble practice problems VERY closely). [Amazing lectures, Gives good feedback, Test heavy]</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" hidden="1" outlineLevel="1" ht="30" customHeight="1">
       <c r="A74" s="107" t="inlineStr"/>
       <c r="B74" s="107" t="inlineStr">
         <is>
-          <t>2023-05-26</t>
+          <t>2023-10-25</t>
         </is>
       </c>
       <c r="C74" s="107" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D74" s="107" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>5/1</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
         <is>
-          <t>Amazing professor who truly wants his students to learn and succeed. Grading: 90% from 3 exams, 10% from HW. Thought this course was a very quantitative, fast-paced, and difficult class to get adjusted to. I struggling at first as I failed (D+) both midterm 1 and midterm 2 (post-curve). Got an A on the final exam (post-curve). Ended with a B. [Clear grading criteria, Caring, Graded by few things]</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+          <t>great professor with clear lectures, easy homework and tests [Amazing lectures, Caring, Respected]</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" hidden="1" outlineLevel="1" ht="75" customHeight="1">
       <c r="A75" s="105" t="inlineStr"/>
       <c r="B75" s="105" t="inlineStr">
         <is>
-          <t>2023-05-09</t>
+          <t>2023-06-21</t>
         </is>
       </c>
       <c r="C75" s="105" t="inlineStr">
         <is>
-          <t>Not sure yet</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D75" s="105" t="inlineStr">
@@ -3045,76 +3163,76 @@
       </c>
       <c r="E75" s="8" t="inlineStr">
         <is>
-          <t>He's a really caring and understanding professor. Although Econ 351 itself can be tough, he makes the lectures engaging and tries his best to help us understand. Doing the homework and practice chapter samples are really helpful for the tests! [Clear grading criteria, Gives good feedback, Caring]</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" hidden="1" outlineLevel="1" ht="90" customHeight="1">
+          <t>Take this class +1 !! Prof. Martinez explains the lectures thoroughly, provides real-world examples, and his pace is perfect. He is determined to help students succeed by going above and beyond to provide office hours (especially before exams) and exam review/revision afterward. Test-heavy, but the content is relevant to lectures and homework. [Amazing lectures, Caring, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" hidden="1" outlineLevel="1" ht="75" customHeight="1">
       <c r="A76" s="107" t="inlineStr"/>
       <c r="B76" s="107" t="inlineStr">
         <is>
-          <t>2023-05-06</t>
+          <t>2023-05-26</t>
         </is>
       </c>
       <c r="C76" s="107" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D76" s="107" t="inlineStr">
         <is>
-          <t>5/4</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
         <is>
-          <t>Professor Marquina is a very kind and sweet guy. You can tell he genuinely cares for his students, he consistently gave extra office hours and met with me 1-on-1 after my poor 2nd midterm performance, encouraged and strategized with me on how I could improve. 2 midterms &amp; 1 final, very challenging course content. Get ready to put in the work [Caring, Graded by few things, Accessible outside class]</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+          <t>Amazing professor who truly wants his students to learn and succeed. Grading: 90% from 3 exams, 10% from HW. Thought this course was a very quantitative, fast-paced, and difficult class to get adjusted to. I struggling at first as I failed (D+) both midterm 1 and midterm 2 (post-curve). Got an A on the final exam (post-curve). Ended with a B. [Clear grading criteria, Caring, Graded by few things]</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" hidden="1" outlineLevel="1" ht="60" customHeight="1">
       <c r="A77" s="105" t="inlineStr"/>
       <c r="B77" s="105" t="inlineStr">
         <is>
-          <t>2023-04-26</t>
+          <t>2023-05-09</t>
         </is>
       </c>
       <c r="C77" s="105" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Not sure yet</t>
         </is>
       </c>
       <c r="D77" s="105" t="inlineStr">
         <is>
-          <t>5/2</t>
+          <t>5/3</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
         <is>
-          <t>Take this class!!!!!!! He is such a nice guy and is always willing to meet with students, whether that means just re explaining something after class, holding office hours, or scheduling 1 on 1 time to meet with you and talk through questions or go over tests. If you pay any attention in the lectures you won't have any trouble.</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+          <t>He's a really caring and understanding professor. Although Econ 351 itself can be tough, he makes the lectures engaging and tries his best to help us understand. Doing the homework and practice chapter samples are really helpful for the tests! [Clear grading criteria, Gives good feedback, Caring]</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" hidden="1" outlineLevel="1" ht="90" customHeight="1">
       <c r="A78" s="107" t="inlineStr"/>
       <c r="B78" s="107" t="inlineStr">
         <is>
-          <t>2023-04-26</t>
+          <t>2023-05-06</t>
         </is>
       </c>
       <c r="C78" s="107" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D78" s="107" t="inlineStr">
         <is>
-          <t>5/3</t>
+          <t>5/4</t>
         </is>
       </c>
       <c r="E78" s="11" t="inlineStr">
         <is>
-          <t>Prof. Martinez is a fairly new professor, but he's one of the best I've had. Although the course is decently tough, if you took AP Econ in Highschool, you'll be fine. Otherwise, he provides very good lectures and is very accessible if you have questions. The hw is harder than the tests, and the practice problems are identical/very similar to tests.</t>
+          <t>Professor Marquina is a very kind and sweet guy. You can tell he genuinely cares for his students, he consistently gave extra office hours and met with me 1-on-1 after my poor 2nd midterm performance, encouraged and strategized with me on how I could improve. 2 midterms &amp; 1 final, very challenging course content. Get ready to put in the work [Caring, Graded by few things, Accessible outside class]</t>
         </is>
       </c>
     </row>
@@ -3122,30 +3240,30 @@
       <c r="A79" s="105" t="inlineStr"/>
       <c r="B79" s="105" t="inlineStr">
         <is>
-          <t>2023-04-06</t>
+          <t>2023-04-26</t>
         </is>
       </c>
       <c r="C79" s="105" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D79" s="105" t="inlineStr">
         <is>
-          <t>5/3</t>
+          <t>5/2</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
         <is>
-          <t>Despite the difficulty of Micro, Professor Martinez-Marquina's lectures are engaging, practical, and interactive. He emphasizes building intuition to see the world from a different perspective and is readily available for support outside of class. Professor Martinez-Marquina's passion and expertise in the subject matter further enrich his lectures. [Amazing lectures, Inspirational, Respected]</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+          <t>Take this class!!!!!!! He is such a nice guy and is always willing to meet with students, whether that means just re explaining something after class, holding office hours, or scheduling 1 on 1 time to meet with you and talk through questions or go over tests. If you pay any attention in the lectures you won't have any trouble.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" hidden="1" outlineLevel="1" ht="75" customHeight="1">
       <c r="A80" s="107" t="inlineStr"/>
       <c r="B80" s="107" t="inlineStr">
         <is>
-          <t>2023-04-06</t>
+          <t>2023-04-26</t>
         </is>
       </c>
       <c r="C80" s="107" t="inlineStr">
@@ -3155,12 +3273,12 @@
       </c>
       <c r="D80" s="107" t="inlineStr">
         <is>
-          <t>5/4</t>
+          <t>5/3</t>
         </is>
       </c>
       <c r="E80" s="11" t="inlineStr">
         <is>
-          <t>Thought he was going to be hard since he was new, but ended up being one of the most chill professors I've had. Makes homework harder than the exams, but uses examples similar to slides. Keeps lectures entertaining. [Amazing lectures, Caring]</t>
+          <t>Prof. Martinez is a fairly new professor, but he's one of the best I've had. Although the course is decently tough, if you took AP Econ in Highschool, you'll be fine. Otherwise, he provides very good lectures and is very accessible if you have questions. The hw is harder than the tests, and the practice problems are identical/very similar to tests.</t>
         </is>
       </c>
     </row>
@@ -3168,34 +3286,30 @@
       <c r="A81" s="105" t="inlineStr"/>
       <c r="B81" s="105" t="inlineStr">
         <is>
-          <t>2023-04-05</t>
+          <t>2023-04-06</t>
         </is>
       </c>
       <c r="C81" s="105" t="inlineStr">
         <is>
-          <t>Incomplete</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D81" s="105" t="inlineStr">
         <is>
-          <t>5/5</t>
+          <t>5/3</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
         <is>
-          <t>The hardest class at usc, but he makes it worth it. Great professor overall - willing to work with students to help with exams and understanding the material. His lectures go by very fast, and his accent can be hard to understand at first. Go to office hours, read the textbook, pay attention and go to every single class...and maybe you'll pass. [Caring, Test heavy, Accessible outside class]</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" hidden="1" outlineLevel="1" ht="75" customHeight="1">
-      <c r="A82" s="106" t="inlineStr">
-        <is>
-          <t>SPAN-290</t>
-        </is>
-      </c>
+          <t>Despite the difficulty of Micro, Professor Martinez-Marquina's lectures are engaging, practical, and interactive. He emphasizes building intuition to see the world from a different perspective and is readily available for support outside of class. Professor Martinez-Marquina's passion and expertise in the subject matter further enrich his lectures. [Amazing lectures, Inspirational, Respected]</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="A82" s="107" t="inlineStr"/>
       <c r="B82" s="107" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2023-04-06</t>
         </is>
       </c>
       <c r="C82" s="107" t="inlineStr">
@@ -3205,58 +3319,62 @@
       </c>
       <c r="D82" s="107" t="inlineStr">
         <is>
-          <t>5/2</t>
+          <t>5/4</t>
         </is>
       </c>
       <c r="E82" s="11" t="inlineStr">
         <is>
-          <t>Prof. Steinberg was engaging during lectures. We were assigned 2 readings per week, and I still passed the class by only attending lectures (no reading). If you follow along in class and take good notes, and refer to the slides him and the TAs post, you'll be in for an easy A and learn a ton! [Get ready to read, Amazing lectures, Hilarious]</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+          <t>Thought he was going to be hard since he was new, but ended up being one of the most chill professors I've had. Makes homework harder than the exams, but uses examples similar to slides. Keeps lectures entertaining. [Amazing lectures, Caring]</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" hidden="1" outlineLevel="1" ht="75" customHeight="1">
       <c r="A83" s="105" t="inlineStr"/>
       <c r="B83" s="105" t="inlineStr">
         <is>
-          <t>2024-05-18</t>
+          <t>2023-04-05</t>
         </is>
       </c>
       <c r="C83" s="105" t="inlineStr">
         <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="D83" s="105" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>The hardest class at usc, but he makes it worth it. Great professor overall - willing to work with students to help with exams and understanding the material. His lectures go by very fast, and his accent can be hard to understand at first. Go to office hours, read the textbook, pay attention and go to every single class...and maybe you'll pass. [Caring, Test heavy, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A84" s="106" t="inlineStr">
+        <is>
+          <t>JS-310</t>
+        </is>
+      </c>
+      <c r="B84" s="107" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="C84" s="107" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D83" s="105" t="inlineStr">
+      <c r="D84" s="107" t="inlineStr">
         <is>
           <t>5/2</t>
         </is>
       </c>
-      <c r="E83" s="8" t="inlineStr">
-        <is>
-          <t>Be prepared to share a little bit in class about the readings - even if you don't read them. The class was fairly easy, involved some in-class reading quizzes and weekly assignments, but nothing too bad. One in-class midterm and take home final. Somewhat approachable, but overall easy grader.</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" hidden="1" outlineLevel="1" ht="75" customHeight="1">
-      <c r="A84" s="107" t="inlineStr"/>
-      <c r="B84" s="107" t="inlineStr">
-        <is>
-          <t>2020-12-16</t>
-        </is>
-      </c>
-      <c r="C84" s="107" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D84" s="107" t="inlineStr">
-        <is>
-          <t>5/4</t>
-        </is>
-      </c>
       <c r="E84" s="11" t="inlineStr">
         <is>
-          <t>hands down one of the best professors in the Spanish department. there's a ton of reading but it's worth it; fantastic curation of books, lectures are brilliant and his dry and subtle sense of humor keeps you engaged and laughing. all around wholesome fun that leaves you wishing covid was over so you could take it in person [Gives good feedback, Get ready to read, Hilarious]</t>
+          <t>Professor Brylak's SLL-310 is one of the best classes you can take for GE credit. Lectures are extremely engaging and based on the weekly readings, which can be a bit dense but are pretty chill as long as you do them consistently. Grades are based on weekly reading quizzes (very easy) and oral presentations that are honestly pretty fun. Take him! [Get ready to read, Hilarious, Caring]</t>
         </is>
       </c>
     </row>
@@ -3264,30 +3382,30 @@
       <c r="A85" s="105" t="inlineStr"/>
       <c r="B85" s="105" t="inlineStr">
         <is>
-          <t>2017-01-11</t>
+          <t>2025-12-03</t>
         </is>
       </c>
       <c r="C85" s="105" t="inlineStr">
         <is>
-          <t>A-</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="D85" s="105" t="inlineStr">
         <is>
-          <t>4/2</t>
+          <t>5/1</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
         <is>
-          <t>He's great and speaks perfect Spanish. He isn't harsh if you don't speak perfectly or know every word. He grades pretty easily and I'm surprised I didn't get a solid A. Overall, would take him again. [GROUP PROJECTS]</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+          <t>I love him; he is truly the best. He is so passionate about what he teaches, and he cares for every single student. I recommend him to ANY and EVERYONE. [Inspirational, Hilarious, Caring]</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" hidden="1" outlineLevel="1" ht="75" customHeight="1">
       <c r="A86" s="107" t="inlineStr"/>
       <c r="B86" s="107" t="inlineStr">
         <is>
-          <t>2016-12-15</t>
+          <t>2024-12-17</t>
         </is>
       </c>
       <c r="C86" s="107" t="inlineStr">
@@ -3297,1369 +3415,1759 @@
       </c>
       <c r="D86" s="107" t="inlineStr">
         <is>
-          <t>5/2</t>
+          <t>4/1</t>
         </is>
       </c>
       <c r="E86" s="11" t="inlineStr">
         <is>
-          <t>A lot of reading (books), but lectures are very interesting. He is well-read and knows a lot of literature. Two papers and one presentation but he's an easy grader. Be prepared to discuss the books. [Get ready to read, Hilarious, Amazing lectures]</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+          <t>Had Prof Brylak for SLL 310! Very funny guy but sometimes goes off on confusing tangents. Weekly reading quizzes are very easy, and you honestly don't really have to do the reading to do the quizzes. Also had 2 pretty long papers, and the instructions those were not very clear. Overall, interesting class and he is very knowledgeable and caring! [Get ready to read, Hilarious]</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" hidden="1" outlineLevel="1" ht="90" customHeight="1">
       <c r="A87" s="105" t="inlineStr"/>
       <c r="B87" s="105" t="inlineStr">
         <is>
+          <t>2024-05-22</t>
+        </is>
+      </c>
+      <c r="C87" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D87" s="105" t="inlineStr">
+        <is>
+          <t>5/1</t>
+        </is>
+      </c>
+      <c r="E87" s="8" t="inlineStr">
+        <is>
+          <t>Cannot recommend prof Brylak more! He is truly an intelligent, caring, and overall amazing teacher. He somehow always has a tidbit of knowledge for whatever tangents we go on and is fantastic at facilitating discussion. He's so engaging, a great presence and I'm very happy I took his class. Assigns ~75-100 pg/week but is a very nice grader! [Get ready to read, Participation matters, Amazing lectures]</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="A88" s="107" t="inlineStr"/>
+      <c r="B88" s="107" t="inlineStr">
+        <is>
+          <t>2024-05-15</t>
+        </is>
+      </c>
+      <c r="C88" s="107" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D88" s="107" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E88" s="11" t="inlineStr">
+        <is>
+          <t>One of my most fun classes in college. Professor Brylak is energetic, hilarious, and very interesting. The assigned reading and videos are usually interesting. Read and watch them so you do not miss out. His assigned papers are vague, but he is not a difficult grader. [Get ready to read, Lots of homework, Hilarious]</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A89" s="105" t="inlineStr"/>
+      <c r="B89" s="105" t="inlineStr">
+        <is>
+          <t>2024-02-13</t>
+        </is>
+      </c>
+      <c r="C89" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D89" s="105" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E89" s="8" t="inlineStr">
+        <is>
+          <t>I cannot love this class more!!! Highly recommended!!! Instead of lecturing by himself, he prepares guiding questions for us to discuss and follow our thoughts to deepen in the direction. He is very knowledgeable to answer all of the unexpected tangent questions. A lot of reading but it's worth it, test and final paper are easy. [Get ready to read, Amazing lectures, Caring]</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A90" s="107" t="inlineStr"/>
+      <c r="B90" s="107" t="inlineStr">
+        <is>
+          <t>2023-11-04</t>
+        </is>
+      </c>
+      <c r="C90" s="107" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="D90" s="107" t="inlineStr">
+        <is>
+          <t>5/1</t>
+        </is>
+      </c>
+      <c r="E90" s="11" t="inlineStr">
+        <is>
+          <t>I took his Easter European Apocalyptic and Post-Apocalyptic Fiction course, and I would highly recommend it. His class is very entertaining and is open to a lot of fun conversation. I had to read around a hundred pages a week and write one page a week, but the weekly papers are graded on completion. [Get ready to read, Amazing lectures, Caring]</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A91" s="105" t="inlineStr"/>
+      <c r="B91" s="105" t="inlineStr">
+        <is>
+          <t>2022-05-21</t>
+        </is>
+      </c>
+      <c r="C91" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D91" s="105" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E91" s="8" t="inlineStr">
+        <is>
+          <t>I really enjoyed Professor Brylak's lectures, they were very interesting and I learned a lot from him. We had to read around 100 pages each week and write a one page response paper, but other than that, he is a very easy grader and it made my seminar experience very chill and fun. Take his gesm even if you have no background on the subject! [Participation matters, Amazing lectures, Caring]</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" hidden="1" outlineLevel="1" ht="30" customHeight="1">
+      <c r="A92" s="107" t="inlineStr"/>
+      <c r="B92" s="107" t="inlineStr">
+        <is>
+          <t>2022-05-13</t>
+        </is>
+      </c>
+      <c r="C92" s="107" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D92" s="107" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E92" s="11" t="inlineStr">
+        <is>
+          <t>Professor Brylak knows his stuff and is a very easy grader. [Amazing lectures, Clear grading criteria, Caring]</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A93" s="105" t="inlineStr"/>
+      <c r="B93" s="105" t="inlineStr">
+        <is>
+          <t>2022-04-28</t>
+        </is>
+      </c>
+      <c r="C93" s="105" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="D93" s="105" t="inlineStr">
+        <is>
+          <t>5/1</t>
+        </is>
+      </c>
+      <c r="E93" s="8" t="inlineStr">
+        <is>
+          <t>The professor is very passionate about the class, so it is very refreshing to see enthusiasm about the topic. The class itself seems very difficult when looking at the name of the class, but it is actually very interesting and easy. Because the professor is an easy grader, I would consider this class stress-free, interesting, and an easy A. [Get ready to read, Respected, Accessible outside class]</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" hidden="1" outlineLevel="1" ht="45" customHeight="1">
+      <c r="A94" s="107" t="inlineStr"/>
+      <c r="B94" s="107" t="inlineStr">
+        <is>
+          <t>2021-12-10</t>
+        </is>
+      </c>
+      <c r="C94" s="107" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D94" s="107" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E94" s="11" t="inlineStr">
+        <is>
+          <t>Great professor! His lectures have a lot of tangents but he's very passionate about the subject so it makes it engaging. A decent amount of reading but easy grading and overall not too much work - a good GESM to take.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" hidden="1" outlineLevel="1" ht="30" customHeight="1">
+      <c r="A95" s="105" t="inlineStr"/>
+      <c r="B95" s="105" t="inlineStr">
+        <is>
+          <t>2021-12-02</t>
+        </is>
+      </c>
+      <c r="C95" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D95" s="105" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E95" s="8" t="inlineStr">
+        <is>
+          <t>Genuinely a sweetheart and loves his classes [Amazing lectures, Lecture heavy, Caring]</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A96" s="104" t="inlineStr">
+        <is>
+          <t>SPAN-290</t>
+        </is>
+      </c>
+      <c r="B96" s="105" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C96" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D96" s="105" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E96" s="8" t="inlineStr">
+        <is>
+          <t>Prof. Steinberg was engaging during lectures. We were assigned 2 readings per week, and I still passed the class by only attending lectures (no reading). If you follow along in class and take good notes, and refer to the slides him and the TAs post, you'll be in for an easy A and learn a ton! [Get ready to read, Amazing lectures, Hilarious]</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="A97" s="107" t="inlineStr"/>
+      <c r="B97" s="107" t="inlineStr">
+        <is>
+          <t>2024-05-18</t>
+        </is>
+      </c>
+      <c r="C97" s="107" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D97" s="107" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E97" s="11" t="inlineStr">
+        <is>
+          <t>Be prepared to share a little bit in class about the readings - even if you don't read them. The class was fairly easy, involved some in-class reading quizzes and weekly assignments, but nothing too bad. One in-class midterm and take home final. Somewhat approachable, but overall easy grader.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" hidden="1" outlineLevel="1" ht="75" customHeight="1">
+      <c r="A98" s="105" t="inlineStr"/>
+      <c r="B98" s="105" t="inlineStr">
+        <is>
+          <t>2020-12-16</t>
+        </is>
+      </c>
+      <c r="C98" s="105" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D98" s="105" t="inlineStr">
+        <is>
+          <t>5/4</t>
+        </is>
+      </c>
+      <c r="E98" s="8" t="inlineStr">
+        <is>
+          <t>hands down one of the best professors in the Spanish department. there's a ton of reading but it's worth it; fantastic curation of books, lectures are brilliant and his dry and subtle sense of humor keeps you engaged and laughing. all around wholesome fun that leaves you wishing covid was over so you could take it in person [Gives good feedback, Get ready to read, Hilarious]</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" hidden="1" outlineLevel="1" ht="45" customHeight="1">
+      <c r="A99" s="107" t="inlineStr"/>
+      <c r="B99" s="107" t="inlineStr">
+        <is>
+          <t>2017-01-11</t>
+        </is>
+      </c>
+      <c r="C99" s="107" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="D99" s="107" t="inlineStr">
+        <is>
+          <t>4/2</t>
+        </is>
+      </c>
+      <c r="E99" s="11" t="inlineStr">
+        <is>
+          <t>He's great and speaks perfect Spanish. He isn't harsh if you don't speak perfectly or know every word. He grades pretty easily and I'm surprised I didn't get a solid A. Overall, would take him again. [GROUP PROJECTS]</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="A100" s="105" t="inlineStr"/>
+      <c r="B100" s="105" t="inlineStr">
+        <is>
+          <t>2016-12-15</t>
+        </is>
+      </c>
+      <c r="C100" s="105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D100" s="105" t="inlineStr">
+        <is>
+          <t>5/2</t>
+        </is>
+      </c>
+      <c r="E100" s="8" t="inlineStr">
+        <is>
+          <t>A lot of reading (books), but lectures are very interesting. He is well-read and knows a lot of literature. Two papers and one presentation but he's an easy grader. Be prepared to discuss the books. [Get ready to read, Hilarious, Amazing lectures]</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="A101" s="107" t="inlineStr"/>
+      <c r="B101" s="107" t="inlineStr">
+        <is>
           <t>2016-04-22</t>
         </is>
       </c>
-      <c r="C87" s="105" t="inlineStr">
+      <c r="C101" s="107" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="D87" s="105" t="inlineStr">
+      <c r="D101" s="107" t="inlineStr">
         <is>
           <t>2/1</t>
         </is>
       </c>
-      <c r="E87" s="8" t="inlineStr">
+      <c r="E101" s="11" t="inlineStr">
         <is>
           <t>Professor Steinberg is an amazing person and instructor he allows you to voice your opinions but also leads you along the way. He assigns alot of reading but it is totally worth it. Lectures are a must and participation is required but the hard work is worth the trouble.</t>
         </is>
       </c>
     </row>
-    <row r="88" hidden="1" outlineLevel="1"/>
-    <row r="89" hidden="1" outlineLevel="1">
-      <c r="A89" s="91" t="inlineStr">
+    <row r="102" hidden="1" outlineLevel="1"/>
+    <row r="103" hidden="1" outlineLevel="1">
+      <c r="A103" s="91" t="inlineStr">
         <is>
           <t>RMP data as of 2026-08-21. Source: ratemyprofessors.com. Avg reviewer grade = mean of self-reported letter grades (4.0 scale); not all reviewers report a grade.</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="28" customHeight="1">
-      <c r="A91" s="4" t="inlineStr">
+    <row r="105" ht="28" customHeight="1">
+      <c r="A105" s="4" t="inlineStr">
         <is>
           <t>Connect prep (e.g. BUAD-304 Personal Assessments) is ungraded class prep - not part of Participation or other graded categories.</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="32" customHeight="1">
-      <c r="A92" s="5" t="inlineStr">
+    <row r="106" ht="32" customHeight="1">
+      <c r="A106" s="5" t="inlineStr">
         <is>
           <t>Start here (graded): 2026-09-04 - ECON-351 - Homework: Homework 1 (Chapter 4) — Brightspace, due 11:59 pm</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="6" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="6" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="B94" s="6" t="inlineStr">
+      <c r="B108" s="6" t="inlineStr">
         <is>
           <t>Reading</t>
         </is>
       </c>
-      <c r="C94" s="6" t="inlineStr">
+      <c r="C108" s="6" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D94" s="6" t="inlineStr">
+      <c r="D108" s="6" t="inlineStr">
         <is>
           <t>Papers</t>
         </is>
       </c>
-      <c r="E94" s="6" t="inlineStr">
+      <c r="E108" s="6" t="inlineStr">
         <is>
           <t>Group Project</t>
         </is>
       </c>
-      <c r="F94" s="6" t="inlineStr">
+      <c r="F108" s="6" t="inlineStr">
         <is>
           <t>External certs</t>
         </is>
       </c>
-      <c r="G94" s="6" t="inlineStr">
+      <c r="G108" s="6" t="inlineStr">
         <is>
           <t>Connect prep</t>
         </is>
       </c>
-      <c r="H94" s="6" t="inlineStr">
+      <c r="H108" s="6" t="inlineStr">
         <is>
           <t>First assignment</t>
         </is>
       </c>
-      <c r="I94" s="6" t="inlineStr">
+      <c r="I108" s="6" t="inlineStr">
         <is>
           <t>Assign due</t>
         </is>
       </c>
-      <c r="J94" s="6" t="inlineStr">
+      <c r="J108" s="6" t="inlineStr">
         <is>
           <t>First major</t>
         </is>
       </c>
-      <c r="K94" s="6" t="inlineStr">
+      <c r="K108" s="6" t="inlineStr">
         <is>
           <t>Major due</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="7">
+    <row r="109">
+      <c r="A109" s="7">
         <f>HYPERLINK("#'BUAD-281'!A1","BUAD-281")</f>
         <v/>
       </c>
-      <c r="B95" s="8" t="inlineStr">
+      <c r="B109" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C95" s="8" t="inlineStr">
+      <c r="C109" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D95" s="8" t="inlineStr">
+      <c r="D109" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E95" s="8" t="inlineStr">
+      <c r="E109" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F95" s="9" t="inlineStr">
+      <c r="F109" s="9" t="inlineStr">
         <is>
           <t>LinkedIn Learning Excel Certification, Stukent Simternship</t>
         </is>
       </c>
-      <c r="G95" s="8" t="inlineStr">
+      <c r="G109" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H95" s="8" t="inlineStr">
+      <c r="H109" s="8" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
         </is>
       </c>
-      <c r="I95" s="8" t="inlineStr">
+      <c r="I109" s="8" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="J95" s="8" t="inlineStr">
+      <c r="J109" s="8" t="inlineStr">
         <is>
           <t>Midterm 1</t>
         </is>
       </c>
-      <c r="K95" s="8" t="inlineStr">
+      <c r="K109" s="8" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="10">
+    <row r="110">
+      <c r="A110" s="10">
         <f>HYPERLINK("#'BUAD-304'!A1","BUAD-304")</f>
         <v/>
       </c>
-      <c r="B96" s="11" t="inlineStr">
+      <c r="B110" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C96" s="11" t="inlineStr">
+      <c r="C110" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D96" s="11" t="inlineStr">
+      <c r="D110" s="11" t="inlineStr">
         <is>
           <t>Final Reflection Paper, Team Project Paper</t>
         </is>
       </c>
-      <c r="E96" s="11" t="inlineStr">
+      <c r="E110" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F96" s="11" t="inlineStr">
+      <c r="F110" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G96" s="12" t="inlineStr">
+      <c r="G110" s="12" t="inlineStr">
         <is>
           <t>Ungraded prep</t>
         </is>
       </c>
-      <c r="H96" s="11" t="inlineStr">
+      <c r="H110" s="11" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.01 - What is my Big thinking</t>
         </is>
       </c>
-      <c r="I96" s="11" t="inlineStr">
+      <c r="I110" s="11" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="J96" s="11" t="inlineStr">
+      <c r="J110" s="11" t="inlineStr">
         <is>
           <t>Thomas Green Case Analysis Memo</t>
         </is>
       </c>
-      <c r="K96" s="11" t="inlineStr">
+      <c r="K110" s="11" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="7">
+    <row r="111">
+      <c r="A111" s="7">
         <f>HYPERLINK("#'ECON-351'!A1","ECON-351")</f>
         <v/>
       </c>
-      <c r="B97" s="8" t="inlineStr">
+      <c r="B111" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C97" s="8" t="inlineStr">
+      <c r="C111" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D97" s="8" t="inlineStr">
+      <c r="D111" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E97" s="8" t="inlineStr">
+      <c r="E111" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F97" s="8" t="inlineStr">
+      <c r="F111" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G97" s="8" t="inlineStr">
+      <c r="G111" s="8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H97" s="8" t="inlineStr">
+      <c r="H111" s="8" t="inlineStr">
         <is>
           <t>Homework 1 (Chapter 4) — Brightspace, due 11:59 pm</t>
         </is>
       </c>
-      <c r="I97" s="8" t="inlineStr">
+      <c r="I111" s="8" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="J97" s="8" t="inlineStr">
+      <c r="J111" s="8" t="inlineStr">
         <is>
           <t>First midterm exam</t>
         </is>
       </c>
-      <c r="K97" s="8" t="inlineStr">
+      <c r="K111" s="8" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="10">
+    <row r="112">
+      <c r="A112" s="10">
         <f>HYPERLINK("#'HIST-103'!A1","HIST-103")</f>
         <v/>
       </c>
-      <c r="B98" s="11" t="inlineStr">
+      <c r="B112" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C98" s="11" t="inlineStr">
+      <c r="C112" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D98" s="11" t="inlineStr">
+      <c r="D112" s="11" t="inlineStr">
         <is>
           <t>Sleep Paper, Witchcraft Paper</t>
         </is>
       </c>
-      <c r="E98" s="11" t="inlineStr">
+      <c r="E112" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F98" s="11" t="inlineStr">
+      <c r="F112" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G98" s="11" t="inlineStr">
+      <c r="G112" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H98" s="11" t="inlineStr">
+      <c r="H112" s="11" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
         </is>
       </c>
-      <c r="I98" s="11" t="inlineStr">
+      <c r="I112" s="11" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="J98" s="11" t="inlineStr">
+      <c r="J112" s="11" t="inlineStr">
         <is>
           <t>Sleep Paper</t>
         </is>
       </c>
-      <c r="K98" s="11" t="inlineStr">
+      <c r="K112" s="11" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="7">
+    <row r="113">
+      <c r="A113" s="7">
+        <f>HYPERLINK("#'JS-310'!A1","JS-310")</f>
+        <v/>
+      </c>
+      <c r="B113" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C113" s="8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D113" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E113" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F113" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G113" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H113" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I113" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J113" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K113" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="10">
         <f>HYPERLINK("#'SPAN-290'!A1","SPAN-290")</f>
         <v/>
       </c>
-      <c r="B99" s="8" t="inlineStr">
+      <c r="B114" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C99" s="8" t="inlineStr">
+      <c r="C114" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D99" s="8" t="inlineStr">
+      <c r="D114" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E99" s="8" t="inlineStr">
+      <c r="E114" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F99" s="8" t="inlineStr">
+      <c r="F114" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G99" s="8" t="inlineStr">
+      <c r="G114" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H99" s="8" t="inlineStr">
+      <c r="H114" s="11" t="inlineStr">
         <is>
           <t>Essay 1</t>
         </is>
       </c>
-      <c r="I99" s="8" t="inlineStr">
+      <c r="I114" s="11" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="J99" s="8" t="inlineStr">
+      <c r="J114" s="11" t="inlineStr">
         <is>
           <t>Essay 1</t>
         </is>
       </c>
-      <c r="K99" s="8" t="inlineStr">
+      <c r="K114" s="11" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="13" t="inlineStr">
+    <row r="116">
+      <c r="A116" s="13" t="inlineStr">
         <is>
           <t>Do First - August 2026 - graded assignments (first per class always listed)</t>
         </is>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="14" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="14" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="B102" s="14" t="inlineStr">
+      <c r="B117" s="14" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="C102" s="14" t="inlineStr">
+      <c r="C117" s="14" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D102" s="14" t="inlineStr">
+      <c r="D117" s="14" t="inlineStr">
         <is>
           <t>Graded?</t>
         </is>
       </c>
-      <c r="E102" s="14" t="inlineStr">
+      <c r="E117" s="14" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="8" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="8" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="B103" s="8" t="inlineStr">
+      <c r="B118" s="8" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="C103" s="15" t="inlineStr">
+      <c r="C118" s="15" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D103" s="8" t="inlineStr">
+      <c r="D118" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E103" s="8" t="inlineStr">
+      <c r="E118" s="8" t="inlineStr">
         <is>
           <t>Homework 1 (Chapter 4) — Brightspace, due 11:59 pm</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="11" t="inlineStr">
+    <row r="119">
+      <c r="A119" s="11" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="B104" s="11" t="inlineStr">
+      <c r="B119" s="11" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C104" s="46" t="inlineStr">
+      <c r="C119" s="46" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D104" s="11" t="inlineStr">
+      <c r="D119" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E104" s="11" t="inlineStr">
+      <c r="E119" s="11" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="8" t="inlineStr">
+    <row r="120">
+      <c r="A120" s="8" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="B105" s="8" t="inlineStr">
+      <c r="B120" s="8" t="inlineStr">
         <is>
           <t>HIST-103</t>
         </is>
       </c>
-      <c r="C105" s="25" t="inlineStr">
+      <c r="C120" s="25" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D105" s="8" t="inlineStr">
+      <c r="D120" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E105" s="8" t="inlineStr">
+      <c r="E120" s="8" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="11" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="11" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="B106" s="11" t="inlineStr">
+      <c r="B121" s="11" t="inlineStr">
         <is>
           <t>SPAN-290</t>
         </is>
       </c>
-      <c r="C106" s="16" t="inlineStr">
+      <c r="C121" s="16" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D106" s="11" t="inlineStr">
+      <c r="D121" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E106" s="11" t="inlineStr">
+      <c r="E121" s="11" t="inlineStr">
         <is>
           <t>Essay 1</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" s="17" t="inlineStr">
+    <row r="123">
+      <c r="A123" s="17" t="inlineStr">
         <is>
           <t>Do First - August 2026 - Connect prep only (ungraded, not Participation)</t>
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" s="18" t="inlineStr">
+    <row r="124">
+      <c r="A124" s="18" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="B109" s="18" t="inlineStr">
+      <c r="B124" s="18" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="C109" s="18" t="inlineStr">
+      <c r="C124" s="18" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D109" s="18" t="inlineStr">
+      <c r="D124" s="18" t="inlineStr">
         <is>
           <t>Graded?</t>
         </is>
       </c>
-      <c r="E109" s="18" t="inlineStr">
+      <c r="E124" s="18" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" s="19" t="inlineStr">
+    <row r="125">
+      <c r="A125" s="19" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B110" s="19" t="inlineStr">
+      <c r="B125" s="19" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C110" s="20" t="inlineStr">
+      <c r="C125" s="20" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D110" s="21" t="inlineStr">
+      <c r="D125" s="21" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E110" s="19" t="inlineStr">
+      <c r="E125" s="19" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
         </is>
       </c>
     </row>
-    <row r="111">
-      <c r="A111" s="22" t="inlineStr">
+    <row r="126">
+      <c r="A126" s="22" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B111" s="22" t="inlineStr">
+      <c r="B126" s="22" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C111" s="23" t="inlineStr">
+      <c r="C126" s="23" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D111" s="24" t="inlineStr">
+      <c r="D126" s="24" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E111" s="22" t="inlineStr">
+      <c r="E126" s="22" t="inlineStr">
         <is>
           <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" s="13" t="inlineStr">
+    <row r="128">
+      <c r="A128" s="13" t="inlineStr">
         <is>
           <t>Upcoming graded assignments (next 45 days)</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="14" t="inlineStr">
+    <row r="129">
+      <c r="A129" s="14" t="inlineStr">
         <is>
           <t>Due</t>
         </is>
       </c>
-      <c r="B114" s="14" t="inlineStr">
+      <c r="B129" s="14" t="inlineStr">
         <is>
           <t>Class</t>
         </is>
       </c>
-      <c r="C114" s="14" t="inlineStr">
+      <c r="C129" s="14" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="D114" s="14" t="inlineStr">
+      <c r="D129" s="14" t="inlineStr">
         <is>
           <t>Graded?</t>
         </is>
       </c>
-      <c r="E114" s="14" t="inlineStr">
+      <c r="E129" s="14" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" s="8" t="inlineStr">
+    <row r="130">
+      <c r="A130" s="8" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>
       </c>
-      <c r="B115" s="8" t="inlineStr">
+      <c r="B130" s="8" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="C115" s="15" t="inlineStr">
+      <c r="C130" s="15" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D115" s="8" t="inlineStr">
+      <c r="D130" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E115" s="8" t="inlineStr">
+      <c r="E130" s="8" t="inlineStr">
         <is>
           <t>Homework 1 (Chapter 4) — Brightspace, due 11:59 pm</t>
         </is>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" s="11" t="inlineStr">
+    <row r="131">
+      <c r="A131" s="11" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="B116" s="11" t="inlineStr">
+      <c r="B131" s="11" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C116" s="46" t="inlineStr">
+      <c r="C131" s="46" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D116" s="11" t="inlineStr">
+      <c r="D131" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E116" s="11" t="inlineStr">
+      <c r="E131" s="11" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
         </is>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" s="8" t="inlineStr">
+    <row r="132">
+      <c r="A132" s="8" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="B117" s="8" t="inlineStr">
+      <c r="B132" s="8" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="C117" s="15" t="inlineStr">
+      <c r="C132" s="15" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D117" s="8" t="inlineStr">
+      <c r="D132" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E117" s="8" t="inlineStr">
+      <c r="E132" s="8" t="inlineStr">
         <is>
           <t>Homework 2 (Chapter 9) — Brightspace, due 11:59 pm</t>
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" s="11" t="inlineStr">
+    <row r="133">
+      <c r="A133" s="11" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="B118" s="11" t="inlineStr">
+      <c r="B133" s="11" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="C118" s="120" t="inlineStr">
+      <c r="C133" s="120" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="D118" s="11" t="inlineStr">
+      <c r="D133" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E118" s="11" t="inlineStr">
+      <c r="E133" s="11" t="inlineStr">
         <is>
           <t>Midterm 1 — covers Chapters 4 and 9</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="8" t="inlineStr">
+    <row r="134">
+      <c r="A134" s="8" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="B119" s="8" t="inlineStr">
+      <c r="B134" s="8" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="C119" s="25" t="inlineStr">
+      <c r="C134" s="25" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D119" s="8" t="inlineStr">
+      <c r="D134" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E119" s="8" t="inlineStr">
+      <c r="E134" s="8" t="inlineStr">
         <is>
           <t>First midterm exam</t>
         </is>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" s="11" t="inlineStr">
+    <row r="135">
+      <c r="A135" s="11" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="B120" s="11" t="inlineStr">
+      <c r="B135" s="11" t="inlineStr">
         <is>
           <t>HIST-103</t>
         </is>
       </c>
-      <c r="C120" s="16" t="inlineStr">
+      <c r="C135" s="16" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D120" s="11" t="inlineStr">
+      <c r="D135" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E120" s="11" t="inlineStr">
+      <c r="E135" s="11" t="inlineStr">
         <is>
           <t>Sleep Paper Due</t>
         </is>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" s="8" t="inlineStr">
+    <row r="136">
+      <c r="A136" s="8" t="inlineStr">
         <is>
           <t>2026-09-15</t>
         </is>
       </c>
-      <c r="B121" s="8" t="inlineStr">
+      <c r="B136" s="8" t="inlineStr">
         <is>
           <t>HIST-103</t>
         </is>
       </c>
-      <c r="C121" s="25" t="inlineStr">
+      <c r="C136" s="25" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D121" s="8" t="inlineStr">
+      <c r="D136" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E121" s="8" t="inlineStr">
+      <c r="E136" s="8" t="inlineStr">
         <is>
           <t>Sleep Paper</t>
         </is>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" s="11" t="inlineStr">
+    <row r="137">
+      <c r="A137" s="11" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="B122" s="11" t="inlineStr">
+      <c r="B137" s="11" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C122" s="46" t="inlineStr">
+      <c r="C137" s="46" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D122" s="11" t="inlineStr">
+      <c r="D137" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E122" s="11" t="inlineStr">
+      <c r="E137" s="11" t="inlineStr">
         <is>
           <t>Class 7 (9/16) - 3-24, 3-28, 3-32; 15 Points</t>
         </is>
       </c>
     </row>
-    <row r="123">
-      <c r="A123" s="8" t="inlineStr">
+    <row r="138">
+      <c r="A138" s="8" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="B123" s="8" t="inlineStr">
+      <c r="B138" s="8" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C123" s="25" t="inlineStr">
+      <c r="C138" s="25" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D123" s="8" t="inlineStr">
+      <c r="D138" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E123" s="8" t="inlineStr">
+      <c r="E138" s="8" t="inlineStr">
         <is>
           <t>Thomas Green Case Analysis Memo</t>
         </is>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" s="11" t="inlineStr">
+    <row r="139">
+      <c r="A139" s="11" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>
       </c>
-      <c r="B124" s="11" t="inlineStr">
+      <c r="B139" s="11" t="inlineStr">
         <is>
           <t>HIST-103</t>
         </is>
       </c>
-      <c r="C124" s="16" t="inlineStr">
+      <c r="C139" s="16" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D124" s="11" t="inlineStr">
+      <c r="D139" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E124" s="11" t="inlineStr">
+      <c r="E139" s="11" t="inlineStr">
         <is>
           <t>Final Exam</t>
         </is>
       </c>
     </row>
-    <row r="125">
-      <c r="A125" s="8" t="inlineStr">
+    <row r="140">
+      <c r="A140" s="8" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="B125" s="8" t="inlineStr">
+      <c r="B140" s="8" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="C125" s="15" t="inlineStr">
+      <c r="C140" s="15" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D125" s="8" t="inlineStr">
+      <c r="D140" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E125" s="8" t="inlineStr">
+      <c r="E140" s="8" t="inlineStr">
         <is>
           <t>Homework 3 — Brightspace, due 11:59 pm</t>
         </is>
       </c>
     </row>
-    <row r="126">
-      <c r="A126" s="11" t="inlineStr">
+    <row r="141">
+      <c r="A141" s="11" t="inlineStr">
         <is>
           <t>2026-09-18</t>
         </is>
       </c>
-      <c r="B126" s="11" t="inlineStr">
+      <c r="B141" s="11" t="inlineStr">
         <is>
           <t>SPAN-290</t>
         </is>
       </c>
-      <c r="C126" s="16" t="inlineStr">
+      <c r="C141" s="16" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D126" s="11" t="inlineStr">
+      <c r="D141" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E126" s="11" t="inlineStr">
+      <c r="E141" s="11" t="inlineStr">
         <is>
           <t>Essay 1</t>
         </is>
       </c>
     </row>
-    <row r="127">
-      <c r="A127" s="8" t="inlineStr">
+    <row r="142">
+      <c r="A142" s="8" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="B127" s="8" t="inlineStr">
+      <c r="B142" s="8" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C127" s="15" t="inlineStr">
+      <c r="C142" s="15" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D127" s="8" t="inlineStr">
+      <c r="D142" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E127" s="8" t="inlineStr">
+      <c r="E142" s="8" t="inlineStr">
         <is>
           <t>Class 8 (9/21) - 5-27 5-46; 10 Points</t>
         </is>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" s="11" t="inlineStr">
+    <row r="143">
+      <c r="A143" s="11" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="B128" s="11" t="inlineStr">
+      <c r="B143" s="11" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C128" s="46" t="inlineStr">
+      <c r="C143" s="46" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D128" s="11" t="inlineStr">
+      <c r="D143" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E128" s="11" t="inlineStr">
+      <c r="E143" s="11" t="inlineStr">
         <is>
           <t>Class 9 (9/23) - 4-21, 4-22; 10 Points</t>
         </is>
       </c>
     </row>
-    <row r="129">
-      <c r="A129" s="8" t="inlineStr">
+    <row r="144">
+      <c r="A144" s="8" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="B129" s="8" t="inlineStr">
+      <c r="B144" s="8" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="C129" s="15" t="inlineStr">
+      <c r="C144" s="15" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D129" s="8" t="inlineStr">
+      <c r="D144" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E129" s="8" t="inlineStr">
+      <c r="E144" s="8" t="inlineStr">
         <is>
           <t>Homework 4 (Chapter 3) — Brightspace, due 11:59 pm</t>
         </is>
       </c>
     </row>
-    <row r="130">
-      <c r="A130" s="11" t="inlineStr">
+    <row r="145">
+      <c r="A145" s="11" t="inlineStr">
         <is>
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="B130" s="11" t="inlineStr">
+      <c r="B145" s="11" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C130" s="90" t="inlineStr">
+      <c r="C145" s="90" t="inlineStr">
         <is>
           <t>Research</t>
         </is>
       </c>
-      <c r="D130" s="11" t="inlineStr">
+      <c r="D145" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E130" s="11" t="inlineStr">
+      <c r="E145" s="11" t="inlineStr">
         <is>
           <t>Research: Setup deadline (registration, prescreening, contacts)</t>
         </is>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" s="8" t="inlineStr">
+    <row r="146">
+      <c r="A146" s="8" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="B131" s="8" t="inlineStr">
+      <c r="B146" s="8" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C131" s="15" t="inlineStr">
+      <c r="C146" s="15" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D131" s="8" t="inlineStr">
+      <c r="D146" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E131" s="8" t="inlineStr">
+      <c r="E146" s="8" t="inlineStr">
         <is>
           <t>Class 10 (9/28) - 8-28, 8-29; 10 Points</t>
         </is>
       </c>
     </row>
-    <row r="132">
-      <c r="A132" s="11" t="inlineStr">
+    <row r="147">
+      <c r="A147" s="11" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="B132" s="11" t="inlineStr">
+      <c r="B147" s="11" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C132" s="16" t="inlineStr">
+      <c r="C147" s="16" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D132" s="11" t="inlineStr">
+      <c r="D147" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E132" s="11" t="inlineStr">
+      <c r="E147" s="11" t="inlineStr">
         <is>
           <t>Team project proposal &amp; team contract</t>
         </is>
       </c>
     </row>
-    <row r="133">
-      <c r="A133" s="8" t="inlineStr">
+    <row r="148">
+      <c r="A148" s="8" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="B133" s="8" t="inlineStr">
+      <c r="B148" s="8" t="inlineStr">
         <is>
           <t>BUAD-304</t>
         </is>
       </c>
-      <c r="C133" s="25" t="inlineStr">
+      <c r="C148" s="25" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D133" s="8" t="inlineStr">
+      <c r="D148" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E133" s="8" t="inlineStr">
+      <c r="E148" s="8" t="inlineStr">
         <is>
           <t>Proposal &amp; Team Contract</t>
         </is>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" s="11" t="inlineStr">
+    <row r="149">
+      <c r="A149" s="11" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B134" s="11" t="inlineStr">
+      <c r="B149" s="11" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C134" s="120" t="inlineStr">
+      <c r="C149" s="120" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="D134" s="11" t="inlineStr">
+      <c r="D149" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E134" s="11" t="inlineStr">
+      <c r="E149" s="11" t="inlineStr">
         <is>
           <t>9/30 Midterm 1: 250 Points Chapters 1, 2, 3, 4, 5, 8</t>
         </is>
       </c>
     </row>
-    <row r="135">
-      <c r="A135" s="8" t="inlineStr">
+    <row r="150">
+      <c r="A150" s="8" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B135" s="8" t="inlineStr">
+      <c r="B150" s="8" t="inlineStr">
         <is>
           <t>BUAD-281</t>
         </is>
       </c>
-      <c r="C135" s="25" t="inlineStr">
+      <c r="C150" s="25" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D135" s="8" t="inlineStr">
+      <c r="D150" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E135" s="8" t="inlineStr">
+      <c r="E150" s="8" t="inlineStr">
         <is>
           <t>Midterm 1</t>
         </is>
       </c>
     </row>
-    <row r="136">
-      <c r="A136" s="11" t="inlineStr">
+    <row r="151">
+      <c r="A151" s="11" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="B136" s="11" t="inlineStr">
+      <c r="B151" s="11" t="inlineStr">
         <is>
           <t>SPAN-290</t>
         </is>
       </c>
-      <c r="C136" s="120" t="inlineStr">
+      <c r="C151" s="120" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="D136" s="11" t="inlineStr">
+      <c r="D151" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E136" s="11" t="inlineStr">
+      <c r="E151" s="11" t="inlineStr">
         <is>
           <t>Midterm Exam (in class)</t>
         </is>
       </c>
     </row>
-    <row r="137">
-      <c r="A137" s="8" t="inlineStr">
+    <row r="152">
+      <c r="A152" s="8" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="B137" s="8" t="inlineStr">
+      <c r="B152" s="8" t="inlineStr">
         <is>
           <t>SPAN-290</t>
         </is>
       </c>
-      <c r="C137" s="25" t="inlineStr">
+      <c r="C152" s="25" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D137" s="8" t="inlineStr">
+      <c r="D152" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E137" s="8" t="inlineStr">
+      <c r="E152" s="8" t="inlineStr">
         <is>
           <t>Midterm Exam</t>
         </is>
       </c>
     </row>
-    <row r="138">
-      <c r="A138" s="11" t="inlineStr">
+    <row r="153">
+      <c r="A153" s="11" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B138" s="11" t="inlineStr">
+      <c r="B153" s="11" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="C138" s="46" t="inlineStr">
+      <c r="C153" s="46" t="inlineStr">
         <is>
           <t>Homework</t>
         </is>
       </c>
-      <c r="D138" s="11" t="inlineStr">
+      <c r="D153" s="11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E138" s="11" t="inlineStr">
+      <c r="E153" s="11" t="inlineStr">
         <is>
           <t>Homework 5 (Chapter 5) — Brightspace, due 11:59 pm</t>
         </is>
       </c>
     </row>
-    <row r="139">
-      <c r="A139" s="8" t="inlineStr">
+    <row r="154">
+      <c r="A154" s="8" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="B139" s="8" t="inlineStr">
+      <c r="B154" s="8" t="inlineStr">
         <is>
           <t>ECON-351</t>
         </is>
       </c>
-      <c r="C139" s="25" t="inlineStr">
+      <c r="C154" s="25" t="inlineStr">
         <is>
           <t>Assignment</t>
         </is>
       </c>
-      <c r="D139" s="8" t="inlineStr">
+      <c r="D154" s="8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E139" s="8" t="inlineStr">
+      <c r="E154" s="8" t="inlineStr">
         <is>
           <t>AI Forecast Project — Part I</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="84">
+  <mergeCells count="97">
     <mergeCell ref="E36:K36"/>
+    <mergeCell ref="E101:K101"/>
+    <mergeCell ref="E91:K91"/>
     <mergeCell ref="E85:K85"/>
+    <mergeCell ref="E100:K100"/>
     <mergeCell ref="E75:K75"/>
-    <mergeCell ref="E22:K22"/>
     <mergeCell ref="E53:K53"/>
+    <mergeCell ref="E93:K93"/>
     <mergeCell ref="C17:K17"/>
     <mergeCell ref="E55:K55"/>
-    <mergeCell ref="A108:K108"/>
     <mergeCell ref="E67:K67"/>
     <mergeCell ref="E39:K39"/>
     <mergeCell ref="E48:K48"/>
-    <mergeCell ref="A101:K101"/>
+    <mergeCell ref="C19:K19"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="E29:K29"/>
     <mergeCell ref="E38:K38"/>
     <mergeCell ref="E31:K31"/>
     <mergeCell ref="E40:K40"/>
     <mergeCell ref="C14:K14"/>
-    <mergeCell ref="A19:K19"/>
+    <mergeCell ref="E95:K95"/>
+    <mergeCell ref="E89:K89"/>
     <mergeCell ref="E26:K26"/>
     <mergeCell ref="E76:K76"/>
     <mergeCell ref="E25:K25"/>
     <mergeCell ref="E66:K66"/>
     <mergeCell ref="E58:K58"/>
+    <mergeCell ref="A128:K128"/>
     <mergeCell ref="E50:K50"/>
     <mergeCell ref="E68:K68"/>
     <mergeCell ref="E42:K42"/>
+    <mergeCell ref="A105:K105"/>
     <mergeCell ref="E52:K52"/>
     <mergeCell ref="E83:K83"/>
+    <mergeCell ref="E92:K92"/>
     <mergeCell ref="E44:K44"/>
-    <mergeCell ref="A91:K91"/>
+    <mergeCell ref="C18:K18"/>
+    <mergeCell ref="A116:K116"/>
+    <mergeCell ref="E94:K94"/>
     <mergeCell ref="E69:K69"/>
     <mergeCell ref="E84:K84"/>
     <mergeCell ref="E78:K78"/>
@@ -4670,7 +5178,6 @@
     <mergeCell ref="E86:K86"/>
     <mergeCell ref="E80:K80"/>
     <mergeCell ref="E61:K61"/>
-    <mergeCell ref="A92:K92"/>
     <mergeCell ref="E70:K70"/>
     <mergeCell ref="E57:K57"/>
     <mergeCell ref="E54:K54"/>
@@ -4679,31 +5186,34 @@
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="E41:K41"/>
     <mergeCell ref="E81:K81"/>
+    <mergeCell ref="A103:K103"/>
     <mergeCell ref="E47:K47"/>
     <mergeCell ref="E56:K56"/>
+    <mergeCell ref="E96:K96"/>
     <mergeCell ref="E43:K43"/>
     <mergeCell ref="E24:K24"/>
     <mergeCell ref="E33:K33"/>
-    <mergeCell ref="A89:K89"/>
-    <mergeCell ref="A12:K12"/>
+    <mergeCell ref="E98:K98"/>
+    <mergeCell ref="A21:K21"/>
+    <mergeCell ref="E88:K88"/>
     <mergeCell ref="E82:K82"/>
-    <mergeCell ref="A113:K113"/>
     <mergeCell ref="E35:K35"/>
+    <mergeCell ref="A106:K106"/>
     <mergeCell ref="E28:K28"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="E60:K60"/>
     <mergeCell ref="E74:K74"/>
     <mergeCell ref="E45:K45"/>
     <mergeCell ref="C16:K16"/>
+    <mergeCell ref="A123:K123"/>
     <mergeCell ref="E37:K37"/>
-    <mergeCell ref="E21:K21"/>
+    <mergeCell ref="E97:K97"/>
     <mergeCell ref="E62:K62"/>
     <mergeCell ref="E71:K71"/>
     <mergeCell ref="E23:K23"/>
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="E64:K64"/>
     <mergeCell ref="E79:K79"/>
-    <mergeCell ref="C13:K13"/>
     <mergeCell ref="E73:K73"/>
     <mergeCell ref="E51:K51"/>
     <mergeCell ref="E87:K87"/>
@@ -4711,6 +5221,9 @@
     <mergeCell ref="C15:K15"/>
     <mergeCell ref="E65:K65"/>
     <mergeCell ref="E34:K34"/>
+    <mergeCell ref="E90:K90"/>
+    <mergeCell ref="E99:K99"/>
+    <mergeCell ref="A13:K13"/>
     <mergeCell ref="E49:K49"/>
     <mergeCell ref="E27:K27"/>
   </mergeCells>
@@ -4720,6 +5233,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10171,4 +10685,564 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="008C564B"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="194" t="inlineStr">
+        <is>
+          <t>JS-310 — The Eastern European Jewish Experience through Literature and Film</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="28">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/sources/js-310-source.pdf","SEE HERE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="29" t="inlineStr">
+        <is>
+          <t>Instructor</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Andrzej Brylak / Yulia Dubasova</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fall 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>Required for an A</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>90% (90-100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>Grading scale</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>A – 90 – 100% B – 80 – 89% C – 70 – 79% D – 60 – 69% F – Below 60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="195" t="inlineStr">
+        <is>
+          <t>Weekly Quizzes 30%  |  Midterm Oral Exam 20%  |  Final Oral Exam 20%  |  Midterm Quiz 15%  |  Final Quiz 15%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="196" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B9" s="196" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="C9" s="196" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="D9" s="196" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="E9" s="196" t="inlineStr">
+        <is>
+          <t>Group Project</t>
+        </is>
+      </c>
+      <c r="F9" s="196" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="197" t="inlineStr">
+        <is>
+          <t>Weekly Quizzes</t>
+        </is>
+      </c>
+      <c r="B10" s="214" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="C10" s="215" t="inlineStr"/>
+      <c r="D10" s="215" t="inlineStr"/>
+      <c r="E10" s="215" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F10" s="200">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/js-310-weekly-quizzes.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="201" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B11" s="216" t="inlineStr"/>
+      <c r="C11" s="216" t="inlineStr"/>
+      <c r="D11" s="216" t="inlineStr"/>
+      <c r="E11" s="216" t="inlineStr"/>
+      <c r="F11" s="203" t="inlineStr">
+        <is>
+          <t>Week 1 — Eastern European Jewish Experience: Historical Introduction — (Text on Brightspace); Antony Polonsky, Jews in P</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="201" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B12" s="216" t="inlineStr"/>
+      <c r="C12" s="216" t="inlineStr"/>
+      <c r="D12" s="216" t="inlineStr"/>
+      <c r="E12" s="216" t="inlineStr"/>
+      <c r="F12" s="203" t="inlineStr">
+        <is>
+          <t>Week 10 — Irony in Holocaust Literature — Imre Kertesz, Fatelessness, pp. 99-189</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="201" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B13" s="216" t="inlineStr"/>
+      <c r="C13" s="216" t="inlineStr"/>
+      <c r="D13" s="216" t="inlineStr"/>
+      <c r="E13" s="216" t="inlineStr"/>
+      <c r="F13" s="203" t="inlineStr">
+        <is>
+          <t>Week 11 — Testimony as a Genre. Ethics and Poetics. — Imre Kertesz, Fatelessness, pp. 189- 262; Film: Everything is Illu</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="201" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B14" s="216" t="inlineStr"/>
+      <c r="C14" s="216" t="inlineStr"/>
+      <c r="D14" s="216" t="inlineStr"/>
+      <c r="E14" s="216" t="inlineStr"/>
+      <c r="F14" s="203" t="inlineStr">
+        <is>
+          <t>Week 12 — Jewish American Literature — Gary Shteyngart, Super Sad True Love Story, pp. 1- 98</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="201" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B15" s="216" t="inlineStr"/>
+      <c r="C15" s="216" t="inlineStr"/>
+      <c r="D15" s="216" t="inlineStr"/>
+      <c r="E15" s="216" t="inlineStr"/>
+      <c r="F15" s="203" t="inlineStr">
+        <is>
+          <t>Week 13 — Eastern European Influence on Contemporary Jewish Identity i — Gary Shteyngart, Super Sad True Love Story, pp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="201" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B16" s="216" t="inlineStr"/>
+      <c r="C16" s="216" t="inlineStr"/>
+      <c r="D16" s="216" t="inlineStr"/>
+      <c r="E16" s="216" t="inlineStr"/>
+      <c r="F16" s="203" t="inlineStr">
+        <is>
+          <t>Week 14 — Jewishness and Postmodernism — Gary Shteyngart, Super Sad True Love Story, pp. 203- 330</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="201" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B17" s="216" t="inlineStr"/>
+      <c r="C17" s="216" t="inlineStr"/>
+      <c r="D17" s="216" t="inlineStr"/>
+      <c r="E17" s="216" t="inlineStr"/>
+      <c r="F17" s="203" t="inlineStr">
+        <is>
+          <t>Week 14 — Jews and Money — Film: Uncut Gems, dir. Safdie Brothers</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="201" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B18" s="216" t="inlineStr"/>
+      <c r="C18" s="216" t="inlineStr"/>
+      <c r="D18" s="216" t="inlineStr"/>
+      <c r="E18" s="216" t="inlineStr"/>
+      <c r="F18" s="203" t="inlineStr">
+        <is>
+          <t>Week 2 — Small Town Jewish Life — Sholem Aleichem, Tevye the Dairyman and Motl the Cantor’s Son, pp. 1-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="201" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B19" s="216" t="inlineStr"/>
+      <c r="C19" s="216" t="inlineStr"/>
+      <c r="D19" s="216" t="inlineStr"/>
+      <c r="E19" s="216" t="inlineStr"/>
+      <c r="F19" s="203" t="inlineStr">
+        <is>
+          <t>Week 3 — Tradition vs Modernity — Sholem Aleichem, Tevye the Dairyman and Motl the Cantor’s Son, pp. 135</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="201" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B20" s="216" t="inlineStr"/>
+      <c r="C20" s="216" t="inlineStr"/>
+      <c r="D20" s="216" t="inlineStr"/>
+      <c r="E20" s="216" t="inlineStr"/>
+      <c r="F20" s="203" t="inlineStr">
+        <is>
+          <t>Week 4 — Jewish Emigration — Sholem Aleichem, Tevye the Dairyman and Motl the Cantor’s Son, pp. 235</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="201" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B21" s="216" t="inlineStr"/>
+      <c r="C21" s="216" t="inlineStr"/>
+      <c r="D21" s="216" t="inlineStr"/>
+      <c r="E21" s="216" t="inlineStr"/>
+      <c r="F21" s="203" t="inlineStr">
+        <is>
+          <t>Week 5 — Americanization — Sholem Aleichem, Tevye the Dairyman and Motl the Cantor’s Son, pp. 281</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="201" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B22" s="216" t="inlineStr"/>
+      <c r="C22" s="216" t="inlineStr"/>
+      <c r="D22" s="216" t="inlineStr"/>
+      <c r="E22" s="216" t="inlineStr"/>
+      <c r="F22" s="203" t="inlineStr">
+        <is>
+          <t>Week 6 — Jewish Criminal Underground — Issac Babel, Odessa Stories, pp. 1-103</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="201" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B23" s="216" t="inlineStr"/>
+      <c r="C23" s="216" t="inlineStr"/>
+      <c r="D23" s="216" t="inlineStr"/>
+      <c r="E23" s="216" t="inlineStr"/>
+      <c r="F23" s="203" t="inlineStr">
+        <is>
+          <t>Week 7 — Jewish Childhood — Isaac Babel, Odessa Stories, pp. 103-175</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="201" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B24" s="216" t="inlineStr"/>
+      <c r="C24" s="216" t="inlineStr"/>
+      <c r="D24" s="216" t="inlineStr"/>
+      <c r="E24" s="216" t="inlineStr"/>
+      <c r="F24" s="203" t="inlineStr">
+        <is>
+          <t>Week 8 — Holocaust and the Problem of Its Representation — Film: Unzere Kinder, dir. Natan Gross.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="201" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B25" s="216" t="inlineStr"/>
+      <c r="C25" s="216" t="inlineStr"/>
+      <c r="D25" s="216" t="inlineStr"/>
+      <c r="E25" s="216" t="inlineStr"/>
+      <c r="F25" s="203" t="inlineStr">
+        <is>
+          <t>Week 9 — Holocaust Literature: Characteristics — Imre Kertesz, Fatelessness, pp. 1-99</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="204" t="inlineStr">
+        <is>
+          <t>Midterm Oral Exam</t>
+        </is>
+      </c>
+      <c r="B26" s="214" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="C26" s="217" t="inlineStr"/>
+      <c r="D26" s="217" t="inlineStr"/>
+      <c r="E26" s="217" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F26" s="206">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/js-310-midterm-oral-exam.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="207" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B27" s="216" t="inlineStr"/>
+      <c r="C27" s="216" t="inlineStr"/>
+      <c r="D27" s="216" t="inlineStr"/>
+      <c r="E27" s="216" t="inlineStr"/>
+      <c r="F27" s="203" t="inlineStr">
+        <is>
+          <t>Midterm Oral Exam — instructional week 8 (15-min quote presentation, 60 pts max)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="197" t="inlineStr">
+        <is>
+          <t>Final Oral Exam</t>
+        </is>
+      </c>
+      <c r="B28" s="214" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="C28" s="215" t="inlineStr"/>
+      <c r="D28" s="215" t="inlineStr"/>
+      <c r="E28" s="215" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F28" s="200">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/js-310-final-oral-exam.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="207" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B29" s="216" t="inlineStr"/>
+      <c r="C29" s="216" t="inlineStr"/>
+      <c r="D29" s="216" t="inlineStr"/>
+      <c r="E29" s="216" t="inlineStr"/>
+      <c r="F29" s="203" t="inlineStr">
+        <is>
+          <t>Final Oral Exam — last instructional week (15-min presentation on Love/Tradition/Jewishness/Violence/Humor across 3 read</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="204" t="inlineStr">
+        <is>
+          <t>Midterm Quiz</t>
+        </is>
+      </c>
+      <c r="B30" s="214" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="C30" s="217" t="inlineStr"/>
+      <c r="D30" s="217" t="inlineStr"/>
+      <c r="E30" s="217" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F30" s="206">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/js-310-midterm-quiz.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="208" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="B31" s="216" t="inlineStr"/>
+      <c r="C31" s="216" t="inlineStr"/>
+      <c r="D31" s="216" t="inlineStr"/>
+      <c r="E31" s="216" t="inlineStr"/>
+      <c r="F31" s="203" t="inlineStr">
+        <is>
+          <t>Midterm Quiz — Thursday, instructional week 7 (20 questions, closed-ended)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="197" t="inlineStr">
+        <is>
+          <t>Final Quiz</t>
+        </is>
+      </c>
+      <c r="B32" s="214" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="C32" s="215" t="inlineStr"/>
+      <c r="D32" s="215" t="inlineStr"/>
+      <c r="E32" s="215" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F32" s="200">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/documents/js-310-final-quiz.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="208" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="B33" s="216" t="inlineStr"/>
+      <c r="C33" s="216" t="inlineStr"/>
+      <c r="D33" s="216" t="inlineStr"/>
+      <c r="E33" s="216" t="inlineStr"/>
+      <c r="F33" s="203" t="inlineStr">
+        <is>
+          <t>Final Quiz — same format as midterm, second half of semester</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="29" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B34" s="209" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="B6:F6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Mark five BUAD-304 Connect assessments as VORBEI
Completed: 3.01, 3.04, 5.01, 11.02, and 12.01 self-assessments.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -11,9 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-281" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ECON-351" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-304" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SPAN-290" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JS-310" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SPAN-290" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JS-310" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-304" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -512,7 +512,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="243">
+  <cellXfs count="248">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1200,6 +1200,21 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="48" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="28" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4020,12 +4035,12 @@
       </c>
       <c r="H110" s="11" t="inlineStr">
         <is>
-          <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
+          <t>Connect: Sharpen Companion</t>
         </is>
       </c>
       <c r="I110" s="11" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="J110" s="11" t="inlineStr">
@@ -4442,7 +4457,7 @@
     <row r="125">
       <c r="A125" s="19" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B125" s="19" t="inlineStr">
@@ -4462,7 +4477,7 @@
       </c>
       <c r="E125" s="19" t="inlineStr">
         <is>
-          <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
+          <t>Connect: Sharpen Companion</t>
         </is>
       </c>
     </row>
@@ -8639,1243 +8654,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001F77B4"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G54"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="66" t="inlineStr">
-        <is>
-          <t>BUAD-304 — Organizational Behavior and Leadership</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="28">
-        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/sources/buad-304-source.pdf","SEE HERE")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="29" t="inlineStr">
-        <is>
-          <t>Instructor</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Christine El Haddad</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="29" t="inlineStr">
-        <is>
-          <t>Term</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Fall 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="29" t="inlineStr">
-        <is>
-          <t>Required for an A</t>
-        </is>
-      </c>
-      <c r="B5" s="30" t="inlineStr">
-        <is>
-          <t>Curved (class rank)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="29" t="inlineStr">
-        <is>
-          <t>Grading scale</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Weighted score (% of points earned) + class average + student ranking (relative grading - no fixed A threshold in syllabus)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="67" t="inlineStr">
-        <is>
-          <t>Final Exam 25%  |  Participation 15%  |  Midterm Exam 15%  |  Team Project Paper 15%  |  Final Reflection Paper 10%  |  Presentation 10%  |  Case Analysis Assignments 5%  |  Proposal &amp; Team Contract 3%  |  Self &amp; Peer Evaluation 2%</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="29" t="inlineStr">
-        <is>
-          <t>Connect prep</t>
-        </is>
-      </c>
-      <c r="B8" s="68" t="inlineStr">
-        <is>
-          <t>Ungraded - Connect self-assessments are class prep, not part of Participation or other grades.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="69" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B10" s="69" t="inlineStr">
-        <is>
-          <t>Weight</t>
-        </is>
-      </c>
-      <c r="C10" s="69" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="D10" s="69" t="inlineStr">
-        <is>
-          <t>Due Date</t>
-        </is>
-      </c>
-      <c r="E10" s="69" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="F10" s="69" t="inlineStr">
-        <is>
-          <t>Group Project</t>
-        </is>
-      </c>
-      <c r="G10" s="69" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="70" t="inlineStr">
-        <is>
-          <t>Final Exam</t>
-        </is>
-      </c>
-      <c r="B11" s="230" t="inlineStr">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-      <c r="C11" s="231" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D11" s="231" t="inlineStr">
-        <is>
-          <t>2026-12-09</t>
-        </is>
-      </c>
-      <c r="E11" s="231" t="inlineStr"/>
-      <c r="F11" s="231" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G11" s="73">
-        <f>HYPERLINK("documents/buad-304-final-exam.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="74" t="inlineStr">
-        <is>
-          <t>Exam</t>
-        </is>
-      </c>
-      <c r="B12" s="232" t="inlineStr"/>
-      <c r="C12" s="232" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D12" s="232" t="inlineStr">
-        <is>
-          <t>2026-12-09</t>
-        </is>
-      </c>
-      <c r="E12" s="232" t="inlineStr"/>
-      <c r="F12" s="232" t="inlineStr"/>
-      <c r="G12" s="76" t="inlineStr">
-        <is>
-          <t>Final Exam</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="77" t="inlineStr">
-        <is>
-          <t>Participation</t>
-        </is>
-      </c>
-      <c r="B13" s="230" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="C13" s="233" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D13" s="233" t="inlineStr">
-        <is>
-          <t>2026-12-04</t>
-        </is>
-      </c>
-      <c r="E13" s="233" t="inlineStr"/>
-      <c r="F13" s="233" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G13" s="79">
-        <f>HYPERLINK("documents/buad-304-participation.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="80" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B14" s="232" t="inlineStr"/>
-      <c r="C14" s="232" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D14" s="232" t="inlineStr"/>
-      <c r="E14" s="232" t="inlineStr"/>
-      <c r="F14" s="232" t="inlineStr"/>
-      <c r="G14" s="76" t="inlineStr">
-        <is>
-          <t>Research: SONA registration opens</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="80" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B15" s="232" t="inlineStr"/>
-      <c r="C15" s="232" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="D15" s="232" t="inlineStr"/>
-      <c r="E15" s="232" t="inlineStr"/>
-      <c r="F15" s="232" t="inlineStr"/>
-      <c r="G15" s="76" t="inlineStr">
-        <is>
-          <t>Research: Prescreening questionnaire opens</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="80" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B16" s="232" t="inlineStr"/>
-      <c r="C16" s="232" t="inlineStr"/>
-      <c r="D16" s="232" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="E16" s="232" t="inlineStr"/>
-      <c r="F16" s="232" t="inlineStr"/>
-      <c r="G16" s="76" t="inlineStr">
-        <is>
-          <t>Research: Setup deadline (registration, prescreening, contacts)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="80" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B17" s="232" t="inlineStr"/>
-      <c r="C17" s="232" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="D17" s="232" t="inlineStr"/>
-      <c r="E17" s="232" t="inlineStr"/>
-      <c r="F17" s="232" t="inlineStr"/>
-      <c r="G17" s="76" t="inlineStr">
-        <is>
-          <t>Research: Study invitations begin (after setup)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="80" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B18" s="232" t="inlineStr"/>
-      <c r="C18" s="232" t="inlineStr"/>
-      <c r="D18" s="232" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="E18" s="232" t="inlineStr"/>
-      <c r="F18" s="232" t="inlineStr"/>
-      <c r="G18" s="76" t="inlineStr">
-        <is>
-          <t>Research: Employee contact surveys sent</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="81" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B19" s="232" t="inlineStr">
-        <is>
-          <t>Not in syllabus (% of 15%)</t>
-        </is>
-      </c>
-      <c r="C19" s="232" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D19" s="232" t="inlineStr">
-        <is>
-          <t>2026-12-04</t>
-        </is>
-      </c>
-      <c r="E19" s="232" t="inlineStr"/>
-      <c r="F19" s="232" t="inlineStr"/>
-      <c r="G19" s="76" t="inlineStr">
-        <is>
-          <t>Active Class Participation — attend MW sessions prepared; contribute to discussions and in-class activities (2 free abse</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="81" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B20" s="232" t="inlineStr">
-        <is>
-          <t>Not in syllabus (% of 15%)</t>
-        </is>
-      </c>
-      <c r="C20" s="232" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="D20" s="232" t="inlineStr">
-        <is>
-          <t>2026-12-04</t>
-        </is>
-      </c>
-      <c r="E20" s="232" t="inlineStr"/>
-      <c r="F20" s="232" t="inlineStr"/>
-      <c r="G20" s="76" t="inlineStr">
-        <is>
-          <t>Team Engagement — effective engagement with project team throughout semester</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="80" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B21" s="232" t="inlineStr">
-        <is>
-          <t>Not in syllabus (% of 15%)</t>
-        </is>
-      </c>
-      <c r="C21" s="232" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D21" s="232" t="inlineStr">
-        <is>
-          <t>2026-12-04</t>
-        </is>
-      </c>
-      <c r="E21" s="232" t="inlineStr"/>
-      <c r="F21" s="232" t="inlineStr"/>
-      <c r="G21" s="76" t="inlineStr">
-        <is>
-          <t>Research Studies — complete 2.0 credits via SONA (register, setup, lab studies)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="80" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="B22" s="232" t="inlineStr"/>
-      <c r="C22" s="232" t="inlineStr"/>
-      <c r="D22" s="232" t="inlineStr">
-        <is>
-          <t>2026-12-04</t>
-        </is>
-      </c>
-      <c r="E22" s="232" t="inlineStr"/>
-      <c r="F22" s="232" t="inlineStr"/>
-      <c r="G22" s="76" t="inlineStr">
-        <is>
-          <t>Research: Complete 2.0 research credits</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="70" t="inlineStr">
-        <is>
-          <t>Midterm Exam</t>
-        </is>
-      </c>
-      <c r="B23" s="230" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="C23" s="231" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D23" s="231" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E23" s="231" t="inlineStr"/>
-      <c r="F23" s="231" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G23" s="73">
-        <f>HYPERLINK("documents/buad-304-midterm-exam.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="74" t="inlineStr">
-        <is>
-          <t>Exam</t>
-        </is>
-      </c>
-      <c r="B24" s="232" t="inlineStr"/>
-      <c r="C24" s="232" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D24" s="232" t="inlineStr">
-        <is>
-          <t>2026-10-14</t>
-        </is>
-      </c>
-      <c r="E24" s="232" t="inlineStr"/>
-      <c r="F24" s="232" t="inlineStr"/>
-      <c r="G24" s="76" t="inlineStr">
-        <is>
-          <t>Midterm Exam</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="77" t="inlineStr">
-        <is>
-          <t>Team Project Paper</t>
-        </is>
-      </c>
-      <c r="B25" s="230" t="inlineStr">
-        <is>
-          <t>15%</t>
-        </is>
-      </c>
-      <c r="C25" s="233" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D25" s="233" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="E25" s="233" t="inlineStr"/>
-      <c r="F25" s="233" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G25" s="79">
-        <f>HYPERLINK("documents/buad-304-team-project-paper.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="81" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B26" s="232" t="inlineStr"/>
-      <c r="C26" s="232" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D26" s="232" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E26" s="232" t="inlineStr"/>
-      <c r="F26" s="232" t="inlineStr"/>
-      <c r="G26" s="76" t="inlineStr">
-        <is>
-          <t>Team project outline</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="81" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B27" s="232" t="inlineStr"/>
-      <c r="C27" s="232" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D27" s="232" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="E27" s="232" t="inlineStr"/>
-      <c r="F27" s="232" t="inlineStr"/>
-      <c r="G27" s="76" t="inlineStr">
-        <is>
-          <t>Team project paper</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="70" t="inlineStr">
-        <is>
-          <t>Final Reflection Paper</t>
-        </is>
-      </c>
-      <c r="B28" s="230" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="C28" s="231" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D28" s="231" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E28" s="231" t="inlineStr"/>
-      <c r="F28" s="231" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G28" s="73">
-        <f>HYPERLINK("documents/buad-304-final-reflection-paper.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="81" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B29" s="232" t="inlineStr"/>
-      <c r="C29" s="232" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D29" s="232" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="E29" s="232" t="inlineStr"/>
-      <c r="F29" s="232" t="inlineStr"/>
-      <c r="G29" s="76" t="inlineStr">
-        <is>
-          <t>Personal Reflection Paper</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="77" t="inlineStr">
-        <is>
-          <t>Presentation</t>
-        </is>
-      </c>
-      <c r="B30" s="230" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="C30" s="233" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D30" s="233" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="E30" s="233" t="inlineStr"/>
-      <c r="F30" s="233" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G30" s="79">
-        <f>HYPERLINK("documents/buad-304-presentation.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="81" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B31" s="232" t="inlineStr"/>
-      <c r="C31" s="232" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D31" s="232" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="E31" s="232" t="inlineStr"/>
-      <c r="F31" s="232" t="inlineStr"/>
-      <c r="G31" s="76" t="inlineStr">
-        <is>
-          <t>Presentation slides</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="70" t="inlineStr">
-        <is>
-          <t>Case Analysis Assignments</t>
-        </is>
-      </c>
-      <c r="B32" s="230" t="inlineStr">
-        <is>
-          <t>5%</t>
-        </is>
-      </c>
-      <c r="C32" s="231" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="D32" s="231" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="E32" s="231" t="inlineStr"/>
-      <c r="F32" s="231" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G32" s="73">
-        <f>HYPERLINK("documents/buad-304-case-analysis-assignments.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="81" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B33" s="232" t="inlineStr"/>
-      <c r="C33" s="232" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="D33" s="232" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="E33" s="232" t="inlineStr"/>
-      <c r="F33" s="232" t="inlineStr"/>
-      <c r="G33" s="76" t="inlineStr">
-        <is>
-          <t>Thomas Green Case Analysis Memo</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="81" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B34" s="232" t="inlineStr"/>
-      <c r="C34" s="232" t="inlineStr">
-        <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="D34" s="232" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="E34" s="232" t="inlineStr"/>
-      <c r="F34" s="232" t="inlineStr"/>
-      <c r="G34" s="76" t="inlineStr">
-        <is>
-          <t>SkillsForTomorrow Analysis Memo</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="77" t="inlineStr">
-        <is>
-          <t>Proposal &amp; Team Contract</t>
-        </is>
-      </c>
-      <c r="B35" s="230" t="inlineStr">
-        <is>
-          <t>3%</t>
-        </is>
-      </c>
-      <c r="C35" s="233" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D35" s="233" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E35" s="233" t="inlineStr"/>
-      <c r="F35" s="233" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G35" s="79">
-        <f>HYPERLINK("documents/buad-304-proposal-team-contract.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="81" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B36" s="232" t="inlineStr"/>
-      <c r="C36" s="232" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D36" s="232" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E36" s="232" t="inlineStr"/>
-      <c r="F36" s="232" t="inlineStr"/>
-      <c r="G36" s="76" t="inlineStr">
-        <is>
-          <t>Team project proposal &amp; team contract</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="70" t="inlineStr">
-        <is>
-          <t>Self &amp; Peer Evaluation</t>
-        </is>
-      </c>
-      <c r="B37" s="230" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="C37" s="231" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D37" s="231" t="inlineStr">
-        <is>
-          <t>2026-11-18</t>
-        </is>
-      </c>
-      <c r="E37" s="231" t="inlineStr"/>
-      <c r="F37" s="231" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G37" s="73">
-        <f>HYPERLINK("documents/buad-304-self-peer-evaluation.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="81" t="inlineStr">
-        <is>
-          <t>Assignment</t>
-        </is>
-      </c>
-      <c r="B38" s="232" t="inlineStr"/>
-      <c r="C38" s="232" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="D38" s="232" t="inlineStr">
-        <is>
-          <t>2026-11-18</t>
-        </is>
-      </c>
-      <c r="E38" s="232" t="inlineStr"/>
-      <c r="F38" s="232" t="inlineStr"/>
-      <c r="G38" s="76" t="inlineStr">
-        <is>
-          <t>Self &amp; peer evaluation</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="77" t="inlineStr">
-        <is>
-          <t>Personal Assessments (Connect)</t>
-        </is>
-      </c>
-      <c r="B39" s="230" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C39" s="233" t="inlineStr"/>
-      <c r="D39" s="233" t="inlineStr">
-        <is>
-          <t>2026-12-20</t>
-        </is>
-      </c>
-      <c r="E39" s="233" t="inlineStr"/>
-      <c r="F39" s="233" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G39" s="79">
-        <f>HYPERLINK("documents/buad-304-personal-assessments-connect.pdf","Open PDF")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B40" s="232" t="inlineStr"/>
-      <c r="C40" s="232" t="inlineStr"/>
-      <c r="D40" s="232" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="E40" s="234" t="inlineStr">
-        <is>
-          <t>VORBEI</t>
-        </is>
-      </c>
-      <c r="F40" s="232" t="inlineStr"/>
-      <c r="G40" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B41" s="232" t="inlineStr"/>
-      <c r="C41" s="232" t="inlineStr"/>
-      <c r="D41" s="232" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="E41" s="232" t="inlineStr"/>
-      <c r="F41" s="232" t="inlineStr"/>
-      <c r="G41" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B42" s="232" t="inlineStr"/>
-      <c r="C42" s="232" t="inlineStr"/>
-      <c r="D42" s="232" t="inlineStr">
-        <is>
-          <t>2026-09-02</t>
-        </is>
-      </c>
-      <c r="E42" s="232" t="inlineStr"/>
-      <c r="F42" s="232" t="inlineStr"/>
-      <c r="G42" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 5.01 - Assessing Your</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B43" s="232" t="inlineStr"/>
-      <c r="C43" s="232" t="inlineStr"/>
-      <c r="D43" s="232" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-      <c r="E43" s="232" t="inlineStr"/>
-      <c r="F43" s="232" t="inlineStr"/>
-      <c r="G43" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Sharpen Companion</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B44" s="232" t="inlineStr"/>
-      <c r="C44" s="232" t="inlineStr"/>
-      <c r="D44" s="232" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="E44" s="232" t="inlineStr"/>
-      <c r="F44" s="232" t="inlineStr"/>
-      <c r="G44" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 11.01 - What is my</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B45" s="232" t="inlineStr"/>
-      <c r="C45" s="232" t="inlineStr"/>
-      <c r="D45" s="232" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="E45" s="232" t="inlineStr"/>
-      <c r="F45" s="232" t="inlineStr"/>
-      <c r="G45" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 11.02 - What is my</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B46" s="232" t="inlineStr"/>
-      <c r="C46" s="232" t="inlineStr"/>
-      <c r="D46" s="232" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-      <c r="E46" s="232" t="inlineStr"/>
-      <c r="F46" s="232" t="inlineStr"/>
-      <c r="G46" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 12.01 - What kind of</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B47" s="232" t="inlineStr"/>
-      <c r="C47" s="232" t="inlineStr"/>
-      <c r="D47" s="232" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E47" s="232" t="inlineStr"/>
-      <c r="F47" s="232" t="inlineStr"/>
-      <c r="G47" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 10.5 - Preferred Conflict</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B48" s="232" t="inlineStr"/>
-      <c r="C48" s="232" t="inlineStr"/>
-      <c r="D48" s="232" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="E48" s="232" t="inlineStr"/>
-      <c r="F48" s="232" t="inlineStr"/>
-      <c r="G48" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 9.01 - Assessing My</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B49" s="232" t="inlineStr"/>
-      <c r="C49" s="232" t="inlineStr"/>
-      <c r="D49" s="232" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E49" s="232" t="inlineStr"/>
-      <c r="F49" s="232" t="inlineStr"/>
-      <c r="G49" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 8.01 - Group</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B50" s="232" t="inlineStr"/>
-      <c r="C50" s="232" t="inlineStr"/>
-      <c r="D50" s="232" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="E50" s="232" t="inlineStr"/>
-      <c r="F50" s="232" t="inlineStr"/>
-      <c r="G50" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 14.02 - What Type of Organizational Culture Do I</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B51" s="232" t="inlineStr"/>
-      <c r="C51" s="232" t="inlineStr"/>
-      <c r="D51" s="232" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
-      </c>
-      <c r="E51" s="232" t="inlineStr"/>
-      <c r="F51" s="232" t="inlineStr"/>
-      <c r="G51" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 16.02 - What Is Your</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B52" s="232" t="inlineStr"/>
-      <c r="C52" s="232" t="inlineStr"/>
-      <c r="D52" s="232" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
-      </c>
-      <c r="E52" s="232" t="inlineStr"/>
-      <c r="F52" s="232" t="inlineStr"/>
-      <c r="G52" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 16.03 - Assessing Your</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="82" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="B53" s="232" t="inlineStr"/>
-      <c r="C53" s="232" t="inlineStr"/>
-      <c r="D53" s="232" t="inlineStr">
-        <is>
-          <t>2026-12-20</t>
-        </is>
-      </c>
-      <c r="E53" s="232" t="inlineStr"/>
-      <c r="F53" s="232" t="inlineStr"/>
-      <c r="G53" s="76" t="inlineStr">
-        <is>
-          <t>Connect: Self-Assessment 12.02 - Which influence</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="29" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B54" s="83" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A7:G7"/>
-    <mergeCell ref="B6:G6"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
     <tabColor rgb="002CA02C"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -11118,7 +9896,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="008C564B"/>
@@ -11706,4 +10484,1257 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001F77B4"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="66" t="inlineStr">
+        <is>
+          <t>BUAD-304 — Organizational Behavior and Leadership</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="28">
+        <f>HYPERLINK("https://raw.githubusercontent.com/vengeanceaiUSC/Syllabus-/cursor/add-syllabus-dissector-skill-a676/output/sources/buad-304-source.pdf","SEE HERE")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="29" t="inlineStr">
+        <is>
+          <t>Instructor</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Christine El Haddad</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fall 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>Required for an A</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>Curved (class rank)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>Grading scale</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Weighted score (% of points earned) + class average + student ranking (relative grading - no fixed A threshold in syllabus)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="67" t="inlineStr">
+        <is>
+          <t>Final Exam 25%  |  Participation 15%  |  Midterm Exam 15%  |  Team Project Paper 15%  |  Final Reflection Paper 10%  |  Presentation 10%  |  Case Analysis Assignments 5%  |  Proposal &amp; Team Contract 3%  |  Self &amp; Peer Evaluation 2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>Connect prep</t>
+        </is>
+      </c>
+      <c r="B8" s="68" t="inlineStr">
+        <is>
+          <t>Ungraded - Connect self-assessments are class prep, not part of Participation or other grades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="69" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B10" s="69" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="C10" s="69" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="D10" s="69" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="E10" s="69" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F10" s="69" t="inlineStr">
+        <is>
+          <t>Group Project</t>
+        </is>
+      </c>
+      <c r="G10" s="69" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="70" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+      <c r="B11" s="243" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="C11" s="244" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D11" s="244" t="inlineStr">
+        <is>
+          <t>2026-12-09</t>
+        </is>
+      </c>
+      <c r="E11" s="244" t="inlineStr"/>
+      <c r="F11" s="244" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G11" s="73">
+        <f>HYPERLINK("documents/buad-304-final-exam.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="74" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="B12" s="245" t="inlineStr"/>
+      <c r="C12" s="245" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D12" s="245" t="inlineStr">
+        <is>
+          <t>2026-12-09</t>
+        </is>
+      </c>
+      <c r="E12" s="245" t="inlineStr"/>
+      <c r="F12" s="245" t="inlineStr"/>
+      <c r="G12" s="76" t="inlineStr">
+        <is>
+          <t>Final Exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="77" t="inlineStr">
+        <is>
+          <t>Participation</t>
+        </is>
+      </c>
+      <c r="B13" s="243" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="C13" s="246" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D13" s="246" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E13" s="246" t="inlineStr"/>
+      <c r="F13" s="246" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G13" s="79">
+        <f>HYPERLINK("documents/buad-304-participation.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="80" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B14" s="245" t="inlineStr"/>
+      <c r="C14" s="245" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D14" s="245" t="inlineStr"/>
+      <c r="E14" s="245" t="inlineStr"/>
+      <c r="F14" s="245" t="inlineStr"/>
+      <c r="G14" s="76" t="inlineStr">
+        <is>
+          <t>Research: SONA registration opens</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="80" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B15" s="245" t="inlineStr"/>
+      <c r="C15" s="245" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="D15" s="245" t="inlineStr"/>
+      <c r="E15" s="245" t="inlineStr"/>
+      <c r="F15" s="245" t="inlineStr"/>
+      <c r="G15" s="76" t="inlineStr">
+        <is>
+          <t>Research: Prescreening questionnaire opens</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="80" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B16" s="245" t="inlineStr"/>
+      <c r="C16" s="245" t="inlineStr"/>
+      <c r="D16" s="245" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E16" s="245" t="inlineStr"/>
+      <c r="F16" s="245" t="inlineStr"/>
+      <c r="G16" s="76" t="inlineStr">
+        <is>
+          <t>Research: Setup deadline (registration, prescreening, contacts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="80" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B17" s="245" t="inlineStr"/>
+      <c r="C17" s="245" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="D17" s="245" t="inlineStr"/>
+      <c r="E17" s="245" t="inlineStr"/>
+      <c r="F17" s="245" t="inlineStr"/>
+      <c r="G17" s="76" t="inlineStr">
+        <is>
+          <t>Research: Study invitations begin (after setup)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="80" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B18" s="245" t="inlineStr"/>
+      <c r="C18" s="245" t="inlineStr"/>
+      <c r="D18" s="245" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="E18" s="245" t="inlineStr"/>
+      <c r="F18" s="245" t="inlineStr"/>
+      <c r="G18" s="76" t="inlineStr">
+        <is>
+          <t>Research: Employee contact surveys sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B19" s="245" t="inlineStr">
+        <is>
+          <t>Not in syllabus (% of 15%)</t>
+        </is>
+      </c>
+      <c r="C19" s="245" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D19" s="245" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E19" s="245" t="inlineStr"/>
+      <c r="F19" s="245" t="inlineStr"/>
+      <c r="G19" s="76" t="inlineStr">
+        <is>
+          <t>Active Class Participation — attend MW sessions prepared; contribute to discussions and in-class activities (2 free abse</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B20" s="245" t="inlineStr">
+        <is>
+          <t>Not in syllabus (% of 15%)</t>
+        </is>
+      </c>
+      <c r="C20" s="245" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="D20" s="245" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E20" s="245" t="inlineStr"/>
+      <c r="F20" s="245" t="inlineStr"/>
+      <c r="G20" s="76" t="inlineStr">
+        <is>
+          <t>Team Engagement — effective engagement with project team throughout semester</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="80" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B21" s="245" t="inlineStr">
+        <is>
+          <t>Not in syllabus (% of 15%)</t>
+        </is>
+      </c>
+      <c r="C21" s="245" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D21" s="245" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E21" s="245" t="inlineStr"/>
+      <c r="F21" s="245" t="inlineStr"/>
+      <c r="G21" s="76" t="inlineStr">
+        <is>
+          <t>Research Studies — complete 2.0 credits via SONA (register, setup, lab studies)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="80" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="B22" s="245" t="inlineStr"/>
+      <c r="C22" s="245" t="inlineStr"/>
+      <c r="D22" s="245" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="E22" s="245" t="inlineStr"/>
+      <c r="F22" s="245" t="inlineStr"/>
+      <c r="G22" s="76" t="inlineStr">
+        <is>
+          <t>Research: Complete 2.0 research credits</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="70" t="inlineStr">
+        <is>
+          <t>Midterm Exam</t>
+        </is>
+      </c>
+      <c r="B23" s="243" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="C23" s="244" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D23" s="244" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E23" s="244" t="inlineStr"/>
+      <c r="F23" s="244" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G23" s="73">
+        <f>HYPERLINK("documents/buad-304-midterm-exam.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="74" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="B24" s="245" t="inlineStr"/>
+      <c r="C24" s="245" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="D24" s="245" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="E24" s="245" t="inlineStr"/>
+      <c r="F24" s="245" t="inlineStr"/>
+      <c r="G24" s="76" t="inlineStr">
+        <is>
+          <t>Midterm Exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="77" t="inlineStr">
+        <is>
+          <t>Team Project Paper</t>
+        </is>
+      </c>
+      <c r="B25" s="243" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="C25" s="246" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D25" s="246" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E25" s="246" t="inlineStr"/>
+      <c r="F25" s="246" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G25" s="79">
+        <f>HYPERLINK("documents/buad-304-team-project-paper.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B26" s="245" t="inlineStr"/>
+      <c r="C26" s="245" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D26" s="245" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E26" s="245" t="inlineStr"/>
+      <c r="F26" s="245" t="inlineStr"/>
+      <c r="G26" s="76" t="inlineStr">
+        <is>
+          <t>Team project outline</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B27" s="245" t="inlineStr"/>
+      <c r="C27" s="245" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D27" s="245" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E27" s="245" t="inlineStr"/>
+      <c r="F27" s="245" t="inlineStr"/>
+      <c r="G27" s="76" t="inlineStr">
+        <is>
+          <t>Team project paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="70" t="inlineStr">
+        <is>
+          <t>Final Reflection Paper</t>
+        </is>
+      </c>
+      <c r="B28" s="243" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C28" s="244" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D28" s="244" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E28" s="244" t="inlineStr"/>
+      <c r="F28" s="244" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G28" s="73">
+        <f>HYPERLINK("documents/buad-304-final-reflection-paper.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B29" s="245" t="inlineStr"/>
+      <c r="C29" s="245" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D29" s="245" t="inlineStr">
+        <is>
+          <t>2026-12-02</t>
+        </is>
+      </c>
+      <c r="E29" s="245" t="inlineStr"/>
+      <c r="F29" s="245" t="inlineStr"/>
+      <c r="G29" s="76" t="inlineStr">
+        <is>
+          <t>Personal Reflection Paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="77" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="B30" s="243" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C30" s="246" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D30" s="246" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E30" s="246" t="inlineStr"/>
+      <c r="F30" s="246" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G30" s="79">
+        <f>HYPERLINK("documents/buad-304-presentation.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B31" s="245" t="inlineStr"/>
+      <c r="C31" s="245" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D31" s="245" t="inlineStr">
+        <is>
+          <t>2026-11-09</t>
+        </is>
+      </c>
+      <c r="E31" s="245" t="inlineStr"/>
+      <c r="F31" s="245" t="inlineStr"/>
+      <c r="G31" s="76" t="inlineStr">
+        <is>
+          <t>Presentation slides</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="70" t="inlineStr">
+        <is>
+          <t>Case Analysis Assignments</t>
+        </is>
+      </c>
+      <c r="B32" s="243" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="C32" s="244" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D32" s="244" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E32" s="244" t="inlineStr"/>
+      <c r="F32" s="244" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G32" s="73">
+        <f>HYPERLINK("documents/buad-304-case-analysis-assignments.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B33" s="245" t="inlineStr"/>
+      <c r="C33" s="245" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D33" s="245" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E33" s="245" t="inlineStr"/>
+      <c r="F33" s="245" t="inlineStr"/>
+      <c r="G33" s="76" t="inlineStr">
+        <is>
+          <t>Thomas Green Case Analysis Memo</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B34" s="245" t="inlineStr"/>
+      <c r="C34" s="245" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="D34" s="245" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E34" s="245" t="inlineStr"/>
+      <c r="F34" s="245" t="inlineStr"/>
+      <c r="G34" s="76" t="inlineStr">
+        <is>
+          <t>SkillsForTomorrow Analysis Memo</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="77" t="inlineStr">
+        <is>
+          <t>Proposal &amp; Team Contract</t>
+        </is>
+      </c>
+      <c r="B35" s="243" t="inlineStr">
+        <is>
+          <t>3%</t>
+        </is>
+      </c>
+      <c r="C35" s="246" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D35" s="246" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E35" s="246" t="inlineStr"/>
+      <c r="F35" s="246" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G35" s="79">
+        <f>HYPERLINK("documents/buad-304-proposal-team-contract.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B36" s="245" t="inlineStr"/>
+      <c r="C36" s="245" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D36" s="245" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E36" s="245" t="inlineStr"/>
+      <c r="F36" s="245" t="inlineStr"/>
+      <c r="G36" s="76" t="inlineStr">
+        <is>
+          <t>Team project proposal &amp; team contract</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="70" t="inlineStr">
+        <is>
+          <t>Self &amp; Peer Evaluation</t>
+        </is>
+      </c>
+      <c r="B37" s="243" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="C37" s="244" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D37" s="244" t="inlineStr">
+        <is>
+          <t>2026-11-18</t>
+        </is>
+      </c>
+      <c r="E37" s="244" t="inlineStr"/>
+      <c r="F37" s="244" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G37" s="73">
+        <f>HYPERLINK("documents/buad-304-self-peer-evaluation.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="81" t="inlineStr">
+        <is>
+          <t>Assignment</t>
+        </is>
+      </c>
+      <c r="B38" s="245" t="inlineStr"/>
+      <c r="C38" s="245" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D38" s="245" t="inlineStr">
+        <is>
+          <t>2026-11-18</t>
+        </is>
+      </c>
+      <c r="E38" s="245" t="inlineStr"/>
+      <c r="F38" s="245" t="inlineStr"/>
+      <c r="G38" s="76" t="inlineStr">
+        <is>
+          <t>Self &amp; peer evaluation</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="77" t="inlineStr">
+        <is>
+          <t>Personal Assessments (Connect)</t>
+        </is>
+      </c>
+      <c r="B39" s="243" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C39" s="246" t="inlineStr"/>
+      <c r="D39" s="246" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E39" s="246" t="inlineStr"/>
+      <c r="F39" s="246" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G39" s="79">
+        <f>HYPERLINK("documents/buad-304-personal-assessments-connect.pdf","Open PDF")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B40" s="245" t="inlineStr"/>
+      <c r="C40" s="245" t="inlineStr"/>
+      <c r="D40" s="245" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E40" s="247" t="inlineStr">
+        <is>
+          <t>VORBEI</t>
+        </is>
+      </c>
+      <c r="F40" s="245" t="inlineStr"/>
+      <c r="G40" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 3.01 - What is my Big thinking about your topics and</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B41" s="245" t="inlineStr"/>
+      <c r="C41" s="245" t="inlineStr"/>
+      <c r="D41" s="245" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="E41" s="247" t="inlineStr">
+        <is>
+          <t>VORBEI</t>
+        </is>
+      </c>
+      <c r="F41" s="245" t="inlineStr"/>
+      <c r="G41" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 3.04 - What Is Your Level</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B42" s="245" t="inlineStr"/>
+      <c r="C42" s="245" t="inlineStr"/>
+      <c r="D42" s="245" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E42" s="247" t="inlineStr">
+        <is>
+          <t>VORBEI</t>
+        </is>
+      </c>
+      <c r="F42" s="245" t="inlineStr"/>
+      <c r="G42" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 5.01 - Assessing Your</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B43" s="245" t="inlineStr"/>
+      <c r="C43" s="245" t="inlineStr"/>
+      <c r="D43" s="245" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="E43" s="245" t="inlineStr"/>
+      <c r="F43" s="245" t="inlineStr"/>
+      <c r="G43" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Sharpen Companion</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B44" s="245" t="inlineStr"/>
+      <c r="C44" s="245" t="inlineStr"/>
+      <c r="D44" s="245" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="E44" s="245" t="inlineStr"/>
+      <c r="F44" s="245" t="inlineStr"/>
+      <c r="G44" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 11.01 - What is my</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B45" s="245" t="inlineStr"/>
+      <c r="C45" s="245" t="inlineStr"/>
+      <c r="D45" s="245" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="E45" s="247" t="inlineStr">
+        <is>
+          <t>VORBEI</t>
+        </is>
+      </c>
+      <c r="F45" s="245" t="inlineStr"/>
+      <c r="G45" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 11.02 - What is my</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B46" s="245" t="inlineStr"/>
+      <c r="C46" s="245" t="inlineStr"/>
+      <c r="D46" s="245" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="E46" s="247" t="inlineStr">
+        <is>
+          <t>VORBEI</t>
+        </is>
+      </c>
+      <c r="F46" s="245" t="inlineStr"/>
+      <c r="G46" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 12.01 - What kind of</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B47" s="245" t="inlineStr"/>
+      <c r="C47" s="245" t="inlineStr"/>
+      <c r="D47" s="245" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E47" s="245" t="inlineStr"/>
+      <c r="F47" s="245" t="inlineStr"/>
+      <c r="G47" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 10.5 - Preferred Conflict</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B48" s="245" t="inlineStr"/>
+      <c r="C48" s="245" t="inlineStr"/>
+      <c r="D48" s="245" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="E48" s="245" t="inlineStr"/>
+      <c r="F48" s="245" t="inlineStr"/>
+      <c r="G48" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 9.01 - Assessing My</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B49" s="245" t="inlineStr"/>
+      <c r="C49" s="245" t="inlineStr"/>
+      <c r="D49" s="245" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E49" s="245" t="inlineStr"/>
+      <c r="F49" s="245" t="inlineStr"/>
+      <c r="G49" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 8.01 - Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B50" s="245" t="inlineStr"/>
+      <c r="C50" s="245" t="inlineStr"/>
+      <c r="D50" s="245" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="E50" s="245" t="inlineStr"/>
+      <c r="F50" s="245" t="inlineStr"/>
+      <c r="G50" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 14.02 - What Type of Organizational Culture Do I</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B51" s="245" t="inlineStr"/>
+      <c r="C51" s="245" t="inlineStr"/>
+      <c r="D51" s="245" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="E51" s="245" t="inlineStr"/>
+      <c r="F51" s="245" t="inlineStr"/>
+      <c r="G51" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 16.02 - What Is Your</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B52" s="245" t="inlineStr"/>
+      <c r="C52" s="245" t="inlineStr"/>
+      <c r="D52" s="245" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="E52" s="245" t="inlineStr"/>
+      <c r="F52" s="245" t="inlineStr"/>
+      <c r="G52" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 16.03 - Assessing Your</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="82" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="B53" s="245" t="inlineStr"/>
+      <c r="C53" s="245" t="inlineStr"/>
+      <c r="D53" s="245" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="E53" s="245" t="inlineStr"/>
+      <c r="F53" s="245" t="inlineStr"/>
+      <c r="G53" s="76" t="inlineStr">
+        <is>
+          <t>Connect: Self-Assessment 12.02 - Which influence</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="29" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B54" s="83" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="B6:G6"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Graduation Plan sheet to syllabi workbook
Import graduation-plan.csv as a styled Excel tab after Overview, with
hyperlinks to dissected course sheets when a matching class exists.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/syllabi.xlsx
+++ b/output/syllabi.xlsx
@@ -8,13 +8,14 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-281" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-304" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ECON-351" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SPAN-290" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JS-310" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ANTH-202" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graduation Plan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-281" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BUAD-304" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ECON-351" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HIST-103" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SPAN-290" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JS-310" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ANTH-202" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -200,7 +201,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="49">
+  <fills count="52">
     <fill>
       <patternFill/>
     </fill>
@@ -442,6 +443,21 @@
         <fgColor rgb="00F6F3F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00548235"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0070AD47"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6E0B4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -513,7 +529,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="294">
+  <cellXfs count="303">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1355,6 +1371,33 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="49" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="50" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="51" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7043,6 +7086,667 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00548235"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="294" t="inlineStr">
+        <is>
+          <t>Graduation Plan — Marshall BBA (128 units)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="295" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="B2" s="295" t="inlineStr">
+        <is>
+          <t>Course Code</t>
+        </is>
+      </c>
+      <c r="C2" s="295" t="inlineStr">
+        <is>
+          <t>Course Title</t>
+        </is>
+      </c>
+      <c r="D2" s="295" t="inlineStr">
+        <is>
+          <t>Requirement Satisfied</t>
+        </is>
+      </c>
+      <c r="E2" s="295" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="F2" s="295" t="inlineStr">
+        <is>
+          <t>Semester Total</t>
+        </is>
+      </c>
+      <c r="G2" s="295" t="inlineStr">
+        <is>
+          <t>Cumulative Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="296" t="inlineStr">
+        <is>
+          <t>Prior Credit</t>
+        </is>
+      </c>
+      <c r="B3" s="297" t="inlineStr"/>
+      <c r="C3" s="298" t="inlineStr">
+        <is>
+          <t>Transfer / Prior USC Work</t>
+        </is>
+      </c>
+      <c r="D3" s="297" t="inlineStr"/>
+      <c r="E3" s="297" t="inlineStr"/>
+      <c r="F3" s="297" t="inlineStr"/>
+      <c r="G3" s="297" t="inlineStr">
+        <is>
+          <t>51.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="296" t="inlineStr">
+        <is>
+          <t>Fall 2026</t>
+        </is>
+      </c>
+      <c r="B4" s="299">
+        <f>HYPERLINK("#'BUAD-304'!A1","BUAD 304")</f>
+        <v/>
+      </c>
+      <c r="C4" s="300" t="inlineStr">
+        <is>
+          <t>Organizational Behavior and Leadership</t>
+        </is>
+      </c>
+      <c r="D4" s="301" t="inlineStr">
+        <is>
+          <t>Marshall Core</t>
+        </is>
+      </c>
+      <c r="E4" s="301" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F4" s="301" t="inlineStr">
+        <is>
+          <t>12.0</t>
+        </is>
+      </c>
+      <c r="G4" s="301" t="inlineStr">
+        <is>
+          <t>63.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="297" t="inlineStr"/>
+      <c r="B5" s="302">
+        <f>HYPERLINK("#'ECON-351'!A1","ECON 351")</f>
+        <v/>
+      </c>
+      <c r="C5" s="298" t="inlineStr">
+        <is>
+          <t>Microeconomics for Business</t>
+        </is>
+      </c>
+      <c r="D5" s="297" t="inlineStr">
+        <is>
+          <t>Marshall Core / Econ</t>
+        </is>
+      </c>
+      <c r="E5" s="297" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F5" s="297" t="inlineStr"/>
+      <c r="G5" s="297" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="301" t="inlineStr"/>
+      <c r="B6" s="301" t="inlineStr">
+        <is>
+          <t>Rel 137</t>
+        </is>
+      </c>
+      <c r="C6" s="300" t="inlineStr">
+        <is>
+          <t>Intro to Islam</t>
+        </is>
+      </c>
+      <c r="D6" s="301" t="inlineStr">
+        <is>
+          <t>GE Category B</t>
+        </is>
+      </c>
+      <c r="E6" s="301" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F6" s="301" t="inlineStr"/>
+      <c r="G6" s="301" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="296" t="inlineStr">
+        <is>
+          <t>Spring 2027</t>
+        </is>
+      </c>
+      <c r="B7" s="302">
+        <f>HYPERLINK("#'BUAD-281'!A1","BUAD 281")</f>
+        <v/>
+      </c>
+      <c r="C7" s="298" t="inlineStr">
+        <is>
+          <t>Introduction to Managerial Accounting</t>
+        </is>
+      </c>
+      <c r="D7" s="297" t="inlineStr">
+        <is>
+          <t>Marshall Core</t>
+        </is>
+      </c>
+      <c r="E7" s="297" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="F7" s="297" t="inlineStr">
+        <is>
+          <t>15.0</t>
+        </is>
+      </c>
+      <c r="G7" s="297" t="inlineStr">
+        <is>
+          <t>78.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="301" t="inlineStr"/>
+      <c r="B8" s="301" t="inlineStr">
+        <is>
+          <t>BUAD 306</t>
+        </is>
+      </c>
+      <c r="C8" s="300" t="inlineStr">
+        <is>
+          <t>Business Finance</t>
+        </is>
+      </c>
+      <c r="D8" s="301" t="inlineStr">
+        <is>
+          <t>Marshall Core</t>
+        </is>
+      </c>
+      <c r="E8" s="301" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F8" s="301" t="inlineStr"/>
+      <c r="G8" s="301" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="297" t="inlineStr"/>
+      <c r="B9" s="297" t="inlineStr">
+        <is>
+          <t>ECON 352</t>
+        </is>
+      </c>
+      <c r="C9" s="298" t="inlineStr">
+        <is>
+          <t>Macroeconomics for Business</t>
+        </is>
+      </c>
+      <c r="D9" s="297" t="inlineStr">
+        <is>
+          <t>Major Requirement</t>
+        </is>
+      </c>
+      <c r="E9" s="297" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F9" s="297" t="inlineStr"/>
+      <c r="G9" s="297" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="301" t="inlineStr"/>
+      <c r="B10" s="301" t="inlineStr">
+        <is>
+          <t>GE-C Course</t>
+        </is>
+      </c>
+      <c r="C10" s="300" t="inlineStr">
+        <is>
+          <t>Approved Social Analysis Course</t>
+        </is>
+      </c>
+      <c r="D10" s="301" t="inlineStr">
+        <is>
+          <t>GE Category C</t>
+        </is>
+      </c>
+      <c r="E10" s="301" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F10" s="301" t="inlineStr"/>
+      <c r="G10" s="301" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="296" t="inlineStr">
+        <is>
+          <t>Fall 2027</t>
+        </is>
+      </c>
+      <c r="B11" s="297" t="inlineStr">
+        <is>
+          <t>BUAD 302</t>
+        </is>
+      </c>
+      <c r="C11" s="298" t="inlineStr">
+        <is>
+          <t>Communication Strategy for Business</t>
+        </is>
+      </c>
+      <c r="D11" s="297" t="inlineStr">
+        <is>
+          <t>Marshall Core</t>
+        </is>
+      </c>
+      <c r="E11" s="297" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F11" s="297" t="inlineStr">
+        <is>
+          <t>12.0</t>
+        </is>
+      </c>
+      <c r="G11" s="297" t="inlineStr">
+        <is>
+          <t>90.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="301" t="inlineStr"/>
+      <c r="B12" s="301" t="inlineStr">
+        <is>
+          <t>BUAD 310</t>
+        </is>
+      </c>
+      <c r="C12" s="300" t="inlineStr">
+        <is>
+          <t>Applied Business Statistics</t>
+        </is>
+      </c>
+      <c r="D12" s="301" t="inlineStr">
+        <is>
+          <t>Marshall Core</t>
+        </is>
+      </c>
+      <c r="E12" s="301" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F12" s="301" t="inlineStr"/>
+      <c r="G12" s="301" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="297" t="inlineStr"/>
+      <c r="B13" s="297" t="inlineStr">
+        <is>
+          <t>GE-D Course</t>
+        </is>
+      </c>
+      <c r="C13" s="298" t="inlineStr">
+        <is>
+          <t>Approved Life Sciences Course</t>
+        </is>
+      </c>
+      <c r="D13" s="297" t="inlineStr">
+        <is>
+          <t>GE Category D</t>
+        </is>
+      </c>
+      <c r="E13" s="297" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F13" s="297" t="inlineStr"/>
+      <c r="G13" s="297" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="296" t="inlineStr">
+        <is>
+          <t>Spring 2028</t>
+        </is>
+      </c>
+      <c r="B14" s="301" t="inlineStr">
+        <is>
+          <t>BUAD 311</t>
+        </is>
+      </c>
+      <c r="C14" s="300" t="inlineStr">
+        <is>
+          <t>Operations Management</t>
+        </is>
+      </c>
+      <c r="D14" s="301" t="inlineStr">
+        <is>
+          <t>Marshall Core</t>
+        </is>
+      </c>
+      <c r="E14" s="301" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F14" s="301" t="inlineStr">
+        <is>
+          <t>12.0</t>
+        </is>
+      </c>
+      <c r="G14" s="301" t="inlineStr">
+        <is>
+          <t>102.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="297" t="inlineStr"/>
+      <c r="B15" s="297" t="inlineStr">
+        <is>
+          <t>WRIT 340</t>
+        </is>
+      </c>
+      <c r="C15" s="298" t="inlineStr">
+        <is>
+          <t>Advanced Writing</t>
+        </is>
+      </c>
+      <c r="D15" s="297" t="inlineStr">
+        <is>
+          <t>Upper Division Writing</t>
+        </is>
+      </c>
+      <c r="E15" s="297" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F15" s="297" t="inlineStr"/>
+      <c r="G15" s="297" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="301" t="inlineStr"/>
+      <c r="B16" s="301" t="inlineStr">
+        <is>
+          <t>GE-E Course</t>
+        </is>
+      </c>
+      <c r="C16" s="300" t="inlineStr">
+        <is>
+          <t>Approved Physical Sciences Course</t>
+        </is>
+      </c>
+      <c r="D16" s="301" t="inlineStr">
+        <is>
+          <t>GE Category E</t>
+        </is>
+      </c>
+      <c r="E16" s="301" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F16" s="301" t="inlineStr"/>
+      <c r="G16" s="301" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="296" t="inlineStr">
+        <is>
+          <t>Fall 2028</t>
+        </is>
+      </c>
+      <c r="B17" s="297" t="inlineStr">
+        <is>
+          <t>BUAD 425</t>
+        </is>
+      </c>
+      <c r="C17" s="298" t="inlineStr">
+        <is>
+          <t>Data Analysis for Decision Making</t>
+        </is>
+      </c>
+      <c r="D17" s="297" t="inlineStr">
+        <is>
+          <t>Marshall Core</t>
+        </is>
+      </c>
+      <c r="E17" s="297" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="F17" s="297" t="inlineStr">
+        <is>
+          <t>14.0</t>
+        </is>
+      </c>
+      <c r="G17" s="297" t="inlineStr">
+        <is>
+          <t>116.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="301" t="inlineStr"/>
+      <c r="B18" s="301" t="inlineStr">
+        <is>
+          <t>Elective</t>
+        </is>
+      </c>
+      <c r="C18" s="300" t="inlineStr">
+        <is>
+          <t>Upper-Division Marshall Elective (1 of 3)</t>
+        </is>
+      </c>
+      <c r="D18" s="301" t="inlineStr">
+        <is>
+          <t>Major Elective</t>
+        </is>
+      </c>
+      <c r="E18" s="301" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F18" s="301" t="inlineStr"/>
+      <c r="G18" s="301" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="297" t="inlineStr"/>
+      <c r="B19" s="297" t="inlineStr">
+        <is>
+          <t>Elective</t>
+        </is>
+      </c>
+      <c r="C19" s="298" t="inlineStr">
+        <is>
+          <t>Upper-Division Marshall Elective (2 of 3)</t>
+        </is>
+      </c>
+      <c r="D19" s="297" t="inlineStr">
+        <is>
+          <t>Major Elective</t>
+        </is>
+      </c>
+      <c r="E19" s="297" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F19" s="297" t="inlineStr"/>
+      <c r="G19" s="297" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="301" t="inlineStr"/>
+      <c r="B20" s="301" t="inlineStr">
+        <is>
+          <t>Elective</t>
+        </is>
+      </c>
+      <c r="C20" s="300" t="inlineStr">
+        <is>
+          <t>General Free Elective</t>
+        </is>
+      </c>
+      <c r="D20" s="301" t="inlineStr">
+        <is>
+          <t>Degree Units</t>
+        </is>
+      </c>
+      <c r="E20" s="301" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F20" s="301" t="inlineStr"/>
+      <c r="G20" s="301" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="296" t="inlineStr">
+        <is>
+          <t>Spring 2029</t>
+        </is>
+      </c>
+      <c r="B21" s="297" t="inlineStr">
+        <is>
+          <t>BUAD 497</t>
+        </is>
+      </c>
+      <c r="C21" s="298" t="inlineStr">
+        <is>
+          <t>Strategic Management</t>
+        </is>
+      </c>
+      <c r="D21" s="297" t="inlineStr">
+        <is>
+          <t>Capstone Core</t>
+        </is>
+      </c>
+      <c r="E21" s="297" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F21" s="297" t="inlineStr">
+        <is>
+          <t>12.0</t>
+        </is>
+      </c>
+      <c r="G21" s="297" t="inlineStr">
+        <is>
+          <t>128.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="301" t="inlineStr"/>
+      <c r="B22" s="301" t="inlineStr">
+        <is>
+          <t>Elective</t>
+        </is>
+      </c>
+      <c r="C22" s="300" t="inlineStr">
+        <is>
+          <t>Upper-Division Marshall Elective (3 of 3)</t>
+        </is>
+      </c>
+      <c r="D22" s="301" t="inlineStr">
+        <is>
+          <t>Major Elective</t>
+        </is>
+      </c>
+      <c r="E22" s="301" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F22" s="301" t="inlineStr"/>
+      <c r="G22" s="301" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="297" t="inlineStr"/>
+      <c r="B23" s="297" t="inlineStr">
+        <is>
+          <t>Elective</t>
+        </is>
+      </c>
+      <c r="C23" s="298" t="inlineStr">
+        <is>
+          <t>General Free Elective</t>
+        </is>
+      </c>
+      <c r="D23" s="297" t="inlineStr">
+        <is>
+          <t>Degree Units</t>
+        </is>
+      </c>
+      <c r="E23" s="297" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="F23" s="297" t="inlineStr"/>
+      <c r="G23" s="297" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00FF7F0E"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -7182,19 +7886,19 @@
           <t>Midterm 1</t>
         </is>
       </c>
-      <c r="B11" s="265" t="inlineStr">
+      <c r="B11" s="290" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C11" s="266" t="inlineStr"/>
-      <c r="D11" s="266" t="inlineStr">
+      <c r="C11" s="291" t="inlineStr"/>
+      <c r="D11" s="291" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="E11" s="266" t="inlineStr"/>
-      <c r="F11" s="266" t="inlineStr">
+      <c r="E11" s="291" t="inlineStr"/>
+      <c r="F11" s="291" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -7210,15 +7914,15 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B12" s="267" t="inlineStr"/>
-      <c r="C12" s="267" t="inlineStr"/>
-      <c r="D12" s="267" t="inlineStr">
+      <c r="B12" s="292" t="inlineStr"/>
+      <c r="C12" s="292" t="inlineStr"/>
+      <c r="D12" s="292" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="E12" s="267" t="inlineStr"/>
-      <c r="F12" s="267" t="inlineStr"/>
+      <c r="E12" s="292" t="inlineStr"/>
+      <c r="F12" s="292" t="inlineStr"/>
       <c r="G12" s="58" t="inlineStr">
         <is>
           <t>9/30 Midterm 1: 250 Points Chapters 1, 2, 3, 4, 5, 8</t>
@@ -7231,19 +7935,19 @@
           <t>Midterm 2</t>
         </is>
       </c>
-      <c r="B13" s="265" t="inlineStr">
+      <c r="B13" s="290" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C13" s="268" t="inlineStr"/>
-      <c r="D13" s="268" t="inlineStr">
+      <c r="C13" s="293" t="inlineStr"/>
+      <c r="D13" s="293" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E13" s="268" t="inlineStr"/>
-      <c r="F13" s="268" t="inlineStr">
+      <c r="E13" s="293" t="inlineStr"/>
+      <c r="F13" s="293" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -7259,15 +7963,15 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B14" s="267" t="inlineStr"/>
-      <c r="C14" s="267" t="inlineStr"/>
-      <c r="D14" s="267" t="inlineStr">
+      <c r="B14" s="292" t="inlineStr"/>
+      <c r="C14" s="292" t="inlineStr"/>
+      <c r="D14" s="292" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="E14" s="267" t="inlineStr"/>
-      <c r="F14" s="267" t="inlineStr"/>
+      <c r="E14" s="292" t="inlineStr"/>
+      <c r="F14" s="292" t="inlineStr"/>
       <c r="G14" s="58" t="inlineStr">
         <is>
           <t>10/26 Midterm 2: 250 Points Chapters 6, 7, 9, &amp; 16</t>
@@ -7280,19 +7984,19 @@
           <t>Final Exam</t>
         </is>
       </c>
-      <c r="B15" s="265" t="inlineStr">
+      <c r="B15" s="290" t="inlineStr">
         <is>
           <t>250 pts</t>
         </is>
       </c>
-      <c r="C15" s="266" t="inlineStr"/>
-      <c r="D15" s="266" t="inlineStr">
+      <c r="C15" s="291" t="inlineStr"/>
+      <c r="D15" s="291" t="inlineStr">
         <is>
           <t>2026-12-16</t>
         </is>
       </c>
-      <c r="E15" s="266" t="inlineStr"/>
-      <c r="F15" s="266" t="inlineStr">
+      <c r="E15" s="291" t="inlineStr"/>
+      <c r="F15" s="291" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -7308,15 +8012,15 @@
           <t>Exam</t>
         </is>
       </c>
-      <c r="B16" s="267" t="inlineStr"/>
-      <c r="C16" s="267" t="inlineStr"/>
-      <c r="D16" s="267" t="inlineStr">
+      <c r="B16" s="292" t="inlineStr"/>
+      <c r="C16" s="292" t="inlineStr"/>
+      <c r="D16" s="292" t="inlineStr">
         <is>
           <t>2026-12-16</t>
         </is>
       </c>
-      <c r="E16" s="267" t="inlineStr"/>
-      <c r="F16" s="267" t="inlineStr"/>
+      <c r="E16" s="292" t="inlineStr"/>
+      <c r="F16" s="292" t="inlineStr"/>
       <c r="G16" s="58" t="inlineStr">
         <is>
           <t>Final Exam</t>
@@ -7329,19 +8033,19 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B17" s="265" t="inlineStr">
+      <c r="B17" s="290" t="inlineStr">
         <is>
           <t>170 pts</t>
         </is>
       </c>
-      <c r="C17" s="268" t="inlineStr"/>
-      <c r="D17" s="268" t="inlineStr">
+      <c r="C17" s="293" t="inlineStr"/>
+      <c r="D17" s="293" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E17" s="268" t="inlineStr"/>
-      <c r="F17" s="268" t="inlineStr">
+      <c r="E17" s="293" t="inlineStr"/>
+      <c r="F17" s="293" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -7357,15 +8061,15 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B18" s="267" t="inlineStr"/>
-      <c r="C18" s="267" t="inlineStr"/>
-      <c r="D18" s="267" t="inlineStr">
+      <c r="B18" s="292" t="inlineStr"/>
+      <c r="C18" s="292" t="inlineStr"/>
+      <c r="D18" s="292" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="E18" s="267" t="inlineStr"/>
-      <c r="F18" s="267" t="inlineStr"/>
+      <c r="E18" s="292" t="inlineStr"/>
+      <c r="F18" s="292" t="inlineStr"/>
       <c r="G18" s="58" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - Product Cost Accumulation: Job; Order Co: Chapter 3</t>
@@ -7378,15 +8082,15 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B19" s="267" t="inlineStr"/>
-      <c r="C19" s="267" t="inlineStr"/>
-      <c r="D19" s="267" t="inlineStr">
+      <c r="B19" s="292" t="inlineStr"/>
+      <c r="C19" s="292" t="inlineStr"/>
+      <c r="D19" s="292" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="E19" s="267" t="inlineStr"/>
-      <c r="F19" s="267" t="inlineStr"/>
+      <c r="E19" s="292" t="inlineStr"/>
+      <c r="F19" s="292" t="inlineStr"/>
       <c r="G19" s="58" t="inlineStr">
         <is>
           <t>Class 5 (9/9) - 2-29, 2-30, 2-40; 15 Points</t>
@@ -7399,15 +8103,15 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B20" s="267" t="inlineStr"/>
-      <c r="C20" s="267" t="inlineStr"/>
-      <c r="D20" s="267" t="inlineStr">
+      <c r="B20" s="292" t="inlineStr"/>
+      <c r="C20" s="292" t="inlineStr"/>
+      <c r="D20" s="292" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E20" s="267" t="inlineStr"/>
-      <c r="F20" s="267" t="inlineStr"/>
+      <c r="E20" s="292" t="inlineStr"/>
+      <c r="F20" s="292" t="inlineStr"/>
       <c r="G20" s="58" t="inlineStr">
         <is>
           <t>Class 7 (9/16) - Activity Based Costing: Chapter 5- ONLY; LO 5.1, 2, 4 &amp; 5</t>
@@ -7420,15 +8124,15 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B21" s="267" t="inlineStr"/>
-      <c r="C21" s="267" t="inlineStr"/>
-      <c r="D21" s="267" t="inlineStr">
+      <c r="B21" s="292" t="inlineStr"/>
+      <c r="C21" s="292" t="inlineStr"/>
+      <c r="D21" s="292" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="E21" s="267" t="inlineStr"/>
-      <c r="F21" s="267" t="inlineStr"/>
+      <c r="E21" s="292" t="inlineStr"/>
+      <c r="F21" s="292" t="inlineStr"/>
       <c r="G21" s="58" t="inlineStr">
         <is>
           <t>Class 7 (9/16) - 3-24, 3-28, 3-32; 15 Points</t>
@@ -7441,15 +8145,15 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B22" s="267" t="inlineStr"/>
-      <c r="C22" s="267" t="inlineStr"/>
-      <c r="D22" s="267" t="inlineStr">
+      <c r="B22" s="292" t="inlineStr"/>
+      <c r="C22" s="292" t="inlineStr"/>
+      <c r="D22" s="292" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="E22" s="267" t="inlineStr"/>
-      <c r="F22" s="267" t="inlineStr"/>
+      <c r="E22" s="292" t="inlineStr"/>
+      <c r="F22" s="292" t="inlineStr"/>
       <c r="G22" s="58" t="inlineStr">
         <is>
           <t>Class 8 (9/21) - Product Cost Accumulation: Pro-; cess Co: Chapter 4- ONLY; LO 4.1, 3, 4, &amp; 5</t>
@@ -7462,15 +8166,15 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B23" s="267" t="inlineStr"/>
-      <c r="C23" s="267" t="inlineStr"/>
-      <c r="D23" s="267" t="inlineStr">
+      <c r="B23" s="292" t="inlineStr"/>
+      <c r="C23" s="292" t="inlineStr"/>
+      <c r="D23" s="292" t="inlineStr">
         <is>
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="E23" s="267" t="inlineStr"/>
-      <c r="F23" s="267" t="inlineStr"/>
+      <c r="E23" s="292" t="inlineStr"/>
+      <c r="F23" s="292" t="inlineStr"/>
       <c r="G23" s="58" t="inlineStr">
         <is>
           <t>Class 8 (9/21) - 5-27 5-46; 10 Points</t>
@@ -7483,15 +8187,15 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B24" s="267" t="inlineStr"/>
-      <c r="C24" s="267" t="inlineStr"/>
-      <c r="D24" s="267" t="inlineStr">
+      <c r="B24" s="292" t="inlineStr"/>
+      <c r="C24" s="292" t="inlineStr"/>
+      <c r="D24" s="292" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="E24" s="267" t="inlineStr"/>
-      <c r="F24" s="267" t="inlineStr"/>
+      <c r="E24" s="292" t="inlineStr"/>
+      <c r="F24" s="292" t="inlineStr"/>
       <c r="G24" s="58" t="inlineStr">
         <is>
           <t>Class 9 (9/23) - Cost of Quality &amp; ESG &amp;; Overview of; • : Chapter 8 - ONLY; LO 8.7, 8, 9</t>
@@ -7504,15 +8208,15 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B25" s="267" t="inlineStr"/>
-      <c r="C25" s="267" t="inlineStr"/>
-      <c r="D25" s="267" t="inlineStr">
+      <c r="B25" s="292" t="inlineStr"/>
+      <c r="C25" s="292" t="inlineStr"/>
+      <c r="D25" s="292" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="E25" s="267" t="inlineStr"/>
-      <c r="F25" s="267" t="inlineStr"/>
+      <c r="E25" s="292" t="inlineStr"/>
+      <c r="F25" s="292" t="inlineStr"/>
       <c r="G25" s="58" t="inlineStr">
         <is>
           <t>Class 9 (9/23) - 4-21, 4-22; 10 Points</t>
@@ -7525,15 +8229,15 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B26" s="267" t="inlineStr"/>
-      <c r="C26" s="267" t="inlineStr"/>
-      <c r="D26" s="267" t="inlineStr">
+      <c r="B26" s="292" t="inlineStr"/>
+      <c r="C26" s="292" t="inlineStr"/>
+      <c r="D26" s="292" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E26" s="267" t="inlineStr"/>
-      <c r="F26" s="267" t="inlineStr"/>
+      <c r="E26" s="292" t="inlineStr"/>
+      <c r="F26" s="292" t="inlineStr"/>
       <c r="G26" s="58" t="inlineStr">
         <is>
           <t>Class 10 (9/28) - Catchup &amp; Midterm Review</t>
@@ -7546,15 +8250,15 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B27" s="267" t="inlineStr"/>
-      <c r="C27" s="267" t="inlineStr"/>
-      <c r="D27" s="267" t="inlineStr">
+      <c r="B27" s="292" t="inlineStr"/>
+      <c r="C27" s="292" t="inlineStr"/>
+      <c r="D27" s="292" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="E27" s="267" t="inlineStr"/>
-      <c r="F27" s="267" t="inlineStr"/>
+      <c r="E27" s="292" t="inlineStr"/>
+      <c r="F27" s="292" t="inlineStr"/>
       <c r="G27" s="58" t="inlineStr">
         <is>
           <t>Class 10 (9/28) - 8-28, 8-29; 10 Points</t>
@@ -7567,15 +8271,15 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B28" s="267" t="inlineStr"/>
-      <c r="C28" s="267" t="inlineStr"/>
-      <c r="D28" s="267" t="inlineStr">
+      <c r="B28" s="292" t="inlineStr"/>
+      <c r="C28" s="292" t="inlineStr"/>
+      <c r="D28" s="292" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="E28" s="267" t="inlineStr"/>
-      <c r="F28" s="267" t="inlineStr"/>
+      <c r="E28" s="292" t="inlineStr"/>
+      <c r="F28" s="292" t="inlineStr"/>
       <c r="G28" s="58" t="inlineStr">
         <is>
           <t>Class 12 (10/7) - Cost volume profit analysis: Chapter 7</t>
@@ -7588,15 +8292,15 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B29" s="267" t="inlineStr"/>
-      <c r="C29" s="267" t="inlineStr"/>
-      <c r="D29" s="267" t="inlineStr">
+      <c r="B29" s="292" t="inlineStr"/>
+      <c r="C29" s="292" t="inlineStr"/>
+      <c r="D29" s="292" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="E29" s="267" t="inlineStr"/>
-      <c r="F29" s="267" t="inlineStr"/>
+      <c r="E29" s="292" t="inlineStr"/>
+      <c r="F29" s="292" t="inlineStr"/>
       <c r="G29" s="58" t="inlineStr">
         <is>
           <t>Class 12 (10/7) - 6-24, 6-25, 6-34; 15 Points</t>
@@ -7609,15 +8313,15 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B30" s="267" t="inlineStr"/>
-      <c r="C30" s="267" t="inlineStr"/>
-      <c r="D30" s="267" t="inlineStr">
+      <c r="B30" s="292" t="inlineStr"/>
+      <c r="C30" s="292" t="inlineStr"/>
+      <c r="D30" s="292" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E30" s="267" t="inlineStr"/>
-      <c r="F30" s="267" t="inlineStr"/>
+      <c r="E30" s="292" t="inlineStr"/>
+      <c r="F30" s="292" t="inlineStr"/>
       <c r="G30" s="58" t="inlineStr">
         <is>
           <t>Class 14 (10/14) - Financial planning and analysis:; Static: Chapter 9</t>
@@ -7630,15 +8334,15 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B31" s="267" t="inlineStr"/>
-      <c r="C31" s="267" t="inlineStr"/>
-      <c r="D31" s="267" t="inlineStr">
+      <c r="B31" s="292" t="inlineStr"/>
+      <c r="C31" s="292" t="inlineStr"/>
+      <c r="D31" s="292" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="E31" s="267" t="inlineStr"/>
-      <c r="F31" s="267" t="inlineStr"/>
+      <c r="E31" s="292" t="inlineStr"/>
+      <c r="F31" s="292" t="inlineStr"/>
       <c r="G31" s="58" t="inlineStr">
         <is>
           <t>Class 14 (10/14) - 7-29, 7-33, 7-40; 15 Points</t>
@@ -7651,15 +8355,15 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B32" s="267" t="inlineStr"/>
-      <c r="C32" s="267" t="inlineStr"/>
-      <c r="D32" s="267" t="inlineStr">
+      <c r="B32" s="292" t="inlineStr"/>
+      <c r="C32" s="292" t="inlineStr"/>
+      <c r="D32" s="292" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E32" s="267" t="inlineStr"/>
-      <c r="F32" s="267" t="inlineStr"/>
+      <c r="E32" s="292" t="inlineStr"/>
+      <c r="F32" s="292" t="inlineStr"/>
       <c r="G32" s="58" t="inlineStr">
         <is>
           <t>Class 15 (10/19) - Capital Budgeting; Practice Midterm Ques: Chapter 16- ONLY; LO 16.1, 2, 3</t>
@@ -7672,15 +8376,15 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B33" s="267" t="inlineStr"/>
-      <c r="C33" s="267" t="inlineStr"/>
-      <c r="D33" s="267" t="inlineStr">
+      <c r="B33" s="292" t="inlineStr"/>
+      <c r="C33" s="292" t="inlineStr"/>
+      <c r="D33" s="292" t="inlineStr">
         <is>
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="E33" s="267" t="inlineStr"/>
-      <c r="F33" s="267" t="inlineStr"/>
+      <c r="E33" s="292" t="inlineStr"/>
+      <c r="F33" s="292" t="inlineStr"/>
       <c r="G33" s="58" t="inlineStr">
         <is>
           <t>Class 15 (10/19) - 9-25, 9-28, 9-37; 15 - Points</t>
@@ -7693,15 +8397,15 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B34" s="267" t="inlineStr"/>
-      <c r="C34" s="267" t="inlineStr"/>
-      <c r="D34" s="267" t="inlineStr">
+      <c r="B34" s="292" t="inlineStr"/>
+      <c r="C34" s="292" t="inlineStr"/>
+      <c r="D34" s="292" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E34" s="267" t="inlineStr"/>
-      <c r="F34" s="267" t="inlineStr"/>
+      <c r="E34" s="292" t="inlineStr"/>
+      <c r="F34" s="292" t="inlineStr"/>
       <c r="G34" s="58" t="inlineStr">
         <is>
           <t>Class 16 (10/21) - Catchup &amp; Midterm Review</t>
@@ -7714,15 +8418,15 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B35" s="267" t="inlineStr"/>
-      <c r="C35" s="267" t="inlineStr"/>
-      <c r="D35" s="267" t="inlineStr">
+      <c r="B35" s="292" t="inlineStr"/>
+      <c r="C35" s="292" t="inlineStr"/>
+      <c r="D35" s="292" t="inlineStr">
         <is>
           <t>2026-10-21</t>
         </is>
       </c>
-      <c r="E35" s="267" t="inlineStr"/>
-      <c r="F35" s="267" t="inlineStr"/>
+      <c r="E35" s="292" t="inlineStr"/>
+      <c r="F35" s="292" t="inlineStr"/>
       <c r="G35" s="58" t="inlineStr">
         <is>
           <t>Class 16 (10/21) - 16-28, 16-40; 10 Points</t>
@@ -7735,15 +8439,15 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B36" s="267" t="inlineStr"/>
-      <c r="C36" s="267" t="inlineStr"/>
-      <c r="D36" s="267" t="inlineStr">
+      <c r="B36" s="292" t="inlineStr"/>
+      <c r="C36" s="292" t="inlineStr"/>
+      <c r="D36" s="292" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="E36" s="267" t="inlineStr"/>
-      <c r="F36" s="267" t="inlineStr"/>
+      <c r="E36" s="292" t="inlineStr"/>
+      <c r="F36" s="292" t="inlineStr"/>
       <c r="G36" s="58" t="inlineStr">
         <is>
           <t>Class 19 (11/4) - Sales Variance Analysis; Flexible Budget: Chapter 11 - ONLY; LO 11.1, 11.2 &amp;; Appendix B</t>
@@ -7756,15 +8460,15 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B37" s="267" t="inlineStr"/>
-      <c r="C37" s="267" t="inlineStr"/>
-      <c r="D37" s="267" t="inlineStr">
+      <c r="B37" s="292" t="inlineStr"/>
+      <c r="C37" s="292" t="inlineStr"/>
+      <c r="D37" s="292" t="inlineStr">
         <is>
           <t>2026-11-04</t>
         </is>
       </c>
-      <c r="E37" s="267" t="inlineStr"/>
-      <c r="F37" s="267" t="inlineStr"/>
+      <c r="E37" s="292" t="inlineStr"/>
+      <c r="F37" s="292" t="inlineStr"/>
       <c r="G37" s="58" t="inlineStr">
         <is>
           <t>Class 19 (11/4) - 10-26, 10-30; 10 Points</t>
@@ -7777,15 +8481,15 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B38" s="267" t="inlineStr"/>
-      <c r="C38" s="267" t="inlineStr"/>
-      <c r="D38" s="267" t="inlineStr">
+      <c r="B38" s="292" t="inlineStr"/>
+      <c r="C38" s="292" t="inlineStr"/>
+      <c r="D38" s="292" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E38" s="267" t="inlineStr"/>
-      <c r="F38" s="267" t="inlineStr"/>
+      <c r="E38" s="292" t="inlineStr"/>
+      <c r="F38" s="292" t="inlineStr"/>
       <c r="G38" s="58" t="inlineStr">
         <is>
           <t>Class 20 (11/9) - Investment Centers: Chapter 13- ONLY; LO 13-1, 2, 3, 4</t>
@@ -7798,15 +8502,15 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B39" s="267" t="inlineStr"/>
-      <c r="C39" s="267" t="inlineStr"/>
-      <c r="D39" s="267" t="inlineStr">
+      <c r="B39" s="292" t="inlineStr"/>
+      <c r="C39" s="292" t="inlineStr"/>
+      <c r="D39" s="292" t="inlineStr">
         <is>
           <t>2026-11-09</t>
         </is>
       </c>
-      <c r="E39" s="267" t="inlineStr"/>
-      <c r="F39" s="267" t="inlineStr"/>
+      <c r="E39" s="292" t="inlineStr"/>
+      <c r="F39" s="292" t="inlineStr"/>
       <c r="G39" s="58" t="inlineStr">
         <is>
           <t>Class 20 (11/9) - 11-31, 11-52; 10 Points</t>
@@ -7819,15 +8523,15 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B40" s="267" t="inlineStr"/>
-      <c r="C40" s="267" t="inlineStr"/>
-      <c r="D40" s="267" t="inlineStr">
+      <c r="B40" s="292" t="inlineStr"/>
+      <c r="C40" s="292" t="inlineStr"/>
+      <c r="D40" s="292" t="inlineStr">
         <is>
           <t>2026-11-16</t>
         </is>
       </c>
-      <c r="E40" s="267" t="inlineStr"/>
-      <c r="F40" s="267" t="inlineStr"/>
+      <c r="E40" s="292" t="inlineStr"/>
+      <c r="F40" s="292" t="inlineStr"/>
       <c r="G40" s="58" t="inlineStr">
         <is>
           <t>Class 21 (11/16) - AI &amp; FP&amp;A</t>
@@ -7840,15 +8544,15 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B41" s="267" t="inlineStr"/>
-      <c r="C41" s="267" t="inlineStr"/>
-      <c r="D41" s="267" t="inlineStr">
+      <c r="B41" s="292" t="inlineStr"/>
+      <c r="C41" s="292" t="inlineStr"/>
+      <c r="D41" s="292" t="inlineStr">
         <is>
           <t>2026-11-16</t>
         </is>
       </c>
-      <c r="E41" s="267" t="inlineStr"/>
-      <c r="F41" s="267" t="inlineStr"/>
+      <c r="E41" s="292" t="inlineStr"/>
+      <c r="F41" s="292" t="inlineStr"/>
       <c r="G41" s="58" t="inlineStr">
         <is>
           <t>Class 21 (11/16) - 13-29, 13-33; 10 Points</t>
@@ -7861,15 +8565,15 @@
           <t>Reading</t>
         </is>
       </c>
-      <c r="B42" s="267" t="inlineStr"/>
-      <c r="C42" s="267" t="inlineStr"/>
-      <c r="D42" s="267" t="inlineStr">
+      <c r="B42" s="292" t="inlineStr"/>
+      <c r="C42" s="292" t="inlineStr"/>
+      <c r="D42" s="292" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E42" s="267" t="inlineStr"/>
-      <c r="F42" s="267" t="inlineStr"/>
+      <c r="E42" s="292" t="inlineStr"/>
+      <c r="F42" s="292" t="inlineStr"/>
       <c r="G42" s="58" t="inlineStr">
         <is>
           <t>Class 2 (12/2) - Catchup &amp; Final Review; Practice Final Questions Posted to Brightspace at; 5:00 PM</t>
@@ -7882,15 +8586,15 @@
           <t>Homework</t>
         </is>
       </c>
-      <c r="B43" s="267" t="inlineStr"/>
-      <c r="C43" s="267" t="inlineStr"/>
-      <c r="D43" s="267" t="inlineStr">
+      <c r="B43" s="292" t="inlineStr"/>
+      <c r="C43" s="292" t="inlineStr"/>
+      <c r="D43" s="292" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E43" s="267" t="inlineStr"/>
-      <c r="F43" s="267" t="inlineStr"/>
+      <c r="E43" s="292" t="inlineStr"/>
+      <c r="F43" s="292" t="inlineStr"/>
       <c r="G43" s="58" t="inlineStr">
         <is>
           <t>Class 2 (12/2) - 14-35, 14-41; 10 Points; Assignments listed Be-; low Due by11:59 PM; Linked In Learning; E</t>
@@ -7903,23 +8607,23 @@
           <t>LinkedIn Learning Excel Certification</t>
         </is>
       </c>
-      <c r="B44" s="265" t="inlineStr">
+      <c r="B44" s="290" t="inlineStr">
         <is>
           <t>75 pts</t>
         </is>
       </c>
-      <c r="C44" s="266" t="inlineStr">
+      <c r="C44" s="291" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D44" s="266" t="inlineStr">
+      <c r="D44" s="291" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E44" s="266" t="inlineStr"/>
-      <c r="F44" s="266" t="inlineStr">
+      <c r="E44" s="291" t="inlineStr"/>
+      <c r="F44" s="291" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -7935,19 +8639,19 @@
           <t>Certification</t>
         </is>
       </c>
-      <c r="B45" s="267" t="inlineStr"/>
-      <c r="C45" s="267" t="inlineStr">
+      <c r="B45" s="292" t="inlineStr"/>
+      <c r="C45" s="292" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D45" s="267" t="inlineStr">
+      <c r="D45" s="292" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E45" s="267" t="inlineStr"/>
-      <c r="F45" s="267" t="inlineStr"/>
+      <c r="E45" s="292" t="inlineStr"/>
+      <c r="F45" s="292" t="inlineStr"/>
       <c r="G45" s="58" t="inlineStr">
         <is>
           <t>LinkedIn Learning Excel Certification</t>
@@ -7960,23 +8664,23 @@
           <t>Stukent Simternship</t>
         </is>
       </c>
-      <c r="B46" s="265" t="inlineStr">
+      <c r="B46" s="290" t="inlineStr">
         <is>
           <t>75 pts</t>
         </is>
       </c>
-      <c r="C46" s="268" t="inlineStr">
+      <c r="C46" s="293" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D46" s="268" t="inlineStr">
+      <c r="D46" s="293" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E46" s="268" t="inlineStr"/>
-      <c r="F46" s="268" t="inlineStr">
+      <c r="E46" s="293" t="inlineStr"/>
+      <c r="F46" s="293" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -7992,19 +8696,19 @@
           <t>Certification</t>
         </is>
       </c>
-      <c r="B47" s="267" t="inlineStr"/>
-      <c r="C47" s="267" t="inlineStr">
+      <c r="B47" s="292" t="inlineStr"/>
+      <c r="C47" s="292" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
-      <c r="D47" s="267" t="inlineStr">
+      <c r="D47" s="292" t="inlineStr">
         <is>
           <t>2026-12-02</t>
         </is>
       </c>
-      <c r="E47" s="267" t="inlineStr"/>
-      <c r="F47" s="267" t="inlineStr"/>
+      <c r="E47" s="292" t="inlineStr"/>
+      <c r="F47" s="292" t="inlineStr"/>
       <c r="G47" s="58" t="inlineStr">
         <is>
           <t>Stukent Simternship</t>
@@ -8037,7 +8741,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001F77B4"/>
@@ -9292,7 +9996,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="009467BD"/>
@@ -10511,7 +11215,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00D62728"/>
@@ -11515,7 +12219,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002CA02C"/>
@@ -12762,7 +13466,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="008C564B"/>
@@ -13354,7 +14058,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00FF7F0E"/>

</xml_diff>